<commit_message>
M1-17: acceso con WhatsApp o correo + PIN
- Usuario por WhatsApp (cambiable) con correo opcional; PIN de 6 dígitos o contraseña fuerte para roles sensibles
- Activación por enlace de un solo uso (WhatsApp de quien invita, sin costo) y reinicio por administrador
- Recuperación por correo; sin SMS en el MVP
- Bloqueo tras 5 intentos, límite por IP y sesión de 90 días
- Cambio de número con autoservicio (exige PIN) y registro en bitácora
- Bitácora de solo-añadir (AuditEvent)
- Pantallas: entrar, activar, recuperar, mi cuenta e invitar; componentes Alert y AuthLayout
- Documentación: v3.3 y matriz de trazabilidad actualizada

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/trazabilidad/Matriz de Trazabilidad MDF.xlsx
+++ b/docs/trazabilidad/Matriz de Trazabilidad MDF.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Origen v1" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Matriz'!$A$1:$N$92</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Matriz'!$A$1:$N$94</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -897,31 +897,31 @@
         </is>
       </c>
       <c r="B5" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$92,$A5)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$94,$A5)</f>
         <v/>
       </c>
       <c r="C5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$92,$A5,Matriz!$L$2:$L$92,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$94,$A5,Matriz!$L$2:$L$94,"Pendiente")</f>
         <v/>
       </c>
       <c r="D5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$92,$A5,Matriz!$L$2:$L$92,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$94,$A5,Matriz!$L$2:$L$94,"En diseño")</f>
         <v/>
       </c>
       <c r="E5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$92,$A5,Matriz!$L$2:$L$92,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$94,$A5,Matriz!$L$2:$L$94,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$92,$A5,Matriz!$L$2:$L$92,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$94,$A5,Matriz!$L$2:$L$94,"En pruebas")</f>
         <v/>
       </c>
       <c r="G5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$92,$A5,Matriz!$L$2:$L$92,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$94,$A5,Matriz!$L$2:$L$94,"Hecho")</f>
         <v/>
       </c>
       <c r="H5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$92,$A5,Matriz!$L$2:$L$92,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$94,$A5,Matriz!$L$2:$L$94,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I5" s="13">
@@ -936,31 +936,31 @@
         </is>
       </c>
       <c r="B6" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$92,$A6)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$94,$A6)</f>
         <v/>
       </c>
       <c r="C6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$92,$A6,Matriz!$L$2:$L$92,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$94,$A6,Matriz!$L$2:$L$94,"Pendiente")</f>
         <v/>
       </c>
       <c r="D6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$92,$A6,Matriz!$L$2:$L$92,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$94,$A6,Matriz!$L$2:$L$94,"En diseño")</f>
         <v/>
       </c>
       <c r="E6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$92,$A6,Matriz!$L$2:$L$92,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$94,$A6,Matriz!$L$2:$L$94,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$92,$A6,Matriz!$L$2:$L$92,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$94,$A6,Matriz!$L$2:$L$94,"En pruebas")</f>
         <v/>
       </c>
       <c r="G6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$92,$A6,Matriz!$L$2:$L$92,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$94,$A6,Matriz!$L$2:$L$94,"Hecho")</f>
         <v/>
       </c>
       <c r="H6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$92,$A6,Matriz!$L$2:$L$92,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$94,$A6,Matriz!$L$2:$L$94,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I6" s="13">
@@ -975,31 +975,31 @@
         </is>
       </c>
       <c r="B7" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$92,$A7)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$94,$A7)</f>
         <v/>
       </c>
       <c r="C7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$92,$A7,Matriz!$L$2:$L$92,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$94,$A7,Matriz!$L$2:$L$94,"Pendiente")</f>
         <v/>
       </c>
       <c r="D7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$92,$A7,Matriz!$L$2:$L$92,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$94,$A7,Matriz!$L$2:$L$94,"En diseño")</f>
         <v/>
       </c>
       <c r="E7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$92,$A7,Matriz!$L$2:$L$92,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$94,$A7,Matriz!$L$2:$L$94,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$92,$A7,Matriz!$L$2:$L$92,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$94,$A7,Matriz!$L$2:$L$94,"En pruebas")</f>
         <v/>
       </c>
       <c r="G7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$92,$A7,Matriz!$L$2:$L$92,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$94,$A7,Matriz!$L$2:$L$94,"Hecho")</f>
         <v/>
       </c>
       <c r="H7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$92,$A7,Matriz!$L$2:$L$92,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$94,$A7,Matriz!$L$2:$L$94,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I7" s="13">
@@ -1014,31 +1014,31 @@
         </is>
       </c>
       <c r="B8" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$92,$A8)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$94,$A8)</f>
         <v/>
       </c>
       <c r="C8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$92,$A8,Matriz!$L$2:$L$92,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$94,$A8,Matriz!$L$2:$L$94,"Pendiente")</f>
         <v/>
       </c>
       <c r="D8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$92,$A8,Matriz!$L$2:$L$92,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$94,$A8,Matriz!$L$2:$L$94,"En diseño")</f>
         <v/>
       </c>
       <c r="E8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$92,$A8,Matriz!$L$2:$L$92,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$94,$A8,Matriz!$L$2:$L$94,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$92,$A8,Matriz!$L$2:$L$92,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$94,$A8,Matriz!$L$2:$L$94,"En pruebas")</f>
         <v/>
       </c>
       <c r="G8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$92,$A8,Matriz!$L$2:$L$92,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$94,$A8,Matriz!$L$2:$L$94,"Hecho")</f>
         <v/>
       </c>
       <c r="H8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$92,$A8,Matriz!$L$2:$L$92,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$94,$A8,Matriz!$L$2:$L$94,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I8" s="13">
@@ -1053,31 +1053,31 @@
         </is>
       </c>
       <c r="B9" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$92,$A9)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$94,$A9)</f>
         <v/>
       </c>
       <c r="C9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$92,$A9,Matriz!$L$2:$L$92,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$94,$A9,Matriz!$L$2:$L$94,"Pendiente")</f>
         <v/>
       </c>
       <c r="D9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$92,$A9,Matriz!$L$2:$L$92,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$94,$A9,Matriz!$L$2:$L$94,"En diseño")</f>
         <v/>
       </c>
       <c r="E9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$92,$A9,Matriz!$L$2:$L$92,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$94,$A9,Matriz!$L$2:$L$94,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$92,$A9,Matriz!$L$2:$L$92,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$94,$A9,Matriz!$L$2:$L$94,"En pruebas")</f>
         <v/>
       </c>
       <c r="G9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$92,$A9,Matriz!$L$2:$L$92,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$94,$A9,Matriz!$L$2:$L$94,"Hecho")</f>
         <v/>
       </c>
       <c r="H9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$92,$A9,Matriz!$L$2:$L$92,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$94,$A9,Matriz!$L$2:$L$94,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I9" s="13">
@@ -1092,31 +1092,31 @@
         </is>
       </c>
       <c r="B10" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$92,$A10)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$94,$A10)</f>
         <v/>
       </c>
       <c r="C10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$92,$A10,Matriz!$L$2:$L$92,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$94,$A10,Matriz!$L$2:$L$94,"Pendiente")</f>
         <v/>
       </c>
       <c r="D10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$92,$A10,Matriz!$L$2:$L$92,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$94,$A10,Matriz!$L$2:$L$94,"En diseño")</f>
         <v/>
       </c>
       <c r="E10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$92,$A10,Matriz!$L$2:$L$92,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$94,$A10,Matriz!$L$2:$L$94,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$92,$A10,Matriz!$L$2:$L$92,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$94,$A10,Matriz!$L$2:$L$94,"En pruebas")</f>
         <v/>
       </c>
       <c r="G10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$92,$A10,Matriz!$L$2:$L$92,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$94,$A10,Matriz!$L$2:$L$94,"Hecho")</f>
         <v/>
       </c>
       <c r="H10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$92,$A10,Matriz!$L$2:$L$92,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$94,$A10,Matriz!$L$2:$L$94,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I10" s="13">
@@ -1131,31 +1131,31 @@
         </is>
       </c>
       <c r="B11" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$92,$A11)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$94,$A11)</f>
         <v/>
       </c>
       <c r="C11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$92,$A11,Matriz!$L$2:$L$92,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$94,$A11,Matriz!$L$2:$L$94,"Pendiente")</f>
         <v/>
       </c>
       <c r="D11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$92,$A11,Matriz!$L$2:$L$92,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$94,$A11,Matriz!$L$2:$L$94,"En diseño")</f>
         <v/>
       </c>
       <c r="E11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$92,$A11,Matriz!$L$2:$L$92,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$94,$A11,Matriz!$L$2:$L$94,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$92,$A11,Matriz!$L$2:$L$92,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$94,$A11,Matriz!$L$2:$L$94,"En pruebas")</f>
         <v/>
       </c>
       <c r="G11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$92,$A11,Matriz!$L$2:$L$92,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$94,$A11,Matriz!$L$2:$L$94,"Hecho")</f>
         <v/>
       </c>
       <c r="H11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$92,$A11,Matriz!$L$2:$L$92,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$94,$A11,Matriz!$L$2:$L$94,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I11" s="13">
@@ -1256,31 +1256,31 @@
         </is>
       </c>
       <c r="B16" s="12">
-        <f>COUNTIF(Matriz!$H$2:$H$92,$A16)</f>
+        <f>COUNTIF(Matriz!$H$2:$H$94,$A16)</f>
         <v/>
       </c>
       <c r="C16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$92,$A16,Matriz!$L$2:$L$92,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$94,$A16,Matriz!$L$2:$L$94,"Pendiente")</f>
         <v/>
       </c>
       <c r="D16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$92,$A16,Matriz!$L$2:$L$92,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$94,$A16,Matriz!$L$2:$L$94,"En diseño")</f>
         <v/>
       </c>
       <c r="E16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$92,$A16,Matriz!$L$2:$L$92,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$94,$A16,Matriz!$L$2:$L$94,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$92,$A16,Matriz!$L$2:$L$92,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$94,$A16,Matriz!$L$2:$L$94,"En pruebas")</f>
         <v/>
       </c>
       <c r="G16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$92,$A16,Matriz!$L$2:$L$92,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$94,$A16,Matriz!$L$2:$L$94,"Hecho")</f>
         <v/>
       </c>
       <c r="H16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$92,$A16,Matriz!$L$2:$L$92,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$94,$A16,Matriz!$L$2:$L$94,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I16" s="13">
@@ -1295,31 +1295,31 @@
         </is>
       </c>
       <c r="B17" s="12">
-        <f>COUNTIF(Matriz!$H$2:$H$92,$A17)</f>
+        <f>COUNTIF(Matriz!$H$2:$H$94,$A17)</f>
         <v/>
       </c>
       <c r="C17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$92,$A17,Matriz!$L$2:$L$92,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$94,$A17,Matriz!$L$2:$L$94,"Pendiente")</f>
         <v/>
       </c>
       <c r="D17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$92,$A17,Matriz!$L$2:$L$92,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$94,$A17,Matriz!$L$2:$L$94,"En diseño")</f>
         <v/>
       </c>
       <c r="E17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$92,$A17,Matriz!$L$2:$L$92,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$94,$A17,Matriz!$L$2:$L$94,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$92,$A17,Matriz!$L$2:$L$92,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$94,$A17,Matriz!$L$2:$L$94,"En pruebas")</f>
         <v/>
       </c>
       <c r="G17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$92,$A17,Matriz!$L$2:$L$92,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$94,$A17,Matriz!$L$2:$L$94,"Hecho")</f>
         <v/>
       </c>
       <c r="H17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$92,$A17,Matriz!$L$2:$L$92,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$94,$A17,Matriz!$L$2:$L$94,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I17" s="13">
@@ -1334,31 +1334,31 @@
         </is>
       </c>
       <c r="B18" s="12">
-        <f>COUNTIF(Matriz!$H$2:$H$92,$A18)</f>
+        <f>COUNTIF(Matriz!$H$2:$H$94,$A18)</f>
         <v/>
       </c>
       <c r="C18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$92,$A18,Matriz!$L$2:$L$92,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$94,$A18,Matriz!$L$2:$L$94,"Pendiente")</f>
         <v/>
       </c>
       <c r="D18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$92,$A18,Matriz!$L$2:$L$92,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$94,$A18,Matriz!$L$2:$L$94,"En diseño")</f>
         <v/>
       </c>
       <c r="E18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$92,$A18,Matriz!$L$2:$L$92,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$94,$A18,Matriz!$L$2:$L$94,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$92,$A18,Matriz!$L$2:$L$92,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$94,$A18,Matriz!$L$2:$L$94,"En pruebas")</f>
         <v/>
       </c>
       <c r="G18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$92,$A18,Matriz!$L$2:$L$92,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$94,$A18,Matriz!$L$2:$L$94,"Hecho")</f>
         <v/>
       </c>
       <c r="H18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$92,$A18,Matriz!$L$2:$L$92,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$94,$A18,Matriz!$L$2:$L$94,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I18" s="13">
@@ -1373,31 +1373,31 @@
         </is>
       </c>
       <c r="B19" s="12">
-        <f>COUNTIF(Matriz!$H$2:$H$92,$A19)</f>
+        <f>COUNTIF(Matriz!$H$2:$H$94,$A19)</f>
         <v/>
       </c>
       <c r="C19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$92,$A19,Matriz!$L$2:$L$92,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$94,$A19,Matriz!$L$2:$L$94,"Pendiente")</f>
         <v/>
       </c>
       <c r="D19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$92,$A19,Matriz!$L$2:$L$92,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$94,$A19,Matriz!$L$2:$L$94,"En diseño")</f>
         <v/>
       </c>
       <c r="E19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$92,$A19,Matriz!$L$2:$L$92,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$94,$A19,Matriz!$L$2:$L$94,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$92,$A19,Matriz!$L$2:$L$92,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$94,$A19,Matriz!$L$2:$L$94,"En pruebas")</f>
         <v/>
       </c>
       <c r="G19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$92,$A19,Matriz!$L$2:$L$92,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$94,$A19,Matriz!$L$2:$L$94,"Hecho")</f>
         <v/>
       </c>
       <c r="H19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$92,$A19,Matriz!$L$2:$L$92,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$94,$A19,Matriz!$L$2:$L$94,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I19" s="13">
@@ -1498,31 +1498,31 @@
         </is>
       </c>
       <c r="B24" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$92,$A24)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$94,$A24)</f>
         <v/>
       </c>
       <c r="C24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$92,$A24,Matriz!$L$2:$L$92,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$94,$A24,Matriz!$L$2:$L$94,"Pendiente")</f>
         <v/>
       </c>
       <c r="D24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$92,$A24,Matriz!$L$2:$L$92,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$94,$A24,Matriz!$L$2:$L$94,"En diseño")</f>
         <v/>
       </c>
       <c r="E24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$92,$A24,Matriz!$L$2:$L$92,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$94,$A24,Matriz!$L$2:$L$94,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$92,$A24,Matriz!$L$2:$L$92,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$94,$A24,Matriz!$L$2:$L$94,"En pruebas")</f>
         <v/>
       </c>
       <c r="G24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$92,$A24,Matriz!$L$2:$L$92,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$94,$A24,Matriz!$L$2:$L$94,"Hecho")</f>
         <v/>
       </c>
       <c r="H24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$92,$A24,Matriz!$L$2:$L$92,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$94,$A24,Matriz!$L$2:$L$94,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I24" s="13">
@@ -1537,31 +1537,31 @@
         </is>
       </c>
       <c r="B25" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$92,$A25)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$94,$A25)</f>
         <v/>
       </c>
       <c r="C25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$92,$A25,Matriz!$L$2:$L$92,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$94,$A25,Matriz!$L$2:$L$94,"Pendiente")</f>
         <v/>
       </c>
       <c r="D25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$92,$A25,Matriz!$L$2:$L$92,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$94,$A25,Matriz!$L$2:$L$94,"En diseño")</f>
         <v/>
       </c>
       <c r="E25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$92,$A25,Matriz!$L$2:$L$92,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$94,$A25,Matriz!$L$2:$L$94,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$92,$A25,Matriz!$L$2:$L$92,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$94,$A25,Matriz!$L$2:$L$94,"En pruebas")</f>
         <v/>
       </c>
       <c r="G25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$92,$A25,Matriz!$L$2:$L$92,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$94,$A25,Matriz!$L$2:$L$94,"Hecho")</f>
         <v/>
       </c>
       <c r="H25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$92,$A25,Matriz!$L$2:$L$92,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$94,$A25,Matriz!$L$2:$L$94,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I25" s="13">
@@ -1576,31 +1576,31 @@
         </is>
       </c>
       <c r="B26" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$92,$A26)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$94,$A26)</f>
         <v/>
       </c>
       <c r="C26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$92,$A26,Matriz!$L$2:$L$92,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$94,$A26,Matriz!$L$2:$L$94,"Pendiente")</f>
         <v/>
       </c>
       <c r="D26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$92,$A26,Matriz!$L$2:$L$92,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$94,$A26,Matriz!$L$2:$L$94,"En diseño")</f>
         <v/>
       </c>
       <c r="E26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$92,$A26,Matriz!$L$2:$L$92,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$94,$A26,Matriz!$L$2:$L$94,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$92,$A26,Matriz!$L$2:$L$92,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$94,$A26,Matriz!$L$2:$L$94,"En pruebas")</f>
         <v/>
       </c>
       <c r="G26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$92,$A26,Matriz!$L$2:$L$92,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$94,$A26,Matriz!$L$2:$L$94,"Hecho")</f>
         <v/>
       </c>
       <c r="H26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$92,$A26,Matriz!$L$2:$L$92,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$94,$A26,Matriz!$L$2:$L$94,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I26" s="13">
@@ -1615,31 +1615,31 @@
         </is>
       </c>
       <c r="B27" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$92,$A27)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$94,$A27)</f>
         <v/>
       </c>
       <c r="C27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$92,$A27,Matriz!$L$2:$L$92,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$94,$A27,Matriz!$L$2:$L$94,"Pendiente")</f>
         <v/>
       </c>
       <c r="D27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$92,$A27,Matriz!$L$2:$L$92,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$94,$A27,Matriz!$L$2:$L$94,"En diseño")</f>
         <v/>
       </c>
       <c r="E27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$92,$A27,Matriz!$L$2:$L$92,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$94,$A27,Matriz!$L$2:$L$94,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$92,$A27,Matriz!$L$2:$L$92,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$94,$A27,Matriz!$L$2:$L$94,"En pruebas")</f>
         <v/>
       </c>
       <c r="G27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$92,$A27,Matriz!$L$2:$L$92,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$94,$A27,Matriz!$L$2:$L$94,"Hecho")</f>
         <v/>
       </c>
       <c r="H27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$92,$A27,Matriz!$L$2:$L$92,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$94,$A27,Matriz!$L$2:$L$94,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I27" s="13">
@@ -1654,31 +1654,31 @@
         </is>
       </c>
       <c r="B28" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$92,$A28)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$94,$A28)</f>
         <v/>
       </c>
       <c r="C28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$92,$A28,Matriz!$L$2:$L$92,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$94,$A28,Matriz!$L$2:$L$94,"Pendiente")</f>
         <v/>
       </c>
       <c r="D28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$92,$A28,Matriz!$L$2:$L$92,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$94,$A28,Matriz!$L$2:$L$94,"En diseño")</f>
         <v/>
       </c>
       <c r="E28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$92,$A28,Matriz!$L$2:$L$92,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$94,$A28,Matriz!$L$2:$L$94,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$92,$A28,Matriz!$L$2:$L$92,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$94,$A28,Matriz!$L$2:$L$94,"En pruebas")</f>
         <v/>
       </c>
       <c r="G28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$92,$A28,Matriz!$L$2:$L$92,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$94,$A28,Matriz!$L$2:$L$94,"Hecho")</f>
         <v/>
       </c>
       <c r="H28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$92,$A28,Matriz!$L$2:$L$92,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$94,$A28,Matriz!$L$2:$L$94,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I28" s="13">
@@ -1693,31 +1693,31 @@
         </is>
       </c>
       <c r="B29" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$92,$A29)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$94,$A29)</f>
         <v/>
       </c>
       <c r="C29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$92,$A29,Matriz!$L$2:$L$92,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$94,$A29,Matriz!$L$2:$L$94,"Pendiente")</f>
         <v/>
       </c>
       <c r="D29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$92,$A29,Matriz!$L$2:$L$92,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$94,$A29,Matriz!$L$2:$L$94,"En diseño")</f>
         <v/>
       </c>
       <c r="E29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$92,$A29,Matriz!$L$2:$L$92,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$94,$A29,Matriz!$L$2:$L$94,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$92,$A29,Matriz!$L$2:$L$92,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$94,$A29,Matriz!$L$2:$L$94,"En pruebas")</f>
         <v/>
       </c>
       <c r="G29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$92,$A29,Matriz!$L$2:$L$92,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$94,$A29,Matriz!$L$2:$L$94,"Hecho")</f>
         <v/>
       </c>
       <c r="H29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$92,$A29,Matriz!$L$2:$L$92,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$94,$A29,Matriz!$L$2:$L$94,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I29" s="13">
@@ -1732,31 +1732,31 @@
         </is>
       </c>
       <c r="B30" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$92,$A30)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$94,$A30)</f>
         <v/>
       </c>
       <c r="C30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$92,$A30,Matriz!$L$2:$L$92,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$94,$A30,Matriz!$L$2:$L$94,"Pendiente")</f>
         <v/>
       </c>
       <c r="D30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$92,$A30,Matriz!$L$2:$L$92,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$94,$A30,Matriz!$L$2:$L$94,"En diseño")</f>
         <v/>
       </c>
       <c r="E30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$92,$A30,Matriz!$L$2:$L$92,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$94,$A30,Matriz!$L$2:$L$94,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$92,$A30,Matriz!$L$2:$L$92,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$94,$A30,Matriz!$L$2:$L$94,"En pruebas")</f>
         <v/>
       </c>
       <c r="G30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$92,$A30,Matriz!$L$2:$L$92,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$94,$A30,Matriz!$L$2:$L$94,"Hecho")</f>
         <v/>
       </c>
       <c r="H30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$92,$A30,Matriz!$L$2:$L$92,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$94,$A30,Matriz!$L$2:$L$94,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I30" s="13">
@@ -1818,7 +1818,7 @@
         </is>
       </c>
       <c r="B35" s="12">
-        <f>COUNTIF(Matriz!$K$2:$K$92,A35)</f>
+        <f>COUNTIF(Matriz!$K$2:$K$94,A35)</f>
         <v/>
       </c>
     </row>
@@ -1829,7 +1829,7 @@
         </is>
       </c>
       <c r="B36" s="12">
-        <f>COUNTIF(Matriz!$K$2:$K$92,A36)</f>
+        <f>COUNTIF(Matriz!$K$2:$K$94,A36)</f>
         <v/>
       </c>
     </row>
@@ -1840,7 +1840,7 @@
         </is>
       </c>
       <c r="B37" s="12">
-        <f>COUNTIF(Matriz!$K$2:$K$92,A37)</f>
+        <f>COUNTIF(Matriz!$K$2:$K$94,A37)</f>
         <v/>
       </c>
     </row>
@@ -1851,7 +1851,7 @@
         </is>
       </c>
       <c r="B38" s="12">
-        <f>COUNTIF(Matriz!$K$2:$K$92,A38)</f>
+        <f>COUNTIF(Matriz!$K$2:$K$94,A38)</f>
         <v/>
       </c>
     </row>
@@ -1866,7 +1866,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N92"/>
+  <dimension ref="A1:N94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3442,12 +3442,12 @@
       </c>
       <c r="C25" s="19" t="inlineStr">
         <is>
-          <t>Acceso con número de WhatsApp y PIN de 6 dígitos. La cuenta se activa con un enlace enviado por WhatsApp (sin costo). La recuperación del PIN se hace por SMS o con apoyo del líder o administrador.</t>
+          <t>Acceso con número de WhatsApp o correo y PIN de 6 dígitos (contraseña de 10+ caracteres para roles sensibles como Pastor, Tesorero y Administrador). La cuenta se activa con un enlace de un solo uso que caduca, enviado desde el WhatsApp de quien invita (sin costo). Recuperación: reinicio por Líder o administrador y enlace por correo si lo tiene. Sin SMS en el MVP.</t>
         </is>
       </c>
       <c r="D25" s="21" t="inlineStr">
         <is>
-          <t>Nuevo v3.1</t>
+          <t>Nuevo v3.1 / v3.3</t>
         </is>
       </c>
       <c r="E25" s="19" t="inlineStr">
@@ -3472,12 +3472,12 @@
       </c>
       <c r="I25" s="19" t="inlineStr">
         <is>
-          <t>Como usuario quiero entrar con mi WhatsApp y un PIN sencillo.</t>
+          <t>Como usuario quiero entrar con mi WhatsApp o correo y un PIN sencillo.</t>
         </is>
       </c>
       <c r="J25" s="19" t="inlineStr">
         <is>
-          <t>Activar la cuenta con enlace, entrar con PIN de 6 dígitos, bloqueo tras intentos fallidos y recuperación por SMS.</t>
+          <t>Activar la cuenta con enlace de un solo uso, entrar con PIN de 6 dígitos (contraseña fuerte en roles sensibles), bloqueo tras 5 intentos y recuperación por Líder, administrador o correo.</t>
         </is>
       </c>
       <c r="K25" s="19" t="inlineStr">
@@ -3487,11 +3487,19 @@
       </c>
       <c r="L25" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M25" s="19" t="inlineStr"/>
-      <c r="N25" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M25" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/m1-17-acceso · 32 pruebas de backend y 4 de frontend pasan</t>
+        </is>
+      </c>
+      <c r="N25" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-05 · Falta probar en dispositivos reales (Android/iOS) y con un Líder.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="18" t="inlineStr">
@@ -3624,52 +3632,52 @@
     <row r="28">
       <c r="A28" s="18" t="inlineStr">
         <is>
-          <t>M2A-01</t>
+          <t>M1-21</t>
         </is>
       </c>
       <c r="B28" s="19" t="inlineStr">
         <is>
-          <t>M2A Cursos de Vida</t>
+          <t>M1 Identidad y comunicación</t>
         </is>
       </c>
       <c r="C28" s="19" t="inlineStr">
         <is>
-          <t>Catálogo dinámico de cursos; se pueden crear nuevos sin intervención técnica. Incluye «Resolución de Varones» y «Toma de Buenas Decisiones», omitidos en v2.</t>
-        </is>
-      </c>
-      <c r="D28" s="22" t="inlineStr">
-        <is>
-          <t>Recuperado v1</t>
+          <t>Cambio de número: el usuario lo actualiza con su PIN actual, el Líder recibe un aviso y queda en bitácora. Si perdió número y teléfono, el Líder o administrador reinicia su acceso. La identidad estable es un ID interno, no el número. El aviso al Líder se activa cuando exista el módulo de Grupos.</t>
+        </is>
+      </c>
+      <c r="D28" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3.3</t>
         </is>
       </c>
       <c r="E28" s="19" t="inlineStr">
         <is>
-          <t>Fuera del MVP</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="F28" s="19" t="inlineStr">
         <is>
-          <t>Fase 3</t>
+          <t>Fase 0</t>
         </is>
       </c>
       <c r="G28" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sprint 1</t>
         </is>
       </c>
       <c r="H28" s="19" t="inlineStr">
         <is>
-          <t>Posterior</t>
-        </is>
-      </c>
-      <c r="I28" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
-        </is>
-      </c>
-      <c r="J28" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
+          <t>H1 · 18-oct (núcleo Fase 0)</t>
+        </is>
+      </c>
+      <c r="I28" s="19" t="inlineStr">
+        <is>
+          <t>Como persona que cambió de número quiero actualizarlo sin perder mi historial.</t>
+        </is>
+      </c>
+      <c r="J28" s="19" t="inlineStr">
+        <is>
+          <t>Cambio con el PIN actual, aviso al Líder y registro en bitácora; si perdió número y teléfono, el Líder o administrador reinicia el acceso.</t>
         </is>
       </c>
       <c r="K28" s="19" t="inlineStr">
@@ -3679,61 +3687,69 @@
       </c>
       <c r="L28" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M28" s="19" t="inlineStr"/>
-      <c r="N28" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M28" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/m1-17-acceso · 32 pruebas de backend y 4 de frontend pasan</t>
+        </is>
+      </c>
+      <c r="N28" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-05 · El aviso al Líder se activa cuando exista Grupos (Sprint 3).</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="18" t="inlineStr">
         <is>
-          <t>M2A-02</t>
+          <t>M1-22</t>
         </is>
       </c>
       <c r="B29" s="19" t="inlineStr">
         <is>
-          <t>M2A Cursos de Vida</t>
+          <t>M1 Identidad y comunicación</t>
         </is>
       </c>
       <c r="C29" s="19" t="inlineStr">
         <is>
-          <t>Flexibilidad operativa: sin día ni horario fijo; el día y el ponente pueden cambiar entre ediciones.</t>
-        </is>
-      </c>
-      <c r="D29" s="19" t="inlineStr">
-        <is>
-          <t>v1 / v2</t>
+          <t>Bloqueo de cuenta tras 5 intentos fallidos durante 15 minutos (configurable), limitación de intentos por IP y sesión de 90 días renovable con el uso.</t>
+        </is>
+      </c>
+      <c r="D29" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3.3</t>
         </is>
       </c>
       <c r="E29" s="19" t="inlineStr">
         <is>
-          <t>Fuera del MVP</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="F29" s="19" t="inlineStr">
         <is>
-          <t>Fase 3</t>
+          <t>Fase 0</t>
         </is>
       </c>
       <c r="G29" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sprint 0</t>
         </is>
       </c>
       <c r="H29" s="19" t="inlineStr">
         <is>
-          <t>Posterior</t>
-        </is>
-      </c>
-      <c r="I29" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
-        </is>
-      </c>
-      <c r="J29" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
+          <t>H1 · 18-oct (núcleo Fase 0)</t>
+        </is>
+      </c>
+      <c r="I29" s="19" t="inlineStr">
+        <is>
+          <t>Como iglesia queremos proteger las cuentas de intentos de adivinar el PIN.</t>
+        </is>
+      </c>
+      <c r="J29" s="19" t="inlineStr">
+        <is>
+          <t>Tras 5 intentos fallidos la cuenta se bloquea 15 minutos; sesión de 90 días renovable.</t>
         </is>
       </c>
       <c r="K29" s="19" t="inlineStr">
@@ -3743,16 +3759,24 @@
       </c>
       <c r="L29" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M29" s="19" t="inlineStr"/>
-      <c r="N29" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M29" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/m1-17-acceso · 32 pruebas de backend y 4 de frontend pasan</t>
+        </is>
+      </c>
+      <c r="N29" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-05 · Límite de intentos por IP: 30 por minuto.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="18" t="inlineStr">
         <is>
-          <t>M2A-03</t>
+          <t>M2A-01</t>
         </is>
       </c>
       <c r="B30" s="19" t="inlineStr">
@@ -3762,12 +3786,12 @@
       </c>
       <c r="C30" s="19" t="inlineStr">
         <is>
-          <t>Reposición de clases: el inscrito puede reponer en otro grupo o con otro ponente, a decisión de quien imparte.</t>
-        </is>
-      </c>
-      <c r="D30" s="19" t="inlineStr">
-        <is>
-          <t>v1 / v2</t>
+          <t>Catálogo dinámico de cursos; se pueden crear nuevos sin intervención técnica. Incluye «Resolución de Varones» y «Toma de Buenas Decisiones», omitidos en v2.</t>
+        </is>
+      </c>
+      <c r="D30" s="22" t="inlineStr">
+        <is>
+          <t>Recuperado v1</t>
         </is>
       </c>
       <c r="E30" s="19" t="inlineStr">
@@ -3816,7 +3840,7 @@
     <row r="31">
       <c r="A31" s="18" t="inlineStr">
         <is>
-          <t>M2A-04</t>
+          <t>M2A-02</t>
         </is>
       </c>
       <c r="B31" s="19" t="inlineStr">
@@ -3826,7 +3850,7 @@
       </c>
       <c r="C31" s="19" t="inlineStr">
         <is>
-          <t>Registro de asistencia por sesión.</t>
+          <t>Flexibilidad operativa: sin día ni horario fijo; el día y el ponente pueden cambiar entre ediciones.</t>
         </is>
       </c>
       <c r="D31" s="19" t="inlineStr">
@@ -3880,7 +3904,7 @@
     <row r="32">
       <c r="A32" s="18" t="inlineStr">
         <is>
-          <t>M2A-05</t>
+          <t>M2A-03</t>
         </is>
       </c>
       <c r="B32" s="19" t="inlineStr">
@@ -3890,7 +3914,7 @@
       </c>
       <c r="C32" s="19" t="inlineStr">
         <is>
-          <t>Seguimiento de tareas o actividades opcionales (no sumativas).</t>
+          <t>Reposición de clases: el inscrito puede reponer en otro grupo o con otro ponente, a decisión de quien imparte.</t>
         </is>
       </c>
       <c r="D32" s="19" t="inlineStr">
@@ -3944,7 +3968,7 @@
     <row r="33">
       <c r="A33" s="18" t="inlineStr">
         <is>
-          <t>M2A-06</t>
+          <t>M2A-04</t>
         </is>
       </c>
       <c r="B33" s="19" t="inlineStr">
@@ -3954,7 +3978,7 @@
       </c>
       <c r="C33" s="19" t="inlineStr">
         <is>
-          <t>Inscripción: quién se inscribe, cuándo lo hizo, si tiene adeudo y qué incluye el costo (materiales, hospedaje, etc.).</t>
+          <t>Registro de asistencia por sesión.</t>
         </is>
       </c>
       <c r="D33" s="19" t="inlineStr">
@@ -4008,7 +4032,7 @@
     <row r="34">
       <c r="A34" s="18" t="inlineStr">
         <is>
-          <t>M2A-07</t>
+          <t>M2A-05</t>
         </is>
       </c>
       <c r="B34" s="19" t="inlineStr">
@@ -4018,12 +4042,12 @@
       </c>
       <c r="C34" s="19" t="inlineStr">
         <is>
-          <t>Registro de pagos, saldo de adeudos y recibo. Por definir: captura manual vs. pasarela de pago, y si se requiere corte de caja.</t>
-        </is>
-      </c>
-      <c r="D34" s="21" t="inlineStr">
-        <is>
-          <t>Nuevo v3</t>
+          <t>Seguimiento de tareas o actividades opcionales (no sumativas).</t>
+        </is>
+      </c>
+      <c r="D34" s="19" t="inlineStr">
+        <is>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E34" s="19" t="inlineStr">
@@ -4058,7 +4082,7 @@
       </c>
       <c r="K34" s="19" t="inlineStr">
         <is>
-          <t>Por definir</t>
+          <t>VoBo pendiente</t>
         </is>
       </c>
       <c r="L34" s="19" t="inlineStr">
@@ -4072,7 +4096,7 @@
     <row r="35">
       <c r="A35" s="18" t="inlineStr">
         <is>
-          <t>M2A-08</t>
+          <t>M2A-06</t>
         </is>
       </c>
       <c r="B35" s="19" t="inlineStr">
@@ -4082,12 +4106,12 @@
       </c>
       <c r="C35" s="19" t="inlineStr">
         <is>
-          <t>Tablero del curso tipo mensajería para avisos antes del curso y días posteriores, con notificación a los inscritos.</t>
-        </is>
-      </c>
-      <c r="D35" s="22" t="inlineStr">
-        <is>
-          <t>Recuperado v1</t>
+          <t>Inscripción: quién se inscribe, cuándo lo hizo, si tiene adeudo y qué incluye el costo (materiales, hospedaje, etc.).</t>
+        </is>
+      </c>
+      <c r="D35" s="19" t="inlineStr">
+        <is>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E35" s="19" t="inlineStr">
@@ -4136,7 +4160,7 @@
     <row r="36">
       <c r="A36" s="18" t="inlineStr">
         <is>
-          <t>M2A-09</t>
+          <t>M2A-07</t>
         </is>
       </c>
       <c r="B36" s="19" t="inlineStr">
@@ -4146,12 +4170,12 @@
       </c>
       <c r="C36" s="19" t="inlineStr">
         <is>
-          <t>Evaluación docente configurable: formulario diseñable (tipo Google Forms) aplicado al finalizar el curso.</t>
-        </is>
-      </c>
-      <c r="D36" s="19" t="inlineStr">
-        <is>
-          <t>v1 / v2</t>
+          <t>Registro de pagos, saldo de adeudos y recibo. Por definir: captura manual vs. pasarela de pago, y si se requiere corte de caja.</t>
+        </is>
+      </c>
+      <c r="D36" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3</t>
         </is>
       </c>
       <c r="E36" s="19" t="inlineStr">
@@ -4186,7 +4210,7 @@
       </c>
       <c r="K36" s="19" t="inlineStr">
         <is>
-          <t>VoBo pendiente</t>
+          <t>Por definir</t>
         </is>
       </c>
       <c r="L36" s="19" t="inlineStr">
@@ -4200,7 +4224,7 @@
     <row r="37">
       <c r="A37" s="18" t="inlineStr">
         <is>
-          <t>M2A-10</t>
+          <t>M2A-08</t>
         </is>
       </c>
       <c r="B37" s="19" t="inlineStr">
@@ -4210,7 +4234,7 @@
       </c>
       <c r="C37" s="19" t="inlineStr">
         <is>
-          <t>Evolución del ponente: historial de evaluaciones por ponente a lo largo del tiempo y entre ediciones.</t>
+          <t>Tablero del curso tipo mensajería para avisos antes del curso y días posteriores, con notificación a los inscritos.</t>
         </is>
       </c>
       <c r="D37" s="22" t="inlineStr">
@@ -4264,7 +4288,7 @@
     <row r="38">
       <c r="A38" s="18" t="inlineStr">
         <is>
-          <t>M2A-11</t>
+          <t>M2A-09</t>
         </is>
       </c>
       <c r="B38" s="19" t="inlineStr">
@@ -4274,7 +4298,7 @@
       </c>
       <c r="C38" s="19" t="inlineStr">
         <is>
-          <t>Reconocimiento de participación (diploma) opcional por curso.</t>
+          <t>Evaluación docente configurable: formulario diseñable (tipo Google Forms) aplicado al finalizar el curso.</t>
         </is>
       </c>
       <c r="D38" s="19" t="inlineStr">
@@ -4328,22 +4352,22 @@
     <row r="39">
       <c r="A39" s="18" t="inlineStr">
         <is>
-          <t>M2B-01</t>
+          <t>M2A-10</t>
         </is>
       </c>
       <c r="B39" s="19" t="inlineStr">
         <is>
-          <t>M2B Cursos escolarizados</t>
+          <t>M2A Cursos de Vida</t>
         </is>
       </c>
       <c r="C39" s="19" t="inlineStr">
         <is>
-          <t>Control riguroso de asistencia.</t>
-        </is>
-      </c>
-      <c r="D39" s="19" t="inlineStr">
-        <is>
-          <t>v1 / v2</t>
+          <t>Evolución del ponente: historial de evaluaciones por ponente a lo largo del tiempo y entre ediciones.</t>
+        </is>
+      </c>
+      <c r="D39" s="22" t="inlineStr">
+        <is>
+          <t>Recuperado v1</t>
         </is>
       </c>
       <c r="E39" s="19" t="inlineStr">
@@ -4392,17 +4416,17 @@
     <row r="40">
       <c r="A40" s="18" t="inlineStr">
         <is>
-          <t>M2B-02</t>
+          <t>M2A-11</t>
         </is>
       </c>
       <c r="B40" s="19" t="inlineStr">
         <is>
-          <t>M2B Cursos escolarizados</t>
+          <t>M2A Cursos de Vida</t>
         </is>
       </c>
       <c r="C40" s="19" t="inlineStr">
         <is>
-          <t>Entrega de tareas y trabajos continuos (incluidos trabajos extra).</t>
+          <t>Reconocimiento de participación (diploma) opcional por curso.</t>
         </is>
       </c>
       <c r="D40" s="19" t="inlineStr">
@@ -4456,7 +4480,7 @@
     <row r="41">
       <c r="A41" s="18" t="inlineStr">
         <is>
-          <t>M2B-03</t>
+          <t>M2B-01</t>
         </is>
       </c>
       <c r="B41" s="19" t="inlineStr">
@@ -4466,7 +4490,7 @@
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>Ponderación de calificaciones y exámenes finales.</t>
+          <t>Control riguroso de asistencia.</t>
         </is>
       </c>
       <c r="D41" s="19" t="inlineStr">
@@ -4520,7 +4544,7 @@
     <row r="42">
       <c r="A42" s="18" t="inlineStr">
         <is>
-          <t>M2B-04</t>
+          <t>M2B-02</t>
         </is>
       </c>
       <c r="B42" s="19" t="inlineStr">
@@ -4530,12 +4554,12 @@
       </c>
       <c r="C42" s="19" t="inlineStr">
         <is>
-          <t>Creador de exámenes en línea: opción múltiple, preguntas abiertas, falso/verdadero y respuesta corta.</t>
+          <t>Entrega de tareas y trabajos continuos (incluidos trabajos extra).</t>
         </is>
       </c>
       <c r="D42" s="19" t="inlineStr">
         <is>
-          <t>v2</t>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E42" s="19" t="inlineStr">
@@ -4584,7 +4608,7 @@
     <row r="43">
       <c r="A43" s="18" t="inlineStr">
         <is>
-          <t>M2B-05</t>
+          <t>M2B-03</t>
         </is>
       </c>
       <c r="B43" s="19" t="inlineStr">
@@ -4594,7 +4618,7 @@
       </c>
       <c r="C43" s="19" t="inlineStr">
         <is>
-          <t>Boleta digital con el formato definido por la iglesia. Por definir: formato oficial de la boleta.</t>
+          <t>Ponderación de calificaciones y exámenes finales.</t>
         </is>
       </c>
       <c r="D43" s="19" t="inlineStr">
@@ -4634,7 +4658,7 @@
       </c>
       <c r="K43" s="19" t="inlineStr">
         <is>
-          <t>Por definir</t>
+          <t>VoBo pendiente</t>
         </is>
       </c>
       <c r="L43" s="19" t="inlineStr">
@@ -4648,7 +4672,7 @@
     <row r="44">
       <c r="A44" s="18" t="inlineStr">
         <is>
-          <t>M2B-06</t>
+          <t>M2B-04</t>
         </is>
       </c>
       <c r="B44" s="19" t="inlineStr">
@@ -4658,7 +4682,7 @@
       </c>
       <c r="C44" s="19" t="inlineStr">
         <is>
-          <t>Historial académico permanente en el Expediente Digital, aunque cambie el maestro o el alumno pierda su comprobante.</t>
+          <t>Creador de exámenes en línea: opción múltiple, preguntas abiertas, falso/verdadero y respuesta corta.</t>
         </is>
       </c>
       <c r="D44" s="19" t="inlineStr">
@@ -4712,57 +4736,57 @@
     <row r="45">
       <c r="A45" s="18" t="inlineStr">
         <is>
-          <t>M3-01</t>
+          <t>M2B-05</t>
         </is>
       </c>
       <c r="B45" s="19" t="inlineStr">
         <is>
-          <t>M3 Grupos de Conexión</t>
+          <t>M2B Cursos escolarizados</t>
         </is>
       </c>
       <c r="C45" s="19" t="inlineStr">
         <is>
-          <t>Estructura del grupo con roles: Supervisor (supervisa uno o varios grupos y reporta al Pastor), Líder, Secretario, Anfitrión y Tesorero.</t>
+          <t>Boleta digital con el formato definido por la iglesia. Por definir: formato oficial de la boleta.</t>
         </is>
       </c>
       <c r="D45" s="19" t="inlineStr">
         <is>
-          <t>v3 + Obs. 4</t>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E45" s="19" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Fuera del MVP</t>
         </is>
       </c>
       <c r="F45" s="19" t="inlineStr">
         <is>
-          <t>Fase 1</t>
+          <t>Fase 3</t>
         </is>
       </c>
       <c r="G45" s="19" t="inlineStr">
         <is>
-          <t>Sprint 3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H45" s="19" t="inlineStr">
         <is>
-          <t>H3 · MVP (Grupos)</t>
-        </is>
-      </c>
-      <c r="I45" s="19" t="inlineStr">
-        <is>
-          <t>Como supervisor quiero asignar Líder, Secretario, Anfitrión y Tesorero a cada grupo.</t>
-        </is>
-      </c>
-      <c r="J45" s="19" t="inlineStr">
-        <is>
-          <t>Un grupo tiene sus roles asignados; un supervisor ve varios grupos.</t>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="I45" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
+        </is>
+      </c>
+      <c r="J45" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
         </is>
       </c>
       <c r="K45" s="19" t="inlineStr">
         <is>
-          <t>VoBo pendiente</t>
+          <t>Por definir</t>
         </is>
       </c>
       <c r="L45" s="19" t="inlineStr">
@@ -4776,52 +4800,52 @@
     <row r="46">
       <c r="A46" s="18" t="inlineStr">
         <is>
-          <t>M3-02</t>
+          <t>M2B-06</t>
         </is>
       </c>
       <c r="B46" s="19" t="inlineStr">
         <is>
-          <t>M3 Grupos de Conexión</t>
+          <t>M2B Cursos escolarizados</t>
         </is>
       </c>
       <c r="C46" s="19" t="inlineStr">
         <is>
-          <t>Distribución del estudio semanal dentro de la app, sustituyendo el envío por WhatsApp.</t>
+          <t>Historial académico permanente en el Expediente Digital, aunque cambie el maestro o el alumno pierda su comprobante.</t>
         </is>
       </c>
       <c r="D46" s="19" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>v2</t>
         </is>
       </c>
       <c r="E46" s="19" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Fuera del MVP</t>
         </is>
       </c>
       <c r="F46" s="19" t="inlineStr">
         <is>
-          <t>Fase 1</t>
+          <t>Fase 3</t>
         </is>
       </c>
       <c r="G46" s="19" t="inlineStr">
         <is>
-          <t>Sprint 3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H46" s="19" t="inlineStr">
         <is>
-          <t>H3 · MVP (Grupos)</t>
-        </is>
-      </c>
-      <c r="I46" s="19" t="inlineStr">
-        <is>
-          <t>Como líder quiero recibir el estudio semanal en la app en lugar de WhatsApp.</t>
-        </is>
-      </c>
-      <c r="J46" s="19" t="inlineStr">
-        <is>
-          <t>Publicar el material de la semana; el líder lo abre y queda marca de lectura.</t>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="I46" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
+        </is>
+      </c>
+      <c r="J46" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
         </is>
       </c>
       <c r="K46" s="19" t="inlineStr">
@@ -4840,7 +4864,7 @@
     <row r="47">
       <c r="A47" s="18" t="inlineStr">
         <is>
-          <t>M3-03</t>
+          <t>M3-01</t>
         </is>
       </c>
       <c r="B47" s="19" t="inlineStr">
@@ -4850,12 +4874,12 @@
       </c>
       <c r="C47" s="19" t="inlineStr">
         <is>
-          <t>Pase de lista digital por Secretario o Líder, con captura sin conexión y sincronización posterior.</t>
+          <t>Estructura del grupo con roles: Supervisor (supervisa uno o varios grupos y reporta al Pastor), Líder, Secretario, Anfitrión y Tesorero.</t>
         </is>
       </c>
       <c r="D47" s="19" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>v3 + Obs. 4</t>
         </is>
       </c>
       <c r="E47" s="19" t="inlineStr">
@@ -4880,12 +4904,12 @@
       </c>
       <c r="I47" s="19" t="inlineStr">
         <is>
-          <t>Como secretario quiero pasar lista aunque no haya señal.</t>
+          <t>Como supervisor quiero asignar Líder, Secretario, Anfitrión y Tesorero a cada grupo.</t>
         </is>
       </c>
       <c r="J47" s="19" t="inlineStr">
         <is>
-          <t>Pasar lista en modo avión; al reconectar se sincroniza sin duplicados.</t>
+          <t>Un grupo tiene sus roles asignados; un supervisor ve varios grupos.</t>
         </is>
       </c>
       <c r="K47" s="19" t="inlineStr">
@@ -4904,7 +4928,7 @@
     <row r="48">
       <c r="A48" s="18" t="inlineStr">
         <is>
-          <t>M3-04</t>
+          <t>M3-02</t>
         </is>
       </c>
       <c r="B48" s="19" t="inlineStr">
@@ -4914,12 +4938,12 @@
       </c>
       <c r="C48" s="19" t="inlineStr">
         <is>
-          <t>Ofrendas regulares y especiales. El Tesorero cuenta y avala la cifra con firma electrónica simple (usuario, fecha y hora, monto y código de confirmación). Si su cifra difiere de la capturada, se registra la diferencia.</t>
+          <t>Distribución del estudio semanal dentro de la app, sustituyendo el envío por WhatsApp.</t>
         </is>
       </c>
       <c r="D48" s="19" t="inlineStr">
         <is>
-          <t>v3 + Obs. 4</t>
+          <t>v3</t>
         </is>
       </c>
       <c r="E48" s="19" t="inlineStr">
@@ -4934,7 +4958,7 @@
       </c>
       <c r="G48" s="19" t="inlineStr">
         <is>
-          <t>Sprint 4</t>
+          <t>Sprint 3</t>
         </is>
       </c>
       <c r="H48" s="19" t="inlineStr">
@@ -4944,12 +4968,12 @@
       </c>
       <c r="I48" s="19" t="inlineStr">
         <is>
-          <t>Como tesorero quiero contar y avalar la ofrenda del grupo.</t>
+          <t>Como líder quiero recibir el estudio semanal en la app en lugar de WhatsApp.</t>
         </is>
       </c>
       <c r="J48" s="19" t="inlineStr">
         <is>
-          <t>Capturar monto; el Tesorero captura su cifra; si difiere se registra la diferencia; con aval no se edita sin motivo.</t>
+          <t>Publicar el material de la semana; el líder lo abre y queda marca de lectura.</t>
         </is>
       </c>
       <c r="K48" s="19" t="inlineStr">
@@ -4968,7 +4992,7 @@
     <row r="49">
       <c r="A49" s="18" t="inlineStr">
         <is>
-          <t>M3-05</t>
+          <t>M3-03</t>
         </is>
       </c>
       <c r="B49" s="19" t="inlineStr">
@@ -4978,7 +5002,7 @@
       </c>
       <c r="C49" s="19" t="inlineStr">
         <is>
-          <t>Formulario dinámico de peticiones de oración, con seguimiento pastoral.</t>
+          <t>Pase de lista digital por Secretario o Líder, con captura sin conexión y sincronización posterior.</t>
         </is>
       </c>
       <c r="D49" s="19" t="inlineStr">
@@ -4998,7 +5022,7 @@
       </c>
       <c r="G49" s="19" t="inlineStr">
         <is>
-          <t>Sprint 4</t>
+          <t>Sprint 3</t>
         </is>
       </c>
       <c r="H49" s="19" t="inlineStr">
@@ -5008,12 +5032,12 @@
       </c>
       <c r="I49" s="19" t="inlineStr">
         <is>
-          <t>Como líder quiero recoger peticiones de oración con un formulario configurable.</t>
+          <t>Como secretario quiero pasar lista aunque no haya señal.</t>
         </is>
       </c>
       <c r="J49" s="19" t="inlineStr">
         <is>
-          <t>Capturar una petición; el formulario se edita sin código.</t>
+          <t>Pasar lista en modo avión; al reconectar se sincroniza sin duplicados.</t>
         </is>
       </c>
       <c r="K49" s="19" t="inlineStr">
@@ -5032,7 +5056,7 @@
     <row r="50">
       <c r="A50" s="18" t="inlineStr">
         <is>
-          <t>M3-06</t>
+          <t>M3-04</t>
         </is>
       </c>
       <c r="B50" s="19" t="inlineStr">
@@ -5042,12 +5066,12 @@
       </c>
       <c r="C50" s="19" t="inlineStr">
         <is>
-          <t>Peticiones de oración visibles solo para Líder y roles superiores. Retención de 1 mes o tiempo configurable, con borrado automático.</t>
-        </is>
-      </c>
-      <c r="D50" s="21" t="inlineStr">
-        <is>
-          <t>Resp. P8</t>
+          <t>Ofrendas regulares y especiales. El Tesorero cuenta y avala la cifra con firma electrónica simple (usuario, fecha y hora, monto y reingreso de su PIN). Si su cifra difiere de la capturada, se registra la diferencia.</t>
+        </is>
+      </c>
+      <c r="D50" s="19" t="inlineStr">
+        <is>
+          <t>v3 + Obs. 4</t>
         </is>
       </c>
       <c r="E50" s="19" t="inlineStr">
@@ -5072,12 +5096,12 @@
       </c>
       <c r="I50" s="19" t="inlineStr">
         <is>
-          <t>Como pastor quiero que las peticiones solo las vea el Líder y superiores y se borren al vencer.</t>
+          <t>Como tesorero quiero contar y avalar la ofrenda del grupo.</t>
         </is>
       </c>
       <c r="J50" s="19" t="inlineStr">
         <is>
-          <t>El Secretario no las ve; tras el plazo configurable (por defecto 30 días) se eliminan.</t>
+          <t>Capturar monto; el Tesorero captura su cifra y confirma con su PIN; si difiere se registra la diferencia; con aval no se edita sin motivo.</t>
         </is>
       </c>
       <c r="K50" s="19" t="inlineStr">
@@ -5096,7 +5120,7 @@
     <row r="51">
       <c r="A51" s="18" t="inlineStr">
         <is>
-          <t>M3-07</t>
+          <t>M3-05</t>
         </is>
       </c>
       <c r="B51" s="19" t="inlineStr">
@@ -5106,7 +5130,7 @@
       </c>
       <c r="C51" s="19" t="inlineStr">
         <is>
-          <t>Reportes de supervisión: dashboards de asistencia, ofrendas y crecimiento por grupo, según permisos.</t>
+          <t>Formulario dinámico de peticiones de oración, con seguimiento pastoral.</t>
         </is>
       </c>
       <c r="D51" s="19" t="inlineStr">
@@ -5116,7 +5140,7 @@
       </c>
       <c r="E51" s="19" t="inlineStr">
         <is>
-          <t>MVP básico</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="F51" s="19" t="inlineStr">
@@ -5126,7 +5150,7 @@
       </c>
       <c r="G51" s="19" t="inlineStr">
         <is>
-          <t>Sprint 5</t>
+          <t>Sprint 4</t>
         </is>
       </c>
       <c r="H51" s="19" t="inlineStr">
@@ -5136,12 +5160,12 @@
       </c>
       <c r="I51" s="19" t="inlineStr">
         <is>
-          <t>Como supervisor quiero ver la salud de mis grupos.</t>
+          <t>Como líder quiero recoger peticiones de oración con un formulario configurable.</t>
         </is>
       </c>
       <c r="J51" s="19" t="inlineStr">
         <is>
-          <t>El dashboard muestra asistencia, ofrendas y crecimiento según permisos.</t>
+          <t>Capturar una petición; el formulario se edita sin código.</t>
         </is>
       </c>
       <c r="K51" s="19" t="inlineStr">
@@ -5160,7 +5184,7 @@
     <row r="52">
       <c r="A52" s="18" t="inlineStr">
         <is>
-          <t>M3-08</t>
+          <t>M3-06</t>
         </is>
       </c>
       <c r="B52" s="19" t="inlineStr">
@@ -5170,47 +5194,47 @@
       </c>
       <c r="C52" s="19" t="inlineStr">
         <is>
-          <t>Ubicación de zona del grupo para que personas cercanas lo encuentren, sin exponer el domicilio exacto. Por definir.</t>
-        </is>
-      </c>
-      <c r="D52" s="19" t="inlineStr">
-        <is>
-          <t>v3</t>
+          <t>Peticiones de oración visibles solo para Líder y roles superiores. Retención de 1 mes o tiempo configurable, con borrado automático.</t>
+        </is>
+      </c>
+      <c r="D52" s="21" t="inlineStr">
+        <is>
+          <t>Resp. P8</t>
         </is>
       </c>
       <c r="E52" s="19" t="inlineStr">
         <is>
-          <t>Fuera del MVP</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="F52" s="19" t="inlineStr">
         <is>
-          <t>Fase 4</t>
+          <t>Fase 1</t>
         </is>
       </c>
       <c r="G52" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sprint 4</t>
         </is>
       </c>
       <c r="H52" s="19" t="inlineStr">
         <is>
-          <t>Posterior</t>
-        </is>
-      </c>
-      <c r="I52" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
-        </is>
-      </c>
-      <c r="J52" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
+          <t>H3 · MVP (Grupos)</t>
+        </is>
+      </c>
+      <c r="I52" s="19" t="inlineStr">
+        <is>
+          <t>Como pastor quiero que las peticiones solo las vea el Líder y superiores y se borren al vencer.</t>
+        </is>
+      </c>
+      <c r="J52" s="19" t="inlineStr">
+        <is>
+          <t>El Secretario no las ve; tras el plazo configurable (por defecto 30 días) se eliminan.</t>
         </is>
       </c>
       <c r="K52" s="19" t="inlineStr">
         <is>
-          <t>Por definir</t>
+          <t>VoBo pendiente</t>
         </is>
       </c>
       <c r="L52" s="19" t="inlineStr">
@@ -5224,7 +5248,7 @@
     <row r="53">
       <c r="A53" s="18" t="inlineStr">
         <is>
-          <t>M3-09</t>
+          <t>M3-07</t>
         </is>
       </c>
       <c r="B53" s="19" t="inlineStr">
@@ -5234,17 +5258,17 @@
       </c>
       <c r="C53" s="19" t="inlineStr">
         <is>
-          <t>A un grupo asisten miembros de la iglesia (vecinos o no) e invitados del grupo que no asisten a la iglesia. Los invitados se registran como Contacto con datos mínimos y se les puede invitar a consolidación.</t>
-        </is>
-      </c>
-      <c r="D53" s="21" t="inlineStr">
-        <is>
-          <t>Corrección v3.2</t>
+          <t>Reportes de supervisión: dashboards de asistencia, ofrendas y crecimiento por grupo, según permisos.</t>
+        </is>
+      </c>
+      <c r="D53" s="19" t="inlineStr">
+        <is>
+          <t>v3</t>
         </is>
       </c>
       <c r="E53" s="19" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>MVP básico</t>
         </is>
       </c>
       <c r="F53" s="19" t="inlineStr">
@@ -5254,7 +5278,7 @@
       </c>
       <c r="G53" s="19" t="inlineStr">
         <is>
-          <t>Sprint 3</t>
+          <t>Sprint 5</t>
         </is>
       </c>
       <c r="H53" s="19" t="inlineStr">
@@ -5264,12 +5288,12 @@
       </c>
       <c r="I53" s="19" t="inlineStr">
         <is>
-          <t>Como secretario quiero registrar invitados del grupo con datos mínimos.</t>
+          <t>Como supervisor quiero ver la salud de mis grupos.</t>
         </is>
       </c>
       <c r="J53" s="19" t="inlineStr">
         <is>
-          <t>Registrar un invitado como Contacto y marcarlo presente.</t>
+          <t>El dashboard muestra asistencia, ofrendas y crecimiento según permisos.</t>
         </is>
       </c>
       <c r="K53" s="19" t="inlineStr">
@@ -5288,7 +5312,7 @@
     <row r="54">
       <c r="A54" s="18" t="inlineStr">
         <is>
-          <t>M3-10</t>
+          <t>M3-08</t>
         </is>
       </c>
       <c r="B54" s="19" t="inlineStr">
@@ -5298,42 +5322,42 @@
       </c>
       <c r="C54" s="19" t="inlineStr">
         <is>
-          <t>Confidencialidad de ofrendas y asistencias: consulta limitada por rol (matriz por definir) y modificación restringida, todo en bitácora.</t>
-        </is>
-      </c>
-      <c r="D54" s="21" t="inlineStr">
-        <is>
-          <t>Obs. 5</t>
+          <t>Ubicación de zona del grupo para que personas cercanas lo encuentren, sin exponer el domicilio exacto. Por definir.</t>
+        </is>
+      </c>
+      <c r="D54" s="19" t="inlineStr">
+        <is>
+          <t>v3</t>
         </is>
       </c>
       <c r="E54" s="19" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Fuera del MVP</t>
         </is>
       </c>
       <c r="F54" s="19" t="inlineStr">
         <is>
-          <t>Fase 1</t>
+          <t>Fase 4</t>
         </is>
       </c>
       <c r="G54" s="19" t="inlineStr">
         <is>
-          <t>Sprint 4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H54" s="19" t="inlineStr">
         <is>
-          <t>H3 · MVP (Grupos)</t>
-        </is>
-      </c>
-      <c r="I54" s="19" t="inlineStr">
-        <is>
-          <t>Como pastor quiero que ofrendas y asistencias sean confidenciales.</t>
-        </is>
-      </c>
-      <c r="J54" s="19" t="inlineStr">
-        <is>
-          <t>La matriz de la sección 3.3 del v3.2 se cumple en pruebas por cada rol.</t>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="I54" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
+        </is>
+      </c>
+      <c r="J54" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
         </is>
       </c>
       <c r="K54" s="19" t="inlineStr">
@@ -5352,7 +5376,7 @@
     <row r="55">
       <c r="A55" s="18" t="inlineStr">
         <is>
-          <t>M3-11</t>
+          <t>M3-09</t>
         </is>
       </c>
       <c r="B55" s="19" t="inlineStr">
@@ -5362,12 +5386,12 @@
       </c>
       <c r="C55" s="19" t="inlineStr">
         <is>
-          <t>Dashboard y tablero de mensajes del grupo.</t>
+          <t>A un grupo asisten miembros de la iglesia (vecinos o no) e invitados del grupo que no asisten a la iglesia. Los invitados se registran como Contacto con datos mínimos y se les puede invitar a consolidación.</t>
         </is>
       </c>
       <c r="D55" s="21" t="inlineStr">
         <is>
-          <t>Obs. 7</t>
+          <t>Corrección v3.2</t>
         </is>
       </c>
       <c r="E55" s="19" t="inlineStr">
@@ -5382,7 +5406,7 @@
       </c>
       <c r="G55" s="19" t="inlineStr">
         <is>
-          <t>Sprint 5</t>
+          <t>Sprint 3</t>
         </is>
       </c>
       <c r="H55" s="19" t="inlineStr">
@@ -5392,12 +5416,12 @@
       </c>
       <c r="I55" s="19" t="inlineStr">
         <is>
-          <t>Como líder quiero un tablero de mensajes de mi grupo.</t>
+          <t>Como secretario quiero registrar invitados del grupo con datos mínimos.</t>
         </is>
       </c>
       <c r="J55" s="19" t="inlineStr">
         <is>
-          <t>Publicar y leer mensajes del grupo.</t>
+          <t>Registrar un invitado como Contacto y marcarlo presente.</t>
         </is>
       </c>
       <c r="K55" s="19" t="inlineStr">
@@ -5416,57 +5440,57 @@
     <row r="56">
       <c r="A56" s="18" t="inlineStr">
         <is>
-          <t>M4-01</t>
+          <t>M3-10</t>
         </is>
       </c>
       <c r="B56" s="19" t="inlineStr">
         <is>
-          <t>M4 Kids Check-In/Out</t>
+          <t>M3 Grupos de Conexión</t>
         </is>
       </c>
       <c r="C56" s="19" t="inlineStr">
         <is>
-          <t>Sustitución de la ficha física de papel.</t>
-        </is>
-      </c>
-      <c r="D56" s="19" t="inlineStr">
-        <is>
-          <t>v1 / v2</t>
+          <t>Confidencialidad de ofrendas y asistencias: consulta limitada por rol (matriz por definir) y modificación restringida, todo en bitácora.</t>
+        </is>
+      </c>
+      <c r="D56" s="21" t="inlineStr">
+        <is>
+          <t>Obs. 5</t>
         </is>
       </c>
       <c r="E56" s="19" t="inlineStr">
         <is>
-          <t>Fuera del MVP</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="F56" s="19" t="inlineStr">
         <is>
-          <t>Fase 2</t>
+          <t>Fase 1</t>
         </is>
       </c>
       <c r="G56" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sprint 4</t>
         </is>
       </c>
       <c r="H56" s="19" t="inlineStr">
         <is>
-          <t>Posterior</t>
-        </is>
-      </c>
-      <c r="I56" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
-        </is>
-      </c>
-      <c r="J56" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
+          <t>H3 · MVP (Grupos)</t>
+        </is>
+      </c>
+      <c r="I56" s="19" t="inlineStr">
+        <is>
+          <t>Como pastor quiero que ofrendas y asistencias sean confidenciales.</t>
+        </is>
+      </c>
+      <c r="J56" s="19" t="inlineStr">
+        <is>
+          <t>La matriz de la sección 3.3 del v3.2 se cumple en pruebas por cada rol.</t>
         </is>
       </c>
       <c r="K56" s="19" t="inlineStr">
         <is>
-          <t>VoBo pendiente</t>
+          <t>Por definir</t>
         </is>
       </c>
       <c r="L56" s="19" t="inlineStr">
@@ -5480,52 +5504,52 @@
     <row r="57">
       <c r="A57" s="18" t="inlineStr">
         <is>
-          <t>M4-02</t>
+          <t>M3-11</t>
         </is>
       </c>
       <c r="B57" s="19" t="inlineStr">
         <is>
-          <t>M4 Kids Check-In/Out</t>
+          <t>M3 Grupos de Conexión</t>
         </is>
       </c>
       <c r="C57" s="19" t="inlineStr">
         <is>
-          <t>Registro de ingreso del menor con salón o clase asignada y generación de código único.</t>
+          <t>Dashboard y tablero de mensajes del grupo.</t>
         </is>
       </c>
       <c r="D57" s="21" t="inlineStr">
         <is>
-          <t>v1 + Nuevo v3</t>
+          <t>Obs. 7</t>
         </is>
       </c>
       <c r="E57" s="19" t="inlineStr">
         <is>
-          <t>Fuera del MVP</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="F57" s="19" t="inlineStr">
         <is>
-          <t>Fase 2</t>
+          <t>Fase 1</t>
         </is>
       </c>
       <c r="G57" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sprint 5</t>
         </is>
       </c>
       <c r="H57" s="19" t="inlineStr">
         <is>
-          <t>Posterior</t>
-        </is>
-      </c>
-      <c r="I57" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
-        </is>
-      </c>
-      <c r="J57" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
+          <t>H3 · MVP (Grupos)</t>
+        </is>
+      </c>
+      <c r="I57" s="19" t="inlineStr">
+        <is>
+          <t>Como líder quiero un tablero de mensajes de mi grupo.</t>
+        </is>
+      </c>
+      <c r="J57" s="19" t="inlineStr">
+        <is>
+          <t>Publicar y leer mensajes del grupo.</t>
         </is>
       </c>
       <c r="K57" s="19" t="inlineStr">
@@ -5544,7 +5568,7 @@
     <row r="58">
       <c r="A58" s="18" t="inlineStr">
         <is>
-          <t>M4-03</t>
+          <t>M4-01</t>
         </is>
       </c>
       <c r="B58" s="19" t="inlineStr">
@@ -5554,12 +5578,12 @@
       </c>
       <c r="C58" s="19" t="inlineStr">
         <is>
-          <t>Código QR dinámico o OTP temporal en la PWA del padre o tutor.</t>
+          <t>Sustitución de la ficha física de papel.</t>
         </is>
       </c>
       <c r="D58" s="19" t="inlineStr">
         <is>
-          <t>v2</t>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E58" s="19" t="inlineStr">
@@ -5608,7 +5632,7 @@
     <row r="59">
       <c r="A59" s="18" t="inlineStr">
         <is>
-          <t>M4-04</t>
+          <t>M4-02</t>
         </is>
       </c>
       <c r="B59" s="19" t="inlineStr">
@@ -5618,12 +5642,12 @@
       </c>
       <c r="C59" s="19" t="inlineStr">
         <is>
-          <t>Validación al entregar: el servidor de Kids escanea el código y confirma identidad y fotografía del tutor autorizado en el Expediente Digital.</t>
-        </is>
-      </c>
-      <c r="D59" s="19" t="inlineStr">
-        <is>
-          <t>v2</t>
+          <t>Registro de ingreso del menor con salón o clase asignada y generación de código único.</t>
+        </is>
+      </c>
+      <c r="D59" s="21" t="inlineStr">
+        <is>
+          <t>v1 + Nuevo v3</t>
         </is>
       </c>
       <c r="E59" s="19" t="inlineStr">
@@ -5672,7 +5696,7 @@
     <row r="60">
       <c r="A60" s="18" t="inlineStr">
         <is>
-          <t>M4-05</t>
+          <t>M4-03</t>
         </is>
       </c>
       <c r="B60" s="19" t="inlineStr">
@@ -5682,12 +5706,12 @@
       </c>
       <c r="C60" s="19" t="inlineStr">
         <is>
-          <t>Alternativa para tutores sin smartphone, sin batería o sin conexión (p. ej. código por SMS o comprobante imprimible con identificación). Por definir.</t>
-        </is>
-      </c>
-      <c r="D60" s="21" t="inlineStr">
-        <is>
-          <t>Nuevo v3</t>
+          <t>Código QR dinámico o OTP temporal en la PWA del padre o tutor.</t>
+        </is>
+      </c>
+      <c r="D60" s="19" t="inlineStr">
+        <is>
+          <t>v2</t>
         </is>
       </c>
       <c r="E60" s="19" t="inlineStr">
@@ -5722,7 +5746,7 @@
       </c>
       <c r="K60" s="19" t="inlineStr">
         <is>
-          <t>Por definir</t>
+          <t>VoBo pendiente</t>
         </is>
       </c>
       <c r="L60" s="19" t="inlineStr">
@@ -5736,7 +5760,7 @@
     <row r="61">
       <c r="A61" s="18" t="inlineStr">
         <is>
-          <t>M4-06</t>
+          <t>M4-04</t>
         </is>
       </c>
       <c r="B61" s="19" t="inlineStr">
@@ -5746,12 +5770,12 @@
       </c>
       <c r="C61" s="19" t="inlineStr">
         <is>
-          <t>Autorización temporal de un tercero para recoger al menor, con aprobación del tutor registrado.</t>
-        </is>
-      </c>
-      <c r="D61" s="21" t="inlineStr">
-        <is>
-          <t>Nuevo v3</t>
+          <t>Validación al entregar: el servidor de Kids escanea el código y confirma identidad y fotografía del tutor autorizado en el Expediente Digital.</t>
+        </is>
+      </c>
+      <c r="D61" s="19" t="inlineStr">
+        <is>
+          <t>v2</t>
         </is>
       </c>
       <c r="E61" s="19" t="inlineStr">
@@ -5800,7 +5824,7 @@
     <row r="62">
       <c r="A62" s="18" t="inlineStr">
         <is>
-          <t>M4-07</t>
+          <t>M4-05</t>
         </is>
       </c>
       <c r="B62" s="19" t="inlineStr">
@@ -5810,7 +5834,7 @@
       </c>
       <c r="C62" s="19" t="inlineStr">
         <is>
-          <t>Caducidad del código y bitácora de cada entrega (quién recogió, quién entregó, hora).</t>
+          <t>Alternativa para tutores sin smartphone, sin batería o sin conexión (p. ej. código por SMS o comprobante imprimible con identificación). Por definir.</t>
         </is>
       </c>
       <c r="D62" s="21" t="inlineStr">
@@ -5850,7 +5874,7 @@
       </c>
       <c r="K62" s="19" t="inlineStr">
         <is>
-          <t>VoBo pendiente</t>
+          <t>Por definir</t>
         </is>
       </c>
       <c r="L62" s="19" t="inlineStr">
@@ -5864,7 +5888,7 @@
     <row r="63">
       <c r="A63" s="18" t="inlineStr">
         <is>
-          <t>M4-08</t>
+          <t>M4-06</t>
         </is>
       </c>
       <c r="B63" s="19" t="inlineStr">
@@ -5874,7 +5898,7 @@
       </c>
       <c r="C63" s="19" t="inlineStr">
         <is>
-          <t>Funcionamiento sin conexión o con conexión degradada para el check-out.</t>
+          <t>Autorización temporal de un tercero para recoger al menor, con aprobación del tutor registrado.</t>
         </is>
       </c>
       <c r="D63" s="21" t="inlineStr">
@@ -5928,52 +5952,52 @@
     <row r="64">
       <c r="A64" s="18" t="inlineStr">
         <is>
-          <t>M5-01</t>
+          <t>M4-07</t>
         </is>
       </c>
       <c r="B64" s="19" t="inlineStr">
         <is>
-          <t>M5 Áreas y servidores</t>
+          <t>M4 Kids Check-In/Out</t>
         </is>
       </c>
       <c r="C64" s="19" t="inlineStr">
         <is>
-          <t>Catálogo mínimo de áreas y asignación de servidores. Versión reducida del módulo 5, necesaria para permisos por área. Sirve como primer censo.</t>
-        </is>
-      </c>
-      <c r="D64" s="19" t="inlineStr">
-        <is>
-          <t>v3</t>
+          <t>Caducidad del código y bitácora de cada entrega (quién recogió, quién entregó, hora).</t>
+        </is>
+      </c>
+      <c r="D64" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3</t>
         </is>
       </c>
       <c r="E64" s="19" t="inlineStr">
         <is>
-          <t>MVP mínimo</t>
+          <t>Fuera del MVP</t>
         </is>
       </c>
       <c r="F64" s="19" t="inlineStr">
         <is>
-          <t>Fase 0</t>
+          <t>Fase 2</t>
         </is>
       </c>
       <c r="G64" s="19" t="inlineStr">
         <is>
-          <t>Sprint 1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H64" s="19" t="inlineStr">
         <is>
-          <t>H2 · Fase 0 completa</t>
-        </is>
-      </c>
-      <c r="I64" s="19" t="inlineStr">
-        <is>
-          <t>Como pastor quiero un catálogo de áreas con su personal para conocer la estructura.</t>
-        </is>
-      </c>
-      <c r="J64" s="19" t="inlineStr">
-        <is>
-          <t>Crear un área, asignar servidores y ver el conteo real.</t>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="I64" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
+        </is>
+      </c>
+      <c r="J64" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
         </is>
       </c>
       <c r="K64" s="19" t="inlineStr">
@@ -5992,22 +6016,22 @@
     <row r="65">
       <c r="A65" s="18" t="inlineStr">
         <is>
-          <t>M5-02</t>
+          <t>M4-08</t>
         </is>
       </c>
       <c r="B65" s="19" t="inlineStr">
         <is>
-          <t>M5 Áreas y servidores</t>
+          <t>M4 Kids Check-In/Out</t>
         </is>
       </c>
       <c r="C65" s="19" t="inlineStr">
         <is>
-          <t>Roles jerárquicos dentro de cada área (directores, líderes, maestros, servidores).</t>
-        </is>
-      </c>
-      <c r="D65" s="19" t="inlineStr">
-        <is>
-          <t>v1</t>
+          <t>Funcionamiento sin conexión o con conexión degradada para el check-out.</t>
+        </is>
+      </c>
+      <c r="D65" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3</t>
         </is>
       </c>
       <c r="E65" s="19" t="inlineStr">
@@ -6017,7 +6041,7 @@
       </c>
       <c r="F65" s="19" t="inlineStr">
         <is>
-          <t>Fase 4</t>
+          <t>Fase 2</t>
         </is>
       </c>
       <c r="G65" s="19" t="inlineStr">
@@ -6056,7 +6080,7 @@
     <row r="66">
       <c r="A66" s="18" t="inlineStr">
         <is>
-          <t>M5-03</t>
+          <t>M5-01</t>
         </is>
       </c>
       <c r="B66" s="19" t="inlineStr">
@@ -6066,42 +6090,42 @@
       </c>
       <c r="C66" s="19" t="inlineStr">
         <is>
-          <t>Organigrama y número real de servidores activos, directores y líderes por área.</t>
+          <t>Catálogo mínimo de áreas y asignación de servidores. Versión reducida del módulo 5, necesaria para permisos por área. Sirve como primer censo.</t>
         </is>
       </c>
       <c r="D66" s="19" t="inlineStr">
         <is>
-          <t>v2</t>
+          <t>v3</t>
         </is>
       </c>
       <c r="E66" s="19" t="inlineStr">
         <is>
-          <t>Fuera del MVP</t>
+          <t>MVP mínimo</t>
         </is>
       </c>
       <c r="F66" s="19" t="inlineStr">
         <is>
-          <t>Fase 4</t>
+          <t>Fase 0</t>
         </is>
       </c>
       <c r="G66" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sprint 1</t>
         </is>
       </c>
       <c r="H66" s="19" t="inlineStr">
         <is>
-          <t>Posterior</t>
-        </is>
-      </c>
-      <c r="I66" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
-        </is>
-      </c>
-      <c r="J66" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
+          <t>H2 · Fase 0 completa</t>
+        </is>
+      </c>
+      <c r="I66" s="19" t="inlineStr">
+        <is>
+          <t>Como pastor quiero un catálogo de áreas con su personal para conocer la estructura.</t>
+        </is>
+      </c>
+      <c r="J66" s="19" t="inlineStr">
+        <is>
+          <t>Crear un área, asignar servidores y ver el conteo real.</t>
         </is>
       </c>
       <c r="K66" s="19" t="inlineStr">
@@ -6120,7 +6144,7 @@
     <row r="67">
       <c r="A67" s="18" t="inlineStr">
         <is>
-          <t>M5-04</t>
+          <t>M5-02</t>
         </is>
       </c>
       <c r="B67" s="19" t="inlineStr">
@@ -6130,12 +6154,12 @@
       </c>
       <c r="C67" s="19" t="inlineStr">
         <is>
-          <t>Control de asistencia a turnos o servicios.</t>
+          <t>Roles jerárquicos dentro de cada área (directores, líderes, maestros, servidores).</t>
         </is>
       </c>
       <c r="D67" s="19" t="inlineStr">
         <is>
-          <t>v1 / v2</t>
+          <t>v1</t>
         </is>
       </c>
       <c r="E67" s="19" t="inlineStr">
@@ -6184,7 +6208,7 @@
     <row r="68">
       <c r="A68" s="18" t="inlineStr">
         <is>
-          <t>M5-05</t>
+          <t>M5-03</t>
         </is>
       </c>
       <c r="B68" s="19" t="inlineStr">
@@ -6194,12 +6218,12 @@
       </c>
       <c r="C68" s="19" t="inlineStr">
         <is>
-          <t>Tablero de avisos y notificaciones interno por área.</t>
+          <t>Organigrama y número real de servidores activos, directores y líderes por área.</t>
         </is>
       </c>
       <c r="D68" s="19" t="inlineStr">
         <is>
-          <t>v1 / v2</t>
+          <t>v2</t>
         </is>
       </c>
       <c r="E68" s="19" t="inlineStr">
@@ -6248,7 +6272,7 @@
     <row r="69">
       <c r="A69" s="18" t="inlineStr">
         <is>
-          <t>M5-06</t>
+          <t>M5-04</t>
         </is>
       </c>
       <c r="B69" s="19" t="inlineStr">
@@ -6258,7 +6282,7 @@
       </c>
       <c r="C69" s="19" t="inlineStr">
         <is>
-          <t>Gestión financiera por área: caja chica y gastos operativos.</t>
+          <t>Control de asistencia a turnos o servicios.</t>
         </is>
       </c>
       <c r="D69" s="19" t="inlineStr">
@@ -6312,22 +6336,22 @@
     <row r="70">
       <c r="A70" s="18" t="inlineStr">
         <is>
-          <t>M6-01</t>
+          <t>M5-05</t>
         </is>
       </c>
       <c r="B70" s="19" t="inlineStr">
         <is>
-          <t>M6 Ministerios de servicio</t>
+          <t>M5 Áreas y servidores</t>
         </is>
       </c>
       <c r="C70" s="19" t="inlineStr">
         <is>
-          <t>Control de personal propio de cada ministerio.</t>
-        </is>
-      </c>
-      <c r="D70" s="22" t="inlineStr">
-        <is>
-          <t>Recuperado v1</t>
+          <t>Tablero de avisos y notificaciones interno por área.</t>
+        </is>
+      </c>
+      <c r="D70" s="19" t="inlineStr">
+        <is>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E70" s="19" t="inlineStr">
@@ -6376,17 +6400,17 @@
     <row r="71">
       <c r="A71" s="18" t="inlineStr">
         <is>
-          <t>M6-02</t>
+          <t>M5-06</t>
         </is>
       </c>
       <c r="B71" s="19" t="inlineStr">
         <is>
-          <t>M6 Ministerios de servicio</t>
+          <t>M5 Áreas y servidores</t>
         </is>
       </c>
       <c r="C71" s="19" t="inlineStr">
         <is>
-          <t>Menú o catálogo digital interactivo (público o interno), autogestionado.</t>
+          <t>Gestión financiera por área: caja chica y gastos operativos.</t>
         </is>
       </c>
       <c r="D71" s="19" t="inlineStr">
@@ -6440,7 +6464,7 @@
     <row r="72">
       <c r="A72" s="18" t="inlineStr">
         <is>
-          <t>M6-03</t>
+          <t>M6-01</t>
         </is>
       </c>
       <c r="B72" s="19" t="inlineStr">
@@ -6450,12 +6474,12 @@
       </c>
       <c r="C72" s="19" t="inlineStr">
         <is>
-          <t>Calendario de turnos: días regulares de servicio y eventos especiales.</t>
-        </is>
-      </c>
-      <c r="D72" s="19" t="inlineStr">
-        <is>
-          <t>v1 / v2</t>
+          <t>Control de personal propio de cada ministerio.</t>
+        </is>
+      </c>
+      <c r="D72" s="22" t="inlineStr">
+        <is>
+          <t>Recuperado v1</t>
         </is>
       </c>
       <c r="E72" s="19" t="inlineStr">
@@ -6504,7 +6528,7 @@
     <row r="73">
       <c r="A73" s="18" t="inlineStr">
         <is>
-          <t>M6-04</t>
+          <t>M6-02</t>
         </is>
       </c>
       <c r="B73" s="19" t="inlineStr">
@@ -6514,7 +6538,7 @@
       </c>
       <c r="C73" s="19" t="inlineStr">
         <is>
-          <t>Registro de asistentes o personas atendidas.</t>
+          <t>Menú o catálogo digital interactivo (público o interno), autogestionado.</t>
         </is>
       </c>
       <c r="D73" s="19" t="inlineStr">
@@ -6568,7 +6592,7 @@
     <row r="74">
       <c r="A74" s="18" t="inlineStr">
         <is>
-          <t>M6-05</t>
+          <t>M6-03</t>
         </is>
       </c>
       <c r="B74" s="19" t="inlineStr">
@@ -6578,7 +6602,7 @@
       </c>
       <c r="C74" s="19" t="inlineStr">
         <is>
-          <t>Control de gastos y de inventario básico.</t>
+          <t>Calendario de turnos: días regulares de servicio y eventos especiales.</t>
         </is>
       </c>
       <c r="D74" s="19" t="inlineStr">
@@ -6632,7 +6656,7 @@
     <row r="75">
       <c r="A75" s="18" t="inlineStr">
         <is>
-          <t>M6-06</t>
+          <t>M6-04</t>
         </is>
       </c>
       <c r="B75" s="19" t="inlineStr">
@@ -6642,7 +6666,7 @@
       </c>
       <c r="C75" s="19" t="inlineStr">
         <is>
-          <t>Canal de comunicación directo con el área de Administración General.</t>
+          <t>Registro de asistentes o personas atendidas.</t>
         </is>
       </c>
       <c r="D75" s="19" t="inlineStr">
@@ -6696,7 +6720,7 @@
     <row r="76">
       <c r="A76" s="18" t="inlineStr">
         <is>
-          <t>M6-07</t>
+          <t>M6-05</t>
         </is>
       </c>
       <c r="B76" s="19" t="inlineStr">
@@ -6706,12 +6730,12 @@
       </c>
       <c r="C76" s="19" t="inlineStr">
         <is>
-          <t>Servicio Médico: los datos de salud de las personas atendidas requieren tratamiento de datos sensibles. Por definir alcance.</t>
-        </is>
-      </c>
-      <c r="D76" s="21" t="inlineStr">
-        <is>
-          <t>Nuevo v3</t>
+          <t>Control de gastos y de inventario básico.</t>
+        </is>
+      </c>
+      <c r="D76" s="19" t="inlineStr">
+        <is>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E76" s="19" t="inlineStr">
@@ -6746,7 +6770,7 @@
       </c>
       <c r="K76" s="19" t="inlineStr">
         <is>
-          <t>Por definir</t>
+          <t>VoBo pendiente</t>
         </is>
       </c>
       <c r="L76" s="19" t="inlineStr">
@@ -6760,17 +6784,17 @@
     <row r="77">
       <c r="A77" s="18" t="inlineStr">
         <is>
-          <t>M7-01</t>
+          <t>M6-06</t>
         </is>
       </c>
       <c r="B77" s="19" t="inlineStr">
         <is>
-          <t>M7 Eventos y aforo</t>
+          <t>M6 Ministerios de servicio</t>
         </is>
       </c>
       <c r="C77" s="19" t="inlineStr">
         <is>
-          <t>Eventos abiertos o evangelísticos con formulario de inscripción rápida, sin requerir historial previo.</t>
+          <t>Canal de comunicación directo con el área de Administración General.</t>
         </is>
       </c>
       <c r="D77" s="19" t="inlineStr">
@@ -6824,22 +6848,22 @@
     <row r="78">
       <c r="A78" s="18" t="inlineStr">
         <is>
-          <t>M7-02</t>
+          <t>M6-07</t>
         </is>
       </c>
       <c r="B78" s="19" t="inlineStr">
         <is>
-          <t>M7 Eventos y aforo</t>
+          <t>M6 Ministerios de servicio</t>
         </is>
       </c>
       <c r="C78" s="19" t="inlineStr">
         <is>
-          <t>Consolidación (inducción de personas que asisten por primera vez) como tipo de evento.</t>
-        </is>
-      </c>
-      <c r="D78" s="22" t="inlineStr">
-        <is>
-          <t>Recuperado v1</t>
+          <t>Servicio Médico: los datos de salud de las personas atendidas requieren tratamiento de datos sensibles. Por definir alcance.</t>
+        </is>
+      </c>
+      <c r="D78" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3</t>
         </is>
       </c>
       <c r="E78" s="19" t="inlineStr">
@@ -6874,7 +6898,7 @@
       </c>
       <c r="K78" s="19" t="inlineStr">
         <is>
-          <t>VoBo pendiente</t>
+          <t>Por definir</t>
         </is>
       </c>
       <c r="L78" s="19" t="inlineStr">
@@ -6888,7 +6912,7 @@
     <row r="79">
       <c r="A79" s="18" t="inlineStr">
         <is>
-          <t>M7-03</t>
+          <t>M7-01</t>
         </is>
       </c>
       <c r="B79" s="19" t="inlineStr">
@@ -6898,12 +6922,12 @@
       </c>
       <c r="C79" s="19" t="inlineStr">
         <is>
-          <t>Encargados de evento (personal de la iglesia únicamente; no se controla personal externo).</t>
-        </is>
-      </c>
-      <c r="D79" s="22" t="inlineStr">
-        <is>
-          <t>Recuperado v1</t>
+          <t>Eventos abiertos o evangelísticos con formulario de inscripción rápida, sin requerir historial previo.</t>
+        </is>
+      </c>
+      <c r="D79" s="19" t="inlineStr">
+        <is>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E79" s="19" t="inlineStr">
@@ -6952,7 +6976,7 @@
     <row r="80">
       <c r="A80" s="18" t="inlineStr">
         <is>
-          <t>M7-04</t>
+          <t>M7-02</t>
         </is>
       </c>
       <c r="B80" s="19" t="inlineStr">
@@ -6962,12 +6986,12 @@
       </c>
       <c r="C80" s="19" t="inlineStr">
         <is>
-          <t>Control de cupo en tiempo real que bloquea el sobrecupo en eventos con aforo limitado (ej. 30 o 50 lugares).</t>
-        </is>
-      </c>
-      <c r="D80" s="19" t="inlineStr">
-        <is>
-          <t>v1 / v2</t>
+          <t>Consolidación (inducción de personas que asisten por primera vez) como tipo de evento.</t>
+        </is>
+      </c>
+      <c r="D80" s="22" t="inlineStr">
+        <is>
+          <t>Recuperado v1</t>
         </is>
       </c>
       <c r="E80" s="19" t="inlineStr">
@@ -7016,7 +7040,7 @@
     <row r="81">
       <c r="A81" s="18" t="inlineStr">
         <is>
-          <t>M7-05</t>
+          <t>M7-03</t>
         </is>
       </c>
       <c r="B81" s="19" t="inlineStr">
@@ -7026,12 +7050,12 @@
       </c>
       <c r="C81" s="19" t="inlineStr">
         <is>
-          <t>Control de asistentes sin lista previa, para aforo y para dar a conocer la iglesia.</t>
-        </is>
-      </c>
-      <c r="D81" s="19" t="inlineStr">
-        <is>
-          <t>v1</t>
+          <t>Encargados de evento (personal de la iglesia únicamente; no se controla personal externo).</t>
+        </is>
+      </c>
+      <c r="D81" s="22" t="inlineStr">
+        <is>
+          <t>Recuperado v1</t>
         </is>
       </c>
       <c r="E81" s="19" t="inlineStr">
@@ -7080,7 +7104,7 @@
     <row r="82">
       <c r="A82" s="18" t="inlineStr">
         <is>
-          <t>M7-06</t>
+          <t>M7-04</t>
         </is>
       </c>
       <c r="B82" s="19" t="inlineStr">
@@ -7090,12 +7114,12 @@
       </c>
       <c r="C82" s="19" t="inlineStr">
         <is>
-          <t>Seguimiento de personas nuevas: conversión de un invitado a Expediente Digital y canalización a un curso o Grupo de Conexión.</t>
-        </is>
-      </c>
-      <c r="D82" s="21" t="inlineStr">
-        <is>
-          <t>Nuevo v3</t>
+          <t>Control de cupo en tiempo real que bloquea el sobrecupo en eventos con aforo limitado (ej. 30 o 50 lugares).</t>
+        </is>
+      </c>
+      <c r="D82" s="19" t="inlineStr">
+        <is>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E82" s="19" t="inlineStr">
@@ -7144,52 +7168,52 @@
     <row r="83">
       <c r="A83" s="18" t="inlineStr">
         <is>
-          <t>NF-01</t>
+          <t>M7-05</t>
         </is>
       </c>
       <c r="B83" s="19" t="inlineStr">
         <is>
-          <t>No funcionales</t>
+          <t>M7 Eventos y aforo</t>
         </is>
       </c>
       <c r="C83" s="19" t="inlineStr">
         <is>
-          <t>Cumplimiento de la LFPDPPP: aviso de privacidad, consentimiento y derechos ARCO.</t>
+          <t>Control de asistentes sin lista previa, para aforo y para dar a conocer la iglesia.</t>
         </is>
       </c>
       <c r="D83" s="19" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>v1</t>
         </is>
       </c>
       <c r="E83" s="19" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Fuera del MVP</t>
         </is>
       </c>
       <c r="F83" s="19" t="inlineStr">
         <is>
-          <t>Fase 0</t>
+          <t>Fase 4</t>
         </is>
       </c>
       <c r="G83" s="19" t="inlineStr">
         <is>
-          <t>Sprint 1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H83" s="19" t="inlineStr">
         <is>
-          <t>H1 · 18-oct (núcleo Fase 0)</t>
-        </is>
-      </c>
-      <c r="I83" s="19" t="inlineStr">
-        <is>
-          <t>Como iglesia queremos cumplir con la LFPDPPP.</t>
-        </is>
-      </c>
-      <c r="J83" s="19" t="inlineStr">
-        <is>
-          <t>Aviso de privacidad, consentimiento y atención de derechos ARCO disponibles.</t>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="I83" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
+        </is>
+      </c>
+      <c r="J83" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
         </is>
       </c>
       <c r="K83" s="19" t="inlineStr">
@@ -7208,52 +7232,52 @@
     <row r="84">
       <c r="A84" s="18" t="inlineStr">
         <is>
-          <t>NF-02</t>
+          <t>M7-06</t>
         </is>
       </c>
       <c r="B84" s="19" t="inlineStr">
         <is>
-          <t>No funcionales</t>
+          <t>M7 Eventos y aforo</t>
         </is>
       </c>
       <c r="C84" s="19" t="inlineStr">
         <is>
-          <t>Cifrado en tránsito y en reposo. Cifrado adicional a nivel de campo para peticiones de oración.</t>
-        </is>
-      </c>
-      <c r="D84" s="19" t="inlineStr">
-        <is>
-          <t>v3</t>
+          <t>Seguimiento de personas nuevas: conversión de un invitado a Expediente Digital y canalización a un curso o Grupo de Conexión.</t>
+        </is>
+      </c>
+      <c r="D84" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3</t>
         </is>
       </c>
       <c r="E84" s="19" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Fuera del MVP</t>
         </is>
       </c>
       <c r="F84" s="19" t="inlineStr">
         <is>
-          <t>Fase 0</t>
+          <t>Fase 4</t>
         </is>
       </c>
       <c r="G84" s="19" t="inlineStr">
         <is>
-          <t>Sprint 0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H84" s="19" t="inlineStr">
         <is>
-          <t>H1 · 18-oct (núcleo Fase 0)</t>
-        </is>
-      </c>
-      <c r="I84" s="19" t="inlineStr">
-        <is>
-          <t>Como iglesia queremos proteger los datos sensibles.</t>
-        </is>
-      </c>
-      <c r="J84" s="19" t="inlineStr">
-        <is>
-          <t>HTTPS obligatorio y peticiones de oración ilegibles directamente en la base.</t>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="I84" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
+        </is>
+      </c>
+      <c r="J84" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
         </is>
       </c>
       <c r="K84" s="19" t="inlineStr">
@@ -7272,7 +7296,7 @@
     <row r="85">
       <c r="A85" s="18" t="inlineStr">
         <is>
-          <t>NF-03</t>
+          <t>NF-01</t>
         </is>
       </c>
       <c r="B85" s="19" t="inlineStr">
@@ -7282,7 +7306,7 @@
       </c>
       <c r="C85" s="19" t="inlineStr">
         <is>
-          <t>Bitácora de auditoría de solo-añadir: quién consultó o modificó expedientes, ofrendas y asistencias.</t>
+          <t>Cumplimiento de la LFPDPPP: aviso de privacidad, consentimiento y derechos ARCO.</t>
         </is>
       </c>
       <c r="D85" s="19" t="inlineStr">
@@ -7312,12 +7336,12 @@
       </c>
       <c r="I85" s="19" t="inlineStr">
         <is>
-          <t>Como pastor quiero una bitácora que nadie pueda alterar.</t>
+          <t>Como iglesia queremos cumplir con la LFPDPPP.</t>
         </is>
       </c>
       <c r="J85" s="19" t="inlineStr">
         <is>
-          <t>El usuario de la aplicación no puede actualizar ni borrar registros de bitácora.</t>
+          <t>Aviso de privacidad, consentimiento y atención de derechos ARCO disponibles.</t>
         </is>
       </c>
       <c r="K85" s="19" t="inlineStr">
@@ -7336,7 +7360,7 @@
     <row r="86">
       <c r="A86" s="18" t="inlineStr">
         <is>
-          <t>NF-04</t>
+          <t>NF-02</t>
         </is>
       </c>
       <c r="B86" s="19" t="inlineStr">
@@ -7346,7 +7370,7 @@
       </c>
       <c r="C86" s="19" t="inlineStr">
         <is>
-          <t>Respaldos automáticos diarios cifrados y prueba periódica de restauración.</t>
+          <t>Cifrado en tránsito y en reposo. Cifrado adicional a nivel de campo para peticiones de oración.</t>
         </is>
       </c>
       <c r="D86" s="19" t="inlineStr">
@@ -7376,12 +7400,12 @@
       </c>
       <c r="I86" s="19" t="inlineStr">
         <is>
-          <t>Como iglesia queremos no perder información.</t>
+          <t>Como iglesia queremos proteger los datos sensibles.</t>
         </is>
       </c>
       <c r="J86" s="19" t="inlineStr">
         <is>
-          <t>Respaldo diario cifrado y restauración probada en un ambiente de pruebas.</t>
+          <t>HTTPS obligatorio y peticiones de oración ilegibles directamente en la base.</t>
         </is>
       </c>
       <c r="K86" s="19" t="inlineStr">
@@ -7400,7 +7424,7 @@
     <row r="87">
       <c r="A87" s="18" t="inlineStr">
         <is>
-          <t>NF-05</t>
+          <t>NF-03</t>
         </is>
       </c>
       <c r="B87" s="19" t="inlineStr">
@@ -7410,61 +7434,69 @@
       </c>
       <c r="C87" s="19" t="inlineStr">
         <is>
-          <t>Disponibilidad esperada en horarios de servicio (fines de semana y reuniones de grupo). Por definir meta.</t>
-        </is>
-      </c>
-      <c r="D87" s="21" t="inlineStr">
-        <is>
-          <t>Nuevo v3</t>
+          <t>Bitácora de auditoría de solo-añadir: quién consultó o modificó expedientes, ofrendas y asistencias.</t>
+        </is>
+      </c>
+      <c r="D87" s="19" t="inlineStr">
+        <is>
+          <t>v3</t>
         </is>
       </c>
       <c r="E87" s="19" t="inlineStr">
         <is>
-          <t>Fuera del MVP</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="F87" s="19" t="inlineStr">
         <is>
-          <t>Transversal</t>
+          <t>Fase 0</t>
         </is>
       </c>
       <c r="G87" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sprint 1</t>
         </is>
       </c>
       <c r="H87" s="19" t="inlineStr">
         <is>
-          <t>Posterior</t>
-        </is>
-      </c>
-      <c r="I87" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
-        </is>
-      </c>
-      <c r="J87" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
+          <t>H1 · 18-oct (núcleo Fase 0)</t>
+        </is>
+      </c>
+      <c r="I87" s="19" t="inlineStr">
+        <is>
+          <t>Como pastor quiero una bitácora que nadie pueda alterar.</t>
+        </is>
+      </c>
+      <c r="J87" s="19" t="inlineStr">
+        <is>
+          <t>El usuario de la aplicación no puede actualizar ni borrar registros de bitácora.</t>
         </is>
       </c>
       <c r="K87" s="19" t="inlineStr">
         <is>
-          <t>Por definir</t>
+          <t>VoBo pendiente</t>
         </is>
       </c>
       <c r="L87" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M87" s="19" t="inlineStr"/>
-      <c r="N87" s="19" t="inlineStr"/>
+          <t>En desarrollo</t>
+        </is>
+      </c>
+      <c r="M87" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/m1-17-acceso · bitácora de solo-añadir a nivel de aplicación</t>
+        </is>
+      </c>
+      <c r="N87" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-05 · Falta reforzarla en la base de datos (permisos) en el Sprint 1.</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="18" t="inlineStr">
         <is>
-          <t>NF-06</t>
+          <t>NF-04</t>
         </is>
       </c>
       <c r="B88" s="19" t="inlineStr">
@@ -7474,7 +7506,7 @@
       </c>
       <c r="C88" s="19" t="inlineStr">
         <is>
-          <t>Pase de lista sin conexión con sincronización posterior (reuniones en domicilios con mala señal).</t>
+          <t>Respaldos automáticos diarios cifrados y prueba periódica de restauración.</t>
         </is>
       </c>
       <c r="D88" s="19" t="inlineStr">
@@ -7494,22 +7526,22 @@
       </c>
       <c r="G88" s="19" t="inlineStr">
         <is>
-          <t>Sprint 3</t>
+          <t>Sprint 0</t>
         </is>
       </c>
       <c r="H88" s="19" t="inlineStr">
         <is>
-          <t>H3 · MVP (Grupos)</t>
+          <t>H1 · 18-oct (núcleo Fase 0)</t>
         </is>
       </c>
       <c r="I88" s="19" t="inlineStr">
         <is>
-          <t>Como secretario quiero que el pase de lista funcione sin señal.</t>
+          <t>Como iglesia queremos no perder información.</t>
         </is>
       </c>
       <c r="J88" s="19" t="inlineStr">
         <is>
-          <t>Prueba en modo avión y sincronización al reconectar.</t>
+          <t>Respaldo diario cifrado y restauración probada en un ambiente de pruebas.</t>
         </is>
       </c>
       <c r="K88" s="19" t="inlineStr">
@@ -7528,7 +7560,7 @@
     <row r="89">
       <c r="A89" s="18" t="inlineStr">
         <is>
-          <t>NF-07</t>
+          <t>NF-05</t>
         </is>
       </c>
       <c r="B89" s="19" t="inlineStr">
@@ -7538,47 +7570,47 @@
       </c>
       <c r="C89" s="19" t="inlineStr">
         <is>
-          <t>Funciona en Android, iOS y escritorio. En iOS, las notificaciones push requieren instalar la PWA; el respaldo por WhatsApp cubre el resto.</t>
-        </is>
-      </c>
-      <c r="D89" s="19" t="inlineStr">
-        <is>
-          <t>v3</t>
+          <t>Disponibilidad esperada en horarios de servicio (fines de semana y reuniones de grupo). Por definir meta.</t>
+        </is>
+      </c>
+      <c r="D89" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3</t>
         </is>
       </c>
       <c r="E89" s="19" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Fuera del MVP</t>
         </is>
       </c>
       <c r="F89" s="19" t="inlineStr">
         <is>
-          <t>Fase 0</t>
+          <t>Transversal</t>
         </is>
       </c>
       <c r="G89" s="19" t="inlineStr">
         <is>
-          <t>Sprint 0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H89" s="19" t="inlineStr">
         <is>
-          <t>H1 · 18-oct (núcleo Fase 0)</t>
-        </is>
-      </c>
-      <c r="I89" s="19" t="inlineStr">
-        <is>
-          <t>Como usuario quiero usar el sistema en mi dispositivo.</t>
-        </is>
-      </c>
-      <c r="J89" s="19" t="inlineStr">
-        <is>
-          <t>Pruebas en Android, iOS y escritorio; push en iOS con la PWA instalada y respaldo por WhatsApp.</t>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="I89" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
+        </is>
+      </c>
+      <c r="J89" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
         </is>
       </c>
       <c r="K89" s="19" t="inlineStr">
         <is>
-          <t>VoBo pendiente</t>
+          <t>Por definir</t>
         </is>
       </c>
       <c r="L89" s="19" t="inlineStr">
@@ -7592,7 +7624,7 @@
     <row r="90">
       <c r="A90" s="18" t="inlineStr">
         <is>
-          <t>NF-08</t>
+          <t>NF-06</t>
         </is>
       </c>
       <c r="B90" s="19" t="inlineStr">
@@ -7602,12 +7634,12 @@
       </c>
       <c r="C90" s="19" t="inlineStr">
         <is>
-          <t>Dimensionamiento para ~1,000 personas, con picos los fines de semana, y margen de crecimiento.</t>
-        </is>
-      </c>
-      <c r="D90" s="21" t="inlineStr">
-        <is>
-          <t>Resp. P8</t>
+          <t>Pase de lista sin conexión con sincronización posterior (reuniones en domicilios con mala señal).</t>
+        </is>
+      </c>
+      <c r="D90" s="19" t="inlineStr">
+        <is>
+          <t>v3</t>
         </is>
       </c>
       <c r="E90" s="19" t="inlineStr">
@@ -7622,22 +7654,22 @@
       </c>
       <c r="G90" s="19" t="inlineStr">
         <is>
-          <t>Sprint 0</t>
+          <t>Sprint 3</t>
         </is>
       </c>
       <c r="H90" s="19" t="inlineStr">
         <is>
-          <t>H1 · 18-oct (núcleo Fase 0)</t>
+          <t>H3 · MVP (Grupos)</t>
         </is>
       </c>
       <c r="I90" s="19" t="inlineStr">
         <is>
-          <t>Como iglesia queremos que el sistema soporte a ~1,000 personas.</t>
+          <t>Como secretario quiero que el pase de lista funcione sin señal.</t>
         </is>
       </c>
       <c r="J90" s="19" t="inlineStr">
         <is>
-          <t>Prueba de carga con volumen representativo (por definir) sin degradación.</t>
+          <t>Prueba en modo avión y sincronización al reconectar.</t>
         </is>
       </c>
       <c r="K90" s="19" t="inlineStr">
@@ -7656,7 +7688,7 @@
     <row r="91">
       <c r="A91" s="18" t="inlineStr">
         <is>
-          <t>NF-09</t>
+          <t>NF-07</t>
         </is>
       </c>
       <c r="B91" s="19" t="inlineStr">
@@ -7666,42 +7698,42 @@
       </c>
       <c r="C91" s="19" t="inlineStr">
         <is>
-          <t>Reportes transversales: asistencia, finanzas, crecimiento de la iglesia, exportables a Excel y PDF.</t>
-        </is>
-      </c>
-      <c r="D91" s="21" t="inlineStr">
-        <is>
-          <t>Nuevo v3</t>
+          <t>Funciona en Android, iOS y escritorio. En iOS, las notificaciones push requieren instalar la PWA; el respaldo por WhatsApp cubre el resto.</t>
+        </is>
+      </c>
+      <c r="D91" s="19" t="inlineStr">
+        <is>
+          <t>v3</t>
         </is>
       </c>
       <c r="E91" s="19" t="inlineStr">
         <is>
-          <t>Fuera del MVP</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="F91" s="19" t="inlineStr">
         <is>
-          <t>Transversal</t>
+          <t>Fase 0</t>
         </is>
       </c>
       <c r="G91" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sprint 0</t>
         </is>
       </c>
       <c r="H91" s="19" t="inlineStr">
         <is>
-          <t>Posterior</t>
-        </is>
-      </c>
-      <c r="I91" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
-        </is>
-      </c>
-      <c r="J91" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
+          <t>H1 · 18-oct (núcleo Fase 0)</t>
+        </is>
+      </c>
+      <c r="I91" s="19" t="inlineStr">
+        <is>
+          <t>Como usuario quiero usar el sistema en mi dispositivo.</t>
+        </is>
+      </c>
+      <c r="J91" s="19" t="inlineStr">
+        <is>
+          <t>Pruebas en Android, iOS y escritorio; push en iOS con la PWA instalada y respaldo por WhatsApp.</t>
         </is>
       </c>
       <c r="K91" s="19" t="inlineStr">
@@ -7720,7 +7752,7 @@
     <row r="92">
       <c r="A92" s="18" t="inlineStr">
         <is>
-          <t>NF-10</t>
+          <t>NF-08</t>
         </is>
       </c>
       <c r="B92" s="19" t="inlineStr">
@@ -7730,12 +7762,12 @@
       </c>
       <c r="C92" s="19" t="inlineStr">
         <is>
-          <t>Usabilidad para personas mayores: tipografía grande, alto contraste, flujos cortos (ver sección 5).</t>
-        </is>
-      </c>
-      <c r="D92" s="19" t="inlineStr">
-        <is>
-          <t>v3 + Obs. 1</t>
+          <t>Dimensionamiento para ~1,000 personas, con picos los fines de semana, y margen de crecimiento.</t>
+        </is>
+      </c>
+      <c r="D92" s="21" t="inlineStr">
+        <is>
+          <t>Resp. P8</t>
         </is>
       </c>
       <c r="E92" s="19" t="inlineStr">
@@ -7760,12 +7792,12 @@
       </c>
       <c r="I92" s="19" t="inlineStr">
         <is>
-          <t>Como persona mayor quiero una interfaz fácil de leer y usar.</t>
+          <t>Como iglesia queremos que el sistema soporte a ~1,000 personas.</t>
         </is>
       </c>
       <c r="J92" s="19" t="inlineStr">
         <is>
-          <t>Texto base 18 px, botones de al menos 48 px, contraste AA; prueba con usuarios mayores.</t>
+          <t>Prueba de carga con volumen representativo (por definir) sin degradación.</t>
         </is>
       </c>
       <c r="K92" s="19" t="inlineStr">
@@ -7781,9 +7813,137 @@
       <c r="M92" s="19" t="inlineStr"/>
       <c r="N92" s="19" t="inlineStr"/>
     </row>
+    <row r="93">
+      <c r="A93" s="18" t="inlineStr">
+        <is>
+          <t>NF-09</t>
+        </is>
+      </c>
+      <c r="B93" s="19" t="inlineStr">
+        <is>
+          <t>No funcionales</t>
+        </is>
+      </c>
+      <c r="C93" s="19" t="inlineStr">
+        <is>
+          <t>Reportes transversales: asistencia, finanzas, crecimiento de la iglesia, exportables a Excel y PDF.</t>
+        </is>
+      </c>
+      <c r="D93" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3</t>
+        </is>
+      </c>
+      <c r="E93" s="19" t="inlineStr">
+        <is>
+          <t>Fuera del MVP</t>
+        </is>
+      </c>
+      <c r="F93" s="19" t="inlineStr">
+        <is>
+          <t>Transversal</t>
+        </is>
+      </c>
+      <c r="G93" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H93" s="19" t="inlineStr">
+        <is>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="I93" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
+        </is>
+      </c>
+      <c r="J93" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
+        </is>
+      </c>
+      <c r="K93" s="19" t="inlineStr">
+        <is>
+          <t>VoBo pendiente</t>
+        </is>
+      </c>
+      <c r="L93" s="19" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M93" s="19" t="inlineStr"/>
+      <c r="N93" s="19" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="18" t="inlineStr">
+        <is>
+          <t>NF-10</t>
+        </is>
+      </c>
+      <c r="B94" s="19" t="inlineStr">
+        <is>
+          <t>No funcionales</t>
+        </is>
+      </c>
+      <c r="C94" s="19" t="inlineStr">
+        <is>
+          <t>Usabilidad para personas mayores: tipografía grande, alto contraste, flujos cortos (ver sección 5).</t>
+        </is>
+      </c>
+      <c r="D94" s="19" t="inlineStr">
+        <is>
+          <t>v3 + Obs. 1</t>
+        </is>
+      </c>
+      <c r="E94" s="19" t="inlineStr">
+        <is>
+          <t>MVP</t>
+        </is>
+      </c>
+      <c r="F94" s="19" t="inlineStr">
+        <is>
+          <t>Fase 0</t>
+        </is>
+      </c>
+      <c r="G94" s="19" t="inlineStr">
+        <is>
+          <t>Sprint 0</t>
+        </is>
+      </c>
+      <c r="H94" s="19" t="inlineStr">
+        <is>
+          <t>H1 · 18-oct (núcleo Fase 0)</t>
+        </is>
+      </c>
+      <c r="I94" s="19" t="inlineStr">
+        <is>
+          <t>Como persona mayor quiero una interfaz fácil de leer y usar.</t>
+        </is>
+      </c>
+      <c r="J94" s="19" t="inlineStr">
+        <is>
+          <t>Texto base 18 px, botones de al menos 48 px, contraste AA; prueba con usuarios mayores.</t>
+        </is>
+      </c>
+      <c r="K94" s="19" t="inlineStr">
+        <is>
+          <t>VoBo pendiente</t>
+        </is>
+      </c>
+      <c r="L94" s="19" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M94" s="19" t="inlineStr"/>
+      <c r="N94" s="19" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N92"/>
-  <conditionalFormatting sqref="L2:L92">
+  <autoFilter ref="A1:N94"/>
+  <conditionalFormatting sqref="L2:L94">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$L2="Hecho"</formula>
     </cfRule>
@@ -7800,7 +7960,7 @@
       <formula>$L2="Bloqueado"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K2:K92">
+  <conditionalFormatting sqref="K2:K94">
     <cfRule type="expression" priority="6" dxfId="0">
       <formula>$K2="Aprobado"</formula>
     </cfRule>
@@ -7808,16 +7968,16 @@
       <formula>$K2="Por definir"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H2:H92">
+  <conditionalFormatting sqref="H2:H94">
     <cfRule type="expression" priority="8" dxfId="5">
       <formula>LEFT($H2,2)="H1"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="L2:L92" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="L2:L94" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Pendiente,En diseño,En desarrollo,En pruebas,Hecho,Bloqueado"</formula1>
     </dataValidation>
-    <dataValidation sqref="K2:K92" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="K2:K94" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"VoBo pendiente,Aprobado,Por definir,Rechazado"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Corrige createsuperuser: la credencial se guarda con hash
El comando de Django envía `password`; el manager solo aceptaba `pin`, por lo que
la contraseña habría quedado en texto plano. Ahora acepta ambos y se agrega prueba.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/trazabilidad/Matriz de Trazabilidad MDF.xlsx
+++ b/docs/trazabilidad/Matriz de Trazabilidad MDF.xlsx
@@ -3492,7 +3492,7 @@
       </c>
       <c r="M25" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/m1-17-acceso · 32 pruebas de backend y 4 de frontend pasan</t>
+          <t>Rama feature/m1-17-acceso · 33 pruebas de backend y 4 de frontend pasan</t>
         </is>
       </c>
       <c r="N25" s="19" t="inlineStr">
@@ -3692,7 +3692,7 @@
       </c>
       <c r="M28" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/m1-17-acceso · 32 pruebas de backend y 4 de frontend pasan</t>
+          <t>Rama feature/m1-17-acceso · 33 pruebas de backend y 4 de frontend pasan</t>
         </is>
       </c>
       <c r="N28" s="19" t="inlineStr">
@@ -3764,7 +3764,7 @@
       </c>
       <c r="M29" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/m1-17-acceso · 32 pruebas de backend y 4 de frontend pasan</t>
+          <t>Rama feature/m1-17-acceso · 33 pruebas de backend y 4 de frontend pasan</t>
         </is>
       </c>
       <c r="N29" s="19" t="inlineStr">

</xml_diff>

<commit_message>
Matriz: M1-17 marcado como hecho tras prueba manual
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/trazabilidad/Matriz de Trazabilidad MDF.xlsx
+++ b/docs/trazabilidad/Matriz de Trazabilidad MDF.xlsx
@@ -3487,17 +3487,17 @@
       </c>
       <c r="L25" s="19" t="inlineStr">
         <is>
-          <t>En pruebas</t>
+          <t>Hecho</t>
         </is>
       </c>
       <c r="M25" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/m1-17-acceso · 33 pruebas de backend y 4 de frontend pasan</t>
+          <t>Rama feature/m1-17-acceso · 33 pruebas de backend y 4 de frontend pasan · Flujo invitar, activar y entrar probado por Edgar en navegador de escritorio</t>
         </is>
       </c>
       <c r="N25" s="19" t="inlineStr">
         <is>
-          <t>2026-10-05 · Falta probar en dispositivos reales (Android/iOS) y con un Líder.</t>
+          <t>2026-10-05 · Pendiente repetir la prueba en Android/iOS (se cubre con NF-07).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
M1-01: expediente digital con los campos de la Radiografía de miembros GC
- Persona con tres niveles de registro, procedencia, datos de la Radiografía y campos extra
- Catálogo de 14 procesos discipulares y avance por persona (fecha y maestro)
- Consentimiento versionado (aviso genérico) al dar de alta y al activar la cuenta
- Historial de movimientos con fecha y motivo; altas, bajas y reactivación
- Alta rápida de contacto con detección de duplicados por WhatsApp; búsqueda sin acentos
- Foto en carpeta local con ruta en la base de datos, reducida y servida solo con sesión
- Consultas y cambios en bitácora; pantallas de lista, alta y ficha
- Componentes nuevos del sistema de diseño (select, textarea, casilla, sección, avatar, archivo)
- Documentación v3.4 y matriz de trazabilidad

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/trazabilidad/Matriz de Trazabilidad MDF.xlsx
+++ b/docs/trazabilidad/Matriz de Trazabilidad MDF.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Origen v1" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Matriz'!$A$1:$N$94</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Matriz'!$A$1:$N$95</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -897,31 +897,31 @@
         </is>
       </c>
       <c r="B5" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$94,$A5)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$95,$A5)</f>
         <v/>
       </c>
       <c r="C5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$94,$A5,Matriz!$L$2:$L$94,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$95,$A5,Matriz!$L$2:$L$95,"Pendiente")</f>
         <v/>
       </c>
       <c r="D5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$94,$A5,Matriz!$L$2:$L$94,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$95,$A5,Matriz!$L$2:$L$95,"En diseño")</f>
         <v/>
       </c>
       <c r="E5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$94,$A5,Matriz!$L$2:$L$94,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$95,$A5,Matriz!$L$2:$L$95,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$94,$A5,Matriz!$L$2:$L$94,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$95,$A5,Matriz!$L$2:$L$95,"En pruebas")</f>
         <v/>
       </c>
       <c r="G5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$94,$A5,Matriz!$L$2:$L$94,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$95,$A5,Matriz!$L$2:$L$95,"Hecho")</f>
         <v/>
       </c>
       <c r="H5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$94,$A5,Matriz!$L$2:$L$94,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$95,$A5,Matriz!$L$2:$L$95,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I5" s="13">
@@ -936,31 +936,31 @@
         </is>
       </c>
       <c r="B6" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$94,$A6)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$95,$A6)</f>
         <v/>
       </c>
       <c r="C6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$94,$A6,Matriz!$L$2:$L$94,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$95,$A6,Matriz!$L$2:$L$95,"Pendiente")</f>
         <v/>
       </c>
       <c r="D6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$94,$A6,Matriz!$L$2:$L$94,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$95,$A6,Matriz!$L$2:$L$95,"En diseño")</f>
         <v/>
       </c>
       <c r="E6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$94,$A6,Matriz!$L$2:$L$94,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$95,$A6,Matriz!$L$2:$L$95,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$94,$A6,Matriz!$L$2:$L$94,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$95,$A6,Matriz!$L$2:$L$95,"En pruebas")</f>
         <v/>
       </c>
       <c r="G6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$94,$A6,Matriz!$L$2:$L$94,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$95,$A6,Matriz!$L$2:$L$95,"Hecho")</f>
         <v/>
       </c>
       <c r="H6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$94,$A6,Matriz!$L$2:$L$94,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$95,$A6,Matriz!$L$2:$L$95,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I6" s="13">
@@ -975,31 +975,31 @@
         </is>
       </c>
       <c r="B7" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$94,$A7)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$95,$A7)</f>
         <v/>
       </c>
       <c r="C7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$94,$A7,Matriz!$L$2:$L$94,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$95,$A7,Matriz!$L$2:$L$95,"Pendiente")</f>
         <v/>
       </c>
       <c r="D7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$94,$A7,Matriz!$L$2:$L$94,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$95,$A7,Matriz!$L$2:$L$95,"En diseño")</f>
         <v/>
       </c>
       <c r="E7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$94,$A7,Matriz!$L$2:$L$94,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$95,$A7,Matriz!$L$2:$L$95,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$94,$A7,Matriz!$L$2:$L$94,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$95,$A7,Matriz!$L$2:$L$95,"En pruebas")</f>
         <v/>
       </c>
       <c r="G7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$94,$A7,Matriz!$L$2:$L$94,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$95,$A7,Matriz!$L$2:$L$95,"Hecho")</f>
         <v/>
       </c>
       <c r="H7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$94,$A7,Matriz!$L$2:$L$94,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$95,$A7,Matriz!$L$2:$L$95,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I7" s="13">
@@ -1014,31 +1014,31 @@
         </is>
       </c>
       <c r="B8" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$94,$A8)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$95,$A8)</f>
         <v/>
       </c>
       <c r="C8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$94,$A8,Matriz!$L$2:$L$94,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$95,$A8,Matriz!$L$2:$L$95,"Pendiente")</f>
         <v/>
       </c>
       <c r="D8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$94,$A8,Matriz!$L$2:$L$94,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$95,$A8,Matriz!$L$2:$L$95,"En diseño")</f>
         <v/>
       </c>
       <c r="E8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$94,$A8,Matriz!$L$2:$L$94,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$95,$A8,Matriz!$L$2:$L$95,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$94,$A8,Matriz!$L$2:$L$94,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$95,$A8,Matriz!$L$2:$L$95,"En pruebas")</f>
         <v/>
       </c>
       <c r="G8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$94,$A8,Matriz!$L$2:$L$94,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$95,$A8,Matriz!$L$2:$L$95,"Hecho")</f>
         <v/>
       </c>
       <c r="H8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$94,$A8,Matriz!$L$2:$L$94,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$95,$A8,Matriz!$L$2:$L$95,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I8" s="13">
@@ -1053,31 +1053,31 @@
         </is>
       </c>
       <c r="B9" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$94,$A9)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$95,$A9)</f>
         <v/>
       </c>
       <c r="C9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$94,$A9,Matriz!$L$2:$L$94,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$95,$A9,Matriz!$L$2:$L$95,"Pendiente")</f>
         <v/>
       </c>
       <c r="D9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$94,$A9,Matriz!$L$2:$L$94,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$95,$A9,Matriz!$L$2:$L$95,"En diseño")</f>
         <v/>
       </c>
       <c r="E9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$94,$A9,Matriz!$L$2:$L$94,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$95,$A9,Matriz!$L$2:$L$95,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$94,$A9,Matriz!$L$2:$L$94,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$95,$A9,Matriz!$L$2:$L$95,"En pruebas")</f>
         <v/>
       </c>
       <c r="G9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$94,$A9,Matriz!$L$2:$L$94,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$95,$A9,Matriz!$L$2:$L$95,"Hecho")</f>
         <v/>
       </c>
       <c r="H9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$94,$A9,Matriz!$L$2:$L$94,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$95,$A9,Matriz!$L$2:$L$95,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I9" s="13">
@@ -1092,31 +1092,31 @@
         </is>
       </c>
       <c r="B10" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$94,$A10)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$95,$A10)</f>
         <v/>
       </c>
       <c r="C10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$94,$A10,Matriz!$L$2:$L$94,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$95,$A10,Matriz!$L$2:$L$95,"Pendiente")</f>
         <v/>
       </c>
       <c r="D10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$94,$A10,Matriz!$L$2:$L$94,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$95,$A10,Matriz!$L$2:$L$95,"En diseño")</f>
         <v/>
       </c>
       <c r="E10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$94,$A10,Matriz!$L$2:$L$94,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$95,$A10,Matriz!$L$2:$L$95,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$94,$A10,Matriz!$L$2:$L$94,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$95,$A10,Matriz!$L$2:$L$95,"En pruebas")</f>
         <v/>
       </c>
       <c r="G10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$94,$A10,Matriz!$L$2:$L$94,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$95,$A10,Matriz!$L$2:$L$95,"Hecho")</f>
         <v/>
       </c>
       <c r="H10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$94,$A10,Matriz!$L$2:$L$94,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$95,$A10,Matriz!$L$2:$L$95,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I10" s="13">
@@ -1131,31 +1131,31 @@
         </is>
       </c>
       <c r="B11" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$94,$A11)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$95,$A11)</f>
         <v/>
       </c>
       <c r="C11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$94,$A11,Matriz!$L$2:$L$94,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$95,$A11,Matriz!$L$2:$L$95,"Pendiente")</f>
         <v/>
       </c>
       <c r="D11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$94,$A11,Matriz!$L$2:$L$94,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$95,$A11,Matriz!$L$2:$L$95,"En diseño")</f>
         <v/>
       </c>
       <c r="E11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$94,$A11,Matriz!$L$2:$L$94,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$95,$A11,Matriz!$L$2:$L$95,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$94,$A11,Matriz!$L$2:$L$94,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$95,$A11,Matriz!$L$2:$L$95,"En pruebas")</f>
         <v/>
       </c>
       <c r="G11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$94,$A11,Matriz!$L$2:$L$94,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$95,$A11,Matriz!$L$2:$L$95,"Hecho")</f>
         <v/>
       </c>
       <c r="H11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$94,$A11,Matriz!$L$2:$L$94,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$95,$A11,Matriz!$L$2:$L$95,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I11" s="13">
@@ -1256,31 +1256,31 @@
         </is>
       </c>
       <c r="B16" s="12">
-        <f>COUNTIF(Matriz!$H$2:$H$94,$A16)</f>
+        <f>COUNTIF(Matriz!$H$2:$H$95,$A16)</f>
         <v/>
       </c>
       <c r="C16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$94,$A16,Matriz!$L$2:$L$94,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$95,$A16,Matriz!$L$2:$L$95,"Pendiente")</f>
         <v/>
       </c>
       <c r="D16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$94,$A16,Matriz!$L$2:$L$94,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$95,$A16,Matriz!$L$2:$L$95,"En diseño")</f>
         <v/>
       </c>
       <c r="E16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$94,$A16,Matriz!$L$2:$L$94,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$95,$A16,Matriz!$L$2:$L$95,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$94,$A16,Matriz!$L$2:$L$94,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$95,$A16,Matriz!$L$2:$L$95,"En pruebas")</f>
         <v/>
       </c>
       <c r="G16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$94,$A16,Matriz!$L$2:$L$94,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$95,$A16,Matriz!$L$2:$L$95,"Hecho")</f>
         <v/>
       </c>
       <c r="H16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$94,$A16,Matriz!$L$2:$L$94,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$95,$A16,Matriz!$L$2:$L$95,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I16" s="13">
@@ -1295,31 +1295,31 @@
         </is>
       </c>
       <c r="B17" s="12">
-        <f>COUNTIF(Matriz!$H$2:$H$94,$A17)</f>
+        <f>COUNTIF(Matriz!$H$2:$H$95,$A17)</f>
         <v/>
       </c>
       <c r="C17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$94,$A17,Matriz!$L$2:$L$94,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$95,$A17,Matriz!$L$2:$L$95,"Pendiente")</f>
         <v/>
       </c>
       <c r="D17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$94,$A17,Matriz!$L$2:$L$94,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$95,$A17,Matriz!$L$2:$L$95,"En diseño")</f>
         <v/>
       </c>
       <c r="E17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$94,$A17,Matriz!$L$2:$L$94,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$95,$A17,Matriz!$L$2:$L$95,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$94,$A17,Matriz!$L$2:$L$94,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$95,$A17,Matriz!$L$2:$L$95,"En pruebas")</f>
         <v/>
       </c>
       <c r="G17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$94,$A17,Matriz!$L$2:$L$94,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$95,$A17,Matriz!$L$2:$L$95,"Hecho")</f>
         <v/>
       </c>
       <c r="H17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$94,$A17,Matriz!$L$2:$L$94,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$95,$A17,Matriz!$L$2:$L$95,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I17" s="13">
@@ -1334,31 +1334,31 @@
         </is>
       </c>
       <c r="B18" s="12">
-        <f>COUNTIF(Matriz!$H$2:$H$94,$A18)</f>
+        <f>COUNTIF(Matriz!$H$2:$H$95,$A18)</f>
         <v/>
       </c>
       <c r="C18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$94,$A18,Matriz!$L$2:$L$94,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$95,$A18,Matriz!$L$2:$L$95,"Pendiente")</f>
         <v/>
       </c>
       <c r="D18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$94,$A18,Matriz!$L$2:$L$94,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$95,$A18,Matriz!$L$2:$L$95,"En diseño")</f>
         <v/>
       </c>
       <c r="E18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$94,$A18,Matriz!$L$2:$L$94,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$95,$A18,Matriz!$L$2:$L$95,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$94,$A18,Matriz!$L$2:$L$94,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$95,$A18,Matriz!$L$2:$L$95,"En pruebas")</f>
         <v/>
       </c>
       <c r="G18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$94,$A18,Matriz!$L$2:$L$94,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$95,$A18,Matriz!$L$2:$L$95,"Hecho")</f>
         <v/>
       </c>
       <c r="H18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$94,$A18,Matriz!$L$2:$L$94,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$95,$A18,Matriz!$L$2:$L$95,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I18" s="13">
@@ -1373,31 +1373,31 @@
         </is>
       </c>
       <c r="B19" s="12">
-        <f>COUNTIF(Matriz!$H$2:$H$94,$A19)</f>
+        <f>COUNTIF(Matriz!$H$2:$H$95,$A19)</f>
         <v/>
       </c>
       <c r="C19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$94,$A19,Matriz!$L$2:$L$94,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$95,$A19,Matriz!$L$2:$L$95,"Pendiente")</f>
         <v/>
       </c>
       <c r="D19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$94,$A19,Matriz!$L$2:$L$94,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$95,$A19,Matriz!$L$2:$L$95,"En diseño")</f>
         <v/>
       </c>
       <c r="E19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$94,$A19,Matriz!$L$2:$L$94,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$95,$A19,Matriz!$L$2:$L$95,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$94,$A19,Matriz!$L$2:$L$94,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$95,$A19,Matriz!$L$2:$L$95,"En pruebas")</f>
         <v/>
       </c>
       <c r="G19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$94,$A19,Matriz!$L$2:$L$94,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$95,$A19,Matriz!$L$2:$L$95,"Hecho")</f>
         <v/>
       </c>
       <c r="H19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$94,$A19,Matriz!$L$2:$L$94,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$95,$A19,Matriz!$L$2:$L$95,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I19" s="13">
@@ -1498,31 +1498,31 @@
         </is>
       </c>
       <c r="B24" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$94,$A24)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$95,$A24)</f>
         <v/>
       </c>
       <c r="C24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$94,$A24,Matriz!$L$2:$L$94,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$95,$A24,Matriz!$L$2:$L$95,"Pendiente")</f>
         <v/>
       </c>
       <c r="D24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$94,$A24,Matriz!$L$2:$L$94,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$95,$A24,Matriz!$L$2:$L$95,"En diseño")</f>
         <v/>
       </c>
       <c r="E24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$94,$A24,Matriz!$L$2:$L$94,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$95,$A24,Matriz!$L$2:$L$95,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$94,$A24,Matriz!$L$2:$L$94,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$95,$A24,Matriz!$L$2:$L$95,"En pruebas")</f>
         <v/>
       </c>
       <c r="G24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$94,$A24,Matriz!$L$2:$L$94,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$95,$A24,Matriz!$L$2:$L$95,"Hecho")</f>
         <v/>
       </c>
       <c r="H24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$94,$A24,Matriz!$L$2:$L$94,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$95,$A24,Matriz!$L$2:$L$95,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I24" s="13">
@@ -1537,31 +1537,31 @@
         </is>
       </c>
       <c r="B25" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$94,$A25)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$95,$A25)</f>
         <v/>
       </c>
       <c r="C25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$94,$A25,Matriz!$L$2:$L$94,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$95,$A25,Matriz!$L$2:$L$95,"Pendiente")</f>
         <v/>
       </c>
       <c r="D25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$94,$A25,Matriz!$L$2:$L$94,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$95,$A25,Matriz!$L$2:$L$95,"En diseño")</f>
         <v/>
       </c>
       <c r="E25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$94,$A25,Matriz!$L$2:$L$94,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$95,$A25,Matriz!$L$2:$L$95,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$94,$A25,Matriz!$L$2:$L$94,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$95,$A25,Matriz!$L$2:$L$95,"En pruebas")</f>
         <v/>
       </c>
       <c r="G25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$94,$A25,Matriz!$L$2:$L$94,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$95,$A25,Matriz!$L$2:$L$95,"Hecho")</f>
         <v/>
       </c>
       <c r="H25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$94,$A25,Matriz!$L$2:$L$94,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$95,$A25,Matriz!$L$2:$L$95,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I25" s="13">
@@ -1576,31 +1576,31 @@
         </is>
       </c>
       <c r="B26" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$94,$A26)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$95,$A26)</f>
         <v/>
       </c>
       <c r="C26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$94,$A26,Matriz!$L$2:$L$94,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$95,$A26,Matriz!$L$2:$L$95,"Pendiente")</f>
         <v/>
       </c>
       <c r="D26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$94,$A26,Matriz!$L$2:$L$94,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$95,$A26,Matriz!$L$2:$L$95,"En diseño")</f>
         <v/>
       </c>
       <c r="E26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$94,$A26,Matriz!$L$2:$L$94,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$95,$A26,Matriz!$L$2:$L$95,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$94,$A26,Matriz!$L$2:$L$94,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$95,$A26,Matriz!$L$2:$L$95,"En pruebas")</f>
         <v/>
       </c>
       <c r="G26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$94,$A26,Matriz!$L$2:$L$94,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$95,$A26,Matriz!$L$2:$L$95,"Hecho")</f>
         <v/>
       </c>
       <c r="H26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$94,$A26,Matriz!$L$2:$L$94,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$95,$A26,Matriz!$L$2:$L$95,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I26" s="13">
@@ -1615,31 +1615,31 @@
         </is>
       </c>
       <c r="B27" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$94,$A27)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$95,$A27)</f>
         <v/>
       </c>
       <c r="C27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$94,$A27,Matriz!$L$2:$L$94,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$95,$A27,Matriz!$L$2:$L$95,"Pendiente")</f>
         <v/>
       </c>
       <c r="D27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$94,$A27,Matriz!$L$2:$L$94,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$95,$A27,Matriz!$L$2:$L$95,"En diseño")</f>
         <v/>
       </c>
       <c r="E27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$94,$A27,Matriz!$L$2:$L$94,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$95,$A27,Matriz!$L$2:$L$95,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$94,$A27,Matriz!$L$2:$L$94,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$95,$A27,Matriz!$L$2:$L$95,"En pruebas")</f>
         <v/>
       </c>
       <c r="G27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$94,$A27,Matriz!$L$2:$L$94,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$95,$A27,Matriz!$L$2:$L$95,"Hecho")</f>
         <v/>
       </c>
       <c r="H27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$94,$A27,Matriz!$L$2:$L$94,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$95,$A27,Matriz!$L$2:$L$95,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I27" s="13">
@@ -1654,31 +1654,31 @@
         </is>
       </c>
       <c r="B28" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$94,$A28)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$95,$A28)</f>
         <v/>
       </c>
       <c r="C28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$94,$A28,Matriz!$L$2:$L$94,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$95,$A28,Matriz!$L$2:$L$95,"Pendiente")</f>
         <v/>
       </c>
       <c r="D28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$94,$A28,Matriz!$L$2:$L$94,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$95,$A28,Matriz!$L$2:$L$95,"En diseño")</f>
         <v/>
       </c>
       <c r="E28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$94,$A28,Matriz!$L$2:$L$94,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$95,$A28,Matriz!$L$2:$L$95,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$94,$A28,Matriz!$L$2:$L$94,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$95,$A28,Matriz!$L$2:$L$95,"En pruebas")</f>
         <v/>
       </c>
       <c r="G28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$94,$A28,Matriz!$L$2:$L$94,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$95,$A28,Matriz!$L$2:$L$95,"Hecho")</f>
         <v/>
       </c>
       <c r="H28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$94,$A28,Matriz!$L$2:$L$94,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$95,$A28,Matriz!$L$2:$L$95,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I28" s="13">
@@ -1693,31 +1693,31 @@
         </is>
       </c>
       <c r="B29" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$94,$A29)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$95,$A29)</f>
         <v/>
       </c>
       <c r="C29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$94,$A29,Matriz!$L$2:$L$94,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$95,$A29,Matriz!$L$2:$L$95,"Pendiente")</f>
         <v/>
       </c>
       <c r="D29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$94,$A29,Matriz!$L$2:$L$94,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$95,$A29,Matriz!$L$2:$L$95,"En diseño")</f>
         <v/>
       </c>
       <c r="E29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$94,$A29,Matriz!$L$2:$L$94,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$95,$A29,Matriz!$L$2:$L$95,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$94,$A29,Matriz!$L$2:$L$94,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$95,$A29,Matriz!$L$2:$L$95,"En pruebas")</f>
         <v/>
       </c>
       <c r="G29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$94,$A29,Matriz!$L$2:$L$94,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$95,$A29,Matriz!$L$2:$L$95,"Hecho")</f>
         <v/>
       </c>
       <c r="H29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$94,$A29,Matriz!$L$2:$L$94,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$95,$A29,Matriz!$L$2:$L$95,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I29" s="13">
@@ -1732,31 +1732,31 @@
         </is>
       </c>
       <c r="B30" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$94,$A30)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$95,$A30)</f>
         <v/>
       </c>
       <c r="C30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$94,$A30,Matriz!$L$2:$L$94,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$95,$A30,Matriz!$L$2:$L$95,"Pendiente")</f>
         <v/>
       </c>
       <c r="D30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$94,$A30,Matriz!$L$2:$L$94,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$95,$A30,Matriz!$L$2:$L$95,"En diseño")</f>
         <v/>
       </c>
       <c r="E30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$94,$A30,Matriz!$L$2:$L$94,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$95,$A30,Matriz!$L$2:$L$95,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$94,$A30,Matriz!$L$2:$L$94,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$95,$A30,Matriz!$L$2:$L$95,"En pruebas")</f>
         <v/>
       </c>
       <c r="G30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$94,$A30,Matriz!$L$2:$L$94,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$95,$A30,Matriz!$L$2:$L$95,"Hecho")</f>
         <v/>
       </c>
       <c r="H30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$94,$A30,Matriz!$L$2:$L$94,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$95,$A30,Matriz!$L$2:$L$95,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I30" s="13">
@@ -1818,7 +1818,7 @@
         </is>
       </c>
       <c r="B35" s="12">
-        <f>COUNTIF(Matriz!$K$2:$K$94,A35)</f>
+        <f>COUNTIF(Matriz!$K$2:$K$95,A35)</f>
         <v/>
       </c>
     </row>
@@ -1829,7 +1829,7 @@
         </is>
       </c>
       <c r="B36" s="12">
-        <f>COUNTIF(Matriz!$K$2:$K$94,A36)</f>
+        <f>COUNTIF(Matriz!$K$2:$K$95,A36)</f>
         <v/>
       </c>
     </row>
@@ -1840,7 +1840,7 @@
         </is>
       </c>
       <c r="B37" s="12">
-        <f>COUNTIF(Matriz!$K$2:$K$94,A37)</f>
+        <f>COUNTIF(Matriz!$K$2:$K$95,A37)</f>
         <v/>
       </c>
     </row>
@@ -1851,7 +1851,7 @@
         </is>
       </c>
       <c r="B38" s="12">
-        <f>COUNTIF(Matriz!$K$2:$K$94,A38)</f>
+        <f>COUNTIF(Matriz!$K$2:$K$95,A38)</f>
         <v/>
       </c>
     </row>
@@ -1866,7 +1866,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N94"/>
+  <dimension ref="A1:N95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2482,12 +2482,12 @@
       </c>
       <c r="C10" s="19" t="inlineStr">
         <is>
-          <t>Expediente Digital Único (EDU) con foto, datos personales, historial de cursos, trayectoria de servicio e historial de grupos de conexión. En el MVP se llenan datos personales, foto y grupos.</t>
+          <t>Expediente Digital Único (EDU) con los campos de la «Radiografía de miembros GC»: foto; nombre, apellidos, fecha de nacimiento (la edad se calcula); calle y número, colonia, código postal, alcaldía; teléfono fijo y celular; correo; grupo de conexión, líder y sector (texto provisional hasta el módulo de Grupos); tiempo en Mundo de Fe; ministerios en que sirve; devocional personal; Oración de Familias en Acción; otros cursos y observaciones. La foto se guarda en una carpeta del servidor con su ruta en la base de datos y solo se ve con sesión y permisos.</t>
         </is>
       </c>
       <c r="D10" s="19" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>v3 + Radiografía</t>
         </is>
       </c>
       <c r="E10" s="19" t="inlineStr">
@@ -2512,12 +2512,12 @@
       </c>
       <c r="I10" s="19" t="inlineStr">
         <is>
-          <t>Como pastor quiero un expediente por persona con foto y datos para conocer a mi gente.</t>
+          <t>Como pastor quiero un expediente por persona con los datos de la Radiografía de miembros GC para conocer a mi gente.</t>
         </is>
       </c>
       <c r="J10" s="19" t="inlineStr">
         <is>
-          <t>Crear un EDU con foto, datos personales y grupo, y consultarlo con el rol adecuado.</t>
+          <t>Crear un EDU con foto y los campos de la Radiografía, buscarlo sin importar acentos y consultarlo con el rol adecuado; la foto solo se ve con sesión.</t>
         </is>
       </c>
       <c r="K10" s="19" t="inlineStr">
@@ -2527,11 +2527,19 @@
       </c>
       <c r="L10" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M10" s="19" t="inlineStr"/>
-      <c r="N10" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M10" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/m1-01-expediente · 56 pruebas de backend y 6 de frontend pasan</t>
+        </is>
+      </c>
+      <c r="N10" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-05 · Falta revisar con la iglesia que los campos y el orden de la Radiografía estén completos.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="18" t="inlineStr">
@@ -3122,7 +3130,7 @@
       </c>
       <c r="C20" s="19" t="inlineStr">
         <is>
-          <t>Aviso de privacidad y consentimiento al registrar a cualquier persona, con consentimiento reforzado para foto y datos de menores.</t>
+          <t>Aviso de privacidad y consentimiento al registrar a cualquier persona o activar una cuenta, con consentimiento aparte para la foto. Cada consentimiento guarda la versión del aviso y la fecha. Por ahora el texto es genérico de ejemplo y debe sustituirse por el oficial antes de producción.</t>
         </is>
       </c>
       <c r="D20" s="19" t="inlineStr">
@@ -3167,11 +3175,19 @@
       </c>
       <c r="L20" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M20" s="19" t="inlineStr"/>
-      <c r="N20" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M20" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/m1-01-expediente · 56 pruebas de backend y 6 de frontend pasan</t>
+        </is>
+      </c>
+      <c r="N20" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-05 · Texto del aviso genérico; sustituir por el oficial antes de producción.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="18" t="inlineStr">
@@ -3231,11 +3247,19 @@
       </c>
       <c r="L21" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M21" s="19" t="inlineStr"/>
-      <c r="N21" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M21" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/m1-01-expediente · 56 pruebas de backend y 6 de frontend pasan</t>
+        </is>
+      </c>
+      <c r="N21" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-05 · Niveles contacto → participante → expediente completo; duplicados por WhatsApp.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="18" t="inlineStr">
@@ -3295,11 +3319,19 @@
       </c>
       <c r="L22" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M22" s="19" t="inlineStr"/>
-      <c r="N22" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M22" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/m1-01-expediente · 56 pruebas de backend y 6 de frontend pasan</t>
+        </is>
+      </c>
+      <c r="N22" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-05 · Procedencia en el alta y en la ficha.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="18" t="inlineStr">
@@ -3359,11 +3391,19 @@
       </c>
       <c r="L23" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M23" s="19" t="inlineStr"/>
-      <c r="N23" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M23" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/m1-01-expediente · 56 pruebas de backend y 6 de frontend pasan</t>
+        </is>
+      </c>
+      <c r="N23" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-05 · Historial de movimientos con fecha y motivo.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="18" t="inlineStr">
@@ -3423,11 +3463,19 @@
       </c>
       <c r="L24" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M24" s="19" t="inlineStr"/>
-      <c r="N24" s="19" t="inlineStr"/>
+          <t>En desarrollo</t>
+        </is>
+      </c>
+      <c r="M24" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/m1-01-expediente · 56 pruebas de backend y 6 de frontend pasan</t>
+        </is>
+      </c>
+      <c r="N24" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-05 · Consultas y cambios de personas ya quedan en bitácora; falta restringir por rol (RBAC).</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="18" t="inlineStr">
@@ -3776,52 +3824,52 @@
     <row r="30">
       <c r="A30" s="18" t="inlineStr">
         <is>
-          <t>M2A-01</t>
+          <t>M1-23</t>
         </is>
       </c>
       <c r="B30" s="19" t="inlineStr">
         <is>
-          <t>M2A Cursos de Vida</t>
+          <t>M1 Identidad y comunicación</t>
         </is>
       </c>
       <c r="C30" s="19" t="inlineStr">
         <is>
-          <t>Catálogo dinámico de cursos; se pueden crear nuevos sin intervención técnica. Incluye «Resolución de Varones» y «Toma de Buenas Decisiones», omitidos en v2.</t>
-        </is>
-      </c>
-      <c r="D30" s="22" t="inlineStr">
-        <is>
-          <t>Recuperado v1</t>
+          <t>Procesos de desarrollo discipular: catálogo configurable (14 procesos de la Radiografía: Nacimiento Espiritual, Consolidación, Peniel, Bautismo en el Espíritu Santo, Bautismo en Agua, Sanidad Total, Fundamentos de la Vida Cristiana, Fundamentos Doctrinales, Fundamentos de Liderazgo, Avanzado hacia la Meta, Visión G. de Conexión, Espíritu Santo, Panorama Bíblico y Lanzamiento) y avance por persona con fecha y nombre del maestro.</t>
+        </is>
+      </c>
+      <c r="D30" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3.4</t>
         </is>
       </c>
       <c r="E30" s="19" t="inlineStr">
         <is>
-          <t>Fuera del MVP</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="F30" s="19" t="inlineStr">
         <is>
-          <t>Fase 3</t>
+          <t>Fase 0</t>
         </is>
       </c>
       <c r="G30" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sprint 1</t>
         </is>
       </c>
       <c r="H30" s="19" t="inlineStr">
         <is>
-          <t>Posterior</t>
-        </is>
-      </c>
-      <c r="I30" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
-        </is>
-      </c>
-      <c r="J30" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
+          <t>H1 · 18-oct (núcleo Fase 0)</t>
+        </is>
+      </c>
+      <c r="I30" s="19" t="inlineStr">
+        <is>
+          <t>Como líder quiero registrar los procesos de discipulado que ha cursado cada persona, con fecha y maestro.</t>
+        </is>
+      </c>
+      <c r="J30" s="19" t="inlineStr">
+        <is>
+          <t>Marcar procesos del catálogo con fecha y maestro, guardarlos y verlos en la ficha; el catálogo es configurable.</t>
         </is>
       </c>
       <c r="K30" s="19" t="inlineStr">
@@ -3831,16 +3879,24 @@
       </c>
       <c r="L30" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M30" s="19" t="inlineStr"/>
-      <c r="N30" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M30" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/m1-01-expediente · 56 pruebas de backend y 6 de frontend pasan</t>
+        </is>
+      </c>
+      <c r="N30" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-05 · 14 procesos sembrados desde la Radiografía.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="18" t="inlineStr">
         <is>
-          <t>M2A-02</t>
+          <t>M2A-01</t>
         </is>
       </c>
       <c r="B31" s="19" t="inlineStr">
@@ -3850,12 +3906,12 @@
       </c>
       <c r="C31" s="19" t="inlineStr">
         <is>
-          <t>Flexibilidad operativa: sin día ni horario fijo; el día y el ponente pueden cambiar entre ediciones.</t>
-        </is>
-      </c>
-      <c r="D31" s="19" t="inlineStr">
-        <is>
-          <t>v1 / v2</t>
+          <t>Catálogo dinámico de cursos; se pueden crear nuevos sin intervención técnica. Incluye «Resolución de Varones» y «Toma de Buenas Decisiones», omitidos en v2.</t>
+        </is>
+      </c>
+      <c r="D31" s="22" t="inlineStr">
+        <is>
+          <t>Recuperado v1</t>
         </is>
       </c>
       <c r="E31" s="19" t="inlineStr">
@@ -3904,7 +3960,7 @@
     <row r="32">
       <c r="A32" s="18" t="inlineStr">
         <is>
-          <t>M2A-03</t>
+          <t>M2A-02</t>
         </is>
       </c>
       <c r="B32" s="19" t="inlineStr">
@@ -3914,7 +3970,7 @@
       </c>
       <c r="C32" s="19" t="inlineStr">
         <is>
-          <t>Reposición de clases: el inscrito puede reponer en otro grupo o con otro ponente, a decisión de quien imparte.</t>
+          <t>Flexibilidad operativa: sin día ni horario fijo; el día y el ponente pueden cambiar entre ediciones.</t>
         </is>
       </c>
       <c r="D32" s="19" t="inlineStr">
@@ -3968,7 +4024,7 @@
     <row r="33">
       <c r="A33" s="18" t="inlineStr">
         <is>
-          <t>M2A-04</t>
+          <t>M2A-03</t>
         </is>
       </c>
       <c r="B33" s="19" t="inlineStr">
@@ -3978,7 +4034,7 @@
       </c>
       <c r="C33" s="19" t="inlineStr">
         <is>
-          <t>Registro de asistencia por sesión.</t>
+          <t>Reposición de clases: el inscrito puede reponer en otro grupo o con otro ponente, a decisión de quien imparte.</t>
         </is>
       </c>
       <c r="D33" s="19" t="inlineStr">
@@ -4032,7 +4088,7 @@
     <row r="34">
       <c r="A34" s="18" t="inlineStr">
         <is>
-          <t>M2A-05</t>
+          <t>M2A-04</t>
         </is>
       </c>
       <c r="B34" s="19" t="inlineStr">
@@ -4042,7 +4098,7 @@
       </c>
       <c r="C34" s="19" t="inlineStr">
         <is>
-          <t>Seguimiento de tareas o actividades opcionales (no sumativas).</t>
+          <t>Registro de asistencia por sesión.</t>
         </is>
       </c>
       <c r="D34" s="19" t="inlineStr">
@@ -4096,7 +4152,7 @@
     <row r="35">
       <c r="A35" s="18" t="inlineStr">
         <is>
-          <t>M2A-06</t>
+          <t>M2A-05</t>
         </is>
       </c>
       <c r="B35" s="19" t="inlineStr">
@@ -4106,7 +4162,7 @@
       </c>
       <c r="C35" s="19" t="inlineStr">
         <is>
-          <t>Inscripción: quién se inscribe, cuándo lo hizo, si tiene adeudo y qué incluye el costo (materiales, hospedaje, etc.).</t>
+          <t>Seguimiento de tareas o actividades opcionales (no sumativas).</t>
         </is>
       </c>
       <c r="D35" s="19" t="inlineStr">
@@ -4160,7 +4216,7 @@
     <row r="36">
       <c r="A36" s="18" t="inlineStr">
         <is>
-          <t>M2A-07</t>
+          <t>M2A-06</t>
         </is>
       </c>
       <c r="B36" s="19" t="inlineStr">
@@ -4170,12 +4226,12 @@
       </c>
       <c r="C36" s="19" t="inlineStr">
         <is>
-          <t>Registro de pagos, saldo de adeudos y recibo. Por definir: captura manual vs. pasarela de pago, y si se requiere corte de caja.</t>
-        </is>
-      </c>
-      <c r="D36" s="21" t="inlineStr">
-        <is>
-          <t>Nuevo v3</t>
+          <t>Inscripción: quién se inscribe, cuándo lo hizo, si tiene adeudo y qué incluye el costo (materiales, hospedaje, etc.).</t>
+        </is>
+      </c>
+      <c r="D36" s="19" t="inlineStr">
+        <is>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E36" s="19" t="inlineStr">
@@ -4210,7 +4266,7 @@
       </c>
       <c r="K36" s="19" t="inlineStr">
         <is>
-          <t>Por definir</t>
+          <t>VoBo pendiente</t>
         </is>
       </c>
       <c r="L36" s="19" t="inlineStr">
@@ -4224,7 +4280,7 @@
     <row r="37">
       <c r="A37" s="18" t="inlineStr">
         <is>
-          <t>M2A-08</t>
+          <t>M2A-07</t>
         </is>
       </c>
       <c r="B37" s="19" t="inlineStr">
@@ -4234,12 +4290,12 @@
       </c>
       <c r="C37" s="19" t="inlineStr">
         <is>
-          <t>Tablero del curso tipo mensajería para avisos antes del curso y días posteriores, con notificación a los inscritos.</t>
-        </is>
-      </c>
-      <c r="D37" s="22" t="inlineStr">
-        <is>
-          <t>Recuperado v1</t>
+          <t>Registro de pagos, saldo de adeudos y recibo. Por definir: captura manual vs. pasarela de pago, y si se requiere corte de caja.</t>
+        </is>
+      </c>
+      <c r="D37" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3</t>
         </is>
       </c>
       <c r="E37" s="19" t="inlineStr">
@@ -4274,7 +4330,7 @@
       </c>
       <c r="K37" s="19" t="inlineStr">
         <is>
-          <t>VoBo pendiente</t>
+          <t>Por definir</t>
         </is>
       </c>
       <c r="L37" s="19" t="inlineStr">
@@ -4288,7 +4344,7 @@
     <row r="38">
       <c r="A38" s="18" t="inlineStr">
         <is>
-          <t>M2A-09</t>
+          <t>M2A-08</t>
         </is>
       </c>
       <c r="B38" s="19" t="inlineStr">
@@ -4298,12 +4354,12 @@
       </c>
       <c r="C38" s="19" t="inlineStr">
         <is>
-          <t>Evaluación docente configurable: formulario diseñable (tipo Google Forms) aplicado al finalizar el curso.</t>
-        </is>
-      </c>
-      <c r="D38" s="19" t="inlineStr">
-        <is>
-          <t>v1 / v2</t>
+          <t>Tablero del curso tipo mensajería para avisos antes del curso y días posteriores, con notificación a los inscritos.</t>
+        </is>
+      </c>
+      <c r="D38" s="22" t="inlineStr">
+        <is>
+          <t>Recuperado v1</t>
         </is>
       </c>
       <c r="E38" s="19" t="inlineStr">
@@ -4352,7 +4408,7 @@
     <row r="39">
       <c r="A39" s="18" t="inlineStr">
         <is>
-          <t>M2A-10</t>
+          <t>M2A-09</t>
         </is>
       </c>
       <c r="B39" s="19" t="inlineStr">
@@ -4362,12 +4418,12 @@
       </c>
       <c r="C39" s="19" t="inlineStr">
         <is>
-          <t>Evolución del ponente: historial de evaluaciones por ponente a lo largo del tiempo y entre ediciones.</t>
-        </is>
-      </c>
-      <c r="D39" s="22" t="inlineStr">
-        <is>
-          <t>Recuperado v1</t>
+          <t>Evaluación docente configurable: formulario diseñable (tipo Google Forms) aplicado al finalizar el curso.</t>
+        </is>
+      </c>
+      <c r="D39" s="19" t="inlineStr">
+        <is>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E39" s="19" t="inlineStr">
@@ -4416,7 +4472,7 @@
     <row r="40">
       <c r="A40" s="18" t="inlineStr">
         <is>
-          <t>M2A-11</t>
+          <t>M2A-10</t>
         </is>
       </c>
       <c r="B40" s="19" t="inlineStr">
@@ -4426,12 +4482,12 @@
       </c>
       <c r="C40" s="19" t="inlineStr">
         <is>
-          <t>Reconocimiento de participación (diploma) opcional por curso.</t>
-        </is>
-      </c>
-      <c r="D40" s="19" t="inlineStr">
-        <is>
-          <t>v1 / v2</t>
+          <t>Evolución del ponente: historial de evaluaciones por ponente a lo largo del tiempo y entre ediciones.</t>
+        </is>
+      </c>
+      <c r="D40" s="22" t="inlineStr">
+        <is>
+          <t>Recuperado v1</t>
         </is>
       </c>
       <c r="E40" s="19" t="inlineStr">
@@ -4480,17 +4536,17 @@
     <row r="41">
       <c r="A41" s="18" t="inlineStr">
         <is>
-          <t>M2B-01</t>
+          <t>M2A-11</t>
         </is>
       </c>
       <c r="B41" s="19" t="inlineStr">
         <is>
-          <t>M2B Cursos escolarizados</t>
+          <t>M2A Cursos de Vida</t>
         </is>
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>Control riguroso de asistencia.</t>
+          <t>Reconocimiento de participación (diploma) opcional por curso.</t>
         </is>
       </c>
       <c r="D41" s="19" t="inlineStr">
@@ -4544,7 +4600,7 @@
     <row r="42">
       <c r="A42" s="18" t="inlineStr">
         <is>
-          <t>M2B-02</t>
+          <t>M2B-01</t>
         </is>
       </c>
       <c r="B42" s="19" t="inlineStr">
@@ -4554,7 +4610,7 @@
       </c>
       <c r="C42" s="19" t="inlineStr">
         <is>
-          <t>Entrega de tareas y trabajos continuos (incluidos trabajos extra).</t>
+          <t>Control riguroso de asistencia.</t>
         </is>
       </c>
       <c r="D42" s="19" t="inlineStr">
@@ -4608,7 +4664,7 @@
     <row r="43">
       <c r="A43" s="18" t="inlineStr">
         <is>
-          <t>M2B-03</t>
+          <t>M2B-02</t>
         </is>
       </c>
       <c r="B43" s="19" t="inlineStr">
@@ -4618,7 +4674,7 @@
       </c>
       <c r="C43" s="19" t="inlineStr">
         <is>
-          <t>Ponderación de calificaciones y exámenes finales.</t>
+          <t>Entrega de tareas y trabajos continuos (incluidos trabajos extra).</t>
         </is>
       </c>
       <c r="D43" s="19" t="inlineStr">
@@ -4672,7 +4728,7 @@
     <row r="44">
       <c r="A44" s="18" t="inlineStr">
         <is>
-          <t>M2B-04</t>
+          <t>M2B-03</t>
         </is>
       </c>
       <c r="B44" s="19" t="inlineStr">
@@ -4682,12 +4738,12 @@
       </c>
       <c r="C44" s="19" t="inlineStr">
         <is>
-          <t>Creador de exámenes en línea: opción múltiple, preguntas abiertas, falso/verdadero y respuesta corta.</t>
+          <t>Ponderación de calificaciones y exámenes finales.</t>
         </is>
       </c>
       <c r="D44" s="19" t="inlineStr">
         <is>
-          <t>v2</t>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E44" s="19" t="inlineStr">
@@ -4736,7 +4792,7 @@
     <row r="45">
       <c r="A45" s="18" t="inlineStr">
         <is>
-          <t>M2B-05</t>
+          <t>M2B-04</t>
         </is>
       </c>
       <c r="B45" s="19" t="inlineStr">
@@ -4746,12 +4802,12 @@
       </c>
       <c r="C45" s="19" t="inlineStr">
         <is>
-          <t>Boleta digital con el formato definido por la iglesia. Por definir: formato oficial de la boleta.</t>
+          <t>Creador de exámenes en línea: opción múltiple, preguntas abiertas, falso/verdadero y respuesta corta.</t>
         </is>
       </c>
       <c r="D45" s="19" t="inlineStr">
         <is>
-          <t>v1 / v2</t>
+          <t>v2</t>
         </is>
       </c>
       <c r="E45" s="19" t="inlineStr">
@@ -4786,7 +4842,7 @@
       </c>
       <c r="K45" s="19" t="inlineStr">
         <is>
-          <t>Por definir</t>
+          <t>VoBo pendiente</t>
         </is>
       </c>
       <c r="L45" s="19" t="inlineStr">
@@ -4800,7 +4856,7 @@
     <row r="46">
       <c r="A46" s="18" t="inlineStr">
         <is>
-          <t>M2B-06</t>
+          <t>M2B-05</t>
         </is>
       </c>
       <c r="B46" s="19" t="inlineStr">
@@ -4810,12 +4866,12 @@
       </c>
       <c r="C46" s="19" t="inlineStr">
         <is>
-          <t>Historial académico permanente en el Expediente Digital, aunque cambie el maestro o el alumno pierda su comprobante.</t>
+          <t>Boleta digital con el formato definido por la iglesia. Por definir: formato oficial de la boleta.</t>
         </is>
       </c>
       <c r="D46" s="19" t="inlineStr">
         <is>
-          <t>v2</t>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E46" s="19" t="inlineStr">
@@ -4850,7 +4906,7 @@
       </c>
       <c r="K46" s="19" t="inlineStr">
         <is>
-          <t>VoBo pendiente</t>
+          <t>Por definir</t>
         </is>
       </c>
       <c r="L46" s="19" t="inlineStr">
@@ -4864,52 +4920,52 @@
     <row r="47">
       <c r="A47" s="18" t="inlineStr">
         <is>
-          <t>M3-01</t>
+          <t>M2B-06</t>
         </is>
       </c>
       <c r="B47" s="19" t="inlineStr">
         <is>
-          <t>M3 Grupos de Conexión</t>
+          <t>M2B Cursos escolarizados</t>
         </is>
       </c>
       <c r="C47" s="19" t="inlineStr">
         <is>
-          <t>Estructura del grupo con roles: Supervisor (supervisa uno o varios grupos y reporta al Pastor), Líder, Secretario, Anfitrión y Tesorero.</t>
+          <t>Historial académico permanente en el Expediente Digital, aunque cambie el maestro o el alumno pierda su comprobante.</t>
         </is>
       </c>
       <c r="D47" s="19" t="inlineStr">
         <is>
-          <t>v3 + Obs. 4</t>
+          <t>v2</t>
         </is>
       </c>
       <c r="E47" s="19" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Fuera del MVP</t>
         </is>
       </c>
       <c r="F47" s="19" t="inlineStr">
         <is>
-          <t>Fase 1</t>
+          <t>Fase 3</t>
         </is>
       </c>
       <c r="G47" s="19" t="inlineStr">
         <is>
-          <t>Sprint 3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H47" s="19" t="inlineStr">
         <is>
-          <t>H3 · MVP (Grupos)</t>
-        </is>
-      </c>
-      <c r="I47" s="19" t="inlineStr">
-        <is>
-          <t>Como supervisor quiero asignar Líder, Secretario, Anfitrión y Tesorero a cada grupo.</t>
-        </is>
-      </c>
-      <c r="J47" s="19" t="inlineStr">
-        <is>
-          <t>Un grupo tiene sus roles asignados; un supervisor ve varios grupos.</t>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="I47" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
+        </is>
+      </c>
+      <c r="J47" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
         </is>
       </c>
       <c r="K47" s="19" t="inlineStr">
@@ -4928,7 +4984,7 @@
     <row r="48">
       <c r="A48" s="18" t="inlineStr">
         <is>
-          <t>M3-02</t>
+          <t>M3-01</t>
         </is>
       </c>
       <c r="B48" s="19" t="inlineStr">
@@ -4938,12 +4994,12 @@
       </c>
       <c r="C48" s="19" t="inlineStr">
         <is>
-          <t>Distribución del estudio semanal dentro de la app, sustituyendo el envío por WhatsApp.</t>
+          <t>Estructura del grupo con roles: Supervisor (supervisa uno o varios grupos y reporta al Pastor), Líder, Secretario, Anfitrión y Tesorero.</t>
         </is>
       </c>
       <c r="D48" s="19" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>v3 + Obs. 4</t>
         </is>
       </c>
       <c r="E48" s="19" t="inlineStr">
@@ -4968,12 +5024,12 @@
       </c>
       <c r="I48" s="19" t="inlineStr">
         <is>
-          <t>Como líder quiero recibir el estudio semanal en la app en lugar de WhatsApp.</t>
+          <t>Como supervisor quiero asignar Líder, Secretario, Anfitrión y Tesorero a cada grupo.</t>
         </is>
       </c>
       <c r="J48" s="19" t="inlineStr">
         <is>
-          <t>Publicar el material de la semana; el líder lo abre y queda marca de lectura.</t>
+          <t>Un grupo tiene sus roles asignados; un supervisor ve varios grupos.</t>
         </is>
       </c>
       <c r="K48" s="19" t="inlineStr">
@@ -4992,7 +5048,7 @@
     <row r="49">
       <c r="A49" s="18" t="inlineStr">
         <is>
-          <t>M3-03</t>
+          <t>M3-02</t>
         </is>
       </c>
       <c r="B49" s="19" t="inlineStr">
@@ -5002,7 +5058,7 @@
       </c>
       <c r="C49" s="19" t="inlineStr">
         <is>
-          <t>Pase de lista digital por Secretario o Líder, con captura sin conexión y sincronización posterior.</t>
+          <t>Distribución del estudio semanal dentro de la app, sustituyendo el envío por WhatsApp.</t>
         </is>
       </c>
       <c r="D49" s="19" t="inlineStr">
@@ -5032,12 +5088,12 @@
       </c>
       <c r="I49" s="19" t="inlineStr">
         <is>
-          <t>Como secretario quiero pasar lista aunque no haya señal.</t>
+          <t>Como líder quiero recibir el estudio semanal en la app en lugar de WhatsApp.</t>
         </is>
       </c>
       <c r="J49" s="19" t="inlineStr">
         <is>
-          <t>Pasar lista en modo avión; al reconectar se sincroniza sin duplicados.</t>
+          <t>Publicar el material de la semana; el líder lo abre y queda marca de lectura.</t>
         </is>
       </c>
       <c r="K49" s="19" t="inlineStr">
@@ -5056,7 +5112,7 @@
     <row r="50">
       <c r="A50" s="18" t="inlineStr">
         <is>
-          <t>M3-04</t>
+          <t>M3-03</t>
         </is>
       </c>
       <c r="B50" s="19" t="inlineStr">
@@ -5066,12 +5122,12 @@
       </c>
       <c r="C50" s="19" t="inlineStr">
         <is>
-          <t>Ofrendas regulares y especiales. El Tesorero cuenta y avala la cifra con firma electrónica simple (usuario, fecha y hora, monto y reingreso de su PIN). Si su cifra difiere de la capturada, se registra la diferencia.</t>
+          <t>Pase de lista digital por Secretario o Líder, con captura sin conexión y sincronización posterior.</t>
         </is>
       </c>
       <c r="D50" s="19" t="inlineStr">
         <is>
-          <t>v3 + Obs. 4</t>
+          <t>v3</t>
         </is>
       </c>
       <c r="E50" s="19" t="inlineStr">
@@ -5086,7 +5142,7 @@
       </c>
       <c r="G50" s="19" t="inlineStr">
         <is>
-          <t>Sprint 4</t>
+          <t>Sprint 3</t>
         </is>
       </c>
       <c r="H50" s="19" t="inlineStr">
@@ -5096,12 +5152,12 @@
       </c>
       <c r="I50" s="19" t="inlineStr">
         <is>
-          <t>Como tesorero quiero contar y avalar la ofrenda del grupo.</t>
+          <t>Como secretario quiero pasar lista aunque no haya señal.</t>
         </is>
       </c>
       <c r="J50" s="19" t="inlineStr">
         <is>
-          <t>Capturar monto; el Tesorero captura su cifra y confirma con su PIN; si difiere se registra la diferencia; con aval no se edita sin motivo.</t>
+          <t>Pasar lista en modo avión; al reconectar se sincroniza sin duplicados.</t>
         </is>
       </c>
       <c r="K50" s="19" t="inlineStr">
@@ -5120,7 +5176,7 @@
     <row r="51">
       <c r="A51" s="18" t="inlineStr">
         <is>
-          <t>M3-05</t>
+          <t>M3-04</t>
         </is>
       </c>
       <c r="B51" s="19" t="inlineStr">
@@ -5130,12 +5186,12 @@
       </c>
       <c r="C51" s="19" t="inlineStr">
         <is>
-          <t>Formulario dinámico de peticiones de oración, con seguimiento pastoral.</t>
+          <t>Ofrendas regulares y especiales. El Tesorero cuenta y avala la cifra con firma electrónica simple (usuario, fecha y hora, monto y reingreso de su PIN). Si su cifra difiere de la capturada, se registra la diferencia.</t>
         </is>
       </c>
       <c r="D51" s="19" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>v3 + Obs. 4</t>
         </is>
       </c>
       <c r="E51" s="19" t="inlineStr">
@@ -5160,12 +5216,12 @@
       </c>
       <c r="I51" s="19" t="inlineStr">
         <is>
-          <t>Como líder quiero recoger peticiones de oración con un formulario configurable.</t>
+          <t>Como tesorero quiero contar y avalar la ofrenda del grupo.</t>
         </is>
       </c>
       <c r="J51" s="19" t="inlineStr">
         <is>
-          <t>Capturar una petición; el formulario se edita sin código.</t>
+          <t>Capturar monto; el Tesorero captura su cifra y confirma con su PIN; si difiere se registra la diferencia; con aval no se edita sin motivo.</t>
         </is>
       </c>
       <c r="K51" s="19" t="inlineStr">
@@ -5184,7 +5240,7 @@
     <row r="52">
       <c r="A52" s="18" t="inlineStr">
         <is>
-          <t>M3-06</t>
+          <t>M3-05</t>
         </is>
       </c>
       <c r="B52" s="19" t="inlineStr">
@@ -5194,12 +5250,12 @@
       </c>
       <c r="C52" s="19" t="inlineStr">
         <is>
-          <t>Peticiones de oración visibles solo para Líder y roles superiores. Retención de 1 mes o tiempo configurable, con borrado automático.</t>
-        </is>
-      </c>
-      <c r="D52" s="21" t="inlineStr">
-        <is>
-          <t>Resp. P8</t>
+          <t>Formulario dinámico de peticiones de oración, con seguimiento pastoral.</t>
+        </is>
+      </c>
+      <c r="D52" s="19" t="inlineStr">
+        <is>
+          <t>v3</t>
         </is>
       </c>
       <c r="E52" s="19" t="inlineStr">
@@ -5224,12 +5280,12 @@
       </c>
       <c r="I52" s="19" t="inlineStr">
         <is>
-          <t>Como pastor quiero que las peticiones solo las vea el Líder y superiores y se borren al vencer.</t>
+          <t>Como líder quiero recoger peticiones de oración con un formulario configurable.</t>
         </is>
       </c>
       <c r="J52" s="19" t="inlineStr">
         <is>
-          <t>El Secretario no las ve; tras el plazo configurable (por defecto 30 días) se eliminan.</t>
+          <t>Capturar una petición; el formulario se edita sin código.</t>
         </is>
       </c>
       <c r="K52" s="19" t="inlineStr">
@@ -5248,7 +5304,7 @@
     <row r="53">
       <c r="A53" s="18" t="inlineStr">
         <is>
-          <t>M3-07</t>
+          <t>M3-06</t>
         </is>
       </c>
       <c r="B53" s="19" t="inlineStr">
@@ -5258,17 +5314,17 @@
       </c>
       <c r="C53" s="19" t="inlineStr">
         <is>
-          <t>Reportes de supervisión: dashboards de asistencia, ofrendas y crecimiento por grupo, según permisos.</t>
-        </is>
-      </c>
-      <c r="D53" s="19" t="inlineStr">
-        <is>
-          <t>v3</t>
+          <t>Peticiones de oración visibles solo para Líder y roles superiores. Retención de 1 mes o tiempo configurable, con borrado automático.</t>
+        </is>
+      </c>
+      <c r="D53" s="21" t="inlineStr">
+        <is>
+          <t>Resp. P8</t>
         </is>
       </c>
       <c r="E53" s="19" t="inlineStr">
         <is>
-          <t>MVP básico</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="F53" s="19" t="inlineStr">
@@ -5278,7 +5334,7 @@
       </c>
       <c r="G53" s="19" t="inlineStr">
         <is>
-          <t>Sprint 5</t>
+          <t>Sprint 4</t>
         </is>
       </c>
       <c r="H53" s="19" t="inlineStr">
@@ -5288,12 +5344,12 @@
       </c>
       <c r="I53" s="19" t="inlineStr">
         <is>
-          <t>Como supervisor quiero ver la salud de mis grupos.</t>
+          <t>Como pastor quiero que las peticiones solo las vea el Líder y superiores y se borren al vencer.</t>
         </is>
       </c>
       <c r="J53" s="19" t="inlineStr">
         <is>
-          <t>El dashboard muestra asistencia, ofrendas y crecimiento según permisos.</t>
+          <t>El Secretario no las ve; tras el plazo configurable (por defecto 30 días) se eliminan.</t>
         </is>
       </c>
       <c r="K53" s="19" t="inlineStr">
@@ -5312,7 +5368,7 @@
     <row r="54">
       <c r="A54" s="18" t="inlineStr">
         <is>
-          <t>M3-08</t>
+          <t>M3-07</t>
         </is>
       </c>
       <c r="B54" s="19" t="inlineStr">
@@ -5322,7 +5378,7 @@
       </c>
       <c r="C54" s="19" t="inlineStr">
         <is>
-          <t>Ubicación de zona del grupo para que personas cercanas lo encuentren, sin exponer el domicilio exacto. Por definir.</t>
+          <t>Reportes de supervisión: dashboards de asistencia, ofrendas y crecimiento por grupo, según permisos.</t>
         </is>
       </c>
       <c r="D54" s="19" t="inlineStr">
@@ -5332,37 +5388,37 @@
       </c>
       <c r="E54" s="19" t="inlineStr">
         <is>
-          <t>Fuera del MVP</t>
+          <t>MVP básico</t>
         </is>
       </c>
       <c r="F54" s="19" t="inlineStr">
         <is>
-          <t>Fase 4</t>
+          <t>Fase 1</t>
         </is>
       </c>
       <c r="G54" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sprint 5</t>
         </is>
       </c>
       <c r="H54" s="19" t="inlineStr">
         <is>
-          <t>Posterior</t>
-        </is>
-      </c>
-      <c r="I54" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
-        </is>
-      </c>
-      <c r="J54" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
+          <t>H3 · MVP (Grupos)</t>
+        </is>
+      </c>
+      <c r="I54" s="19" t="inlineStr">
+        <is>
+          <t>Como supervisor quiero ver la salud de mis grupos.</t>
+        </is>
+      </c>
+      <c r="J54" s="19" t="inlineStr">
+        <is>
+          <t>El dashboard muestra asistencia, ofrendas y crecimiento según permisos.</t>
         </is>
       </c>
       <c r="K54" s="19" t="inlineStr">
         <is>
-          <t>Por definir</t>
+          <t>VoBo pendiente</t>
         </is>
       </c>
       <c r="L54" s="19" t="inlineStr">
@@ -5376,7 +5432,7 @@
     <row r="55">
       <c r="A55" s="18" t="inlineStr">
         <is>
-          <t>M3-09</t>
+          <t>M3-08</t>
         </is>
       </c>
       <c r="B55" s="19" t="inlineStr">
@@ -5386,47 +5442,47 @@
       </c>
       <c r="C55" s="19" t="inlineStr">
         <is>
-          <t>A un grupo asisten miembros de la iglesia (vecinos o no) e invitados del grupo que no asisten a la iglesia. Los invitados se registran como Contacto con datos mínimos y se les puede invitar a consolidación.</t>
-        </is>
-      </c>
-      <c r="D55" s="21" t="inlineStr">
-        <is>
-          <t>Corrección v3.2</t>
+          <t>Ubicación de zona del grupo para que personas cercanas lo encuentren, sin exponer el domicilio exacto. Por definir.</t>
+        </is>
+      </c>
+      <c r="D55" s="19" t="inlineStr">
+        <is>
+          <t>v3</t>
         </is>
       </c>
       <c r="E55" s="19" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Fuera del MVP</t>
         </is>
       </c>
       <c r="F55" s="19" t="inlineStr">
         <is>
-          <t>Fase 1</t>
+          <t>Fase 4</t>
         </is>
       </c>
       <c r="G55" s="19" t="inlineStr">
         <is>
-          <t>Sprint 3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H55" s="19" t="inlineStr">
         <is>
-          <t>H3 · MVP (Grupos)</t>
-        </is>
-      </c>
-      <c r="I55" s="19" t="inlineStr">
-        <is>
-          <t>Como secretario quiero registrar invitados del grupo con datos mínimos.</t>
-        </is>
-      </c>
-      <c r="J55" s="19" t="inlineStr">
-        <is>
-          <t>Registrar un invitado como Contacto y marcarlo presente.</t>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="I55" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
+        </is>
+      </c>
+      <c r="J55" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
         </is>
       </c>
       <c r="K55" s="19" t="inlineStr">
         <is>
-          <t>VoBo pendiente</t>
+          <t>Por definir</t>
         </is>
       </c>
       <c r="L55" s="19" t="inlineStr">
@@ -5440,7 +5496,7 @@
     <row r="56">
       <c r="A56" s="18" t="inlineStr">
         <is>
-          <t>M3-10</t>
+          <t>M3-09</t>
         </is>
       </c>
       <c r="B56" s="19" t="inlineStr">
@@ -5450,12 +5506,12 @@
       </c>
       <c r="C56" s="19" t="inlineStr">
         <is>
-          <t>Confidencialidad de ofrendas y asistencias: consulta limitada por rol (matriz por definir) y modificación restringida, todo en bitácora.</t>
+          <t>A un grupo asisten miembros de la iglesia (vecinos o no) e invitados del grupo que no asisten a la iglesia. Los invitados se registran como Contacto con datos mínimos y se les puede invitar a consolidación.</t>
         </is>
       </c>
       <c r="D56" s="21" t="inlineStr">
         <is>
-          <t>Obs. 5</t>
+          <t>Corrección v3.2</t>
         </is>
       </c>
       <c r="E56" s="19" t="inlineStr">
@@ -5470,7 +5526,7 @@
       </c>
       <c r="G56" s="19" t="inlineStr">
         <is>
-          <t>Sprint 4</t>
+          <t>Sprint 3</t>
         </is>
       </c>
       <c r="H56" s="19" t="inlineStr">
@@ -5480,17 +5536,17 @@
       </c>
       <c r="I56" s="19" t="inlineStr">
         <is>
-          <t>Como pastor quiero que ofrendas y asistencias sean confidenciales.</t>
+          <t>Como secretario quiero registrar invitados del grupo con datos mínimos.</t>
         </is>
       </c>
       <c r="J56" s="19" t="inlineStr">
         <is>
-          <t>La matriz de la sección 3.3 del v3.2 se cumple en pruebas por cada rol.</t>
+          <t>Registrar un invitado como Contacto y marcarlo presente.</t>
         </is>
       </c>
       <c r="K56" s="19" t="inlineStr">
         <is>
-          <t>Por definir</t>
+          <t>VoBo pendiente</t>
         </is>
       </c>
       <c r="L56" s="19" t="inlineStr">
@@ -5504,7 +5560,7 @@
     <row r="57">
       <c r="A57" s="18" t="inlineStr">
         <is>
-          <t>M3-11</t>
+          <t>M3-10</t>
         </is>
       </c>
       <c r="B57" s="19" t="inlineStr">
@@ -5514,12 +5570,12 @@
       </c>
       <c r="C57" s="19" t="inlineStr">
         <is>
-          <t>Dashboard y tablero de mensajes del grupo.</t>
+          <t>Confidencialidad de ofrendas y asistencias: consulta limitada por rol (matriz por definir) y modificación restringida, todo en bitácora.</t>
         </is>
       </c>
       <c r="D57" s="21" t="inlineStr">
         <is>
-          <t>Obs. 7</t>
+          <t>Obs. 5</t>
         </is>
       </c>
       <c r="E57" s="19" t="inlineStr">
@@ -5534,7 +5590,7 @@
       </c>
       <c r="G57" s="19" t="inlineStr">
         <is>
-          <t>Sprint 5</t>
+          <t>Sprint 4</t>
         </is>
       </c>
       <c r="H57" s="19" t="inlineStr">
@@ -5544,17 +5600,17 @@
       </c>
       <c r="I57" s="19" t="inlineStr">
         <is>
-          <t>Como líder quiero un tablero de mensajes de mi grupo.</t>
+          <t>Como pastor quiero que ofrendas y asistencias sean confidenciales.</t>
         </is>
       </c>
       <c r="J57" s="19" t="inlineStr">
         <is>
-          <t>Publicar y leer mensajes del grupo.</t>
+          <t>La matriz de la sección 3.3 del v3.2 se cumple en pruebas por cada rol.</t>
         </is>
       </c>
       <c r="K57" s="19" t="inlineStr">
         <is>
-          <t>VoBo pendiente</t>
+          <t>Por definir</t>
         </is>
       </c>
       <c r="L57" s="19" t="inlineStr">
@@ -5568,52 +5624,52 @@
     <row r="58">
       <c r="A58" s="18" t="inlineStr">
         <is>
-          <t>M4-01</t>
+          <t>M3-11</t>
         </is>
       </c>
       <c r="B58" s="19" t="inlineStr">
         <is>
-          <t>M4 Kids Check-In/Out</t>
+          <t>M3 Grupos de Conexión</t>
         </is>
       </c>
       <c r="C58" s="19" t="inlineStr">
         <is>
-          <t>Sustitución de la ficha física de papel.</t>
-        </is>
-      </c>
-      <c r="D58" s="19" t="inlineStr">
-        <is>
-          <t>v1 / v2</t>
+          <t>Dashboard y tablero de mensajes del grupo.</t>
+        </is>
+      </c>
+      <c r="D58" s="21" t="inlineStr">
+        <is>
+          <t>Obs. 7</t>
         </is>
       </c>
       <c r="E58" s="19" t="inlineStr">
         <is>
-          <t>Fuera del MVP</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="F58" s="19" t="inlineStr">
         <is>
-          <t>Fase 2</t>
+          <t>Fase 1</t>
         </is>
       </c>
       <c r="G58" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sprint 5</t>
         </is>
       </c>
       <c r="H58" s="19" t="inlineStr">
         <is>
-          <t>Posterior</t>
-        </is>
-      </c>
-      <c r="I58" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
-        </is>
-      </c>
-      <c r="J58" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
+          <t>H3 · MVP (Grupos)</t>
+        </is>
+      </c>
+      <c r="I58" s="19" t="inlineStr">
+        <is>
+          <t>Como líder quiero un tablero de mensajes de mi grupo.</t>
+        </is>
+      </c>
+      <c r="J58" s="19" t="inlineStr">
+        <is>
+          <t>Publicar y leer mensajes del grupo.</t>
         </is>
       </c>
       <c r="K58" s="19" t="inlineStr">
@@ -5632,7 +5688,7 @@
     <row r="59">
       <c r="A59" s="18" t="inlineStr">
         <is>
-          <t>M4-02</t>
+          <t>M4-01</t>
         </is>
       </c>
       <c r="B59" s="19" t="inlineStr">
@@ -5642,12 +5698,12 @@
       </c>
       <c r="C59" s="19" t="inlineStr">
         <is>
-          <t>Registro de ingreso del menor con salón o clase asignada y generación de código único.</t>
-        </is>
-      </c>
-      <c r="D59" s="21" t="inlineStr">
-        <is>
-          <t>v1 + Nuevo v3</t>
+          <t>Sustitución de la ficha física de papel.</t>
+        </is>
+      </c>
+      <c r="D59" s="19" t="inlineStr">
+        <is>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E59" s="19" t="inlineStr">
@@ -5696,7 +5752,7 @@
     <row r="60">
       <c r="A60" s="18" t="inlineStr">
         <is>
-          <t>M4-03</t>
+          <t>M4-02</t>
         </is>
       </c>
       <c r="B60" s="19" t="inlineStr">
@@ -5706,12 +5762,12 @@
       </c>
       <c r="C60" s="19" t="inlineStr">
         <is>
-          <t>Código QR dinámico o OTP temporal en la PWA del padre o tutor.</t>
-        </is>
-      </c>
-      <c r="D60" s="19" t="inlineStr">
-        <is>
-          <t>v2</t>
+          <t>Registro de ingreso del menor con salón o clase asignada y generación de código único.</t>
+        </is>
+      </c>
+      <c r="D60" s="21" t="inlineStr">
+        <is>
+          <t>v1 + Nuevo v3</t>
         </is>
       </c>
       <c r="E60" s="19" t="inlineStr">
@@ -5760,7 +5816,7 @@
     <row r="61">
       <c r="A61" s="18" t="inlineStr">
         <is>
-          <t>M4-04</t>
+          <t>M4-03</t>
         </is>
       </c>
       <c r="B61" s="19" t="inlineStr">
@@ -5770,7 +5826,7 @@
       </c>
       <c r="C61" s="19" t="inlineStr">
         <is>
-          <t>Validación al entregar: el servidor de Kids escanea el código y confirma identidad y fotografía del tutor autorizado en el Expediente Digital.</t>
+          <t>Código QR dinámico o OTP temporal en la PWA del padre o tutor.</t>
         </is>
       </c>
       <c r="D61" s="19" t="inlineStr">
@@ -5824,7 +5880,7 @@
     <row r="62">
       <c r="A62" s="18" t="inlineStr">
         <is>
-          <t>M4-05</t>
+          <t>M4-04</t>
         </is>
       </c>
       <c r="B62" s="19" t="inlineStr">
@@ -5834,12 +5890,12 @@
       </c>
       <c r="C62" s="19" t="inlineStr">
         <is>
-          <t>Alternativa para tutores sin smartphone, sin batería o sin conexión (p. ej. código por SMS o comprobante imprimible con identificación). Por definir.</t>
-        </is>
-      </c>
-      <c r="D62" s="21" t="inlineStr">
-        <is>
-          <t>Nuevo v3</t>
+          <t>Validación al entregar: el servidor de Kids escanea el código y confirma identidad y fotografía del tutor autorizado en el Expediente Digital.</t>
+        </is>
+      </c>
+      <c r="D62" s="19" t="inlineStr">
+        <is>
+          <t>v2</t>
         </is>
       </c>
       <c r="E62" s="19" t="inlineStr">
@@ -5874,7 +5930,7 @@
       </c>
       <c r="K62" s="19" t="inlineStr">
         <is>
-          <t>Por definir</t>
+          <t>VoBo pendiente</t>
         </is>
       </c>
       <c r="L62" s="19" t="inlineStr">
@@ -5888,7 +5944,7 @@
     <row r="63">
       <c r="A63" s="18" t="inlineStr">
         <is>
-          <t>M4-06</t>
+          <t>M4-05</t>
         </is>
       </c>
       <c r="B63" s="19" t="inlineStr">
@@ -5898,7 +5954,7 @@
       </c>
       <c r="C63" s="19" t="inlineStr">
         <is>
-          <t>Autorización temporal de un tercero para recoger al menor, con aprobación del tutor registrado.</t>
+          <t>Alternativa para tutores sin smartphone, sin batería o sin conexión (p. ej. código por SMS o comprobante imprimible con identificación). Por definir.</t>
         </is>
       </c>
       <c r="D63" s="21" t="inlineStr">
@@ -5938,7 +5994,7 @@
       </c>
       <c r="K63" s="19" t="inlineStr">
         <is>
-          <t>VoBo pendiente</t>
+          <t>Por definir</t>
         </is>
       </c>
       <c r="L63" s="19" t="inlineStr">
@@ -5952,7 +6008,7 @@
     <row r="64">
       <c r="A64" s="18" t="inlineStr">
         <is>
-          <t>M4-07</t>
+          <t>M4-06</t>
         </is>
       </c>
       <c r="B64" s="19" t="inlineStr">
@@ -5962,7 +6018,7 @@
       </c>
       <c r="C64" s="19" t="inlineStr">
         <is>
-          <t>Caducidad del código y bitácora de cada entrega (quién recogió, quién entregó, hora).</t>
+          <t>Autorización temporal de un tercero para recoger al menor, con aprobación del tutor registrado.</t>
         </is>
       </c>
       <c r="D64" s="21" t="inlineStr">
@@ -6016,7 +6072,7 @@
     <row r="65">
       <c r="A65" s="18" t="inlineStr">
         <is>
-          <t>M4-08</t>
+          <t>M4-07</t>
         </is>
       </c>
       <c r="B65" s="19" t="inlineStr">
@@ -6026,7 +6082,7 @@
       </c>
       <c r="C65" s="19" t="inlineStr">
         <is>
-          <t>Funcionamiento sin conexión o con conexión degradada para el check-out.</t>
+          <t>Caducidad del código y bitácora de cada entrega (quién recogió, quién entregó, hora).</t>
         </is>
       </c>
       <c r="D65" s="21" t="inlineStr">
@@ -6080,52 +6136,52 @@
     <row r="66">
       <c r="A66" s="18" t="inlineStr">
         <is>
-          <t>M5-01</t>
+          <t>M4-08</t>
         </is>
       </c>
       <c r="B66" s="19" t="inlineStr">
         <is>
-          <t>M5 Áreas y servidores</t>
+          <t>M4 Kids Check-In/Out</t>
         </is>
       </c>
       <c r="C66" s="19" t="inlineStr">
         <is>
-          <t>Catálogo mínimo de áreas y asignación de servidores. Versión reducida del módulo 5, necesaria para permisos por área. Sirve como primer censo.</t>
-        </is>
-      </c>
-      <c r="D66" s="19" t="inlineStr">
-        <is>
-          <t>v3</t>
+          <t>Funcionamiento sin conexión o con conexión degradada para el check-out.</t>
+        </is>
+      </c>
+      <c r="D66" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3</t>
         </is>
       </c>
       <c r="E66" s="19" t="inlineStr">
         <is>
-          <t>MVP mínimo</t>
+          <t>Fuera del MVP</t>
         </is>
       </c>
       <c r="F66" s="19" t="inlineStr">
         <is>
-          <t>Fase 0</t>
+          <t>Fase 2</t>
         </is>
       </c>
       <c r="G66" s="19" t="inlineStr">
         <is>
-          <t>Sprint 1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H66" s="19" t="inlineStr">
         <is>
-          <t>H2 · Fase 0 completa</t>
-        </is>
-      </c>
-      <c r="I66" s="19" t="inlineStr">
-        <is>
-          <t>Como pastor quiero un catálogo de áreas con su personal para conocer la estructura.</t>
-        </is>
-      </c>
-      <c r="J66" s="19" t="inlineStr">
-        <is>
-          <t>Crear un área, asignar servidores y ver el conteo real.</t>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="I66" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
+        </is>
+      </c>
+      <c r="J66" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
         </is>
       </c>
       <c r="K66" s="19" t="inlineStr">
@@ -6144,7 +6200,7 @@
     <row r="67">
       <c r="A67" s="18" t="inlineStr">
         <is>
-          <t>M5-02</t>
+          <t>M5-01</t>
         </is>
       </c>
       <c r="B67" s="19" t="inlineStr">
@@ -6154,42 +6210,42 @@
       </c>
       <c r="C67" s="19" t="inlineStr">
         <is>
-          <t>Roles jerárquicos dentro de cada área (directores, líderes, maestros, servidores).</t>
+          <t>Catálogo mínimo de áreas y asignación de servidores. Versión reducida del módulo 5, necesaria para permisos por área. Sirve como primer censo.</t>
         </is>
       </c>
       <c r="D67" s="19" t="inlineStr">
         <is>
-          <t>v1</t>
+          <t>v3</t>
         </is>
       </c>
       <c r="E67" s="19" t="inlineStr">
         <is>
-          <t>Fuera del MVP</t>
+          <t>MVP mínimo</t>
         </is>
       </c>
       <c r="F67" s="19" t="inlineStr">
         <is>
-          <t>Fase 4</t>
+          <t>Fase 0</t>
         </is>
       </c>
       <c r="G67" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sprint 1</t>
         </is>
       </c>
       <c r="H67" s="19" t="inlineStr">
         <is>
-          <t>Posterior</t>
-        </is>
-      </c>
-      <c r="I67" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
-        </is>
-      </c>
-      <c r="J67" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
+          <t>H2 · Fase 0 completa</t>
+        </is>
+      </c>
+      <c r="I67" s="19" t="inlineStr">
+        <is>
+          <t>Como pastor quiero un catálogo de áreas con su personal para conocer la estructura.</t>
+        </is>
+      </c>
+      <c r="J67" s="19" t="inlineStr">
+        <is>
+          <t>Crear un área, asignar servidores y ver el conteo real.</t>
         </is>
       </c>
       <c r="K67" s="19" t="inlineStr">
@@ -6208,7 +6264,7 @@
     <row r="68">
       <c r="A68" s="18" t="inlineStr">
         <is>
-          <t>M5-03</t>
+          <t>M5-02</t>
         </is>
       </c>
       <c r="B68" s="19" t="inlineStr">
@@ -6218,12 +6274,12 @@
       </c>
       <c r="C68" s="19" t="inlineStr">
         <is>
-          <t>Organigrama y número real de servidores activos, directores y líderes por área.</t>
+          <t>Roles jerárquicos dentro de cada área (directores, líderes, maestros, servidores).</t>
         </is>
       </c>
       <c r="D68" s="19" t="inlineStr">
         <is>
-          <t>v2</t>
+          <t>v1</t>
         </is>
       </c>
       <c r="E68" s="19" t="inlineStr">
@@ -6272,7 +6328,7 @@
     <row r="69">
       <c r="A69" s="18" t="inlineStr">
         <is>
-          <t>M5-04</t>
+          <t>M5-03</t>
         </is>
       </c>
       <c r="B69" s="19" t="inlineStr">
@@ -6282,12 +6338,12 @@
       </c>
       <c r="C69" s="19" t="inlineStr">
         <is>
-          <t>Control de asistencia a turnos o servicios.</t>
+          <t>Organigrama y número real de servidores activos, directores y líderes por área.</t>
         </is>
       </c>
       <c r="D69" s="19" t="inlineStr">
         <is>
-          <t>v1 / v2</t>
+          <t>v2</t>
         </is>
       </c>
       <c r="E69" s="19" t="inlineStr">
@@ -6336,7 +6392,7 @@
     <row r="70">
       <c r="A70" s="18" t="inlineStr">
         <is>
-          <t>M5-05</t>
+          <t>M5-04</t>
         </is>
       </c>
       <c r="B70" s="19" t="inlineStr">
@@ -6346,7 +6402,7 @@
       </c>
       <c r="C70" s="19" t="inlineStr">
         <is>
-          <t>Tablero de avisos y notificaciones interno por área.</t>
+          <t>Control de asistencia a turnos o servicios.</t>
         </is>
       </c>
       <c r="D70" s="19" t="inlineStr">
@@ -6400,7 +6456,7 @@
     <row r="71">
       <c r="A71" s="18" t="inlineStr">
         <is>
-          <t>M5-06</t>
+          <t>M5-05</t>
         </is>
       </c>
       <c r="B71" s="19" t="inlineStr">
@@ -6410,7 +6466,7 @@
       </c>
       <c r="C71" s="19" t="inlineStr">
         <is>
-          <t>Gestión financiera por área: caja chica y gastos operativos.</t>
+          <t>Tablero de avisos y notificaciones interno por área.</t>
         </is>
       </c>
       <c r="D71" s="19" t="inlineStr">
@@ -6464,22 +6520,22 @@
     <row r="72">
       <c r="A72" s="18" t="inlineStr">
         <is>
-          <t>M6-01</t>
+          <t>M5-06</t>
         </is>
       </c>
       <c r="B72" s="19" t="inlineStr">
         <is>
-          <t>M6 Ministerios de servicio</t>
+          <t>M5 Áreas y servidores</t>
         </is>
       </c>
       <c r="C72" s="19" t="inlineStr">
         <is>
-          <t>Control de personal propio de cada ministerio.</t>
-        </is>
-      </c>
-      <c r="D72" s="22" t="inlineStr">
-        <is>
-          <t>Recuperado v1</t>
+          <t>Gestión financiera por área: caja chica y gastos operativos.</t>
+        </is>
+      </c>
+      <c r="D72" s="19" t="inlineStr">
+        <is>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E72" s="19" t="inlineStr">
@@ -6528,7 +6584,7 @@
     <row r="73">
       <c r="A73" s="18" t="inlineStr">
         <is>
-          <t>M6-02</t>
+          <t>M6-01</t>
         </is>
       </c>
       <c r="B73" s="19" t="inlineStr">
@@ -6538,12 +6594,12 @@
       </c>
       <c r="C73" s="19" t="inlineStr">
         <is>
-          <t>Menú o catálogo digital interactivo (público o interno), autogestionado.</t>
-        </is>
-      </c>
-      <c r="D73" s="19" t="inlineStr">
-        <is>
-          <t>v1 / v2</t>
+          <t>Control de personal propio de cada ministerio.</t>
+        </is>
+      </c>
+      <c r="D73" s="22" t="inlineStr">
+        <is>
+          <t>Recuperado v1</t>
         </is>
       </c>
       <c r="E73" s="19" t="inlineStr">
@@ -6592,7 +6648,7 @@
     <row r="74">
       <c r="A74" s="18" t="inlineStr">
         <is>
-          <t>M6-03</t>
+          <t>M6-02</t>
         </is>
       </c>
       <c r="B74" s="19" t="inlineStr">
@@ -6602,7 +6658,7 @@
       </c>
       <c r="C74" s="19" t="inlineStr">
         <is>
-          <t>Calendario de turnos: días regulares de servicio y eventos especiales.</t>
+          <t>Menú o catálogo digital interactivo (público o interno), autogestionado.</t>
         </is>
       </c>
       <c r="D74" s="19" t="inlineStr">
@@ -6656,7 +6712,7 @@
     <row r="75">
       <c r="A75" s="18" t="inlineStr">
         <is>
-          <t>M6-04</t>
+          <t>M6-03</t>
         </is>
       </c>
       <c r="B75" s="19" t="inlineStr">
@@ -6666,7 +6722,7 @@
       </c>
       <c r="C75" s="19" t="inlineStr">
         <is>
-          <t>Registro de asistentes o personas atendidas.</t>
+          <t>Calendario de turnos: días regulares de servicio y eventos especiales.</t>
         </is>
       </c>
       <c r="D75" s="19" t="inlineStr">
@@ -6720,7 +6776,7 @@
     <row r="76">
       <c r="A76" s="18" t="inlineStr">
         <is>
-          <t>M6-05</t>
+          <t>M6-04</t>
         </is>
       </c>
       <c r="B76" s="19" t="inlineStr">
@@ -6730,7 +6786,7 @@
       </c>
       <c r="C76" s="19" t="inlineStr">
         <is>
-          <t>Control de gastos y de inventario básico.</t>
+          <t>Registro de asistentes o personas atendidas.</t>
         </is>
       </c>
       <c r="D76" s="19" t="inlineStr">
@@ -6784,7 +6840,7 @@
     <row r="77">
       <c r="A77" s="18" t="inlineStr">
         <is>
-          <t>M6-06</t>
+          <t>M6-05</t>
         </is>
       </c>
       <c r="B77" s="19" t="inlineStr">
@@ -6794,7 +6850,7 @@
       </c>
       <c r="C77" s="19" t="inlineStr">
         <is>
-          <t>Canal de comunicación directo con el área de Administración General.</t>
+          <t>Control de gastos y de inventario básico.</t>
         </is>
       </c>
       <c r="D77" s="19" t="inlineStr">
@@ -6848,7 +6904,7 @@
     <row r="78">
       <c r="A78" s="18" t="inlineStr">
         <is>
-          <t>M6-07</t>
+          <t>M6-06</t>
         </is>
       </c>
       <c r="B78" s="19" t="inlineStr">
@@ -6858,12 +6914,12 @@
       </c>
       <c r="C78" s="19" t="inlineStr">
         <is>
-          <t>Servicio Médico: los datos de salud de las personas atendidas requieren tratamiento de datos sensibles. Por definir alcance.</t>
-        </is>
-      </c>
-      <c r="D78" s="21" t="inlineStr">
-        <is>
-          <t>Nuevo v3</t>
+          <t>Canal de comunicación directo con el área de Administración General.</t>
+        </is>
+      </c>
+      <c r="D78" s="19" t="inlineStr">
+        <is>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E78" s="19" t="inlineStr">
@@ -6898,7 +6954,7 @@
       </c>
       <c r="K78" s="19" t="inlineStr">
         <is>
-          <t>Por definir</t>
+          <t>VoBo pendiente</t>
         </is>
       </c>
       <c r="L78" s="19" t="inlineStr">
@@ -6912,22 +6968,22 @@
     <row r="79">
       <c r="A79" s="18" t="inlineStr">
         <is>
-          <t>M7-01</t>
+          <t>M6-07</t>
         </is>
       </c>
       <c r="B79" s="19" t="inlineStr">
         <is>
-          <t>M7 Eventos y aforo</t>
+          <t>M6 Ministerios de servicio</t>
         </is>
       </c>
       <c r="C79" s="19" t="inlineStr">
         <is>
-          <t>Eventos abiertos o evangelísticos con formulario de inscripción rápida, sin requerir historial previo.</t>
-        </is>
-      </c>
-      <c r="D79" s="19" t="inlineStr">
-        <is>
-          <t>v1 / v2</t>
+          <t>Servicio Médico: los datos de salud de las personas atendidas requieren tratamiento de datos sensibles. Por definir alcance.</t>
+        </is>
+      </c>
+      <c r="D79" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3</t>
         </is>
       </c>
       <c r="E79" s="19" t="inlineStr">
@@ -6962,7 +7018,7 @@
       </c>
       <c r="K79" s="19" t="inlineStr">
         <is>
-          <t>VoBo pendiente</t>
+          <t>Por definir</t>
         </is>
       </c>
       <c r="L79" s="19" t="inlineStr">
@@ -6976,7 +7032,7 @@
     <row r="80">
       <c r="A80" s="18" t="inlineStr">
         <is>
-          <t>M7-02</t>
+          <t>M7-01</t>
         </is>
       </c>
       <c r="B80" s="19" t="inlineStr">
@@ -6986,12 +7042,12 @@
       </c>
       <c r="C80" s="19" t="inlineStr">
         <is>
-          <t>Consolidación (inducción de personas que asisten por primera vez) como tipo de evento.</t>
-        </is>
-      </c>
-      <c r="D80" s="22" t="inlineStr">
-        <is>
-          <t>Recuperado v1</t>
+          <t>Eventos abiertos o evangelísticos con formulario de inscripción rápida, sin requerir historial previo.</t>
+        </is>
+      </c>
+      <c r="D80" s="19" t="inlineStr">
+        <is>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E80" s="19" t="inlineStr">
@@ -7040,7 +7096,7 @@
     <row r="81">
       <c r="A81" s="18" t="inlineStr">
         <is>
-          <t>M7-03</t>
+          <t>M7-02</t>
         </is>
       </c>
       <c r="B81" s="19" t="inlineStr">
@@ -7050,7 +7106,7 @@
       </c>
       <c r="C81" s="19" t="inlineStr">
         <is>
-          <t>Encargados de evento (personal de la iglesia únicamente; no se controla personal externo).</t>
+          <t>Consolidación (inducción de personas que asisten por primera vez) como tipo de evento.</t>
         </is>
       </c>
       <c r="D81" s="22" t="inlineStr">
@@ -7104,7 +7160,7 @@
     <row r="82">
       <c r="A82" s="18" t="inlineStr">
         <is>
-          <t>M7-04</t>
+          <t>M7-03</t>
         </is>
       </c>
       <c r="B82" s="19" t="inlineStr">
@@ -7114,12 +7170,12 @@
       </c>
       <c r="C82" s="19" t="inlineStr">
         <is>
-          <t>Control de cupo en tiempo real que bloquea el sobrecupo en eventos con aforo limitado (ej. 30 o 50 lugares).</t>
-        </is>
-      </c>
-      <c r="D82" s="19" t="inlineStr">
-        <is>
-          <t>v1 / v2</t>
+          <t>Encargados de evento (personal de la iglesia únicamente; no se controla personal externo).</t>
+        </is>
+      </c>
+      <c r="D82" s="22" t="inlineStr">
+        <is>
+          <t>Recuperado v1</t>
         </is>
       </c>
       <c r="E82" s="19" t="inlineStr">
@@ -7168,7 +7224,7 @@
     <row r="83">
       <c r="A83" s="18" t="inlineStr">
         <is>
-          <t>M7-05</t>
+          <t>M7-04</t>
         </is>
       </c>
       <c r="B83" s="19" t="inlineStr">
@@ -7178,12 +7234,12 @@
       </c>
       <c r="C83" s="19" t="inlineStr">
         <is>
-          <t>Control de asistentes sin lista previa, para aforo y para dar a conocer la iglesia.</t>
+          <t>Control de cupo en tiempo real que bloquea el sobrecupo en eventos con aforo limitado (ej. 30 o 50 lugares).</t>
         </is>
       </c>
       <c r="D83" s="19" t="inlineStr">
         <is>
-          <t>v1</t>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E83" s="19" t="inlineStr">
@@ -7232,7 +7288,7 @@
     <row r="84">
       <c r="A84" s="18" t="inlineStr">
         <is>
-          <t>M7-06</t>
+          <t>M7-05</t>
         </is>
       </c>
       <c r="B84" s="19" t="inlineStr">
@@ -7242,12 +7298,12 @@
       </c>
       <c r="C84" s="19" t="inlineStr">
         <is>
-          <t>Seguimiento de personas nuevas: conversión de un invitado a Expediente Digital y canalización a un curso o Grupo de Conexión.</t>
-        </is>
-      </c>
-      <c r="D84" s="21" t="inlineStr">
-        <is>
-          <t>Nuevo v3</t>
+          <t>Control de asistentes sin lista previa, para aforo y para dar a conocer la iglesia.</t>
+        </is>
+      </c>
+      <c r="D84" s="19" t="inlineStr">
+        <is>
+          <t>v1</t>
         </is>
       </c>
       <c r="E84" s="19" t="inlineStr">
@@ -7296,52 +7352,52 @@
     <row r="85">
       <c r="A85" s="18" t="inlineStr">
         <is>
-          <t>NF-01</t>
+          <t>M7-06</t>
         </is>
       </c>
       <c r="B85" s="19" t="inlineStr">
         <is>
-          <t>No funcionales</t>
+          <t>M7 Eventos y aforo</t>
         </is>
       </c>
       <c r="C85" s="19" t="inlineStr">
         <is>
-          <t>Cumplimiento de la LFPDPPP: aviso de privacidad, consentimiento y derechos ARCO.</t>
-        </is>
-      </c>
-      <c r="D85" s="19" t="inlineStr">
-        <is>
-          <t>v3</t>
+          <t>Seguimiento de personas nuevas: conversión de un invitado a Expediente Digital y canalización a un curso o Grupo de Conexión.</t>
+        </is>
+      </c>
+      <c r="D85" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3</t>
         </is>
       </c>
       <c r="E85" s="19" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Fuera del MVP</t>
         </is>
       </c>
       <c r="F85" s="19" t="inlineStr">
         <is>
-          <t>Fase 0</t>
+          <t>Fase 4</t>
         </is>
       </c>
       <c r="G85" s="19" t="inlineStr">
         <is>
-          <t>Sprint 1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H85" s="19" t="inlineStr">
         <is>
-          <t>H1 · 18-oct (núcleo Fase 0)</t>
-        </is>
-      </c>
-      <c r="I85" s="19" t="inlineStr">
-        <is>
-          <t>Como iglesia queremos cumplir con la LFPDPPP.</t>
-        </is>
-      </c>
-      <c r="J85" s="19" t="inlineStr">
-        <is>
-          <t>Aviso de privacidad, consentimiento y atención de derechos ARCO disponibles.</t>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="I85" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
+        </is>
+      </c>
+      <c r="J85" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
         </is>
       </c>
       <c r="K85" s="19" t="inlineStr">
@@ -7360,7 +7416,7 @@
     <row r="86">
       <c r="A86" s="18" t="inlineStr">
         <is>
-          <t>NF-02</t>
+          <t>NF-01</t>
         </is>
       </c>
       <c r="B86" s="19" t="inlineStr">
@@ -7370,7 +7426,7 @@
       </c>
       <c r="C86" s="19" t="inlineStr">
         <is>
-          <t>Cifrado en tránsito y en reposo. Cifrado adicional a nivel de campo para peticiones de oración.</t>
+          <t>Cumplimiento de la LFPDPPP: aviso de privacidad, consentimiento y derechos ARCO.</t>
         </is>
       </c>
       <c r="D86" s="19" t="inlineStr">
@@ -7390,7 +7446,7 @@
       </c>
       <c r="G86" s="19" t="inlineStr">
         <is>
-          <t>Sprint 0</t>
+          <t>Sprint 1</t>
         </is>
       </c>
       <c r="H86" s="19" t="inlineStr">
@@ -7400,12 +7456,12 @@
       </c>
       <c r="I86" s="19" t="inlineStr">
         <is>
-          <t>Como iglesia queremos proteger los datos sensibles.</t>
+          <t>Como iglesia queremos cumplir con la LFPDPPP.</t>
         </is>
       </c>
       <c r="J86" s="19" t="inlineStr">
         <is>
-          <t>HTTPS obligatorio y peticiones de oración ilegibles directamente en la base.</t>
+          <t>Aviso de privacidad, consentimiento y atención de derechos ARCO disponibles.</t>
         </is>
       </c>
       <c r="K86" s="19" t="inlineStr">
@@ -7424,7 +7480,7 @@
     <row r="87">
       <c r="A87" s="18" t="inlineStr">
         <is>
-          <t>NF-03</t>
+          <t>NF-02</t>
         </is>
       </c>
       <c r="B87" s="19" t="inlineStr">
@@ -7434,7 +7490,7 @@
       </c>
       <c r="C87" s="19" t="inlineStr">
         <is>
-          <t>Bitácora de auditoría de solo-añadir: quién consultó o modificó expedientes, ofrendas y asistencias.</t>
+          <t>Cifrado en tránsito y en reposo. Cifrado adicional a nivel de campo para peticiones de oración.</t>
         </is>
       </c>
       <c r="D87" s="19" t="inlineStr">
@@ -7454,7 +7510,7 @@
       </c>
       <c r="G87" s="19" t="inlineStr">
         <is>
-          <t>Sprint 1</t>
+          <t>Sprint 0</t>
         </is>
       </c>
       <c r="H87" s="19" t="inlineStr">
@@ -7464,12 +7520,12 @@
       </c>
       <c r="I87" s="19" t="inlineStr">
         <is>
-          <t>Como pastor quiero una bitácora que nadie pueda alterar.</t>
+          <t>Como iglesia queremos proteger los datos sensibles.</t>
         </is>
       </c>
       <c r="J87" s="19" t="inlineStr">
         <is>
-          <t>El usuario de la aplicación no puede actualizar ni borrar registros de bitácora.</t>
+          <t>HTTPS obligatorio y peticiones de oración ilegibles directamente en la base.</t>
         </is>
       </c>
       <c r="K87" s="19" t="inlineStr">
@@ -7479,24 +7535,16 @@
       </c>
       <c r="L87" s="19" t="inlineStr">
         <is>
-          <t>En desarrollo</t>
-        </is>
-      </c>
-      <c r="M87" s="19" t="inlineStr">
-        <is>
-          <t>Rama feature/m1-17-acceso · bitácora de solo-añadir a nivel de aplicación</t>
-        </is>
-      </c>
-      <c r="N87" s="19" t="inlineStr">
-        <is>
-          <t>2026-10-05 · Falta reforzarla en la base de datos (permisos) en el Sprint 1.</t>
-        </is>
-      </c>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M87" s="19" t="inlineStr"/>
+      <c r="N87" s="19" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="18" t="inlineStr">
         <is>
-          <t>NF-04</t>
+          <t>NF-03</t>
         </is>
       </c>
       <c r="B88" s="19" t="inlineStr">
@@ -7506,7 +7554,7 @@
       </c>
       <c r="C88" s="19" t="inlineStr">
         <is>
-          <t>Respaldos automáticos diarios cifrados y prueba periódica de restauración.</t>
+          <t>Bitácora de auditoría de solo-añadir: quién consultó o modificó expedientes, ofrendas y asistencias.</t>
         </is>
       </c>
       <c r="D88" s="19" t="inlineStr">
@@ -7526,7 +7574,7 @@
       </c>
       <c r="G88" s="19" t="inlineStr">
         <is>
-          <t>Sprint 0</t>
+          <t>Sprint 1</t>
         </is>
       </c>
       <c r="H88" s="19" t="inlineStr">
@@ -7536,12 +7584,12 @@
       </c>
       <c r="I88" s="19" t="inlineStr">
         <is>
-          <t>Como iglesia queremos no perder información.</t>
+          <t>Como pastor quiero una bitácora que nadie pueda alterar.</t>
         </is>
       </c>
       <c r="J88" s="19" t="inlineStr">
         <is>
-          <t>Respaldo diario cifrado y restauración probada en un ambiente de pruebas.</t>
+          <t>El usuario de la aplicación no puede actualizar ni borrar registros de bitácora.</t>
         </is>
       </c>
       <c r="K88" s="19" t="inlineStr">
@@ -7551,16 +7599,24 @@
       </c>
       <c r="L88" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M88" s="19" t="inlineStr"/>
-      <c r="N88" s="19" t="inlineStr"/>
+          <t>En desarrollo</t>
+        </is>
+      </c>
+      <c r="M88" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/m1-17-acceso · bitácora de solo-añadir a nivel de aplicación</t>
+        </is>
+      </c>
+      <c r="N88" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-05 · Falta reforzarla en la base de datos (permisos) en el Sprint 1.</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="18" t="inlineStr">
         <is>
-          <t>NF-05</t>
+          <t>NF-04</t>
         </is>
       </c>
       <c r="B89" s="19" t="inlineStr">
@@ -7570,47 +7626,47 @@
       </c>
       <c r="C89" s="19" t="inlineStr">
         <is>
-          <t>Disponibilidad esperada en horarios de servicio (fines de semana y reuniones de grupo). Por definir meta.</t>
-        </is>
-      </c>
-      <c r="D89" s="21" t="inlineStr">
-        <is>
-          <t>Nuevo v3</t>
+          <t>Respaldos automáticos diarios cifrados y prueba periódica de restauración.</t>
+        </is>
+      </c>
+      <c r="D89" s="19" t="inlineStr">
+        <is>
+          <t>v3</t>
         </is>
       </c>
       <c r="E89" s="19" t="inlineStr">
         <is>
-          <t>Fuera del MVP</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="F89" s="19" t="inlineStr">
         <is>
-          <t>Transversal</t>
+          <t>Fase 0</t>
         </is>
       </c>
       <c r="G89" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sprint 0</t>
         </is>
       </c>
       <c r="H89" s="19" t="inlineStr">
         <is>
-          <t>Posterior</t>
-        </is>
-      </c>
-      <c r="I89" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
-        </is>
-      </c>
-      <c r="J89" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
+          <t>H1 · 18-oct (núcleo Fase 0)</t>
+        </is>
+      </c>
+      <c r="I89" s="19" t="inlineStr">
+        <is>
+          <t>Como iglesia queremos no perder información.</t>
+        </is>
+      </c>
+      <c r="J89" s="19" t="inlineStr">
+        <is>
+          <t>Respaldo diario cifrado y restauración probada en un ambiente de pruebas.</t>
         </is>
       </c>
       <c r="K89" s="19" t="inlineStr">
         <is>
-          <t>Por definir</t>
+          <t>VoBo pendiente</t>
         </is>
       </c>
       <c r="L89" s="19" t="inlineStr">
@@ -7624,7 +7680,7 @@
     <row r="90">
       <c r="A90" s="18" t="inlineStr">
         <is>
-          <t>NF-06</t>
+          <t>NF-05</t>
         </is>
       </c>
       <c r="B90" s="19" t="inlineStr">
@@ -7634,47 +7690,47 @@
       </c>
       <c r="C90" s="19" t="inlineStr">
         <is>
-          <t>Pase de lista sin conexión con sincronización posterior (reuniones en domicilios con mala señal).</t>
-        </is>
-      </c>
-      <c r="D90" s="19" t="inlineStr">
-        <is>
-          <t>v3</t>
+          <t>Disponibilidad esperada en horarios de servicio (fines de semana y reuniones de grupo). Por definir meta.</t>
+        </is>
+      </c>
+      <c r="D90" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3</t>
         </is>
       </c>
       <c r="E90" s="19" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Fuera del MVP</t>
         </is>
       </c>
       <c r="F90" s="19" t="inlineStr">
         <is>
-          <t>Fase 0</t>
+          <t>Transversal</t>
         </is>
       </c>
       <c r="G90" s="19" t="inlineStr">
         <is>
-          <t>Sprint 3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H90" s="19" t="inlineStr">
         <is>
-          <t>H3 · MVP (Grupos)</t>
-        </is>
-      </c>
-      <c r="I90" s="19" t="inlineStr">
-        <is>
-          <t>Como secretario quiero que el pase de lista funcione sin señal.</t>
-        </is>
-      </c>
-      <c r="J90" s="19" t="inlineStr">
-        <is>
-          <t>Prueba en modo avión y sincronización al reconectar.</t>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="I90" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
+        </is>
+      </c>
+      <c r="J90" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
         </is>
       </c>
       <c r="K90" s="19" t="inlineStr">
         <is>
-          <t>VoBo pendiente</t>
+          <t>Por definir</t>
         </is>
       </c>
       <c r="L90" s="19" t="inlineStr">
@@ -7688,7 +7744,7 @@
     <row r="91">
       <c r="A91" s="18" t="inlineStr">
         <is>
-          <t>NF-07</t>
+          <t>NF-06</t>
         </is>
       </c>
       <c r="B91" s="19" t="inlineStr">
@@ -7698,7 +7754,7 @@
       </c>
       <c r="C91" s="19" t="inlineStr">
         <is>
-          <t>Funciona en Android, iOS y escritorio. En iOS, las notificaciones push requieren instalar la PWA; el respaldo por WhatsApp cubre el resto.</t>
+          <t>Pase de lista sin conexión con sincronización posterior (reuniones en domicilios con mala señal).</t>
         </is>
       </c>
       <c r="D91" s="19" t="inlineStr">
@@ -7718,22 +7774,22 @@
       </c>
       <c r="G91" s="19" t="inlineStr">
         <is>
-          <t>Sprint 0</t>
+          <t>Sprint 3</t>
         </is>
       </c>
       <c r="H91" s="19" t="inlineStr">
         <is>
-          <t>H1 · 18-oct (núcleo Fase 0)</t>
+          <t>H3 · MVP (Grupos)</t>
         </is>
       </c>
       <c r="I91" s="19" t="inlineStr">
         <is>
-          <t>Como usuario quiero usar el sistema en mi dispositivo.</t>
+          <t>Como secretario quiero que el pase de lista funcione sin señal.</t>
         </is>
       </c>
       <c r="J91" s="19" t="inlineStr">
         <is>
-          <t>Pruebas en Android, iOS y escritorio; push en iOS con la PWA instalada y respaldo por WhatsApp.</t>
+          <t>Prueba en modo avión y sincronización al reconectar.</t>
         </is>
       </c>
       <c r="K91" s="19" t="inlineStr">
@@ -7752,7 +7808,7 @@
     <row r="92">
       <c r="A92" s="18" t="inlineStr">
         <is>
-          <t>NF-08</t>
+          <t>NF-07</t>
         </is>
       </c>
       <c r="B92" s="19" t="inlineStr">
@@ -7762,12 +7818,12 @@
       </c>
       <c r="C92" s="19" t="inlineStr">
         <is>
-          <t>Dimensionamiento para ~1,000 personas, con picos los fines de semana, y margen de crecimiento.</t>
-        </is>
-      </c>
-      <c r="D92" s="21" t="inlineStr">
-        <is>
-          <t>Resp. P8</t>
+          <t>Funciona en Android, iOS y escritorio. En iOS, las notificaciones push requieren instalar la PWA; el respaldo por WhatsApp cubre el resto.</t>
+        </is>
+      </c>
+      <c r="D92" s="19" t="inlineStr">
+        <is>
+          <t>v3</t>
         </is>
       </c>
       <c r="E92" s="19" t="inlineStr">
@@ -7792,12 +7848,12 @@
       </c>
       <c r="I92" s="19" t="inlineStr">
         <is>
-          <t>Como iglesia queremos que el sistema soporte a ~1,000 personas.</t>
+          <t>Como usuario quiero usar el sistema en mi dispositivo.</t>
         </is>
       </c>
       <c r="J92" s="19" t="inlineStr">
         <is>
-          <t>Prueba de carga con volumen representativo (por definir) sin degradación.</t>
+          <t>Pruebas en Android, iOS y escritorio; push en iOS con la PWA instalada y respaldo por WhatsApp.</t>
         </is>
       </c>
       <c r="K92" s="19" t="inlineStr">
@@ -7816,7 +7872,7 @@
     <row r="93">
       <c r="A93" s="18" t="inlineStr">
         <is>
-          <t>NF-09</t>
+          <t>NF-08</t>
         </is>
       </c>
       <c r="B93" s="19" t="inlineStr">
@@ -7826,42 +7882,42 @@
       </c>
       <c r="C93" s="19" t="inlineStr">
         <is>
-          <t>Reportes transversales: asistencia, finanzas, crecimiento de la iglesia, exportables a Excel y PDF.</t>
+          <t>Dimensionamiento para ~1,000 personas, con picos los fines de semana, y margen de crecimiento.</t>
         </is>
       </c>
       <c r="D93" s="21" t="inlineStr">
         <is>
-          <t>Nuevo v3</t>
+          <t>Resp. P8</t>
         </is>
       </c>
       <c r="E93" s="19" t="inlineStr">
         <is>
-          <t>Fuera del MVP</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="F93" s="19" t="inlineStr">
         <is>
-          <t>Transversal</t>
+          <t>Fase 0</t>
         </is>
       </c>
       <c r="G93" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sprint 0</t>
         </is>
       </c>
       <c r="H93" s="19" t="inlineStr">
         <is>
-          <t>Posterior</t>
-        </is>
-      </c>
-      <c r="I93" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
-        </is>
-      </c>
-      <c r="J93" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
+          <t>H1 · 18-oct (núcleo Fase 0)</t>
+        </is>
+      </c>
+      <c r="I93" s="19" t="inlineStr">
+        <is>
+          <t>Como iglesia queremos que el sistema soporte a ~1,000 personas.</t>
+        </is>
+      </c>
+      <c r="J93" s="19" t="inlineStr">
+        <is>
+          <t>Prueba de carga con volumen representativo (por definir) sin degradación.</t>
         </is>
       </c>
       <c r="K93" s="19" t="inlineStr">
@@ -7880,7 +7936,7 @@
     <row r="94">
       <c r="A94" s="18" t="inlineStr">
         <is>
-          <t>NF-10</t>
+          <t>NF-09</t>
         </is>
       </c>
       <c r="B94" s="19" t="inlineStr">
@@ -7890,42 +7946,42 @@
       </c>
       <c r="C94" s="19" t="inlineStr">
         <is>
-          <t>Usabilidad para personas mayores: tipografía grande, alto contraste, flujos cortos (ver sección 5).</t>
-        </is>
-      </c>
-      <c r="D94" s="19" t="inlineStr">
-        <is>
-          <t>v3 + Obs. 1</t>
+          <t>Reportes transversales: asistencia, finanzas, crecimiento de la iglesia, exportables a Excel y PDF.</t>
+        </is>
+      </c>
+      <c r="D94" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3</t>
         </is>
       </c>
       <c r="E94" s="19" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Fuera del MVP</t>
         </is>
       </c>
       <c r="F94" s="19" t="inlineStr">
         <is>
-          <t>Fase 0</t>
+          <t>Transversal</t>
         </is>
       </c>
       <c r="G94" s="19" t="inlineStr">
         <is>
-          <t>Sprint 0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H94" s="19" t="inlineStr">
         <is>
-          <t>H1 · 18-oct (núcleo Fase 0)</t>
-        </is>
-      </c>
-      <c r="I94" s="19" t="inlineStr">
-        <is>
-          <t>Como persona mayor quiero una interfaz fácil de leer y usar.</t>
-        </is>
-      </c>
-      <c r="J94" s="19" t="inlineStr">
-        <is>
-          <t>Texto base 18 px, botones de al menos 48 px, contraste AA; prueba con usuarios mayores.</t>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="I94" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
+        </is>
+      </c>
+      <c r="J94" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
         </is>
       </c>
       <c r="K94" s="19" t="inlineStr">
@@ -7941,9 +7997,73 @@
       <c r="M94" s="19" t="inlineStr"/>
       <c r="N94" s="19" t="inlineStr"/>
     </row>
+    <row r="95">
+      <c r="A95" s="18" t="inlineStr">
+        <is>
+          <t>NF-10</t>
+        </is>
+      </c>
+      <c r="B95" s="19" t="inlineStr">
+        <is>
+          <t>No funcionales</t>
+        </is>
+      </c>
+      <c r="C95" s="19" t="inlineStr">
+        <is>
+          <t>Usabilidad para personas mayores: tipografía grande, alto contraste, flujos cortos (ver sección 5).</t>
+        </is>
+      </c>
+      <c r="D95" s="19" t="inlineStr">
+        <is>
+          <t>v3 + Obs. 1</t>
+        </is>
+      </c>
+      <c r="E95" s="19" t="inlineStr">
+        <is>
+          <t>MVP</t>
+        </is>
+      </c>
+      <c r="F95" s="19" t="inlineStr">
+        <is>
+          <t>Fase 0</t>
+        </is>
+      </c>
+      <c r="G95" s="19" t="inlineStr">
+        <is>
+          <t>Sprint 0</t>
+        </is>
+      </c>
+      <c r="H95" s="19" t="inlineStr">
+        <is>
+          <t>H1 · 18-oct (núcleo Fase 0)</t>
+        </is>
+      </c>
+      <c r="I95" s="19" t="inlineStr">
+        <is>
+          <t>Como persona mayor quiero una interfaz fácil de leer y usar.</t>
+        </is>
+      </c>
+      <c r="J95" s="19" t="inlineStr">
+        <is>
+          <t>Texto base 18 px, botones de al menos 48 px, contraste AA; prueba con usuarios mayores.</t>
+        </is>
+      </c>
+      <c r="K95" s="19" t="inlineStr">
+        <is>
+          <t>VoBo pendiente</t>
+        </is>
+      </c>
+      <c r="L95" s="19" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M95" s="19" t="inlineStr"/>
+      <c r="N95" s="19" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N94"/>
-  <conditionalFormatting sqref="L2:L94">
+  <autoFilter ref="A1:N95"/>
+  <conditionalFormatting sqref="L2:L95">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$L2="Hecho"</formula>
     </cfRule>
@@ -7960,7 +8080,7 @@
       <formula>$L2="Bloqueado"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K2:K94">
+  <conditionalFormatting sqref="K2:K95">
     <cfRule type="expression" priority="6" dxfId="0">
       <formula>$K2="Aprobado"</formula>
     </cfRule>
@@ -7968,16 +8088,16 @@
       <formula>$K2="Por definir"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H2:H94">
+  <conditionalFormatting sqref="H2:H95">
     <cfRule type="expression" priority="8" dxfId="5">
       <formula>LEFT($H2,2)="H1"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="L2:L94" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="L2:L95" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Pendiente,En diseño,En desarrollo,En pruebas,Hecho,Bloqueado"</formula1>
     </dataValidation>
-    <dataValidation sqref="K2:K94" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="K2:K95" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"VoBo pendiente,Aprobado,Por definir,Rechazado"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
M1-07: roles y permisos (RBAC) según la matriz de confidencialidad
- Catálogo de 9 roles con permisos configurables y asignación por usuario
- Permisos exigidos en personas, invitaciones y reinicios; nadie otorga un rol más alto que el suyo
- Roles sensibles exigen contraseña fuerte; cambios de roles en bitácora
- El administrador técnico no accede a expedientes (matriz); createsuperuser le asigna ese rol
- Pantalla Roles, navegación por permisos y comando asignar_rol
- Matriz de trazabilidad actualizada

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/trazabilidad/Matriz de Trazabilidad MDF.xlsx
+++ b/docs/trazabilidad/Matriz de Trazabilidad MDF.xlsx
@@ -2919,11 +2919,19 @@
       </c>
       <c r="L16" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M16" s="19" t="inlineStr"/>
-      <c r="N16" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M16" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/m1-07-roles · 67 pruebas de backend y 6 de frontend pasan</t>
+        </is>
+      </c>
+      <c r="N16" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-10 · 9 roles sembrados según la matriz aprobada; asignación desde la pantalla Roles.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="18" t="inlineStr">
@@ -2983,11 +2991,19 @@
       </c>
       <c r="L17" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M17" s="19" t="inlineStr"/>
-      <c r="N17" s="19" t="inlineStr"/>
+          <t>En desarrollo</t>
+        </is>
+      </c>
+      <c r="M17" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/m1-07-roles · 67 pruebas de backend y 6 de frontend pasan</t>
+        </is>
+      </c>
+      <c r="N17" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-10 · Permisos por rol listos; el alcance por grupo/área llega con el módulo de Grupos.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="18" t="inlineStr">
@@ -3468,7 +3484,7 @@
       </c>
       <c r="M24" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/m1-01-expediente · 56 pruebas de backend y 6 de frontend pasan</t>
+          <t>Rama feature/m1-07-roles · 67 pruebas de backend y 6 de frontend pasan</t>
         </is>
       </c>
       <c r="N24" s="19" t="inlineStr">

</xml_diff>

<commit_message>
NF-03: bitácora inmutable en la base de datos y pantalla de consulta
- Trigger de PostgreSQL que rechaza UPDATE, DELETE y TRUNCATE sobre la bitácora
- El actor pasa a PROTECT (los usuarios se desactivan, no se borran)
- Endpoint /api/auditoria/ con filtros y permiso bitacora.ver; consultarla queda registrada
- Pantalla Bitácora; matriz de trazabilidad actualizada

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/trazabilidad/Matriz de Trazabilidad MDF.xlsx
+++ b/docs/trazabilidad/Matriz de Trazabilidad MDF.xlsx
@@ -7615,17 +7615,17 @@
       </c>
       <c r="L88" s="19" t="inlineStr">
         <is>
-          <t>En desarrollo</t>
+          <t>En pruebas</t>
         </is>
       </c>
       <c r="M88" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/m1-17-acceso · bitácora de solo-añadir a nivel de aplicación</t>
+          <t>Rama feature/nf-03-bitacora · 69 pruebas de backend pasan</t>
         </is>
       </c>
       <c r="N88" s="19" t="inlineStr">
         <is>
-          <t>2026-10-05 · Falta reforzarla en la base de datos (permisos) en el Sprint 1.</t>
+          <t>2026-10-10 · Bloqueo en aplicación y trigger de PostgreSQL (UPDATE/DELETE/TRUNCATE); pantalla de consulta con permiso bitacora.ver.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
M3: Grupos de Conexión (estructura, pase de lista, estudio semanal) con alcance por grupo
- Grupos con tipo (conexión o reunión de líderes), día y hora; roles por grupo (supervisor, líder,
  secretario, anfitrión, tesorero, asistente); invitados como Contacto sin duplicar por WhatsApp
- Alcance por grupo según la matriz de confidencialidad (M1-08): cada quien ve solo sus grupos
- Reuniones semanales y pase de lista (secretario el mismo día, líder siempre, supervisor consulta)
- Estudio semanal: PDF adultos, PDF niños y audio con soporte de Range para iPhone
- Permisos nuevos grupos.ver_todos, grupos.gestionar y grupos.material
- Pantallas: grupos, grupo, reunión con pase de lista y estudio; documentación v3.5 y matriz

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/trazabilidad/Matriz de Trazabilidad MDF.xlsx
+++ b/docs/trazabilidad/Matriz de Trazabilidad MDF.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Origen v1" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Matriz'!$A$1:$N$95</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Matriz'!$A$1:$N$96</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -897,31 +897,31 @@
         </is>
       </c>
       <c r="B5" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$95,$A5)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$96,$A5)</f>
         <v/>
       </c>
       <c r="C5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$95,$A5,Matriz!$L$2:$L$95,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$96,$A5,Matriz!$L$2:$L$96,"Pendiente")</f>
         <v/>
       </c>
       <c r="D5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$95,$A5,Matriz!$L$2:$L$95,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$96,$A5,Matriz!$L$2:$L$96,"En diseño")</f>
         <v/>
       </c>
       <c r="E5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$95,$A5,Matriz!$L$2:$L$95,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$96,$A5,Matriz!$L$2:$L$96,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$95,$A5,Matriz!$L$2:$L$95,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$96,$A5,Matriz!$L$2:$L$96,"En pruebas")</f>
         <v/>
       </c>
       <c r="G5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$95,$A5,Matriz!$L$2:$L$95,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$96,$A5,Matriz!$L$2:$L$96,"Hecho")</f>
         <v/>
       </c>
       <c r="H5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$95,$A5,Matriz!$L$2:$L$95,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$96,$A5,Matriz!$L$2:$L$96,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I5" s="13">
@@ -936,31 +936,31 @@
         </is>
       </c>
       <c r="B6" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$95,$A6)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$96,$A6)</f>
         <v/>
       </c>
       <c r="C6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$95,$A6,Matriz!$L$2:$L$95,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$96,$A6,Matriz!$L$2:$L$96,"Pendiente")</f>
         <v/>
       </c>
       <c r="D6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$95,$A6,Matriz!$L$2:$L$95,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$96,$A6,Matriz!$L$2:$L$96,"En diseño")</f>
         <v/>
       </c>
       <c r="E6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$95,$A6,Matriz!$L$2:$L$95,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$96,$A6,Matriz!$L$2:$L$96,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$95,$A6,Matriz!$L$2:$L$95,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$96,$A6,Matriz!$L$2:$L$96,"En pruebas")</f>
         <v/>
       </c>
       <c r="G6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$95,$A6,Matriz!$L$2:$L$95,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$96,$A6,Matriz!$L$2:$L$96,"Hecho")</f>
         <v/>
       </c>
       <c r="H6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$95,$A6,Matriz!$L$2:$L$95,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$96,$A6,Matriz!$L$2:$L$96,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I6" s="13">
@@ -975,31 +975,31 @@
         </is>
       </c>
       <c r="B7" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$95,$A7)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$96,$A7)</f>
         <v/>
       </c>
       <c r="C7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$95,$A7,Matriz!$L$2:$L$95,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$96,$A7,Matriz!$L$2:$L$96,"Pendiente")</f>
         <v/>
       </c>
       <c r="D7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$95,$A7,Matriz!$L$2:$L$95,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$96,$A7,Matriz!$L$2:$L$96,"En diseño")</f>
         <v/>
       </c>
       <c r="E7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$95,$A7,Matriz!$L$2:$L$95,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$96,$A7,Matriz!$L$2:$L$96,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$95,$A7,Matriz!$L$2:$L$95,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$96,$A7,Matriz!$L$2:$L$96,"En pruebas")</f>
         <v/>
       </c>
       <c r="G7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$95,$A7,Matriz!$L$2:$L$95,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$96,$A7,Matriz!$L$2:$L$96,"Hecho")</f>
         <v/>
       </c>
       <c r="H7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$95,$A7,Matriz!$L$2:$L$95,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$96,$A7,Matriz!$L$2:$L$96,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I7" s="13">
@@ -1014,31 +1014,31 @@
         </is>
       </c>
       <c r="B8" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$95,$A8)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$96,$A8)</f>
         <v/>
       </c>
       <c r="C8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$95,$A8,Matriz!$L$2:$L$95,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$96,$A8,Matriz!$L$2:$L$96,"Pendiente")</f>
         <v/>
       </c>
       <c r="D8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$95,$A8,Matriz!$L$2:$L$95,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$96,$A8,Matriz!$L$2:$L$96,"En diseño")</f>
         <v/>
       </c>
       <c r="E8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$95,$A8,Matriz!$L$2:$L$95,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$96,$A8,Matriz!$L$2:$L$96,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$95,$A8,Matriz!$L$2:$L$95,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$96,$A8,Matriz!$L$2:$L$96,"En pruebas")</f>
         <v/>
       </c>
       <c r="G8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$95,$A8,Matriz!$L$2:$L$95,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$96,$A8,Matriz!$L$2:$L$96,"Hecho")</f>
         <v/>
       </c>
       <c r="H8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$95,$A8,Matriz!$L$2:$L$95,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$96,$A8,Matriz!$L$2:$L$96,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I8" s="13">
@@ -1053,31 +1053,31 @@
         </is>
       </c>
       <c r="B9" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$95,$A9)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$96,$A9)</f>
         <v/>
       </c>
       <c r="C9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$95,$A9,Matriz!$L$2:$L$95,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$96,$A9,Matriz!$L$2:$L$96,"Pendiente")</f>
         <v/>
       </c>
       <c r="D9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$95,$A9,Matriz!$L$2:$L$95,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$96,$A9,Matriz!$L$2:$L$96,"En diseño")</f>
         <v/>
       </c>
       <c r="E9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$95,$A9,Matriz!$L$2:$L$95,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$96,$A9,Matriz!$L$2:$L$96,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$95,$A9,Matriz!$L$2:$L$95,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$96,$A9,Matriz!$L$2:$L$96,"En pruebas")</f>
         <v/>
       </c>
       <c r="G9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$95,$A9,Matriz!$L$2:$L$95,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$96,$A9,Matriz!$L$2:$L$96,"Hecho")</f>
         <v/>
       </c>
       <c r="H9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$95,$A9,Matriz!$L$2:$L$95,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$96,$A9,Matriz!$L$2:$L$96,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I9" s="13">
@@ -1092,31 +1092,31 @@
         </is>
       </c>
       <c r="B10" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$95,$A10)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$96,$A10)</f>
         <v/>
       </c>
       <c r="C10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$95,$A10,Matriz!$L$2:$L$95,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$96,$A10,Matriz!$L$2:$L$96,"Pendiente")</f>
         <v/>
       </c>
       <c r="D10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$95,$A10,Matriz!$L$2:$L$95,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$96,$A10,Matriz!$L$2:$L$96,"En diseño")</f>
         <v/>
       </c>
       <c r="E10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$95,$A10,Matriz!$L$2:$L$95,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$96,$A10,Matriz!$L$2:$L$96,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$95,$A10,Matriz!$L$2:$L$95,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$96,$A10,Matriz!$L$2:$L$96,"En pruebas")</f>
         <v/>
       </c>
       <c r="G10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$95,$A10,Matriz!$L$2:$L$95,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$96,$A10,Matriz!$L$2:$L$96,"Hecho")</f>
         <v/>
       </c>
       <c r="H10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$95,$A10,Matriz!$L$2:$L$95,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$96,$A10,Matriz!$L$2:$L$96,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I10" s="13">
@@ -1131,31 +1131,31 @@
         </is>
       </c>
       <c r="B11" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$95,$A11)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$96,$A11)</f>
         <v/>
       </c>
       <c r="C11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$95,$A11,Matriz!$L$2:$L$95,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$96,$A11,Matriz!$L$2:$L$96,"Pendiente")</f>
         <v/>
       </c>
       <c r="D11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$95,$A11,Matriz!$L$2:$L$95,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$96,$A11,Matriz!$L$2:$L$96,"En diseño")</f>
         <v/>
       </c>
       <c r="E11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$95,$A11,Matriz!$L$2:$L$95,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$96,$A11,Matriz!$L$2:$L$96,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$95,$A11,Matriz!$L$2:$L$95,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$96,$A11,Matriz!$L$2:$L$96,"En pruebas")</f>
         <v/>
       </c>
       <c r="G11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$95,$A11,Matriz!$L$2:$L$95,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$96,$A11,Matriz!$L$2:$L$96,"Hecho")</f>
         <v/>
       </c>
       <c r="H11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$95,$A11,Matriz!$L$2:$L$95,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$96,$A11,Matriz!$L$2:$L$96,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I11" s="13">
@@ -1256,31 +1256,31 @@
         </is>
       </c>
       <c r="B16" s="12">
-        <f>COUNTIF(Matriz!$H$2:$H$95,$A16)</f>
+        <f>COUNTIF(Matriz!$H$2:$H$96,$A16)</f>
         <v/>
       </c>
       <c r="C16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$95,$A16,Matriz!$L$2:$L$95,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$96,$A16,Matriz!$L$2:$L$96,"Pendiente")</f>
         <v/>
       </c>
       <c r="D16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$95,$A16,Matriz!$L$2:$L$95,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$96,$A16,Matriz!$L$2:$L$96,"En diseño")</f>
         <v/>
       </c>
       <c r="E16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$95,$A16,Matriz!$L$2:$L$95,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$96,$A16,Matriz!$L$2:$L$96,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$95,$A16,Matriz!$L$2:$L$95,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$96,$A16,Matriz!$L$2:$L$96,"En pruebas")</f>
         <v/>
       </c>
       <c r="G16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$95,$A16,Matriz!$L$2:$L$95,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$96,$A16,Matriz!$L$2:$L$96,"Hecho")</f>
         <v/>
       </c>
       <c r="H16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$95,$A16,Matriz!$L$2:$L$95,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$96,$A16,Matriz!$L$2:$L$96,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I16" s="13">
@@ -1295,31 +1295,31 @@
         </is>
       </c>
       <c r="B17" s="12">
-        <f>COUNTIF(Matriz!$H$2:$H$95,$A17)</f>
+        <f>COUNTIF(Matriz!$H$2:$H$96,$A17)</f>
         <v/>
       </c>
       <c r="C17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$95,$A17,Matriz!$L$2:$L$95,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$96,$A17,Matriz!$L$2:$L$96,"Pendiente")</f>
         <v/>
       </c>
       <c r="D17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$95,$A17,Matriz!$L$2:$L$95,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$96,$A17,Matriz!$L$2:$L$96,"En diseño")</f>
         <v/>
       </c>
       <c r="E17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$95,$A17,Matriz!$L$2:$L$95,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$96,$A17,Matriz!$L$2:$L$96,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$95,$A17,Matriz!$L$2:$L$95,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$96,$A17,Matriz!$L$2:$L$96,"En pruebas")</f>
         <v/>
       </c>
       <c r="G17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$95,$A17,Matriz!$L$2:$L$95,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$96,$A17,Matriz!$L$2:$L$96,"Hecho")</f>
         <v/>
       </c>
       <c r="H17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$95,$A17,Matriz!$L$2:$L$95,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$96,$A17,Matriz!$L$2:$L$96,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I17" s="13">
@@ -1334,31 +1334,31 @@
         </is>
       </c>
       <c r="B18" s="12">
-        <f>COUNTIF(Matriz!$H$2:$H$95,$A18)</f>
+        <f>COUNTIF(Matriz!$H$2:$H$96,$A18)</f>
         <v/>
       </c>
       <c r="C18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$95,$A18,Matriz!$L$2:$L$95,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$96,$A18,Matriz!$L$2:$L$96,"Pendiente")</f>
         <v/>
       </c>
       <c r="D18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$95,$A18,Matriz!$L$2:$L$95,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$96,$A18,Matriz!$L$2:$L$96,"En diseño")</f>
         <v/>
       </c>
       <c r="E18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$95,$A18,Matriz!$L$2:$L$95,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$96,$A18,Matriz!$L$2:$L$96,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$95,$A18,Matriz!$L$2:$L$95,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$96,$A18,Matriz!$L$2:$L$96,"En pruebas")</f>
         <v/>
       </c>
       <c r="G18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$95,$A18,Matriz!$L$2:$L$95,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$96,$A18,Matriz!$L$2:$L$96,"Hecho")</f>
         <v/>
       </c>
       <c r="H18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$95,$A18,Matriz!$L$2:$L$95,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$96,$A18,Matriz!$L$2:$L$96,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I18" s="13">
@@ -1373,31 +1373,31 @@
         </is>
       </c>
       <c r="B19" s="12">
-        <f>COUNTIF(Matriz!$H$2:$H$95,$A19)</f>
+        <f>COUNTIF(Matriz!$H$2:$H$96,$A19)</f>
         <v/>
       </c>
       <c r="C19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$95,$A19,Matriz!$L$2:$L$95,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$96,$A19,Matriz!$L$2:$L$96,"Pendiente")</f>
         <v/>
       </c>
       <c r="D19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$95,$A19,Matriz!$L$2:$L$95,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$96,$A19,Matriz!$L$2:$L$96,"En diseño")</f>
         <v/>
       </c>
       <c r="E19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$95,$A19,Matriz!$L$2:$L$95,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$96,$A19,Matriz!$L$2:$L$96,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$95,$A19,Matriz!$L$2:$L$95,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$96,$A19,Matriz!$L$2:$L$96,"En pruebas")</f>
         <v/>
       </c>
       <c r="G19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$95,$A19,Matriz!$L$2:$L$95,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$96,$A19,Matriz!$L$2:$L$96,"Hecho")</f>
         <v/>
       </c>
       <c r="H19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$95,$A19,Matriz!$L$2:$L$95,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$96,$A19,Matriz!$L$2:$L$96,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I19" s="13">
@@ -1498,31 +1498,31 @@
         </is>
       </c>
       <c r="B24" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$95,$A24)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$96,$A24)</f>
         <v/>
       </c>
       <c r="C24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$95,$A24,Matriz!$L$2:$L$95,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$96,$A24,Matriz!$L$2:$L$96,"Pendiente")</f>
         <v/>
       </c>
       <c r="D24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$95,$A24,Matriz!$L$2:$L$95,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$96,$A24,Matriz!$L$2:$L$96,"En diseño")</f>
         <v/>
       </c>
       <c r="E24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$95,$A24,Matriz!$L$2:$L$95,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$96,$A24,Matriz!$L$2:$L$96,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$95,$A24,Matriz!$L$2:$L$95,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$96,$A24,Matriz!$L$2:$L$96,"En pruebas")</f>
         <v/>
       </c>
       <c r="G24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$95,$A24,Matriz!$L$2:$L$95,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$96,$A24,Matriz!$L$2:$L$96,"Hecho")</f>
         <v/>
       </c>
       <c r="H24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$95,$A24,Matriz!$L$2:$L$95,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$96,$A24,Matriz!$L$2:$L$96,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I24" s="13">
@@ -1537,31 +1537,31 @@
         </is>
       </c>
       <c r="B25" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$95,$A25)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$96,$A25)</f>
         <v/>
       </c>
       <c r="C25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$95,$A25,Matriz!$L$2:$L$95,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$96,$A25,Matriz!$L$2:$L$96,"Pendiente")</f>
         <v/>
       </c>
       <c r="D25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$95,$A25,Matriz!$L$2:$L$95,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$96,$A25,Matriz!$L$2:$L$96,"En diseño")</f>
         <v/>
       </c>
       <c r="E25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$95,$A25,Matriz!$L$2:$L$95,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$96,$A25,Matriz!$L$2:$L$96,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$95,$A25,Matriz!$L$2:$L$95,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$96,$A25,Matriz!$L$2:$L$96,"En pruebas")</f>
         <v/>
       </c>
       <c r="G25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$95,$A25,Matriz!$L$2:$L$95,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$96,$A25,Matriz!$L$2:$L$96,"Hecho")</f>
         <v/>
       </c>
       <c r="H25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$95,$A25,Matriz!$L$2:$L$95,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$96,$A25,Matriz!$L$2:$L$96,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I25" s="13">
@@ -1576,31 +1576,31 @@
         </is>
       </c>
       <c r="B26" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$95,$A26)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$96,$A26)</f>
         <v/>
       </c>
       <c r="C26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$95,$A26,Matriz!$L$2:$L$95,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$96,$A26,Matriz!$L$2:$L$96,"Pendiente")</f>
         <v/>
       </c>
       <c r="D26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$95,$A26,Matriz!$L$2:$L$95,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$96,$A26,Matriz!$L$2:$L$96,"En diseño")</f>
         <v/>
       </c>
       <c r="E26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$95,$A26,Matriz!$L$2:$L$95,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$96,$A26,Matriz!$L$2:$L$96,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$95,$A26,Matriz!$L$2:$L$95,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$96,$A26,Matriz!$L$2:$L$96,"En pruebas")</f>
         <v/>
       </c>
       <c r="G26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$95,$A26,Matriz!$L$2:$L$95,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$96,$A26,Matriz!$L$2:$L$96,"Hecho")</f>
         <v/>
       </c>
       <c r="H26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$95,$A26,Matriz!$L$2:$L$95,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$96,$A26,Matriz!$L$2:$L$96,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I26" s="13">
@@ -1615,31 +1615,31 @@
         </is>
       </c>
       <c r="B27" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$95,$A27)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$96,$A27)</f>
         <v/>
       </c>
       <c r="C27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$95,$A27,Matriz!$L$2:$L$95,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$96,$A27,Matriz!$L$2:$L$96,"Pendiente")</f>
         <v/>
       </c>
       <c r="D27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$95,$A27,Matriz!$L$2:$L$95,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$96,$A27,Matriz!$L$2:$L$96,"En diseño")</f>
         <v/>
       </c>
       <c r="E27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$95,$A27,Matriz!$L$2:$L$95,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$96,$A27,Matriz!$L$2:$L$96,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$95,$A27,Matriz!$L$2:$L$95,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$96,$A27,Matriz!$L$2:$L$96,"En pruebas")</f>
         <v/>
       </c>
       <c r="G27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$95,$A27,Matriz!$L$2:$L$95,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$96,$A27,Matriz!$L$2:$L$96,"Hecho")</f>
         <v/>
       </c>
       <c r="H27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$95,$A27,Matriz!$L$2:$L$95,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$96,$A27,Matriz!$L$2:$L$96,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I27" s="13">
@@ -1654,31 +1654,31 @@
         </is>
       </c>
       <c r="B28" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$95,$A28)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$96,$A28)</f>
         <v/>
       </c>
       <c r="C28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$95,$A28,Matriz!$L$2:$L$95,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$96,$A28,Matriz!$L$2:$L$96,"Pendiente")</f>
         <v/>
       </c>
       <c r="D28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$95,$A28,Matriz!$L$2:$L$95,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$96,$A28,Matriz!$L$2:$L$96,"En diseño")</f>
         <v/>
       </c>
       <c r="E28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$95,$A28,Matriz!$L$2:$L$95,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$96,$A28,Matriz!$L$2:$L$96,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$95,$A28,Matriz!$L$2:$L$95,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$96,$A28,Matriz!$L$2:$L$96,"En pruebas")</f>
         <v/>
       </c>
       <c r="G28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$95,$A28,Matriz!$L$2:$L$95,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$96,$A28,Matriz!$L$2:$L$96,"Hecho")</f>
         <v/>
       </c>
       <c r="H28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$95,$A28,Matriz!$L$2:$L$95,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$96,$A28,Matriz!$L$2:$L$96,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I28" s="13">
@@ -1693,31 +1693,31 @@
         </is>
       </c>
       <c r="B29" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$95,$A29)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$96,$A29)</f>
         <v/>
       </c>
       <c r="C29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$95,$A29,Matriz!$L$2:$L$95,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$96,$A29,Matriz!$L$2:$L$96,"Pendiente")</f>
         <v/>
       </c>
       <c r="D29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$95,$A29,Matriz!$L$2:$L$95,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$96,$A29,Matriz!$L$2:$L$96,"En diseño")</f>
         <v/>
       </c>
       <c r="E29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$95,$A29,Matriz!$L$2:$L$95,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$96,$A29,Matriz!$L$2:$L$96,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$95,$A29,Matriz!$L$2:$L$95,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$96,$A29,Matriz!$L$2:$L$96,"En pruebas")</f>
         <v/>
       </c>
       <c r="G29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$95,$A29,Matriz!$L$2:$L$95,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$96,$A29,Matriz!$L$2:$L$96,"Hecho")</f>
         <v/>
       </c>
       <c r="H29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$95,$A29,Matriz!$L$2:$L$95,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$96,$A29,Matriz!$L$2:$L$96,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I29" s="13">
@@ -1732,31 +1732,31 @@
         </is>
       </c>
       <c r="B30" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$95,$A30)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$96,$A30)</f>
         <v/>
       </c>
       <c r="C30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$95,$A30,Matriz!$L$2:$L$95,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$96,$A30,Matriz!$L$2:$L$96,"Pendiente")</f>
         <v/>
       </c>
       <c r="D30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$95,$A30,Matriz!$L$2:$L$95,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$96,$A30,Matriz!$L$2:$L$96,"En diseño")</f>
         <v/>
       </c>
       <c r="E30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$95,$A30,Matriz!$L$2:$L$95,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$96,$A30,Matriz!$L$2:$L$96,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$95,$A30,Matriz!$L$2:$L$95,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$96,$A30,Matriz!$L$2:$L$96,"En pruebas")</f>
         <v/>
       </c>
       <c r="G30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$95,$A30,Matriz!$L$2:$L$95,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$96,$A30,Matriz!$L$2:$L$96,"Hecho")</f>
         <v/>
       </c>
       <c r="H30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$95,$A30,Matriz!$L$2:$L$95,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$96,$A30,Matriz!$L$2:$L$96,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I30" s="13">
@@ -1818,7 +1818,7 @@
         </is>
       </c>
       <c r="B35" s="12">
-        <f>COUNTIF(Matriz!$K$2:$K$95,A35)</f>
+        <f>COUNTIF(Matriz!$K$2:$K$96,A35)</f>
         <v/>
       </c>
     </row>
@@ -1829,7 +1829,7 @@
         </is>
       </c>
       <c r="B36" s="12">
-        <f>COUNTIF(Matriz!$K$2:$K$95,A36)</f>
+        <f>COUNTIF(Matriz!$K$2:$K$96,A36)</f>
         <v/>
       </c>
     </row>
@@ -1840,7 +1840,7 @@
         </is>
       </c>
       <c r="B37" s="12">
-        <f>COUNTIF(Matriz!$K$2:$K$95,A37)</f>
+        <f>COUNTIF(Matriz!$K$2:$K$96,A37)</f>
         <v/>
       </c>
     </row>
@@ -1851,7 +1851,7 @@
         </is>
       </c>
       <c r="B38" s="12">
-        <f>COUNTIF(Matriz!$K$2:$K$95,A38)</f>
+        <f>COUNTIF(Matriz!$K$2:$K$96,A38)</f>
         <v/>
       </c>
     </row>
@@ -1866,7 +1866,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N95"/>
+  <dimension ref="A1:N96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2991,17 +2991,17 @@
       </c>
       <c r="L17" s="19" t="inlineStr">
         <is>
-          <t>En desarrollo</t>
+          <t>En pruebas</t>
         </is>
       </c>
       <c r="M17" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/m1-07-roles · 67 pruebas de backend y 6 de frontend pasan</t>
+          <t>Rama feature/m3-grupos · 88 pruebas de backend y 7 de frontend pasan</t>
         </is>
       </c>
       <c r="N17" s="19" t="inlineStr">
         <is>
-          <t>2026-10-10 · Permisos por rol listos; el alcance por grupo/área llega con el módulo de Grupos.</t>
+          <t>2026-10-24 · Alcance por grupo implementado en el módulo Grupos.</t>
         </is>
       </c>
     </row>
@@ -5055,11 +5055,19 @@
       </c>
       <c r="L48" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M48" s="19" t="inlineStr"/>
-      <c r="N48" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M48" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/m3-grupos · 88 pruebas de backend y 7 de frontend pasan</t>
+        </is>
+      </c>
+      <c r="N48" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-24 · Supervisor, Líder, Secretario, Anfitrión, Tesorero y Asistente por grupo; falta probar con líderes reales.</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="18" t="inlineStr">
@@ -5074,12 +5082,12 @@
       </c>
       <c r="C49" s="19" t="inlineStr">
         <is>
-          <t>Distribución del estudio semanal dentro de la app, sustituyendo el envío por WhatsApp.</t>
+          <t>Estudio semanal dentro de la app: un registro por semana con PDF para adultos, PDF para niños y audio de la lectura (PDF hasta 15 MB; audio hasta 40 MB). Lo publican Pastor o Anciano y los líderes lo abren desde la reunión, sustituyendo el envío por WhatsApp. El audio admite adelantar y retroceder en iPhone.</t>
         </is>
       </c>
       <c r="D49" s="19" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>v1 / v2 + Respuesta</t>
         </is>
       </c>
       <c r="E49" s="19" t="inlineStr">
@@ -5119,11 +5127,19 @@
       </c>
       <c r="L49" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M49" s="19" t="inlineStr"/>
-      <c r="N49" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M49" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/m3-grupos · 88 pruebas de backend y 7 de frontend pasan</t>
+        </is>
+      </c>
+      <c r="N49" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-24 · PDF adultos, PDF niños y audio por semana; audio con Range para iPhone. Pendiente probar en iOS.</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="18" t="inlineStr">
@@ -5138,7 +5154,7 @@
       </c>
       <c r="C50" s="19" t="inlineStr">
         <is>
-          <t>Pase de lista digital por Secretario o Líder, con captura sin conexión y sincronización posterior.</t>
+          <t>Pase de lista digital por Secretario o Líder. El Secretario captura y corrige el mismo día; el Líder modifica siempre; el Supervisor solo consulta. La captura sin conexión (NF-06) queda para la siguiente entrega.</t>
         </is>
       </c>
       <c r="D50" s="19" t="inlineStr">
@@ -5183,11 +5199,19 @@
       </c>
       <c r="L50" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M50" s="19" t="inlineStr"/>
-      <c r="N50" s="19" t="inlineStr"/>
+          <t>En desarrollo</t>
+        </is>
+      </c>
+      <c r="M50" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/m3-grupos · 88 pruebas de backend y 7 de frontend pasan</t>
+        </is>
+      </c>
+      <c r="N50" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-24 · Pase de lista listo; falta modo sin conexión (NF-06).</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="18" t="inlineStr">
@@ -5567,11 +5591,19 @@
       </c>
       <c r="L56" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M56" s="19" t="inlineStr"/>
-      <c r="N56" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M56" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/m3-grupos · 88 pruebas de backend y 7 de frontend pasan</t>
+        </is>
+      </c>
+      <c r="N56" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-24 · Invitados registrados como Contacto con consentimiento y sin duplicar por WhatsApp.</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="18" t="inlineStr">
@@ -5704,42 +5736,42 @@
     <row r="59">
       <c r="A59" s="18" t="inlineStr">
         <is>
-          <t>M4-01</t>
+          <t>M3-12</t>
         </is>
       </c>
       <c r="B59" s="19" t="inlineStr">
         <is>
-          <t>M4 Kids Check-In/Out</t>
+          <t>M3 Grupos de Conexión</t>
         </is>
       </c>
       <c r="C59" s="19" t="inlineStr">
         <is>
-          <t>Sustitución de la ficha física de papel.</t>
-        </is>
-      </c>
-      <c r="D59" s="19" t="inlineStr">
-        <is>
-          <t>v1 / v2</t>
+          <t>Reuniones: cada grupo se reúne una vez por semana en casa del líder (día y hora por grupo) y existe una reunión general de líderes, modelada como un grupo de tipo «Líderes».</t>
+        </is>
+      </c>
+      <c r="D59" s="21" t="inlineStr">
+        <is>
+          <t>Respuesta</t>
         </is>
       </c>
       <c r="E59" s="19" t="inlineStr">
         <is>
-          <t>Fuera del MVP</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="F59" s="19" t="inlineStr">
         <is>
-          <t>Fase 2</t>
+          <t>Fase 1</t>
         </is>
       </c>
       <c r="G59" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sprint 3</t>
         </is>
       </c>
       <c r="H59" s="19" t="inlineStr">
         <is>
-          <t>Posterior</t>
+          <t>H3 · MVP (Grupos)</t>
         </is>
       </c>
       <c r="I59" s="20" t="inlineStr">
@@ -5759,16 +5791,24 @@
       </c>
       <c r="L59" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M59" s="19" t="inlineStr"/>
-      <c r="N59" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M59" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/m3-grupos · 88 pruebas de backend y 7 de frontend pasan</t>
+        </is>
+      </c>
+      <c r="N59" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-24 · Una reunión semanal por grupo y grupo tipo Líderes.</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="18" t="inlineStr">
         <is>
-          <t>M4-02</t>
+          <t>M4-01</t>
         </is>
       </c>
       <c r="B60" s="19" t="inlineStr">
@@ -5778,12 +5818,12 @@
       </c>
       <c r="C60" s="19" t="inlineStr">
         <is>
-          <t>Registro de ingreso del menor con salón o clase asignada y generación de código único.</t>
-        </is>
-      </c>
-      <c r="D60" s="21" t="inlineStr">
-        <is>
-          <t>v1 + Nuevo v3</t>
+          <t>Sustitución de la ficha física de papel.</t>
+        </is>
+      </c>
+      <c r="D60" s="19" t="inlineStr">
+        <is>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E60" s="19" t="inlineStr">
@@ -5832,7 +5872,7 @@
     <row r="61">
       <c r="A61" s="18" t="inlineStr">
         <is>
-          <t>M4-03</t>
+          <t>M4-02</t>
         </is>
       </c>
       <c r="B61" s="19" t="inlineStr">
@@ -5842,12 +5882,12 @@
       </c>
       <c r="C61" s="19" t="inlineStr">
         <is>
-          <t>Código QR dinámico o OTP temporal en la PWA del padre o tutor.</t>
-        </is>
-      </c>
-      <c r="D61" s="19" t="inlineStr">
-        <is>
-          <t>v2</t>
+          <t>Registro de ingreso del menor con salón o clase asignada y generación de código único.</t>
+        </is>
+      </c>
+      <c r="D61" s="21" t="inlineStr">
+        <is>
+          <t>v1 + Nuevo v3</t>
         </is>
       </c>
       <c r="E61" s="19" t="inlineStr">
@@ -5896,7 +5936,7 @@
     <row r="62">
       <c r="A62" s="18" t="inlineStr">
         <is>
-          <t>M4-04</t>
+          <t>M4-03</t>
         </is>
       </c>
       <c r="B62" s="19" t="inlineStr">
@@ -5906,7 +5946,7 @@
       </c>
       <c r="C62" s="19" t="inlineStr">
         <is>
-          <t>Validación al entregar: el servidor de Kids escanea el código y confirma identidad y fotografía del tutor autorizado en el Expediente Digital.</t>
+          <t>Código QR dinámico o OTP temporal en la PWA del padre o tutor.</t>
         </is>
       </c>
       <c r="D62" s="19" t="inlineStr">
@@ -5960,7 +6000,7 @@
     <row r="63">
       <c r="A63" s="18" t="inlineStr">
         <is>
-          <t>M4-05</t>
+          <t>M4-04</t>
         </is>
       </c>
       <c r="B63" s="19" t="inlineStr">
@@ -5970,12 +6010,12 @@
       </c>
       <c r="C63" s="19" t="inlineStr">
         <is>
-          <t>Alternativa para tutores sin smartphone, sin batería o sin conexión (p. ej. código por SMS o comprobante imprimible con identificación). Por definir.</t>
-        </is>
-      </c>
-      <c r="D63" s="21" t="inlineStr">
-        <is>
-          <t>Nuevo v3</t>
+          <t>Validación al entregar: el servidor de Kids escanea el código y confirma identidad y fotografía del tutor autorizado en el Expediente Digital.</t>
+        </is>
+      </c>
+      <c r="D63" s="19" t="inlineStr">
+        <is>
+          <t>v2</t>
         </is>
       </c>
       <c r="E63" s="19" t="inlineStr">
@@ -6010,7 +6050,7 @@
       </c>
       <c r="K63" s="19" t="inlineStr">
         <is>
-          <t>Por definir</t>
+          <t>VoBo pendiente</t>
         </is>
       </c>
       <c r="L63" s="19" t="inlineStr">
@@ -6024,7 +6064,7 @@
     <row r="64">
       <c r="A64" s="18" t="inlineStr">
         <is>
-          <t>M4-06</t>
+          <t>M4-05</t>
         </is>
       </c>
       <c r="B64" s="19" t="inlineStr">
@@ -6034,7 +6074,7 @@
       </c>
       <c r="C64" s="19" t="inlineStr">
         <is>
-          <t>Autorización temporal de un tercero para recoger al menor, con aprobación del tutor registrado.</t>
+          <t>Alternativa para tutores sin smartphone, sin batería o sin conexión (p. ej. código por SMS o comprobante imprimible con identificación). Por definir.</t>
         </is>
       </c>
       <c r="D64" s="21" t="inlineStr">
@@ -6074,7 +6114,7 @@
       </c>
       <c r="K64" s="19" t="inlineStr">
         <is>
-          <t>VoBo pendiente</t>
+          <t>Por definir</t>
         </is>
       </c>
       <c r="L64" s="19" t="inlineStr">
@@ -6088,7 +6128,7 @@
     <row r="65">
       <c r="A65" s="18" t="inlineStr">
         <is>
-          <t>M4-07</t>
+          <t>M4-06</t>
         </is>
       </c>
       <c r="B65" s="19" t="inlineStr">
@@ -6098,7 +6138,7 @@
       </c>
       <c r="C65" s="19" t="inlineStr">
         <is>
-          <t>Caducidad del código y bitácora de cada entrega (quién recogió, quién entregó, hora).</t>
+          <t>Autorización temporal de un tercero para recoger al menor, con aprobación del tutor registrado.</t>
         </is>
       </c>
       <c r="D65" s="21" t="inlineStr">
@@ -6152,7 +6192,7 @@
     <row r="66">
       <c r="A66" s="18" t="inlineStr">
         <is>
-          <t>M4-08</t>
+          <t>M4-07</t>
         </is>
       </c>
       <c r="B66" s="19" t="inlineStr">
@@ -6162,7 +6202,7 @@
       </c>
       <c r="C66" s="19" t="inlineStr">
         <is>
-          <t>Funcionamiento sin conexión o con conexión degradada para el check-out.</t>
+          <t>Caducidad del código y bitácora de cada entrega (quién recogió, quién entregó, hora).</t>
         </is>
       </c>
       <c r="D66" s="21" t="inlineStr">
@@ -6216,52 +6256,52 @@
     <row r="67">
       <c r="A67" s="18" t="inlineStr">
         <is>
-          <t>M5-01</t>
+          <t>M4-08</t>
         </is>
       </c>
       <c r="B67" s="19" t="inlineStr">
         <is>
-          <t>M5 Áreas y servidores</t>
+          <t>M4 Kids Check-In/Out</t>
         </is>
       </c>
       <c r="C67" s="19" t="inlineStr">
         <is>
-          <t>Catálogo mínimo de áreas y asignación de servidores. Versión reducida del módulo 5, necesaria para permisos por área. Sirve como primer censo.</t>
-        </is>
-      </c>
-      <c r="D67" s="19" t="inlineStr">
-        <is>
-          <t>v3</t>
+          <t>Funcionamiento sin conexión o con conexión degradada para el check-out.</t>
+        </is>
+      </c>
+      <c r="D67" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3</t>
         </is>
       </c>
       <c r="E67" s="19" t="inlineStr">
         <is>
-          <t>MVP mínimo</t>
+          <t>Fuera del MVP</t>
         </is>
       </c>
       <c r="F67" s="19" t="inlineStr">
         <is>
-          <t>Fase 0</t>
+          <t>Fase 2</t>
         </is>
       </c>
       <c r="G67" s="19" t="inlineStr">
         <is>
-          <t>Sprint 1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H67" s="19" t="inlineStr">
         <is>
-          <t>H2 · Fase 0 completa</t>
-        </is>
-      </c>
-      <c r="I67" s="19" t="inlineStr">
-        <is>
-          <t>Como pastor quiero un catálogo de áreas con su personal para conocer la estructura.</t>
-        </is>
-      </c>
-      <c r="J67" s="19" t="inlineStr">
-        <is>
-          <t>Crear un área, asignar servidores y ver el conteo real.</t>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="I67" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
+        </is>
+      </c>
+      <c r="J67" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
         </is>
       </c>
       <c r="K67" s="19" t="inlineStr">
@@ -6280,7 +6320,7 @@
     <row r="68">
       <c r="A68" s="18" t="inlineStr">
         <is>
-          <t>M5-02</t>
+          <t>M5-01</t>
         </is>
       </c>
       <c r="B68" s="19" t="inlineStr">
@@ -6290,42 +6330,42 @@
       </c>
       <c r="C68" s="19" t="inlineStr">
         <is>
-          <t>Roles jerárquicos dentro de cada área (directores, líderes, maestros, servidores).</t>
+          <t>Catálogo mínimo de áreas y asignación de servidores. Versión reducida del módulo 5, necesaria para permisos por área. Sirve como primer censo.</t>
         </is>
       </c>
       <c r="D68" s="19" t="inlineStr">
         <is>
-          <t>v1</t>
+          <t>v3</t>
         </is>
       </c>
       <c r="E68" s="19" t="inlineStr">
         <is>
-          <t>Fuera del MVP</t>
+          <t>MVP mínimo</t>
         </is>
       </c>
       <c r="F68" s="19" t="inlineStr">
         <is>
-          <t>Fase 4</t>
+          <t>Fase 0</t>
         </is>
       </c>
       <c r="G68" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sprint 1</t>
         </is>
       </c>
       <c r="H68" s="19" t="inlineStr">
         <is>
-          <t>Posterior</t>
-        </is>
-      </c>
-      <c r="I68" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
-        </is>
-      </c>
-      <c r="J68" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
+          <t>H2 · Fase 0 completa</t>
+        </is>
+      </c>
+      <c r="I68" s="19" t="inlineStr">
+        <is>
+          <t>Como pastor quiero un catálogo de áreas con su personal para conocer la estructura.</t>
+        </is>
+      </c>
+      <c r="J68" s="19" t="inlineStr">
+        <is>
+          <t>Crear un área, asignar servidores y ver el conteo real.</t>
         </is>
       </c>
       <c r="K68" s="19" t="inlineStr">
@@ -6344,7 +6384,7 @@
     <row r="69">
       <c r="A69" s="18" t="inlineStr">
         <is>
-          <t>M5-03</t>
+          <t>M5-02</t>
         </is>
       </c>
       <c r="B69" s="19" t="inlineStr">
@@ -6354,12 +6394,12 @@
       </c>
       <c r="C69" s="19" t="inlineStr">
         <is>
-          <t>Organigrama y número real de servidores activos, directores y líderes por área.</t>
+          <t>Roles jerárquicos dentro de cada área (directores, líderes, maestros, servidores).</t>
         </is>
       </c>
       <c r="D69" s="19" t="inlineStr">
         <is>
-          <t>v2</t>
+          <t>v1</t>
         </is>
       </c>
       <c r="E69" s="19" t="inlineStr">
@@ -6408,7 +6448,7 @@
     <row r="70">
       <c r="A70" s="18" t="inlineStr">
         <is>
-          <t>M5-04</t>
+          <t>M5-03</t>
         </is>
       </c>
       <c r="B70" s="19" t="inlineStr">
@@ -6418,12 +6458,12 @@
       </c>
       <c r="C70" s="19" t="inlineStr">
         <is>
-          <t>Control de asistencia a turnos o servicios.</t>
+          <t>Organigrama y número real de servidores activos, directores y líderes por área.</t>
         </is>
       </c>
       <c r="D70" s="19" t="inlineStr">
         <is>
-          <t>v1 / v2</t>
+          <t>v2</t>
         </is>
       </c>
       <c r="E70" s="19" t="inlineStr">
@@ -6472,7 +6512,7 @@
     <row r="71">
       <c r="A71" s="18" t="inlineStr">
         <is>
-          <t>M5-05</t>
+          <t>M5-04</t>
         </is>
       </c>
       <c r="B71" s="19" t="inlineStr">
@@ -6482,7 +6522,7 @@
       </c>
       <c r="C71" s="19" t="inlineStr">
         <is>
-          <t>Tablero de avisos y notificaciones interno por área.</t>
+          <t>Control de asistencia a turnos o servicios.</t>
         </is>
       </c>
       <c r="D71" s="19" t="inlineStr">
@@ -6536,7 +6576,7 @@
     <row r="72">
       <c r="A72" s="18" t="inlineStr">
         <is>
-          <t>M5-06</t>
+          <t>M5-05</t>
         </is>
       </c>
       <c r="B72" s="19" t="inlineStr">
@@ -6546,7 +6586,7 @@
       </c>
       <c r="C72" s="19" t="inlineStr">
         <is>
-          <t>Gestión financiera por área: caja chica y gastos operativos.</t>
+          <t>Tablero de avisos y notificaciones interno por área.</t>
         </is>
       </c>
       <c r="D72" s="19" t="inlineStr">
@@ -6600,22 +6640,22 @@
     <row r="73">
       <c r="A73" s="18" t="inlineStr">
         <is>
-          <t>M6-01</t>
+          <t>M5-06</t>
         </is>
       </c>
       <c r="B73" s="19" t="inlineStr">
         <is>
-          <t>M6 Ministerios de servicio</t>
+          <t>M5 Áreas y servidores</t>
         </is>
       </c>
       <c r="C73" s="19" t="inlineStr">
         <is>
-          <t>Control de personal propio de cada ministerio.</t>
-        </is>
-      </c>
-      <c r="D73" s="22" t="inlineStr">
-        <is>
-          <t>Recuperado v1</t>
+          <t>Gestión financiera por área: caja chica y gastos operativos.</t>
+        </is>
+      </c>
+      <c r="D73" s="19" t="inlineStr">
+        <is>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E73" s="19" t="inlineStr">
@@ -6664,7 +6704,7 @@
     <row r="74">
       <c r="A74" s="18" t="inlineStr">
         <is>
-          <t>M6-02</t>
+          <t>M6-01</t>
         </is>
       </c>
       <c r="B74" s="19" t="inlineStr">
@@ -6674,12 +6714,12 @@
       </c>
       <c r="C74" s="19" t="inlineStr">
         <is>
-          <t>Menú o catálogo digital interactivo (público o interno), autogestionado.</t>
-        </is>
-      </c>
-      <c r="D74" s="19" t="inlineStr">
-        <is>
-          <t>v1 / v2</t>
+          <t>Control de personal propio de cada ministerio.</t>
+        </is>
+      </c>
+      <c r="D74" s="22" t="inlineStr">
+        <is>
+          <t>Recuperado v1</t>
         </is>
       </c>
       <c r="E74" s="19" t="inlineStr">
@@ -6728,7 +6768,7 @@
     <row r="75">
       <c r="A75" s="18" t="inlineStr">
         <is>
-          <t>M6-03</t>
+          <t>M6-02</t>
         </is>
       </c>
       <c r="B75" s="19" t="inlineStr">
@@ -6738,7 +6778,7 @@
       </c>
       <c r="C75" s="19" t="inlineStr">
         <is>
-          <t>Calendario de turnos: días regulares de servicio y eventos especiales.</t>
+          <t>Menú o catálogo digital interactivo (público o interno), autogestionado.</t>
         </is>
       </c>
       <c r="D75" s="19" t="inlineStr">
@@ -6792,7 +6832,7 @@
     <row r="76">
       <c r="A76" s="18" t="inlineStr">
         <is>
-          <t>M6-04</t>
+          <t>M6-03</t>
         </is>
       </c>
       <c r="B76" s="19" t="inlineStr">
@@ -6802,7 +6842,7 @@
       </c>
       <c r="C76" s="19" t="inlineStr">
         <is>
-          <t>Registro de asistentes o personas atendidas.</t>
+          <t>Calendario de turnos: días regulares de servicio y eventos especiales.</t>
         </is>
       </c>
       <c r="D76" s="19" t="inlineStr">
@@ -6856,7 +6896,7 @@
     <row r="77">
       <c r="A77" s="18" t="inlineStr">
         <is>
-          <t>M6-05</t>
+          <t>M6-04</t>
         </is>
       </c>
       <c r="B77" s="19" t="inlineStr">
@@ -6866,7 +6906,7 @@
       </c>
       <c r="C77" s="19" t="inlineStr">
         <is>
-          <t>Control de gastos y de inventario básico.</t>
+          <t>Registro de asistentes o personas atendidas.</t>
         </is>
       </c>
       <c r="D77" s="19" t="inlineStr">
@@ -6920,7 +6960,7 @@
     <row r="78">
       <c r="A78" s="18" t="inlineStr">
         <is>
-          <t>M6-06</t>
+          <t>M6-05</t>
         </is>
       </c>
       <c r="B78" s="19" t="inlineStr">
@@ -6930,7 +6970,7 @@
       </c>
       <c r="C78" s="19" t="inlineStr">
         <is>
-          <t>Canal de comunicación directo con el área de Administración General.</t>
+          <t>Control de gastos y de inventario básico.</t>
         </is>
       </c>
       <c r="D78" s="19" t="inlineStr">
@@ -6984,7 +7024,7 @@
     <row r="79">
       <c r="A79" s="18" t="inlineStr">
         <is>
-          <t>M6-07</t>
+          <t>M6-06</t>
         </is>
       </c>
       <c r="B79" s="19" t="inlineStr">
@@ -6994,12 +7034,12 @@
       </c>
       <c r="C79" s="19" t="inlineStr">
         <is>
-          <t>Servicio Médico: los datos de salud de las personas atendidas requieren tratamiento de datos sensibles. Por definir alcance.</t>
-        </is>
-      </c>
-      <c r="D79" s="21" t="inlineStr">
-        <is>
-          <t>Nuevo v3</t>
+          <t>Canal de comunicación directo con el área de Administración General.</t>
+        </is>
+      </c>
+      <c r="D79" s="19" t="inlineStr">
+        <is>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E79" s="19" t="inlineStr">
@@ -7034,7 +7074,7 @@
       </c>
       <c r="K79" s="19" t="inlineStr">
         <is>
-          <t>Por definir</t>
+          <t>VoBo pendiente</t>
         </is>
       </c>
       <c r="L79" s="19" t="inlineStr">
@@ -7048,22 +7088,22 @@
     <row r="80">
       <c r="A80" s="18" t="inlineStr">
         <is>
-          <t>M7-01</t>
+          <t>M6-07</t>
         </is>
       </c>
       <c r="B80" s="19" t="inlineStr">
         <is>
-          <t>M7 Eventos y aforo</t>
+          <t>M6 Ministerios de servicio</t>
         </is>
       </c>
       <c r="C80" s="19" t="inlineStr">
         <is>
-          <t>Eventos abiertos o evangelísticos con formulario de inscripción rápida, sin requerir historial previo.</t>
-        </is>
-      </c>
-      <c r="D80" s="19" t="inlineStr">
-        <is>
-          <t>v1 / v2</t>
+          <t>Servicio Médico: los datos de salud de las personas atendidas requieren tratamiento de datos sensibles. Por definir alcance.</t>
+        </is>
+      </c>
+      <c r="D80" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3</t>
         </is>
       </c>
       <c r="E80" s="19" t="inlineStr">
@@ -7098,7 +7138,7 @@
       </c>
       <c r="K80" s="19" t="inlineStr">
         <is>
-          <t>VoBo pendiente</t>
+          <t>Por definir</t>
         </is>
       </c>
       <c r="L80" s="19" t="inlineStr">
@@ -7112,7 +7152,7 @@
     <row r="81">
       <c r="A81" s="18" t="inlineStr">
         <is>
-          <t>M7-02</t>
+          <t>M7-01</t>
         </is>
       </c>
       <c r="B81" s="19" t="inlineStr">
@@ -7122,12 +7162,12 @@
       </c>
       <c r="C81" s="19" t="inlineStr">
         <is>
-          <t>Consolidación (inducción de personas que asisten por primera vez) como tipo de evento.</t>
-        </is>
-      </c>
-      <c r="D81" s="22" t="inlineStr">
-        <is>
-          <t>Recuperado v1</t>
+          <t>Eventos abiertos o evangelísticos con formulario de inscripción rápida, sin requerir historial previo.</t>
+        </is>
+      </c>
+      <c r="D81" s="19" t="inlineStr">
+        <is>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E81" s="19" t="inlineStr">
@@ -7176,7 +7216,7 @@
     <row r="82">
       <c r="A82" s="18" t="inlineStr">
         <is>
-          <t>M7-03</t>
+          <t>M7-02</t>
         </is>
       </c>
       <c r="B82" s="19" t="inlineStr">
@@ -7186,7 +7226,7 @@
       </c>
       <c r="C82" s="19" t="inlineStr">
         <is>
-          <t>Encargados de evento (personal de la iglesia únicamente; no se controla personal externo).</t>
+          <t>Consolidación (inducción de personas que asisten por primera vez) como tipo de evento.</t>
         </is>
       </c>
       <c r="D82" s="22" t="inlineStr">
@@ -7240,7 +7280,7 @@
     <row r="83">
       <c r="A83" s="18" t="inlineStr">
         <is>
-          <t>M7-04</t>
+          <t>M7-03</t>
         </is>
       </c>
       <c r="B83" s="19" t="inlineStr">
@@ -7250,12 +7290,12 @@
       </c>
       <c r="C83" s="19" t="inlineStr">
         <is>
-          <t>Control de cupo en tiempo real que bloquea el sobrecupo en eventos con aforo limitado (ej. 30 o 50 lugares).</t>
-        </is>
-      </c>
-      <c r="D83" s="19" t="inlineStr">
-        <is>
-          <t>v1 / v2</t>
+          <t>Encargados de evento (personal de la iglesia únicamente; no se controla personal externo).</t>
+        </is>
+      </c>
+      <c r="D83" s="22" t="inlineStr">
+        <is>
+          <t>Recuperado v1</t>
         </is>
       </c>
       <c r="E83" s="19" t="inlineStr">
@@ -7304,7 +7344,7 @@
     <row r="84">
       <c r="A84" s="18" t="inlineStr">
         <is>
-          <t>M7-05</t>
+          <t>M7-04</t>
         </is>
       </c>
       <c r="B84" s="19" t="inlineStr">
@@ -7314,12 +7354,12 @@
       </c>
       <c r="C84" s="19" t="inlineStr">
         <is>
-          <t>Control de asistentes sin lista previa, para aforo y para dar a conocer la iglesia.</t>
+          <t>Control de cupo en tiempo real que bloquea el sobrecupo en eventos con aforo limitado (ej. 30 o 50 lugares).</t>
         </is>
       </c>
       <c r="D84" s="19" t="inlineStr">
         <is>
-          <t>v1</t>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E84" s="19" t="inlineStr">
@@ -7368,7 +7408,7 @@
     <row r="85">
       <c r="A85" s="18" t="inlineStr">
         <is>
-          <t>M7-06</t>
+          <t>M7-05</t>
         </is>
       </c>
       <c r="B85" s="19" t="inlineStr">
@@ -7378,12 +7418,12 @@
       </c>
       <c r="C85" s="19" t="inlineStr">
         <is>
-          <t>Seguimiento de personas nuevas: conversión de un invitado a Expediente Digital y canalización a un curso o Grupo de Conexión.</t>
-        </is>
-      </c>
-      <c r="D85" s="21" t="inlineStr">
-        <is>
-          <t>Nuevo v3</t>
+          <t>Control de asistentes sin lista previa, para aforo y para dar a conocer la iglesia.</t>
+        </is>
+      </c>
+      <c r="D85" s="19" t="inlineStr">
+        <is>
+          <t>v1</t>
         </is>
       </c>
       <c r="E85" s="19" t="inlineStr">
@@ -7432,52 +7472,52 @@
     <row r="86">
       <c r="A86" s="18" t="inlineStr">
         <is>
-          <t>NF-01</t>
+          <t>M7-06</t>
         </is>
       </c>
       <c r="B86" s="19" t="inlineStr">
         <is>
-          <t>No funcionales</t>
+          <t>M7 Eventos y aforo</t>
         </is>
       </c>
       <c r="C86" s="19" t="inlineStr">
         <is>
-          <t>Cumplimiento de la LFPDPPP: aviso de privacidad, consentimiento y derechos ARCO.</t>
-        </is>
-      </c>
-      <c r="D86" s="19" t="inlineStr">
-        <is>
-          <t>v3</t>
+          <t>Seguimiento de personas nuevas: conversión de un invitado a Expediente Digital y canalización a un curso o Grupo de Conexión.</t>
+        </is>
+      </c>
+      <c r="D86" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3</t>
         </is>
       </c>
       <c r="E86" s="19" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Fuera del MVP</t>
         </is>
       </c>
       <c r="F86" s="19" t="inlineStr">
         <is>
-          <t>Fase 0</t>
+          <t>Fase 4</t>
         </is>
       </c>
       <c r="G86" s="19" t="inlineStr">
         <is>
-          <t>Sprint 1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H86" s="19" t="inlineStr">
         <is>
-          <t>H1 · 18-oct (núcleo Fase 0)</t>
-        </is>
-      </c>
-      <c r="I86" s="19" t="inlineStr">
-        <is>
-          <t>Como iglesia queremos cumplir con la LFPDPPP.</t>
-        </is>
-      </c>
-      <c r="J86" s="19" t="inlineStr">
-        <is>
-          <t>Aviso de privacidad, consentimiento y atención de derechos ARCO disponibles.</t>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="I86" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
+        </is>
+      </c>
+      <c r="J86" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
         </is>
       </c>
       <c r="K86" s="19" t="inlineStr">
@@ -7496,7 +7536,7 @@
     <row r="87">
       <c r="A87" s="18" t="inlineStr">
         <is>
-          <t>NF-02</t>
+          <t>NF-01</t>
         </is>
       </c>
       <c r="B87" s="19" t="inlineStr">
@@ -7506,7 +7546,7 @@
       </c>
       <c r="C87" s="19" t="inlineStr">
         <is>
-          <t>Cifrado en tránsito y en reposo. Cifrado adicional a nivel de campo para peticiones de oración.</t>
+          <t>Cumplimiento de la LFPDPPP: aviso de privacidad, consentimiento y derechos ARCO.</t>
         </is>
       </c>
       <c r="D87" s="19" t="inlineStr">
@@ -7526,7 +7566,7 @@
       </c>
       <c r="G87" s="19" t="inlineStr">
         <is>
-          <t>Sprint 0</t>
+          <t>Sprint 1</t>
         </is>
       </c>
       <c r="H87" s="19" t="inlineStr">
@@ -7536,12 +7576,12 @@
       </c>
       <c r="I87" s="19" t="inlineStr">
         <is>
-          <t>Como iglesia queremos proteger los datos sensibles.</t>
+          <t>Como iglesia queremos cumplir con la LFPDPPP.</t>
         </is>
       </c>
       <c r="J87" s="19" t="inlineStr">
         <is>
-          <t>HTTPS obligatorio y peticiones de oración ilegibles directamente en la base.</t>
+          <t>Aviso de privacidad, consentimiento y atención de derechos ARCO disponibles.</t>
         </is>
       </c>
       <c r="K87" s="19" t="inlineStr">
@@ -7560,7 +7600,7 @@
     <row r="88">
       <c r="A88" s="18" t="inlineStr">
         <is>
-          <t>NF-03</t>
+          <t>NF-02</t>
         </is>
       </c>
       <c r="B88" s="19" t="inlineStr">
@@ -7570,7 +7610,7 @@
       </c>
       <c r="C88" s="19" t="inlineStr">
         <is>
-          <t>Bitácora de auditoría de solo-añadir: quién consultó o modificó expedientes, ofrendas y asistencias.</t>
+          <t>Cifrado en tránsito y en reposo. Cifrado adicional a nivel de campo para peticiones de oración.</t>
         </is>
       </c>
       <c r="D88" s="19" t="inlineStr">
@@ -7590,7 +7630,7 @@
       </c>
       <c r="G88" s="19" t="inlineStr">
         <is>
-          <t>Sprint 1</t>
+          <t>Sprint 0</t>
         </is>
       </c>
       <c r="H88" s="19" t="inlineStr">
@@ -7600,12 +7640,12 @@
       </c>
       <c r="I88" s="19" t="inlineStr">
         <is>
-          <t>Como pastor quiero una bitácora que nadie pueda alterar.</t>
+          <t>Como iglesia queremos proteger los datos sensibles.</t>
         </is>
       </c>
       <c r="J88" s="19" t="inlineStr">
         <is>
-          <t>El usuario de la aplicación no puede actualizar ni borrar registros de bitácora.</t>
+          <t>HTTPS obligatorio y peticiones de oración ilegibles directamente en la base.</t>
         </is>
       </c>
       <c r="K88" s="19" t="inlineStr">
@@ -7615,24 +7655,16 @@
       </c>
       <c r="L88" s="19" t="inlineStr">
         <is>
-          <t>En pruebas</t>
-        </is>
-      </c>
-      <c r="M88" s="19" t="inlineStr">
-        <is>
-          <t>Rama feature/nf-03-bitacora · 69 pruebas de backend pasan</t>
-        </is>
-      </c>
-      <c r="N88" s="19" t="inlineStr">
-        <is>
-          <t>2026-10-10 · Bloqueo en aplicación y trigger de PostgreSQL (UPDATE/DELETE/TRUNCATE); pantalla de consulta con permiso bitacora.ver.</t>
-        </is>
-      </c>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M88" s="19" t="inlineStr"/>
+      <c r="N88" s="19" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="18" t="inlineStr">
         <is>
-          <t>NF-04</t>
+          <t>NF-03</t>
         </is>
       </c>
       <c r="B89" s="19" t="inlineStr">
@@ -7642,7 +7674,7 @@
       </c>
       <c r="C89" s="19" t="inlineStr">
         <is>
-          <t>Respaldos automáticos diarios cifrados y prueba periódica de restauración.</t>
+          <t>Bitácora de auditoría de solo-añadir: quién consultó o modificó expedientes, ofrendas y asistencias.</t>
         </is>
       </c>
       <c r="D89" s="19" t="inlineStr">
@@ -7662,7 +7694,7 @@
       </c>
       <c r="G89" s="19" t="inlineStr">
         <is>
-          <t>Sprint 0</t>
+          <t>Sprint 1</t>
         </is>
       </c>
       <c r="H89" s="19" t="inlineStr">
@@ -7672,12 +7704,12 @@
       </c>
       <c r="I89" s="19" t="inlineStr">
         <is>
-          <t>Como iglesia queremos no perder información.</t>
+          <t>Como pastor quiero una bitácora que nadie pueda alterar.</t>
         </is>
       </c>
       <c r="J89" s="19" t="inlineStr">
         <is>
-          <t>Respaldo diario cifrado y restauración probada en un ambiente de pruebas.</t>
+          <t>El usuario de la aplicación no puede actualizar ni borrar registros de bitácora.</t>
         </is>
       </c>
       <c r="K89" s="19" t="inlineStr">
@@ -7687,16 +7719,24 @@
       </c>
       <c r="L89" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M89" s="19" t="inlineStr"/>
-      <c r="N89" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M89" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/nf-03-bitacora · 69 pruebas de backend pasan</t>
+        </is>
+      </c>
+      <c r="N89" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-10 · Bloqueo en aplicación y trigger de PostgreSQL (UPDATE/DELETE/TRUNCATE); pantalla de consulta con permiso bitacora.ver.</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="18" t="inlineStr">
         <is>
-          <t>NF-05</t>
+          <t>NF-04</t>
         </is>
       </c>
       <c r="B90" s="19" t="inlineStr">
@@ -7706,47 +7746,47 @@
       </c>
       <c r="C90" s="19" t="inlineStr">
         <is>
-          <t>Disponibilidad esperada en horarios de servicio (fines de semana y reuniones de grupo). Por definir meta.</t>
-        </is>
-      </c>
-      <c r="D90" s="21" t="inlineStr">
-        <is>
-          <t>Nuevo v3</t>
+          <t>Respaldos automáticos diarios cifrados y prueba periódica de restauración.</t>
+        </is>
+      </c>
+      <c r="D90" s="19" t="inlineStr">
+        <is>
+          <t>v3</t>
         </is>
       </c>
       <c r="E90" s="19" t="inlineStr">
         <is>
-          <t>Fuera del MVP</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="F90" s="19" t="inlineStr">
         <is>
-          <t>Transversal</t>
+          <t>Fase 0</t>
         </is>
       </c>
       <c r="G90" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sprint 0</t>
         </is>
       </c>
       <c r="H90" s="19" t="inlineStr">
         <is>
-          <t>Posterior</t>
-        </is>
-      </c>
-      <c r="I90" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
-        </is>
-      </c>
-      <c r="J90" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
+          <t>H1 · 18-oct (núcleo Fase 0)</t>
+        </is>
+      </c>
+      <c r="I90" s="19" t="inlineStr">
+        <is>
+          <t>Como iglesia queremos no perder información.</t>
+        </is>
+      </c>
+      <c r="J90" s="19" t="inlineStr">
+        <is>
+          <t>Respaldo diario cifrado y restauración probada en un ambiente de pruebas.</t>
         </is>
       </c>
       <c r="K90" s="19" t="inlineStr">
         <is>
-          <t>Por definir</t>
+          <t>VoBo pendiente</t>
         </is>
       </c>
       <c r="L90" s="19" t="inlineStr">
@@ -7760,7 +7800,7 @@
     <row r="91">
       <c r="A91" s="18" t="inlineStr">
         <is>
-          <t>NF-06</t>
+          <t>NF-05</t>
         </is>
       </c>
       <c r="B91" s="19" t="inlineStr">
@@ -7770,47 +7810,47 @@
       </c>
       <c r="C91" s="19" t="inlineStr">
         <is>
-          <t>Pase de lista sin conexión con sincronización posterior (reuniones en domicilios con mala señal).</t>
-        </is>
-      </c>
-      <c r="D91" s="19" t="inlineStr">
-        <is>
-          <t>v3</t>
+          <t>Disponibilidad esperada en horarios de servicio (fines de semana y reuniones de grupo). Por definir meta.</t>
+        </is>
+      </c>
+      <c r="D91" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3</t>
         </is>
       </c>
       <c r="E91" s="19" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Fuera del MVP</t>
         </is>
       </c>
       <c r="F91" s="19" t="inlineStr">
         <is>
-          <t>Fase 0</t>
+          <t>Transversal</t>
         </is>
       </c>
       <c r="G91" s="19" t="inlineStr">
         <is>
-          <t>Sprint 3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H91" s="19" t="inlineStr">
         <is>
-          <t>H3 · MVP (Grupos)</t>
-        </is>
-      </c>
-      <c r="I91" s="19" t="inlineStr">
-        <is>
-          <t>Como secretario quiero que el pase de lista funcione sin señal.</t>
-        </is>
-      </c>
-      <c r="J91" s="19" t="inlineStr">
-        <is>
-          <t>Prueba en modo avión y sincronización al reconectar.</t>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="I91" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
+        </is>
+      </c>
+      <c r="J91" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
         </is>
       </c>
       <c r="K91" s="19" t="inlineStr">
         <is>
-          <t>VoBo pendiente</t>
+          <t>Por definir</t>
         </is>
       </c>
       <c r="L91" s="19" t="inlineStr">
@@ -7824,7 +7864,7 @@
     <row r="92">
       <c r="A92" s="18" t="inlineStr">
         <is>
-          <t>NF-07</t>
+          <t>NF-06</t>
         </is>
       </c>
       <c r="B92" s="19" t="inlineStr">
@@ -7834,7 +7874,7 @@
       </c>
       <c r="C92" s="19" t="inlineStr">
         <is>
-          <t>Funciona en Android, iOS y escritorio. En iOS, las notificaciones push requieren instalar la PWA; el respaldo por WhatsApp cubre el resto.</t>
+          <t>Pase de lista sin conexión con sincronización posterior (reuniones en domicilios con mala señal).</t>
         </is>
       </c>
       <c r="D92" s="19" t="inlineStr">
@@ -7854,22 +7894,22 @@
       </c>
       <c r="G92" s="19" t="inlineStr">
         <is>
-          <t>Sprint 0</t>
+          <t>Sprint 3</t>
         </is>
       </c>
       <c r="H92" s="19" t="inlineStr">
         <is>
-          <t>H1 · 18-oct (núcleo Fase 0)</t>
+          <t>H3 · MVP (Grupos)</t>
         </is>
       </c>
       <c r="I92" s="19" t="inlineStr">
         <is>
-          <t>Como usuario quiero usar el sistema en mi dispositivo.</t>
+          <t>Como secretario quiero que el pase de lista funcione sin señal.</t>
         </is>
       </c>
       <c r="J92" s="19" t="inlineStr">
         <is>
-          <t>Pruebas en Android, iOS y escritorio; push en iOS con la PWA instalada y respaldo por WhatsApp.</t>
+          <t>Prueba en modo avión y sincronización al reconectar.</t>
         </is>
       </c>
       <c r="K92" s="19" t="inlineStr">
@@ -7888,7 +7928,7 @@
     <row r="93">
       <c r="A93" s="18" t="inlineStr">
         <is>
-          <t>NF-08</t>
+          <t>NF-07</t>
         </is>
       </c>
       <c r="B93" s="19" t="inlineStr">
@@ -7898,12 +7938,12 @@
       </c>
       <c r="C93" s="19" t="inlineStr">
         <is>
-          <t>Dimensionamiento para ~1,000 personas, con picos los fines de semana, y margen de crecimiento.</t>
-        </is>
-      </c>
-      <c r="D93" s="21" t="inlineStr">
-        <is>
-          <t>Resp. P8</t>
+          <t>Funciona en Android, iOS y escritorio. En iOS, las notificaciones push requieren instalar la PWA; el respaldo por WhatsApp cubre el resto.</t>
+        </is>
+      </c>
+      <c r="D93" s="19" t="inlineStr">
+        <is>
+          <t>v3</t>
         </is>
       </c>
       <c r="E93" s="19" t="inlineStr">
@@ -7928,12 +7968,12 @@
       </c>
       <c r="I93" s="19" t="inlineStr">
         <is>
-          <t>Como iglesia queremos que el sistema soporte a ~1,000 personas.</t>
+          <t>Como usuario quiero usar el sistema en mi dispositivo.</t>
         </is>
       </c>
       <c r="J93" s="19" t="inlineStr">
         <is>
-          <t>Prueba de carga con volumen representativo (por definir) sin degradación.</t>
+          <t>Pruebas en Android, iOS y escritorio; push en iOS con la PWA instalada y respaldo por WhatsApp.</t>
         </is>
       </c>
       <c r="K93" s="19" t="inlineStr">
@@ -7952,7 +7992,7 @@
     <row r="94">
       <c r="A94" s="18" t="inlineStr">
         <is>
-          <t>NF-09</t>
+          <t>NF-08</t>
         </is>
       </c>
       <c r="B94" s="19" t="inlineStr">
@@ -7962,42 +8002,42 @@
       </c>
       <c r="C94" s="19" t="inlineStr">
         <is>
-          <t>Reportes transversales: asistencia, finanzas, crecimiento de la iglesia, exportables a Excel y PDF.</t>
+          <t>Dimensionamiento para ~1,000 personas, con picos los fines de semana, y margen de crecimiento.</t>
         </is>
       </c>
       <c r="D94" s="21" t="inlineStr">
         <is>
-          <t>Nuevo v3</t>
+          <t>Resp. P8</t>
         </is>
       </c>
       <c r="E94" s="19" t="inlineStr">
         <is>
-          <t>Fuera del MVP</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="F94" s="19" t="inlineStr">
         <is>
-          <t>Transversal</t>
+          <t>Fase 0</t>
         </is>
       </c>
       <c r="G94" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sprint 0</t>
         </is>
       </c>
       <c r="H94" s="19" t="inlineStr">
         <is>
-          <t>Posterior</t>
-        </is>
-      </c>
-      <c r="I94" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
-        </is>
-      </c>
-      <c r="J94" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
+          <t>H1 · 18-oct (núcleo Fase 0)</t>
+        </is>
+      </c>
+      <c r="I94" s="19" t="inlineStr">
+        <is>
+          <t>Como iglesia queremos que el sistema soporte a ~1,000 personas.</t>
+        </is>
+      </c>
+      <c r="J94" s="19" t="inlineStr">
+        <is>
+          <t>Prueba de carga con volumen representativo (por definir) sin degradación.</t>
         </is>
       </c>
       <c r="K94" s="19" t="inlineStr">
@@ -8016,7 +8056,7 @@
     <row r="95">
       <c r="A95" s="18" t="inlineStr">
         <is>
-          <t>NF-10</t>
+          <t>NF-09</t>
         </is>
       </c>
       <c r="B95" s="19" t="inlineStr">
@@ -8026,42 +8066,42 @@
       </c>
       <c r="C95" s="19" t="inlineStr">
         <is>
-          <t>Usabilidad para personas mayores: tipografía grande, alto contraste, flujos cortos (ver sección 5).</t>
-        </is>
-      </c>
-      <c r="D95" s="19" t="inlineStr">
-        <is>
-          <t>v3 + Obs. 1</t>
+          <t>Reportes transversales: asistencia, finanzas, crecimiento de la iglesia, exportables a Excel y PDF.</t>
+        </is>
+      </c>
+      <c r="D95" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3</t>
         </is>
       </c>
       <c r="E95" s="19" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Fuera del MVP</t>
         </is>
       </c>
       <c r="F95" s="19" t="inlineStr">
         <is>
-          <t>Fase 0</t>
+          <t>Transversal</t>
         </is>
       </c>
       <c r="G95" s="19" t="inlineStr">
         <is>
-          <t>Sprint 0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H95" s="19" t="inlineStr">
         <is>
-          <t>H1 · 18-oct (núcleo Fase 0)</t>
-        </is>
-      </c>
-      <c r="I95" s="19" t="inlineStr">
-        <is>
-          <t>Como persona mayor quiero una interfaz fácil de leer y usar.</t>
-        </is>
-      </c>
-      <c r="J95" s="19" t="inlineStr">
-        <is>
-          <t>Texto base 18 px, botones de al menos 48 px, contraste AA; prueba con usuarios mayores.</t>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="I95" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
+        </is>
+      </c>
+      <c r="J95" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
         </is>
       </c>
       <c r="K95" s="19" t="inlineStr">
@@ -8077,9 +8117,73 @@
       <c r="M95" s="19" t="inlineStr"/>
       <c r="N95" s="19" t="inlineStr"/>
     </row>
+    <row r="96">
+      <c r="A96" s="18" t="inlineStr">
+        <is>
+          <t>NF-10</t>
+        </is>
+      </c>
+      <c r="B96" s="19" t="inlineStr">
+        <is>
+          <t>No funcionales</t>
+        </is>
+      </c>
+      <c r="C96" s="19" t="inlineStr">
+        <is>
+          <t>Usabilidad para personas mayores: tipografía grande, alto contraste, flujos cortos (ver sección 5).</t>
+        </is>
+      </c>
+      <c r="D96" s="19" t="inlineStr">
+        <is>
+          <t>v3 + Obs. 1</t>
+        </is>
+      </c>
+      <c r="E96" s="19" t="inlineStr">
+        <is>
+          <t>MVP</t>
+        </is>
+      </c>
+      <c r="F96" s="19" t="inlineStr">
+        <is>
+          <t>Fase 0</t>
+        </is>
+      </c>
+      <c r="G96" s="19" t="inlineStr">
+        <is>
+          <t>Sprint 0</t>
+        </is>
+      </c>
+      <c r="H96" s="19" t="inlineStr">
+        <is>
+          <t>H1 · 18-oct (núcleo Fase 0)</t>
+        </is>
+      </c>
+      <c r="I96" s="19" t="inlineStr">
+        <is>
+          <t>Como persona mayor quiero una interfaz fácil de leer y usar.</t>
+        </is>
+      </c>
+      <c r="J96" s="19" t="inlineStr">
+        <is>
+          <t>Texto base 18 px, botones de al menos 48 px, contraste AA; prueba con usuarios mayores.</t>
+        </is>
+      </c>
+      <c r="K96" s="19" t="inlineStr">
+        <is>
+          <t>VoBo pendiente</t>
+        </is>
+      </c>
+      <c r="L96" s="19" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M96" s="19" t="inlineStr"/>
+      <c r="N96" s="19" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N95"/>
-  <conditionalFormatting sqref="L2:L95">
+  <autoFilter ref="A1:N96"/>
+  <conditionalFormatting sqref="L2:L96">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$L2="Hecho"</formula>
     </cfRule>
@@ -8096,7 +8200,7 @@
       <formula>$L2="Bloqueado"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K2:K95">
+  <conditionalFormatting sqref="K2:K96">
     <cfRule type="expression" priority="6" dxfId="0">
       <formula>$K2="Aprobado"</formula>
     </cfRule>
@@ -8104,16 +8208,16 @@
       <formula>$K2="Por definir"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H2:H95">
+  <conditionalFormatting sqref="H2:H96">
     <cfRule type="expression" priority="8" dxfId="5">
       <formula>LEFT($H2,2)="H1"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="L2:L95" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="L2:L96" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Pendiente,En diseño,En desarrollo,En pruebas,Hecho,Bloqueado"</formula1>
     </dataValidation>
-    <dataValidation sqref="K2:K95" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="K2:K96" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"VoBo pendiente,Aprobado,Por definir,Rechazado"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
M3-04: ofrendas del grupo con aval del Tesorero
- Ofrenda regular o especial por reunión; captura del Secretario (Pastor por excepción)
- El Tesorero cuenta, escribe su cifra y avala reescribiendo su PIN (con bloqueo por intentos);
  la diferencia queda registrada; nadie avala su propia captura
- Corrección con motivo, vuelve a pendiente y exige nuevo aval; historial de movimientos
- Confidencialidad según la matriz: Líder y Supervisor consultan, Pastor ve todo, Anciano sin finanzas
- Todo en bitácora; pantallas de captura en la reunión y de ofrendas por avalar
- Documentación v3.6 y matriz de trazabilidad

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/trazabilidad/Matriz de Trazabilidad MDF.xlsx
+++ b/docs/trazabilidad/Matriz de Trazabilidad MDF.xlsx
@@ -5226,7 +5226,7 @@
       </c>
       <c r="C51" s="19" t="inlineStr">
         <is>
-          <t>Ofrendas regulares y especiales. El Tesorero cuenta y avala la cifra con firma electrónica simple (usuario, fecha y hora, monto y reingreso de su PIN). Si su cifra difiere de la capturada, se registra la diferencia.</t>
+          <t>Ofrendas regulares y especiales (con concepto) por reunión, cuantificables. El Secretario captura el monto; el Tesorero cuenta, escribe su cifra y avala volviendo a escribir su PIN. Si su cifra coincide queda «Avalada»; si no, se registra la diferencia y queda «Con diferencia». Una ofrenda ya capturada solo se corrige con motivo y vuelve a pendiente para un nuevo aval. Quien capturó no puede avalar su propia captura. Líder y Supervisor solo consultan, el Pastor consulta todo y el Anciano no ve finanzas. Todo movimiento queda en bitácora.</t>
         </is>
       </c>
       <c r="D51" s="19" t="inlineStr">
@@ -5271,11 +5271,19 @@
       </c>
       <c r="L51" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M51" s="19" t="inlineStr"/>
-      <c r="N51" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M51" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/m3-ofrendas · 111 pruebas de backend y 14 de frontend pasan</t>
+        </is>
+      </c>
+      <c r="N51" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-24 · Probado de punta a punta con Secretaria y Tesorero distintos; falta validarlo con la iglesia (por ejemplo, qué pasa si el grupo no tiene Secretario).</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="18" t="inlineStr">

</xml_diff>

<commit_message>
M3-04/M3-13: suplencias del Líder, diferencias visibles y parámetros configurables
- El Líder captura si el grupo no tiene Secretario y avala si no tiene Tesorero (nunca su propia
  captura; el Pastor también puede avalar). Toda suplencia queda marcada en movimientos y bitácora
- Aviso visible de ofrendas con diferencia en la lista y el detalle del grupo, la reunión y la
  pantalla del Tesorero, para quien puede consultar
- Parámetros configurables (monto máximo y una regular por reunión) con pantalla de Configuración,
  permiso config.gestionar y cada cambio en bitácora
- Se retira la restricción única en base de datos: la regla ahora es configurable
- Documentación v3.7 y matriz de trazabilidad

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/trazabilidad/Matriz de Trazabilidad MDF.xlsx
+++ b/docs/trazabilidad/Matriz de Trazabilidad MDF.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Origen v1" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Matriz'!$A$1:$N$96</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Matriz'!$A$1:$N$97</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -897,31 +897,31 @@
         </is>
       </c>
       <c r="B5" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$96,$A5)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$97,$A5)</f>
         <v/>
       </c>
       <c r="C5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A5,Matriz!$L$2:$L$96,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A5,Matriz!$L$2:$L$97,"Pendiente")</f>
         <v/>
       </c>
       <c r="D5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A5,Matriz!$L$2:$L$96,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A5,Matriz!$L$2:$L$97,"En diseño")</f>
         <v/>
       </c>
       <c r="E5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A5,Matriz!$L$2:$L$96,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A5,Matriz!$L$2:$L$97,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A5,Matriz!$L$2:$L$96,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A5,Matriz!$L$2:$L$97,"En pruebas")</f>
         <v/>
       </c>
       <c r="G5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A5,Matriz!$L$2:$L$96,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A5,Matriz!$L$2:$L$97,"Hecho")</f>
         <v/>
       </c>
       <c r="H5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A5,Matriz!$L$2:$L$96,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A5,Matriz!$L$2:$L$97,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I5" s="13">
@@ -936,31 +936,31 @@
         </is>
       </c>
       <c r="B6" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$96,$A6)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$97,$A6)</f>
         <v/>
       </c>
       <c r="C6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A6,Matriz!$L$2:$L$96,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A6,Matriz!$L$2:$L$97,"Pendiente")</f>
         <v/>
       </c>
       <c r="D6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A6,Matriz!$L$2:$L$96,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A6,Matriz!$L$2:$L$97,"En diseño")</f>
         <v/>
       </c>
       <c r="E6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A6,Matriz!$L$2:$L$96,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A6,Matriz!$L$2:$L$97,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A6,Matriz!$L$2:$L$96,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A6,Matriz!$L$2:$L$97,"En pruebas")</f>
         <v/>
       </c>
       <c r="G6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A6,Matriz!$L$2:$L$96,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A6,Matriz!$L$2:$L$97,"Hecho")</f>
         <v/>
       </c>
       <c r="H6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A6,Matriz!$L$2:$L$96,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A6,Matriz!$L$2:$L$97,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I6" s="13">
@@ -975,31 +975,31 @@
         </is>
       </c>
       <c r="B7" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$96,$A7)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$97,$A7)</f>
         <v/>
       </c>
       <c r="C7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A7,Matriz!$L$2:$L$96,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A7,Matriz!$L$2:$L$97,"Pendiente")</f>
         <v/>
       </c>
       <c r="D7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A7,Matriz!$L$2:$L$96,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A7,Matriz!$L$2:$L$97,"En diseño")</f>
         <v/>
       </c>
       <c r="E7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A7,Matriz!$L$2:$L$96,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A7,Matriz!$L$2:$L$97,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A7,Matriz!$L$2:$L$96,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A7,Matriz!$L$2:$L$97,"En pruebas")</f>
         <v/>
       </c>
       <c r="G7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A7,Matriz!$L$2:$L$96,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A7,Matriz!$L$2:$L$97,"Hecho")</f>
         <v/>
       </c>
       <c r="H7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A7,Matriz!$L$2:$L$96,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A7,Matriz!$L$2:$L$97,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I7" s="13">
@@ -1014,31 +1014,31 @@
         </is>
       </c>
       <c r="B8" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$96,$A8)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$97,$A8)</f>
         <v/>
       </c>
       <c r="C8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A8,Matriz!$L$2:$L$96,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A8,Matriz!$L$2:$L$97,"Pendiente")</f>
         <v/>
       </c>
       <c r="D8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A8,Matriz!$L$2:$L$96,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A8,Matriz!$L$2:$L$97,"En diseño")</f>
         <v/>
       </c>
       <c r="E8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A8,Matriz!$L$2:$L$96,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A8,Matriz!$L$2:$L$97,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A8,Matriz!$L$2:$L$96,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A8,Matriz!$L$2:$L$97,"En pruebas")</f>
         <v/>
       </c>
       <c r="G8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A8,Matriz!$L$2:$L$96,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A8,Matriz!$L$2:$L$97,"Hecho")</f>
         <v/>
       </c>
       <c r="H8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A8,Matriz!$L$2:$L$96,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A8,Matriz!$L$2:$L$97,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I8" s="13">
@@ -1053,31 +1053,31 @@
         </is>
       </c>
       <c r="B9" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$96,$A9)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$97,$A9)</f>
         <v/>
       </c>
       <c r="C9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A9,Matriz!$L$2:$L$96,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A9,Matriz!$L$2:$L$97,"Pendiente")</f>
         <v/>
       </c>
       <c r="D9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A9,Matriz!$L$2:$L$96,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A9,Matriz!$L$2:$L$97,"En diseño")</f>
         <v/>
       </c>
       <c r="E9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A9,Matriz!$L$2:$L$96,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A9,Matriz!$L$2:$L$97,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A9,Matriz!$L$2:$L$96,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A9,Matriz!$L$2:$L$97,"En pruebas")</f>
         <v/>
       </c>
       <c r="G9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A9,Matriz!$L$2:$L$96,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A9,Matriz!$L$2:$L$97,"Hecho")</f>
         <v/>
       </c>
       <c r="H9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A9,Matriz!$L$2:$L$96,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A9,Matriz!$L$2:$L$97,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I9" s="13">
@@ -1092,31 +1092,31 @@
         </is>
       </c>
       <c r="B10" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$96,$A10)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$97,$A10)</f>
         <v/>
       </c>
       <c r="C10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A10,Matriz!$L$2:$L$96,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A10,Matriz!$L$2:$L$97,"Pendiente")</f>
         <v/>
       </c>
       <c r="D10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A10,Matriz!$L$2:$L$96,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A10,Matriz!$L$2:$L$97,"En diseño")</f>
         <v/>
       </c>
       <c r="E10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A10,Matriz!$L$2:$L$96,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A10,Matriz!$L$2:$L$97,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A10,Matriz!$L$2:$L$96,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A10,Matriz!$L$2:$L$97,"En pruebas")</f>
         <v/>
       </c>
       <c r="G10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A10,Matriz!$L$2:$L$96,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A10,Matriz!$L$2:$L$97,"Hecho")</f>
         <v/>
       </c>
       <c r="H10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A10,Matriz!$L$2:$L$96,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A10,Matriz!$L$2:$L$97,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I10" s="13">
@@ -1131,31 +1131,31 @@
         </is>
       </c>
       <c r="B11" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$96,$A11)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$97,$A11)</f>
         <v/>
       </c>
       <c r="C11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A11,Matriz!$L$2:$L$96,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A11,Matriz!$L$2:$L$97,"Pendiente")</f>
         <v/>
       </c>
       <c r="D11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A11,Matriz!$L$2:$L$96,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A11,Matriz!$L$2:$L$97,"En diseño")</f>
         <v/>
       </c>
       <c r="E11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A11,Matriz!$L$2:$L$96,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A11,Matriz!$L$2:$L$97,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A11,Matriz!$L$2:$L$96,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A11,Matriz!$L$2:$L$97,"En pruebas")</f>
         <v/>
       </c>
       <c r="G11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A11,Matriz!$L$2:$L$96,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A11,Matriz!$L$2:$L$97,"Hecho")</f>
         <v/>
       </c>
       <c r="H11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A11,Matriz!$L$2:$L$96,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A11,Matriz!$L$2:$L$97,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I11" s="13">
@@ -1256,31 +1256,31 @@
         </is>
       </c>
       <c r="B16" s="12">
-        <f>COUNTIF(Matriz!$H$2:$H$96,$A16)</f>
+        <f>COUNTIF(Matriz!$H$2:$H$97,$A16)</f>
         <v/>
       </c>
       <c r="C16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$96,$A16,Matriz!$L$2:$L$96,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$97,$A16,Matriz!$L$2:$L$97,"Pendiente")</f>
         <v/>
       </c>
       <c r="D16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$96,$A16,Matriz!$L$2:$L$96,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$97,$A16,Matriz!$L$2:$L$97,"En diseño")</f>
         <v/>
       </c>
       <c r="E16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$96,$A16,Matriz!$L$2:$L$96,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$97,$A16,Matriz!$L$2:$L$97,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$96,$A16,Matriz!$L$2:$L$96,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$97,$A16,Matriz!$L$2:$L$97,"En pruebas")</f>
         <v/>
       </c>
       <c r="G16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$96,$A16,Matriz!$L$2:$L$96,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$97,$A16,Matriz!$L$2:$L$97,"Hecho")</f>
         <v/>
       </c>
       <c r="H16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$96,$A16,Matriz!$L$2:$L$96,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$97,$A16,Matriz!$L$2:$L$97,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I16" s="13">
@@ -1295,31 +1295,31 @@
         </is>
       </c>
       <c r="B17" s="12">
-        <f>COUNTIF(Matriz!$H$2:$H$96,$A17)</f>
+        <f>COUNTIF(Matriz!$H$2:$H$97,$A17)</f>
         <v/>
       </c>
       <c r="C17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$96,$A17,Matriz!$L$2:$L$96,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$97,$A17,Matriz!$L$2:$L$97,"Pendiente")</f>
         <v/>
       </c>
       <c r="D17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$96,$A17,Matriz!$L$2:$L$96,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$97,$A17,Matriz!$L$2:$L$97,"En diseño")</f>
         <v/>
       </c>
       <c r="E17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$96,$A17,Matriz!$L$2:$L$96,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$97,$A17,Matriz!$L$2:$L$97,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$96,$A17,Matriz!$L$2:$L$96,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$97,$A17,Matriz!$L$2:$L$97,"En pruebas")</f>
         <v/>
       </c>
       <c r="G17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$96,$A17,Matriz!$L$2:$L$96,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$97,$A17,Matriz!$L$2:$L$97,"Hecho")</f>
         <v/>
       </c>
       <c r="H17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$96,$A17,Matriz!$L$2:$L$96,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$97,$A17,Matriz!$L$2:$L$97,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I17" s="13">
@@ -1334,31 +1334,31 @@
         </is>
       </c>
       <c r="B18" s="12">
-        <f>COUNTIF(Matriz!$H$2:$H$96,$A18)</f>
+        <f>COUNTIF(Matriz!$H$2:$H$97,$A18)</f>
         <v/>
       </c>
       <c r="C18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$96,$A18,Matriz!$L$2:$L$96,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$97,$A18,Matriz!$L$2:$L$97,"Pendiente")</f>
         <v/>
       </c>
       <c r="D18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$96,$A18,Matriz!$L$2:$L$96,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$97,$A18,Matriz!$L$2:$L$97,"En diseño")</f>
         <v/>
       </c>
       <c r="E18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$96,$A18,Matriz!$L$2:$L$96,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$97,$A18,Matriz!$L$2:$L$97,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$96,$A18,Matriz!$L$2:$L$96,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$97,$A18,Matriz!$L$2:$L$97,"En pruebas")</f>
         <v/>
       </c>
       <c r="G18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$96,$A18,Matriz!$L$2:$L$96,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$97,$A18,Matriz!$L$2:$L$97,"Hecho")</f>
         <v/>
       </c>
       <c r="H18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$96,$A18,Matriz!$L$2:$L$96,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$97,$A18,Matriz!$L$2:$L$97,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I18" s="13">
@@ -1373,31 +1373,31 @@
         </is>
       </c>
       <c r="B19" s="12">
-        <f>COUNTIF(Matriz!$H$2:$H$96,$A19)</f>
+        <f>COUNTIF(Matriz!$H$2:$H$97,$A19)</f>
         <v/>
       </c>
       <c r="C19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$96,$A19,Matriz!$L$2:$L$96,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$97,$A19,Matriz!$L$2:$L$97,"Pendiente")</f>
         <v/>
       </c>
       <c r="D19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$96,$A19,Matriz!$L$2:$L$96,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$97,$A19,Matriz!$L$2:$L$97,"En diseño")</f>
         <v/>
       </c>
       <c r="E19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$96,$A19,Matriz!$L$2:$L$96,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$97,$A19,Matriz!$L$2:$L$97,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$96,$A19,Matriz!$L$2:$L$96,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$97,$A19,Matriz!$L$2:$L$97,"En pruebas")</f>
         <v/>
       </c>
       <c r="G19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$96,$A19,Matriz!$L$2:$L$96,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$97,$A19,Matriz!$L$2:$L$97,"Hecho")</f>
         <v/>
       </c>
       <c r="H19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$96,$A19,Matriz!$L$2:$L$96,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$97,$A19,Matriz!$L$2:$L$97,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I19" s="13">
@@ -1498,31 +1498,31 @@
         </is>
       </c>
       <c r="B24" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$96,$A24)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$97,$A24)</f>
         <v/>
       </c>
       <c r="C24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A24,Matriz!$L$2:$L$96,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A24,Matriz!$L$2:$L$97,"Pendiente")</f>
         <v/>
       </c>
       <c r="D24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A24,Matriz!$L$2:$L$96,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A24,Matriz!$L$2:$L$97,"En diseño")</f>
         <v/>
       </c>
       <c r="E24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A24,Matriz!$L$2:$L$96,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A24,Matriz!$L$2:$L$97,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A24,Matriz!$L$2:$L$96,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A24,Matriz!$L$2:$L$97,"En pruebas")</f>
         <v/>
       </c>
       <c r="G24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A24,Matriz!$L$2:$L$96,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A24,Matriz!$L$2:$L$97,"Hecho")</f>
         <v/>
       </c>
       <c r="H24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A24,Matriz!$L$2:$L$96,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A24,Matriz!$L$2:$L$97,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I24" s="13">
@@ -1537,31 +1537,31 @@
         </is>
       </c>
       <c r="B25" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$96,$A25)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$97,$A25)</f>
         <v/>
       </c>
       <c r="C25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A25,Matriz!$L$2:$L$96,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A25,Matriz!$L$2:$L$97,"Pendiente")</f>
         <v/>
       </c>
       <c r="D25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A25,Matriz!$L$2:$L$96,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A25,Matriz!$L$2:$L$97,"En diseño")</f>
         <v/>
       </c>
       <c r="E25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A25,Matriz!$L$2:$L$96,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A25,Matriz!$L$2:$L$97,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A25,Matriz!$L$2:$L$96,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A25,Matriz!$L$2:$L$97,"En pruebas")</f>
         <v/>
       </c>
       <c r="G25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A25,Matriz!$L$2:$L$96,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A25,Matriz!$L$2:$L$97,"Hecho")</f>
         <v/>
       </c>
       <c r="H25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A25,Matriz!$L$2:$L$96,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A25,Matriz!$L$2:$L$97,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I25" s="13">
@@ -1576,31 +1576,31 @@
         </is>
       </c>
       <c r="B26" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$96,$A26)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$97,$A26)</f>
         <v/>
       </c>
       <c r="C26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A26,Matriz!$L$2:$L$96,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A26,Matriz!$L$2:$L$97,"Pendiente")</f>
         <v/>
       </c>
       <c r="D26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A26,Matriz!$L$2:$L$96,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A26,Matriz!$L$2:$L$97,"En diseño")</f>
         <v/>
       </c>
       <c r="E26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A26,Matriz!$L$2:$L$96,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A26,Matriz!$L$2:$L$97,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A26,Matriz!$L$2:$L$96,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A26,Matriz!$L$2:$L$97,"En pruebas")</f>
         <v/>
       </c>
       <c r="G26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A26,Matriz!$L$2:$L$96,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A26,Matriz!$L$2:$L$97,"Hecho")</f>
         <v/>
       </c>
       <c r="H26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A26,Matriz!$L$2:$L$96,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A26,Matriz!$L$2:$L$97,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I26" s="13">
@@ -1615,31 +1615,31 @@
         </is>
       </c>
       <c r="B27" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$96,$A27)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$97,$A27)</f>
         <v/>
       </c>
       <c r="C27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A27,Matriz!$L$2:$L$96,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A27,Matriz!$L$2:$L$97,"Pendiente")</f>
         <v/>
       </c>
       <c r="D27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A27,Matriz!$L$2:$L$96,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A27,Matriz!$L$2:$L$97,"En diseño")</f>
         <v/>
       </c>
       <c r="E27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A27,Matriz!$L$2:$L$96,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A27,Matriz!$L$2:$L$97,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A27,Matriz!$L$2:$L$96,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A27,Matriz!$L$2:$L$97,"En pruebas")</f>
         <v/>
       </c>
       <c r="G27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A27,Matriz!$L$2:$L$96,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A27,Matriz!$L$2:$L$97,"Hecho")</f>
         <v/>
       </c>
       <c r="H27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A27,Matriz!$L$2:$L$96,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A27,Matriz!$L$2:$L$97,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I27" s="13">
@@ -1654,31 +1654,31 @@
         </is>
       </c>
       <c r="B28" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$96,$A28)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$97,$A28)</f>
         <v/>
       </c>
       <c r="C28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A28,Matriz!$L$2:$L$96,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A28,Matriz!$L$2:$L$97,"Pendiente")</f>
         <v/>
       </c>
       <c r="D28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A28,Matriz!$L$2:$L$96,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A28,Matriz!$L$2:$L$97,"En diseño")</f>
         <v/>
       </c>
       <c r="E28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A28,Matriz!$L$2:$L$96,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A28,Matriz!$L$2:$L$97,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A28,Matriz!$L$2:$L$96,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A28,Matriz!$L$2:$L$97,"En pruebas")</f>
         <v/>
       </c>
       <c r="G28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A28,Matriz!$L$2:$L$96,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A28,Matriz!$L$2:$L$97,"Hecho")</f>
         <v/>
       </c>
       <c r="H28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A28,Matriz!$L$2:$L$96,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A28,Matriz!$L$2:$L$97,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I28" s="13">
@@ -1693,31 +1693,31 @@
         </is>
       </c>
       <c r="B29" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$96,$A29)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$97,$A29)</f>
         <v/>
       </c>
       <c r="C29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A29,Matriz!$L$2:$L$96,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A29,Matriz!$L$2:$L$97,"Pendiente")</f>
         <v/>
       </c>
       <c r="D29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A29,Matriz!$L$2:$L$96,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A29,Matriz!$L$2:$L$97,"En diseño")</f>
         <v/>
       </c>
       <c r="E29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A29,Matriz!$L$2:$L$96,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A29,Matriz!$L$2:$L$97,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A29,Matriz!$L$2:$L$96,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A29,Matriz!$L$2:$L$97,"En pruebas")</f>
         <v/>
       </c>
       <c r="G29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A29,Matriz!$L$2:$L$96,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A29,Matriz!$L$2:$L$97,"Hecho")</f>
         <v/>
       </c>
       <c r="H29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A29,Matriz!$L$2:$L$96,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A29,Matriz!$L$2:$L$97,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I29" s="13">
@@ -1732,31 +1732,31 @@
         </is>
       </c>
       <c r="B30" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$96,$A30)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$97,$A30)</f>
         <v/>
       </c>
       <c r="C30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A30,Matriz!$L$2:$L$96,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A30,Matriz!$L$2:$L$97,"Pendiente")</f>
         <v/>
       </c>
       <c r="D30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A30,Matriz!$L$2:$L$96,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A30,Matriz!$L$2:$L$97,"En diseño")</f>
         <v/>
       </c>
       <c r="E30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A30,Matriz!$L$2:$L$96,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A30,Matriz!$L$2:$L$97,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A30,Matriz!$L$2:$L$96,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A30,Matriz!$L$2:$L$97,"En pruebas")</f>
         <v/>
       </c>
       <c r="G30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A30,Matriz!$L$2:$L$96,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A30,Matriz!$L$2:$L$97,"Hecho")</f>
         <v/>
       </c>
       <c r="H30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A30,Matriz!$L$2:$L$96,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A30,Matriz!$L$2:$L$97,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I30" s="13">
@@ -1818,7 +1818,7 @@
         </is>
       </c>
       <c r="B35" s="12">
-        <f>COUNTIF(Matriz!$K$2:$K$96,A35)</f>
+        <f>COUNTIF(Matriz!$K$2:$K$97,A35)</f>
         <v/>
       </c>
     </row>
@@ -1829,7 +1829,7 @@
         </is>
       </c>
       <c r="B36" s="12">
-        <f>COUNTIF(Matriz!$K$2:$K$96,A36)</f>
+        <f>COUNTIF(Matriz!$K$2:$K$97,A36)</f>
         <v/>
       </c>
     </row>
@@ -1840,7 +1840,7 @@
         </is>
       </c>
       <c r="B37" s="12">
-        <f>COUNTIF(Matriz!$K$2:$K$96,A37)</f>
+        <f>COUNTIF(Matriz!$K$2:$K$97,A37)</f>
         <v/>
       </c>
     </row>
@@ -1851,7 +1851,7 @@
         </is>
       </c>
       <c r="B38" s="12">
-        <f>COUNTIF(Matriz!$K$2:$K$96,A38)</f>
+        <f>COUNTIF(Matriz!$K$2:$K$97,A38)</f>
         <v/>
       </c>
     </row>
@@ -1866,7 +1866,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N96"/>
+  <dimension ref="A1:N97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5226,7 +5226,7 @@
       </c>
       <c r="C51" s="19" t="inlineStr">
         <is>
-          <t>Ofrendas regulares y especiales (con concepto) por reunión, cuantificables. El Secretario captura el monto; el Tesorero cuenta, escribe su cifra y avala volviendo a escribir su PIN. Si su cifra coincide queda «Avalada»; si no, se registra la diferencia y queda «Con diferencia». Una ofrenda ya capturada solo se corrige con motivo y vuelve a pendiente para un nuevo aval. Quien capturó no puede avalar su propia captura. Líder y Supervisor solo consultan, el Pastor consulta todo y el Anciano no ve finanzas. Todo movimiento queda en bitácora.</t>
+          <t>Ofrendas regulares y especiales (con concepto) por reunión, cuantificables. El Secretario captura el monto; si el grupo no tiene Secretario, lo suple el Líder. El Tesorero cuenta, escribe su cifra y avala volviendo a escribir su PIN; si el grupo no tiene Tesorero, avalan el Líder o el Pastor, nunca quien capturó. Si la cifra coincide queda «Avalada»; si no, se registra la diferencia y queda «Con diferencia», con aviso visible en el grupo, la reunión y la pantalla del Tesorero para quien pueda consultar. Una ofrenda ya capturada solo se corrige con motivo y vuelve a pendiente para un nuevo aval. El Pastor consulta todo, el Líder y el Supervisor consultan y el Anciano no ve finanzas. Toda suplencia, captura, aval y corrección queda en bitácora.</t>
         </is>
       </c>
       <c r="D51" s="19" t="inlineStr">
@@ -5276,12 +5276,12 @@
       </c>
       <c r="M51" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/m3-ofrendas · 111 pruebas de backend y 14 de frontend pasan</t>
+          <t>Rama feature/m3-ofrendas-ajustes · 121 pruebas de backend y 14 de frontend pasan</t>
         </is>
       </c>
       <c r="N51" s="19" t="inlineStr">
         <is>
-          <t>2026-10-24 · Probado de punta a punta con Secretaria y Tesorero distintos; falta validarlo con la iglesia (por ejemplo, qué pasa si el grupo no tiene Secretario).</t>
+          <t>2026-10-24 · Con suplencias del Líder, diferencias visibles y límites configurables. Falta validar con la iglesia.</t>
         </is>
       </c>
     </row>
@@ -5816,42 +5816,42 @@
     <row r="60">
       <c r="A60" s="18" t="inlineStr">
         <is>
-          <t>M4-01</t>
+          <t>M3-13</t>
         </is>
       </c>
       <c r="B60" s="19" t="inlineStr">
         <is>
-          <t>M4 Kids Check-In/Out</t>
+          <t>M3 Grupos de Conexión</t>
         </is>
       </c>
       <c r="C60" s="19" t="inlineStr">
         <is>
-          <t>Sustitución de la ficha física de papel.</t>
-        </is>
-      </c>
-      <c r="D60" s="19" t="inlineStr">
-        <is>
-          <t>v1 / v2</t>
+          <t>Parámetros configurables sin programar, con pantalla de Configuración y cada cambio en bitácora: monto máximo por ofrenda (1,000,000 por defecto) y si se permite una sola ofrenda regular por reunión. Solo Pastor y Administrador Técnico.</t>
+        </is>
+      </c>
+      <c r="D60" s="21" t="inlineStr">
+        <is>
+          <t>Respuesta</t>
         </is>
       </c>
       <c r="E60" s="19" t="inlineStr">
         <is>
-          <t>Fuera del MVP</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="F60" s="19" t="inlineStr">
         <is>
-          <t>Fase 2</t>
+          <t>Fase 1</t>
         </is>
       </c>
       <c r="G60" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sprint 4</t>
         </is>
       </c>
       <c r="H60" s="19" t="inlineStr">
         <is>
-          <t>Posterior</t>
+          <t>H3 · MVP (Grupos)</t>
         </is>
       </c>
       <c r="I60" s="20" t="inlineStr">
@@ -5871,16 +5871,24 @@
       </c>
       <c r="L60" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M60" s="19" t="inlineStr"/>
-      <c r="N60" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M60" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/m3-ofrendas-ajustes · 121 pruebas de backend y 14 de frontend pasan</t>
+        </is>
+      </c>
+      <c r="N60" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-24 · Pantalla Configuración: monto máximo y una regular por reunión.</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="18" t="inlineStr">
         <is>
-          <t>M4-02</t>
+          <t>M4-01</t>
         </is>
       </c>
       <c r="B61" s="19" t="inlineStr">
@@ -5890,12 +5898,12 @@
       </c>
       <c r="C61" s="19" t="inlineStr">
         <is>
-          <t>Registro de ingreso del menor con salón o clase asignada y generación de código único.</t>
-        </is>
-      </c>
-      <c r="D61" s="21" t="inlineStr">
-        <is>
-          <t>v1 + Nuevo v3</t>
+          <t>Sustitución de la ficha física de papel.</t>
+        </is>
+      </c>
+      <c r="D61" s="19" t="inlineStr">
+        <is>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E61" s="19" t="inlineStr">
@@ -5944,7 +5952,7 @@
     <row r="62">
       <c r="A62" s="18" t="inlineStr">
         <is>
-          <t>M4-03</t>
+          <t>M4-02</t>
         </is>
       </c>
       <c r="B62" s="19" t="inlineStr">
@@ -5954,12 +5962,12 @@
       </c>
       <c r="C62" s="19" t="inlineStr">
         <is>
-          <t>Código QR dinámico o OTP temporal en la PWA del padre o tutor.</t>
-        </is>
-      </c>
-      <c r="D62" s="19" t="inlineStr">
-        <is>
-          <t>v2</t>
+          <t>Registro de ingreso del menor con salón o clase asignada y generación de código único.</t>
+        </is>
+      </c>
+      <c r="D62" s="21" t="inlineStr">
+        <is>
+          <t>v1 + Nuevo v3</t>
         </is>
       </c>
       <c r="E62" s="19" t="inlineStr">
@@ -6008,7 +6016,7 @@
     <row r="63">
       <c r="A63" s="18" t="inlineStr">
         <is>
-          <t>M4-04</t>
+          <t>M4-03</t>
         </is>
       </c>
       <c r="B63" s="19" t="inlineStr">
@@ -6018,7 +6026,7 @@
       </c>
       <c r="C63" s="19" t="inlineStr">
         <is>
-          <t>Validación al entregar: el servidor de Kids escanea el código y confirma identidad y fotografía del tutor autorizado en el Expediente Digital.</t>
+          <t>Código QR dinámico o OTP temporal en la PWA del padre o tutor.</t>
         </is>
       </c>
       <c r="D63" s="19" t="inlineStr">
@@ -6072,7 +6080,7 @@
     <row r="64">
       <c r="A64" s="18" t="inlineStr">
         <is>
-          <t>M4-05</t>
+          <t>M4-04</t>
         </is>
       </c>
       <c r="B64" s="19" t="inlineStr">
@@ -6082,12 +6090,12 @@
       </c>
       <c r="C64" s="19" t="inlineStr">
         <is>
-          <t>Alternativa para tutores sin smartphone, sin batería o sin conexión (p. ej. código por SMS o comprobante imprimible con identificación). Por definir.</t>
-        </is>
-      </c>
-      <c r="D64" s="21" t="inlineStr">
-        <is>
-          <t>Nuevo v3</t>
+          <t>Validación al entregar: el servidor de Kids escanea el código y confirma identidad y fotografía del tutor autorizado en el Expediente Digital.</t>
+        </is>
+      </c>
+      <c r="D64" s="19" t="inlineStr">
+        <is>
+          <t>v2</t>
         </is>
       </c>
       <c r="E64" s="19" t="inlineStr">
@@ -6122,7 +6130,7 @@
       </c>
       <c r="K64" s="19" t="inlineStr">
         <is>
-          <t>Por definir</t>
+          <t>VoBo pendiente</t>
         </is>
       </c>
       <c r="L64" s="19" t="inlineStr">
@@ -6136,7 +6144,7 @@
     <row r="65">
       <c r="A65" s="18" t="inlineStr">
         <is>
-          <t>M4-06</t>
+          <t>M4-05</t>
         </is>
       </c>
       <c r="B65" s="19" t="inlineStr">
@@ -6146,7 +6154,7 @@
       </c>
       <c r="C65" s="19" t="inlineStr">
         <is>
-          <t>Autorización temporal de un tercero para recoger al menor, con aprobación del tutor registrado.</t>
+          <t>Alternativa para tutores sin smartphone, sin batería o sin conexión (p. ej. código por SMS o comprobante imprimible con identificación). Por definir.</t>
         </is>
       </c>
       <c r="D65" s="21" t="inlineStr">
@@ -6186,7 +6194,7 @@
       </c>
       <c r="K65" s="19" t="inlineStr">
         <is>
-          <t>VoBo pendiente</t>
+          <t>Por definir</t>
         </is>
       </c>
       <c r="L65" s="19" t="inlineStr">
@@ -6200,7 +6208,7 @@
     <row r="66">
       <c r="A66" s="18" t="inlineStr">
         <is>
-          <t>M4-07</t>
+          <t>M4-06</t>
         </is>
       </c>
       <c r="B66" s="19" t="inlineStr">
@@ -6210,7 +6218,7 @@
       </c>
       <c r="C66" s="19" t="inlineStr">
         <is>
-          <t>Caducidad del código y bitácora de cada entrega (quién recogió, quién entregó, hora).</t>
+          <t>Autorización temporal de un tercero para recoger al menor, con aprobación del tutor registrado.</t>
         </is>
       </c>
       <c r="D66" s="21" t="inlineStr">
@@ -6264,7 +6272,7 @@
     <row r="67">
       <c r="A67" s="18" t="inlineStr">
         <is>
-          <t>M4-08</t>
+          <t>M4-07</t>
         </is>
       </c>
       <c r="B67" s="19" t="inlineStr">
@@ -6274,7 +6282,7 @@
       </c>
       <c r="C67" s="19" t="inlineStr">
         <is>
-          <t>Funcionamiento sin conexión o con conexión degradada para el check-out.</t>
+          <t>Caducidad del código y bitácora de cada entrega (quién recogió, quién entregó, hora).</t>
         </is>
       </c>
       <c r="D67" s="21" t="inlineStr">
@@ -6328,52 +6336,52 @@
     <row r="68">
       <c r="A68" s="18" t="inlineStr">
         <is>
-          <t>M5-01</t>
+          <t>M4-08</t>
         </is>
       </c>
       <c r="B68" s="19" t="inlineStr">
         <is>
-          <t>M5 Áreas y servidores</t>
+          <t>M4 Kids Check-In/Out</t>
         </is>
       </c>
       <c r="C68" s="19" t="inlineStr">
         <is>
-          <t>Catálogo mínimo de áreas y asignación de servidores. Versión reducida del módulo 5, necesaria para permisos por área. Sirve como primer censo.</t>
-        </is>
-      </c>
-      <c r="D68" s="19" t="inlineStr">
-        <is>
-          <t>v3</t>
+          <t>Funcionamiento sin conexión o con conexión degradada para el check-out.</t>
+        </is>
+      </c>
+      <c r="D68" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3</t>
         </is>
       </c>
       <c r="E68" s="19" t="inlineStr">
         <is>
-          <t>MVP mínimo</t>
+          <t>Fuera del MVP</t>
         </is>
       </c>
       <c r="F68" s="19" t="inlineStr">
         <is>
-          <t>Fase 0</t>
+          <t>Fase 2</t>
         </is>
       </c>
       <c r="G68" s="19" t="inlineStr">
         <is>
-          <t>Sprint 1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H68" s="19" t="inlineStr">
         <is>
-          <t>H2 · Fase 0 completa</t>
-        </is>
-      </c>
-      <c r="I68" s="19" t="inlineStr">
-        <is>
-          <t>Como pastor quiero un catálogo de áreas con su personal para conocer la estructura.</t>
-        </is>
-      </c>
-      <c r="J68" s="19" t="inlineStr">
-        <is>
-          <t>Crear un área, asignar servidores y ver el conteo real.</t>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="I68" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
+        </is>
+      </c>
+      <c r="J68" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
         </is>
       </c>
       <c r="K68" s="19" t="inlineStr">
@@ -6392,7 +6400,7 @@
     <row r="69">
       <c r="A69" s="18" t="inlineStr">
         <is>
-          <t>M5-02</t>
+          <t>M5-01</t>
         </is>
       </c>
       <c r="B69" s="19" t="inlineStr">
@@ -6402,42 +6410,42 @@
       </c>
       <c r="C69" s="19" t="inlineStr">
         <is>
-          <t>Roles jerárquicos dentro de cada área (directores, líderes, maestros, servidores).</t>
+          <t>Catálogo mínimo de áreas y asignación de servidores. Versión reducida del módulo 5, necesaria para permisos por área. Sirve como primer censo.</t>
         </is>
       </c>
       <c r="D69" s="19" t="inlineStr">
         <is>
-          <t>v1</t>
+          <t>v3</t>
         </is>
       </c>
       <c r="E69" s="19" t="inlineStr">
         <is>
-          <t>Fuera del MVP</t>
+          <t>MVP mínimo</t>
         </is>
       </c>
       <c r="F69" s="19" t="inlineStr">
         <is>
-          <t>Fase 4</t>
+          <t>Fase 0</t>
         </is>
       </c>
       <c r="G69" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sprint 1</t>
         </is>
       </c>
       <c r="H69" s="19" t="inlineStr">
         <is>
-          <t>Posterior</t>
-        </is>
-      </c>
-      <c r="I69" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
-        </is>
-      </c>
-      <c r="J69" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
+          <t>H2 · Fase 0 completa</t>
+        </is>
+      </c>
+      <c r="I69" s="19" t="inlineStr">
+        <is>
+          <t>Como pastor quiero un catálogo de áreas con su personal para conocer la estructura.</t>
+        </is>
+      </c>
+      <c r="J69" s="19" t="inlineStr">
+        <is>
+          <t>Crear un área, asignar servidores y ver el conteo real.</t>
         </is>
       </c>
       <c r="K69" s="19" t="inlineStr">
@@ -6456,7 +6464,7 @@
     <row r="70">
       <c r="A70" s="18" t="inlineStr">
         <is>
-          <t>M5-03</t>
+          <t>M5-02</t>
         </is>
       </c>
       <c r="B70" s="19" t="inlineStr">
@@ -6466,12 +6474,12 @@
       </c>
       <c r="C70" s="19" t="inlineStr">
         <is>
-          <t>Organigrama y número real de servidores activos, directores y líderes por área.</t>
+          <t>Roles jerárquicos dentro de cada área (directores, líderes, maestros, servidores).</t>
         </is>
       </c>
       <c r="D70" s="19" t="inlineStr">
         <is>
-          <t>v2</t>
+          <t>v1</t>
         </is>
       </c>
       <c r="E70" s="19" t="inlineStr">
@@ -6520,7 +6528,7 @@
     <row r="71">
       <c r="A71" s="18" t="inlineStr">
         <is>
-          <t>M5-04</t>
+          <t>M5-03</t>
         </is>
       </c>
       <c r="B71" s="19" t="inlineStr">
@@ -6530,12 +6538,12 @@
       </c>
       <c r="C71" s="19" t="inlineStr">
         <is>
-          <t>Control de asistencia a turnos o servicios.</t>
+          <t>Organigrama y número real de servidores activos, directores y líderes por área.</t>
         </is>
       </c>
       <c r="D71" s="19" t="inlineStr">
         <is>
-          <t>v1 / v2</t>
+          <t>v2</t>
         </is>
       </c>
       <c r="E71" s="19" t="inlineStr">
@@ -6584,7 +6592,7 @@
     <row r="72">
       <c r="A72" s="18" t="inlineStr">
         <is>
-          <t>M5-05</t>
+          <t>M5-04</t>
         </is>
       </c>
       <c r="B72" s="19" t="inlineStr">
@@ -6594,7 +6602,7 @@
       </c>
       <c r="C72" s="19" t="inlineStr">
         <is>
-          <t>Tablero de avisos y notificaciones interno por área.</t>
+          <t>Control de asistencia a turnos o servicios.</t>
         </is>
       </c>
       <c r="D72" s="19" t="inlineStr">
@@ -6648,7 +6656,7 @@
     <row r="73">
       <c r="A73" s="18" t="inlineStr">
         <is>
-          <t>M5-06</t>
+          <t>M5-05</t>
         </is>
       </c>
       <c r="B73" s="19" t="inlineStr">
@@ -6658,7 +6666,7 @@
       </c>
       <c r="C73" s="19" t="inlineStr">
         <is>
-          <t>Gestión financiera por área: caja chica y gastos operativos.</t>
+          <t>Tablero de avisos y notificaciones interno por área.</t>
         </is>
       </c>
       <c r="D73" s="19" t="inlineStr">
@@ -6712,22 +6720,22 @@
     <row r="74">
       <c r="A74" s="18" t="inlineStr">
         <is>
-          <t>M6-01</t>
+          <t>M5-06</t>
         </is>
       </c>
       <c r="B74" s="19" t="inlineStr">
         <is>
-          <t>M6 Ministerios de servicio</t>
+          <t>M5 Áreas y servidores</t>
         </is>
       </c>
       <c r="C74" s="19" t="inlineStr">
         <is>
-          <t>Control de personal propio de cada ministerio.</t>
-        </is>
-      </c>
-      <c r="D74" s="22" t="inlineStr">
-        <is>
-          <t>Recuperado v1</t>
+          <t>Gestión financiera por área: caja chica y gastos operativos.</t>
+        </is>
+      </c>
+      <c r="D74" s="19" t="inlineStr">
+        <is>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E74" s="19" t="inlineStr">
@@ -6776,7 +6784,7 @@
     <row r="75">
       <c r="A75" s="18" t="inlineStr">
         <is>
-          <t>M6-02</t>
+          <t>M6-01</t>
         </is>
       </c>
       <c r="B75" s="19" t="inlineStr">
@@ -6786,12 +6794,12 @@
       </c>
       <c r="C75" s="19" t="inlineStr">
         <is>
-          <t>Menú o catálogo digital interactivo (público o interno), autogestionado.</t>
-        </is>
-      </c>
-      <c r="D75" s="19" t="inlineStr">
-        <is>
-          <t>v1 / v2</t>
+          <t>Control de personal propio de cada ministerio.</t>
+        </is>
+      </c>
+      <c r="D75" s="22" t="inlineStr">
+        <is>
+          <t>Recuperado v1</t>
         </is>
       </c>
       <c r="E75" s="19" t="inlineStr">
@@ -6840,7 +6848,7 @@
     <row r="76">
       <c r="A76" s="18" t="inlineStr">
         <is>
-          <t>M6-03</t>
+          <t>M6-02</t>
         </is>
       </c>
       <c r="B76" s="19" t="inlineStr">
@@ -6850,7 +6858,7 @@
       </c>
       <c r="C76" s="19" t="inlineStr">
         <is>
-          <t>Calendario de turnos: días regulares de servicio y eventos especiales.</t>
+          <t>Menú o catálogo digital interactivo (público o interno), autogestionado.</t>
         </is>
       </c>
       <c r="D76" s="19" t="inlineStr">
@@ -6904,7 +6912,7 @@
     <row r="77">
       <c r="A77" s="18" t="inlineStr">
         <is>
-          <t>M6-04</t>
+          <t>M6-03</t>
         </is>
       </c>
       <c r="B77" s="19" t="inlineStr">
@@ -6914,7 +6922,7 @@
       </c>
       <c r="C77" s="19" t="inlineStr">
         <is>
-          <t>Registro de asistentes o personas atendidas.</t>
+          <t>Calendario de turnos: días regulares de servicio y eventos especiales.</t>
         </is>
       </c>
       <c r="D77" s="19" t="inlineStr">
@@ -6968,7 +6976,7 @@
     <row r="78">
       <c r="A78" s="18" t="inlineStr">
         <is>
-          <t>M6-05</t>
+          <t>M6-04</t>
         </is>
       </c>
       <c r="B78" s="19" t="inlineStr">
@@ -6978,7 +6986,7 @@
       </c>
       <c r="C78" s="19" t="inlineStr">
         <is>
-          <t>Control de gastos y de inventario básico.</t>
+          <t>Registro de asistentes o personas atendidas.</t>
         </is>
       </c>
       <c r="D78" s="19" t="inlineStr">
@@ -7032,7 +7040,7 @@
     <row r="79">
       <c r="A79" s="18" t="inlineStr">
         <is>
-          <t>M6-06</t>
+          <t>M6-05</t>
         </is>
       </c>
       <c r="B79" s="19" t="inlineStr">
@@ -7042,7 +7050,7 @@
       </c>
       <c r="C79" s="19" t="inlineStr">
         <is>
-          <t>Canal de comunicación directo con el área de Administración General.</t>
+          <t>Control de gastos y de inventario básico.</t>
         </is>
       </c>
       <c r="D79" s="19" t="inlineStr">
@@ -7096,7 +7104,7 @@
     <row r="80">
       <c r="A80" s="18" t="inlineStr">
         <is>
-          <t>M6-07</t>
+          <t>M6-06</t>
         </is>
       </c>
       <c r="B80" s="19" t="inlineStr">
@@ -7106,12 +7114,12 @@
       </c>
       <c r="C80" s="19" t="inlineStr">
         <is>
-          <t>Servicio Médico: los datos de salud de las personas atendidas requieren tratamiento de datos sensibles. Por definir alcance.</t>
-        </is>
-      </c>
-      <c r="D80" s="21" t="inlineStr">
-        <is>
-          <t>Nuevo v3</t>
+          <t>Canal de comunicación directo con el área de Administración General.</t>
+        </is>
+      </c>
+      <c r="D80" s="19" t="inlineStr">
+        <is>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E80" s="19" t="inlineStr">
@@ -7146,7 +7154,7 @@
       </c>
       <c r="K80" s="19" t="inlineStr">
         <is>
-          <t>Por definir</t>
+          <t>VoBo pendiente</t>
         </is>
       </c>
       <c r="L80" s="19" t="inlineStr">
@@ -7160,22 +7168,22 @@
     <row r="81">
       <c r="A81" s="18" t="inlineStr">
         <is>
-          <t>M7-01</t>
+          <t>M6-07</t>
         </is>
       </c>
       <c r="B81" s="19" t="inlineStr">
         <is>
-          <t>M7 Eventos y aforo</t>
+          <t>M6 Ministerios de servicio</t>
         </is>
       </c>
       <c r="C81" s="19" t="inlineStr">
         <is>
-          <t>Eventos abiertos o evangelísticos con formulario de inscripción rápida, sin requerir historial previo.</t>
-        </is>
-      </c>
-      <c r="D81" s="19" t="inlineStr">
-        <is>
-          <t>v1 / v2</t>
+          <t>Servicio Médico: los datos de salud de las personas atendidas requieren tratamiento de datos sensibles. Por definir alcance.</t>
+        </is>
+      </c>
+      <c r="D81" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3</t>
         </is>
       </c>
       <c r="E81" s="19" t="inlineStr">
@@ -7210,7 +7218,7 @@
       </c>
       <c r="K81" s="19" t="inlineStr">
         <is>
-          <t>VoBo pendiente</t>
+          <t>Por definir</t>
         </is>
       </c>
       <c r="L81" s="19" t="inlineStr">
@@ -7224,7 +7232,7 @@
     <row r="82">
       <c r="A82" s="18" t="inlineStr">
         <is>
-          <t>M7-02</t>
+          <t>M7-01</t>
         </is>
       </c>
       <c r="B82" s="19" t="inlineStr">
@@ -7234,12 +7242,12 @@
       </c>
       <c r="C82" s="19" t="inlineStr">
         <is>
-          <t>Consolidación (inducción de personas que asisten por primera vez) como tipo de evento.</t>
-        </is>
-      </c>
-      <c r="D82" s="22" t="inlineStr">
-        <is>
-          <t>Recuperado v1</t>
+          <t>Eventos abiertos o evangelísticos con formulario de inscripción rápida, sin requerir historial previo.</t>
+        </is>
+      </c>
+      <c r="D82" s="19" t="inlineStr">
+        <is>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E82" s="19" t="inlineStr">
@@ -7288,7 +7296,7 @@
     <row r="83">
       <c r="A83" s="18" t="inlineStr">
         <is>
-          <t>M7-03</t>
+          <t>M7-02</t>
         </is>
       </c>
       <c r="B83" s="19" t="inlineStr">
@@ -7298,7 +7306,7 @@
       </c>
       <c r="C83" s="19" t="inlineStr">
         <is>
-          <t>Encargados de evento (personal de la iglesia únicamente; no se controla personal externo).</t>
+          <t>Consolidación (inducción de personas que asisten por primera vez) como tipo de evento.</t>
         </is>
       </c>
       <c r="D83" s="22" t="inlineStr">
@@ -7352,7 +7360,7 @@
     <row r="84">
       <c r="A84" s="18" t="inlineStr">
         <is>
-          <t>M7-04</t>
+          <t>M7-03</t>
         </is>
       </c>
       <c r="B84" s="19" t="inlineStr">
@@ -7362,12 +7370,12 @@
       </c>
       <c r="C84" s="19" t="inlineStr">
         <is>
-          <t>Control de cupo en tiempo real que bloquea el sobrecupo en eventos con aforo limitado (ej. 30 o 50 lugares).</t>
-        </is>
-      </c>
-      <c r="D84" s="19" t="inlineStr">
-        <is>
-          <t>v1 / v2</t>
+          <t>Encargados de evento (personal de la iglesia únicamente; no se controla personal externo).</t>
+        </is>
+      </c>
+      <c r="D84" s="22" t="inlineStr">
+        <is>
+          <t>Recuperado v1</t>
         </is>
       </c>
       <c r="E84" s="19" t="inlineStr">
@@ -7416,7 +7424,7 @@
     <row r="85">
       <c r="A85" s="18" t="inlineStr">
         <is>
-          <t>M7-05</t>
+          <t>M7-04</t>
         </is>
       </c>
       <c r="B85" s="19" t="inlineStr">
@@ -7426,12 +7434,12 @@
       </c>
       <c r="C85" s="19" t="inlineStr">
         <is>
-          <t>Control de asistentes sin lista previa, para aforo y para dar a conocer la iglesia.</t>
+          <t>Control de cupo en tiempo real que bloquea el sobrecupo en eventos con aforo limitado (ej. 30 o 50 lugares).</t>
         </is>
       </c>
       <c r="D85" s="19" t="inlineStr">
         <is>
-          <t>v1</t>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E85" s="19" t="inlineStr">
@@ -7480,7 +7488,7 @@
     <row r="86">
       <c r="A86" s="18" t="inlineStr">
         <is>
-          <t>M7-06</t>
+          <t>M7-05</t>
         </is>
       </c>
       <c r="B86" s="19" t="inlineStr">
@@ -7490,12 +7498,12 @@
       </c>
       <c r="C86" s="19" t="inlineStr">
         <is>
-          <t>Seguimiento de personas nuevas: conversión de un invitado a Expediente Digital y canalización a un curso o Grupo de Conexión.</t>
-        </is>
-      </c>
-      <c r="D86" s="21" t="inlineStr">
-        <is>
-          <t>Nuevo v3</t>
+          <t>Control de asistentes sin lista previa, para aforo y para dar a conocer la iglesia.</t>
+        </is>
+      </c>
+      <c r="D86" s="19" t="inlineStr">
+        <is>
+          <t>v1</t>
         </is>
       </c>
       <c r="E86" s="19" t="inlineStr">
@@ -7544,52 +7552,52 @@
     <row r="87">
       <c r="A87" s="18" t="inlineStr">
         <is>
-          <t>NF-01</t>
+          <t>M7-06</t>
         </is>
       </c>
       <c r="B87" s="19" t="inlineStr">
         <is>
-          <t>No funcionales</t>
+          <t>M7 Eventos y aforo</t>
         </is>
       </c>
       <c r="C87" s="19" t="inlineStr">
         <is>
-          <t>Cumplimiento de la LFPDPPP: aviso de privacidad, consentimiento y derechos ARCO.</t>
-        </is>
-      </c>
-      <c r="D87" s="19" t="inlineStr">
-        <is>
-          <t>v3</t>
+          <t>Seguimiento de personas nuevas: conversión de un invitado a Expediente Digital y canalización a un curso o Grupo de Conexión.</t>
+        </is>
+      </c>
+      <c r="D87" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3</t>
         </is>
       </c>
       <c r="E87" s="19" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Fuera del MVP</t>
         </is>
       </c>
       <c r="F87" s="19" t="inlineStr">
         <is>
-          <t>Fase 0</t>
+          <t>Fase 4</t>
         </is>
       </c>
       <c r="G87" s="19" t="inlineStr">
         <is>
-          <t>Sprint 1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H87" s="19" t="inlineStr">
         <is>
-          <t>H1 · 18-oct (núcleo Fase 0)</t>
-        </is>
-      </c>
-      <c r="I87" s="19" t="inlineStr">
-        <is>
-          <t>Como iglesia queremos cumplir con la LFPDPPP.</t>
-        </is>
-      </c>
-      <c r="J87" s="19" t="inlineStr">
-        <is>
-          <t>Aviso de privacidad, consentimiento y atención de derechos ARCO disponibles.</t>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="I87" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
+        </is>
+      </c>
+      <c r="J87" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
         </is>
       </c>
       <c r="K87" s="19" t="inlineStr">
@@ -7608,7 +7616,7 @@
     <row r="88">
       <c r="A88" s="18" t="inlineStr">
         <is>
-          <t>NF-02</t>
+          <t>NF-01</t>
         </is>
       </c>
       <c r="B88" s="19" t="inlineStr">
@@ -7618,7 +7626,7 @@
       </c>
       <c r="C88" s="19" t="inlineStr">
         <is>
-          <t>Cifrado en tránsito y en reposo. Cifrado adicional a nivel de campo para peticiones de oración.</t>
+          <t>Cumplimiento de la LFPDPPP: aviso de privacidad, consentimiento y derechos ARCO.</t>
         </is>
       </c>
       <c r="D88" s="19" t="inlineStr">
@@ -7638,7 +7646,7 @@
       </c>
       <c r="G88" s="19" t="inlineStr">
         <is>
-          <t>Sprint 0</t>
+          <t>Sprint 1</t>
         </is>
       </c>
       <c r="H88" s="19" t="inlineStr">
@@ -7648,12 +7656,12 @@
       </c>
       <c r="I88" s="19" t="inlineStr">
         <is>
-          <t>Como iglesia queremos proteger los datos sensibles.</t>
+          <t>Como iglesia queremos cumplir con la LFPDPPP.</t>
         </is>
       </c>
       <c r="J88" s="19" t="inlineStr">
         <is>
-          <t>HTTPS obligatorio y peticiones de oración ilegibles directamente en la base.</t>
+          <t>Aviso de privacidad, consentimiento y atención de derechos ARCO disponibles.</t>
         </is>
       </c>
       <c r="K88" s="19" t="inlineStr">
@@ -7672,7 +7680,7 @@
     <row r="89">
       <c r="A89" s="18" t="inlineStr">
         <is>
-          <t>NF-03</t>
+          <t>NF-02</t>
         </is>
       </c>
       <c r="B89" s="19" t="inlineStr">
@@ -7682,7 +7690,7 @@
       </c>
       <c r="C89" s="19" t="inlineStr">
         <is>
-          <t>Bitácora de auditoría de solo-añadir: quién consultó o modificó expedientes, ofrendas y asistencias.</t>
+          <t>Cifrado en tránsito y en reposo. Cifrado adicional a nivel de campo para peticiones de oración.</t>
         </is>
       </c>
       <c r="D89" s="19" t="inlineStr">
@@ -7702,7 +7710,7 @@
       </c>
       <c r="G89" s="19" t="inlineStr">
         <is>
-          <t>Sprint 1</t>
+          <t>Sprint 0</t>
         </is>
       </c>
       <c r="H89" s="19" t="inlineStr">
@@ -7712,12 +7720,12 @@
       </c>
       <c r="I89" s="19" t="inlineStr">
         <is>
-          <t>Como pastor quiero una bitácora que nadie pueda alterar.</t>
+          <t>Como iglesia queremos proteger los datos sensibles.</t>
         </is>
       </c>
       <c r="J89" s="19" t="inlineStr">
         <is>
-          <t>El usuario de la aplicación no puede actualizar ni borrar registros de bitácora.</t>
+          <t>HTTPS obligatorio y peticiones de oración ilegibles directamente en la base.</t>
         </is>
       </c>
       <c r="K89" s="19" t="inlineStr">
@@ -7727,24 +7735,16 @@
       </c>
       <c r="L89" s="19" t="inlineStr">
         <is>
-          <t>En pruebas</t>
-        </is>
-      </c>
-      <c r="M89" s="19" t="inlineStr">
-        <is>
-          <t>Rama feature/nf-03-bitacora · 69 pruebas de backend pasan</t>
-        </is>
-      </c>
-      <c r="N89" s="19" t="inlineStr">
-        <is>
-          <t>2026-10-10 · Bloqueo en aplicación y trigger de PostgreSQL (UPDATE/DELETE/TRUNCATE); pantalla de consulta con permiso bitacora.ver.</t>
-        </is>
-      </c>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M89" s="19" t="inlineStr"/>
+      <c r="N89" s="19" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="18" t="inlineStr">
         <is>
-          <t>NF-04</t>
+          <t>NF-03</t>
         </is>
       </c>
       <c r="B90" s="19" t="inlineStr">
@@ -7754,7 +7754,7 @@
       </c>
       <c r="C90" s="19" t="inlineStr">
         <is>
-          <t>Respaldos automáticos diarios cifrados y prueba periódica de restauración.</t>
+          <t>Bitácora de auditoría de solo-añadir: quién consultó o modificó expedientes, ofrendas y asistencias.</t>
         </is>
       </c>
       <c r="D90" s="19" t="inlineStr">
@@ -7774,7 +7774,7 @@
       </c>
       <c r="G90" s="19" t="inlineStr">
         <is>
-          <t>Sprint 0</t>
+          <t>Sprint 1</t>
         </is>
       </c>
       <c r="H90" s="19" t="inlineStr">
@@ -7784,12 +7784,12 @@
       </c>
       <c r="I90" s="19" t="inlineStr">
         <is>
-          <t>Como iglesia queremos no perder información.</t>
+          <t>Como pastor quiero una bitácora que nadie pueda alterar.</t>
         </is>
       </c>
       <c r="J90" s="19" t="inlineStr">
         <is>
-          <t>Respaldo diario cifrado y restauración probada en un ambiente de pruebas.</t>
+          <t>El usuario de la aplicación no puede actualizar ni borrar registros de bitácora.</t>
         </is>
       </c>
       <c r="K90" s="19" t="inlineStr">
@@ -7799,16 +7799,24 @@
       </c>
       <c r="L90" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M90" s="19" t="inlineStr"/>
-      <c r="N90" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M90" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/nf-03-bitacora · 69 pruebas de backend pasan</t>
+        </is>
+      </c>
+      <c r="N90" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-10 · Bloqueo en aplicación y trigger de PostgreSQL (UPDATE/DELETE/TRUNCATE); pantalla de consulta con permiso bitacora.ver.</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="18" t="inlineStr">
         <is>
-          <t>NF-05</t>
+          <t>NF-04</t>
         </is>
       </c>
       <c r="B91" s="19" t="inlineStr">
@@ -7818,47 +7826,47 @@
       </c>
       <c r="C91" s="19" t="inlineStr">
         <is>
-          <t>Disponibilidad esperada en horarios de servicio (fines de semana y reuniones de grupo). Por definir meta.</t>
-        </is>
-      </c>
-      <c r="D91" s="21" t="inlineStr">
-        <is>
-          <t>Nuevo v3</t>
+          <t>Respaldos automáticos diarios cifrados y prueba periódica de restauración.</t>
+        </is>
+      </c>
+      <c r="D91" s="19" t="inlineStr">
+        <is>
+          <t>v3</t>
         </is>
       </c>
       <c r="E91" s="19" t="inlineStr">
         <is>
-          <t>Fuera del MVP</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="F91" s="19" t="inlineStr">
         <is>
-          <t>Transversal</t>
+          <t>Fase 0</t>
         </is>
       </c>
       <c r="G91" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sprint 0</t>
         </is>
       </c>
       <c r="H91" s="19" t="inlineStr">
         <is>
-          <t>Posterior</t>
-        </is>
-      </c>
-      <c r="I91" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
-        </is>
-      </c>
-      <c r="J91" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
+          <t>H1 · 18-oct (núcleo Fase 0)</t>
+        </is>
+      </c>
+      <c r="I91" s="19" t="inlineStr">
+        <is>
+          <t>Como iglesia queremos no perder información.</t>
+        </is>
+      </c>
+      <c r="J91" s="19" t="inlineStr">
+        <is>
+          <t>Respaldo diario cifrado y restauración probada en un ambiente de pruebas.</t>
         </is>
       </c>
       <c r="K91" s="19" t="inlineStr">
         <is>
-          <t>Por definir</t>
+          <t>VoBo pendiente</t>
         </is>
       </c>
       <c r="L91" s="19" t="inlineStr">
@@ -7872,7 +7880,7 @@
     <row r="92">
       <c r="A92" s="18" t="inlineStr">
         <is>
-          <t>NF-06</t>
+          <t>NF-05</t>
         </is>
       </c>
       <c r="B92" s="19" t="inlineStr">
@@ -7882,47 +7890,47 @@
       </c>
       <c r="C92" s="19" t="inlineStr">
         <is>
-          <t>Pase de lista sin conexión con sincronización posterior (reuniones en domicilios con mala señal).</t>
-        </is>
-      </c>
-      <c r="D92" s="19" t="inlineStr">
-        <is>
-          <t>v3</t>
+          <t>Disponibilidad esperada en horarios de servicio (fines de semana y reuniones de grupo). Por definir meta.</t>
+        </is>
+      </c>
+      <c r="D92" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3</t>
         </is>
       </c>
       <c r="E92" s="19" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Fuera del MVP</t>
         </is>
       </c>
       <c r="F92" s="19" t="inlineStr">
         <is>
-          <t>Fase 0</t>
+          <t>Transversal</t>
         </is>
       </c>
       <c r="G92" s="19" t="inlineStr">
         <is>
-          <t>Sprint 3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H92" s="19" t="inlineStr">
         <is>
-          <t>H3 · MVP (Grupos)</t>
-        </is>
-      </c>
-      <c r="I92" s="19" t="inlineStr">
-        <is>
-          <t>Como secretario quiero que el pase de lista funcione sin señal.</t>
-        </is>
-      </c>
-      <c r="J92" s="19" t="inlineStr">
-        <is>
-          <t>Prueba en modo avión y sincronización al reconectar.</t>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="I92" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
+        </is>
+      </c>
+      <c r="J92" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
         </is>
       </c>
       <c r="K92" s="19" t="inlineStr">
         <is>
-          <t>VoBo pendiente</t>
+          <t>Por definir</t>
         </is>
       </c>
       <c r="L92" s="19" t="inlineStr">
@@ -7936,7 +7944,7 @@
     <row r="93">
       <c r="A93" s="18" t="inlineStr">
         <is>
-          <t>NF-07</t>
+          <t>NF-06</t>
         </is>
       </c>
       <c r="B93" s="19" t="inlineStr">
@@ -7946,7 +7954,7 @@
       </c>
       <c r="C93" s="19" t="inlineStr">
         <is>
-          <t>Funciona en Android, iOS y escritorio. En iOS, las notificaciones push requieren instalar la PWA; el respaldo por WhatsApp cubre el resto.</t>
+          <t>Pase de lista sin conexión con sincronización posterior (reuniones en domicilios con mala señal).</t>
         </is>
       </c>
       <c r="D93" s="19" t="inlineStr">
@@ -7966,22 +7974,22 @@
       </c>
       <c r="G93" s="19" t="inlineStr">
         <is>
-          <t>Sprint 0</t>
+          <t>Sprint 3</t>
         </is>
       </c>
       <c r="H93" s="19" t="inlineStr">
         <is>
-          <t>H1 · 18-oct (núcleo Fase 0)</t>
+          <t>H3 · MVP (Grupos)</t>
         </is>
       </c>
       <c r="I93" s="19" t="inlineStr">
         <is>
-          <t>Como usuario quiero usar el sistema en mi dispositivo.</t>
+          <t>Como secretario quiero que el pase de lista funcione sin señal.</t>
         </is>
       </c>
       <c r="J93" s="19" t="inlineStr">
         <is>
-          <t>Pruebas en Android, iOS y escritorio; push en iOS con la PWA instalada y respaldo por WhatsApp.</t>
+          <t>Prueba en modo avión y sincronización al reconectar.</t>
         </is>
       </c>
       <c r="K93" s="19" t="inlineStr">
@@ -8000,7 +8008,7 @@
     <row r="94">
       <c r="A94" s="18" t="inlineStr">
         <is>
-          <t>NF-08</t>
+          <t>NF-07</t>
         </is>
       </c>
       <c r="B94" s="19" t="inlineStr">
@@ -8010,12 +8018,12 @@
       </c>
       <c r="C94" s="19" t="inlineStr">
         <is>
-          <t>Dimensionamiento para ~1,000 personas, con picos los fines de semana, y margen de crecimiento.</t>
-        </is>
-      </c>
-      <c r="D94" s="21" t="inlineStr">
-        <is>
-          <t>Resp. P8</t>
+          <t>Funciona en Android, iOS y escritorio. En iOS, las notificaciones push requieren instalar la PWA; el respaldo por WhatsApp cubre el resto.</t>
+        </is>
+      </c>
+      <c r="D94" s="19" t="inlineStr">
+        <is>
+          <t>v3</t>
         </is>
       </c>
       <c r="E94" s="19" t="inlineStr">
@@ -8040,12 +8048,12 @@
       </c>
       <c r="I94" s="19" t="inlineStr">
         <is>
-          <t>Como iglesia queremos que el sistema soporte a ~1,000 personas.</t>
+          <t>Como usuario quiero usar el sistema en mi dispositivo.</t>
         </is>
       </c>
       <c r="J94" s="19" t="inlineStr">
         <is>
-          <t>Prueba de carga con volumen representativo (por definir) sin degradación.</t>
+          <t>Pruebas en Android, iOS y escritorio; push en iOS con la PWA instalada y respaldo por WhatsApp.</t>
         </is>
       </c>
       <c r="K94" s="19" t="inlineStr">
@@ -8064,7 +8072,7 @@
     <row r="95">
       <c r="A95" s="18" t="inlineStr">
         <is>
-          <t>NF-09</t>
+          <t>NF-08</t>
         </is>
       </c>
       <c r="B95" s="19" t="inlineStr">
@@ -8074,42 +8082,42 @@
       </c>
       <c r="C95" s="19" t="inlineStr">
         <is>
-          <t>Reportes transversales: asistencia, finanzas, crecimiento de la iglesia, exportables a Excel y PDF.</t>
+          <t>Dimensionamiento para ~1,000 personas, con picos los fines de semana, y margen de crecimiento.</t>
         </is>
       </c>
       <c r="D95" s="21" t="inlineStr">
         <is>
-          <t>Nuevo v3</t>
+          <t>Resp. P8</t>
         </is>
       </c>
       <c r="E95" s="19" t="inlineStr">
         <is>
-          <t>Fuera del MVP</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="F95" s="19" t="inlineStr">
         <is>
-          <t>Transversal</t>
+          <t>Fase 0</t>
         </is>
       </c>
       <c r="G95" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sprint 0</t>
         </is>
       </c>
       <c r="H95" s="19" t="inlineStr">
         <is>
-          <t>Posterior</t>
-        </is>
-      </c>
-      <c r="I95" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
-        </is>
-      </c>
-      <c r="J95" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
+          <t>H1 · 18-oct (núcleo Fase 0)</t>
+        </is>
+      </c>
+      <c r="I95" s="19" t="inlineStr">
+        <is>
+          <t>Como iglesia queremos que el sistema soporte a ~1,000 personas.</t>
+        </is>
+      </c>
+      <c r="J95" s="19" t="inlineStr">
+        <is>
+          <t>Prueba de carga con volumen representativo (por definir) sin degradación.</t>
         </is>
       </c>
       <c r="K95" s="19" t="inlineStr">
@@ -8128,7 +8136,7 @@
     <row r="96">
       <c r="A96" s="18" t="inlineStr">
         <is>
-          <t>NF-10</t>
+          <t>NF-09</t>
         </is>
       </c>
       <c r="B96" s="19" t="inlineStr">
@@ -8138,42 +8146,42 @@
       </c>
       <c r="C96" s="19" t="inlineStr">
         <is>
-          <t>Usabilidad para personas mayores: tipografía grande, alto contraste, flujos cortos (ver sección 5).</t>
-        </is>
-      </c>
-      <c r="D96" s="19" t="inlineStr">
-        <is>
-          <t>v3 + Obs. 1</t>
+          <t>Reportes transversales: asistencia, finanzas, crecimiento de la iglesia, exportables a Excel y PDF.</t>
+        </is>
+      </c>
+      <c r="D96" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3</t>
         </is>
       </c>
       <c r="E96" s="19" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Fuera del MVP</t>
         </is>
       </c>
       <c r="F96" s="19" t="inlineStr">
         <is>
-          <t>Fase 0</t>
+          <t>Transversal</t>
         </is>
       </c>
       <c r="G96" s="19" t="inlineStr">
         <is>
-          <t>Sprint 0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H96" s="19" t="inlineStr">
         <is>
-          <t>H1 · 18-oct (núcleo Fase 0)</t>
-        </is>
-      </c>
-      <c r="I96" s="19" t="inlineStr">
-        <is>
-          <t>Como persona mayor quiero una interfaz fácil de leer y usar.</t>
-        </is>
-      </c>
-      <c r="J96" s="19" t="inlineStr">
-        <is>
-          <t>Texto base 18 px, botones de al menos 48 px, contraste AA; prueba con usuarios mayores.</t>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="I96" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
+        </is>
+      </c>
+      <c r="J96" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
         </is>
       </c>
       <c r="K96" s="19" t="inlineStr">
@@ -8189,9 +8197,73 @@
       <c r="M96" s="19" t="inlineStr"/>
       <c r="N96" s="19" t="inlineStr"/>
     </row>
+    <row r="97">
+      <c r="A97" s="18" t="inlineStr">
+        <is>
+          <t>NF-10</t>
+        </is>
+      </c>
+      <c r="B97" s="19" t="inlineStr">
+        <is>
+          <t>No funcionales</t>
+        </is>
+      </c>
+      <c r="C97" s="19" t="inlineStr">
+        <is>
+          <t>Usabilidad para personas mayores: tipografía grande, alto contraste, flujos cortos (ver sección 5).</t>
+        </is>
+      </c>
+      <c r="D97" s="19" t="inlineStr">
+        <is>
+          <t>v3 + Obs. 1</t>
+        </is>
+      </c>
+      <c r="E97" s="19" t="inlineStr">
+        <is>
+          <t>MVP</t>
+        </is>
+      </c>
+      <c r="F97" s="19" t="inlineStr">
+        <is>
+          <t>Fase 0</t>
+        </is>
+      </c>
+      <c r="G97" s="19" t="inlineStr">
+        <is>
+          <t>Sprint 0</t>
+        </is>
+      </c>
+      <c r="H97" s="19" t="inlineStr">
+        <is>
+          <t>H1 · 18-oct (núcleo Fase 0)</t>
+        </is>
+      </c>
+      <c r="I97" s="19" t="inlineStr">
+        <is>
+          <t>Como persona mayor quiero una interfaz fácil de leer y usar.</t>
+        </is>
+      </c>
+      <c r="J97" s="19" t="inlineStr">
+        <is>
+          <t>Texto base 18 px, botones de al menos 48 px, contraste AA; prueba con usuarios mayores.</t>
+        </is>
+      </c>
+      <c r="K97" s="19" t="inlineStr">
+        <is>
+          <t>VoBo pendiente</t>
+        </is>
+      </c>
+      <c r="L97" s="19" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M97" s="19" t="inlineStr"/>
+      <c r="N97" s="19" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N96"/>
-  <conditionalFormatting sqref="L2:L96">
+  <autoFilter ref="A1:N97"/>
+  <conditionalFormatting sqref="L2:L97">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$L2="Hecho"</formula>
     </cfRule>
@@ -8208,7 +8280,7 @@
       <formula>$L2="Bloqueado"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K2:K96">
+  <conditionalFormatting sqref="K2:K97">
     <cfRule type="expression" priority="6" dxfId="0">
       <formula>$K2="Aprobado"</formula>
     </cfRule>
@@ -8216,16 +8288,16 @@
       <formula>$K2="Por definir"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H2:H96">
+  <conditionalFormatting sqref="H2:H97">
     <cfRule type="expression" priority="8" dxfId="5">
       <formula>LEFT($H2,2)="H1"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="L2:L96" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="L2:L97" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Pendiente,En diseño,En desarrollo,En pruebas,Hecho,Bloqueado"</formula1>
     </dataValidation>
-    <dataValidation sqref="K2:K96" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="K2:K97" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"VoBo pendiente,Aprobado,Por definir,Rechazado"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
NF-06: pase de lista sin conexión y corrección del service worker
- Cola local de listas con la hora real de captura; se envía sola al volver la señal
- Servidor: la regla del Secretario "solo el mismo día" se evalúa contra el día de la captura
  (ventana de 7 días, reloj adelantado acotado), no pisa cambios más recientes, es idempotente
  y queda en bitácora como diferida
- Lectura sin conexión de sesión, grupos y reuniones (NetworkFirst); sin finanzas, personas ni
  estudios; la copia se borra al cerrar sesión
- Modo /grupos/:id/hoy para pasar lista sin señal; aviso de conexión y de pendientes con "Enviar
  ahora" y "Descartar" para rechazos definitivos
- Corrige el service worker: ya no responde con la app a PDF, audio del estudio ni /admin/
- React Query en modo "always" para que el service worker y la cola funcionen sin red
- Documentación v3.8 y matriz de trazabilidad

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/trazabilidad/Matriz de Trazabilidad MDF.xlsx
+++ b/docs/trazabilidad/Matriz de Trazabilidad MDF.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Origen v1" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Matriz'!$A$1:$N$96</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Matriz'!$A$1:$N$97</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -897,31 +897,31 @@
         </is>
       </c>
       <c r="B5" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$96,$A5)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$97,$A5)</f>
         <v/>
       </c>
       <c r="C5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A5,Matriz!$L$2:$L$96,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A5,Matriz!$L$2:$L$97,"Pendiente")</f>
         <v/>
       </c>
       <c r="D5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A5,Matriz!$L$2:$L$96,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A5,Matriz!$L$2:$L$97,"En diseño")</f>
         <v/>
       </c>
       <c r="E5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A5,Matriz!$L$2:$L$96,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A5,Matriz!$L$2:$L$97,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A5,Matriz!$L$2:$L$96,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A5,Matriz!$L$2:$L$97,"En pruebas")</f>
         <v/>
       </c>
       <c r="G5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A5,Matriz!$L$2:$L$96,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A5,Matriz!$L$2:$L$97,"Hecho")</f>
         <v/>
       </c>
       <c r="H5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A5,Matriz!$L$2:$L$96,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A5,Matriz!$L$2:$L$97,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I5" s="13">
@@ -936,31 +936,31 @@
         </is>
       </c>
       <c r="B6" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$96,$A6)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$97,$A6)</f>
         <v/>
       </c>
       <c r="C6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A6,Matriz!$L$2:$L$96,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A6,Matriz!$L$2:$L$97,"Pendiente")</f>
         <v/>
       </c>
       <c r="D6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A6,Matriz!$L$2:$L$96,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A6,Matriz!$L$2:$L$97,"En diseño")</f>
         <v/>
       </c>
       <c r="E6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A6,Matriz!$L$2:$L$96,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A6,Matriz!$L$2:$L$97,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A6,Matriz!$L$2:$L$96,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A6,Matriz!$L$2:$L$97,"En pruebas")</f>
         <v/>
       </c>
       <c r="G6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A6,Matriz!$L$2:$L$96,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A6,Matriz!$L$2:$L$97,"Hecho")</f>
         <v/>
       </c>
       <c r="H6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A6,Matriz!$L$2:$L$96,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A6,Matriz!$L$2:$L$97,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I6" s="13">
@@ -975,31 +975,31 @@
         </is>
       </c>
       <c r="B7" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$96,$A7)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$97,$A7)</f>
         <v/>
       </c>
       <c r="C7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A7,Matriz!$L$2:$L$96,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A7,Matriz!$L$2:$L$97,"Pendiente")</f>
         <v/>
       </c>
       <c r="D7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A7,Matriz!$L$2:$L$96,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A7,Matriz!$L$2:$L$97,"En diseño")</f>
         <v/>
       </c>
       <c r="E7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A7,Matriz!$L$2:$L$96,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A7,Matriz!$L$2:$L$97,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A7,Matriz!$L$2:$L$96,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A7,Matriz!$L$2:$L$97,"En pruebas")</f>
         <v/>
       </c>
       <c r="G7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A7,Matriz!$L$2:$L$96,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A7,Matriz!$L$2:$L$97,"Hecho")</f>
         <v/>
       </c>
       <c r="H7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A7,Matriz!$L$2:$L$96,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A7,Matriz!$L$2:$L$97,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I7" s="13">
@@ -1014,31 +1014,31 @@
         </is>
       </c>
       <c r="B8" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$96,$A8)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$97,$A8)</f>
         <v/>
       </c>
       <c r="C8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A8,Matriz!$L$2:$L$96,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A8,Matriz!$L$2:$L$97,"Pendiente")</f>
         <v/>
       </c>
       <c r="D8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A8,Matriz!$L$2:$L$96,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A8,Matriz!$L$2:$L$97,"En diseño")</f>
         <v/>
       </c>
       <c r="E8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A8,Matriz!$L$2:$L$96,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A8,Matriz!$L$2:$L$97,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A8,Matriz!$L$2:$L$96,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A8,Matriz!$L$2:$L$97,"En pruebas")</f>
         <v/>
       </c>
       <c r="G8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A8,Matriz!$L$2:$L$96,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A8,Matriz!$L$2:$L$97,"Hecho")</f>
         <v/>
       </c>
       <c r="H8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A8,Matriz!$L$2:$L$96,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A8,Matriz!$L$2:$L$97,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I8" s="13">
@@ -1053,31 +1053,31 @@
         </is>
       </c>
       <c r="B9" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$96,$A9)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$97,$A9)</f>
         <v/>
       </c>
       <c r="C9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A9,Matriz!$L$2:$L$96,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A9,Matriz!$L$2:$L$97,"Pendiente")</f>
         <v/>
       </c>
       <c r="D9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A9,Matriz!$L$2:$L$96,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A9,Matriz!$L$2:$L$97,"En diseño")</f>
         <v/>
       </c>
       <c r="E9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A9,Matriz!$L$2:$L$96,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A9,Matriz!$L$2:$L$97,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A9,Matriz!$L$2:$L$96,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A9,Matriz!$L$2:$L$97,"En pruebas")</f>
         <v/>
       </c>
       <c r="G9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A9,Matriz!$L$2:$L$96,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A9,Matriz!$L$2:$L$97,"Hecho")</f>
         <v/>
       </c>
       <c r="H9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A9,Matriz!$L$2:$L$96,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A9,Matriz!$L$2:$L$97,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I9" s="13">
@@ -1092,31 +1092,31 @@
         </is>
       </c>
       <c r="B10" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$96,$A10)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$97,$A10)</f>
         <v/>
       </c>
       <c r="C10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A10,Matriz!$L$2:$L$96,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A10,Matriz!$L$2:$L$97,"Pendiente")</f>
         <v/>
       </c>
       <c r="D10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A10,Matriz!$L$2:$L$96,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A10,Matriz!$L$2:$L$97,"En diseño")</f>
         <v/>
       </c>
       <c r="E10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A10,Matriz!$L$2:$L$96,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A10,Matriz!$L$2:$L$97,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A10,Matriz!$L$2:$L$96,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A10,Matriz!$L$2:$L$97,"En pruebas")</f>
         <v/>
       </c>
       <c r="G10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A10,Matriz!$L$2:$L$96,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A10,Matriz!$L$2:$L$97,"Hecho")</f>
         <v/>
       </c>
       <c r="H10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A10,Matriz!$L$2:$L$96,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A10,Matriz!$L$2:$L$97,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I10" s="13">
@@ -1131,31 +1131,31 @@
         </is>
       </c>
       <c r="B11" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$96,$A11)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$97,$A11)</f>
         <v/>
       </c>
       <c r="C11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A11,Matriz!$L$2:$L$96,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A11,Matriz!$L$2:$L$97,"Pendiente")</f>
         <v/>
       </c>
       <c r="D11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A11,Matriz!$L$2:$L$96,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A11,Matriz!$L$2:$L$97,"En diseño")</f>
         <v/>
       </c>
       <c r="E11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A11,Matriz!$L$2:$L$96,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A11,Matriz!$L$2:$L$97,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A11,Matriz!$L$2:$L$96,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A11,Matriz!$L$2:$L$97,"En pruebas")</f>
         <v/>
       </c>
       <c r="G11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A11,Matriz!$L$2:$L$96,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A11,Matriz!$L$2:$L$97,"Hecho")</f>
         <v/>
       </c>
       <c r="H11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$96,$A11,Matriz!$L$2:$L$96,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$97,$A11,Matriz!$L$2:$L$97,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I11" s="13">
@@ -1256,31 +1256,31 @@
         </is>
       </c>
       <c r="B16" s="12">
-        <f>COUNTIF(Matriz!$H$2:$H$96,$A16)</f>
+        <f>COUNTIF(Matriz!$H$2:$H$97,$A16)</f>
         <v/>
       </c>
       <c r="C16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$96,$A16,Matriz!$L$2:$L$96,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$97,$A16,Matriz!$L$2:$L$97,"Pendiente")</f>
         <v/>
       </c>
       <c r="D16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$96,$A16,Matriz!$L$2:$L$96,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$97,$A16,Matriz!$L$2:$L$97,"En diseño")</f>
         <v/>
       </c>
       <c r="E16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$96,$A16,Matriz!$L$2:$L$96,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$97,$A16,Matriz!$L$2:$L$97,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$96,$A16,Matriz!$L$2:$L$96,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$97,$A16,Matriz!$L$2:$L$97,"En pruebas")</f>
         <v/>
       </c>
       <c r="G16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$96,$A16,Matriz!$L$2:$L$96,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$97,$A16,Matriz!$L$2:$L$97,"Hecho")</f>
         <v/>
       </c>
       <c r="H16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$96,$A16,Matriz!$L$2:$L$96,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$97,$A16,Matriz!$L$2:$L$97,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I16" s="13">
@@ -1295,31 +1295,31 @@
         </is>
       </c>
       <c r="B17" s="12">
-        <f>COUNTIF(Matriz!$H$2:$H$96,$A17)</f>
+        <f>COUNTIF(Matriz!$H$2:$H$97,$A17)</f>
         <v/>
       </c>
       <c r="C17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$96,$A17,Matriz!$L$2:$L$96,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$97,$A17,Matriz!$L$2:$L$97,"Pendiente")</f>
         <v/>
       </c>
       <c r="D17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$96,$A17,Matriz!$L$2:$L$96,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$97,$A17,Matriz!$L$2:$L$97,"En diseño")</f>
         <v/>
       </c>
       <c r="E17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$96,$A17,Matriz!$L$2:$L$96,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$97,$A17,Matriz!$L$2:$L$97,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$96,$A17,Matriz!$L$2:$L$96,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$97,$A17,Matriz!$L$2:$L$97,"En pruebas")</f>
         <v/>
       </c>
       <c r="G17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$96,$A17,Matriz!$L$2:$L$96,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$97,$A17,Matriz!$L$2:$L$97,"Hecho")</f>
         <v/>
       </c>
       <c r="H17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$96,$A17,Matriz!$L$2:$L$96,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$97,$A17,Matriz!$L$2:$L$97,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I17" s="13">
@@ -1334,31 +1334,31 @@
         </is>
       </c>
       <c r="B18" s="12">
-        <f>COUNTIF(Matriz!$H$2:$H$96,$A18)</f>
+        <f>COUNTIF(Matriz!$H$2:$H$97,$A18)</f>
         <v/>
       </c>
       <c r="C18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$96,$A18,Matriz!$L$2:$L$96,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$97,$A18,Matriz!$L$2:$L$97,"Pendiente")</f>
         <v/>
       </c>
       <c r="D18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$96,$A18,Matriz!$L$2:$L$96,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$97,$A18,Matriz!$L$2:$L$97,"En diseño")</f>
         <v/>
       </c>
       <c r="E18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$96,$A18,Matriz!$L$2:$L$96,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$97,$A18,Matriz!$L$2:$L$97,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$96,$A18,Matriz!$L$2:$L$96,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$97,$A18,Matriz!$L$2:$L$97,"En pruebas")</f>
         <v/>
       </c>
       <c r="G18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$96,$A18,Matriz!$L$2:$L$96,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$97,$A18,Matriz!$L$2:$L$97,"Hecho")</f>
         <v/>
       </c>
       <c r="H18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$96,$A18,Matriz!$L$2:$L$96,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$97,$A18,Matriz!$L$2:$L$97,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I18" s="13">
@@ -1373,31 +1373,31 @@
         </is>
       </c>
       <c r="B19" s="12">
-        <f>COUNTIF(Matriz!$H$2:$H$96,$A19)</f>
+        <f>COUNTIF(Matriz!$H$2:$H$97,$A19)</f>
         <v/>
       </c>
       <c r="C19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$96,$A19,Matriz!$L$2:$L$96,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$97,$A19,Matriz!$L$2:$L$97,"Pendiente")</f>
         <v/>
       </c>
       <c r="D19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$96,$A19,Matriz!$L$2:$L$96,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$97,$A19,Matriz!$L$2:$L$97,"En diseño")</f>
         <v/>
       </c>
       <c r="E19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$96,$A19,Matriz!$L$2:$L$96,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$97,$A19,Matriz!$L$2:$L$97,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$96,$A19,Matriz!$L$2:$L$96,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$97,$A19,Matriz!$L$2:$L$97,"En pruebas")</f>
         <v/>
       </c>
       <c r="G19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$96,$A19,Matriz!$L$2:$L$96,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$97,$A19,Matriz!$L$2:$L$97,"Hecho")</f>
         <v/>
       </c>
       <c r="H19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$96,$A19,Matriz!$L$2:$L$96,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$97,$A19,Matriz!$L$2:$L$97,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I19" s="13">
@@ -1498,31 +1498,31 @@
         </is>
       </c>
       <c r="B24" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$96,$A24)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$97,$A24)</f>
         <v/>
       </c>
       <c r="C24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A24,Matriz!$L$2:$L$96,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A24,Matriz!$L$2:$L$97,"Pendiente")</f>
         <v/>
       </c>
       <c r="D24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A24,Matriz!$L$2:$L$96,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A24,Matriz!$L$2:$L$97,"En diseño")</f>
         <v/>
       </c>
       <c r="E24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A24,Matriz!$L$2:$L$96,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A24,Matriz!$L$2:$L$97,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A24,Matriz!$L$2:$L$96,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A24,Matriz!$L$2:$L$97,"En pruebas")</f>
         <v/>
       </c>
       <c r="G24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A24,Matriz!$L$2:$L$96,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A24,Matriz!$L$2:$L$97,"Hecho")</f>
         <v/>
       </c>
       <c r="H24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A24,Matriz!$L$2:$L$96,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A24,Matriz!$L$2:$L$97,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I24" s="13">
@@ -1537,31 +1537,31 @@
         </is>
       </c>
       <c r="B25" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$96,$A25)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$97,$A25)</f>
         <v/>
       </c>
       <c r="C25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A25,Matriz!$L$2:$L$96,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A25,Matriz!$L$2:$L$97,"Pendiente")</f>
         <v/>
       </c>
       <c r="D25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A25,Matriz!$L$2:$L$96,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A25,Matriz!$L$2:$L$97,"En diseño")</f>
         <v/>
       </c>
       <c r="E25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A25,Matriz!$L$2:$L$96,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A25,Matriz!$L$2:$L$97,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A25,Matriz!$L$2:$L$96,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A25,Matriz!$L$2:$L$97,"En pruebas")</f>
         <v/>
       </c>
       <c r="G25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A25,Matriz!$L$2:$L$96,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A25,Matriz!$L$2:$L$97,"Hecho")</f>
         <v/>
       </c>
       <c r="H25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A25,Matriz!$L$2:$L$96,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A25,Matriz!$L$2:$L$97,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I25" s="13">
@@ -1576,31 +1576,31 @@
         </is>
       </c>
       <c r="B26" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$96,$A26)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$97,$A26)</f>
         <v/>
       </c>
       <c r="C26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A26,Matriz!$L$2:$L$96,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A26,Matriz!$L$2:$L$97,"Pendiente")</f>
         <v/>
       </c>
       <c r="D26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A26,Matriz!$L$2:$L$96,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A26,Matriz!$L$2:$L$97,"En diseño")</f>
         <v/>
       </c>
       <c r="E26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A26,Matriz!$L$2:$L$96,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A26,Matriz!$L$2:$L$97,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A26,Matriz!$L$2:$L$96,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A26,Matriz!$L$2:$L$97,"En pruebas")</f>
         <v/>
       </c>
       <c r="G26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A26,Matriz!$L$2:$L$96,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A26,Matriz!$L$2:$L$97,"Hecho")</f>
         <v/>
       </c>
       <c r="H26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A26,Matriz!$L$2:$L$96,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A26,Matriz!$L$2:$L$97,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I26" s="13">
@@ -1615,31 +1615,31 @@
         </is>
       </c>
       <c r="B27" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$96,$A27)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$97,$A27)</f>
         <v/>
       </c>
       <c r="C27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A27,Matriz!$L$2:$L$96,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A27,Matriz!$L$2:$L$97,"Pendiente")</f>
         <v/>
       </c>
       <c r="D27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A27,Matriz!$L$2:$L$96,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A27,Matriz!$L$2:$L$97,"En diseño")</f>
         <v/>
       </c>
       <c r="E27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A27,Matriz!$L$2:$L$96,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A27,Matriz!$L$2:$L$97,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A27,Matriz!$L$2:$L$96,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A27,Matriz!$L$2:$L$97,"En pruebas")</f>
         <v/>
       </c>
       <c r="G27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A27,Matriz!$L$2:$L$96,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A27,Matriz!$L$2:$L$97,"Hecho")</f>
         <v/>
       </c>
       <c r="H27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A27,Matriz!$L$2:$L$96,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A27,Matriz!$L$2:$L$97,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I27" s="13">
@@ -1654,31 +1654,31 @@
         </is>
       </c>
       <c r="B28" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$96,$A28)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$97,$A28)</f>
         <v/>
       </c>
       <c r="C28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A28,Matriz!$L$2:$L$96,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A28,Matriz!$L$2:$L$97,"Pendiente")</f>
         <v/>
       </c>
       <c r="D28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A28,Matriz!$L$2:$L$96,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A28,Matriz!$L$2:$L$97,"En diseño")</f>
         <v/>
       </c>
       <c r="E28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A28,Matriz!$L$2:$L$96,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A28,Matriz!$L$2:$L$97,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A28,Matriz!$L$2:$L$96,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A28,Matriz!$L$2:$L$97,"En pruebas")</f>
         <v/>
       </c>
       <c r="G28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A28,Matriz!$L$2:$L$96,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A28,Matriz!$L$2:$L$97,"Hecho")</f>
         <v/>
       </c>
       <c r="H28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A28,Matriz!$L$2:$L$96,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A28,Matriz!$L$2:$L$97,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I28" s="13">
@@ -1693,31 +1693,31 @@
         </is>
       </c>
       <c r="B29" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$96,$A29)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$97,$A29)</f>
         <v/>
       </c>
       <c r="C29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A29,Matriz!$L$2:$L$96,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A29,Matriz!$L$2:$L$97,"Pendiente")</f>
         <v/>
       </c>
       <c r="D29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A29,Matriz!$L$2:$L$96,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A29,Matriz!$L$2:$L$97,"En diseño")</f>
         <v/>
       </c>
       <c r="E29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A29,Matriz!$L$2:$L$96,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A29,Matriz!$L$2:$L$97,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A29,Matriz!$L$2:$L$96,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A29,Matriz!$L$2:$L$97,"En pruebas")</f>
         <v/>
       </c>
       <c r="G29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A29,Matriz!$L$2:$L$96,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A29,Matriz!$L$2:$L$97,"Hecho")</f>
         <v/>
       </c>
       <c r="H29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A29,Matriz!$L$2:$L$96,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A29,Matriz!$L$2:$L$97,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I29" s="13">
@@ -1732,31 +1732,31 @@
         </is>
       </c>
       <c r="B30" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$96,$A30)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$97,$A30)</f>
         <v/>
       </c>
       <c r="C30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A30,Matriz!$L$2:$L$96,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A30,Matriz!$L$2:$L$97,"Pendiente")</f>
         <v/>
       </c>
       <c r="D30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A30,Matriz!$L$2:$L$96,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A30,Matriz!$L$2:$L$97,"En diseño")</f>
         <v/>
       </c>
       <c r="E30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A30,Matriz!$L$2:$L$96,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A30,Matriz!$L$2:$L$97,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A30,Matriz!$L$2:$L$96,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A30,Matriz!$L$2:$L$97,"En pruebas")</f>
         <v/>
       </c>
       <c r="G30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A30,Matriz!$L$2:$L$96,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A30,Matriz!$L$2:$L$97,"Hecho")</f>
         <v/>
       </c>
       <c r="H30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$96,$A30,Matriz!$L$2:$L$96,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$97,$A30,Matriz!$L$2:$L$97,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I30" s="13">
@@ -1818,7 +1818,7 @@
         </is>
       </c>
       <c r="B35" s="12">
-        <f>COUNTIF(Matriz!$K$2:$K$96,A35)</f>
+        <f>COUNTIF(Matriz!$K$2:$K$97,A35)</f>
         <v/>
       </c>
     </row>
@@ -1829,7 +1829,7 @@
         </is>
       </c>
       <c r="B36" s="12">
-        <f>COUNTIF(Matriz!$K$2:$K$96,A36)</f>
+        <f>COUNTIF(Matriz!$K$2:$K$97,A36)</f>
         <v/>
       </c>
     </row>
@@ -1840,7 +1840,7 @@
         </is>
       </c>
       <c r="B37" s="12">
-        <f>COUNTIF(Matriz!$K$2:$K$96,A37)</f>
+        <f>COUNTIF(Matriz!$K$2:$K$97,A37)</f>
         <v/>
       </c>
     </row>
@@ -1851,7 +1851,7 @@
         </is>
       </c>
       <c r="B38" s="12">
-        <f>COUNTIF(Matriz!$K$2:$K$96,A38)</f>
+        <f>COUNTIF(Matriz!$K$2:$K$97,A38)</f>
         <v/>
       </c>
     </row>
@@ -1866,7 +1866,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N96"/>
+  <dimension ref="A1:N97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="C50" s="19" t="inlineStr">
         <is>
-          <t>Pase de lista digital por Secretario o Líder. El Secretario captura y corrige el mismo día; el Líder modifica siempre; el Supervisor solo consulta. La captura sin conexión (NF-06) queda para la siguiente entrega.</t>
+          <t>Pase de lista digital por Secretario o Líder. El Secretario captura y corrige el mismo día; el Líder modifica siempre; el Supervisor solo consulta. Funciona sin conexión: la lista se guarda en el teléfono con la hora real de captura y se envía sola al volver la señal, sin pisar cambios más recientes hechos en línea. Una captura sin conexión se acepta hasta 7 días después y se evalúa contra el día en que se hizo; todo queda en bitácora marcado como diferido.</t>
         </is>
       </c>
       <c r="D50" s="19" t="inlineStr">
@@ -5199,17 +5199,17 @@
       </c>
       <c r="L50" s="19" t="inlineStr">
         <is>
-          <t>En desarrollo</t>
+          <t>En pruebas</t>
         </is>
       </c>
       <c r="M50" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/m3-grupos · 88 pruebas de backend y 7 de frontend pasan</t>
+          <t>Rama feature/nf-06-sin-conexion · 117 pruebas de backend y 27 de frontend; probado en Chrome real con service worker</t>
         </is>
       </c>
       <c r="N50" s="19" t="inlineStr">
         <is>
-          <t>2026-10-24 · Pase de lista listo; falta modo sin conexión (NF-06).</t>
+          <t>2026-10-24 · Pase de lista con y sin conexión.</t>
         </is>
       </c>
     </row>
@@ -5226,7 +5226,7 @@
       </c>
       <c r="C51" s="19" t="inlineStr">
         <is>
-          <t>Ofrendas regulares y especiales (con concepto) por reunión, cuantificables. El Secretario captura el monto; el Tesorero cuenta, escribe su cifra y avala volviendo a escribir su PIN. Si su cifra coincide queda «Avalada»; si no, se registra la diferencia y queda «Con diferencia». Una ofrenda ya capturada solo se corrige con motivo y vuelve a pendiente para un nuevo aval. Quien capturó no puede avalar su propia captura. Líder y Supervisor solo consultan, el Pastor consulta todo y el Anciano no ve finanzas. Todo movimiento queda en bitácora.</t>
+          <t>Ofrendas regulares y especiales (con concepto) por reunión, cuantificables. El Secretario captura el monto; si el grupo no tiene Secretario, lo suple el Líder. El Tesorero cuenta, escribe su cifra y avala volviendo a escribir su PIN; si el grupo no tiene Tesorero, avalan el Líder o el Pastor, nunca quien capturó. Si la cifra coincide queda «Avalada»; si no, se registra la diferencia y queda «Con diferencia», con aviso visible en el grupo, la reunión y la pantalla del Tesorero para quien pueda consultar. Una ofrenda ya capturada solo se corrige con motivo y vuelve a pendiente para un nuevo aval. El Pastor consulta todo, el Líder y el Supervisor consultan y el Anciano no ve finanzas. Toda suplencia, captura, aval y corrección queda en bitácora.</t>
         </is>
       </c>
       <c r="D51" s="19" t="inlineStr">
@@ -5276,12 +5276,12 @@
       </c>
       <c r="M51" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/m3-ofrendas · 111 pruebas de backend y 14 de frontend pasan</t>
+          <t>Rama feature/m3-ofrendas-ajustes · 121 pruebas de backend y 14 de frontend pasan</t>
         </is>
       </c>
       <c r="N51" s="19" t="inlineStr">
         <is>
-          <t>2026-10-24 · Probado de punta a punta con Secretaria y Tesorero distintos; falta validarlo con la iglesia (por ejemplo, qué pasa si el grupo no tiene Secretario).</t>
+          <t>2026-10-24 · Con suplencias del Líder, diferencias visibles y límites configurables. Falta validar con la iglesia.</t>
         </is>
       </c>
     </row>
@@ -5816,42 +5816,42 @@
     <row r="60">
       <c r="A60" s="18" t="inlineStr">
         <is>
-          <t>M4-01</t>
+          <t>M3-13</t>
         </is>
       </c>
       <c r="B60" s="19" t="inlineStr">
         <is>
-          <t>M4 Kids Check-In/Out</t>
+          <t>M3 Grupos de Conexión</t>
         </is>
       </c>
       <c r="C60" s="19" t="inlineStr">
         <is>
-          <t>Sustitución de la ficha física de papel.</t>
-        </is>
-      </c>
-      <c r="D60" s="19" t="inlineStr">
-        <is>
-          <t>v1 / v2</t>
+          <t>Parámetros configurables sin programar, con pantalla de Configuración y cada cambio en bitácora: monto máximo por ofrenda (1,000,000 por defecto) y si se permite una sola ofrenda regular por reunión. Solo Pastor y Administrador Técnico.</t>
+        </is>
+      </c>
+      <c r="D60" s="21" t="inlineStr">
+        <is>
+          <t>Respuesta</t>
         </is>
       </c>
       <c r="E60" s="19" t="inlineStr">
         <is>
-          <t>Fuera del MVP</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="F60" s="19" t="inlineStr">
         <is>
-          <t>Fase 2</t>
+          <t>Fase 1</t>
         </is>
       </c>
       <c r="G60" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sprint 4</t>
         </is>
       </c>
       <c r="H60" s="19" t="inlineStr">
         <is>
-          <t>Posterior</t>
+          <t>H3 · MVP (Grupos)</t>
         </is>
       </c>
       <c r="I60" s="20" t="inlineStr">
@@ -5871,16 +5871,24 @@
       </c>
       <c r="L60" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M60" s="19" t="inlineStr"/>
-      <c r="N60" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M60" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/m3-ofrendas-ajustes · 121 pruebas de backend y 14 de frontend pasan</t>
+        </is>
+      </c>
+      <c r="N60" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-24 · Pantalla Configuración: monto máximo y una regular por reunión.</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="18" t="inlineStr">
         <is>
-          <t>M4-02</t>
+          <t>M4-01</t>
         </is>
       </c>
       <c r="B61" s="19" t="inlineStr">
@@ -5890,12 +5898,12 @@
       </c>
       <c r="C61" s="19" t="inlineStr">
         <is>
-          <t>Registro de ingreso del menor con salón o clase asignada y generación de código único.</t>
-        </is>
-      </c>
-      <c r="D61" s="21" t="inlineStr">
-        <is>
-          <t>v1 + Nuevo v3</t>
+          <t>Sustitución de la ficha física de papel.</t>
+        </is>
+      </c>
+      <c r="D61" s="19" t="inlineStr">
+        <is>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E61" s="19" t="inlineStr">
@@ -5944,7 +5952,7 @@
     <row r="62">
       <c r="A62" s="18" t="inlineStr">
         <is>
-          <t>M4-03</t>
+          <t>M4-02</t>
         </is>
       </c>
       <c r="B62" s="19" t="inlineStr">
@@ -5954,12 +5962,12 @@
       </c>
       <c r="C62" s="19" t="inlineStr">
         <is>
-          <t>Código QR dinámico o OTP temporal en la PWA del padre o tutor.</t>
-        </is>
-      </c>
-      <c r="D62" s="19" t="inlineStr">
-        <is>
-          <t>v2</t>
+          <t>Registro de ingreso del menor con salón o clase asignada y generación de código único.</t>
+        </is>
+      </c>
+      <c r="D62" s="21" t="inlineStr">
+        <is>
+          <t>v1 + Nuevo v3</t>
         </is>
       </c>
       <c r="E62" s="19" t="inlineStr">
@@ -6008,7 +6016,7 @@
     <row r="63">
       <c r="A63" s="18" t="inlineStr">
         <is>
-          <t>M4-04</t>
+          <t>M4-03</t>
         </is>
       </c>
       <c r="B63" s="19" t="inlineStr">
@@ -6018,7 +6026,7 @@
       </c>
       <c r="C63" s="19" t="inlineStr">
         <is>
-          <t>Validación al entregar: el servidor de Kids escanea el código y confirma identidad y fotografía del tutor autorizado en el Expediente Digital.</t>
+          <t>Código QR dinámico o OTP temporal en la PWA del padre o tutor.</t>
         </is>
       </c>
       <c r="D63" s="19" t="inlineStr">
@@ -6072,7 +6080,7 @@
     <row r="64">
       <c r="A64" s="18" t="inlineStr">
         <is>
-          <t>M4-05</t>
+          <t>M4-04</t>
         </is>
       </c>
       <c r="B64" s="19" t="inlineStr">
@@ -6082,12 +6090,12 @@
       </c>
       <c r="C64" s="19" t="inlineStr">
         <is>
-          <t>Alternativa para tutores sin smartphone, sin batería o sin conexión (p. ej. código por SMS o comprobante imprimible con identificación). Por definir.</t>
-        </is>
-      </c>
-      <c r="D64" s="21" t="inlineStr">
-        <is>
-          <t>Nuevo v3</t>
+          <t>Validación al entregar: el servidor de Kids escanea el código y confirma identidad y fotografía del tutor autorizado en el Expediente Digital.</t>
+        </is>
+      </c>
+      <c r="D64" s="19" t="inlineStr">
+        <is>
+          <t>v2</t>
         </is>
       </c>
       <c r="E64" s="19" t="inlineStr">
@@ -6122,7 +6130,7 @@
       </c>
       <c r="K64" s="19" t="inlineStr">
         <is>
-          <t>Por definir</t>
+          <t>VoBo pendiente</t>
         </is>
       </c>
       <c r="L64" s="19" t="inlineStr">
@@ -6136,7 +6144,7 @@
     <row r="65">
       <c r="A65" s="18" t="inlineStr">
         <is>
-          <t>M4-06</t>
+          <t>M4-05</t>
         </is>
       </c>
       <c r="B65" s="19" t="inlineStr">
@@ -6146,7 +6154,7 @@
       </c>
       <c r="C65" s="19" t="inlineStr">
         <is>
-          <t>Autorización temporal de un tercero para recoger al menor, con aprobación del tutor registrado.</t>
+          <t>Alternativa para tutores sin smartphone, sin batería o sin conexión (p. ej. código por SMS o comprobante imprimible con identificación). Por definir.</t>
         </is>
       </c>
       <c r="D65" s="21" t="inlineStr">
@@ -6186,7 +6194,7 @@
       </c>
       <c r="K65" s="19" t="inlineStr">
         <is>
-          <t>VoBo pendiente</t>
+          <t>Por definir</t>
         </is>
       </c>
       <c r="L65" s="19" t="inlineStr">
@@ -6200,7 +6208,7 @@
     <row r="66">
       <c r="A66" s="18" t="inlineStr">
         <is>
-          <t>M4-07</t>
+          <t>M4-06</t>
         </is>
       </c>
       <c r="B66" s="19" t="inlineStr">
@@ -6210,7 +6218,7 @@
       </c>
       <c r="C66" s="19" t="inlineStr">
         <is>
-          <t>Caducidad del código y bitácora de cada entrega (quién recogió, quién entregó, hora).</t>
+          <t>Autorización temporal de un tercero para recoger al menor, con aprobación del tutor registrado.</t>
         </is>
       </c>
       <c r="D66" s="21" t="inlineStr">
@@ -6264,7 +6272,7 @@
     <row r="67">
       <c r="A67" s="18" t="inlineStr">
         <is>
-          <t>M4-08</t>
+          <t>M4-07</t>
         </is>
       </c>
       <c r="B67" s="19" t="inlineStr">
@@ -6274,7 +6282,7 @@
       </c>
       <c r="C67" s="19" t="inlineStr">
         <is>
-          <t>Funcionamiento sin conexión o con conexión degradada para el check-out.</t>
+          <t>Caducidad del código y bitácora de cada entrega (quién recogió, quién entregó, hora).</t>
         </is>
       </c>
       <c r="D67" s="21" t="inlineStr">
@@ -6328,52 +6336,52 @@
     <row r="68">
       <c r="A68" s="18" t="inlineStr">
         <is>
-          <t>M5-01</t>
+          <t>M4-08</t>
         </is>
       </c>
       <c r="B68" s="19" t="inlineStr">
         <is>
-          <t>M5 Áreas y servidores</t>
+          <t>M4 Kids Check-In/Out</t>
         </is>
       </c>
       <c r="C68" s="19" t="inlineStr">
         <is>
-          <t>Catálogo mínimo de áreas y asignación de servidores. Versión reducida del módulo 5, necesaria para permisos por área. Sirve como primer censo.</t>
-        </is>
-      </c>
-      <c r="D68" s="19" t="inlineStr">
-        <is>
-          <t>v3</t>
+          <t>Funcionamiento sin conexión o con conexión degradada para el check-out.</t>
+        </is>
+      </c>
+      <c r="D68" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3</t>
         </is>
       </c>
       <c r="E68" s="19" t="inlineStr">
         <is>
-          <t>MVP mínimo</t>
+          <t>Fuera del MVP</t>
         </is>
       </c>
       <c r="F68" s="19" t="inlineStr">
         <is>
-          <t>Fase 0</t>
+          <t>Fase 2</t>
         </is>
       </c>
       <c r="G68" s="19" t="inlineStr">
         <is>
-          <t>Sprint 1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H68" s="19" t="inlineStr">
         <is>
-          <t>H2 · Fase 0 completa</t>
-        </is>
-      </c>
-      <c r="I68" s="19" t="inlineStr">
-        <is>
-          <t>Como pastor quiero un catálogo de áreas con su personal para conocer la estructura.</t>
-        </is>
-      </c>
-      <c r="J68" s="19" t="inlineStr">
-        <is>
-          <t>Crear un área, asignar servidores y ver el conteo real.</t>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="I68" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
+        </is>
+      </c>
+      <c r="J68" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
         </is>
       </c>
       <c r="K68" s="19" t="inlineStr">
@@ -6392,7 +6400,7 @@
     <row r="69">
       <c r="A69" s="18" t="inlineStr">
         <is>
-          <t>M5-02</t>
+          <t>M5-01</t>
         </is>
       </c>
       <c r="B69" s="19" t="inlineStr">
@@ -6402,42 +6410,42 @@
       </c>
       <c r="C69" s="19" t="inlineStr">
         <is>
-          <t>Roles jerárquicos dentro de cada área (directores, líderes, maestros, servidores).</t>
+          <t>Catálogo mínimo de áreas y asignación de servidores. Versión reducida del módulo 5, necesaria para permisos por área. Sirve como primer censo.</t>
         </is>
       </c>
       <c r="D69" s="19" t="inlineStr">
         <is>
-          <t>v1</t>
+          <t>v3</t>
         </is>
       </c>
       <c r="E69" s="19" t="inlineStr">
         <is>
-          <t>Fuera del MVP</t>
+          <t>MVP mínimo</t>
         </is>
       </c>
       <c r="F69" s="19" t="inlineStr">
         <is>
-          <t>Fase 4</t>
+          <t>Fase 0</t>
         </is>
       </c>
       <c r="G69" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sprint 1</t>
         </is>
       </c>
       <c r="H69" s="19" t="inlineStr">
         <is>
-          <t>Posterior</t>
-        </is>
-      </c>
-      <c r="I69" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
-        </is>
-      </c>
-      <c r="J69" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
+          <t>H2 · Fase 0 completa</t>
+        </is>
+      </c>
+      <c r="I69" s="19" t="inlineStr">
+        <is>
+          <t>Como pastor quiero un catálogo de áreas con su personal para conocer la estructura.</t>
+        </is>
+      </c>
+      <c r="J69" s="19" t="inlineStr">
+        <is>
+          <t>Crear un área, asignar servidores y ver el conteo real.</t>
         </is>
       </c>
       <c r="K69" s="19" t="inlineStr">
@@ -6456,7 +6464,7 @@
     <row r="70">
       <c r="A70" s="18" t="inlineStr">
         <is>
-          <t>M5-03</t>
+          <t>M5-02</t>
         </is>
       </c>
       <c r="B70" s="19" t="inlineStr">
@@ -6466,12 +6474,12 @@
       </c>
       <c r="C70" s="19" t="inlineStr">
         <is>
-          <t>Organigrama y número real de servidores activos, directores y líderes por área.</t>
+          <t>Roles jerárquicos dentro de cada área (directores, líderes, maestros, servidores).</t>
         </is>
       </c>
       <c r="D70" s="19" t="inlineStr">
         <is>
-          <t>v2</t>
+          <t>v1</t>
         </is>
       </c>
       <c r="E70" s="19" t="inlineStr">
@@ -6520,7 +6528,7 @@
     <row r="71">
       <c r="A71" s="18" t="inlineStr">
         <is>
-          <t>M5-04</t>
+          <t>M5-03</t>
         </is>
       </c>
       <c r="B71" s="19" t="inlineStr">
@@ -6530,12 +6538,12 @@
       </c>
       <c r="C71" s="19" t="inlineStr">
         <is>
-          <t>Control de asistencia a turnos o servicios.</t>
+          <t>Organigrama y número real de servidores activos, directores y líderes por área.</t>
         </is>
       </c>
       <c r="D71" s="19" t="inlineStr">
         <is>
-          <t>v1 / v2</t>
+          <t>v2</t>
         </is>
       </c>
       <c r="E71" s="19" t="inlineStr">
@@ -6584,7 +6592,7 @@
     <row r="72">
       <c r="A72" s="18" t="inlineStr">
         <is>
-          <t>M5-05</t>
+          <t>M5-04</t>
         </is>
       </c>
       <c r="B72" s="19" t="inlineStr">
@@ -6594,7 +6602,7 @@
       </c>
       <c r="C72" s="19" t="inlineStr">
         <is>
-          <t>Tablero de avisos y notificaciones interno por área.</t>
+          <t>Control de asistencia a turnos o servicios.</t>
         </is>
       </c>
       <c r="D72" s="19" t="inlineStr">
@@ -6648,7 +6656,7 @@
     <row r="73">
       <c r="A73" s="18" t="inlineStr">
         <is>
-          <t>M5-06</t>
+          <t>M5-05</t>
         </is>
       </c>
       <c r="B73" s="19" t="inlineStr">
@@ -6658,7 +6666,7 @@
       </c>
       <c r="C73" s="19" t="inlineStr">
         <is>
-          <t>Gestión financiera por área: caja chica y gastos operativos.</t>
+          <t>Tablero de avisos y notificaciones interno por área.</t>
         </is>
       </c>
       <c r="D73" s="19" t="inlineStr">
@@ -6712,22 +6720,22 @@
     <row r="74">
       <c r="A74" s="18" t="inlineStr">
         <is>
-          <t>M6-01</t>
+          <t>M5-06</t>
         </is>
       </c>
       <c r="B74" s="19" t="inlineStr">
         <is>
-          <t>M6 Ministerios de servicio</t>
+          <t>M5 Áreas y servidores</t>
         </is>
       </c>
       <c r="C74" s="19" t="inlineStr">
         <is>
-          <t>Control de personal propio de cada ministerio.</t>
-        </is>
-      </c>
-      <c r="D74" s="22" t="inlineStr">
-        <is>
-          <t>Recuperado v1</t>
+          <t>Gestión financiera por área: caja chica y gastos operativos.</t>
+        </is>
+      </c>
+      <c r="D74" s="19" t="inlineStr">
+        <is>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E74" s="19" t="inlineStr">
@@ -6776,7 +6784,7 @@
     <row r="75">
       <c r="A75" s="18" t="inlineStr">
         <is>
-          <t>M6-02</t>
+          <t>M6-01</t>
         </is>
       </c>
       <c r="B75" s="19" t="inlineStr">
@@ -6786,12 +6794,12 @@
       </c>
       <c r="C75" s="19" t="inlineStr">
         <is>
-          <t>Menú o catálogo digital interactivo (público o interno), autogestionado.</t>
-        </is>
-      </c>
-      <c r="D75" s="19" t="inlineStr">
-        <is>
-          <t>v1 / v2</t>
+          <t>Control de personal propio de cada ministerio.</t>
+        </is>
+      </c>
+      <c r="D75" s="22" t="inlineStr">
+        <is>
+          <t>Recuperado v1</t>
         </is>
       </c>
       <c r="E75" s="19" t="inlineStr">
@@ -6840,7 +6848,7 @@
     <row r="76">
       <c r="A76" s="18" t="inlineStr">
         <is>
-          <t>M6-03</t>
+          <t>M6-02</t>
         </is>
       </c>
       <c r="B76" s="19" t="inlineStr">
@@ -6850,7 +6858,7 @@
       </c>
       <c r="C76" s="19" t="inlineStr">
         <is>
-          <t>Calendario de turnos: días regulares de servicio y eventos especiales.</t>
+          <t>Menú o catálogo digital interactivo (público o interno), autogestionado.</t>
         </is>
       </c>
       <c r="D76" s="19" t="inlineStr">
@@ -6904,7 +6912,7 @@
     <row r="77">
       <c r="A77" s="18" t="inlineStr">
         <is>
-          <t>M6-04</t>
+          <t>M6-03</t>
         </is>
       </c>
       <c r="B77" s="19" t="inlineStr">
@@ -6914,7 +6922,7 @@
       </c>
       <c r="C77" s="19" t="inlineStr">
         <is>
-          <t>Registro de asistentes o personas atendidas.</t>
+          <t>Calendario de turnos: días regulares de servicio y eventos especiales.</t>
         </is>
       </c>
       <c r="D77" s="19" t="inlineStr">
@@ -6968,7 +6976,7 @@
     <row r="78">
       <c r="A78" s="18" t="inlineStr">
         <is>
-          <t>M6-05</t>
+          <t>M6-04</t>
         </is>
       </c>
       <c r="B78" s="19" t="inlineStr">
@@ -6978,7 +6986,7 @@
       </c>
       <c r="C78" s="19" t="inlineStr">
         <is>
-          <t>Control de gastos y de inventario básico.</t>
+          <t>Registro de asistentes o personas atendidas.</t>
         </is>
       </c>
       <c r="D78" s="19" t="inlineStr">
@@ -7032,7 +7040,7 @@
     <row r="79">
       <c r="A79" s="18" t="inlineStr">
         <is>
-          <t>M6-06</t>
+          <t>M6-05</t>
         </is>
       </c>
       <c r="B79" s="19" t="inlineStr">
@@ -7042,7 +7050,7 @@
       </c>
       <c r="C79" s="19" t="inlineStr">
         <is>
-          <t>Canal de comunicación directo con el área de Administración General.</t>
+          <t>Control de gastos y de inventario básico.</t>
         </is>
       </c>
       <c r="D79" s="19" t="inlineStr">
@@ -7096,7 +7104,7 @@
     <row r="80">
       <c r="A80" s="18" t="inlineStr">
         <is>
-          <t>M6-07</t>
+          <t>M6-06</t>
         </is>
       </c>
       <c r="B80" s="19" t="inlineStr">
@@ -7106,12 +7114,12 @@
       </c>
       <c r="C80" s="19" t="inlineStr">
         <is>
-          <t>Servicio Médico: los datos de salud de las personas atendidas requieren tratamiento de datos sensibles. Por definir alcance.</t>
-        </is>
-      </c>
-      <c r="D80" s="21" t="inlineStr">
-        <is>
-          <t>Nuevo v3</t>
+          <t>Canal de comunicación directo con el área de Administración General.</t>
+        </is>
+      </c>
+      <c r="D80" s="19" t="inlineStr">
+        <is>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E80" s="19" t="inlineStr">
@@ -7146,7 +7154,7 @@
       </c>
       <c r="K80" s="19" t="inlineStr">
         <is>
-          <t>Por definir</t>
+          <t>VoBo pendiente</t>
         </is>
       </c>
       <c r="L80" s="19" t="inlineStr">
@@ -7160,22 +7168,22 @@
     <row r="81">
       <c r="A81" s="18" t="inlineStr">
         <is>
-          <t>M7-01</t>
+          <t>M6-07</t>
         </is>
       </c>
       <c r="B81" s="19" t="inlineStr">
         <is>
-          <t>M7 Eventos y aforo</t>
+          <t>M6 Ministerios de servicio</t>
         </is>
       </c>
       <c r="C81" s="19" t="inlineStr">
         <is>
-          <t>Eventos abiertos o evangelísticos con formulario de inscripción rápida, sin requerir historial previo.</t>
-        </is>
-      </c>
-      <c r="D81" s="19" t="inlineStr">
-        <is>
-          <t>v1 / v2</t>
+          <t>Servicio Médico: los datos de salud de las personas atendidas requieren tratamiento de datos sensibles. Por definir alcance.</t>
+        </is>
+      </c>
+      <c r="D81" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3</t>
         </is>
       </c>
       <c r="E81" s="19" t="inlineStr">
@@ -7210,7 +7218,7 @@
       </c>
       <c r="K81" s="19" t="inlineStr">
         <is>
-          <t>VoBo pendiente</t>
+          <t>Por definir</t>
         </is>
       </c>
       <c r="L81" s="19" t="inlineStr">
@@ -7224,7 +7232,7 @@
     <row r="82">
       <c r="A82" s="18" t="inlineStr">
         <is>
-          <t>M7-02</t>
+          <t>M7-01</t>
         </is>
       </c>
       <c r="B82" s="19" t="inlineStr">
@@ -7234,12 +7242,12 @@
       </c>
       <c r="C82" s="19" t="inlineStr">
         <is>
-          <t>Consolidación (inducción de personas que asisten por primera vez) como tipo de evento.</t>
-        </is>
-      </c>
-      <c r="D82" s="22" t="inlineStr">
-        <is>
-          <t>Recuperado v1</t>
+          <t>Eventos abiertos o evangelísticos con formulario de inscripción rápida, sin requerir historial previo.</t>
+        </is>
+      </c>
+      <c r="D82" s="19" t="inlineStr">
+        <is>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E82" s="19" t="inlineStr">
@@ -7288,7 +7296,7 @@
     <row r="83">
       <c r="A83" s="18" t="inlineStr">
         <is>
-          <t>M7-03</t>
+          <t>M7-02</t>
         </is>
       </c>
       <c r="B83" s="19" t="inlineStr">
@@ -7298,7 +7306,7 @@
       </c>
       <c r="C83" s="19" t="inlineStr">
         <is>
-          <t>Encargados de evento (personal de la iglesia únicamente; no se controla personal externo).</t>
+          <t>Consolidación (inducción de personas que asisten por primera vez) como tipo de evento.</t>
         </is>
       </c>
       <c r="D83" s="22" t="inlineStr">
@@ -7352,7 +7360,7 @@
     <row r="84">
       <c r="A84" s="18" t="inlineStr">
         <is>
-          <t>M7-04</t>
+          <t>M7-03</t>
         </is>
       </c>
       <c r="B84" s="19" t="inlineStr">
@@ -7362,12 +7370,12 @@
       </c>
       <c r="C84" s="19" t="inlineStr">
         <is>
-          <t>Control de cupo en tiempo real que bloquea el sobrecupo en eventos con aforo limitado (ej. 30 o 50 lugares).</t>
-        </is>
-      </c>
-      <c r="D84" s="19" t="inlineStr">
-        <is>
-          <t>v1 / v2</t>
+          <t>Encargados de evento (personal de la iglesia únicamente; no se controla personal externo).</t>
+        </is>
+      </c>
+      <c r="D84" s="22" t="inlineStr">
+        <is>
+          <t>Recuperado v1</t>
         </is>
       </c>
       <c r="E84" s="19" t="inlineStr">
@@ -7416,7 +7424,7 @@
     <row r="85">
       <c r="A85" s="18" t="inlineStr">
         <is>
-          <t>M7-05</t>
+          <t>M7-04</t>
         </is>
       </c>
       <c r="B85" s="19" t="inlineStr">
@@ -7426,12 +7434,12 @@
       </c>
       <c r="C85" s="19" t="inlineStr">
         <is>
-          <t>Control de asistentes sin lista previa, para aforo y para dar a conocer la iglesia.</t>
+          <t>Control de cupo en tiempo real que bloquea el sobrecupo en eventos con aforo limitado (ej. 30 o 50 lugares).</t>
         </is>
       </c>
       <c r="D85" s="19" t="inlineStr">
         <is>
-          <t>v1</t>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E85" s="19" t="inlineStr">
@@ -7480,7 +7488,7 @@
     <row r="86">
       <c r="A86" s="18" t="inlineStr">
         <is>
-          <t>M7-06</t>
+          <t>M7-05</t>
         </is>
       </c>
       <c r="B86" s="19" t="inlineStr">
@@ -7490,12 +7498,12 @@
       </c>
       <c r="C86" s="19" t="inlineStr">
         <is>
-          <t>Seguimiento de personas nuevas: conversión de un invitado a Expediente Digital y canalización a un curso o Grupo de Conexión.</t>
-        </is>
-      </c>
-      <c r="D86" s="21" t="inlineStr">
-        <is>
-          <t>Nuevo v3</t>
+          <t>Control de asistentes sin lista previa, para aforo y para dar a conocer la iglesia.</t>
+        </is>
+      </c>
+      <c r="D86" s="19" t="inlineStr">
+        <is>
+          <t>v1</t>
         </is>
       </c>
       <c r="E86" s="19" t="inlineStr">
@@ -7544,52 +7552,52 @@
     <row r="87">
       <c r="A87" s="18" t="inlineStr">
         <is>
-          <t>NF-01</t>
+          <t>M7-06</t>
         </is>
       </c>
       <c r="B87" s="19" t="inlineStr">
         <is>
-          <t>No funcionales</t>
+          <t>M7 Eventos y aforo</t>
         </is>
       </c>
       <c r="C87" s="19" t="inlineStr">
         <is>
-          <t>Cumplimiento de la LFPDPPP: aviso de privacidad, consentimiento y derechos ARCO.</t>
-        </is>
-      </c>
-      <c r="D87" s="19" t="inlineStr">
-        <is>
-          <t>v3</t>
+          <t>Seguimiento de personas nuevas: conversión de un invitado a Expediente Digital y canalización a un curso o Grupo de Conexión.</t>
+        </is>
+      </c>
+      <c r="D87" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3</t>
         </is>
       </c>
       <c r="E87" s="19" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Fuera del MVP</t>
         </is>
       </c>
       <c r="F87" s="19" t="inlineStr">
         <is>
-          <t>Fase 0</t>
+          <t>Fase 4</t>
         </is>
       </c>
       <c r="G87" s="19" t="inlineStr">
         <is>
-          <t>Sprint 1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H87" s="19" t="inlineStr">
         <is>
-          <t>H1 · 18-oct (núcleo Fase 0)</t>
-        </is>
-      </c>
-      <c r="I87" s="19" t="inlineStr">
-        <is>
-          <t>Como iglesia queremos cumplir con la LFPDPPP.</t>
-        </is>
-      </c>
-      <c r="J87" s="19" t="inlineStr">
-        <is>
-          <t>Aviso de privacidad, consentimiento y atención de derechos ARCO disponibles.</t>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="I87" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
+        </is>
+      </c>
+      <c r="J87" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
         </is>
       </c>
       <c r="K87" s="19" t="inlineStr">
@@ -7608,7 +7616,7 @@
     <row r="88">
       <c r="A88" s="18" t="inlineStr">
         <is>
-          <t>NF-02</t>
+          <t>NF-01</t>
         </is>
       </c>
       <c r="B88" s="19" t="inlineStr">
@@ -7618,7 +7626,7 @@
       </c>
       <c r="C88" s="19" t="inlineStr">
         <is>
-          <t>Cifrado en tránsito y en reposo. Cifrado adicional a nivel de campo para peticiones de oración.</t>
+          <t>Cumplimiento de la LFPDPPP: aviso de privacidad, consentimiento y derechos ARCO.</t>
         </is>
       </c>
       <c r="D88" s="19" t="inlineStr">
@@ -7638,7 +7646,7 @@
       </c>
       <c r="G88" s="19" t="inlineStr">
         <is>
-          <t>Sprint 0</t>
+          <t>Sprint 1</t>
         </is>
       </c>
       <c r="H88" s="19" t="inlineStr">
@@ -7648,12 +7656,12 @@
       </c>
       <c r="I88" s="19" t="inlineStr">
         <is>
-          <t>Como iglesia queremos proteger los datos sensibles.</t>
+          <t>Como iglesia queremos cumplir con la LFPDPPP.</t>
         </is>
       </c>
       <c r="J88" s="19" t="inlineStr">
         <is>
-          <t>HTTPS obligatorio y peticiones de oración ilegibles directamente en la base.</t>
+          <t>Aviso de privacidad, consentimiento y atención de derechos ARCO disponibles.</t>
         </is>
       </c>
       <c r="K88" s="19" t="inlineStr">
@@ -7672,7 +7680,7 @@
     <row r="89">
       <c r="A89" s="18" t="inlineStr">
         <is>
-          <t>NF-03</t>
+          <t>NF-02</t>
         </is>
       </c>
       <c r="B89" s="19" t="inlineStr">
@@ -7682,7 +7690,7 @@
       </c>
       <c r="C89" s="19" t="inlineStr">
         <is>
-          <t>Bitácora de auditoría de solo-añadir: quién consultó o modificó expedientes, ofrendas y asistencias.</t>
+          <t>Cifrado en tránsito y en reposo. Cifrado adicional a nivel de campo para peticiones de oración.</t>
         </is>
       </c>
       <c r="D89" s="19" t="inlineStr">
@@ -7702,7 +7710,7 @@
       </c>
       <c r="G89" s="19" t="inlineStr">
         <is>
-          <t>Sprint 1</t>
+          <t>Sprint 0</t>
         </is>
       </c>
       <c r="H89" s="19" t="inlineStr">
@@ -7712,12 +7720,12 @@
       </c>
       <c r="I89" s="19" t="inlineStr">
         <is>
-          <t>Como pastor quiero una bitácora que nadie pueda alterar.</t>
+          <t>Como iglesia queremos proteger los datos sensibles.</t>
         </is>
       </c>
       <c r="J89" s="19" t="inlineStr">
         <is>
-          <t>El usuario de la aplicación no puede actualizar ni borrar registros de bitácora.</t>
+          <t>HTTPS obligatorio y peticiones de oración ilegibles directamente en la base.</t>
         </is>
       </c>
       <c r="K89" s="19" t="inlineStr">
@@ -7727,24 +7735,16 @@
       </c>
       <c r="L89" s="19" t="inlineStr">
         <is>
-          <t>En pruebas</t>
-        </is>
-      </c>
-      <c r="M89" s="19" t="inlineStr">
-        <is>
-          <t>Rama feature/nf-03-bitacora · 69 pruebas de backend pasan</t>
-        </is>
-      </c>
-      <c r="N89" s="19" t="inlineStr">
-        <is>
-          <t>2026-10-10 · Bloqueo en aplicación y trigger de PostgreSQL (UPDATE/DELETE/TRUNCATE); pantalla de consulta con permiso bitacora.ver.</t>
-        </is>
-      </c>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M89" s="19" t="inlineStr"/>
+      <c r="N89" s="19" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="18" t="inlineStr">
         <is>
-          <t>NF-04</t>
+          <t>NF-03</t>
         </is>
       </c>
       <c r="B90" s="19" t="inlineStr">
@@ -7754,7 +7754,7 @@
       </c>
       <c r="C90" s="19" t="inlineStr">
         <is>
-          <t>Respaldos automáticos diarios cifrados y prueba periódica de restauración.</t>
+          <t>Bitácora de auditoría de solo-añadir: quién consultó o modificó expedientes, ofrendas y asistencias.</t>
         </is>
       </c>
       <c r="D90" s="19" t="inlineStr">
@@ -7774,7 +7774,7 @@
       </c>
       <c r="G90" s="19" t="inlineStr">
         <is>
-          <t>Sprint 0</t>
+          <t>Sprint 1</t>
         </is>
       </c>
       <c r="H90" s="19" t="inlineStr">
@@ -7784,12 +7784,12 @@
       </c>
       <c r="I90" s="19" t="inlineStr">
         <is>
-          <t>Como iglesia queremos no perder información.</t>
+          <t>Como pastor quiero una bitácora que nadie pueda alterar.</t>
         </is>
       </c>
       <c r="J90" s="19" t="inlineStr">
         <is>
-          <t>Respaldo diario cifrado y restauración probada en un ambiente de pruebas.</t>
+          <t>El usuario de la aplicación no puede actualizar ni borrar registros de bitácora.</t>
         </is>
       </c>
       <c r="K90" s="19" t="inlineStr">
@@ -7799,16 +7799,24 @@
       </c>
       <c r="L90" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M90" s="19" t="inlineStr"/>
-      <c r="N90" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M90" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/nf-03-bitacora · 69 pruebas de backend pasan</t>
+        </is>
+      </c>
+      <c r="N90" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-10 · Bloqueo en aplicación y trigger de PostgreSQL (UPDATE/DELETE/TRUNCATE); pantalla de consulta con permiso bitacora.ver.</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="18" t="inlineStr">
         <is>
-          <t>NF-05</t>
+          <t>NF-04</t>
         </is>
       </c>
       <c r="B91" s="19" t="inlineStr">
@@ -7818,47 +7826,47 @@
       </c>
       <c r="C91" s="19" t="inlineStr">
         <is>
-          <t>Disponibilidad esperada en horarios de servicio (fines de semana y reuniones de grupo). Por definir meta.</t>
-        </is>
-      </c>
-      <c r="D91" s="21" t="inlineStr">
-        <is>
-          <t>Nuevo v3</t>
+          <t>Respaldos automáticos diarios cifrados y prueba periódica de restauración.</t>
+        </is>
+      </c>
+      <c r="D91" s="19" t="inlineStr">
+        <is>
+          <t>v3</t>
         </is>
       </c>
       <c r="E91" s="19" t="inlineStr">
         <is>
-          <t>Fuera del MVP</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="F91" s="19" t="inlineStr">
         <is>
-          <t>Transversal</t>
+          <t>Fase 0</t>
         </is>
       </c>
       <c r="G91" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sprint 0</t>
         </is>
       </c>
       <c r="H91" s="19" t="inlineStr">
         <is>
-          <t>Posterior</t>
-        </is>
-      </c>
-      <c r="I91" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
-        </is>
-      </c>
-      <c r="J91" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
+          <t>H1 · 18-oct (núcleo Fase 0)</t>
+        </is>
+      </c>
+      <c r="I91" s="19" t="inlineStr">
+        <is>
+          <t>Como iglesia queremos no perder información.</t>
+        </is>
+      </c>
+      <c r="J91" s="19" t="inlineStr">
+        <is>
+          <t>Respaldo diario cifrado y restauración probada en un ambiente de pruebas.</t>
         </is>
       </c>
       <c r="K91" s="19" t="inlineStr">
         <is>
-          <t>Por definir</t>
+          <t>VoBo pendiente</t>
         </is>
       </c>
       <c r="L91" s="19" t="inlineStr">
@@ -7872,7 +7880,7 @@
     <row r="92">
       <c r="A92" s="18" t="inlineStr">
         <is>
-          <t>NF-06</t>
+          <t>NF-05</t>
         </is>
       </c>
       <c r="B92" s="19" t="inlineStr">
@@ -7882,47 +7890,47 @@
       </c>
       <c r="C92" s="19" t="inlineStr">
         <is>
-          <t>Pase de lista sin conexión con sincronización posterior (reuniones en domicilios con mala señal).</t>
-        </is>
-      </c>
-      <c r="D92" s="19" t="inlineStr">
-        <is>
-          <t>v3</t>
+          <t>Disponibilidad esperada en horarios de servicio (fines de semana y reuniones de grupo). Por definir meta.</t>
+        </is>
+      </c>
+      <c r="D92" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3</t>
         </is>
       </c>
       <c r="E92" s="19" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Fuera del MVP</t>
         </is>
       </c>
       <c r="F92" s="19" t="inlineStr">
         <is>
-          <t>Fase 0</t>
+          <t>Transversal</t>
         </is>
       </c>
       <c r="G92" s="19" t="inlineStr">
         <is>
-          <t>Sprint 3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H92" s="19" t="inlineStr">
         <is>
-          <t>H3 · MVP (Grupos)</t>
-        </is>
-      </c>
-      <c r="I92" s="19" t="inlineStr">
-        <is>
-          <t>Como secretario quiero que el pase de lista funcione sin señal.</t>
-        </is>
-      </c>
-      <c r="J92" s="19" t="inlineStr">
-        <is>
-          <t>Prueba en modo avión y sincronización al reconectar.</t>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="I92" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
+        </is>
+      </c>
+      <c r="J92" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
         </is>
       </c>
       <c r="K92" s="19" t="inlineStr">
         <is>
-          <t>VoBo pendiente</t>
+          <t>Por definir</t>
         </is>
       </c>
       <c r="L92" s="19" t="inlineStr">
@@ -7936,7 +7944,7 @@
     <row r="93">
       <c r="A93" s="18" t="inlineStr">
         <is>
-          <t>NF-07</t>
+          <t>NF-06</t>
         </is>
       </c>
       <c r="B93" s="19" t="inlineStr">
@@ -7946,7 +7954,7 @@
       </c>
       <c r="C93" s="19" t="inlineStr">
         <is>
-          <t>Funciona en Android, iOS y escritorio. En iOS, las notificaciones push requieren instalar la PWA; el respaldo por WhatsApp cubre el resto.</t>
+          <t>Pase de lista sin conexión con sincronización posterior (reuniones en domicilios con mala señal).</t>
         </is>
       </c>
       <c r="D93" s="19" t="inlineStr">
@@ -7966,22 +7974,22 @@
       </c>
       <c r="G93" s="19" t="inlineStr">
         <is>
-          <t>Sprint 0</t>
+          <t>Sprint 3</t>
         </is>
       </c>
       <c r="H93" s="19" t="inlineStr">
         <is>
-          <t>H1 · 18-oct (núcleo Fase 0)</t>
+          <t>H3 · MVP (Grupos)</t>
         </is>
       </c>
       <c r="I93" s="19" t="inlineStr">
         <is>
-          <t>Como usuario quiero usar el sistema en mi dispositivo.</t>
+          <t>Como secretario quiero que el pase de lista funcione sin señal.</t>
         </is>
       </c>
       <c r="J93" s="19" t="inlineStr">
         <is>
-          <t>Pruebas en Android, iOS y escritorio; push en iOS con la PWA instalada y respaldo por WhatsApp.</t>
+          <t>Prueba en modo avión y sincronización al reconectar.</t>
         </is>
       </c>
       <c r="K93" s="19" t="inlineStr">
@@ -7991,16 +7999,24 @@
       </c>
       <c r="L93" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M93" s="19" t="inlineStr"/>
-      <c r="N93" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M93" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/nf-06-sin-conexion · 117 pruebas de backend y 27 de frontend; probado en Chrome real con service worker</t>
+        </is>
+      </c>
+      <c r="N93" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-24 · Probado de punta a punta en Chrome (sin red → cola → sincronización). Pendiente probar en Android e iOS reales.</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="18" t="inlineStr">
         <is>
-          <t>NF-08</t>
+          <t>NF-07</t>
         </is>
       </c>
       <c r="B94" s="19" t="inlineStr">
@@ -8010,12 +8026,12 @@
       </c>
       <c r="C94" s="19" t="inlineStr">
         <is>
-          <t>Dimensionamiento para ~1,000 personas, con picos los fines de semana, y margen de crecimiento.</t>
-        </is>
-      </c>
-      <c r="D94" s="21" t="inlineStr">
-        <is>
-          <t>Resp. P8</t>
+          <t>Funciona en Android, iOS y escritorio. En iOS, las notificaciones push requieren instalar la PWA; el respaldo por WhatsApp cubre el resto.</t>
+        </is>
+      </c>
+      <c r="D94" s="19" t="inlineStr">
+        <is>
+          <t>v3</t>
         </is>
       </c>
       <c r="E94" s="19" t="inlineStr">
@@ -8040,12 +8056,12 @@
       </c>
       <c r="I94" s="19" t="inlineStr">
         <is>
-          <t>Como iglesia queremos que el sistema soporte a ~1,000 personas.</t>
+          <t>Como usuario quiero usar el sistema en mi dispositivo.</t>
         </is>
       </c>
       <c r="J94" s="19" t="inlineStr">
         <is>
-          <t>Prueba de carga con volumen representativo (por definir) sin degradación.</t>
+          <t>Pruebas en Android, iOS y escritorio; push en iOS con la PWA instalada y respaldo por WhatsApp.</t>
         </is>
       </c>
       <c r="K94" s="19" t="inlineStr">
@@ -8064,7 +8080,7 @@
     <row r="95">
       <c r="A95" s="18" t="inlineStr">
         <is>
-          <t>NF-09</t>
+          <t>NF-08</t>
         </is>
       </c>
       <c r="B95" s="19" t="inlineStr">
@@ -8074,42 +8090,42 @@
       </c>
       <c r="C95" s="19" t="inlineStr">
         <is>
-          <t>Reportes transversales: asistencia, finanzas, crecimiento de la iglesia, exportables a Excel y PDF.</t>
+          <t>Dimensionamiento para ~1,000 personas, con picos los fines de semana, y margen de crecimiento.</t>
         </is>
       </c>
       <c r="D95" s="21" t="inlineStr">
         <is>
-          <t>Nuevo v3</t>
+          <t>Resp. P8</t>
         </is>
       </c>
       <c r="E95" s="19" t="inlineStr">
         <is>
-          <t>Fuera del MVP</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="F95" s="19" t="inlineStr">
         <is>
-          <t>Transversal</t>
+          <t>Fase 0</t>
         </is>
       </c>
       <c r="G95" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sprint 0</t>
         </is>
       </c>
       <c r="H95" s="19" t="inlineStr">
         <is>
-          <t>Posterior</t>
-        </is>
-      </c>
-      <c r="I95" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
-        </is>
-      </c>
-      <c r="J95" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
+          <t>H1 · 18-oct (núcleo Fase 0)</t>
+        </is>
+      </c>
+      <c r="I95" s="19" t="inlineStr">
+        <is>
+          <t>Como iglesia queremos que el sistema soporte a ~1,000 personas.</t>
+        </is>
+      </c>
+      <c r="J95" s="19" t="inlineStr">
+        <is>
+          <t>Prueba de carga con volumen representativo (por definir) sin degradación.</t>
         </is>
       </c>
       <c r="K95" s="19" t="inlineStr">
@@ -8128,7 +8144,7 @@
     <row r="96">
       <c r="A96" s="18" t="inlineStr">
         <is>
-          <t>NF-10</t>
+          <t>NF-09</t>
         </is>
       </c>
       <c r="B96" s="19" t="inlineStr">
@@ -8138,42 +8154,42 @@
       </c>
       <c r="C96" s="19" t="inlineStr">
         <is>
-          <t>Usabilidad para personas mayores: tipografía grande, alto contraste, flujos cortos (ver sección 5).</t>
-        </is>
-      </c>
-      <c r="D96" s="19" t="inlineStr">
-        <is>
-          <t>v3 + Obs. 1</t>
+          <t>Reportes transversales: asistencia, finanzas, crecimiento de la iglesia, exportables a Excel y PDF.</t>
+        </is>
+      </c>
+      <c r="D96" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3</t>
         </is>
       </c>
       <c r="E96" s="19" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Fuera del MVP</t>
         </is>
       </c>
       <c r="F96" s="19" t="inlineStr">
         <is>
-          <t>Fase 0</t>
+          <t>Transversal</t>
         </is>
       </c>
       <c r="G96" s="19" t="inlineStr">
         <is>
-          <t>Sprint 0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H96" s="19" t="inlineStr">
         <is>
-          <t>H1 · 18-oct (núcleo Fase 0)</t>
-        </is>
-      </c>
-      <c r="I96" s="19" t="inlineStr">
-        <is>
-          <t>Como persona mayor quiero una interfaz fácil de leer y usar.</t>
-        </is>
-      </c>
-      <c r="J96" s="19" t="inlineStr">
-        <is>
-          <t>Texto base 18 px, botones de al menos 48 px, contraste AA; prueba con usuarios mayores.</t>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="I96" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
+        </is>
+      </c>
+      <c r="J96" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
         </is>
       </c>
       <c r="K96" s="19" t="inlineStr">
@@ -8189,9 +8205,73 @@
       <c r="M96" s="19" t="inlineStr"/>
       <c r="N96" s="19" t="inlineStr"/>
     </row>
+    <row r="97">
+      <c r="A97" s="18" t="inlineStr">
+        <is>
+          <t>NF-10</t>
+        </is>
+      </c>
+      <c r="B97" s="19" t="inlineStr">
+        <is>
+          <t>No funcionales</t>
+        </is>
+      </c>
+      <c r="C97" s="19" t="inlineStr">
+        <is>
+          <t>Usabilidad para personas mayores: tipografía grande, alto contraste, flujos cortos (ver sección 5).</t>
+        </is>
+      </c>
+      <c r="D97" s="19" t="inlineStr">
+        <is>
+          <t>v3 + Obs. 1</t>
+        </is>
+      </c>
+      <c r="E97" s="19" t="inlineStr">
+        <is>
+          <t>MVP</t>
+        </is>
+      </c>
+      <c r="F97" s="19" t="inlineStr">
+        <is>
+          <t>Fase 0</t>
+        </is>
+      </c>
+      <c r="G97" s="19" t="inlineStr">
+        <is>
+          <t>Sprint 0</t>
+        </is>
+      </c>
+      <c r="H97" s="19" t="inlineStr">
+        <is>
+          <t>H1 · 18-oct (núcleo Fase 0)</t>
+        </is>
+      </c>
+      <c r="I97" s="19" t="inlineStr">
+        <is>
+          <t>Como persona mayor quiero una interfaz fácil de leer y usar.</t>
+        </is>
+      </c>
+      <c r="J97" s="19" t="inlineStr">
+        <is>
+          <t>Texto base 18 px, botones de al menos 48 px, contraste AA; prueba con usuarios mayores.</t>
+        </is>
+      </c>
+      <c r="K97" s="19" t="inlineStr">
+        <is>
+          <t>VoBo pendiente</t>
+        </is>
+      </c>
+      <c r="L97" s="19" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M97" s="19" t="inlineStr"/>
+      <c r="N97" s="19" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N96"/>
-  <conditionalFormatting sqref="L2:L96">
+  <autoFilter ref="A1:N97"/>
+  <conditionalFormatting sqref="L2:L97">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$L2="Hecho"</formula>
     </cfRule>
@@ -8208,7 +8288,7 @@
       <formula>$L2="Bloqueado"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K2:K96">
+  <conditionalFormatting sqref="K2:K97">
     <cfRule type="expression" priority="6" dxfId="0">
       <formula>$K2="Aprobado"</formula>
     </cfRule>
@@ -8216,16 +8296,16 @@
       <formula>$K2="Por definir"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H2:H96">
+  <conditionalFormatting sqref="H2:H97">
     <cfRule type="expression" priority="8" dxfId="5">
       <formula>LEFT($H2,2)="H1"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="L2:L96" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="L2:L97" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Pendiente,En diseño,En desarrollo,En pruebas,Hecho,Bloqueado"</formula1>
     </dataValidation>
-    <dataValidation sqref="K2:K96" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="K2:K97" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"VoBo pendiente,Aprobado,Por definir,Rechazado"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
M3-05/M3-06/M3-14: peticiones de oración como componente reutilizable
- Módulo propio con origen registrable: cada petición guarda su origen (tipo, id y etiqueta fija)
  de forma inmutable y lo muestra siempre; Grupos de Conexión es el primer origen
- Formulario configurable y versionado (campos que se desactivan, no se borran) con editor
- Contenido cifrado a nivel de campo (rotación de claves); sin registro en el panel técnico ni en bitácora
- Confidencialidad según la matriz: el Secretario registra pero no lee, el Administrador Técnico nunca
- Retención configurable (30 días) con borrado al consultar y tarea diaria en el despliegue
- Panel reutilizable en la reunión y el grupo, y pantalla global con filtro por origen
- Documentación v3.9 y matriz de trazabilidad

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/trazabilidad/Matriz de Trazabilidad MDF.xlsx
+++ b/docs/trazabilidad/Matriz de Trazabilidad MDF.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Origen v1" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Matriz'!$A$1:$N$97</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Matriz'!$A$1:$N$98</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -897,31 +897,31 @@
         </is>
       </c>
       <c r="B5" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$97,$A5)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$98,$A5)</f>
         <v/>
       </c>
       <c r="C5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$97,$A5,Matriz!$L$2:$L$97,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$98,$A5,Matriz!$L$2:$L$98,"Pendiente")</f>
         <v/>
       </c>
       <c r="D5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$97,$A5,Matriz!$L$2:$L$97,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$98,$A5,Matriz!$L$2:$L$98,"En diseño")</f>
         <v/>
       </c>
       <c r="E5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$97,$A5,Matriz!$L$2:$L$97,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$98,$A5,Matriz!$L$2:$L$98,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$97,$A5,Matriz!$L$2:$L$97,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$98,$A5,Matriz!$L$2:$L$98,"En pruebas")</f>
         <v/>
       </c>
       <c r="G5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$97,$A5,Matriz!$L$2:$L$97,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$98,$A5,Matriz!$L$2:$L$98,"Hecho")</f>
         <v/>
       </c>
       <c r="H5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$97,$A5,Matriz!$L$2:$L$97,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$98,$A5,Matriz!$L$2:$L$98,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I5" s="13">
@@ -936,31 +936,31 @@
         </is>
       </c>
       <c r="B6" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$97,$A6)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$98,$A6)</f>
         <v/>
       </c>
       <c r="C6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$97,$A6,Matriz!$L$2:$L$97,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$98,$A6,Matriz!$L$2:$L$98,"Pendiente")</f>
         <v/>
       </c>
       <c r="D6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$97,$A6,Matriz!$L$2:$L$97,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$98,$A6,Matriz!$L$2:$L$98,"En diseño")</f>
         <v/>
       </c>
       <c r="E6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$97,$A6,Matriz!$L$2:$L$97,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$98,$A6,Matriz!$L$2:$L$98,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$97,$A6,Matriz!$L$2:$L$97,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$98,$A6,Matriz!$L$2:$L$98,"En pruebas")</f>
         <v/>
       </c>
       <c r="G6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$97,$A6,Matriz!$L$2:$L$97,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$98,$A6,Matriz!$L$2:$L$98,"Hecho")</f>
         <v/>
       </c>
       <c r="H6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$97,$A6,Matriz!$L$2:$L$97,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$98,$A6,Matriz!$L$2:$L$98,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I6" s="13">
@@ -975,31 +975,31 @@
         </is>
       </c>
       <c r="B7" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$97,$A7)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$98,$A7)</f>
         <v/>
       </c>
       <c r="C7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$97,$A7,Matriz!$L$2:$L$97,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$98,$A7,Matriz!$L$2:$L$98,"Pendiente")</f>
         <v/>
       </c>
       <c r="D7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$97,$A7,Matriz!$L$2:$L$97,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$98,$A7,Matriz!$L$2:$L$98,"En diseño")</f>
         <v/>
       </c>
       <c r="E7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$97,$A7,Matriz!$L$2:$L$97,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$98,$A7,Matriz!$L$2:$L$98,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$97,$A7,Matriz!$L$2:$L$97,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$98,$A7,Matriz!$L$2:$L$98,"En pruebas")</f>
         <v/>
       </c>
       <c r="G7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$97,$A7,Matriz!$L$2:$L$97,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$98,$A7,Matriz!$L$2:$L$98,"Hecho")</f>
         <v/>
       </c>
       <c r="H7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$97,$A7,Matriz!$L$2:$L$97,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$98,$A7,Matriz!$L$2:$L$98,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I7" s="13">
@@ -1014,31 +1014,31 @@
         </is>
       </c>
       <c r="B8" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$97,$A8)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$98,$A8)</f>
         <v/>
       </c>
       <c r="C8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$97,$A8,Matriz!$L$2:$L$97,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$98,$A8,Matriz!$L$2:$L$98,"Pendiente")</f>
         <v/>
       </c>
       <c r="D8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$97,$A8,Matriz!$L$2:$L$97,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$98,$A8,Matriz!$L$2:$L$98,"En diseño")</f>
         <v/>
       </c>
       <c r="E8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$97,$A8,Matriz!$L$2:$L$97,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$98,$A8,Matriz!$L$2:$L$98,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$97,$A8,Matriz!$L$2:$L$97,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$98,$A8,Matriz!$L$2:$L$98,"En pruebas")</f>
         <v/>
       </c>
       <c r="G8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$97,$A8,Matriz!$L$2:$L$97,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$98,$A8,Matriz!$L$2:$L$98,"Hecho")</f>
         <v/>
       </c>
       <c r="H8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$97,$A8,Matriz!$L$2:$L$97,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$98,$A8,Matriz!$L$2:$L$98,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I8" s="13">
@@ -1053,31 +1053,31 @@
         </is>
       </c>
       <c r="B9" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$97,$A9)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$98,$A9)</f>
         <v/>
       </c>
       <c r="C9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$97,$A9,Matriz!$L$2:$L$97,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$98,$A9,Matriz!$L$2:$L$98,"Pendiente")</f>
         <v/>
       </c>
       <c r="D9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$97,$A9,Matriz!$L$2:$L$97,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$98,$A9,Matriz!$L$2:$L$98,"En diseño")</f>
         <v/>
       </c>
       <c r="E9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$97,$A9,Matriz!$L$2:$L$97,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$98,$A9,Matriz!$L$2:$L$98,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$97,$A9,Matriz!$L$2:$L$97,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$98,$A9,Matriz!$L$2:$L$98,"En pruebas")</f>
         <v/>
       </c>
       <c r="G9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$97,$A9,Matriz!$L$2:$L$97,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$98,$A9,Matriz!$L$2:$L$98,"Hecho")</f>
         <v/>
       </c>
       <c r="H9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$97,$A9,Matriz!$L$2:$L$97,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$98,$A9,Matriz!$L$2:$L$98,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I9" s="13">
@@ -1092,31 +1092,31 @@
         </is>
       </c>
       <c r="B10" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$97,$A10)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$98,$A10)</f>
         <v/>
       </c>
       <c r="C10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$97,$A10,Matriz!$L$2:$L$97,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$98,$A10,Matriz!$L$2:$L$98,"Pendiente")</f>
         <v/>
       </c>
       <c r="D10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$97,$A10,Matriz!$L$2:$L$97,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$98,$A10,Matriz!$L$2:$L$98,"En diseño")</f>
         <v/>
       </c>
       <c r="E10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$97,$A10,Matriz!$L$2:$L$97,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$98,$A10,Matriz!$L$2:$L$98,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$97,$A10,Matriz!$L$2:$L$97,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$98,$A10,Matriz!$L$2:$L$98,"En pruebas")</f>
         <v/>
       </c>
       <c r="G10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$97,$A10,Matriz!$L$2:$L$97,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$98,$A10,Matriz!$L$2:$L$98,"Hecho")</f>
         <v/>
       </c>
       <c r="H10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$97,$A10,Matriz!$L$2:$L$97,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$98,$A10,Matriz!$L$2:$L$98,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I10" s="13">
@@ -1131,31 +1131,31 @@
         </is>
       </c>
       <c r="B11" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$97,$A11)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$98,$A11)</f>
         <v/>
       </c>
       <c r="C11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$97,$A11,Matriz!$L$2:$L$97,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$98,$A11,Matriz!$L$2:$L$98,"Pendiente")</f>
         <v/>
       </c>
       <c r="D11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$97,$A11,Matriz!$L$2:$L$97,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$98,$A11,Matriz!$L$2:$L$98,"En diseño")</f>
         <v/>
       </c>
       <c r="E11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$97,$A11,Matriz!$L$2:$L$97,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$98,$A11,Matriz!$L$2:$L$98,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$97,$A11,Matriz!$L$2:$L$97,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$98,$A11,Matriz!$L$2:$L$98,"En pruebas")</f>
         <v/>
       </c>
       <c r="G11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$97,$A11,Matriz!$L$2:$L$97,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$98,$A11,Matriz!$L$2:$L$98,"Hecho")</f>
         <v/>
       </c>
       <c r="H11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$97,$A11,Matriz!$L$2:$L$97,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$98,$A11,Matriz!$L$2:$L$98,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I11" s="13">
@@ -1256,31 +1256,31 @@
         </is>
       </c>
       <c r="B16" s="12">
-        <f>COUNTIF(Matriz!$H$2:$H$97,$A16)</f>
+        <f>COUNTIF(Matriz!$H$2:$H$98,$A16)</f>
         <v/>
       </c>
       <c r="C16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$97,$A16,Matriz!$L$2:$L$97,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$98,$A16,Matriz!$L$2:$L$98,"Pendiente")</f>
         <v/>
       </c>
       <c r="D16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$97,$A16,Matriz!$L$2:$L$97,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$98,$A16,Matriz!$L$2:$L$98,"En diseño")</f>
         <v/>
       </c>
       <c r="E16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$97,$A16,Matriz!$L$2:$L$97,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$98,$A16,Matriz!$L$2:$L$98,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$97,$A16,Matriz!$L$2:$L$97,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$98,$A16,Matriz!$L$2:$L$98,"En pruebas")</f>
         <v/>
       </c>
       <c r="G16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$97,$A16,Matriz!$L$2:$L$97,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$98,$A16,Matriz!$L$2:$L$98,"Hecho")</f>
         <v/>
       </c>
       <c r="H16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$97,$A16,Matriz!$L$2:$L$97,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$98,$A16,Matriz!$L$2:$L$98,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I16" s="13">
@@ -1295,31 +1295,31 @@
         </is>
       </c>
       <c r="B17" s="12">
-        <f>COUNTIF(Matriz!$H$2:$H$97,$A17)</f>
+        <f>COUNTIF(Matriz!$H$2:$H$98,$A17)</f>
         <v/>
       </c>
       <c r="C17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$97,$A17,Matriz!$L$2:$L$97,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$98,$A17,Matriz!$L$2:$L$98,"Pendiente")</f>
         <v/>
       </c>
       <c r="D17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$97,$A17,Matriz!$L$2:$L$97,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$98,$A17,Matriz!$L$2:$L$98,"En diseño")</f>
         <v/>
       </c>
       <c r="E17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$97,$A17,Matriz!$L$2:$L$97,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$98,$A17,Matriz!$L$2:$L$98,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$97,$A17,Matriz!$L$2:$L$97,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$98,$A17,Matriz!$L$2:$L$98,"En pruebas")</f>
         <v/>
       </c>
       <c r="G17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$97,$A17,Matriz!$L$2:$L$97,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$98,$A17,Matriz!$L$2:$L$98,"Hecho")</f>
         <v/>
       </c>
       <c r="H17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$97,$A17,Matriz!$L$2:$L$97,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$98,$A17,Matriz!$L$2:$L$98,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I17" s="13">
@@ -1334,31 +1334,31 @@
         </is>
       </c>
       <c r="B18" s="12">
-        <f>COUNTIF(Matriz!$H$2:$H$97,$A18)</f>
+        <f>COUNTIF(Matriz!$H$2:$H$98,$A18)</f>
         <v/>
       </c>
       <c r="C18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$97,$A18,Matriz!$L$2:$L$97,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$98,$A18,Matriz!$L$2:$L$98,"Pendiente")</f>
         <v/>
       </c>
       <c r="D18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$97,$A18,Matriz!$L$2:$L$97,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$98,$A18,Matriz!$L$2:$L$98,"En diseño")</f>
         <v/>
       </c>
       <c r="E18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$97,$A18,Matriz!$L$2:$L$97,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$98,$A18,Matriz!$L$2:$L$98,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$97,$A18,Matriz!$L$2:$L$97,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$98,$A18,Matriz!$L$2:$L$98,"En pruebas")</f>
         <v/>
       </c>
       <c r="G18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$97,$A18,Matriz!$L$2:$L$97,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$98,$A18,Matriz!$L$2:$L$98,"Hecho")</f>
         <v/>
       </c>
       <c r="H18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$97,$A18,Matriz!$L$2:$L$97,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$98,$A18,Matriz!$L$2:$L$98,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I18" s="13">
@@ -1373,31 +1373,31 @@
         </is>
       </c>
       <c r="B19" s="12">
-        <f>COUNTIF(Matriz!$H$2:$H$97,$A19)</f>
+        <f>COUNTIF(Matriz!$H$2:$H$98,$A19)</f>
         <v/>
       </c>
       <c r="C19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$97,$A19,Matriz!$L$2:$L$97,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$98,$A19,Matriz!$L$2:$L$98,"Pendiente")</f>
         <v/>
       </c>
       <c r="D19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$97,$A19,Matriz!$L$2:$L$97,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$98,$A19,Matriz!$L$2:$L$98,"En diseño")</f>
         <v/>
       </c>
       <c r="E19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$97,$A19,Matriz!$L$2:$L$97,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$98,$A19,Matriz!$L$2:$L$98,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$97,$A19,Matriz!$L$2:$L$97,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$98,$A19,Matriz!$L$2:$L$98,"En pruebas")</f>
         <v/>
       </c>
       <c r="G19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$97,$A19,Matriz!$L$2:$L$97,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$98,$A19,Matriz!$L$2:$L$98,"Hecho")</f>
         <v/>
       </c>
       <c r="H19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$97,$A19,Matriz!$L$2:$L$97,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$98,$A19,Matriz!$L$2:$L$98,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I19" s="13">
@@ -1498,31 +1498,31 @@
         </is>
       </c>
       <c r="B24" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$97,$A24)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$98,$A24)</f>
         <v/>
       </c>
       <c r="C24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$97,$A24,Matriz!$L$2:$L$97,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$98,$A24,Matriz!$L$2:$L$98,"Pendiente")</f>
         <v/>
       </c>
       <c r="D24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$97,$A24,Matriz!$L$2:$L$97,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$98,$A24,Matriz!$L$2:$L$98,"En diseño")</f>
         <v/>
       </c>
       <c r="E24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$97,$A24,Matriz!$L$2:$L$97,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$98,$A24,Matriz!$L$2:$L$98,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$97,$A24,Matriz!$L$2:$L$97,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$98,$A24,Matriz!$L$2:$L$98,"En pruebas")</f>
         <v/>
       </c>
       <c r="G24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$97,$A24,Matriz!$L$2:$L$97,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$98,$A24,Matriz!$L$2:$L$98,"Hecho")</f>
         <v/>
       </c>
       <c r="H24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$97,$A24,Matriz!$L$2:$L$97,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$98,$A24,Matriz!$L$2:$L$98,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I24" s="13">
@@ -1537,31 +1537,31 @@
         </is>
       </c>
       <c r="B25" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$97,$A25)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$98,$A25)</f>
         <v/>
       </c>
       <c r="C25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$97,$A25,Matriz!$L$2:$L$97,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$98,$A25,Matriz!$L$2:$L$98,"Pendiente")</f>
         <v/>
       </c>
       <c r="D25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$97,$A25,Matriz!$L$2:$L$97,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$98,$A25,Matriz!$L$2:$L$98,"En diseño")</f>
         <v/>
       </c>
       <c r="E25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$97,$A25,Matriz!$L$2:$L$97,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$98,$A25,Matriz!$L$2:$L$98,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$97,$A25,Matriz!$L$2:$L$97,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$98,$A25,Matriz!$L$2:$L$98,"En pruebas")</f>
         <v/>
       </c>
       <c r="G25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$97,$A25,Matriz!$L$2:$L$97,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$98,$A25,Matriz!$L$2:$L$98,"Hecho")</f>
         <v/>
       </c>
       <c r="H25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$97,$A25,Matriz!$L$2:$L$97,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$98,$A25,Matriz!$L$2:$L$98,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I25" s="13">
@@ -1576,31 +1576,31 @@
         </is>
       </c>
       <c r="B26" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$97,$A26)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$98,$A26)</f>
         <v/>
       </c>
       <c r="C26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$97,$A26,Matriz!$L$2:$L$97,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$98,$A26,Matriz!$L$2:$L$98,"Pendiente")</f>
         <v/>
       </c>
       <c r="D26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$97,$A26,Matriz!$L$2:$L$97,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$98,$A26,Matriz!$L$2:$L$98,"En diseño")</f>
         <v/>
       </c>
       <c r="E26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$97,$A26,Matriz!$L$2:$L$97,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$98,$A26,Matriz!$L$2:$L$98,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$97,$A26,Matriz!$L$2:$L$97,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$98,$A26,Matriz!$L$2:$L$98,"En pruebas")</f>
         <v/>
       </c>
       <c r="G26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$97,$A26,Matriz!$L$2:$L$97,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$98,$A26,Matriz!$L$2:$L$98,"Hecho")</f>
         <v/>
       </c>
       <c r="H26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$97,$A26,Matriz!$L$2:$L$97,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$98,$A26,Matriz!$L$2:$L$98,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I26" s="13">
@@ -1615,31 +1615,31 @@
         </is>
       </c>
       <c r="B27" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$97,$A27)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$98,$A27)</f>
         <v/>
       </c>
       <c r="C27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$97,$A27,Matriz!$L$2:$L$97,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$98,$A27,Matriz!$L$2:$L$98,"Pendiente")</f>
         <v/>
       </c>
       <c r="D27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$97,$A27,Matriz!$L$2:$L$97,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$98,$A27,Matriz!$L$2:$L$98,"En diseño")</f>
         <v/>
       </c>
       <c r="E27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$97,$A27,Matriz!$L$2:$L$97,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$98,$A27,Matriz!$L$2:$L$98,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$97,$A27,Matriz!$L$2:$L$97,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$98,$A27,Matriz!$L$2:$L$98,"En pruebas")</f>
         <v/>
       </c>
       <c r="G27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$97,$A27,Matriz!$L$2:$L$97,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$98,$A27,Matriz!$L$2:$L$98,"Hecho")</f>
         <v/>
       </c>
       <c r="H27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$97,$A27,Matriz!$L$2:$L$97,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$98,$A27,Matriz!$L$2:$L$98,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I27" s="13">
@@ -1654,31 +1654,31 @@
         </is>
       </c>
       <c r="B28" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$97,$A28)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$98,$A28)</f>
         <v/>
       </c>
       <c r="C28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$97,$A28,Matriz!$L$2:$L$97,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$98,$A28,Matriz!$L$2:$L$98,"Pendiente")</f>
         <v/>
       </c>
       <c r="D28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$97,$A28,Matriz!$L$2:$L$97,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$98,$A28,Matriz!$L$2:$L$98,"En diseño")</f>
         <v/>
       </c>
       <c r="E28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$97,$A28,Matriz!$L$2:$L$97,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$98,$A28,Matriz!$L$2:$L$98,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$97,$A28,Matriz!$L$2:$L$97,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$98,$A28,Matriz!$L$2:$L$98,"En pruebas")</f>
         <v/>
       </c>
       <c r="G28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$97,$A28,Matriz!$L$2:$L$97,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$98,$A28,Matriz!$L$2:$L$98,"Hecho")</f>
         <v/>
       </c>
       <c r="H28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$97,$A28,Matriz!$L$2:$L$97,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$98,$A28,Matriz!$L$2:$L$98,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I28" s="13">
@@ -1693,31 +1693,31 @@
         </is>
       </c>
       <c r="B29" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$97,$A29)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$98,$A29)</f>
         <v/>
       </c>
       <c r="C29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$97,$A29,Matriz!$L$2:$L$97,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$98,$A29,Matriz!$L$2:$L$98,"Pendiente")</f>
         <v/>
       </c>
       <c r="D29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$97,$A29,Matriz!$L$2:$L$97,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$98,$A29,Matriz!$L$2:$L$98,"En diseño")</f>
         <v/>
       </c>
       <c r="E29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$97,$A29,Matriz!$L$2:$L$97,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$98,$A29,Matriz!$L$2:$L$98,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$97,$A29,Matriz!$L$2:$L$97,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$98,$A29,Matriz!$L$2:$L$98,"En pruebas")</f>
         <v/>
       </c>
       <c r="G29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$97,$A29,Matriz!$L$2:$L$97,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$98,$A29,Matriz!$L$2:$L$98,"Hecho")</f>
         <v/>
       </c>
       <c r="H29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$97,$A29,Matriz!$L$2:$L$97,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$98,$A29,Matriz!$L$2:$L$98,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I29" s="13">
@@ -1732,31 +1732,31 @@
         </is>
       </c>
       <c r="B30" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$97,$A30)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$98,$A30)</f>
         <v/>
       </c>
       <c r="C30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$97,$A30,Matriz!$L$2:$L$97,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$98,$A30,Matriz!$L$2:$L$98,"Pendiente")</f>
         <v/>
       </c>
       <c r="D30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$97,$A30,Matriz!$L$2:$L$97,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$98,$A30,Matriz!$L$2:$L$98,"En diseño")</f>
         <v/>
       </c>
       <c r="E30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$97,$A30,Matriz!$L$2:$L$97,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$98,$A30,Matriz!$L$2:$L$98,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$97,$A30,Matriz!$L$2:$L$97,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$98,$A30,Matriz!$L$2:$L$98,"En pruebas")</f>
         <v/>
       </c>
       <c r="G30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$97,$A30,Matriz!$L$2:$L$97,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$98,$A30,Matriz!$L$2:$L$98,"Hecho")</f>
         <v/>
       </c>
       <c r="H30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$97,$A30,Matriz!$L$2:$L$97,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$98,$A30,Matriz!$L$2:$L$98,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I30" s="13">
@@ -1818,7 +1818,7 @@
         </is>
       </c>
       <c r="B35" s="12">
-        <f>COUNTIF(Matriz!$K$2:$K$97,A35)</f>
+        <f>COUNTIF(Matriz!$K$2:$K$98,A35)</f>
         <v/>
       </c>
     </row>
@@ -1829,7 +1829,7 @@
         </is>
       </c>
       <c r="B36" s="12">
-        <f>COUNTIF(Matriz!$K$2:$K$97,A36)</f>
+        <f>COUNTIF(Matriz!$K$2:$K$98,A36)</f>
         <v/>
       </c>
     </row>
@@ -1840,7 +1840,7 @@
         </is>
       </c>
       <c r="B37" s="12">
-        <f>COUNTIF(Matriz!$K$2:$K$97,A37)</f>
+        <f>COUNTIF(Matriz!$K$2:$K$98,A37)</f>
         <v/>
       </c>
     </row>
@@ -1851,7 +1851,7 @@
         </is>
       </c>
       <c r="B38" s="12">
-        <f>COUNTIF(Matriz!$K$2:$K$97,A38)</f>
+        <f>COUNTIF(Matriz!$K$2:$K$98,A38)</f>
         <v/>
       </c>
     </row>
@@ -1866,7 +1866,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N97"/>
+  <dimension ref="A1:N98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5298,7 +5298,7 @@
       </c>
       <c r="C52" s="19" t="inlineStr">
         <is>
-          <t>Formulario dinámico de peticiones de oración, con seguimiento pastoral.</t>
+          <t>Peticiones de oración con formulario configurable (campos que se agregan, desactivan y reordenan sin programar; cada cambio crea una versión y los campos no se borran). Por defecto: petición, quién la pide y categoría. Las registran el Líder y el Secretario, desde la reunión o desde el grupo; el Pastor también.</t>
         </is>
       </c>
       <c r="D52" s="19" t="inlineStr">
@@ -5343,11 +5343,19 @@
       </c>
       <c r="L52" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M52" s="19" t="inlineStr"/>
-      <c r="N52" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M52" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/m3-peticiones-oracion · 153 pruebas de backend y 30 de frontend pasan; probado contra la base real</t>
+        </is>
+      </c>
+      <c r="N52" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-24 · Formulario configurable y versionado; captura desde la reunión y el grupo.</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="18" t="inlineStr">
@@ -5362,7 +5370,7 @@
       </c>
       <c r="C53" s="19" t="inlineStr">
         <is>
-          <t>Peticiones de oración visibles solo para Líder y roles superiores. Retención de 1 mes o tiempo configurable, con borrado automático.</t>
+          <t>Confidencialidad y retención de las peticiones: solo las ven el Líder de su grupo, el Supervisor de sus grupos, el Pastor y el Anciano (el Secretario las registra pero no las lee; el Administrador Técnico nunca). Se guardan cifradas y se borran automáticamente a los 30 días, configurable. Consultarlas y atenderlas queda en bitácora sin incluir el texto.</t>
         </is>
       </c>
       <c r="D53" s="21" t="inlineStr">
@@ -5407,11 +5415,19 @@
       </c>
       <c r="L53" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M53" s="19" t="inlineStr"/>
-      <c r="N53" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M53" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/m3-peticiones-oracion · 153 pruebas de backend y 30 de frontend pasan; probado contra la base real</t>
+        </is>
+      </c>
+      <c r="N53" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-24 · Cifrado, visibilidad por rol, borrado a los 30 días configurable (tarea diaria en el despliegue).</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="18" t="inlineStr">
@@ -5888,42 +5904,42 @@
     <row r="61">
       <c r="A61" s="18" t="inlineStr">
         <is>
-          <t>M4-01</t>
+          <t>M3-14</t>
         </is>
       </c>
       <c r="B61" s="19" t="inlineStr">
         <is>
-          <t>M4 Kids Check-In/Out</t>
+          <t>M3 Grupos de Conexión</t>
         </is>
       </c>
       <c r="C61" s="19" t="inlineStr">
         <is>
-          <t>Sustitución de la ficha física de papel.</t>
-        </is>
-      </c>
-      <c r="D61" s="19" t="inlineStr">
-        <is>
-          <t>v1 / v2</t>
+          <t>Componente de peticiones reutilizable: cualquier módulo (grupos hoy; cursos o eventos después) se registra como origen y decide quién registra y quién ve. Toda petición guarda su origen de forma inmutable (tipo, identificador y una etiqueta fija, por ejemplo «Grupo de Conexión · Norte · reunión del 22/10/2026») y lo muestra siempre en el listado.</t>
+        </is>
+      </c>
+      <c r="D61" s="21" t="inlineStr">
+        <is>
+          <t>Respuesta</t>
         </is>
       </c>
       <c r="E61" s="19" t="inlineStr">
         <is>
-          <t>Fuera del MVP</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="F61" s="19" t="inlineStr">
         <is>
-          <t>Fase 2</t>
+          <t>Fase 1</t>
         </is>
       </c>
       <c r="G61" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sprint 4</t>
         </is>
       </c>
       <c r="H61" s="19" t="inlineStr">
         <is>
-          <t>Posterior</t>
+          <t>H3 · MVP (Grupos)</t>
         </is>
       </c>
       <c r="I61" s="20" t="inlineStr">
@@ -5943,16 +5959,24 @@
       </c>
       <c r="L61" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M61" s="19" t="inlineStr"/>
-      <c r="N61" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M61" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/m3-peticiones-oracion · 153 pruebas de backend y 30 de frontend pasan; probado contra la base real</t>
+        </is>
+      </c>
+      <c r="N61" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-24 · Origen inmutable y visible; probado con un segundo origen de prueba para verificar la reutilización.</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="18" t="inlineStr">
         <is>
-          <t>M4-02</t>
+          <t>M4-01</t>
         </is>
       </c>
       <c r="B62" s="19" t="inlineStr">
@@ -5962,12 +5986,12 @@
       </c>
       <c r="C62" s="19" t="inlineStr">
         <is>
-          <t>Registro de ingreso del menor con salón o clase asignada y generación de código único.</t>
-        </is>
-      </c>
-      <c r="D62" s="21" t="inlineStr">
-        <is>
-          <t>v1 + Nuevo v3</t>
+          <t>Sustitución de la ficha física de papel.</t>
+        </is>
+      </c>
+      <c r="D62" s="19" t="inlineStr">
+        <is>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E62" s="19" t="inlineStr">
@@ -6016,7 +6040,7 @@
     <row r="63">
       <c r="A63" s="18" t="inlineStr">
         <is>
-          <t>M4-03</t>
+          <t>M4-02</t>
         </is>
       </c>
       <c r="B63" s="19" t="inlineStr">
@@ -6026,12 +6050,12 @@
       </c>
       <c r="C63" s="19" t="inlineStr">
         <is>
-          <t>Código QR dinámico o OTP temporal en la PWA del padre o tutor.</t>
-        </is>
-      </c>
-      <c r="D63" s="19" t="inlineStr">
-        <is>
-          <t>v2</t>
+          <t>Registro de ingreso del menor con salón o clase asignada y generación de código único.</t>
+        </is>
+      </c>
+      <c r="D63" s="21" t="inlineStr">
+        <is>
+          <t>v1 + Nuevo v3</t>
         </is>
       </c>
       <c r="E63" s="19" t="inlineStr">
@@ -6080,7 +6104,7 @@
     <row r="64">
       <c r="A64" s="18" t="inlineStr">
         <is>
-          <t>M4-04</t>
+          <t>M4-03</t>
         </is>
       </c>
       <c r="B64" s="19" t="inlineStr">
@@ -6090,7 +6114,7 @@
       </c>
       <c r="C64" s="19" t="inlineStr">
         <is>
-          <t>Validación al entregar: el servidor de Kids escanea el código y confirma identidad y fotografía del tutor autorizado en el Expediente Digital.</t>
+          <t>Código QR dinámico o OTP temporal en la PWA del padre o tutor.</t>
         </is>
       </c>
       <c r="D64" s="19" t="inlineStr">
@@ -6144,7 +6168,7 @@
     <row r="65">
       <c r="A65" s="18" t="inlineStr">
         <is>
-          <t>M4-05</t>
+          <t>M4-04</t>
         </is>
       </c>
       <c r="B65" s="19" t="inlineStr">
@@ -6154,12 +6178,12 @@
       </c>
       <c r="C65" s="19" t="inlineStr">
         <is>
-          <t>Alternativa para tutores sin smartphone, sin batería o sin conexión (p. ej. código por SMS o comprobante imprimible con identificación). Por definir.</t>
-        </is>
-      </c>
-      <c r="D65" s="21" t="inlineStr">
-        <is>
-          <t>Nuevo v3</t>
+          <t>Validación al entregar: el servidor de Kids escanea el código y confirma identidad y fotografía del tutor autorizado en el Expediente Digital.</t>
+        </is>
+      </c>
+      <c r="D65" s="19" t="inlineStr">
+        <is>
+          <t>v2</t>
         </is>
       </c>
       <c r="E65" s="19" t="inlineStr">
@@ -6194,7 +6218,7 @@
       </c>
       <c r="K65" s="19" t="inlineStr">
         <is>
-          <t>Por definir</t>
+          <t>VoBo pendiente</t>
         </is>
       </c>
       <c r="L65" s="19" t="inlineStr">
@@ -6208,7 +6232,7 @@
     <row r="66">
       <c r="A66" s="18" t="inlineStr">
         <is>
-          <t>M4-06</t>
+          <t>M4-05</t>
         </is>
       </c>
       <c r="B66" s="19" t="inlineStr">
@@ -6218,7 +6242,7 @@
       </c>
       <c r="C66" s="19" t="inlineStr">
         <is>
-          <t>Autorización temporal de un tercero para recoger al menor, con aprobación del tutor registrado.</t>
+          <t>Alternativa para tutores sin smartphone, sin batería o sin conexión (p. ej. código por SMS o comprobante imprimible con identificación). Por definir.</t>
         </is>
       </c>
       <c r="D66" s="21" t="inlineStr">
@@ -6258,7 +6282,7 @@
       </c>
       <c r="K66" s="19" t="inlineStr">
         <is>
-          <t>VoBo pendiente</t>
+          <t>Por definir</t>
         </is>
       </c>
       <c r="L66" s="19" t="inlineStr">
@@ -6272,7 +6296,7 @@
     <row r="67">
       <c r="A67" s="18" t="inlineStr">
         <is>
-          <t>M4-07</t>
+          <t>M4-06</t>
         </is>
       </c>
       <c r="B67" s="19" t="inlineStr">
@@ -6282,7 +6306,7 @@
       </c>
       <c r="C67" s="19" t="inlineStr">
         <is>
-          <t>Caducidad del código y bitácora de cada entrega (quién recogió, quién entregó, hora).</t>
+          <t>Autorización temporal de un tercero para recoger al menor, con aprobación del tutor registrado.</t>
         </is>
       </c>
       <c r="D67" s="21" t="inlineStr">
@@ -6336,7 +6360,7 @@
     <row r="68">
       <c r="A68" s="18" t="inlineStr">
         <is>
-          <t>M4-08</t>
+          <t>M4-07</t>
         </is>
       </c>
       <c r="B68" s="19" t="inlineStr">
@@ -6346,7 +6370,7 @@
       </c>
       <c r="C68" s="19" t="inlineStr">
         <is>
-          <t>Funcionamiento sin conexión o con conexión degradada para el check-out.</t>
+          <t>Caducidad del código y bitácora de cada entrega (quién recogió, quién entregó, hora).</t>
         </is>
       </c>
       <c r="D68" s="21" t="inlineStr">
@@ -6400,52 +6424,52 @@
     <row r="69">
       <c r="A69" s="18" t="inlineStr">
         <is>
-          <t>M5-01</t>
+          <t>M4-08</t>
         </is>
       </c>
       <c r="B69" s="19" t="inlineStr">
         <is>
-          <t>M5 Áreas y servidores</t>
+          <t>M4 Kids Check-In/Out</t>
         </is>
       </c>
       <c r="C69" s="19" t="inlineStr">
         <is>
-          <t>Catálogo mínimo de áreas y asignación de servidores. Versión reducida del módulo 5, necesaria para permisos por área. Sirve como primer censo.</t>
-        </is>
-      </c>
-      <c r="D69" s="19" t="inlineStr">
-        <is>
-          <t>v3</t>
+          <t>Funcionamiento sin conexión o con conexión degradada para el check-out.</t>
+        </is>
+      </c>
+      <c r="D69" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3</t>
         </is>
       </c>
       <c r="E69" s="19" t="inlineStr">
         <is>
-          <t>MVP mínimo</t>
+          <t>Fuera del MVP</t>
         </is>
       </c>
       <c r="F69" s="19" t="inlineStr">
         <is>
-          <t>Fase 0</t>
+          <t>Fase 2</t>
         </is>
       </c>
       <c r="G69" s="19" t="inlineStr">
         <is>
-          <t>Sprint 1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H69" s="19" t="inlineStr">
         <is>
-          <t>H2 · Fase 0 completa</t>
-        </is>
-      </c>
-      <c r="I69" s="19" t="inlineStr">
-        <is>
-          <t>Como pastor quiero un catálogo de áreas con su personal para conocer la estructura.</t>
-        </is>
-      </c>
-      <c r="J69" s="19" t="inlineStr">
-        <is>
-          <t>Crear un área, asignar servidores y ver el conteo real.</t>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="I69" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
+        </is>
+      </c>
+      <c r="J69" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
         </is>
       </c>
       <c r="K69" s="19" t="inlineStr">
@@ -6464,7 +6488,7 @@
     <row r="70">
       <c r="A70" s="18" t="inlineStr">
         <is>
-          <t>M5-02</t>
+          <t>M5-01</t>
         </is>
       </c>
       <c r="B70" s="19" t="inlineStr">
@@ -6474,42 +6498,42 @@
       </c>
       <c r="C70" s="19" t="inlineStr">
         <is>
-          <t>Roles jerárquicos dentro de cada área (directores, líderes, maestros, servidores).</t>
+          <t>Catálogo mínimo de áreas y asignación de servidores. Versión reducida del módulo 5, necesaria para permisos por área. Sirve como primer censo.</t>
         </is>
       </c>
       <c r="D70" s="19" t="inlineStr">
         <is>
-          <t>v1</t>
+          <t>v3</t>
         </is>
       </c>
       <c r="E70" s="19" t="inlineStr">
         <is>
-          <t>Fuera del MVP</t>
+          <t>MVP mínimo</t>
         </is>
       </c>
       <c r="F70" s="19" t="inlineStr">
         <is>
-          <t>Fase 4</t>
+          <t>Fase 0</t>
         </is>
       </c>
       <c r="G70" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sprint 1</t>
         </is>
       </c>
       <c r="H70" s="19" t="inlineStr">
         <is>
-          <t>Posterior</t>
-        </is>
-      </c>
-      <c r="I70" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
-        </is>
-      </c>
-      <c r="J70" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
+          <t>H2 · Fase 0 completa</t>
+        </is>
+      </c>
+      <c r="I70" s="19" t="inlineStr">
+        <is>
+          <t>Como pastor quiero un catálogo de áreas con su personal para conocer la estructura.</t>
+        </is>
+      </c>
+      <c r="J70" s="19" t="inlineStr">
+        <is>
+          <t>Crear un área, asignar servidores y ver el conteo real.</t>
         </is>
       </c>
       <c r="K70" s="19" t="inlineStr">
@@ -6528,7 +6552,7 @@
     <row r="71">
       <c r="A71" s="18" t="inlineStr">
         <is>
-          <t>M5-03</t>
+          <t>M5-02</t>
         </is>
       </c>
       <c r="B71" s="19" t="inlineStr">
@@ -6538,12 +6562,12 @@
       </c>
       <c r="C71" s="19" t="inlineStr">
         <is>
-          <t>Organigrama y número real de servidores activos, directores y líderes por área.</t>
+          <t>Roles jerárquicos dentro de cada área (directores, líderes, maestros, servidores).</t>
         </is>
       </c>
       <c r="D71" s="19" t="inlineStr">
         <is>
-          <t>v2</t>
+          <t>v1</t>
         </is>
       </c>
       <c r="E71" s="19" t="inlineStr">
@@ -6592,7 +6616,7 @@
     <row r="72">
       <c r="A72" s="18" t="inlineStr">
         <is>
-          <t>M5-04</t>
+          <t>M5-03</t>
         </is>
       </c>
       <c r="B72" s="19" t="inlineStr">
@@ -6602,12 +6626,12 @@
       </c>
       <c r="C72" s="19" t="inlineStr">
         <is>
-          <t>Control de asistencia a turnos o servicios.</t>
+          <t>Organigrama y número real de servidores activos, directores y líderes por área.</t>
         </is>
       </c>
       <c r="D72" s="19" t="inlineStr">
         <is>
-          <t>v1 / v2</t>
+          <t>v2</t>
         </is>
       </c>
       <c r="E72" s="19" t="inlineStr">
@@ -6656,7 +6680,7 @@
     <row r="73">
       <c r="A73" s="18" t="inlineStr">
         <is>
-          <t>M5-05</t>
+          <t>M5-04</t>
         </is>
       </c>
       <c r="B73" s="19" t="inlineStr">
@@ -6666,7 +6690,7 @@
       </c>
       <c r="C73" s="19" t="inlineStr">
         <is>
-          <t>Tablero de avisos y notificaciones interno por área.</t>
+          <t>Control de asistencia a turnos o servicios.</t>
         </is>
       </c>
       <c r="D73" s="19" t="inlineStr">
@@ -6720,7 +6744,7 @@
     <row r="74">
       <c r="A74" s="18" t="inlineStr">
         <is>
-          <t>M5-06</t>
+          <t>M5-05</t>
         </is>
       </c>
       <c r="B74" s="19" t="inlineStr">
@@ -6730,7 +6754,7 @@
       </c>
       <c r="C74" s="19" t="inlineStr">
         <is>
-          <t>Gestión financiera por área: caja chica y gastos operativos.</t>
+          <t>Tablero de avisos y notificaciones interno por área.</t>
         </is>
       </c>
       <c r="D74" s="19" t="inlineStr">
@@ -6784,22 +6808,22 @@
     <row r="75">
       <c r="A75" s="18" t="inlineStr">
         <is>
-          <t>M6-01</t>
+          <t>M5-06</t>
         </is>
       </c>
       <c r="B75" s="19" t="inlineStr">
         <is>
-          <t>M6 Ministerios de servicio</t>
+          <t>M5 Áreas y servidores</t>
         </is>
       </c>
       <c r="C75" s="19" t="inlineStr">
         <is>
-          <t>Control de personal propio de cada ministerio.</t>
-        </is>
-      </c>
-      <c r="D75" s="22" t="inlineStr">
-        <is>
-          <t>Recuperado v1</t>
+          <t>Gestión financiera por área: caja chica y gastos operativos.</t>
+        </is>
+      </c>
+      <c r="D75" s="19" t="inlineStr">
+        <is>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E75" s="19" t="inlineStr">
@@ -6848,7 +6872,7 @@
     <row r="76">
       <c r="A76" s="18" t="inlineStr">
         <is>
-          <t>M6-02</t>
+          <t>M6-01</t>
         </is>
       </c>
       <c r="B76" s="19" t="inlineStr">
@@ -6858,12 +6882,12 @@
       </c>
       <c r="C76" s="19" t="inlineStr">
         <is>
-          <t>Menú o catálogo digital interactivo (público o interno), autogestionado.</t>
-        </is>
-      </c>
-      <c r="D76" s="19" t="inlineStr">
-        <is>
-          <t>v1 / v2</t>
+          <t>Control de personal propio de cada ministerio.</t>
+        </is>
+      </c>
+      <c r="D76" s="22" t="inlineStr">
+        <is>
+          <t>Recuperado v1</t>
         </is>
       </c>
       <c r="E76" s="19" t="inlineStr">
@@ -6912,7 +6936,7 @@
     <row r="77">
       <c r="A77" s="18" t="inlineStr">
         <is>
-          <t>M6-03</t>
+          <t>M6-02</t>
         </is>
       </c>
       <c r="B77" s="19" t="inlineStr">
@@ -6922,7 +6946,7 @@
       </c>
       <c r="C77" s="19" t="inlineStr">
         <is>
-          <t>Calendario de turnos: días regulares de servicio y eventos especiales.</t>
+          <t>Menú o catálogo digital interactivo (público o interno), autogestionado.</t>
         </is>
       </c>
       <c r="D77" s="19" t="inlineStr">
@@ -6976,7 +7000,7 @@
     <row r="78">
       <c r="A78" s="18" t="inlineStr">
         <is>
-          <t>M6-04</t>
+          <t>M6-03</t>
         </is>
       </c>
       <c r="B78" s="19" t="inlineStr">
@@ -6986,7 +7010,7 @@
       </c>
       <c r="C78" s="19" t="inlineStr">
         <is>
-          <t>Registro de asistentes o personas atendidas.</t>
+          <t>Calendario de turnos: días regulares de servicio y eventos especiales.</t>
         </is>
       </c>
       <c r="D78" s="19" t="inlineStr">
@@ -7040,7 +7064,7 @@
     <row r="79">
       <c r="A79" s="18" t="inlineStr">
         <is>
-          <t>M6-05</t>
+          <t>M6-04</t>
         </is>
       </c>
       <c r="B79" s="19" t="inlineStr">
@@ -7050,7 +7074,7 @@
       </c>
       <c r="C79" s="19" t="inlineStr">
         <is>
-          <t>Control de gastos y de inventario básico.</t>
+          <t>Registro de asistentes o personas atendidas.</t>
         </is>
       </c>
       <c r="D79" s="19" t="inlineStr">
@@ -7104,7 +7128,7 @@
     <row r="80">
       <c r="A80" s="18" t="inlineStr">
         <is>
-          <t>M6-06</t>
+          <t>M6-05</t>
         </is>
       </c>
       <c r="B80" s="19" t="inlineStr">
@@ -7114,7 +7138,7 @@
       </c>
       <c r="C80" s="19" t="inlineStr">
         <is>
-          <t>Canal de comunicación directo con el área de Administración General.</t>
+          <t>Control de gastos y de inventario básico.</t>
         </is>
       </c>
       <c r="D80" s="19" t="inlineStr">
@@ -7168,7 +7192,7 @@
     <row r="81">
       <c r="A81" s="18" t="inlineStr">
         <is>
-          <t>M6-07</t>
+          <t>M6-06</t>
         </is>
       </c>
       <c r="B81" s="19" t="inlineStr">
@@ -7178,12 +7202,12 @@
       </c>
       <c r="C81" s="19" t="inlineStr">
         <is>
-          <t>Servicio Médico: los datos de salud de las personas atendidas requieren tratamiento de datos sensibles. Por definir alcance.</t>
-        </is>
-      </c>
-      <c r="D81" s="21" t="inlineStr">
-        <is>
-          <t>Nuevo v3</t>
+          <t>Canal de comunicación directo con el área de Administración General.</t>
+        </is>
+      </c>
+      <c r="D81" s="19" t="inlineStr">
+        <is>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E81" s="19" t="inlineStr">
@@ -7218,7 +7242,7 @@
       </c>
       <c r="K81" s="19" t="inlineStr">
         <is>
-          <t>Por definir</t>
+          <t>VoBo pendiente</t>
         </is>
       </c>
       <c r="L81" s="19" t="inlineStr">
@@ -7232,22 +7256,22 @@
     <row r="82">
       <c r="A82" s="18" t="inlineStr">
         <is>
-          <t>M7-01</t>
+          <t>M6-07</t>
         </is>
       </c>
       <c r="B82" s="19" t="inlineStr">
         <is>
-          <t>M7 Eventos y aforo</t>
+          <t>M6 Ministerios de servicio</t>
         </is>
       </c>
       <c r="C82" s="19" t="inlineStr">
         <is>
-          <t>Eventos abiertos o evangelísticos con formulario de inscripción rápida, sin requerir historial previo.</t>
-        </is>
-      </c>
-      <c r="D82" s="19" t="inlineStr">
-        <is>
-          <t>v1 / v2</t>
+          <t>Servicio Médico: los datos de salud de las personas atendidas requieren tratamiento de datos sensibles. Por definir alcance.</t>
+        </is>
+      </c>
+      <c r="D82" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3</t>
         </is>
       </c>
       <c r="E82" s="19" t="inlineStr">
@@ -7282,7 +7306,7 @@
       </c>
       <c r="K82" s="19" t="inlineStr">
         <is>
-          <t>VoBo pendiente</t>
+          <t>Por definir</t>
         </is>
       </c>
       <c r="L82" s="19" t="inlineStr">
@@ -7296,7 +7320,7 @@
     <row r="83">
       <c r="A83" s="18" t="inlineStr">
         <is>
-          <t>M7-02</t>
+          <t>M7-01</t>
         </is>
       </c>
       <c r="B83" s="19" t="inlineStr">
@@ -7306,12 +7330,12 @@
       </c>
       <c r="C83" s="19" t="inlineStr">
         <is>
-          <t>Consolidación (inducción de personas que asisten por primera vez) como tipo de evento.</t>
-        </is>
-      </c>
-      <c r="D83" s="22" t="inlineStr">
-        <is>
-          <t>Recuperado v1</t>
+          <t>Eventos abiertos o evangelísticos con formulario de inscripción rápida, sin requerir historial previo.</t>
+        </is>
+      </c>
+      <c r="D83" s="19" t="inlineStr">
+        <is>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E83" s="19" t="inlineStr">
@@ -7360,7 +7384,7 @@
     <row r="84">
       <c r="A84" s="18" t="inlineStr">
         <is>
-          <t>M7-03</t>
+          <t>M7-02</t>
         </is>
       </c>
       <c r="B84" s="19" t="inlineStr">
@@ -7370,7 +7394,7 @@
       </c>
       <c r="C84" s="19" t="inlineStr">
         <is>
-          <t>Encargados de evento (personal de la iglesia únicamente; no se controla personal externo).</t>
+          <t>Consolidación (inducción de personas que asisten por primera vez) como tipo de evento.</t>
         </is>
       </c>
       <c r="D84" s="22" t="inlineStr">
@@ -7424,7 +7448,7 @@
     <row r="85">
       <c r="A85" s="18" t="inlineStr">
         <is>
-          <t>M7-04</t>
+          <t>M7-03</t>
         </is>
       </c>
       <c r="B85" s="19" t="inlineStr">
@@ -7434,12 +7458,12 @@
       </c>
       <c r="C85" s="19" t="inlineStr">
         <is>
-          <t>Control de cupo en tiempo real que bloquea el sobrecupo en eventos con aforo limitado (ej. 30 o 50 lugares).</t>
-        </is>
-      </c>
-      <c r="D85" s="19" t="inlineStr">
-        <is>
-          <t>v1 / v2</t>
+          <t>Encargados de evento (personal de la iglesia únicamente; no se controla personal externo).</t>
+        </is>
+      </c>
+      <c r="D85" s="22" t="inlineStr">
+        <is>
+          <t>Recuperado v1</t>
         </is>
       </c>
       <c r="E85" s="19" t="inlineStr">
@@ -7488,7 +7512,7 @@
     <row r="86">
       <c r="A86" s="18" t="inlineStr">
         <is>
-          <t>M7-05</t>
+          <t>M7-04</t>
         </is>
       </c>
       <c r="B86" s="19" t="inlineStr">
@@ -7498,12 +7522,12 @@
       </c>
       <c r="C86" s="19" t="inlineStr">
         <is>
-          <t>Control de asistentes sin lista previa, para aforo y para dar a conocer la iglesia.</t>
+          <t>Control de cupo en tiempo real que bloquea el sobrecupo en eventos con aforo limitado (ej. 30 o 50 lugares).</t>
         </is>
       </c>
       <c r="D86" s="19" t="inlineStr">
         <is>
-          <t>v1</t>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E86" s="19" t="inlineStr">
@@ -7552,7 +7576,7 @@
     <row r="87">
       <c r="A87" s="18" t="inlineStr">
         <is>
-          <t>M7-06</t>
+          <t>M7-05</t>
         </is>
       </c>
       <c r="B87" s="19" t="inlineStr">
@@ -7562,12 +7586,12 @@
       </c>
       <c r="C87" s="19" t="inlineStr">
         <is>
-          <t>Seguimiento de personas nuevas: conversión de un invitado a Expediente Digital y canalización a un curso o Grupo de Conexión.</t>
-        </is>
-      </c>
-      <c r="D87" s="21" t="inlineStr">
-        <is>
-          <t>Nuevo v3</t>
+          <t>Control de asistentes sin lista previa, para aforo y para dar a conocer la iglesia.</t>
+        </is>
+      </c>
+      <c r="D87" s="19" t="inlineStr">
+        <is>
+          <t>v1</t>
         </is>
       </c>
       <c r="E87" s="19" t="inlineStr">
@@ -7616,52 +7640,52 @@
     <row r="88">
       <c r="A88" s="18" t="inlineStr">
         <is>
-          <t>NF-01</t>
+          <t>M7-06</t>
         </is>
       </c>
       <c r="B88" s="19" t="inlineStr">
         <is>
-          <t>No funcionales</t>
+          <t>M7 Eventos y aforo</t>
         </is>
       </c>
       <c r="C88" s="19" t="inlineStr">
         <is>
-          <t>Cumplimiento de la LFPDPPP: aviso de privacidad, consentimiento y derechos ARCO.</t>
-        </is>
-      </c>
-      <c r="D88" s="19" t="inlineStr">
-        <is>
-          <t>v3</t>
+          <t>Seguimiento de personas nuevas: conversión de un invitado a Expediente Digital y canalización a un curso o Grupo de Conexión.</t>
+        </is>
+      </c>
+      <c r="D88" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3</t>
         </is>
       </c>
       <c r="E88" s="19" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Fuera del MVP</t>
         </is>
       </c>
       <c r="F88" s="19" t="inlineStr">
         <is>
-          <t>Fase 0</t>
+          <t>Fase 4</t>
         </is>
       </c>
       <c r="G88" s="19" t="inlineStr">
         <is>
-          <t>Sprint 1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H88" s="19" t="inlineStr">
         <is>
-          <t>H1 · 18-oct (núcleo Fase 0)</t>
-        </is>
-      </c>
-      <c r="I88" s="19" t="inlineStr">
-        <is>
-          <t>Como iglesia queremos cumplir con la LFPDPPP.</t>
-        </is>
-      </c>
-      <c r="J88" s="19" t="inlineStr">
-        <is>
-          <t>Aviso de privacidad, consentimiento y atención de derechos ARCO disponibles.</t>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="I88" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
+        </is>
+      </c>
+      <c r="J88" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
         </is>
       </c>
       <c r="K88" s="19" t="inlineStr">
@@ -7680,7 +7704,7 @@
     <row r="89">
       <c r="A89" s="18" t="inlineStr">
         <is>
-          <t>NF-02</t>
+          <t>NF-01</t>
         </is>
       </c>
       <c r="B89" s="19" t="inlineStr">
@@ -7690,7 +7714,7 @@
       </c>
       <c r="C89" s="19" t="inlineStr">
         <is>
-          <t>Cifrado en tránsito y en reposo. Cifrado adicional a nivel de campo para peticiones de oración.</t>
+          <t>Cumplimiento de la LFPDPPP: aviso de privacidad, consentimiento y derechos ARCO.</t>
         </is>
       </c>
       <c r="D89" s="19" t="inlineStr">
@@ -7710,7 +7734,7 @@
       </c>
       <c r="G89" s="19" t="inlineStr">
         <is>
-          <t>Sprint 0</t>
+          <t>Sprint 1</t>
         </is>
       </c>
       <c r="H89" s="19" t="inlineStr">
@@ -7720,12 +7744,12 @@
       </c>
       <c r="I89" s="19" t="inlineStr">
         <is>
-          <t>Como iglesia queremos proteger los datos sensibles.</t>
+          <t>Como iglesia queremos cumplir con la LFPDPPP.</t>
         </is>
       </c>
       <c r="J89" s="19" t="inlineStr">
         <is>
-          <t>HTTPS obligatorio y peticiones de oración ilegibles directamente en la base.</t>
+          <t>Aviso de privacidad, consentimiento y atención de derechos ARCO disponibles.</t>
         </is>
       </c>
       <c r="K89" s="19" t="inlineStr">
@@ -7744,7 +7768,7 @@
     <row r="90">
       <c r="A90" s="18" t="inlineStr">
         <is>
-          <t>NF-03</t>
+          <t>NF-02</t>
         </is>
       </c>
       <c r="B90" s="19" t="inlineStr">
@@ -7754,7 +7778,7 @@
       </c>
       <c r="C90" s="19" t="inlineStr">
         <is>
-          <t>Bitácora de auditoría de solo-añadir: quién consultó o modificó expedientes, ofrendas y asistencias.</t>
+          <t>Cifrado en tránsito y en reposo. Cifrado adicional a nivel de campo para peticiones de oración.</t>
         </is>
       </c>
       <c r="D90" s="19" t="inlineStr">
@@ -7774,7 +7798,7 @@
       </c>
       <c r="G90" s="19" t="inlineStr">
         <is>
-          <t>Sprint 1</t>
+          <t>Sprint 0</t>
         </is>
       </c>
       <c r="H90" s="19" t="inlineStr">
@@ -7784,12 +7808,12 @@
       </c>
       <c r="I90" s="19" t="inlineStr">
         <is>
-          <t>Como pastor quiero una bitácora que nadie pueda alterar.</t>
+          <t>Como iglesia queremos proteger los datos sensibles.</t>
         </is>
       </c>
       <c r="J90" s="19" t="inlineStr">
         <is>
-          <t>El usuario de la aplicación no puede actualizar ni borrar registros de bitácora.</t>
+          <t>HTTPS obligatorio y peticiones de oración ilegibles directamente en la base.</t>
         </is>
       </c>
       <c r="K90" s="19" t="inlineStr">
@@ -7804,19 +7828,19 @@
       </c>
       <c r="M90" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/nf-03-bitacora · 69 pruebas de backend pasan</t>
+          <t>Rama feature/m3-peticiones-oracion · 153 pruebas de backend y 30 de frontend pasan; probado contra la base real</t>
         </is>
       </c>
       <c r="N90" s="19" t="inlineStr">
         <is>
-          <t>2026-10-10 · Bloqueo en aplicación y trigger de PostgreSQL (UPDATE/DELETE/TRUNCATE); pantalla de consulta con permiso bitacora.ver.</t>
+          <t>2026-10-24 · Peticiones cifradas a nivel de campo; falta cifrado en reposo de toda la base (proveedor de nube).</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="18" t="inlineStr">
         <is>
-          <t>NF-04</t>
+          <t>NF-03</t>
         </is>
       </c>
       <c r="B91" s="19" t="inlineStr">
@@ -7826,7 +7850,7 @@
       </c>
       <c r="C91" s="19" t="inlineStr">
         <is>
-          <t>Respaldos automáticos diarios cifrados y prueba periódica de restauración.</t>
+          <t>Bitácora de auditoría de solo-añadir: quién consultó o modificó expedientes, ofrendas y asistencias.</t>
         </is>
       </c>
       <c r="D91" s="19" t="inlineStr">
@@ -7846,7 +7870,7 @@
       </c>
       <c r="G91" s="19" t="inlineStr">
         <is>
-          <t>Sprint 0</t>
+          <t>Sprint 1</t>
         </is>
       </c>
       <c r="H91" s="19" t="inlineStr">
@@ -7856,12 +7880,12 @@
       </c>
       <c r="I91" s="19" t="inlineStr">
         <is>
-          <t>Como iglesia queremos no perder información.</t>
+          <t>Como pastor quiero una bitácora que nadie pueda alterar.</t>
         </is>
       </c>
       <c r="J91" s="19" t="inlineStr">
         <is>
-          <t>Respaldo diario cifrado y restauración probada en un ambiente de pruebas.</t>
+          <t>El usuario de la aplicación no puede actualizar ni borrar registros de bitácora.</t>
         </is>
       </c>
       <c r="K91" s="19" t="inlineStr">
@@ -7871,16 +7895,24 @@
       </c>
       <c r="L91" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M91" s="19" t="inlineStr"/>
-      <c r="N91" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M91" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/nf-03-bitacora · 69 pruebas de backend pasan</t>
+        </is>
+      </c>
+      <c r="N91" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-10 · Bloqueo en aplicación y trigger de PostgreSQL (UPDATE/DELETE/TRUNCATE); pantalla de consulta con permiso bitacora.ver.</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="18" t="inlineStr">
         <is>
-          <t>NF-05</t>
+          <t>NF-04</t>
         </is>
       </c>
       <c r="B92" s="19" t="inlineStr">
@@ -7890,47 +7922,47 @@
       </c>
       <c r="C92" s="19" t="inlineStr">
         <is>
-          <t>Disponibilidad esperada en horarios de servicio (fines de semana y reuniones de grupo). Por definir meta.</t>
-        </is>
-      </c>
-      <c r="D92" s="21" t="inlineStr">
-        <is>
-          <t>Nuevo v3</t>
+          <t>Respaldos automáticos diarios cifrados y prueba periódica de restauración.</t>
+        </is>
+      </c>
+      <c r="D92" s="19" t="inlineStr">
+        <is>
+          <t>v3</t>
         </is>
       </c>
       <c r="E92" s="19" t="inlineStr">
         <is>
-          <t>Fuera del MVP</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="F92" s="19" t="inlineStr">
         <is>
-          <t>Transversal</t>
+          <t>Fase 0</t>
         </is>
       </c>
       <c r="G92" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sprint 0</t>
         </is>
       </c>
       <c r="H92" s="19" t="inlineStr">
         <is>
-          <t>Posterior</t>
-        </is>
-      </c>
-      <c r="I92" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
-        </is>
-      </c>
-      <c r="J92" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
+          <t>H1 · 18-oct (núcleo Fase 0)</t>
+        </is>
+      </c>
+      <c r="I92" s="19" t="inlineStr">
+        <is>
+          <t>Como iglesia queremos no perder información.</t>
+        </is>
+      </c>
+      <c r="J92" s="19" t="inlineStr">
+        <is>
+          <t>Respaldo diario cifrado y restauración probada en un ambiente de pruebas.</t>
         </is>
       </c>
       <c r="K92" s="19" t="inlineStr">
         <is>
-          <t>Por definir</t>
+          <t>VoBo pendiente</t>
         </is>
       </c>
       <c r="L92" s="19" t="inlineStr">
@@ -7944,7 +7976,7 @@
     <row r="93">
       <c r="A93" s="18" t="inlineStr">
         <is>
-          <t>NF-06</t>
+          <t>NF-05</t>
         </is>
       </c>
       <c r="B93" s="19" t="inlineStr">
@@ -7954,69 +7986,61 @@
       </c>
       <c r="C93" s="19" t="inlineStr">
         <is>
-          <t>Pase de lista sin conexión con sincronización posterior (reuniones en domicilios con mala señal).</t>
-        </is>
-      </c>
-      <c r="D93" s="19" t="inlineStr">
-        <is>
-          <t>v3</t>
+          <t>Disponibilidad esperada en horarios de servicio (fines de semana y reuniones de grupo). Por definir meta.</t>
+        </is>
+      </c>
+      <c r="D93" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3</t>
         </is>
       </c>
       <c r="E93" s="19" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Fuera del MVP</t>
         </is>
       </c>
       <c r="F93" s="19" t="inlineStr">
         <is>
-          <t>Fase 0</t>
+          <t>Transversal</t>
         </is>
       </c>
       <c r="G93" s="19" t="inlineStr">
         <is>
-          <t>Sprint 3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H93" s="19" t="inlineStr">
         <is>
-          <t>H3 · MVP (Grupos)</t>
-        </is>
-      </c>
-      <c r="I93" s="19" t="inlineStr">
-        <is>
-          <t>Como secretario quiero que el pase de lista funcione sin señal.</t>
-        </is>
-      </c>
-      <c r="J93" s="19" t="inlineStr">
-        <is>
-          <t>Prueba en modo avión y sincronización al reconectar.</t>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="I93" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
+        </is>
+      </c>
+      <c r="J93" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
         </is>
       </c>
       <c r="K93" s="19" t="inlineStr">
         <is>
-          <t>VoBo pendiente</t>
+          <t>Por definir</t>
         </is>
       </c>
       <c r="L93" s="19" t="inlineStr">
         <is>
-          <t>En pruebas</t>
-        </is>
-      </c>
-      <c r="M93" s="19" t="inlineStr">
-        <is>
-          <t>Rama feature/nf-06-sin-conexion · 117 pruebas de backend y 27 de frontend; probado en Chrome real con service worker</t>
-        </is>
-      </c>
-      <c r="N93" s="19" t="inlineStr">
-        <is>
-          <t>2026-10-24 · Probado de punta a punta en Chrome (sin red → cola → sincronización). Pendiente probar en Android e iOS reales.</t>
-        </is>
-      </c>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M93" s="19" t="inlineStr"/>
+      <c r="N93" s="19" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="18" t="inlineStr">
         <is>
-          <t>NF-07</t>
+          <t>NF-06</t>
         </is>
       </c>
       <c r="B94" s="19" t="inlineStr">
@@ -8026,7 +8050,7 @@
       </c>
       <c r="C94" s="19" t="inlineStr">
         <is>
-          <t>Funciona en Android, iOS y escritorio. En iOS, las notificaciones push requieren instalar la PWA; el respaldo por WhatsApp cubre el resto.</t>
+          <t>Pase de lista sin conexión con sincronización posterior (reuniones en domicilios con mala señal).</t>
         </is>
       </c>
       <c r="D94" s="19" t="inlineStr">
@@ -8046,22 +8070,22 @@
       </c>
       <c r="G94" s="19" t="inlineStr">
         <is>
-          <t>Sprint 0</t>
+          <t>Sprint 3</t>
         </is>
       </c>
       <c r="H94" s="19" t="inlineStr">
         <is>
-          <t>H1 · 18-oct (núcleo Fase 0)</t>
+          <t>H3 · MVP (Grupos)</t>
         </is>
       </c>
       <c r="I94" s="19" t="inlineStr">
         <is>
-          <t>Como usuario quiero usar el sistema en mi dispositivo.</t>
+          <t>Como secretario quiero que el pase de lista funcione sin señal.</t>
         </is>
       </c>
       <c r="J94" s="19" t="inlineStr">
         <is>
-          <t>Pruebas en Android, iOS y escritorio; push en iOS con la PWA instalada y respaldo por WhatsApp.</t>
+          <t>Prueba en modo avión y sincronización al reconectar.</t>
         </is>
       </c>
       <c r="K94" s="19" t="inlineStr">
@@ -8071,16 +8095,24 @@
       </c>
       <c r="L94" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M94" s="19" t="inlineStr"/>
-      <c r="N94" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M94" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/nf-06-sin-conexion · 117 pruebas de backend y 27 de frontend; probado en Chrome real con service worker</t>
+        </is>
+      </c>
+      <c r="N94" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-24 · Probado de punta a punta en Chrome (sin red → cola → sincronización). Pendiente probar en Android e iOS reales.</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="18" t="inlineStr">
         <is>
-          <t>NF-08</t>
+          <t>NF-07</t>
         </is>
       </c>
       <c r="B95" s="19" t="inlineStr">
@@ -8090,12 +8122,12 @@
       </c>
       <c r="C95" s="19" t="inlineStr">
         <is>
-          <t>Dimensionamiento para ~1,000 personas, con picos los fines de semana, y margen de crecimiento.</t>
-        </is>
-      </c>
-      <c r="D95" s="21" t="inlineStr">
-        <is>
-          <t>Resp. P8</t>
+          <t>Funciona en Android, iOS y escritorio. En iOS, las notificaciones push requieren instalar la PWA; el respaldo por WhatsApp cubre el resto.</t>
+        </is>
+      </c>
+      <c r="D95" s="19" t="inlineStr">
+        <is>
+          <t>v3</t>
         </is>
       </c>
       <c r="E95" s="19" t="inlineStr">
@@ -8120,12 +8152,12 @@
       </c>
       <c r="I95" s="19" t="inlineStr">
         <is>
-          <t>Como iglesia queremos que el sistema soporte a ~1,000 personas.</t>
+          <t>Como usuario quiero usar el sistema en mi dispositivo.</t>
         </is>
       </c>
       <c r="J95" s="19" t="inlineStr">
         <is>
-          <t>Prueba de carga con volumen representativo (por definir) sin degradación.</t>
+          <t>Pruebas en Android, iOS y escritorio; push en iOS con la PWA instalada y respaldo por WhatsApp.</t>
         </is>
       </c>
       <c r="K95" s="19" t="inlineStr">
@@ -8144,7 +8176,7 @@
     <row r="96">
       <c r="A96" s="18" t="inlineStr">
         <is>
-          <t>NF-09</t>
+          <t>NF-08</t>
         </is>
       </c>
       <c r="B96" s="19" t="inlineStr">
@@ -8154,42 +8186,42 @@
       </c>
       <c r="C96" s="19" t="inlineStr">
         <is>
-          <t>Reportes transversales: asistencia, finanzas, crecimiento de la iglesia, exportables a Excel y PDF.</t>
+          <t>Dimensionamiento para ~1,000 personas, con picos los fines de semana, y margen de crecimiento.</t>
         </is>
       </c>
       <c r="D96" s="21" t="inlineStr">
         <is>
-          <t>Nuevo v3</t>
+          <t>Resp. P8</t>
         </is>
       </c>
       <c r="E96" s="19" t="inlineStr">
         <is>
-          <t>Fuera del MVP</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="F96" s="19" t="inlineStr">
         <is>
-          <t>Transversal</t>
+          <t>Fase 0</t>
         </is>
       </c>
       <c r="G96" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sprint 0</t>
         </is>
       </c>
       <c r="H96" s="19" t="inlineStr">
         <is>
-          <t>Posterior</t>
-        </is>
-      </c>
-      <c r="I96" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
-        </is>
-      </c>
-      <c r="J96" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
+          <t>H1 · 18-oct (núcleo Fase 0)</t>
+        </is>
+      </c>
+      <c r="I96" s="19" t="inlineStr">
+        <is>
+          <t>Como iglesia queremos que el sistema soporte a ~1,000 personas.</t>
+        </is>
+      </c>
+      <c r="J96" s="19" t="inlineStr">
+        <is>
+          <t>Prueba de carga con volumen representativo (por definir) sin degradación.</t>
         </is>
       </c>
       <c r="K96" s="19" t="inlineStr">
@@ -8208,7 +8240,7 @@
     <row r="97">
       <c r="A97" s="18" t="inlineStr">
         <is>
-          <t>NF-10</t>
+          <t>NF-09</t>
         </is>
       </c>
       <c r="B97" s="19" t="inlineStr">
@@ -8218,42 +8250,42 @@
       </c>
       <c r="C97" s="19" t="inlineStr">
         <is>
-          <t>Usabilidad para personas mayores: tipografía grande, alto contraste, flujos cortos (ver sección 5).</t>
-        </is>
-      </c>
-      <c r="D97" s="19" t="inlineStr">
-        <is>
-          <t>v3 + Obs. 1</t>
+          <t>Reportes transversales: asistencia, finanzas, crecimiento de la iglesia, exportables a Excel y PDF.</t>
+        </is>
+      </c>
+      <c r="D97" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3</t>
         </is>
       </c>
       <c r="E97" s="19" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Fuera del MVP</t>
         </is>
       </c>
       <c r="F97" s="19" t="inlineStr">
         <is>
-          <t>Fase 0</t>
+          <t>Transversal</t>
         </is>
       </c>
       <c r="G97" s="19" t="inlineStr">
         <is>
-          <t>Sprint 0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H97" s="19" t="inlineStr">
         <is>
-          <t>H1 · 18-oct (núcleo Fase 0)</t>
-        </is>
-      </c>
-      <c r="I97" s="19" t="inlineStr">
-        <is>
-          <t>Como persona mayor quiero una interfaz fácil de leer y usar.</t>
-        </is>
-      </c>
-      <c r="J97" s="19" t="inlineStr">
-        <is>
-          <t>Texto base 18 px, botones de al menos 48 px, contraste AA; prueba con usuarios mayores.</t>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="I97" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
+        </is>
+      </c>
+      <c r="J97" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
         </is>
       </c>
       <c r="K97" s="19" t="inlineStr">
@@ -8269,9 +8301,73 @@
       <c r="M97" s="19" t="inlineStr"/>
       <c r="N97" s="19" t="inlineStr"/>
     </row>
+    <row r="98">
+      <c r="A98" s="18" t="inlineStr">
+        <is>
+          <t>NF-10</t>
+        </is>
+      </c>
+      <c r="B98" s="19" t="inlineStr">
+        <is>
+          <t>No funcionales</t>
+        </is>
+      </c>
+      <c r="C98" s="19" t="inlineStr">
+        <is>
+          <t>Usabilidad para personas mayores: tipografía grande, alto contraste, flujos cortos (ver sección 5).</t>
+        </is>
+      </c>
+      <c r="D98" s="19" t="inlineStr">
+        <is>
+          <t>v3 + Obs. 1</t>
+        </is>
+      </c>
+      <c r="E98" s="19" t="inlineStr">
+        <is>
+          <t>MVP</t>
+        </is>
+      </c>
+      <c r="F98" s="19" t="inlineStr">
+        <is>
+          <t>Fase 0</t>
+        </is>
+      </c>
+      <c r="G98" s="19" t="inlineStr">
+        <is>
+          <t>Sprint 0</t>
+        </is>
+      </c>
+      <c r="H98" s="19" t="inlineStr">
+        <is>
+          <t>H1 · 18-oct (núcleo Fase 0)</t>
+        </is>
+      </c>
+      <c r="I98" s="19" t="inlineStr">
+        <is>
+          <t>Como persona mayor quiero una interfaz fácil de leer y usar.</t>
+        </is>
+      </c>
+      <c r="J98" s="19" t="inlineStr">
+        <is>
+          <t>Texto base 18 px, botones de al menos 48 px, contraste AA; prueba con usuarios mayores.</t>
+        </is>
+      </c>
+      <c r="K98" s="19" t="inlineStr">
+        <is>
+          <t>VoBo pendiente</t>
+        </is>
+      </c>
+      <c r="L98" s="19" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M98" s="19" t="inlineStr"/>
+      <c r="N98" s="19" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N97"/>
-  <conditionalFormatting sqref="L2:L97">
+  <autoFilter ref="A1:N98"/>
+  <conditionalFormatting sqref="L2:L98">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$L2="Hecho"</formula>
     </cfRule>
@@ -8288,7 +8384,7 @@
       <formula>$L2="Bloqueado"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K2:K97">
+  <conditionalFormatting sqref="K2:K98">
     <cfRule type="expression" priority="6" dxfId="0">
       <formula>$K2="Aprobado"</formula>
     </cfRule>
@@ -8296,16 +8392,16 @@
       <formula>$K2="Por definir"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H2:H97">
+  <conditionalFormatting sqref="H2:H98">
     <cfRule type="expression" priority="8" dxfId="5">
       <formula>LEFT($H2,2)="H1"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="L2:L97" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="L2:L98" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Pendiente,En diseño,En desarrollo,En pruebas,Hecho,Bloqueado"</formula1>
     </dataValidation>
-    <dataValidation sqref="K2:K97" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="K2:K98" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"VoBo pendiente,Aprobado,Por definir,Rechazado"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Peticiones de oración: alcance de lectura, equipo de oración y nombre oculto
- Cada petición tiene un alcance elegido al registrar: solo líderes, mi grupo o equipo de oración;
  el valor por defecto es configurable (nuevo parámetro de tipo opción en Configuración)
- Rol «Equipo de oración» con su propio permiso, asignable desde Roles: ve las del alcance equipo
  de cualquier origen y nada más
- Quien pertenece al grupo ve las de alcance grupo y equipo; solo líderes y superiores las atienden
- Opción de ocultar el nombre: los campos marcados «identifica a la persona» solo los ven líderes y
  quien la registró
- El registro de orígenes pasa a niveles de acceso (líder y miembro) en lugar de lista de visibles
- Cambia la regla de la matriz de confidencialidad aprobada para peticiones (documentado en v3.10)
- Pantallas: selector de alcance, etiqueta de alcance en cada petición y campo identifica en el editor

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/trazabilidad/Matriz de Trazabilidad MDF.xlsx
+++ b/docs/trazabilidad/Matriz de Trazabilidad MDF.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Origen v1" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Matriz'!$A$1:$N$98</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Matriz'!$A$1:$N$99</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -897,31 +897,31 @@
         </is>
       </c>
       <c r="B5" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$98,$A5)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$99,$A5)</f>
         <v/>
       </c>
       <c r="C5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$98,$A5,Matriz!$L$2:$L$98,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$99,$A5,Matriz!$L$2:$L$99,"Pendiente")</f>
         <v/>
       </c>
       <c r="D5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$98,$A5,Matriz!$L$2:$L$98,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$99,$A5,Matriz!$L$2:$L$99,"En diseño")</f>
         <v/>
       </c>
       <c r="E5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$98,$A5,Matriz!$L$2:$L$98,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$99,$A5,Matriz!$L$2:$L$99,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$98,$A5,Matriz!$L$2:$L$98,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$99,$A5,Matriz!$L$2:$L$99,"En pruebas")</f>
         <v/>
       </c>
       <c r="G5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$98,$A5,Matriz!$L$2:$L$98,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$99,$A5,Matriz!$L$2:$L$99,"Hecho")</f>
         <v/>
       </c>
       <c r="H5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$98,$A5,Matriz!$L$2:$L$98,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$99,$A5,Matriz!$L$2:$L$99,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I5" s="13">
@@ -936,31 +936,31 @@
         </is>
       </c>
       <c r="B6" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$98,$A6)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$99,$A6)</f>
         <v/>
       </c>
       <c r="C6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$98,$A6,Matriz!$L$2:$L$98,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$99,$A6,Matriz!$L$2:$L$99,"Pendiente")</f>
         <v/>
       </c>
       <c r="D6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$98,$A6,Matriz!$L$2:$L$98,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$99,$A6,Matriz!$L$2:$L$99,"En diseño")</f>
         <v/>
       </c>
       <c r="E6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$98,$A6,Matriz!$L$2:$L$98,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$99,$A6,Matriz!$L$2:$L$99,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$98,$A6,Matriz!$L$2:$L$98,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$99,$A6,Matriz!$L$2:$L$99,"En pruebas")</f>
         <v/>
       </c>
       <c r="G6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$98,$A6,Matriz!$L$2:$L$98,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$99,$A6,Matriz!$L$2:$L$99,"Hecho")</f>
         <v/>
       </c>
       <c r="H6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$98,$A6,Matriz!$L$2:$L$98,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$99,$A6,Matriz!$L$2:$L$99,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I6" s="13">
@@ -975,31 +975,31 @@
         </is>
       </c>
       <c r="B7" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$98,$A7)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$99,$A7)</f>
         <v/>
       </c>
       <c r="C7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$98,$A7,Matriz!$L$2:$L$98,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$99,$A7,Matriz!$L$2:$L$99,"Pendiente")</f>
         <v/>
       </c>
       <c r="D7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$98,$A7,Matriz!$L$2:$L$98,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$99,$A7,Matriz!$L$2:$L$99,"En diseño")</f>
         <v/>
       </c>
       <c r="E7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$98,$A7,Matriz!$L$2:$L$98,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$99,$A7,Matriz!$L$2:$L$99,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$98,$A7,Matriz!$L$2:$L$98,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$99,$A7,Matriz!$L$2:$L$99,"En pruebas")</f>
         <v/>
       </c>
       <c r="G7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$98,$A7,Matriz!$L$2:$L$98,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$99,$A7,Matriz!$L$2:$L$99,"Hecho")</f>
         <v/>
       </c>
       <c r="H7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$98,$A7,Matriz!$L$2:$L$98,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$99,$A7,Matriz!$L$2:$L$99,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I7" s="13">
@@ -1014,31 +1014,31 @@
         </is>
       </c>
       <c r="B8" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$98,$A8)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$99,$A8)</f>
         <v/>
       </c>
       <c r="C8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$98,$A8,Matriz!$L$2:$L$98,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$99,$A8,Matriz!$L$2:$L$99,"Pendiente")</f>
         <v/>
       </c>
       <c r="D8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$98,$A8,Matriz!$L$2:$L$98,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$99,$A8,Matriz!$L$2:$L$99,"En diseño")</f>
         <v/>
       </c>
       <c r="E8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$98,$A8,Matriz!$L$2:$L$98,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$99,$A8,Matriz!$L$2:$L$99,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$98,$A8,Matriz!$L$2:$L$98,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$99,$A8,Matriz!$L$2:$L$99,"En pruebas")</f>
         <v/>
       </c>
       <c r="G8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$98,$A8,Matriz!$L$2:$L$98,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$99,$A8,Matriz!$L$2:$L$99,"Hecho")</f>
         <v/>
       </c>
       <c r="H8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$98,$A8,Matriz!$L$2:$L$98,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$99,$A8,Matriz!$L$2:$L$99,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I8" s="13">
@@ -1053,31 +1053,31 @@
         </is>
       </c>
       <c r="B9" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$98,$A9)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$99,$A9)</f>
         <v/>
       </c>
       <c r="C9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$98,$A9,Matriz!$L$2:$L$98,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$99,$A9,Matriz!$L$2:$L$99,"Pendiente")</f>
         <v/>
       </c>
       <c r="D9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$98,$A9,Matriz!$L$2:$L$98,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$99,$A9,Matriz!$L$2:$L$99,"En diseño")</f>
         <v/>
       </c>
       <c r="E9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$98,$A9,Matriz!$L$2:$L$98,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$99,$A9,Matriz!$L$2:$L$99,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$98,$A9,Matriz!$L$2:$L$98,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$99,$A9,Matriz!$L$2:$L$99,"En pruebas")</f>
         <v/>
       </c>
       <c r="G9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$98,$A9,Matriz!$L$2:$L$98,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$99,$A9,Matriz!$L$2:$L$99,"Hecho")</f>
         <v/>
       </c>
       <c r="H9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$98,$A9,Matriz!$L$2:$L$98,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$99,$A9,Matriz!$L$2:$L$99,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I9" s="13">
@@ -1092,31 +1092,31 @@
         </is>
       </c>
       <c r="B10" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$98,$A10)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$99,$A10)</f>
         <v/>
       </c>
       <c r="C10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$98,$A10,Matriz!$L$2:$L$98,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$99,$A10,Matriz!$L$2:$L$99,"Pendiente")</f>
         <v/>
       </c>
       <c r="D10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$98,$A10,Matriz!$L$2:$L$98,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$99,$A10,Matriz!$L$2:$L$99,"En diseño")</f>
         <v/>
       </c>
       <c r="E10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$98,$A10,Matriz!$L$2:$L$98,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$99,$A10,Matriz!$L$2:$L$99,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$98,$A10,Matriz!$L$2:$L$98,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$99,$A10,Matriz!$L$2:$L$99,"En pruebas")</f>
         <v/>
       </c>
       <c r="G10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$98,$A10,Matriz!$L$2:$L$98,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$99,$A10,Matriz!$L$2:$L$99,"Hecho")</f>
         <v/>
       </c>
       <c r="H10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$98,$A10,Matriz!$L$2:$L$98,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$99,$A10,Matriz!$L$2:$L$99,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I10" s="13">
@@ -1131,31 +1131,31 @@
         </is>
       </c>
       <c r="B11" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$98,$A11)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$99,$A11)</f>
         <v/>
       </c>
       <c r="C11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$98,$A11,Matriz!$L$2:$L$98,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$99,$A11,Matriz!$L$2:$L$99,"Pendiente")</f>
         <v/>
       </c>
       <c r="D11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$98,$A11,Matriz!$L$2:$L$98,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$99,$A11,Matriz!$L$2:$L$99,"En diseño")</f>
         <v/>
       </c>
       <c r="E11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$98,$A11,Matriz!$L$2:$L$98,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$99,$A11,Matriz!$L$2:$L$99,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$98,$A11,Matriz!$L$2:$L$98,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$99,$A11,Matriz!$L$2:$L$99,"En pruebas")</f>
         <v/>
       </c>
       <c r="G11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$98,$A11,Matriz!$L$2:$L$98,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$99,$A11,Matriz!$L$2:$L$99,"Hecho")</f>
         <v/>
       </c>
       <c r="H11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$98,$A11,Matriz!$L$2:$L$98,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$99,$A11,Matriz!$L$2:$L$99,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I11" s="13">
@@ -1256,31 +1256,31 @@
         </is>
       </c>
       <c r="B16" s="12">
-        <f>COUNTIF(Matriz!$H$2:$H$98,$A16)</f>
+        <f>COUNTIF(Matriz!$H$2:$H$99,$A16)</f>
         <v/>
       </c>
       <c r="C16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$98,$A16,Matriz!$L$2:$L$98,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$99,$A16,Matriz!$L$2:$L$99,"Pendiente")</f>
         <v/>
       </c>
       <c r="D16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$98,$A16,Matriz!$L$2:$L$98,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$99,$A16,Matriz!$L$2:$L$99,"En diseño")</f>
         <v/>
       </c>
       <c r="E16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$98,$A16,Matriz!$L$2:$L$98,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$99,$A16,Matriz!$L$2:$L$99,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$98,$A16,Matriz!$L$2:$L$98,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$99,$A16,Matriz!$L$2:$L$99,"En pruebas")</f>
         <v/>
       </c>
       <c r="G16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$98,$A16,Matriz!$L$2:$L$98,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$99,$A16,Matriz!$L$2:$L$99,"Hecho")</f>
         <v/>
       </c>
       <c r="H16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$98,$A16,Matriz!$L$2:$L$98,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$99,$A16,Matriz!$L$2:$L$99,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I16" s="13">
@@ -1295,31 +1295,31 @@
         </is>
       </c>
       <c r="B17" s="12">
-        <f>COUNTIF(Matriz!$H$2:$H$98,$A17)</f>
+        <f>COUNTIF(Matriz!$H$2:$H$99,$A17)</f>
         <v/>
       </c>
       <c r="C17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$98,$A17,Matriz!$L$2:$L$98,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$99,$A17,Matriz!$L$2:$L$99,"Pendiente")</f>
         <v/>
       </c>
       <c r="D17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$98,$A17,Matriz!$L$2:$L$98,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$99,$A17,Matriz!$L$2:$L$99,"En diseño")</f>
         <v/>
       </c>
       <c r="E17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$98,$A17,Matriz!$L$2:$L$98,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$99,$A17,Matriz!$L$2:$L$99,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$98,$A17,Matriz!$L$2:$L$98,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$99,$A17,Matriz!$L$2:$L$99,"En pruebas")</f>
         <v/>
       </c>
       <c r="G17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$98,$A17,Matriz!$L$2:$L$98,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$99,$A17,Matriz!$L$2:$L$99,"Hecho")</f>
         <v/>
       </c>
       <c r="H17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$98,$A17,Matriz!$L$2:$L$98,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$99,$A17,Matriz!$L$2:$L$99,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I17" s="13">
@@ -1334,31 +1334,31 @@
         </is>
       </c>
       <c r="B18" s="12">
-        <f>COUNTIF(Matriz!$H$2:$H$98,$A18)</f>
+        <f>COUNTIF(Matriz!$H$2:$H$99,$A18)</f>
         <v/>
       </c>
       <c r="C18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$98,$A18,Matriz!$L$2:$L$98,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$99,$A18,Matriz!$L$2:$L$99,"Pendiente")</f>
         <v/>
       </c>
       <c r="D18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$98,$A18,Matriz!$L$2:$L$98,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$99,$A18,Matriz!$L$2:$L$99,"En diseño")</f>
         <v/>
       </c>
       <c r="E18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$98,$A18,Matriz!$L$2:$L$98,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$99,$A18,Matriz!$L$2:$L$99,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$98,$A18,Matriz!$L$2:$L$98,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$99,$A18,Matriz!$L$2:$L$99,"En pruebas")</f>
         <v/>
       </c>
       <c r="G18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$98,$A18,Matriz!$L$2:$L$98,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$99,$A18,Matriz!$L$2:$L$99,"Hecho")</f>
         <v/>
       </c>
       <c r="H18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$98,$A18,Matriz!$L$2:$L$98,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$99,$A18,Matriz!$L$2:$L$99,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I18" s="13">
@@ -1373,31 +1373,31 @@
         </is>
       </c>
       <c r="B19" s="12">
-        <f>COUNTIF(Matriz!$H$2:$H$98,$A19)</f>
+        <f>COUNTIF(Matriz!$H$2:$H$99,$A19)</f>
         <v/>
       </c>
       <c r="C19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$98,$A19,Matriz!$L$2:$L$98,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$99,$A19,Matriz!$L$2:$L$99,"Pendiente")</f>
         <v/>
       </c>
       <c r="D19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$98,$A19,Matriz!$L$2:$L$98,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$99,$A19,Matriz!$L$2:$L$99,"En diseño")</f>
         <v/>
       </c>
       <c r="E19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$98,$A19,Matriz!$L$2:$L$98,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$99,$A19,Matriz!$L$2:$L$99,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$98,$A19,Matriz!$L$2:$L$98,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$99,$A19,Matriz!$L$2:$L$99,"En pruebas")</f>
         <v/>
       </c>
       <c r="G19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$98,$A19,Matriz!$L$2:$L$98,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$99,$A19,Matriz!$L$2:$L$99,"Hecho")</f>
         <v/>
       </c>
       <c r="H19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$98,$A19,Matriz!$L$2:$L$98,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$99,$A19,Matriz!$L$2:$L$99,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I19" s="13">
@@ -1498,31 +1498,31 @@
         </is>
       </c>
       <c r="B24" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$98,$A24)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$99,$A24)</f>
         <v/>
       </c>
       <c r="C24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$98,$A24,Matriz!$L$2:$L$98,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$99,$A24,Matriz!$L$2:$L$99,"Pendiente")</f>
         <v/>
       </c>
       <c r="D24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$98,$A24,Matriz!$L$2:$L$98,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$99,$A24,Matriz!$L$2:$L$99,"En diseño")</f>
         <v/>
       </c>
       <c r="E24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$98,$A24,Matriz!$L$2:$L$98,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$99,$A24,Matriz!$L$2:$L$99,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$98,$A24,Matriz!$L$2:$L$98,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$99,$A24,Matriz!$L$2:$L$99,"En pruebas")</f>
         <v/>
       </c>
       <c r="G24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$98,$A24,Matriz!$L$2:$L$98,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$99,$A24,Matriz!$L$2:$L$99,"Hecho")</f>
         <v/>
       </c>
       <c r="H24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$98,$A24,Matriz!$L$2:$L$98,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$99,$A24,Matriz!$L$2:$L$99,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I24" s="13">
@@ -1537,31 +1537,31 @@
         </is>
       </c>
       <c r="B25" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$98,$A25)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$99,$A25)</f>
         <v/>
       </c>
       <c r="C25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$98,$A25,Matriz!$L$2:$L$98,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$99,$A25,Matriz!$L$2:$L$99,"Pendiente")</f>
         <v/>
       </c>
       <c r="D25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$98,$A25,Matriz!$L$2:$L$98,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$99,$A25,Matriz!$L$2:$L$99,"En diseño")</f>
         <v/>
       </c>
       <c r="E25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$98,$A25,Matriz!$L$2:$L$98,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$99,$A25,Matriz!$L$2:$L$99,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$98,$A25,Matriz!$L$2:$L$98,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$99,$A25,Matriz!$L$2:$L$99,"En pruebas")</f>
         <v/>
       </c>
       <c r="G25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$98,$A25,Matriz!$L$2:$L$98,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$99,$A25,Matriz!$L$2:$L$99,"Hecho")</f>
         <v/>
       </c>
       <c r="H25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$98,$A25,Matriz!$L$2:$L$98,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$99,$A25,Matriz!$L$2:$L$99,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I25" s="13">
@@ -1576,31 +1576,31 @@
         </is>
       </c>
       <c r="B26" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$98,$A26)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$99,$A26)</f>
         <v/>
       </c>
       <c r="C26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$98,$A26,Matriz!$L$2:$L$98,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$99,$A26,Matriz!$L$2:$L$99,"Pendiente")</f>
         <v/>
       </c>
       <c r="D26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$98,$A26,Matriz!$L$2:$L$98,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$99,$A26,Matriz!$L$2:$L$99,"En diseño")</f>
         <v/>
       </c>
       <c r="E26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$98,$A26,Matriz!$L$2:$L$98,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$99,$A26,Matriz!$L$2:$L$99,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$98,$A26,Matriz!$L$2:$L$98,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$99,$A26,Matriz!$L$2:$L$99,"En pruebas")</f>
         <v/>
       </c>
       <c r="G26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$98,$A26,Matriz!$L$2:$L$98,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$99,$A26,Matriz!$L$2:$L$99,"Hecho")</f>
         <v/>
       </c>
       <c r="H26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$98,$A26,Matriz!$L$2:$L$98,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$99,$A26,Matriz!$L$2:$L$99,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I26" s="13">
@@ -1615,31 +1615,31 @@
         </is>
       </c>
       <c r="B27" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$98,$A27)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$99,$A27)</f>
         <v/>
       </c>
       <c r="C27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$98,$A27,Matriz!$L$2:$L$98,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$99,$A27,Matriz!$L$2:$L$99,"Pendiente")</f>
         <v/>
       </c>
       <c r="D27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$98,$A27,Matriz!$L$2:$L$98,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$99,$A27,Matriz!$L$2:$L$99,"En diseño")</f>
         <v/>
       </c>
       <c r="E27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$98,$A27,Matriz!$L$2:$L$98,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$99,$A27,Matriz!$L$2:$L$99,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$98,$A27,Matriz!$L$2:$L$98,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$99,$A27,Matriz!$L$2:$L$99,"En pruebas")</f>
         <v/>
       </c>
       <c r="G27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$98,$A27,Matriz!$L$2:$L$98,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$99,$A27,Matriz!$L$2:$L$99,"Hecho")</f>
         <v/>
       </c>
       <c r="H27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$98,$A27,Matriz!$L$2:$L$98,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$99,$A27,Matriz!$L$2:$L$99,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I27" s="13">
@@ -1654,31 +1654,31 @@
         </is>
       </c>
       <c r="B28" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$98,$A28)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$99,$A28)</f>
         <v/>
       </c>
       <c r="C28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$98,$A28,Matriz!$L$2:$L$98,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$99,$A28,Matriz!$L$2:$L$99,"Pendiente")</f>
         <v/>
       </c>
       <c r="D28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$98,$A28,Matriz!$L$2:$L$98,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$99,$A28,Matriz!$L$2:$L$99,"En diseño")</f>
         <v/>
       </c>
       <c r="E28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$98,$A28,Matriz!$L$2:$L$98,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$99,$A28,Matriz!$L$2:$L$99,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$98,$A28,Matriz!$L$2:$L$98,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$99,$A28,Matriz!$L$2:$L$99,"En pruebas")</f>
         <v/>
       </c>
       <c r="G28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$98,$A28,Matriz!$L$2:$L$98,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$99,$A28,Matriz!$L$2:$L$99,"Hecho")</f>
         <v/>
       </c>
       <c r="H28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$98,$A28,Matriz!$L$2:$L$98,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$99,$A28,Matriz!$L$2:$L$99,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I28" s="13">
@@ -1693,31 +1693,31 @@
         </is>
       </c>
       <c r="B29" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$98,$A29)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$99,$A29)</f>
         <v/>
       </c>
       <c r="C29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$98,$A29,Matriz!$L$2:$L$98,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$99,$A29,Matriz!$L$2:$L$99,"Pendiente")</f>
         <v/>
       </c>
       <c r="D29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$98,$A29,Matriz!$L$2:$L$98,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$99,$A29,Matriz!$L$2:$L$99,"En diseño")</f>
         <v/>
       </c>
       <c r="E29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$98,$A29,Matriz!$L$2:$L$98,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$99,$A29,Matriz!$L$2:$L$99,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$98,$A29,Matriz!$L$2:$L$98,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$99,$A29,Matriz!$L$2:$L$99,"En pruebas")</f>
         <v/>
       </c>
       <c r="G29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$98,$A29,Matriz!$L$2:$L$98,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$99,$A29,Matriz!$L$2:$L$99,"Hecho")</f>
         <v/>
       </c>
       <c r="H29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$98,$A29,Matriz!$L$2:$L$98,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$99,$A29,Matriz!$L$2:$L$99,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I29" s="13">
@@ -1732,31 +1732,31 @@
         </is>
       </c>
       <c r="B30" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$98,$A30)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$99,$A30)</f>
         <v/>
       </c>
       <c r="C30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$98,$A30,Matriz!$L$2:$L$98,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$99,$A30,Matriz!$L$2:$L$99,"Pendiente")</f>
         <v/>
       </c>
       <c r="D30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$98,$A30,Matriz!$L$2:$L$98,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$99,$A30,Matriz!$L$2:$L$99,"En diseño")</f>
         <v/>
       </c>
       <c r="E30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$98,$A30,Matriz!$L$2:$L$98,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$99,$A30,Matriz!$L$2:$L$99,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$98,$A30,Matriz!$L$2:$L$98,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$99,$A30,Matriz!$L$2:$L$99,"En pruebas")</f>
         <v/>
       </c>
       <c r="G30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$98,$A30,Matriz!$L$2:$L$98,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$99,$A30,Matriz!$L$2:$L$99,"Hecho")</f>
         <v/>
       </c>
       <c r="H30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$98,$A30,Matriz!$L$2:$L$98,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$99,$A30,Matriz!$L$2:$L$99,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I30" s="13">
@@ -1818,7 +1818,7 @@
         </is>
       </c>
       <c r="B35" s="12">
-        <f>COUNTIF(Matriz!$K$2:$K$98,A35)</f>
+        <f>COUNTIF(Matriz!$K$2:$K$99,A35)</f>
         <v/>
       </c>
     </row>
@@ -1829,7 +1829,7 @@
         </is>
       </c>
       <c r="B36" s="12">
-        <f>COUNTIF(Matriz!$K$2:$K$98,A36)</f>
+        <f>COUNTIF(Matriz!$K$2:$K$99,A36)</f>
         <v/>
       </c>
     </row>
@@ -1840,7 +1840,7 @@
         </is>
       </c>
       <c r="B37" s="12">
-        <f>COUNTIF(Matriz!$K$2:$K$98,A37)</f>
+        <f>COUNTIF(Matriz!$K$2:$K$99,A37)</f>
         <v/>
       </c>
     </row>
@@ -1851,7 +1851,7 @@
         </is>
       </c>
       <c r="B38" s="12">
-        <f>COUNTIF(Matriz!$K$2:$K$98,A38)</f>
+        <f>COUNTIF(Matriz!$K$2:$K$99,A38)</f>
         <v/>
       </c>
     </row>
@@ -1866,7 +1866,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N98"/>
+  <dimension ref="A1:N99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5348,7 +5348,7 @@
       </c>
       <c r="M52" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/m3-peticiones-oracion · 153 pruebas de backend y 30 de frontend pasan; probado contra la base real</t>
+          <t>Rama feature/m3-peticiones-oracion · 165 pruebas de backend y 32 de frontend pasan; probado contra la base real</t>
         </is>
       </c>
       <c r="N52" s="19" t="inlineStr">
@@ -5370,12 +5370,12 @@
       </c>
       <c r="C53" s="19" t="inlineStr">
         <is>
-          <t>Confidencialidad y retención de las peticiones: solo las ven el Líder de su grupo, el Supervisor de sus grupos, el Pastor y el Anciano (el Secretario las registra pero no las lee; el Administrador Técnico nunca). Se guardan cifradas y se borran automáticamente a los 30 días, configurable. Consultarlas y atenderlas queda en bitácora sin incluir el texto.</t>
+          <t>Alcance de lectura de cada petición, elegido por quien la registra con autorización de quien la pide: «Solo líderes» (Líder, Supervisor, Pastor y Anciano), «Mi grupo» (todos los integrantes del grupo y los anteriores) o «Equipo de oración» (además, quien tenga el rol Equipo de oración). El alcance por defecto es configurable. Quien registra siempre ve lo que registró; el Administrador Técnico nunca ve el contenido. Solo líderes y superiores marcan una petición como atendida. Se guardan cifradas y se borran automáticamente a los 30 días, configurable. Consultarlas y atenderlas queda en bitácora sin incluir el texto.</t>
         </is>
       </c>
       <c r="D53" s="21" t="inlineStr">
         <is>
-          <t>Resp. P8</t>
+          <t>Resp. P8 + Respuesta</t>
         </is>
       </c>
       <c r="E53" s="19" t="inlineStr">
@@ -5420,12 +5420,12 @@
       </c>
       <c r="M53" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/m3-peticiones-oracion · 153 pruebas de backend y 30 de frontend pasan; probado contra la base real</t>
+          <t>Rama feature/m3-peticiones-oracion · 165 pruebas de backend y 32 de frontend pasan; probado contra la base real</t>
         </is>
       </c>
       <c r="N53" s="19" t="inlineStr">
         <is>
-          <t>2026-10-24 · Cifrado, visibilidad por rol, borrado a los 30 días configurable (tarea diaria en el despliegue).</t>
+          <t>2026-10-24 · Alcance por petición (líderes, grupo, equipo), cifrado y borrado a los 30 días configurable. Cambia la matriz aprobada: actualizar con la iglesia.</t>
         </is>
       </c>
     </row>
@@ -5914,7 +5914,7 @@
       </c>
       <c r="C61" s="19" t="inlineStr">
         <is>
-          <t>Componente de peticiones reutilizable: cualquier módulo (grupos hoy; cursos o eventos después) se registra como origen y decide quién registra y quién ve. Toda petición guarda su origen de forma inmutable (tipo, identificador y una etiqueta fija, por ejemplo «Grupo de Conexión · Norte · reunión del 22/10/2026») y lo muestra siempre en el listado.</t>
+          <t>Componente de peticiones reutilizable: cualquier módulo (grupos hoy; cursos o eventos después) se registra como origen y decide quién registra y qué nivel de acceso tiene cada persona. Toda petición guarda su origen de forma inmutable (tipo, identificador y una etiqueta fija, por ejemplo «Grupo de Conexión · Norte · reunión del 22/10/2026») y lo muestra siempre en el listado.</t>
         </is>
       </c>
       <c r="D61" s="21" t="inlineStr">
@@ -5964,7 +5964,7 @@
       </c>
       <c r="M61" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/m3-peticiones-oracion · 153 pruebas de backend y 30 de frontend pasan; probado contra la base real</t>
+          <t>Rama feature/m3-peticiones-oracion · 165 pruebas de backend y 32 de frontend pasan; probado contra la base real</t>
         </is>
       </c>
       <c r="N61" s="19" t="inlineStr">
@@ -5976,42 +5976,42 @@
     <row r="62">
       <c r="A62" s="18" t="inlineStr">
         <is>
-          <t>M4-01</t>
+          <t>M3-15</t>
         </is>
       </c>
       <c r="B62" s="19" t="inlineStr">
         <is>
-          <t>M4 Kids Check-In/Out</t>
+          <t>M3 Grupos de Conexión</t>
         </is>
       </c>
       <c r="C62" s="19" t="inlineStr">
         <is>
-          <t>Sustitución de la ficha física de papel.</t>
-        </is>
-      </c>
-      <c r="D62" s="19" t="inlineStr">
-        <is>
-          <t>v1 / v2</t>
+          <t>Equipo de oración: rol configurable (Equipo de oración) que se asigna a las personas que se reúnen a orar por las peticiones compartidas con ese alcance; no da acceso a nada más. Opción de ocultar el nombre de quien pide: los campos del formulario marcados «identifica a la persona» solo los ven líderes y quien registró.</t>
+        </is>
+      </c>
+      <c r="D62" s="21" t="inlineStr">
+        <is>
+          <t>Respuesta</t>
         </is>
       </c>
       <c r="E62" s="19" t="inlineStr">
         <is>
-          <t>Fuera del MVP</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="F62" s="19" t="inlineStr">
         <is>
-          <t>Fase 2</t>
+          <t>Fase 1</t>
         </is>
       </c>
       <c r="G62" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sprint 4</t>
         </is>
       </c>
       <c r="H62" s="19" t="inlineStr">
         <is>
-          <t>Posterior</t>
+          <t>H3 · MVP (Grupos)</t>
         </is>
       </c>
       <c r="I62" s="20" t="inlineStr">
@@ -6031,16 +6031,24 @@
       </c>
       <c r="L62" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M62" s="19" t="inlineStr"/>
-      <c r="N62" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M62" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/m3-peticiones-oracion · 165 pruebas de backend y 32 de frontend pasan; probado contra la base real</t>
+        </is>
+      </c>
+      <c r="N62" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-24 · Rol Equipo de oración y nombre oculto; falta definir el texto de privacidad específico.</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="18" t="inlineStr">
         <is>
-          <t>M4-02</t>
+          <t>M4-01</t>
         </is>
       </c>
       <c r="B63" s="19" t="inlineStr">
@@ -6050,12 +6058,12 @@
       </c>
       <c r="C63" s="19" t="inlineStr">
         <is>
-          <t>Registro de ingreso del menor con salón o clase asignada y generación de código único.</t>
-        </is>
-      </c>
-      <c r="D63" s="21" t="inlineStr">
-        <is>
-          <t>v1 + Nuevo v3</t>
+          <t>Sustitución de la ficha física de papel.</t>
+        </is>
+      </c>
+      <c r="D63" s="19" t="inlineStr">
+        <is>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E63" s="19" t="inlineStr">
@@ -6104,7 +6112,7 @@
     <row r="64">
       <c r="A64" s="18" t="inlineStr">
         <is>
-          <t>M4-03</t>
+          <t>M4-02</t>
         </is>
       </c>
       <c r="B64" s="19" t="inlineStr">
@@ -6114,12 +6122,12 @@
       </c>
       <c r="C64" s="19" t="inlineStr">
         <is>
-          <t>Código QR dinámico o OTP temporal en la PWA del padre o tutor.</t>
-        </is>
-      </c>
-      <c r="D64" s="19" t="inlineStr">
-        <is>
-          <t>v2</t>
+          <t>Registro de ingreso del menor con salón o clase asignada y generación de código único.</t>
+        </is>
+      </c>
+      <c r="D64" s="21" t="inlineStr">
+        <is>
+          <t>v1 + Nuevo v3</t>
         </is>
       </c>
       <c r="E64" s="19" t="inlineStr">
@@ -6168,7 +6176,7 @@
     <row r="65">
       <c r="A65" s="18" t="inlineStr">
         <is>
-          <t>M4-04</t>
+          <t>M4-03</t>
         </is>
       </c>
       <c r="B65" s="19" t="inlineStr">
@@ -6178,7 +6186,7 @@
       </c>
       <c r="C65" s="19" t="inlineStr">
         <is>
-          <t>Validación al entregar: el servidor de Kids escanea el código y confirma identidad y fotografía del tutor autorizado en el Expediente Digital.</t>
+          <t>Código QR dinámico o OTP temporal en la PWA del padre o tutor.</t>
         </is>
       </c>
       <c r="D65" s="19" t="inlineStr">
@@ -6232,7 +6240,7 @@
     <row r="66">
       <c r="A66" s="18" t="inlineStr">
         <is>
-          <t>M4-05</t>
+          <t>M4-04</t>
         </is>
       </c>
       <c r="B66" s="19" t="inlineStr">
@@ -6242,12 +6250,12 @@
       </c>
       <c r="C66" s="19" t="inlineStr">
         <is>
-          <t>Alternativa para tutores sin smartphone, sin batería o sin conexión (p. ej. código por SMS o comprobante imprimible con identificación). Por definir.</t>
-        </is>
-      </c>
-      <c r="D66" s="21" t="inlineStr">
-        <is>
-          <t>Nuevo v3</t>
+          <t>Validación al entregar: el servidor de Kids escanea el código y confirma identidad y fotografía del tutor autorizado en el Expediente Digital.</t>
+        </is>
+      </c>
+      <c r="D66" s="19" t="inlineStr">
+        <is>
+          <t>v2</t>
         </is>
       </c>
       <c r="E66" s="19" t="inlineStr">
@@ -6282,7 +6290,7 @@
       </c>
       <c r="K66" s="19" t="inlineStr">
         <is>
-          <t>Por definir</t>
+          <t>VoBo pendiente</t>
         </is>
       </c>
       <c r="L66" s="19" t="inlineStr">
@@ -6296,7 +6304,7 @@
     <row r="67">
       <c r="A67" s="18" t="inlineStr">
         <is>
-          <t>M4-06</t>
+          <t>M4-05</t>
         </is>
       </c>
       <c r="B67" s="19" t="inlineStr">
@@ -6306,7 +6314,7 @@
       </c>
       <c r="C67" s="19" t="inlineStr">
         <is>
-          <t>Autorización temporal de un tercero para recoger al menor, con aprobación del tutor registrado.</t>
+          <t>Alternativa para tutores sin smartphone, sin batería o sin conexión (p. ej. código por SMS o comprobante imprimible con identificación). Por definir.</t>
         </is>
       </c>
       <c r="D67" s="21" t="inlineStr">
@@ -6346,7 +6354,7 @@
       </c>
       <c r="K67" s="19" t="inlineStr">
         <is>
-          <t>VoBo pendiente</t>
+          <t>Por definir</t>
         </is>
       </c>
       <c r="L67" s="19" t="inlineStr">
@@ -6360,7 +6368,7 @@
     <row r="68">
       <c r="A68" s="18" t="inlineStr">
         <is>
-          <t>M4-07</t>
+          <t>M4-06</t>
         </is>
       </c>
       <c r="B68" s="19" t="inlineStr">
@@ -6370,7 +6378,7 @@
       </c>
       <c r="C68" s="19" t="inlineStr">
         <is>
-          <t>Caducidad del código y bitácora de cada entrega (quién recogió, quién entregó, hora).</t>
+          <t>Autorización temporal de un tercero para recoger al menor, con aprobación del tutor registrado.</t>
         </is>
       </c>
       <c r="D68" s="21" t="inlineStr">
@@ -6424,7 +6432,7 @@
     <row r="69">
       <c r="A69" s="18" t="inlineStr">
         <is>
-          <t>M4-08</t>
+          <t>M4-07</t>
         </is>
       </c>
       <c r="B69" s="19" t="inlineStr">
@@ -6434,7 +6442,7 @@
       </c>
       <c r="C69" s="19" t="inlineStr">
         <is>
-          <t>Funcionamiento sin conexión o con conexión degradada para el check-out.</t>
+          <t>Caducidad del código y bitácora de cada entrega (quién recogió, quién entregó, hora).</t>
         </is>
       </c>
       <c r="D69" s="21" t="inlineStr">
@@ -6488,52 +6496,52 @@
     <row r="70">
       <c r="A70" s="18" t="inlineStr">
         <is>
-          <t>M5-01</t>
+          <t>M4-08</t>
         </is>
       </c>
       <c r="B70" s="19" t="inlineStr">
         <is>
-          <t>M5 Áreas y servidores</t>
+          <t>M4 Kids Check-In/Out</t>
         </is>
       </c>
       <c r="C70" s="19" t="inlineStr">
         <is>
-          <t>Catálogo mínimo de áreas y asignación de servidores. Versión reducida del módulo 5, necesaria para permisos por área. Sirve como primer censo.</t>
-        </is>
-      </c>
-      <c r="D70" s="19" t="inlineStr">
-        <is>
-          <t>v3</t>
+          <t>Funcionamiento sin conexión o con conexión degradada para el check-out.</t>
+        </is>
+      </c>
+      <c r="D70" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3</t>
         </is>
       </c>
       <c r="E70" s="19" t="inlineStr">
         <is>
-          <t>MVP mínimo</t>
+          <t>Fuera del MVP</t>
         </is>
       </c>
       <c r="F70" s="19" t="inlineStr">
         <is>
-          <t>Fase 0</t>
+          <t>Fase 2</t>
         </is>
       </c>
       <c r="G70" s="19" t="inlineStr">
         <is>
-          <t>Sprint 1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H70" s="19" t="inlineStr">
         <is>
-          <t>H2 · Fase 0 completa</t>
-        </is>
-      </c>
-      <c r="I70" s="19" t="inlineStr">
-        <is>
-          <t>Como pastor quiero un catálogo de áreas con su personal para conocer la estructura.</t>
-        </is>
-      </c>
-      <c r="J70" s="19" t="inlineStr">
-        <is>
-          <t>Crear un área, asignar servidores y ver el conteo real.</t>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="I70" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
+        </is>
+      </c>
+      <c r="J70" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
         </is>
       </c>
       <c r="K70" s="19" t="inlineStr">
@@ -6552,7 +6560,7 @@
     <row r="71">
       <c r="A71" s="18" t="inlineStr">
         <is>
-          <t>M5-02</t>
+          <t>M5-01</t>
         </is>
       </c>
       <c r="B71" s="19" t="inlineStr">
@@ -6562,42 +6570,42 @@
       </c>
       <c r="C71" s="19" t="inlineStr">
         <is>
-          <t>Roles jerárquicos dentro de cada área (directores, líderes, maestros, servidores).</t>
+          <t>Catálogo mínimo de áreas y asignación de servidores. Versión reducida del módulo 5, necesaria para permisos por área. Sirve como primer censo.</t>
         </is>
       </c>
       <c r="D71" s="19" t="inlineStr">
         <is>
-          <t>v1</t>
+          <t>v3</t>
         </is>
       </c>
       <c r="E71" s="19" t="inlineStr">
         <is>
-          <t>Fuera del MVP</t>
+          <t>MVP mínimo</t>
         </is>
       </c>
       <c r="F71" s="19" t="inlineStr">
         <is>
-          <t>Fase 4</t>
+          <t>Fase 0</t>
         </is>
       </c>
       <c r="G71" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sprint 1</t>
         </is>
       </c>
       <c r="H71" s="19" t="inlineStr">
         <is>
-          <t>Posterior</t>
-        </is>
-      </c>
-      <c r="I71" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
-        </is>
-      </c>
-      <c r="J71" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
+          <t>H2 · Fase 0 completa</t>
+        </is>
+      </c>
+      <c r="I71" s="19" t="inlineStr">
+        <is>
+          <t>Como pastor quiero un catálogo de áreas con su personal para conocer la estructura.</t>
+        </is>
+      </c>
+      <c r="J71" s="19" t="inlineStr">
+        <is>
+          <t>Crear un área, asignar servidores y ver el conteo real.</t>
         </is>
       </c>
       <c r="K71" s="19" t="inlineStr">
@@ -6616,7 +6624,7 @@
     <row r="72">
       <c r="A72" s="18" t="inlineStr">
         <is>
-          <t>M5-03</t>
+          <t>M5-02</t>
         </is>
       </c>
       <c r="B72" s="19" t="inlineStr">
@@ -6626,12 +6634,12 @@
       </c>
       <c r="C72" s="19" t="inlineStr">
         <is>
-          <t>Organigrama y número real de servidores activos, directores y líderes por área.</t>
+          <t>Roles jerárquicos dentro de cada área (directores, líderes, maestros, servidores).</t>
         </is>
       </c>
       <c r="D72" s="19" t="inlineStr">
         <is>
-          <t>v2</t>
+          <t>v1</t>
         </is>
       </c>
       <c r="E72" s="19" t="inlineStr">
@@ -6680,7 +6688,7 @@
     <row r="73">
       <c r="A73" s="18" t="inlineStr">
         <is>
-          <t>M5-04</t>
+          <t>M5-03</t>
         </is>
       </c>
       <c r="B73" s="19" t="inlineStr">
@@ -6690,12 +6698,12 @@
       </c>
       <c r="C73" s="19" t="inlineStr">
         <is>
-          <t>Control de asistencia a turnos o servicios.</t>
+          <t>Organigrama y número real de servidores activos, directores y líderes por área.</t>
         </is>
       </c>
       <c r="D73" s="19" t="inlineStr">
         <is>
-          <t>v1 / v2</t>
+          <t>v2</t>
         </is>
       </c>
       <c r="E73" s="19" t="inlineStr">
@@ -6744,7 +6752,7 @@
     <row r="74">
       <c r="A74" s="18" t="inlineStr">
         <is>
-          <t>M5-05</t>
+          <t>M5-04</t>
         </is>
       </c>
       <c r="B74" s="19" t="inlineStr">
@@ -6754,7 +6762,7 @@
       </c>
       <c r="C74" s="19" t="inlineStr">
         <is>
-          <t>Tablero de avisos y notificaciones interno por área.</t>
+          <t>Control de asistencia a turnos o servicios.</t>
         </is>
       </c>
       <c r="D74" s="19" t="inlineStr">
@@ -6808,7 +6816,7 @@
     <row r="75">
       <c r="A75" s="18" t="inlineStr">
         <is>
-          <t>M5-06</t>
+          <t>M5-05</t>
         </is>
       </c>
       <c r="B75" s="19" t="inlineStr">
@@ -6818,7 +6826,7 @@
       </c>
       <c r="C75" s="19" t="inlineStr">
         <is>
-          <t>Gestión financiera por área: caja chica y gastos operativos.</t>
+          <t>Tablero de avisos y notificaciones interno por área.</t>
         </is>
       </c>
       <c r="D75" s="19" t="inlineStr">
@@ -6872,22 +6880,22 @@
     <row r="76">
       <c r="A76" s="18" t="inlineStr">
         <is>
-          <t>M6-01</t>
+          <t>M5-06</t>
         </is>
       </c>
       <c r="B76" s="19" t="inlineStr">
         <is>
-          <t>M6 Ministerios de servicio</t>
+          <t>M5 Áreas y servidores</t>
         </is>
       </c>
       <c r="C76" s="19" t="inlineStr">
         <is>
-          <t>Control de personal propio de cada ministerio.</t>
-        </is>
-      </c>
-      <c r="D76" s="22" t="inlineStr">
-        <is>
-          <t>Recuperado v1</t>
+          <t>Gestión financiera por área: caja chica y gastos operativos.</t>
+        </is>
+      </c>
+      <c r="D76" s="19" t="inlineStr">
+        <is>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E76" s="19" t="inlineStr">
@@ -6936,7 +6944,7 @@
     <row r="77">
       <c r="A77" s="18" t="inlineStr">
         <is>
-          <t>M6-02</t>
+          <t>M6-01</t>
         </is>
       </c>
       <c r="B77" s="19" t="inlineStr">
@@ -6946,12 +6954,12 @@
       </c>
       <c r="C77" s="19" t="inlineStr">
         <is>
-          <t>Menú o catálogo digital interactivo (público o interno), autogestionado.</t>
-        </is>
-      </c>
-      <c r="D77" s="19" t="inlineStr">
-        <is>
-          <t>v1 / v2</t>
+          <t>Control de personal propio de cada ministerio.</t>
+        </is>
+      </c>
+      <c r="D77" s="22" t="inlineStr">
+        <is>
+          <t>Recuperado v1</t>
         </is>
       </c>
       <c r="E77" s="19" t="inlineStr">
@@ -7000,7 +7008,7 @@
     <row r="78">
       <c r="A78" s="18" t="inlineStr">
         <is>
-          <t>M6-03</t>
+          <t>M6-02</t>
         </is>
       </c>
       <c r="B78" s="19" t="inlineStr">
@@ -7010,7 +7018,7 @@
       </c>
       <c r="C78" s="19" t="inlineStr">
         <is>
-          <t>Calendario de turnos: días regulares de servicio y eventos especiales.</t>
+          <t>Menú o catálogo digital interactivo (público o interno), autogestionado.</t>
         </is>
       </c>
       <c r="D78" s="19" t="inlineStr">
@@ -7064,7 +7072,7 @@
     <row r="79">
       <c r="A79" s="18" t="inlineStr">
         <is>
-          <t>M6-04</t>
+          <t>M6-03</t>
         </is>
       </c>
       <c r="B79" s="19" t="inlineStr">
@@ -7074,7 +7082,7 @@
       </c>
       <c r="C79" s="19" t="inlineStr">
         <is>
-          <t>Registro de asistentes o personas atendidas.</t>
+          <t>Calendario de turnos: días regulares de servicio y eventos especiales.</t>
         </is>
       </c>
       <c r="D79" s="19" t="inlineStr">
@@ -7128,7 +7136,7 @@
     <row r="80">
       <c r="A80" s="18" t="inlineStr">
         <is>
-          <t>M6-05</t>
+          <t>M6-04</t>
         </is>
       </c>
       <c r="B80" s="19" t="inlineStr">
@@ -7138,7 +7146,7 @@
       </c>
       <c r="C80" s="19" t="inlineStr">
         <is>
-          <t>Control de gastos y de inventario básico.</t>
+          <t>Registro de asistentes o personas atendidas.</t>
         </is>
       </c>
       <c r="D80" s="19" t="inlineStr">
@@ -7192,7 +7200,7 @@
     <row r="81">
       <c r="A81" s="18" t="inlineStr">
         <is>
-          <t>M6-06</t>
+          <t>M6-05</t>
         </is>
       </c>
       <c r="B81" s="19" t="inlineStr">
@@ -7202,7 +7210,7 @@
       </c>
       <c r="C81" s="19" t="inlineStr">
         <is>
-          <t>Canal de comunicación directo con el área de Administración General.</t>
+          <t>Control de gastos y de inventario básico.</t>
         </is>
       </c>
       <c r="D81" s="19" t="inlineStr">
@@ -7256,7 +7264,7 @@
     <row r="82">
       <c r="A82" s="18" t="inlineStr">
         <is>
-          <t>M6-07</t>
+          <t>M6-06</t>
         </is>
       </c>
       <c r="B82" s="19" t="inlineStr">
@@ -7266,12 +7274,12 @@
       </c>
       <c r="C82" s="19" t="inlineStr">
         <is>
-          <t>Servicio Médico: los datos de salud de las personas atendidas requieren tratamiento de datos sensibles. Por definir alcance.</t>
-        </is>
-      </c>
-      <c r="D82" s="21" t="inlineStr">
-        <is>
-          <t>Nuevo v3</t>
+          <t>Canal de comunicación directo con el área de Administración General.</t>
+        </is>
+      </c>
+      <c r="D82" s="19" t="inlineStr">
+        <is>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E82" s="19" t="inlineStr">
@@ -7306,7 +7314,7 @@
       </c>
       <c r="K82" s="19" t="inlineStr">
         <is>
-          <t>Por definir</t>
+          <t>VoBo pendiente</t>
         </is>
       </c>
       <c r="L82" s="19" t="inlineStr">
@@ -7320,22 +7328,22 @@
     <row r="83">
       <c r="A83" s="18" t="inlineStr">
         <is>
-          <t>M7-01</t>
+          <t>M6-07</t>
         </is>
       </c>
       <c r="B83" s="19" t="inlineStr">
         <is>
-          <t>M7 Eventos y aforo</t>
+          <t>M6 Ministerios de servicio</t>
         </is>
       </c>
       <c r="C83" s="19" t="inlineStr">
         <is>
-          <t>Eventos abiertos o evangelísticos con formulario de inscripción rápida, sin requerir historial previo.</t>
-        </is>
-      </c>
-      <c r="D83" s="19" t="inlineStr">
-        <is>
-          <t>v1 / v2</t>
+          <t>Servicio Médico: los datos de salud de las personas atendidas requieren tratamiento de datos sensibles. Por definir alcance.</t>
+        </is>
+      </c>
+      <c r="D83" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3</t>
         </is>
       </c>
       <c r="E83" s="19" t="inlineStr">
@@ -7370,7 +7378,7 @@
       </c>
       <c r="K83" s="19" t="inlineStr">
         <is>
-          <t>VoBo pendiente</t>
+          <t>Por definir</t>
         </is>
       </c>
       <c r="L83" s="19" t="inlineStr">
@@ -7384,7 +7392,7 @@
     <row r="84">
       <c r="A84" s="18" t="inlineStr">
         <is>
-          <t>M7-02</t>
+          <t>M7-01</t>
         </is>
       </c>
       <c r="B84" s="19" t="inlineStr">
@@ -7394,12 +7402,12 @@
       </c>
       <c r="C84" s="19" t="inlineStr">
         <is>
-          <t>Consolidación (inducción de personas que asisten por primera vez) como tipo de evento.</t>
-        </is>
-      </c>
-      <c r="D84" s="22" t="inlineStr">
-        <is>
-          <t>Recuperado v1</t>
+          <t>Eventos abiertos o evangelísticos con formulario de inscripción rápida, sin requerir historial previo.</t>
+        </is>
+      </c>
+      <c r="D84" s="19" t="inlineStr">
+        <is>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E84" s="19" t="inlineStr">
@@ -7448,7 +7456,7 @@
     <row r="85">
       <c r="A85" s="18" t="inlineStr">
         <is>
-          <t>M7-03</t>
+          <t>M7-02</t>
         </is>
       </c>
       <c r="B85" s="19" t="inlineStr">
@@ -7458,7 +7466,7 @@
       </c>
       <c r="C85" s="19" t="inlineStr">
         <is>
-          <t>Encargados de evento (personal de la iglesia únicamente; no se controla personal externo).</t>
+          <t>Consolidación (inducción de personas que asisten por primera vez) como tipo de evento.</t>
         </is>
       </c>
       <c r="D85" s="22" t="inlineStr">
@@ -7512,7 +7520,7 @@
     <row r="86">
       <c r="A86" s="18" t="inlineStr">
         <is>
-          <t>M7-04</t>
+          <t>M7-03</t>
         </is>
       </c>
       <c r="B86" s="19" t="inlineStr">
@@ -7522,12 +7530,12 @@
       </c>
       <c r="C86" s="19" t="inlineStr">
         <is>
-          <t>Control de cupo en tiempo real que bloquea el sobrecupo en eventos con aforo limitado (ej. 30 o 50 lugares).</t>
-        </is>
-      </c>
-      <c r="D86" s="19" t="inlineStr">
-        <is>
-          <t>v1 / v2</t>
+          <t>Encargados de evento (personal de la iglesia únicamente; no se controla personal externo).</t>
+        </is>
+      </c>
+      <c r="D86" s="22" t="inlineStr">
+        <is>
+          <t>Recuperado v1</t>
         </is>
       </c>
       <c r="E86" s="19" t="inlineStr">
@@ -7576,7 +7584,7 @@
     <row r="87">
       <c r="A87" s="18" t="inlineStr">
         <is>
-          <t>M7-05</t>
+          <t>M7-04</t>
         </is>
       </c>
       <c r="B87" s="19" t="inlineStr">
@@ -7586,12 +7594,12 @@
       </c>
       <c r="C87" s="19" t="inlineStr">
         <is>
-          <t>Control de asistentes sin lista previa, para aforo y para dar a conocer la iglesia.</t>
+          <t>Control de cupo en tiempo real que bloquea el sobrecupo en eventos con aforo limitado (ej. 30 o 50 lugares).</t>
         </is>
       </c>
       <c r="D87" s="19" t="inlineStr">
         <is>
-          <t>v1</t>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E87" s="19" t="inlineStr">
@@ -7640,7 +7648,7 @@
     <row r="88">
       <c r="A88" s="18" t="inlineStr">
         <is>
-          <t>M7-06</t>
+          <t>M7-05</t>
         </is>
       </c>
       <c r="B88" s="19" t="inlineStr">
@@ -7650,12 +7658,12 @@
       </c>
       <c r="C88" s="19" t="inlineStr">
         <is>
-          <t>Seguimiento de personas nuevas: conversión de un invitado a Expediente Digital y canalización a un curso o Grupo de Conexión.</t>
-        </is>
-      </c>
-      <c r="D88" s="21" t="inlineStr">
-        <is>
-          <t>Nuevo v3</t>
+          <t>Control de asistentes sin lista previa, para aforo y para dar a conocer la iglesia.</t>
+        </is>
+      </c>
+      <c r="D88" s="19" t="inlineStr">
+        <is>
+          <t>v1</t>
         </is>
       </c>
       <c r="E88" s="19" t="inlineStr">
@@ -7704,52 +7712,52 @@
     <row r="89">
       <c r="A89" s="18" t="inlineStr">
         <is>
-          <t>NF-01</t>
+          <t>M7-06</t>
         </is>
       </c>
       <c r="B89" s="19" t="inlineStr">
         <is>
-          <t>No funcionales</t>
+          <t>M7 Eventos y aforo</t>
         </is>
       </c>
       <c r="C89" s="19" t="inlineStr">
         <is>
-          <t>Cumplimiento de la LFPDPPP: aviso de privacidad, consentimiento y derechos ARCO.</t>
-        </is>
-      </c>
-      <c r="D89" s="19" t="inlineStr">
-        <is>
-          <t>v3</t>
+          <t>Seguimiento de personas nuevas: conversión de un invitado a Expediente Digital y canalización a un curso o Grupo de Conexión.</t>
+        </is>
+      </c>
+      <c r="D89" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3</t>
         </is>
       </c>
       <c r="E89" s="19" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Fuera del MVP</t>
         </is>
       </c>
       <c r="F89" s="19" t="inlineStr">
         <is>
-          <t>Fase 0</t>
+          <t>Fase 4</t>
         </is>
       </c>
       <c r="G89" s="19" t="inlineStr">
         <is>
-          <t>Sprint 1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H89" s="19" t="inlineStr">
         <is>
-          <t>H1 · 18-oct (núcleo Fase 0)</t>
-        </is>
-      </c>
-      <c r="I89" s="19" t="inlineStr">
-        <is>
-          <t>Como iglesia queremos cumplir con la LFPDPPP.</t>
-        </is>
-      </c>
-      <c r="J89" s="19" t="inlineStr">
-        <is>
-          <t>Aviso de privacidad, consentimiento y atención de derechos ARCO disponibles.</t>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="I89" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
+        </is>
+      </c>
+      <c r="J89" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
         </is>
       </c>
       <c r="K89" s="19" t="inlineStr">
@@ -7768,7 +7776,7 @@
     <row r="90">
       <c r="A90" s="18" t="inlineStr">
         <is>
-          <t>NF-02</t>
+          <t>NF-01</t>
         </is>
       </c>
       <c r="B90" s="19" t="inlineStr">
@@ -7778,7 +7786,7 @@
       </c>
       <c r="C90" s="19" t="inlineStr">
         <is>
-          <t>Cifrado en tránsito y en reposo. Cifrado adicional a nivel de campo para peticiones de oración.</t>
+          <t>Cumplimiento de la LFPDPPP: aviso de privacidad, consentimiento y derechos ARCO.</t>
         </is>
       </c>
       <c r="D90" s="19" t="inlineStr">
@@ -7798,7 +7806,7 @@
       </c>
       <c r="G90" s="19" t="inlineStr">
         <is>
-          <t>Sprint 0</t>
+          <t>Sprint 1</t>
         </is>
       </c>
       <c r="H90" s="19" t="inlineStr">
@@ -7808,12 +7816,12 @@
       </c>
       <c r="I90" s="19" t="inlineStr">
         <is>
-          <t>Como iglesia queremos proteger los datos sensibles.</t>
+          <t>Como iglesia queremos cumplir con la LFPDPPP.</t>
         </is>
       </c>
       <c r="J90" s="19" t="inlineStr">
         <is>
-          <t>HTTPS obligatorio y peticiones de oración ilegibles directamente en la base.</t>
+          <t>Aviso de privacidad, consentimiento y atención de derechos ARCO disponibles.</t>
         </is>
       </c>
       <c r="K90" s="19" t="inlineStr">
@@ -7823,24 +7831,16 @@
       </c>
       <c r="L90" s="19" t="inlineStr">
         <is>
-          <t>En pruebas</t>
-        </is>
-      </c>
-      <c r="M90" s="19" t="inlineStr">
-        <is>
-          <t>Rama feature/m3-peticiones-oracion · 153 pruebas de backend y 30 de frontend pasan; probado contra la base real</t>
-        </is>
-      </c>
-      <c r="N90" s="19" t="inlineStr">
-        <is>
-          <t>2026-10-24 · Peticiones cifradas a nivel de campo; falta cifrado en reposo de toda la base (proveedor de nube).</t>
-        </is>
-      </c>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M90" s="19" t="inlineStr"/>
+      <c r="N90" s="19" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="18" t="inlineStr">
         <is>
-          <t>NF-03</t>
+          <t>NF-02</t>
         </is>
       </c>
       <c r="B91" s="19" t="inlineStr">
@@ -7850,7 +7850,7 @@
       </c>
       <c r="C91" s="19" t="inlineStr">
         <is>
-          <t>Bitácora de auditoría de solo-añadir: quién consultó o modificó expedientes, ofrendas y asistencias.</t>
+          <t>Cifrado en tránsito y en reposo. Cifrado adicional a nivel de campo para peticiones de oración.</t>
         </is>
       </c>
       <c r="D91" s="19" t="inlineStr">
@@ -7870,7 +7870,7 @@
       </c>
       <c r="G91" s="19" t="inlineStr">
         <is>
-          <t>Sprint 1</t>
+          <t>Sprint 0</t>
         </is>
       </c>
       <c r="H91" s="19" t="inlineStr">
@@ -7880,12 +7880,12 @@
       </c>
       <c r="I91" s="19" t="inlineStr">
         <is>
-          <t>Como pastor quiero una bitácora que nadie pueda alterar.</t>
+          <t>Como iglesia queremos proteger los datos sensibles.</t>
         </is>
       </c>
       <c r="J91" s="19" t="inlineStr">
         <is>
-          <t>El usuario de la aplicación no puede actualizar ni borrar registros de bitácora.</t>
+          <t>HTTPS obligatorio y peticiones de oración ilegibles directamente en la base.</t>
         </is>
       </c>
       <c r="K91" s="19" t="inlineStr">
@@ -7900,19 +7900,19 @@
       </c>
       <c r="M91" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/nf-03-bitacora · 69 pruebas de backend pasan</t>
+          <t>Rama feature/m3-peticiones-oracion · 165 pruebas de backend y 32 de frontend pasan; probado contra la base real</t>
         </is>
       </c>
       <c r="N91" s="19" t="inlineStr">
         <is>
-          <t>2026-10-10 · Bloqueo en aplicación y trigger de PostgreSQL (UPDATE/DELETE/TRUNCATE); pantalla de consulta con permiso bitacora.ver.</t>
+          <t>2026-10-24 · Peticiones cifradas a nivel de campo; falta cifrado en reposo de toda la base (proveedor de nube).</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="18" t="inlineStr">
         <is>
-          <t>NF-04</t>
+          <t>NF-03</t>
         </is>
       </c>
       <c r="B92" s="19" t="inlineStr">
@@ -7922,7 +7922,7 @@
       </c>
       <c r="C92" s="19" t="inlineStr">
         <is>
-          <t>Respaldos automáticos diarios cifrados y prueba periódica de restauración.</t>
+          <t>Bitácora de auditoría de solo-añadir: quién consultó o modificó expedientes, ofrendas y asistencias.</t>
         </is>
       </c>
       <c r="D92" s="19" t="inlineStr">
@@ -7942,7 +7942,7 @@
       </c>
       <c r="G92" s="19" t="inlineStr">
         <is>
-          <t>Sprint 0</t>
+          <t>Sprint 1</t>
         </is>
       </c>
       <c r="H92" s="19" t="inlineStr">
@@ -7952,12 +7952,12 @@
       </c>
       <c r="I92" s="19" t="inlineStr">
         <is>
-          <t>Como iglesia queremos no perder información.</t>
+          <t>Como pastor quiero una bitácora que nadie pueda alterar.</t>
         </is>
       </c>
       <c r="J92" s="19" t="inlineStr">
         <is>
-          <t>Respaldo diario cifrado y restauración probada en un ambiente de pruebas.</t>
+          <t>El usuario de la aplicación no puede actualizar ni borrar registros de bitácora.</t>
         </is>
       </c>
       <c r="K92" s="19" t="inlineStr">
@@ -7967,16 +7967,24 @@
       </c>
       <c r="L92" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M92" s="19" t="inlineStr"/>
-      <c r="N92" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M92" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/nf-03-bitacora · 69 pruebas de backend pasan</t>
+        </is>
+      </c>
+      <c r="N92" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-10 · Bloqueo en aplicación y trigger de PostgreSQL (UPDATE/DELETE/TRUNCATE); pantalla de consulta con permiso bitacora.ver.</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="18" t="inlineStr">
         <is>
-          <t>NF-05</t>
+          <t>NF-04</t>
         </is>
       </c>
       <c r="B93" s="19" t="inlineStr">
@@ -7986,47 +7994,47 @@
       </c>
       <c r="C93" s="19" t="inlineStr">
         <is>
-          <t>Disponibilidad esperada en horarios de servicio (fines de semana y reuniones de grupo). Por definir meta.</t>
-        </is>
-      </c>
-      <c r="D93" s="21" t="inlineStr">
-        <is>
-          <t>Nuevo v3</t>
+          <t>Respaldos automáticos diarios cifrados y prueba periódica de restauración.</t>
+        </is>
+      </c>
+      <c r="D93" s="19" t="inlineStr">
+        <is>
+          <t>v3</t>
         </is>
       </c>
       <c r="E93" s="19" t="inlineStr">
         <is>
-          <t>Fuera del MVP</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="F93" s="19" t="inlineStr">
         <is>
-          <t>Transversal</t>
+          <t>Fase 0</t>
         </is>
       </c>
       <c r="G93" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sprint 0</t>
         </is>
       </c>
       <c r="H93" s="19" t="inlineStr">
         <is>
-          <t>Posterior</t>
-        </is>
-      </c>
-      <c r="I93" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
-        </is>
-      </c>
-      <c r="J93" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
+          <t>H1 · 18-oct (núcleo Fase 0)</t>
+        </is>
+      </c>
+      <c r="I93" s="19" t="inlineStr">
+        <is>
+          <t>Como iglesia queremos no perder información.</t>
+        </is>
+      </c>
+      <c r="J93" s="19" t="inlineStr">
+        <is>
+          <t>Respaldo diario cifrado y restauración probada en un ambiente de pruebas.</t>
         </is>
       </c>
       <c r="K93" s="19" t="inlineStr">
         <is>
-          <t>Por definir</t>
+          <t>VoBo pendiente</t>
         </is>
       </c>
       <c r="L93" s="19" t="inlineStr">
@@ -8040,7 +8048,7 @@
     <row r="94">
       <c r="A94" s="18" t="inlineStr">
         <is>
-          <t>NF-06</t>
+          <t>NF-05</t>
         </is>
       </c>
       <c r="B94" s="19" t="inlineStr">
@@ -8050,69 +8058,61 @@
       </c>
       <c r="C94" s="19" t="inlineStr">
         <is>
-          <t>Pase de lista sin conexión con sincronización posterior (reuniones en domicilios con mala señal).</t>
-        </is>
-      </c>
-      <c r="D94" s="19" t="inlineStr">
-        <is>
-          <t>v3</t>
+          <t>Disponibilidad esperada en horarios de servicio (fines de semana y reuniones de grupo). Por definir meta.</t>
+        </is>
+      </c>
+      <c r="D94" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3</t>
         </is>
       </c>
       <c r="E94" s="19" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Fuera del MVP</t>
         </is>
       </c>
       <c r="F94" s="19" t="inlineStr">
         <is>
-          <t>Fase 0</t>
+          <t>Transversal</t>
         </is>
       </c>
       <c r="G94" s="19" t="inlineStr">
         <is>
-          <t>Sprint 3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H94" s="19" t="inlineStr">
         <is>
-          <t>H3 · MVP (Grupos)</t>
-        </is>
-      </c>
-      <c r="I94" s="19" t="inlineStr">
-        <is>
-          <t>Como secretario quiero que el pase de lista funcione sin señal.</t>
-        </is>
-      </c>
-      <c r="J94" s="19" t="inlineStr">
-        <is>
-          <t>Prueba en modo avión y sincronización al reconectar.</t>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="I94" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
+        </is>
+      </c>
+      <c r="J94" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
         </is>
       </c>
       <c r="K94" s="19" t="inlineStr">
         <is>
-          <t>VoBo pendiente</t>
+          <t>Por definir</t>
         </is>
       </c>
       <c r="L94" s="19" t="inlineStr">
         <is>
-          <t>En pruebas</t>
-        </is>
-      </c>
-      <c r="M94" s="19" t="inlineStr">
-        <is>
-          <t>Rama feature/nf-06-sin-conexion · 117 pruebas de backend y 27 de frontend; probado en Chrome real con service worker</t>
-        </is>
-      </c>
-      <c r="N94" s="19" t="inlineStr">
-        <is>
-          <t>2026-10-24 · Probado de punta a punta en Chrome (sin red → cola → sincronización). Pendiente probar en Android e iOS reales.</t>
-        </is>
-      </c>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M94" s="19" t="inlineStr"/>
+      <c r="N94" s="19" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="18" t="inlineStr">
         <is>
-          <t>NF-07</t>
+          <t>NF-06</t>
         </is>
       </c>
       <c r="B95" s="19" t="inlineStr">
@@ -8122,7 +8122,7 @@
       </c>
       <c r="C95" s="19" t="inlineStr">
         <is>
-          <t>Funciona en Android, iOS y escritorio. En iOS, las notificaciones push requieren instalar la PWA; el respaldo por WhatsApp cubre el resto.</t>
+          <t>Pase de lista sin conexión con sincronización posterior (reuniones en domicilios con mala señal).</t>
         </is>
       </c>
       <c r="D95" s="19" t="inlineStr">
@@ -8142,22 +8142,22 @@
       </c>
       <c r="G95" s="19" t="inlineStr">
         <is>
-          <t>Sprint 0</t>
+          <t>Sprint 3</t>
         </is>
       </c>
       <c r="H95" s="19" t="inlineStr">
         <is>
-          <t>H1 · 18-oct (núcleo Fase 0)</t>
+          <t>H3 · MVP (Grupos)</t>
         </is>
       </c>
       <c r="I95" s="19" t="inlineStr">
         <is>
-          <t>Como usuario quiero usar el sistema en mi dispositivo.</t>
+          <t>Como secretario quiero que el pase de lista funcione sin señal.</t>
         </is>
       </c>
       <c r="J95" s="19" t="inlineStr">
         <is>
-          <t>Pruebas en Android, iOS y escritorio; push en iOS con la PWA instalada y respaldo por WhatsApp.</t>
+          <t>Prueba en modo avión y sincronización al reconectar.</t>
         </is>
       </c>
       <c r="K95" s="19" t="inlineStr">
@@ -8167,16 +8167,24 @@
       </c>
       <c r="L95" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M95" s="19" t="inlineStr"/>
-      <c r="N95" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M95" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/nf-06-sin-conexion · 117 pruebas de backend y 27 de frontend; probado en Chrome real con service worker</t>
+        </is>
+      </c>
+      <c r="N95" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-24 · Probado de punta a punta en Chrome (sin red → cola → sincronización). Pendiente probar en Android e iOS reales.</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="18" t="inlineStr">
         <is>
-          <t>NF-08</t>
+          <t>NF-07</t>
         </is>
       </c>
       <c r="B96" s="19" t="inlineStr">
@@ -8186,12 +8194,12 @@
       </c>
       <c r="C96" s="19" t="inlineStr">
         <is>
-          <t>Dimensionamiento para ~1,000 personas, con picos los fines de semana, y margen de crecimiento.</t>
-        </is>
-      </c>
-      <c r="D96" s="21" t="inlineStr">
-        <is>
-          <t>Resp. P8</t>
+          <t>Funciona en Android, iOS y escritorio. En iOS, las notificaciones push requieren instalar la PWA; el respaldo por WhatsApp cubre el resto.</t>
+        </is>
+      </c>
+      <c r="D96" s="19" t="inlineStr">
+        <is>
+          <t>v3</t>
         </is>
       </c>
       <c r="E96" s="19" t="inlineStr">
@@ -8216,12 +8224,12 @@
       </c>
       <c r="I96" s="19" t="inlineStr">
         <is>
-          <t>Como iglesia queremos que el sistema soporte a ~1,000 personas.</t>
+          <t>Como usuario quiero usar el sistema en mi dispositivo.</t>
         </is>
       </c>
       <c r="J96" s="19" t="inlineStr">
         <is>
-          <t>Prueba de carga con volumen representativo (por definir) sin degradación.</t>
+          <t>Pruebas en Android, iOS y escritorio; push en iOS con la PWA instalada y respaldo por WhatsApp.</t>
         </is>
       </c>
       <c r="K96" s="19" t="inlineStr">
@@ -8240,7 +8248,7 @@
     <row r="97">
       <c r="A97" s="18" t="inlineStr">
         <is>
-          <t>NF-09</t>
+          <t>NF-08</t>
         </is>
       </c>
       <c r="B97" s="19" t="inlineStr">
@@ -8250,42 +8258,42 @@
       </c>
       <c r="C97" s="19" t="inlineStr">
         <is>
-          <t>Reportes transversales: asistencia, finanzas, crecimiento de la iglesia, exportables a Excel y PDF.</t>
+          <t>Dimensionamiento para ~1,000 personas, con picos los fines de semana, y margen de crecimiento.</t>
         </is>
       </c>
       <c r="D97" s="21" t="inlineStr">
         <is>
-          <t>Nuevo v3</t>
+          <t>Resp. P8</t>
         </is>
       </c>
       <c r="E97" s="19" t="inlineStr">
         <is>
-          <t>Fuera del MVP</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="F97" s="19" t="inlineStr">
         <is>
-          <t>Transversal</t>
+          <t>Fase 0</t>
         </is>
       </c>
       <c r="G97" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sprint 0</t>
         </is>
       </c>
       <c r="H97" s="19" t="inlineStr">
         <is>
-          <t>Posterior</t>
-        </is>
-      </c>
-      <c r="I97" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
-        </is>
-      </c>
-      <c r="J97" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
+          <t>H1 · 18-oct (núcleo Fase 0)</t>
+        </is>
+      </c>
+      <c r="I97" s="19" t="inlineStr">
+        <is>
+          <t>Como iglesia queremos que el sistema soporte a ~1,000 personas.</t>
+        </is>
+      </c>
+      <c r="J97" s="19" t="inlineStr">
+        <is>
+          <t>Prueba de carga con volumen representativo (por definir) sin degradación.</t>
         </is>
       </c>
       <c r="K97" s="19" t="inlineStr">
@@ -8304,7 +8312,7 @@
     <row r="98">
       <c r="A98" s="18" t="inlineStr">
         <is>
-          <t>NF-10</t>
+          <t>NF-09</t>
         </is>
       </c>
       <c r="B98" s="19" t="inlineStr">
@@ -8314,42 +8322,42 @@
       </c>
       <c r="C98" s="19" t="inlineStr">
         <is>
-          <t>Usabilidad para personas mayores: tipografía grande, alto contraste, flujos cortos (ver sección 5).</t>
-        </is>
-      </c>
-      <c r="D98" s="19" t="inlineStr">
-        <is>
-          <t>v3 + Obs. 1</t>
+          <t>Reportes transversales: asistencia, finanzas, crecimiento de la iglesia, exportables a Excel y PDF.</t>
+        </is>
+      </c>
+      <c r="D98" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3</t>
         </is>
       </c>
       <c r="E98" s="19" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Fuera del MVP</t>
         </is>
       </c>
       <c r="F98" s="19" t="inlineStr">
         <is>
-          <t>Fase 0</t>
+          <t>Transversal</t>
         </is>
       </c>
       <c r="G98" s="19" t="inlineStr">
         <is>
-          <t>Sprint 0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H98" s="19" t="inlineStr">
         <is>
-          <t>H1 · 18-oct (núcleo Fase 0)</t>
-        </is>
-      </c>
-      <c r="I98" s="19" t="inlineStr">
-        <is>
-          <t>Como persona mayor quiero una interfaz fácil de leer y usar.</t>
-        </is>
-      </c>
-      <c r="J98" s="19" t="inlineStr">
-        <is>
-          <t>Texto base 18 px, botones de al menos 48 px, contraste AA; prueba con usuarios mayores.</t>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="I98" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
+        </is>
+      </c>
+      <c r="J98" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
         </is>
       </c>
       <c r="K98" s="19" t="inlineStr">
@@ -8365,9 +8373,73 @@
       <c r="M98" s="19" t="inlineStr"/>
       <c r="N98" s="19" t="inlineStr"/>
     </row>
+    <row r="99">
+      <c r="A99" s="18" t="inlineStr">
+        <is>
+          <t>NF-10</t>
+        </is>
+      </c>
+      <c r="B99" s="19" t="inlineStr">
+        <is>
+          <t>No funcionales</t>
+        </is>
+      </c>
+      <c r="C99" s="19" t="inlineStr">
+        <is>
+          <t>Usabilidad para personas mayores: tipografía grande, alto contraste, flujos cortos (ver sección 5).</t>
+        </is>
+      </c>
+      <c r="D99" s="19" t="inlineStr">
+        <is>
+          <t>v3 + Obs. 1</t>
+        </is>
+      </c>
+      <c r="E99" s="19" t="inlineStr">
+        <is>
+          <t>MVP</t>
+        </is>
+      </c>
+      <c r="F99" s="19" t="inlineStr">
+        <is>
+          <t>Fase 0</t>
+        </is>
+      </c>
+      <c r="G99" s="19" t="inlineStr">
+        <is>
+          <t>Sprint 0</t>
+        </is>
+      </c>
+      <c r="H99" s="19" t="inlineStr">
+        <is>
+          <t>H1 · 18-oct (núcleo Fase 0)</t>
+        </is>
+      </c>
+      <c r="I99" s="19" t="inlineStr">
+        <is>
+          <t>Como persona mayor quiero una interfaz fácil de leer y usar.</t>
+        </is>
+      </c>
+      <c r="J99" s="19" t="inlineStr">
+        <is>
+          <t>Texto base 18 px, botones de al menos 48 px, contraste AA; prueba con usuarios mayores.</t>
+        </is>
+      </c>
+      <c r="K99" s="19" t="inlineStr">
+        <is>
+          <t>VoBo pendiente</t>
+        </is>
+      </c>
+      <c r="L99" s="19" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M99" s="19" t="inlineStr"/>
+      <c r="N99" s="19" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N98"/>
-  <conditionalFormatting sqref="L2:L98">
+  <autoFilter ref="A1:N99"/>
+  <conditionalFormatting sqref="L2:L99">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$L2="Hecho"</formula>
     </cfRule>
@@ -8384,7 +8456,7 @@
       <formula>$L2="Bloqueado"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K2:K98">
+  <conditionalFormatting sqref="K2:K99">
     <cfRule type="expression" priority="6" dxfId="0">
       <formula>$K2="Aprobado"</formula>
     </cfRule>
@@ -8392,16 +8464,16 @@
       <formula>$K2="Por definir"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H2:H98">
+  <conditionalFormatting sqref="H2:H99">
     <cfRule type="expression" priority="8" dxfId="5">
       <formula>LEFT($H2,2)="H1"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="L2:L98" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="L2:L99" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Pendiente,En diseño,En desarrollo,En pruebas,Hecho,Bloqueado"</formula1>
     </dataValidation>
-    <dataValidation sqref="K2:K98" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="K2:K99" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"VoBo pendiente,Aprobado,Por definir,Rechazado"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Peticiones de oración: leyenda de privacidad al capturar
- Alerta visible en el formulario de captura: pide confirmar que la persona está de acuerdo en
  quién leerá su petición (según el alcance elegido), indica si el nombre queda oculto y los días
  tras los que se borra
- El formulario informa los días de conservación vigentes (configurable) para la leyenda
- Documentación y matriz actualizadas

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/trazabilidad/Matriz de Trazabilidad MDF.xlsx
+++ b/docs/trazabilidad/Matriz de Trazabilidad MDF.xlsx
@@ -5348,7 +5348,7 @@
       </c>
       <c r="M52" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/m3-peticiones-oracion · 165 pruebas de backend y 32 de frontend pasan; probado contra la base real</t>
+          <t>Rama feature/m3-peticiones-oracion · 166 pruebas de backend y 32 de frontend pasan; probado contra la base real</t>
         </is>
       </c>
       <c r="N52" s="19" t="inlineStr">
@@ -5420,7 +5420,7 @@
       </c>
       <c r="M53" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/m3-peticiones-oracion · 165 pruebas de backend y 32 de frontend pasan; probado contra la base real</t>
+          <t>Rama feature/m3-peticiones-oracion · 166 pruebas de backend y 32 de frontend pasan; probado contra la base real</t>
         </is>
       </c>
       <c r="N53" s="19" t="inlineStr">
@@ -5964,7 +5964,7 @@
       </c>
       <c r="M61" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/m3-peticiones-oracion · 165 pruebas de backend y 32 de frontend pasan; probado contra la base real</t>
+          <t>Rama feature/m3-peticiones-oracion · 166 pruebas de backend y 32 de frontend pasan; probado contra la base real</t>
         </is>
       </c>
       <c r="N61" s="19" t="inlineStr">
@@ -5986,7 +5986,7 @@
       </c>
       <c r="C62" s="19" t="inlineStr">
         <is>
-          <t>Equipo de oración: rol configurable (Equipo de oración) que se asigna a las personas que se reúnen a orar por las peticiones compartidas con ese alcance; no da acceso a nada más. Opción de ocultar el nombre de quien pide: los campos del formulario marcados «identifica a la persona» solo los ven líderes y quien registró.</t>
+          <t>Equipo de oración: rol configurable (Equipo de oración) que se asigna a las personas que se reúnen a orar por las peticiones compartidas con ese alcance; no da acceso a nada más. Opción de ocultar el nombre de quien pide: los campos del formulario marcados «identifica a la persona» solo los ven líderes y quien registró. Al capturar se muestra una leyenda que pide confirmar la autorización de quien pide, indica quién la leerá y cuándo se borra.</t>
         </is>
       </c>
       <c r="D62" s="21" t="inlineStr">
@@ -6036,12 +6036,12 @@
       </c>
       <c r="M62" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/m3-peticiones-oracion · 165 pruebas de backend y 32 de frontend pasan; probado contra la base real</t>
+          <t>Rama feature/m3-peticiones-oracion · 166 pruebas de backend y 32 de frontend pasan; probado contra la base real</t>
         </is>
       </c>
       <c r="N62" s="19" t="inlineStr">
         <is>
-          <t>2026-10-24 · Rol Equipo de oración y nombre oculto; falta definir el texto de privacidad específico.</t>
+          <t>2026-10-24 · Rol Equipo de oración, nombre oculto y leyenda de privacidad al capturar. Falta el aviso de privacidad oficial de la iglesia.</t>
         </is>
       </c>
     </row>
@@ -7900,7 +7900,7 @@
       </c>
       <c r="M91" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/m3-peticiones-oracion · 165 pruebas de backend y 32 de frontend pasan; probado contra la base real</t>
+          <t>Rama feature/m3-peticiones-oracion · 166 pruebas de backend y 32 de frontend pasan; probado contra la base real</t>
         </is>
       </c>
       <c r="N91" s="19" t="inlineStr">

</xml_diff>

<commit_message>
M3-07/M3-11/M1-19: dashboard de supervisión, tablero de mensajes y corrección de zona horaria
- Dashboard «Resumen de grupos»: asistencia por semana y por grupo, avisos (sin lista, asistencia
  baja con umbral configurable, ofrendas con diferencia), ofrendas y peticiones solo según rol;
  sin datos de personas; el Secretario y el Tesorero no lo ven
- Tablero de mensajes reutilizable por origen: publican Líder, Supervisor, Secretario y Pastor, leen
  los integrantes; fijados, borrado lógico, no leídos, retención configurable y pantalla «Avisos»
- Componentes Meter y ColumnsChart en el sistema de diseño
- Corrige la zona horaria: «hoy» ya no es la fecha de UTC del servidor sino la de México, para que
  las reuniones de la tarde-noche no se fechen con el día siguiente
- La tarea diaria del despliegue también purga el tablero
- Documentación v3.11 y matriz de trazabilidad

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/trazabilidad/Matriz de Trazabilidad MDF.xlsx
+++ b/docs/trazabilidad/Matriz de Trazabilidad MDF.xlsx
@@ -3642,7 +3642,7 @@
       </c>
       <c r="C27" s="19" t="inlineStr">
         <is>
-          <t>Dashboard y tablero de mensajes por módulo, construidos con un componente genérico reutilizable. En el MVP: Grupos de Conexión y vista general de Fase 0.</t>
+          <t>Dashboard y tablero de mensajes por módulo como componentes genéricos: el tablero (y las peticiones) se registran por origen y cada módulo decide quién publica y quién lee; los gráficos del dashboard viven en el sistema de diseño. Grupos de Conexión es el primer módulo en usarlos.</t>
         </is>
       </c>
       <c r="D27" s="21" t="inlineStr">
@@ -3687,11 +3687,19 @@
       </c>
       <c r="L27" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M27" s="19" t="inlineStr"/>
-      <c r="N27" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M27" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/m3-dashboard-tablero · 195 pruebas de backend y 39 de frontend pasan; probado contra la base real</t>
+        </is>
+      </c>
+      <c r="N27" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-25 · Tablero y gráficas como componentes genéricos; grupos es el primer origen.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="18" t="inlineStr">
@@ -5442,7 +5450,7 @@
       </c>
       <c r="C54" s="19" t="inlineStr">
         <is>
-          <t>Reportes de supervisión: dashboards de asistencia, ofrendas y crecimiento por grupo, según permisos.</t>
+          <t>Dashboard de supervisión («Resumen de grupos») para Supervisor, Líder, Pastor y Anciano sobre los grupos que cada uno puede consultar: asistencia por semana y por grupo, grupos sin lista esta semana, asistencia por debajo de un mínimo configurable (60 % por defecto), ofrendas avaladas, pendientes y con diferencia (solo si el rol ve finanzas) y peticiones activas (solo las que puede leer). No muestra datos de personas. El Secretario y el Tesorero no lo ven.</t>
         </is>
       </c>
       <c r="D54" s="19" t="inlineStr">
@@ -5487,11 +5495,19 @@
       </c>
       <c r="L54" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M54" s="19" t="inlineStr"/>
-      <c r="N54" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M54" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/m3-dashboard-tablero · 195 pruebas de backend y 39 de frontend pasan; probado contra la base real</t>
+        </is>
+      </c>
+      <c r="N54" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-25 · Dashboard con asistencia, avisos y datos según rol; umbral configurable.</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="18" t="inlineStr">
@@ -5706,7 +5722,7 @@
       </c>
       <c r="C58" s="19" t="inlineStr">
         <is>
-          <t>Dashboard y tablero de mensajes del grupo.</t>
+          <t>Tablero de mensajes del grupo: lo publican Líder, Supervisor, Secretario y Pastor; lo leen todos los integrantes activos. Mensajes de hasta 1,000 caracteres, con opción de fijarlos, borrado lógico, contador de mensajes nuevos y conservación configurable (90 días). Pantalla «Avisos» para quien no abre la página del grupo.</t>
         </is>
       </c>
       <c r="D58" s="21" t="inlineStr">
@@ -5751,11 +5767,19 @@
       </c>
       <c r="L58" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M58" s="19" t="inlineStr"/>
-      <c r="N58" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M58" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/m3-dashboard-tablero · 195 pruebas de backend y 39 de frontend pasan; probado contra la base real</t>
+        </is>
+      </c>
+      <c r="N58" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-25 · Tablero con fijados, no leídos y retención configurable; falta notificación push (M1-09).</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="18" t="inlineStr">

</xml_diff>

<commit_message>
M1-09: notificaciones push con sonido y vibración
- App notificaciones: suscripciones por dispositivo, claves VAPID, envío en
  segundo plano con limpieza de dispositivos caducados y prueba de envío.
- Avisan de mensajes nuevos del tablero (solo a quien puede leerlos, sin
  avisar al autor) y de un estudio nuevo de la semana.
- Parámetro configurable para apagar las notificaciones.
- Service worker propio (caché, sin conexión y push); íconos PNG.
- Activación desde Inicio y Mi cuenta; al cerrar sesión el teléfono se da de baja.
- Docs v3.13 (anexo L), matriz y guía de despliegue actualizadas.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/trazabilidad/Matriz de Trazabilidad MDF.xlsx
+++ b/docs/trazabilidad/Matriz de Trazabilidad MDF.xlsx
@@ -3063,11 +3063,19 @@
       </c>
       <c r="L18" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M18" s="19" t="inlineStr"/>
-      <c r="N18" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M18" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/m1-09-notificaciones · pruebas de backend y 66 de frontend pasan; claves VAPID de QA configuradas</t>
+        </is>
+      </c>
+      <c r="N18" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-26 · Notificaciones push con sonido y vibración para mensajes del tablero y estudio nuevo, solo a quien puede leerlos; se activan por dispositivo y se pueden apagar en Configuración. Pendiente: probar en Samsung S23 e iPhone reales y los avisos de la iglesia en general (no ligados a un grupo).</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="18" t="inlineStr">
@@ -5777,7 +5785,7 @@
       </c>
       <c r="N58" s="19" t="inlineStr">
         <is>
-          <t>2026-10-25 · Tablero con fijados, no leídos y retención configurable; falta notificación push (M1-09).</t>
+          <t>2026-10-25 · Tablero con fijados, no leídos y retención configurable; la notificación push de mensajes nuevos se entrega con M1-09.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Correcciones de la primera ronda de pruebas (paso 1)
- Cerrar sesión: la baja del dispositivo de notificaciones tiene un tope de 2 s
  y ya no puede dejar el botón sin respuesta.
- Menú: los ítems de módulo muestran su ícono real en una pastilla de color.
- Invitar > Accesos: desbloquear por «Demasiados intentos» y reiniciar acceso,
  limitado al alcance de quien lo hace y con bitácora.
- Pasar lista: fila completa con palomita.
- Docs v3.14 (anexo M) y matriz con los hallazgos P1-01 a P1-12.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/trazabilidad/Matriz de Trazabilidad MDF.xlsx
+++ b/docs/trazabilidad/Matriz de Trazabilidad MDF.xlsx
@@ -8519,7 +8519,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -9039,6 +9039,330 @@
       <c r="E19" s="24" t="inlineStr">
         <is>
           <t>Incorporado en v3.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="18" t="inlineStr">
+        <is>
+          <t>P1-01</t>
+        </is>
+      </c>
+      <c r="B20" s="24" t="inlineStr">
+        <is>
+          <t>Pruebas 1: «Cerrar sesión» no hace nada.</t>
+        </is>
+      </c>
+      <c r="C20" s="24" t="inlineStr">
+        <is>
+          <t>M1-17</t>
+        </is>
+      </c>
+      <c r="D20" s="24" t="inlineStr">
+        <is>
+          <t>La baja del dispositivo de notificaciones podía quedar esperando sin límite; ahora tiene un tope de 2 s.</t>
+        </is>
+      </c>
+      <c r="E20" s="24" t="inlineStr">
+        <is>
+          <t>Corregido (v3.14)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="18" t="inlineStr">
+        <is>
+          <t>P1-02</t>
+        </is>
+      </c>
+      <c r="B21" s="24" t="inlineStr">
+        <is>
+          <t>Pruebas 1: en el menú solo se veía el ícono de Inicio.</t>
+        </is>
+      </c>
+      <c r="C21" s="24" t="inlineStr">
+        <is>
+          <t>M1-19</t>
+        </is>
+      </c>
+      <c r="D21" s="24" t="inlineStr">
+        <is>
+          <t>Los ítems de módulo dibujaban un cuadro vacío; ahora muestran su ícono en una pastilla del color del módulo.</t>
+        </is>
+      </c>
+      <c r="E21" s="24" t="inlineStr">
+        <is>
+          <t>Corregido (v3.14)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="18" t="inlineStr">
+        <is>
+          <t>P1-03</t>
+        </is>
+      </c>
+      <c r="B22" s="24" t="inlineStr">
+        <is>
+          <t>Pruebas 1: cómo reiniciar el contador tras «Demasiados intentos».</t>
+        </is>
+      </c>
+      <c r="C22" s="24" t="inlineStr">
+        <is>
+          <t>M1-17, M1-07</t>
+        </is>
+      </c>
+      <c r="D22" s="24" t="inlineStr">
+        <is>
+          <t>Pantalla Invitar &gt; Accesos: Desbloquear y Reiniciar acceso, limitado a las personas del alcance de quien lo hace; queda en bitácora.</t>
+        </is>
+      </c>
+      <c r="E22" s="24" t="inlineStr">
+        <is>
+          <t>Corregido (v3.14)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="18" t="inlineStr">
+        <is>
+          <t>P1-04</t>
+        </is>
+      </c>
+      <c r="B23" s="24" t="inlineStr">
+        <is>
+          <t>Pruebas 1: pasar lista con X o palomita.</t>
+        </is>
+      </c>
+      <c r="C23" s="24" t="inlineStr">
+        <is>
+          <t>M3-03</t>
+        </is>
+      </c>
+      <c r="D23" s="24" t="inlineStr">
+        <is>
+          <t>Fila completa tocable con palomita y estado visible.</t>
+        </is>
+      </c>
+      <c r="E23" s="24" t="inlineStr">
+        <is>
+          <t>Corregido (v3.14)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="18" t="inlineStr">
+        <is>
+          <t>P1-05</t>
+        </is>
+      </c>
+      <c r="B24" s="24" t="inlineStr">
+        <is>
+          <t>Pruebas 1: menú con categorías, barra superior con Ocultar menú y Cerrar sesión, inicio como dashboard, tema de color, tablas en Personas y Roles, botón Volver.</t>
+        </is>
+      </c>
+      <c r="C24" s="24" t="inlineStr">
+        <is>
+          <t>M1-19, M1-07</t>
+        </is>
+      </c>
+      <c r="D24" s="24" t="inlineStr">
+        <is>
+          <t>Rediseño de navegación y pantallas de administración.</t>
+        </is>
+      </c>
+      <c r="E24" s="24" t="inlineStr">
+        <is>
+          <t>Planeado (paso 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="18" t="inlineStr">
+        <is>
+          <t>P1-06</t>
+        </is>
+      </c>
+      <c r="B25" s="24" t="inlineStr">
+        <is>
+          <t>Pruebas 1: bitácora con paginación, filtros, semáforo y gráfica de errores.</t>
+        </is>
+      </c>
+      <c r="C25" s="24" t="inlineStr">
+        <is>
+          <t>M1-16</t>
+        </is>
+      </c>
+      <c r="D25" s="24" t="inlineStr">
+        <is>
+          <t>Mejora de la consulta de bitácora.</t>
+        </is>
+      </c>
+      <c r="E25" s="24" t="inlineStr">
+        <is>
+          <t>Planeado (paso 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="18" t="inlineStr">
+        <is>
+          <t>P1-07</t>
+        </is>
+      </c>
+      <c r="B26" s="24" t="inlineStr">
+        <is>
+          <t>Pruebas 1: grupos por sector (ej. Sector K, Casa 6), filtros, editar integrantes, suspender grupo, agrupar por día de reunión.</t>
+        </is>
+      </c>
+      <c r="C26" s="24" t="inlineStr">
+        <is>
+          <t>M3-01, M3-12</t>
+        </is>
+      </c>
+      <c r="D26" s="24" t="inlineStr">
+        <is>
+          <t>Sector como dato del grupo; suspender con observaciones, bitácora y dashboard.</t>
+        </is>
+      </c>
+      <c r="E26" s="24" t="inlineStr">
+        <is>
+          <t>Planeado (paso 3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="18" t="inlineStr">
+        <is>
+          <t>P1-08</t>
+        </is>
+      </c>
+      <c r="B27" s="24" t="inlineStr">
+        <is>
+          <t>Pruebas 1: personas con baja, traslado a otra iglesia, roles visibles y filtros eclesiásticos.</t>
+        </is>
+      </c>
+      <c r="C27" s="24" t="inlineStr">
+        <is>
+          <t>M1-14, M1-13</t>
+        </is>
+      </c>
+      <c r="D27" s="24" t="inlineStr">
+        <is>
+          <t>Pantallas sobre el historial de movimientos; filtros por cursos esperan al módulo de cursos.</t>
+        </is>
+      </c>
+      <c r="E27" s="24" t="inlineStr">
+        <is>
+          <t>Planeado (paso 4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="18" t="inlineStr">
+        <is>
+          <t>P1-09</t>
+        </is>
+      </c>
+      <c r="B28" s="24" t="inlineStr">
+        <is>
+          <t>Pruebas 1: invitar por QR o enlace; el líder aprueba el acceso (como Teams); asignación manual con aviso; rol por defecto.</t>
+        </is>
+      </c>
+      <c r="C28" s="24" t="inlineStr">
+        <is>
+          <t>M1-10, M3-09</t>
+        </is>
+      </c>
+      <c r="D28" s="24" t="inlineStr">
+        <is>
+          <t>Solicitud de ingreso por enlace/QR con aprobación del líder.</t>
+        </is>
+      </c>
+      <c r="E28" s="24" t="inlineStr">
+        <is>
+          <t>Planeado (paso 5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="18" t="inlineStr">
+        <is>
+          <t>P1-10</t>
+        </is>
+      </c>
+      <c r="B29" s="24" t="inlineStr">
+        <is>
+          <t>Pruebas 1: avisos masivos a la iglesia, grupos, ministerios (áreas de servicio) o personas; agrupar los recibidos.</t>
+        </is>
+      </c>
+      <c r="C29" s="24" t="inlineStr">
+        <is>
+          <t>M1-09</t>
+        </is>
+      </c>
+      <c r="D29" s="24" t="inlineStr">
+        <is>
+          <t>Requiere definir ministerios como áreas de servicio.</t>
+        </is>
+      </c>
+      <c r="E29" s="24" t="inlineStr">
+        <is>
+          <t>Planeado (paso 6)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="18" t="inlineStr">
+        <is>
+          <t>P1-11</t>
+        </is>
+      </c>
+      <c r="B30" s="24" t="inlineStr">
+        <is>
+          <t>Pruebas 1: Mi cuenta editable (datos básicos no sensibles; lo administrativo lo edita la secretaria).</t>
+        </is>
+      </c>
+      <c r="C30" s="24" t="inlineStr">
+        <is>
+          <t>M1-11</t>
+        </is>
+      </c>
+      <c r="D30" s="24" t="inlineStr">
+        <is>
+          <t>Campos editables por la persona vs. por administración.</t>
+        </is>
+      </c>
+      <c r="E30" s="24" t="inlineStr">
+        <is>
+          <t>Planeado (paso 7)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="18" t="inlineStr">
+        <is>
+          <t>P1-12</t>
+        </is>
+      </c>
+      <c r="B31" s="24" t="inlineStr">
+        <is>
+          <t>Pruebas 1: el rol de Super Usuario es el único que asigna Administrador técnico.</t>
+        </is>
+      </c>
+      <c r="C31" s="24" t="inlineStr">
+        <is>
+          <t>M1-07</t>
+        </is>
+      </c>
+      <c r="D31" s="24" t="inlineStr">
+        <is>
+          <t>Regla de asignación pendiente de confirmar.</t>
+        </is>
+      </c>
+      <c r="E31" s="24" t="inlineStr">
+        <is>
+          <t>Por confirmar</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Navegación, inicio como dashboard, tablas, bitácora y tema (paso 2)
- Barra superior con Ocultar menú, nombre de la persona y Cerrar sesión
- Menú agrupado por categorías (Operación, Catálogos, Administración)
- Inicio como dashboard: accesos rápidos por permiso y resumen de grupos
- Cinco paletas de color elegibles en Mi cuenta
- Personas y Roles en tablas, con roles visibles y Volver al listado
- Bitácora con semáforo, filtros, paginación y gráfica de errores por día
- Documentos v3.15 (anexo N) y matriz de trazabilidad actualizados

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/trazabilidad/Matriz de Trazabilidad MDF.xlsx
+++ b/docs/trazabilidad/Matriz de Trazabilidad MDF.xlsx
@@ -3487,17 +3487,17 @@
       </c>
       <c r="L24" s="19" t="inlineStr">
         <is>
-          <t>En desarrollo</t>
+          <t>En pruebas</t>
         </is>
       </c>
       <c r="M24" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/m1-07-roles · 67 pruebas de backend y 6 de frontend pasan</t>
+          <t>Rama feature/navegacion-dashboard-paso-2 · pruebas de backend y 77 de frontend pasan; lint, estilos y compilación limpios</t>
         </is>
       </c>
       <c r="N24" s="19" t="inlineStr">
         <is>
-          <t>2026-10-05 · Consultas y cambios de personas ya quedan en bitácora; falta restringir por rol (RBAC).</t>
+          <t>2026-10-27 · Bitácora con niveles tipo semáforo, filtros, paginación y gráfica de errores por día. Consultar el resumen también exige el permiso de bitácora.</t>
         </is>
       </c>
     </row>
@@ -3700,12 +3700,12 @@
       </c>
       <c r="M27" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/m3-dashboard-tablero · 195 pruebas de backend y 39 de frontend pasan; probado contra la base real</t>
+          <t>Rama feature/navegacion-dashboard-paso-2 · pruebas de backend y 77 de frontend pasan; lint, estilos y compilación limpios</t>
         </is>
       </c>
       <c r="N27" s="19" t="inlineStr">
         <is>
-          <t>2026-10-25 · Tablero y gráficas como componentes genéricos; grupos es el primer origen. Mejoras de usabilidad móvil (v3.12): barra con «Más», deshacer, confirmación al descartar.</t>
+          <t>2026-10-27 · Tablero y gráficas como componentes genéricos; grupos es el primer origen. Barra superior con Cerrar sesión, menú por categorías, Inicio como dashboard con accesos rápidos y resumen de grupos, y color de la aplicación elegible (v3.15).</t>
         </is>
       </c>
     </row>
@@ -9168,12 +9168,12 @@
       </c>
       <c r="D24" s="24" t="inlineStr">
         <is>
-          <t>Rediseño de navegación y pantallas de administración.</t>
+          <t>Barra superior, menú por categorías, Inicio como dashboard, cinco paletas de color, tablas en Personas y Roles con «Volver al listado». Pendiente: transición animada del menú.</t>
         </is>
       </c>
       <c r="E24" s="24" t="inlineStr">
         <is>
-          <t>Planeado (paso 2)</t>
+          <t>Hecho (v3.15)</t>
         </is>
       </c>
     </row>
@@ -9195,12 +9195,12 @@
       </c>
       <c r="D25" s="24" t="inlineStr">
         <is>
-          <t>Mejora de la consulta de bitácora.</t>
+          <t>Paginación, filtros por tipo, nivel, persona y fechas, semáforo y gráfica de errores y avisos por día.</t>
         </is>
       </c>
       <c r="E25" s="24" t="inlineStr">
         <is>
-          <t>Planeado (paso 2)</t>
+          <t>Hecho (v3.15)</t>
         </is>
       </c>
     </row>
@@ -9357,12 +9357,12 @@
       </c>
       <c r="D31" s="24" t="inlineStr">
         <is>
-          <t>Regla de asignación pendiente de confirmar.</t>
+          <t>Confirmado por Edgar el 27-oct-2026; el sistema ya lo cumple (nadie otorga un rol más alto que el suyo) y hay prueba.</t>
         </is>
       </c>
       <c r="E31" s="24" t="inlineStr">
         <is>
-          <t>Por confirmar</t>
+          <t>Hecho (v3.15)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Grupos: sector y casa, filtros, suspensión, roles y reuniones por día (paso 3)
- Sector (letra) y casa (número) como datos del grupo; migración que conserva
  el sector escrito antes como texto libre en la colonia
- Filtros del listado por texto, líder, día, sector y estado
- Edición de datos del grupo y cambio de rol de integrantes
- Suspender y reactivar con motivo, bitácora y reflejo en el resumen
- Cada reunión muestra asistencia, observaciones, peticiones y ofrendas
- Documentos v3.16 (anexo O) y matriz de trazabilidad actualizados

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/trazabilidad/Matriz de Trazabilidad MDF.xlsx
+++ b/docs/trazabilidad/Matriz de Trazabilidad MDF.xlsx
@@ -5076,12 +5076,12 @@
       </c>
       <c r="M48" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/m3-grupos · 88 pruebas de backend y 7 de frontend pasan</t>
+          <t>Rama feature/grupos-paso-3 · pruebas de backend y 81 de frontend pasan; lint, estilos y compilación limpios</t>
         </is>
       </c>
       <c r="N48" s="19" t="inlineStr">
         <is>
-          <t>2026-10-24 · Supervisor, Líder, Secretario, Anfitrión, Tesorero y Asistente por grupo; falta probar con líderes reales.</t>
+          <t>2026-10-27 · Supervisor, Líder, Secretario, Anfitrión, Tesorero y Asistente por grupo; ahora con cambio de rol, sector (letra), casa (número) y suspensión con motivo.</t>
         </is>
       </c>
     </row>
@@ -5852,12 +5852,12 @@
       </c>
       <c r="M59" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/m3-grupos · 88 pruebas de backend y 7 de frontend pasan</t>
+          <t>Rama feature/grupos-paso-3 · pruebas de backend y 81 de frontend pasan; lint, estilos y compilación limpios</t>
         </is>
       </c>
       <c r="N59" s="19" t="inlineStr">
         <is>
-          <t>2026-10-24 · Una reunión semanal por grupo y grupo tipo Líderes.</t>
+          <t>2026-10-27 · Una reunión semanal por grupo y grupo tipo Líderes; filtros por día, sector, líder y estado; cada reunión muestra su asistencia, observaciones, peticiones y ofrendas.</t>
         </is>
       </c>
     </row>
@@ -9222,12 +9222,12 @@
       </c>
       <c r="D26" s="24" t="inlineStr">
         <is>
-          <t>Sector como dato del grupo; suspender con observaciones, bitácora y dashboard.</t>
+          <t>Sector (letra) y casa (número), filtros, cambio de rol de integrantes, suspensión con motivo y bitácora, y reuniones con lo ocurrido cada día. Pendiente: nada de este hallazgo.</t>
         </is>
       </c>
       <c r="E26" s="24" t="inlineStr">
         <is>
-          <t>Planeado (paso 3)</t>
+          <t>Hecho (v3.16)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Personas: traslado a otra iglesia, baja con grupos, niveles y filtros (paso 4)
- Traslado a otra iglesia con destino en el historial y bitácora
- Baja y traslado retiran a la persona de sus grupos (membresía inactiva)
- Situación en la iglesia al inicio de la ficha
- Nivel de registro explicado y qué falta para el expediente completo
- Listado con grupos de cada persona y filtros por grupo y rol
- Documentos v3.17 (anexo P) y matriz de trazabilidad actualizados

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/trazabilidad/Matriz de Trazabilidad MDF.xlsx
+++ b/docs/trazabilidad/Matriz de Trazabilidad MDF.xlsx
@@ -3276,12 +3276,12 @@
       </c>
       <c r="M21" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/m1-01-expediente · 56 pruebas de backend y 6 de frontend pasan</t>
+          <t>Rama feature/personas-paso-4 · pruebas de backend y 85 de frontend pasan; lint, estilos y compilación limpios</t>
         </is>
       </c>
       <c r="N21" s="19" t="inlineStr">
         <is>
-          <t>2026-10-05 · Niveles contacto → participante → expediente completo; duplicados por WhatsApp.</t>
+          <t>2026-10-27 · Niveles contacto → participante → expediente completo, ahora explicados en la ficha; duplicados por WhatsApp.</t>
         </is>
       </c>
     </row>
@@ -3420,12 +3420,12 @@
       </c>
       <c r="M23" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/m1-01-expediente · 56 pruebas de backend y 6 de frontend pasan</t>
+          <t>Rama feature/personas-paso-4 · pruebas de backend y 85 de frontend pasan; lint, estilos y compilación limpios</t>
         </is>
       </c>
       <c r="N23" s="19" t="inlineStr">
         <is>
-          <t>2026-10-05 · Historial de movimientos con fecha y motivo.</t>
+          <t>2026-10-27 · Historial de movimientos con fecha y motivo; ahora incluye traslado a otra iglesia con su destino, y la baja retira a la persona de sus grupos.</t>
         </is>
       </c>
     </row>
@@ -9249,12 +9249,12 @@
       </c>
       <c r="D27" s="24" t="inlineStr">
         <is>
-          <t>Pantallas sobre el historial de movimientos; filtros por cursos esperan al módulo de cursos.</t>
+          <t>Traslado a otra iglesia, baja que saca de los grupos, situación al inicio de la ficha, niveles explicados, grupos y filtros por grupo y rol. Pendiente: filtros por cursos (módulo de Cursos).</t>
         </is>
       </c>
       <c r="E27" s="24" t="inlineStr">
         <is>
-          <t>Planeado (paso 4)</t>
+          <t>Hecho (v3.17)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Invitación por enlace o QR con sala de espera y asignación con aviso (paso 5)
- Enlace y QR por grupo (generar, regenerar, desactivar) y página pública
  de sala de espera con aprobación del líder
- Solicitudes pendientes en la ficha del grupo (aprobar, rechazar, avisar por
  WhatsApp) y notificación al líder
- Asignar un grupo desde la ficha de la persona; aviso al líder y a la persona
  cada vez que alguien entra a un grupo
- Rol por defecto Miembro / Asistente al invitar
- Documentos v3.18 (anexo Q) y matriz de trazabilidad actualizados

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/trazabilidad/Matriz de Trazabilidad MDF.xlsx
+++ b/docs/trazabilidad/Matriz de Trazabilidad MDF.xlsx
@@ -3135,11 +3135,19 @@
       </c>
       <c r="L19" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M19" s="19" t="inlineStr"/>
-      <c r="N19" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M19" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/paso-5-invitaciones · pruebas de backend y 93 de frontend pasan; lint, estilos y compilación limpios</t>
+        </is>
+      </c>
+      <c r="N19" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-27 · Rol por defecto Miembro / Asistente al invitar; invitación por enlace o QR con aprobación del líder (sala de espera) y asignación manual desde la ficha de la persona, con notificaciones.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="18" t="inlineStr">
@@ -5644,12 +5652,12 @@
       </c>
       <c r="M56" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/m3-grupos · 88 pruebas de backend y 7 de frontend pasan</t>
+          <t>Rama feature/paso-5-invitaciones · pruebas de backend y 93 de frontend pasan; lint, estilos y compilación limpios</t>
         </is>
       </c>
       <c r="N56" s="19" t="inlineStr">
         <is>
-          <t>2026-10-24 · Invitados registrados como Contacto con consentimiento y sin duplicar por WhatsApp.</t>
+          <t>2026-10-27 · Los invitados entran al grupo como Contacto cuando el líder aprueba su solicitud por enlace o QR.</t>
         </is>
       </c>
     </row>
@@ -9276,12 +9284,12 @@
       </c>
       <c r="D28" s="24" t="inlineStr">
         <is>
-          <t>Solicitud de ingreso por enlace/QR con aprobación del líder.</t>
+          <t>Enlace y QR por grupo, sala de espera con aprobación del líder, asignación manual con aviso y rol por defecto Miembro / Asistente. Pendiente: definir qué rol hace la asignación manual.</t>
         </is>
       </c>
       <c r="E28" s="24" t="inlineStr">
         <is>
-          <t>Planeado (paso 5)</t>
+          <t>Hecho (v3.18)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Administrador de roles y permisos, con el rol Secretaria (paso 6)
- Catálogo de permisos por módulo, pantalla y acción (definido por el código)
- Pantalla Roles y permisos: crear, editar, duplicar, desactivar y reactivar roles
  con una matriz de casillas; todo cambio queda en bitácora
- Reglas de jerarquía: nadie está por encima del Super Usuario, nadie crea o
  edita un rol de su nivel o superior ni concede permisos que no tiene
- Rol Secretaria, igual al Pastor en lo administrativo; el Super Usuario, el
  Pastor y la Secretaria administran roles
- Lo que puede hacer cada persona, por módulo y pantalla, en la asignación de roles
- Documentos v3.19 (anexo R, requisito M1-24) y matriz de trazabilidad actualizados

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/trazabilidad/Matriz de Trazabilidad MDF.xlsx
+++ b/docs/trazabilidad/Matriz de Trazabilidad MDF.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Origen v1" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Matriz'!$A$1:$N$99</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Matriz'!$A$1:$N$100</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -897,31 +897,31 @@
         </is>
       </c>
       <c r="B5" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$99,$A5)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$100,$A5)</f>
         <v/>
       </c>
       <c r="C5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$99,$A5,Matriz!$L$2:$L$99,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$100,$A5,Matriz!$L$2:$L$100,"Pendiente")</f>
         <v/>
       </c>
       <c r="D5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$99,$A5,Matriz!$L$2:$L$99,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$100,$A5,Matriz!$L$2:$L$100,"En diseño")</f>
         <v/>
       </c>
       <c r="E5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$99,$A5,Matriz!$L$2:$L$99,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$100,$A5,Matriz!$L$2:$L$100,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$99,$A5,Matriz!$L$2:$L$99,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$100,$A5,Matriz!$L$2:$L$100,"En pruebas")</f>
         <v/>
       </c>
       <c r="G5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$99,$A5,Matriz!$L$2:$L$99,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$100,$A5,Matriz!$L$2:$L$100,"Hecho")</f>
         <v/>
       </c>
       <c r="H5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$99,$A5,Matriz!$L$2:$L$99,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$100,$A5,Matriz!$L$2:$L$100,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I5" s="13">
@@ -936,31 +936,31 @@
         </is>
       </c>
       <c r="B6" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$99,$A6)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$100,$A6)</f>
         <v/>
       </c>
       <c r="C6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$99,$A6,Matriz!$L$2:$L$99,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$100,$A6,Matriz!$L$2:$L$100,"Pendiente")</f>
         <v/>
       </c>
       <c r="D6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$99,$A6,Matriz!$L$2:$L$99,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$100,$A6,Matriz!$L$2:$L$100,"En diseño")</f>
         <v/>
       </c>
       <c r="E6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$99,$A6,Matriz!$L$2:$L$99,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$100,$A6,Matriz!$L$2:$L$100,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$99,$A6,Matriz!$L$2:$L$99,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$100,$A6,Matriz!$L$2:$L$100,"En pruebas")</f>
         <v/>
       </c>
       <c r="G6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$99,$A6,Matriz!$L$2:$L$99,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$100,$A6,Matriz!$L$2:$L$100,"Hecho")</f>
         <v/>
       </c>
       <c r="H6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$99,$A6,Matriz!$L$2:$L$99,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$100,$A6,Matriz!$L$2:$L$100,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I6" s="13">
@@ -975,31 +975,31 @@
         </is>
       </c>
       <c r="B7" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$99,$A7)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$100,$A7)</f>
         <v/>
       </c>
       <c r="C7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$99,$A7,Matriz!$L$2:$L$99,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$100,$A7,Matriz!$L$2:$L$100,"Pendiente")</f>
         <v/>
       </c>
       <c r="D7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$99,$A7,Matriz!$L$2:$L$99,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$100,$A7,Matriz!$L$2:$L$100,"En diseño")</f>
         <v/>
       </c>
       <c r="E7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$99,$A7,Matriz!$L$2:$L$99,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$100,$A7,Matriz!$L$2:$L$100,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$99,$A7,Matriz!$L$2:$L$99,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$100,$A7,Matriz!$L$2:$L$100,"En pruebas")</f>
         <v/>
       </c>
       <c r="G7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$99,$A7,Matriz!$L$2:$L$99,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$100,$A7,Matriz!$L$2:$L$100,"Hecho")</f>
         <v/>
       </c>
       <c r="H7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$99,$A7,Matriz!$L$2:$L$99,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$100,$A7,Matriz!$L$2:$L$100,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I7" s="13">
@@ -1014,31 +1014,31 @@
         </is>
       </c>
       <c r="B8" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$99,$A8)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$100,$A8)</f>
         <v/>
       </c>
       <c r="C8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$99,$A8,Matriz!$L$2:$L$99,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$100,$A8,Matriz!$L$2:$L$100,"Pendiente")</f>
         <v/>
       </c>
       <c r="D8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$99,$A8,Matriz!$L$2:$L$99,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$100,$A8,Matriz!$L$2:$L$100,"En diseño")</f>
         <v/>
       </c>
       <c r="E8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$99,$A8,Matriz!$L$2:$L$99,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$100,$A8,Matriz!$L$2:$L$100,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$99,$A8,Matriz!$L$2:$L$99,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$100,$A8,Matriz!$L$2:$L$100,"En pruebas")</f>
         <v/>
       </c>
       <c r="G8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$99,$A8,Matriz!$L$2:$L$99,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$100,$A8,Matriz!$L$2:$L$100,"Hecho")</f>
         <v/>
       </c>
       <c r="H8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$99,$A8,Matriz!$L$2:$L$99,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$100,$A8,Matriz!$L$2:$L$100,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I8" s="13">
@@ -1053,31 +1053,31 @@
         </is>
       </c>
       <c r="B9" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$99,$A9)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$100,$A9)</f>
         <v/>
       </c>
       <c r="C9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$99,$A9,Matriz!$L$2:$L$99,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$100,$A9,Matriz!$L$2:$L$100,"Pendiente")</f>
         <v/>
       </c>
       <c r="D9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$99,$A9,Matriz!$L$2:$L$99,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$100,$A9,Matriz!$L$2:$L$100,"En diseño")</f>
         <v/>
       </c>
       <c r="E9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$99,$A9,Matriz!$L$2:$L$99,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$100,$A9,Matriz!$L$2:$L$100,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$99,$A9,Matriz!$L$2:$L$99,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$100,$A9,Matriz!$L$2:$L$100,"En pruebas")</f>
         <v/>
       </c>
       <c r="G9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$99,$A9,Matriz!$L$2:$L$99,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$100,$A9,Matriz!$L$2:$L$100,"Hecho")</f>
         <v/>
       </c>
       <c r="H9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$99,$A9,Matriz!$L$2:$L$99,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$100,$A9,Matriz!$L$2:$L$100,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I9" s="13">
@@ -1092,31 +1092,31 @@
         </is>
       </c>
       <c r="B10" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$99,$A10)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$100,$A10)</f>
         <v/>
       </c>
       <c r="C10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$99,$A10,Matriz!$L$2:$L$99,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$100,$A10,Matriz!$L$2:$L$100,"Pendiente")</f>
         <v/>
       </c>
       <c r="D10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$99,$A10,Matriz!$L$2:$L$99,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$100,$A10,Matriz!$L$2:$L$100,"En diseño")</f>
         <v/>
       </c>
       <c r="E10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$99,$A10,Matriz!$L$2:$L$99,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$100,$A10,Matriz!$L$2:$L$100,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$99,$A10,Matriz!$L$2:$L$99,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$100,$A10,Matriz!$L$2:$L$100,"En pruebas")</f>
         <v/>
       </c>
       <c r="G10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$99,$A10,Matriz!$L$2:$L$99,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$100,$A10,Matriz!$L$2:$L$100,"Hecho")</f>
         <v/>
       </c>
       <c r="H10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$99,$A10,Matriz!$L$2:$L$99,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$100,$A10,Matriz!$L$2:$L$100,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I10" s="13">
@@ -1131,31 +1131,31 @@
         </is>
       </c>
       <c r="B11" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$99,$A11)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$100,$A11)</f>
         <v/>
       </c>
       <c r="C11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$99,$A11,Matriz!$L$2:$L$99,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$100,$A11,Matriz!$L$2:$L$100,"Pendiente")</f>
         <v/>
       </c>
       <c r="D11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$99,$A11,Matriz!$L$2:$L$99,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$100,$A11,Matriz!$L$2:$L$100,"En diseño")</f>
         <v/>
       </c>
       <c r="E11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$99,$A11,Matriz!$L$2:$L$99,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$100,$A11,Matriz!$L$2:$L$100,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$99,$A11,Matriz!$L$2:$L$99,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$100,$A11,Matriz!$L$2:$L$100,"En pruebas")</f>
         <v/>
       </c>
       <c r="G11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$99,$A11,Matriz!$L$2:$L$99,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$100,$A11,Matriz!$L$2:$L$100,"Hecho")</f>
         <v/>
       </c>
       <c r="H11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$99,$A11,Matriz!$L$2:$L$99,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$100,$A11,Matriz!$L$2:$L$100,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I11" s="13">
@@ -1256,31 +1256,31 @@
         </is>
       </c>
       <c r="B16" s="12">
-        <f>COUNTIF(Matriz!$H$2:$H$99,$A16)</f>
+        <f>COUNTIF(Matriz!$H$2:$H$100,$A16)</f>
         <v/>
       </c>
       <c r="C16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$99,$A16,Matriz!$L$2:$L$99,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$100,$A16,Matriz!$L$2:$L$100,"Pendiente")</f>
         <v/>
       </c>
       <c r="D16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$99,$A16,Matriz!$L$2:$L$99,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$100,$A16,Matriz!$L$2:$L$100,"En diseño")</f>
         <v/>
       </c>
       <c r="E16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$99,$A16,Matriz!$L$2:$L$99,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$100,$A16,Matriz!$L$2:$L$100,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$99,$A16,Matriz!$L$2:$L$99,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$100,$A16,Matriz!$L$2:$L$100,"En pruebas")</f>
         <v/>
       </c>
       <c r="G16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$99,$A16,Matriz!$L$2:$L$99,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$100,$A16,Matriz!$L$2:$L$100,"Hecho")</f>
         <v/>
       </c>
       <c r="H16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$99,$A16,Matriz!$L$2:$L$99,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$100,$A16,Matriz!$L$2:$L$100,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I16" s="13">
@@ -1295,31 +1295,31 @@
         </is>
       </c>
       <c r="B17" s="12">
-        <f>COUNTIF(Matriz!$H$2:$H$99,$A17)</f>
+        <f>COUNTIF(Matriz!$H$2:$H$100,$A17)</f>
         <v/>
       </c>
       <c r="C17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$99,$A17,Matriz!$L$2:$L$99,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$100,$A17,Matriz!$L$2:$L$100,"Pendiente")</f>
         <v/>
       </c>
       <c r="D17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$99,$A17,Matriz!$L$2:$L$99,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$100,$A17,Matriz!$L$2:$L$100,"En diseño")</f>
         <v/>
       </c>
       <c r="E17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$99,$A17,Matriz!$L$2:$L$99,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$100,$A17,Matriz!$L$2:$L$100,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$99,$A17,Matriz!$L$2:$L$99,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$100,$A17,Matriz!$L$2:$L$100,"En pruebas")</f>
         <v/>
       </c>
       <c r="G17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$99,$A17,Matriz!$L$2:$L$99,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$100,$A17,Matriz!$L$2:$L$100,"Hecho")</f>
         <v/>
       </c>
       <c r="H17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$99,$A17,Matriz!$L$2:$L$99,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$100,$A17,Matriz!$L$2:$L$100,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I17" s="13">
@@ -1334,31 +1334,31 @@
         </is>
       </c>
       <c r="B18" s="12">
-        <f>COUNTIF(Matriz!$H$2:$H$99,$A18)</f>
+        <f>COUNTIF(Matriz!$H$2:$H$100,$A18)</f>
         <v/>
       </c>
       <c r="C18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$99,$A18,Matriz!$L$2:$L$99,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$100,$A18,Matriz!$L$2:$L$100,"Pendiente")</f>
         <v/>
       </c>
       <c r="D18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$99,$A18,Matriz!$L$2:$L$99,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$100,$A18,Matriz!$L$2:$L$100,"En diseño")</f>
         <v/>
       </c>
       <c r="E18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$99,$A18,Matriz!$L$2:$L$99,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$100,$A18,Matriz!$L$2:$L$100,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$99,$A18,Matriz!$L$2:$L$99,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$100,$A18,Matriz!$L$2:$L$100,"En pruebas")</f>
         <v/>
       </c>
       <c r="G18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$99,$A18,Matriz!$L$2:$L$99,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$100,$A18,Matriz!$L$2:$L$100,"Hecho")</f>
         <v/>
       </c>
       <c r="H18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$99,$A18,Matriz!$L$2:$L$99,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$100,$A18,Matriz!$L$2:$L$100,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I18" s="13">
@@ -1373,31 +1373,31 @@
         </is>
       </c>
       <c r="B19" s="12">
-        <f>COUNTIF(Matriz!$H$2:$H$99,$A19)</f>
+        <f>COUNTIF(Matriz!$H$2:$H$100,$A19)</f>
         <v/>
       </c>
       <c r="C19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$99,$A19,Matriz!$L$2:$L$99,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$100,$A19,Matriz!$L$2:$L$100,"Pendiente")</f>
         <v/>
       </c>
       <c r="D19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$99,$A19,Matriz!$L$2:$L$99,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$100,$A19,Matriz!$L$2:$L$100,"En diseño")</f>
         <v/>
       </c>
       <c r="E19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$99,$A19,Matriz!$L$2:$L$99,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$100,$A19,Matriz!$L$2:$L$100,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$99,$A19,Matriz!$L$2:$L$99,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$100,$A19,Matriz!$L$2:$L$100,"En pruebas")</f>
         <v/>
       </c>
       <c r="G19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$99,$A19,Matriz!$L$2:$L$99,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$100,$A19,Matriz!$L$2:$L$100,"Hecho")</f>
         <v/>
       </c>
       <c r="H19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$99,$A19,Matriz!$L$2:$L$99,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$100,$A19,Matriz!$L$2:$L$100,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I19" s="13">
@@ -1498,31 +1498,31 @@
         </is>
       </c>
       <c r="B24" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$99,$A24)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$100,$A24)</f>
         <v/>
       </c>
       <c r="C24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$99,$A24,Matriz!$L$2:$L$99,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$100,$A24,Matriz!$L$2:$L$100,"Pendiente")</f>
         <v/>
       </c>
       <c r="D24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$99,$A24,Matriz!$L$2:$L$99,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$100,$A24,Matriz!$L$2:$L$100,"En diseño")</f>
         <v/>
       </c>
       <c r="E24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$99,$A24,Matriz!$L$2:$L$99,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$100,$A24,Matriz!$L$2:$L$100,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$99,$A24,Matriz!$L$2:$L$99,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$100,$A24,Matriz!$L$2:$L$100,"En pruebas")</f>
         <v/>
       </c>
       <c r="G24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$99,$A24,Matriz!$L$2:$L$99,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$100,$A24,Matriz!$L$2:$L$100,"Hecho")</f>
         <v/>
       </c>
       <c r="H24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$99,$A24,Matriz!$L$2:$L$99,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$100,$A24,Matriz!$L$2:$L$100,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I24" s="13">
@@ -1537,31 +1537,31 @@
         </is>
       </c>
       <c r="B25" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$99,$A25)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$100,$A25)</f>
         <v/>
       </c>
       <c r="C25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$99,$A25,Matriz!$L$2:$L$99,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$100,$A25,Matriz!$L$2:$L$100,"Pendiente")</f>
         <v/>
       </c>
       <c r="D25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$99,$A25,Matriz!$L$2:$L$99,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$100,$A25,Matriz!$L$2:$L$100,"En diseño")</f>
         <v/>
       </c>
       <c r="E25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$99,$A25,Matriz!$L$2:$L$99,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$100,$A25,Matriz!$L$2:$L$100,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$99,$A25,Matriz!$L$2:$L$99,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$100,$A25,Matriz!$L$2:$L$100,"En pruebas")</f>
         <v/>
       </c>
       <c r="G25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$99,$A25,Matriz!$L$2:$L$99,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$100,$A25,Matriz!$L$2:$L$100,"Hecho")</f>
         <v/>
       </c>
       <c r="H25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$99,$A25,Matriz!$L$2:$L$99,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$100,$A25,Matriz!$L$2:$L$100,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I25" s="13">
@@ -1576,31 +1576,31 @@
         </is>
       </c>
       <c r="B26" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$99,$A26)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$100,$A26)</f>
         <v/>
       </c>
       <c r="C26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$99,$A26,Matriz!$L$2:$L$99,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$100,$A26,Matriz!$L$2:$L$100,"Pendiente")</f>
         <v/>
       </c>
       <c r="D26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$99,$A26,Matriz!$L$2:$L$99,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$100,$A26,Matriz!$L$2:$L$100,"En diseño")</f>
         <v/>
       </c>
       <c r="E26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$99,$A26,Matriz!$L$2:$L$99,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$100,$A26,Matriz!$L$2:$L$100,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$99,$A26,Matriz!$L$2:$L$99,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$100,$A26,Matriz!$L$2:$L$100,"En pruebas")</f>
         <v/>
       </c>
       <c r="G26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$99,$A26,Matriz!$L$2:$L$99,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$100,$A26,Matriz!$L$2:$L$100,"Hecho")</f>
         <v/>
       </c>
       <c r="H26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$99,$A26,Matriz!$L$2:$L$99,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$100,$A26,Matriz!$L$2:$L$100,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I26" s="13">
@@ -1615,31 +1615,31 @@
         </is>
       </c>
       <c r="B27" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$99,$A27)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$100,$A27)</f>
         <v/>
       </c>
       <c r="C27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$99,$A27,Matriz!$L$2:$L$99,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$100,$A27,Matriz!$L$2:$L$100,"Pendiente")</f>
         <v/>
       </c>
       <c r="D27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$99,$A27,Matriz!$L$2:$L$99,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$100,$A27,Matriz!$L$2:$L$100,"En diseño")</f>
         <v/>
       </c>
       <c r="E27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$99,$A27,Matriz!$L$2:$L$99,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$100,$A27,Matriz!$L$2:$L$100,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$99,$A27,Matriz!$L$2:$L$99,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$100,$A27,Matriz!$L$2:$L$100,"En pruebas")</f>
         <v/>
       </c>
       <c r="G27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$99,$A27,Matriz!$L$2:$L$99,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$100,$A27,Matriz!$L$2:$L$100,"Hecho")</f>
         <v/>
       </c>
       <c r="H27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$99,$A27,Matriz!$L$2:$L$99,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$100,$A27,Matriz!$L$2:$L$100,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I27" s="13">
@@ -1654,31 +1654,31 @@
         </is>
       </c>
       <c r="B28" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$99,$A28)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$100,$A28)</f>
         <v/>
       </c>
       <c r="C28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$99,$A28,Matriz!$L$2:$L$99,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$100,$A28,Matriz!$L$2:$L$100,"Pendiente")</f>
         <v/>
       </c>
       <c r="D28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$99,$A28,Matriz!$L$2:$L$99,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$100,$A28,Matriz!$L$2:$L$100,"En diseño")</f>
         <v/>
       </c>
       <c r="E28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$99,$A28,Matriz!$L$2:$L$99,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$100,$A28,Matriz!$L$2:$L$100,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$99,$A28,Matriz!$L$2:$L$99,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$100,$A28,Matriz!$L$2:$L$100,"En pruebas")</f>
         <v/>
       </c>
       <c r="G28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$99,$A28,Matriz!$L$2:$L$99,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$100,$A28,Matriz!$L$2:$L$100,"Hecho")</f>
         <v/>
       </c>
       <c r="H28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$99,$A28,Matriz!$L$2:$L$99,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$100,$A28,Matriz!$L$2:$L$100,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I28" s="13">
@@ -1693,31 +1693,31 @@
         </is>
       </c>
       <c r="B29" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$99,$A29)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$100,$A29)</f>
         <v/>
       </c>
       <c r="C29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$99,$A29,Matriz!$L$2:$L$99,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$100,$A29,Matriz!$L$2:$L$100,"Pendiente")</f>
         <v/>
       </c>
       <c r="D29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$99,$A29,Matriz!$L$2:$L$99,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$100,$A29,Matriz!$L$2:$L$100,"En diseño")</f>
         <v/>
       </c>
       <c r="E29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$99,$A29,Matriz!$L$2:$L$99,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$100,$A29,Matriz!$L$2:$L$100,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$99,$A29,Matriz!$L$2:$L$99,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$100,$A29,Matriz!$L$2:$L$100,"En pruebas")</f>
         <v/>
       </c>
       <c r="G29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$99,$A29,Matriz!$L$2:$L$99,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$100,$A29,Matriz!$L$2:$L$100,"Hecho")</f>
         <v/>
       </c>
       <c r="H29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$99,$A29,Matriz!$L$2:$L$99,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$100,$A29,Matriz!$L$2:$L$100,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I29" s="13">
@@ -1732,31 +1732,31 @@
         </is>
       </c>
       <c r="B30" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$99,$A30)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$100,$A30)</f>
         <v/>
       </c>
       <c r="C30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$99,$A30,Matriz!$L$2:$L$99,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$100,$A30,Matriz!$L$2:$L$100,"Pendiente")</f>
         <v/>
       </c>
       <c r="D30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$99,$A30,Matriz!$L$2:$L$99,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$100,$A30,Matriz!$L$2:$L$100,"En diseño")</f>
         <v/>
       </c>
       <c r="E30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$99,$A30,Matriz!$L$2:$L$99,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$100,$A30,Matriz!$L$2:$L$100,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$99,$A30,Matriz!$L$2:$L$99,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$100,$A30,Matriz!$L$2:$L$100,"En pruebas")</f>
         <v/>
       </c>
       <c r="G30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$99,$A30,Matriz!$L$2:$L$99,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$100,$A30,Matriz!$L$2:$L$100,"Hecho")</f>
         <v/>
       </c>
       <c r="H30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$99,$A30,Matriz!$L$2:$L$99,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$100,$A30,Matriz!$L$2:$L$100,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I30" s="13">
@@ -1818,7 +1818,7 @@
         </is>
       </c>
       <c r="B35" s="12">
-        <f>COUNTIF(Matriz!$K$2:$K$99,A35)</f>
+        <f>COUNTIF(Matriz!$K$2:$K$100,A35)</f>
         <v/>
       </c>
     </row>
@@ -1829,7 +1829,7 @@
         </is>
       </c>
       <c r="B36" s="12">
-        <f>COUNTIF(Matriz!$K$2:$K$99,A36)</f>
+        <f>COUNTIF(Matriz!$K$2:$K$100,A36)</f>
         <v/>
       </c>
     </row>
@@ -1840,7 +1840,7 @@
         </is>
       </c>
       <c r="B37" s="12">
-        <f>COUNTIF(Matriz!$K$2:$K$99,A37)</f>
+        <f>COUNTIF(Matriz!$K$2:$K$100,A37)</f>
         <v/>
       </c>
     </row>
@@ -1851,7 +1851,7 @@
         </is>
       </c>
       <c r="B38" s="12">
-        <f>COUNTIF(Matriz!$K$2:$K$99,A38)</f>
+        <f>COUNTIF(Matriz!$K$2:$K$100,A38)</f>
         <v/>
       </c>
     </row>
@@ -1866,7 +1866,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N99"/>
+  <dimension ref="A1:N100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2924,12 +2924,12 @@
       </c>
       <c r="M16" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/m1-07-roles · 67 pruebas de backend y 6 de frontend pasan</t>
+          <t>Rama feature/paso-6-roles-permisos · pruebas de backend y 97 de frontend pasan; lint, estilos y compilación limpios</t>
         </is>
       </c>
       <c r="N16" s="19" t="inlineStr">
         <is>
-          <t>2026-10-10 · 9 roles sembrados según la matriz aprobada; asignación desde la pantalla Roles.</t>
+          <t>2026-10-29 · Roles base más la Secretaria; asignación con jerarquía (nadie otorga un rol más alto que el suyo, solo el Super Usuario asigna Super Usuario); baja y traslado solo por un superior.</t>
         </is>
       </c>
     </row>
@@ -3936,52 +3936,52 @@
     <row r="31">
       <c r="A31" s="18" t="inlineStr">
         <is>
-          <t>M2A-01</t>
+          <t>M1-24</t>
         </is>
       </c>
       <c r="B31" s="19" t="inlineStr">
         <is>
-          <t>M2A Cursos de Vida</t>
+          <t>M1 Identidad y comunicación</t>
         </is>
       </c>
       <c r="C31" s="19" t="inlineStr">
         <is>
-          <t>Catálogo dinámico de cursos; se pueden crear nuevos sin intervención técnica. Incluye «Resolución de Varones» y «Toma de Buenas Decisiones», omitidos en v2.</t>
-        </is>
-      </c>
-      <c r="D31" s="22" t="inlineStr">
-        <is>
-          <t>Recuperado v1</t>
+          <t>Administrador de roles y permisos: se crean roles y, por módulo, pantalla y acción, se elige lo que cada uno puede hacer. El Super Usuario, el Pastor y la Secretaria lo administran; nadie está por encima del Super Usuario y solo él asigna ese rol. Nadie concede un permiso que no tiene ni crea o cambia un rol de su nivel o superior. Un rol en uso no se desactiva y todo cambio queda en bitácora.</t>
+        </is>
+      </c>
+      <c r="D31" s="21" t="inlineStr">
+        <is>
+          <t>Respuesta v3.19</t>
         </is>
       </c>
       <c r="E31" s="19" t="inlineStr">
         <is>
-          <t>Fuera del MVP</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="F31" s="19" t="inlineStr">
         <is>
-          <t>Fase 3</t>
+          <t>Fase 0</t>
         </is>
       </c>
       <c r="G31" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sprint 5</t>
         </is>
       </c>
       <c r="H31" s="19" t="inlineStr">
         <is>
-          <t>Posterior</t>
-        </is>
-      </c>
-      <c r="I31" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
-        </is>
-      </c>
-      <c r="J31" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
+          <t>H2 · Fase 0 completa</t>
+        </is>
+      </c>
+      <c r="I31" s="19" t="inlineStr">
+        <is>
+          <t>Como administrador quiero crear roles y elegir, por módulo, pantalla y acción, lo que puede hacer cada uno, para que los permisos no se hagan bolas.</t>
+        </is>
+      </c>
+      <c r="J31" s="19" t="inlineStr">
+        <is>
+          <t>Crear un rol con permisos, no poder conceder los que no se tienen ni editar un rol de nivel igual o superior, y ver en la bitácora quién cambió qué.</t>
         </is>
       </c>
       <c r="K31" s="19" t="inlineStr">
@@ -3991,16 +3991,24 @@
       </c>
       <c r="L31" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M31" s="19" t="inlineStr"/>
-      <c r="N31" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M31" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/paso-6-roles-permisos · pruebas de backend y 97 de frontend pasan; lint, estilos y compilación limpios</t>
+        </is>
+      </c>
+      <c r="N31" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-29 · Catálogo de permisos, pantalla de roles con matriz, duplicado y desactivación, rol Secretaria y vista de lo que puede hacer cada persona. Falta: roles de unidad con alcance (siguiente entrega).</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="18" t="inlineStr">
         <is>
-          <t>M2A-02</t>
+          <t>M2A-01</t>
         </is>
       </c>
       <c r="B32" s="19" t="inlineStr">
@@ -4010,12 +4018,12 @@
       </c>
       <c r="C32" s="19" t="inlineStr">
         <is>
-          <t>Flexibilidad operativa: sin día ni horario fijo; el día y el ponente pueden cambiar entre ediciones.</t>
-        </is>
-      </c>
-      <c r="D32" s="19" t="inlineStr">
-        <is>
-          <t>v1 / v2</t>
+          <t>Catálogo dinámico de cursos; se pueden crear nuevos sin intervención técnica. Incluye «Resolución de Varones» y «Toma de Buenas Decisiones», omitidos en v2.</t>
+        </is>
+      </c>
+      <c r="D32" s="22" t="inlineStr">
+        <is>
+          <t>Recuperado v1</t>
         </is>
       </c>
       <c r="E32" s="19" t="inlineStr">
@@ -4064,7 +4072,7 @@
     <row r="33">
       <c r="A33" s="18" t="inlineStr">
         <is>
-          <t>M2A-03</t>
+          <t>M2A-02</t>
         </is>
       </c>
       <c r="B33" s="19" t="inlineStr">
@@ -4074,7 +4082,7 @@
       </c>
       <c r="C33" s="19" t="inlineStr">
         <is>
-          <t>Reposición de clases: el inscrito puede reponer en otro grupo o con otro ponente, a decisión de quien imparte.</t>
+          <t>Flexibilidad operativa: sin día ni horario fijo; el día y el ponente pueden cambiar entre ediciones.</t>
         </is>
       </c>
       <c r="D33" s="19" t="inlineStr">
@@ -4128,7 +4136,7 @@
     <row r="34">
       <c r="A34" s="18" t="inlineStr">
         <is>
-          <t>M2A-04</t>
+          <t>M2A-03</t>
         </is>
       </c>
       <c r="B34" s="19" t="inlineStr">
@@ -4138,7 +4146,7 @@
       </c>
       <c r="C34" s="19" t="inlineStr">
         <is>
-          <t>Registro de asistencia por sesión.</t>
+          <t>Reposición de clases: el inscrito puede reponer en otro grupo o con otro ponente, a decisión de quien imparte.</t>
         </is>
       </c>
       <c r="D34" s="19" t="inlineStr">
@@ -4192,7 +4200,7 @@
     <row r="35">
       <c r="A35" s="18" t="inlineStr">
         <is>
-          <t>M2A-05</t>
+          <t>M2A-04</t>
         </is>
       </c>
       <c r="B35" s="19" t="inlineStr">
@@ -4202,7 +4210,7 @@
       </c>
       <c r="C35" s="19" t="inlineStr">
         <is>
-          <t>Seguimiento de tareas o actividades opcionales (no sumativas).</t>
+          <t>Registro de asistencia por sesión.</t>
         </is>
       </c>
       <c r="D35" s="19" t="inlineStr">
@@ -4256,7 +4264,7 @@
     <row r="36">
       <c r="A36" s="18" t="inlineStr">
         <is>
-          <t>M2A-06</t>
+          <t>M2A-05</t>
         </is>
       </c>
       <c r="B36" s="19" t="inlineStr">
@@ -4266,7 +4274,7 @@
       </c>
       <c r="C36" s="19" t="inlineStr">
         <is>
-          <t>Inscripción: quién se inscribe, cuándo lo hizo, si tiene adeudo y qué incluye el costo (materiales, hospedaje, etc.).</t>
+          <t>Seguimiento de tareas o actividades opcionales (no sumativas).</t>
         </is>
       </c>
       <c r="D36" s="19" t="inlineStr">
@@ -4320,7 +4328,7 @@
     <row r="37">
       <c r="A37" s="18" t="inlineStr">
         <is>
-          <t>M2A-07</t>
+          <t>M2A-06</t>
         </is>
       </c>
       <c r="B37" s="19" t="inlineStr">
@@ -4330,12 +4338,12 @@
       </c>
       <c r="C37" s="19" t="inlineStr">
         <is>
-          <t>Registro de pagos, saldo de adeudos y recibo. Por definir: captura manual vs. pasarela de pago, y si se requiere corte de caja.</t>
-        </is>
-      </c>
-      <c r="D37" s="21" t="inlineStr">
-        <is>
-          <t>Nuevo v3</t>
+          <t>Inscripción: quién se inscribe, cuándo lo hizo, si tiene adeudo y qué incluye el costo (materiales, hospedaje, etc.).</t>
+        </is>
+      </c>
+      <c r="D37" s="19" t="inlineStr">
+        <is>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E37" s="19" t="inlineStr">
@@ -4370,7 +4378,7 @@
       </c>
       <c r="K37" s="19" t="inlineStr">
         <is>
-          <t>Por definir</t>
+          <t>VoBo pendiente</t>
         </is>
       </c>
       <c r="L37" s="19" t="inlineStr">
@@ -4384,7 +4392,7 @@
     <row r="38">
       <c r="A38" s="18" t="inlineStr">
         <is>
-          <t>M2A-08</t>
+          <t>M2A-07</t>
         </is>
       </c>
       <c r="B38" s="19" t="inlineStr">
@@ -4394,12 +4402,12 @@
       </c>
       <c r="C38" s="19" t="inlineStr">
         <is>
-          <t>Tablero del curso tipo mensajería para avisos antes del curso y días posteriores, con notificación a los inscritos.</t>
-        </is>
-      </c>
-      <c r="D38" s="22" t="inlineStr">
-        <is>
-          <t>Recuperado v1</t>
+          <t>Registro de pagos, saldo de adeudos y recibo. Por definir: captura manual vs. pasarela de pago, y si se requiere corte de caja.</t>
+        </is>
+      </c>
+      <c r="D38" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3</t>
         </is>
       </c>
       <c r="E38" s="19" t="inlineStr">
@@ -4434,7 +4442,7 @@
       </c>
       <c r="K38" s="19" t="inlineStr">
         <is>
-          <t>VoBo pendiente</t>
+          <t>Por definir</t>
         </is>
       </c>
       <c r="L38" s="19" t="inlineStr">
@@ -4448,7 +4456,7 @@
     <row r="39">
       <c r="A39" s="18" t="inlineStr">
         <is>
-          <t>M2A-09</t>
+          <t>M2A-08</t>
         </is>
       </c>
       <c r="B39" s="19" t="inlineStr">
@@ -4458,12 +4466,12 @@
       </c>
       <c r="C39" s="19" t="inlineStr">
         <is>
-          <t>Evaluación docente configurable: formulario diseñable (tipo Google Forms) aplicado al finalizar el curso.</t>
-        </is>
-      </c>
-      <c r="D39" s="19" t="inlineStr">
-        <is>
-          <t>v1 / v2</t>
+          <t>Tablero del curso tipo mensajería para avisos antes del curso y días posteriores, con notificación a los inscritos.</t>
+        </is>
+      </c>
+      <c r="D39" s="22" t="inlineStr">
+        <is>
+          <t>Recuperado v1</t>
         </is>
       </c>
       <c r="E39" s="19" t="inlineStr">
@@ -4512,7 +4520,7 @@
     <row r="40">
       <c r="A40" s="18" t="inlineStr">
         <is>
-          <t>M2A-10</t>
+          <t>M2A-09</t>
         </is>
       </c>
       <c r="B40" s="19" t="inlineStr">
@@ -4522,12 +4530,12 @@
       </c>
       <c r="C40" s="19" t="inlineStr">
         <is>
-          <t>Evolución del ponente: historial de evaluaciones por ponente a lo largo del tiempo y entre ediciones.</t>
-        </is>
-      </c>
-      <c r="D40" s="22" t="inlineStr">
-        <is>
-          <t>Recuperado v1</t>
+          <t>Evaluación docente configurable: formulario diseñable (tipo Google Forms) aplicado al finalizar el curso.</t>
+        </is>
+      </c>
+      <c r="D40" s="19" t="inlineStr">
+        <is>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E40" s="19" t="inlineStr">
@@ -4576,7 +4584,7 @@
     <row r="41">
       <c r="A41" s="18" t="inlineStr">
         <is>
-          <t>M2A-11</t>
+          <t>M2A-10</t>
         </is>
       </c>
       <c r="B41" s="19" t="inlineStr">
@@ -4586,12 +4594,12 @@
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>Reconocimiento de participación (diploma) opcional por curso.</t>
-        </is>
-      </c>
-      <c r="D41" s="19" t="inlineStr">
-        <is>
-          <t>v1 / v2</t>
+          <t>Evolución del ponente: historial de evaluaciones por ponente a lo largo del tiempo y entre ediciones.</t>
+        </is>
+      </c>
+      <c r="D41" s="22" t="inlineStr">
+        <is>
+          <t>Recuperado v1</t>
         </is>
       </c>
       <c r="E41" s="19" t="inlineStr">
@@ -4640,17 +4648,17 @@
     <row r="42">
       <c r="A42" s="18" t="inlineStr">
         <is>
-          <t>M2B-01</t>
+          <t>M2A-11</t>
         </is>
       </c>
       <c r="B42" s="19" t="inlineStr">
         <is>
-          <t>M2B Cursos escolarizados</t>
+          <t>M2A Cursos de Vida</t>
         </is>
       </c>
       <c r="C42" s="19" t="inlineStr">
         <is>
-          <t>Control riguroso de asistencia.</t>
+          <t>Reconocimiento de participación (diploma) opcional por curso.</t>
         </is>
       </c>
       <c r="D42" s="19" t="inlineStr">
@@ -4704,7 +4712,7 @@
     <row r="43">
       <c r="A43" s="18" t="inlineStr">
         <is>
-          <t>M2B-02</t>
+          <t>M2B-01</t>
         </is>
       </c>
       <c r="B43" s="19" t="inlineStr">
@@ -4714,7 +4722,7 @@
       </c>
       <c r="C43" s="19" t="inlineStr">
         <is>
-          <t>Entrega de tareas y trabajos continuos (incluidos trabajos extra).</t>
+          <t>Control riguroso de asistencia.</t>
         </is>
       </c>
       <c r="D43" s="19" t="inlineStr">
@@ -4768,7 +4776,7 @@
     <row r="44">
       <c r="A44" s="18" t="inlineStr">
         <is>
-          <t>M2B-03</t>
+          <t>M2B-02</t>
         </is>
       </c>
       <c r="B44" s="19" t="inlineStr">
@@ -4778,7 +4786,7 @@
       </c>
       <c r="C44" s="19" t="inlineStr">
         <is>
-          <t>Ponderación de calificaciones y exámenes finales.</t>
+          <t>Entrega de tareas y trabajos continuos (incluidos trabajos extra).</t>
         </is>
       </c>
       <c r="D44" s="19" t="inlineStr">
@@ -4832,7 +4840,7 @@
     <row r="45">
       <c r="A45" s="18" t="inlineStr">
         <is>
-          <t>M2B-04</t>
+          <t>M2B-03</t>
         </is>
       </c>
       <c r="B45" s="19" t="inlineStr">
@@ -4842,12 +4850,12 @@
       </c>
       <c r="C45" s="19" t="inlineStr">
         <is>
-          <t>Creador de exámenes en línea: opción múltiple, preguntas abiertas, falso/verdadero y respuesta corta.</t>
+          <t>Ponderación de calificaciones y exámenes finales.</t>
         </is>
       </c>
       <c r="D45" s="19" t="inlineStr">
         <is>
-          <t>v2</t>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E45" s="19" t="inlineStr">
@@ -4896,7 +4904,7 @@
     <row r="46">
       <c r="A46" s="18" t="inlineStr">
         <is>
-          <t>M2B-05</t>
+          <t>M2B-04</t>
         </is>
       </c>
       <c r="B46" s="19" t="inlineStr">
@@ -4906,12 +4914,12 @@
       </c>
       <c r="C46" s="19" t="inlineStr">
         <is>
-          <t>Boleta digital con el formato definido por la iglesia. Por definir: formato oficial de la boleta.</t>
+          <t>Creador de exámenes en línea: opción múltiple, preguntas abiertas, falso/verdadero y respuesta corta.</t>
         </is>
       </c>
       <c r="D46" s="19" t="inlineStr">
         <is>
-          <t>v1 / v2</t>
+          <t>v2</t>
         </is>
       </c>
       <c r="E46" s="19" t="inlineStr">
@@ -4946,7 +4954,7 @@
       </c>
       <c r="K46" s="19" t="inlineStr">
         <is>
-          <t>Por definir</t>
+          <t>VoBo pendiente</t>
         </is>
       </c>
       <c r="L46" s="19" t="inlineStr">
@@ -4960,7 +4968,7 @@
     <row r="47">
       <c r="A47" s="18" t="inlineStr">
         <is>
-          <t>M2B-06</t>
+          <t>M2B-05</t>
         </is>
       </c>
       <c r="B47" s="19" t="inlineStr">
@@ -4970,12 +4978,12 @@
       </c>
       <c r="C47" s="19" t="inlineStr">
         <is>
-          <t>Historial académico permanente en el Expediente Digital, aunque cambie el maestro o el alumno pierda su comprobante.</t>
+          <t>Boleta digital con el formato definido por la iglesia. Por definir: formato oficial de la boleta.</t>
         </is>
       </c>
       <c r="D47" s="19" t="inlineStr">
         <is>
-          <t>v2</t>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E47" s="19" t="inlineStr">
@@ -5010,7 +5018,7 @@
       </c>
       <c r="K47" s="19" t="inlineStr">
         <is>
-          <t>VoBo pendiente</t>
+          <t>Por definir</t>
         </is>
       </c>
       <c r="L47" s="19" t="inlineStr">
@@ -5024,52 +5032,52 @@
     <row r="48">
       <c r="A48" s="18" t="inlineStr">
         <is>
-          <t>M3-01</t>
+          <t>M2B-06</t>
         </is>
       </c>
       <c r="B48" s="19" t="inlineStr">
         <is>
-          <t>M3 Grupos de Conexión</t>
+          <t>M2B Cursos escolarizados</t>
         </is>
       </c>
       <c r="C48" s="19" t="inlineStr">
         <is>
-          <t>Estructura del grupo con roles: Supervisor (supervisa uno o varios grupos y reporta al Pastor), Líder, Secretario, Anfitrión y Tesorero.</t>
+          <t>Historial académico permanente en el Expediente Digital, aunque cambie el maestro o el alumno pierda su comprobante.</t>
         </is>
       </c>
       <c r="D48" s="19" t="inlineStr">
         <is>
-          <t>v3 + Obs. 4</t>
+          <t>v2</t>
         </is>
       </c>
       <c r="E48" s="19" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Fuera del MVP</t>
         </is>
       </c>
       <c r="F48" s="19" t="inlineStr">
         <is>
-          <t>Fase 1</t>
+          <t>Fase 3</t>
         </is>
       </c>
       <c r="G48" s="19" t="inlineStr">
         <is>
-          <t>Sprint 3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H48" s="19" t="inlineStr">
         <is>
-          <t>H3 · MVP (Grupos)</t>
-        </is>
-      </c>
-      <c r="I48" s="19" t="inlineStr">
-        <is>
-          <t>Como supervisor quiero asignar Líder, Secretario, Anfitrión y Tesorero a cada grupo.</t>
-        </is>
-      </c>
-      <c r="J48" s="19" t="inlineStr">
-        <is>
-          <t>Un grupo tiene sus roles asignados; un supervisor ve varios grupos.</t>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="I48" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
+        </is>
+      </c>
+      <c r="J48" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
         </is>
       </c>
       <c r="K48" s="19" t="inlineStr">
@@ -5079,24 +5087,16 @@
       </c>
       <c r="L48" s="19" t="inlineStr">
         <is>
-          <t>En pruebas</t>
-        </is>
-      </c>
-      <c r="M48" s="19" t="inlineStr">
-        <is>
-          <t>Rama feature/grupos-paso-3 · pruebas de backend y 81 de frontend pasan; lint, estilos y compilación limpios</t>
-        </is>
-      </c>
-      <c r="N48" s="19" t="inlineStr">
-        <is>
-          <t>2026-10-27 · Supervisor, Líder, Secretario, Anfitrión, Tesorero y Asistente por grupo; ahora con cambio de rol, sector (letra), casa (número) y suspensión con motivo.</t>
-        </is>
-      </c>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M48" s="19" t="inlineStr"/>
+      <c r="N48" s="19" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="18" t="inlineStr">
         <is>
-          <t>M3-02</t>
+          <t>M3-01</t>
         </is>
       </c>
       <c r="B49" s="19" t="inlineStr">
@@ -5106,12 +5106,12 @@
       </c>
       <c r="C49" s="19" t="inlineStr">
         <is>
-          <t>Estudio semanal dentro de la app: un registro por semana con PDF para adultos, PDF para niños y audio de la lectura (PDF hasta 15 MB; audio hasta 40 MB). Lo publican Pastor o Anciano y los líderes lo abren desde la reunión, sustituyendo el envío por WhatsApp. El audio admite adelantar y retroceder en iPhone.</t>
+          <t>Estructura del grupo con roles: Supervisor (supervisa uno o varios grupos y reporta al Pastor), Líder, Secretario, Anfitrión y Tesorero.</t>
         </is>
       </c>
       <c r="D49" s="19" t="inlineStr">
         <is>
-          <t>v1 / v2 + Respuesta</t>
+          <t>v3 + Obs. 4</t>
         </is>
       </c>
       <c r="E49" s="19" t="inlineStr">
@@ -5136,12 +5136,12 @@
       </c>
       <c r="I49" s="19" t="inlineStr">
         <is>
-          <t>Como líder quiero recibir el estudio semanal en la app en lugar de WhatsApp.</t>
+          <t>Como supervisor quiero asignar Líder, Secretario, Anfitrión y Tesorero a cada grupo.</t>
         </is>
       </c>
       <c r="J49" s="19" t="inlineStr">
         <is>
-          <t>Publicar el material de la semana; el líder lo abre y queda marca de lectura.</t>
+          <t>Un grupo tiene sus roles asignados; un supervisor ve varios grupos.</t>
         </is>
       </c>
       <c r="K49" s="19" t="inlineStr">
@@ -5156,19 +5156,19 @@
       </c>
       <c r="M49" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/m3-grupos · 88 pruebas de backend y 7 de frontend pasan</t>
+          <t>Rama feature/grupos-paso-3 · pruebas de backend y 81 de frontend pasan; lint, estilos y compilación limpios</t>
         </is>
       </c>
       <c r="N49" s="19" t="inlineStr">
         <is>
-          <t>2026-10-24 · PDF adultos, PDF niños y audio por semana; audio con Range para iPhone. Pendiente probar en iOS.</t>
+          <t>2026-10-27 · Supervisor, Líder, Secretario, Anfitrión, Tesorero y Asistente por grupo; ahora con cambio de rol, sector (letra), casa (número) y suspensión con motivo.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="18" t="inlineStr">
         <is>
-          <t>M3-03</t>
+          <t>M3-02</t>
         </is>
       </c>
       <c r="B50" s="19" t="inlineStr">
@@ -5178,12 +5178,12 @@
       </c>
       <c r="C50" s="19" t="inlineStr">
         <is>
-          <t>Pase de lista digital por Secretario o Líder. El Secretario captura y corrige el mismo día; el Líder modifica siempre; el Supervisor solo consulta. Funciona sin conexión: la lista se guarda en el teléfono con la hora real de captura y se envía sola al volver la señal, sin pisar cambios más recientes hechos en línea. Una captura sin conexión se acepta hasta 7 días después y se evalúa contra el día en que se hizo; todo queda en bitácora marcado como diferido.</t>
+          <t>Estudio semanal dentro de la app: un registro por semana con PDF para adultos, PDF para niños y audio de la lectura (PDF hasta 15 MB; audio hasta 40 MB). Lo publican Pastor o Anciano y los líderes lo abren desde la reunión, sustituyendo el envío por WhatsApp. El audio admite adelantar y retroceder en iPhone.</t>
         </is>
       </c>
       <c r="D50" s="19" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>v1 / v2 + Respuesta</t>
         </is>
       </c>
       <c r="E50" s="19" t="inlineStr">
@@ -5208,12 +5208,12 @@
       </c>
       <c r="I50" s="19" t="inlineStr">
         <is>
-          <t>Como secretario quiero pasar lista aunque no haya señal.</t>
+          <t>Como líder quiero recibir el estudio semanal en la app en lugar de WhatsApp.</t>
         </is>
       </c>
       <c r="J50" s="19" t="inlineStr">
         <is>
-          <t>Pasar lista en modo avión; al reconectar se sincroniza sin duplicados.</t>
+          <t>Publicar el material de la semana; el líder lo abre y queda marca de lectura.</t>
         </is>
       </c>
       <c r="K50" s="19" t="inlineStr">
@@ -5228,19 +5228,19 @@
       </c>
       <c r="M50" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/nf-06-sin-conexion · 117 pruebas de backend y 27 de frontend; probado en Chrome real con service worker</t>
+          <t>Rama feature/m3-grupos · 88 pruebas de backend y 7 de frontend pasan</t>
         </is>
       </c>
       <c r="N50" s="19" t="inlineStr">
         <is>
-          <t>2026-10-24 · Pase de lista con y sin conexión.</t>
+          <t>2026-10-24 · PDF adultos, PDF niños y audio por semana; audio con Range para iPhone. Pendiente probar en iOS.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="18" t="inlineStr">
         <is>
-          <t>M3-04</t>
+          <t>M3-03</t>
         </is>
       </c>
       <c r="B51" s="19" t="inlineStr">
@@ -5250,12 +5250,12 @@
       </c>
       <c r="C51" s="19" t="inlineStr">
         <is>
-          <t>Ofrendas regulares y especiales (con concepto) por reunión, cuantificables. El Secretario captura el monto; si el grupo no tiene Secretario, lo suple el Líder. El Tesorero cuenta, escribe su cifra y avala volviendo a escribir su PIN; si el grupo no tiene Tesorero, avalan el Líder o el Pastor, nunca quien capturó. Si la cifra coincide queda «Avalada»; si no, se registra la diferencia y queda «Con diferencia», con aviso visible en el grupo, la reunión y la pantalla del Tesorero para quien pueda consultar. Una ofrenda ya capturada solo se corrige con motivo y vuelve a pendiente para un nuevo aval. El Pastor consulta todo, el Líder y el Supervisor consultan y el Anciano no ve finanzas. Toda suplencia, captura, aval y corrección queda en bitácora.</t>
+          <t>Pase de lista digital por Secretario o Líder. El Secretario captura y corrige el mismo día; el Líder modifica siempre; el Supervisor solo consulta. Funciona sin conexión: la lista se guarda en el teléfono con la hora real de captura y se envía sola al volver la señal, sin pisar cambios más recientes hechos en línea. Una captura sin conexión se acepta hasta 7 días después y se evalúa contra el día en que se hizo; todo queda en bitácora marcado como diferido.</t>
         </is>
       </c>
       <c r="D51" s="19" t="inlineStr">
         <is>
-          <t>v3 + Obs. 4</t>
+          <t>v3</t>
         </is>
       </c>
       <c r="E51" s="19" t="inlineStr">
@@ -5270,7 +5270,7 @@
       </c>
       <c r="G51" s="19" t="inlineStr">
         <is>
-          <t>Sprint 4</t>
+          <t>Sprint 3</t>
         </is>
       </c>
       <c r="H51" s="19" t="inlineStr">
@@ -5280,12 +5280,12 @@
       </c>
       <c r="I51" s="19" t="inlineStr">
         <is>
-          <t>Como tesorero quiero contar y avalar la ofrenda del grupo.</t>
+          <t>Como secretario quiero pasar lista aunque no haya señal.</t>
         </is>
       </c>
       <c r="J51" s="19" t="inlineStr">
         <is>
-          <t>Capturar monto; el Tesorero captura su cifra y confirma con su PIN; si difiere se registra la diferencia; con aval no se edita sin motivo.</t>
+          <t>Pasar lista en modo avión; al reconectar se sincroniza sin duplicados.</t>
         </is>
       </c>
       <c r="K51" s="19" t="inlineStr">
@@ -5300,19 +5300,19 @@
       </c>
       <c r="M51" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/m3-ofrendas-ajustes · 121 pruebas de backend y 14 de frontend pasan</t>
+          <t>Rama feature/nf-06-sin-conexion · 117 pruebas de backend y 27 de frontend; probado en Chrome real con service worker</t>
         </is>
       </c>
       <c r="N51" s="19" t="inlineStr">
         <is>
-          <t>2026-10-24 · Con suplencias del Líder, diferencias visibles y límites configurables. Falta validar con la iglesia.</t>
+          <t>2026-10-24 · Pase de lista con y sin conexión.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="18" t="inlineStr">
         <is>
-          <t>M3-05</t>
+          <t>M3-04</t>
         </is>
       </c>
       <c r="B52" s="19" t="inlineStr">
@@ -5322,12 +5322,12 @@
       </c>
       <c r="C52" s="19" t="inlineStr">
         <is>
-          <t>Peticiones de oración con formulario configurable (campos que se agregan, desactivan y reordenan sin programar; cada cambio crea una versión y los campos no se borran). Por defecto: petición, quién la pide y categoría. Las registran el Líder y el Secretario, desde la reunión o desde el grupo; el Pastor también.</t>
+          <t>Ofrendas regulares y especiales (con concepto) por reunión, cuantificables. El Secretario captura el monto; si el grupo no tiene Secretario, lo suple el Líder. El Tesorero cuenta, escribe su cifra y avala volviendo a escribir su PIN; si el grupo no tiene Tesorero, avalan el Líder o el Pastor, nunca quien capturó. Si la cifra coincide queda «Avalada»; si no, se registra la diferencia y queda «Con diferencia», con aviso visible en el grupo, la reunión y la pantalla del Tesorero para quien pueda consultar. Una ofrenda ya capturada solo se corrige con motivo y vuelve a pendiente para un nuevo aval. El Pastor consulta todo, el Líder y el Supervisor consultan y el Anciano no ve finanzas. Toda suplencia, captura, aval y corrección queda en bitácora.</t>
         </is>
       </c>
       <c r="D52" s="19" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>v3 + Obs. 4</t>
         </is>
       </c>
       <c r="E52" s="19" t="inlineStr">
@@ -5352,12 +5352,12 @@
       </c>
       <c r="I52" s="19" t="inlineStr">
         <is>
-          <t>Como líder quiero recoger peticiones de oración con un formulario configurable.</t>
+          <t>Como tesorero quiero contar y avalar la ofrenda del grupo.</t>
         </is>
       </c>
       <c r="J52" s="19" t="inlineStr">
         <is>
-          <t>Capturar una petición; el formulario se edita sin código.</t>
+          <t>Capturar monto; el Tesorero captura su cifra y confirma con su PIN; si difiere se registra la diferencia; con aval no se edita sin motivo.</t>
         </is>
       </c>
       <c r="K52" s="19" t="inlineStr">
@@ -5372,19 +5372,19 @@
       </c>
       <c r="M52" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/m3-peticiones-oracion · 166 pruebas de backend y 32 de frontend pasan; probado contra la base real</t>
+          <t>Rama feature/m3-ofrendas-ajustes · 121 pruebas de backend y 14 de frontend pasan</t>
         </is>
       </c>
       <c r="N52" s="19" t="inlineStr">
         <is>
-          <t>2026-10-24 · Formulario configurable y versionado; captura desde la reunión y el grupo.</t>
+          <t>2026-10-24 · Con suplencias del Líder, diferencias visibles y límites configurables. Falta validar con la iglesia.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="18" t="inlineStr">
         <is>
-          <t>M3-06</t>
+          <t>M3-05</t>
         </is>
       </c>
       <c r="B53" s="19" t="inlineStr">
@@ -5394,12 +5394,12 @@
       </c>
       <c r="C53" s="19" t="inlineStr">
         <is>
-          <t>Alcance de lectura de cada petición, elegido por quien la registra con autorización de quien la pide: «Solo líderes» (Líder, Supervisor, Pastor y Anciano), «Mi grupo» (todos los integrantes del grupo y los anteriores) o «Equipo de oración» (además, quien tenga el rol Equipo de oración). El alcance por defecto es configurable. Quien registra siempre ve lo que registró; el Administrador Técnico nunca ve el contenido. Solo líderes y superiores marcan una petición como atendida. Se guardan cifradas y se borran automáticamente a los 30 días, configurable. Consultarlas y atenderlas queda en bitácora sin incluir el texto.</t>
-        </is>
-      </c>
-      <c r="D53" s="21" t="inlineStr">
-        <is>
-          <t>Resp. P8 + Respuesta</t>
+          <t>Peticiones de oración con formulario configurable (campos que se agregan, desactivan y reordenan sin programar; cada cambio crea una versión y los campos no se borran). Por defecto: petición, quién la pide y categoría. Las registran el Líder y el Secretario, desde la reunión o desde el grupo; el Pastor también.</t>
+        </is>
+      </c>
+      <c r="D53" s="19" t="inlineStr">
+        <is>
+          <t>v3</t>
         </is>
       </c>
       <c r="E53" s="19" t="inlineStr">
@@ -5424,12 +5424,12 @@
       </c>
       <c r="I53" s="19" t="inlineStr">
         <is>
-          <t>Como pastor quiero que las peticiones solo las vea el Líder y superiores y se borren al vencer.</t>
+          <t>Como líder quiero recoger peticiones de oración con un formulario configurable.</t>
         </is>
       </c>
       <c r="J53" s="19" t="inlineStr">
         <is>
-          <t>El Secretario no las ve; tras el plazo configurable (por defecto 30 días) se eliminan.</t>
+          <t>Capturar una petición; el formulario se edita sin código.</t>
         </is>
       </c>
       <c r="K53" s="19" t="inlineStr">
@@ -5449,14 +5449,14 @@
       </c>
       <c r="N53" s="19" t="inlineStr">
         <is>
-          <t>2026-10-24 · Alcance por petición (líderes, grupo, equipo), cifrado y borrado a los 30 días configurable. Cambia la matriz aprobada: actualizar con la iglesia.</t>
+          <t>2026-10-24 · Formulario configurable y versionado; captura desde la reunión y el grupo.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="18" t="inlineStr">
         <is>
-          <t>M3-07</t>
+          <t>M3-06</t>
         </is>
       </c>
       <c r="B54" s="19" t="inlineStr">
@@ -5466,17 +5466,17 @@
       </c>
       <c r="C54" s="19" t="inlineStr">
         <is>
-          <t>Dashboard de supervisión («Resumen de grupos») para Supervisor, Líder, Pastor y Anciano sobre los grupos que cada uno puede consultar: asistencia por semana y por grupo, grupos sin lista esta semana, asistencia por debajo de un mínimo configurable (60 % por defecto), ofrendas avaladas, pendientes y con diferencia (solo si el rol ve finanzas) y peticiones activas (solo las que puede leer). No muestra datos de personas. El Secretario y el Tesorero no lo ven.</t>
-        </is>
-      </c>
-      <c r="D54" s="19" t="inlineStr">
-        <is>
-          <t>v3</t>
+          <t>Alcance de lectura de cada petición, elegido por quien la registra con autorización de quien la pide: «Solo líderes» (Líder, Supervisor, Pastor y Anciano), «Mi grupo» (todos los integrantes del grupo y los anteriores) o «Equipo de oración» (además, quien tenga el rol Equipo de oración). El alcance por defecto es configurable. Quien registra siempre ve lo que registró; el Administrador Técnico nunca ve el contenido. Solo líderes y superiores marcan una petición como atendida. Se guardan cifradas y se borran automáticamente a los 30 días, configurable. Consultarlas y atenderlas queda en bitácora sin incluir el texto.</t>
+        </is>
+      </c>
+      <c r="D54" s="21" t="inlineStr">
+        <is>
+          <t>Resp. P8 + Respuesta</t>
         </is>
       </c>
       <c r="E54" s="19" t="inlineStr">
         <is>
-          <t>MVP básico</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="F54" s="19" t="inlineStr">
@@ -5486,7 +5486,7 @@
       </c>
       <c r="G54" s="19" t="inlineStr">
         <is>
-          <t>Sprint 5</t>
+          <t>Sprint 4</t>
         </is>
       </c>
       <c r="H54" s="19" t="inlineStr">
@@ -5496,12 +5496,12 @@
       </c>
       <c r="I54" s="19" t="inlineStr">
         <is>
-          <t>Como supervisor quiero ver la salud de mis grupos.</t>
+          <t>Como pastor quiero que las peticiones solo las vea el Líder y superiores y se borren al vencer.</t>
         </is>
       </c>
       <c r="J54" s="19" t="inlineStr">
         <is>
-          <t>El dashboard muestra asistencia, ofrendas y crecimiento según permisos.</t>
+          <t>El Secretario no las ve; tras el plazo configurable (por defecto 30 días) se eliminan.</t>
         </is>
       </c>
       <c r="K54" s="19" t="inlineStr">
@@ -5516,19 +5516,19 @@
       </c>
       <c r="M54" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/m3-dashboard-tablero · 195 pruebas de backend y 39 de frontend pasan; probado contra la base real</t>
+          <t>Rama feature/m3-peticiones-oracion · 166 pruebas de backend y 32 de frontend pasan; probado contra la base real</t>
         </is>
       </c>
       <c r="N54" s="19" t="inlineStr">
         <is>
-          <t>2026-10-25 · Dashboard con asistencia, avisos y datos según rol; umbral configurable.</t>
+          <t>2026-10-24 · Alcance por petición (líderes, grupo, equipo), cifrado y borrado a los 30 días configurable. Cambia la matriz aprobada: actualizar con la iglesia.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="18" t="inlineStr">
         <is>
-          <t>M3-08</t>
+          <t>M3-07</t>
         </is>
       </c>
       <c r="B55" s="19" t="inlineStr">
@@ -5538,7 +5538,7 @@
       </c>
       <c r="C55" s="19" t="inlineStr">
         <is>
-          <t>Ubicación de zona del grupo para que personas cercanas lo encuentren, sin exponer el domicilio exacto. Por definir.</t>
+          <t>Dashboard de supervisión («Resumen de grupos») para Supervisor, Líder, Pastor y Anciano sobre los grupos que cada uno puede consultar: asistencia por semana y por grupo, grupos sin lista esta semana, asistencia por debajo de un mínimo configurable (60 % por defecto), ofrendas avaladas, pendientes y con diferencia (solo si el rol ve finanzas) y peticiones activas (solo las que puede leer). No muestra datos de personas. El Secretario y el Tesorero no lo ven.</t>
         </is>
       </c>
       <c r="D55" s="19" t="inlineStr">
@@ -5548,51 +5548,59 @@
       </c>
       <c r="E55" s="19" t="inlineStr">
         <is>
-          <t>Fuera del MVP</t>
+          <t>MVP básico</t>
         </is>
       </c>
       <c r="F55" s="19" t="inlineStr">
         <is>
-          <t>Fase 4</t>
+          <t>Fase 1</t>
         </is>
       </c>
       <c r="G55" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sprint 5</t>
         </is>
       </c>
       <c r="H55" s="19" t="inlineStr">
         <is>
-          <t>Posterior</t>
-        </is>
-      </c>
-      <c r="I55" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
-        </is>
-      </c>
-      <c r="J55" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
+          <t>H3 · MVP (Grupos)</t>
+        </is>
+      </c>
+      <c r="I55" s="19" t="inlineStr">
+        <is>
+          <t>Como supervisor quiero ver la salud de mis grupos.</t>
+        </is>
+      </c>
+      <c r="J55" s="19" t="inlineStr">
+        <is>
+          <t>El dashboard muestra asistencia, ofrendas y crecimiento según permisos.</t>
         </is>
       </c>
       <c r="K55" s="19" t="inlineStr">
         <is>
-          <t>Por definir</t>
+          <t>VoBo pendiente</t>
         </is>
       </c>
       <c r="L55" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M55" s="19" t="inlineStr"/>
-      <c r="N55" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M55" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/m3-dashboard-tablero · 195 pruebas de backend y 39 de frontend pasan; probado contra la base real</t>
+        </is>
+      </c>
+      <c r="N55" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-25 · Dashboard con asistencia, avisos y datos según rol; umbral configurable.</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="18" t="inlineStr">
         <is>
-          <t>M3-09</t>
+          <t>M3-08</t>
         </is>
       </c>
       <c r="B56" s="19" t="inlineStr">
@@ -5602,69 +5610,61 @@
       </c>
       <c r="C56" s="19" t="inlineStr">
         <is>
-          <t>A un grupo asisten miembros de la iglesia (vecinos o no) e invitados del grupo que no asisten a la iglesia. Los invitados se registran como Contacto con datos mínimos y se les puede invitar a consolidación.</t>
-        </is>
-      </c>
-      <c r="D56" s="21" t="inlineStr">
-        <is>
-          <t>Corrección v3.2</t>
+          <t>Ubicación de zona del grupo para que personas cercanas lo encuentren, sin exponer el domicilio exacto. Por definir.</t>
+        </is>
+      </c>
+      <c r="D56" s="19" t="inlineStr">
+        <is>
+          <t>v3</t>
         </is>
       </c>
       <c r="E56" s="19" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Fuera del MVP</t>
         </is>
       </c>
       <c r="F56" s="19" t="inlineStr">
         <is>
-          <t>Fase 1</t>
+          <t>Fase 4</t>
         </is>
       </c>
       <c r="G56" s="19" t="inlineStr">
         <is>
-          <t>Sprint 3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H56" s="19" t="inlineStr">
         <is>
-          <t>H3 · MVP (Grupos)</t>
-        </is>
-      </c>
-      <c r="I56" s="19" t="inlineStr">
-        <is>
-          <t>Como secretario quiero registrar invitados del grupo con datos mínimos.</t>
-        </is>
-      </c>
-      <c r="J56" s="19" t="inlineStr">
-        <is>
-          <t>Registrar un invitado como Contacto y marcarlo presente.</t>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="I56" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
+        </is>
+      </c>
+      <c r="J56" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
         </is>
       </c>
       <c r="K56" s="19" t="inlineStr">
         <is>
-          <t>VoBo pendiente</t>
+          <t>Por definir</t>
         </is>
       </c>
       <c r="L56" s="19" t="inlineStr">
         <is>
-          <t>En pruebas</t>
-        </is>
-      </c>
-      <c r="M56" s="19" t="inlineStr">
-        <is>
-          <t>Rama feature/paso-5-invitaciones · pruebas de backend y 93 de frontend pasan; lint, estilos y compilación limpios</t>
-        </is>
-      </c>
-      <c r="N56" s="19" t="inlineStr">
-        <is>
-          <t>2026-10-27 · Los invitados entran al grupo como Contacto cuando el líder aprueba su solicitud por enlace o QR.</t>
-        </is>
-      </c>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M56" s="19" t="inlineStr"/>
+      <c r="N56" s="19" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="18" t="inlineStr">
         <is>
-          <t>M3-10</t>
+          <t>M3-09</t>
         </is>
       </c>
       <c r="B57" s="19" t="inlineStr">
@@ -5674,12 +5674,12 @@
       </c>
       <c r="C57" s="19" t="inlineStr">
         <is>
-          <t>Confidencialidad de ofrendas y asistencias: consulta limitada por rol (matriz por definir) y modificación restringida, todo en bitácora.</t>
+          <t>A un grupo asisten miembros de la iglesia (vecinos o no) e invitados del grupo que no asisten a la iglesia. Los invitados se registran como Contacto con datos mínimos y se les puede invitar a consolidación.</t>
         </is>
       </c>
       <c r="D57" s="21" t="inlineStr">
         <is>
-          <t>Obs. 5</t>
+          <t>Corrección v3.2</t>
         </is>
       </c>
       <c r="E57" s="19" t="inlineStr">
@@ -5694,7 +5694,7 @@
       </c>
       <c r="G57" s="19" t="inlineStr">
         <is>
-          <t>Sprint 4</t>
+          <t>Sprint 3</t>
         </is>
       </c>
       <c r="H57" s="19" t="inlineStr">
@@ -5704,31 +5704,39 @@
       </c>
       <c r="I57" s="19" t="inlineStr">
         <is>
-          <t>Como pastor quiero que ofrendas y asistencias sean confidenciales.</t>
+          <t>Como secretario quiero registrar invitados del grupo con datos mínimos.</t>
         </is>
       </c>
       <c r="J57" s="19" t="inlineStr">
         <is>
-          <t>La matriz de la sección 3.3 del v3.2 se cumple en pruebas por cada rol.</t>
+          <t>Registrar un invitado como Contacto y marcarlo presente.</t>
         </is>
       </c>
       <c r="K57" s="19" t="inlineStr">
         <is>
-          <t>Por definir</t>
+          <t>VoBo pendiente</t>
         </is>
       </c>
       <c r="L57" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M57" s="19" t="inlineStr"/>
-      <c r="N57" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M57" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/paso-5-invitaciones · pruebas de backend y 93 de frontend pasan; lint, estilos y compilación limpios</t>
+        </is>
+      </c>
+      <c r="N57" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-27 · Los invitados entran al grupo como Contacto cuando el líder aprueba su solicitud por enlace o QR.</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="18" t="inlineStr">
         <is>
-          <t>M3-11</t>
+          <t>M3-10</t>
         </is>
       </c>
       <c r="B58" s="19" t="inlineStr">
@@ -5738,12 +5746,12 @@
       </c>
       <c r="C58" s="19" t="inlineStr">
         <is>
-          <t>Tablero de mensajes del grupo: lo publican Líder, Supervisor, Secretario y Pastor; lo leen todos los integrantes activos. Mensajes de hasta 1,000 caracteres, con opción de fijarlos, borrado lógico, contador de mensajes nuevos y conservación configurable (90 días). Pantalla «Avisos» para quien no abre la página del grupo.</t>
+          <t>Confidencialidad de ofrendas y asistencias: consulta limitada por rol (matriz por definir) y modificación restringida, todo en bitácora.</t>
         </is>
       </c>
       <c r="D58" s="21" t="inlineStr">
         <is>
-          <t>Obs. 7</t>
+          <t>Obs. 5</t>
         </is>
       </c>
       <c r="E58" s="19" t="inlineStr">
@@ -5758,7 +5766,7 @@
       </c>
       <c r="G58" s="19" t="inlineStr">
         <is>
-          <t>Sprint 5</t>
+          <t>Sprint 4</t>
         </is>
       </c>
       <c r="H58" s="19" t="inlineStr">
@@ -5768,39 +5776,31 @@
       </c>
       <c r="I58" s="19" t="inlineStr">
         <is>
-          <t>Como líder quiero un tablero de mensajes de mi grupo.</t>
+          <t>Como pastor quiero que ofrendas y asistencias sean confidenciales.</t>
         </is>
       </c>
       <c r="J58" s="19" t="inlineStr">
         <is>
-          <t>Publicar y leer mensajes del grupo.</t>
+          <t>La matriz de la sección 3.3 del v3.2 se cumple en pruebas por cada rol.</t>
         </is>
       </c>
       <c r="K58" s="19" t="inlineStr">
         <is>
-          <t>VoBo pendiente</t>
+          <t>Por definir</t>
         </is>
       </c>
       <c r="L58" s="19" t="inlineStr">
         <is>
-          <t>En pruebas</t>
-        </is>
-      </c>
-      <c r="M58" s="19" t="inlineStr">
-        <is>
-          <t>Rama feature/m3-dashboard-tablero · 195 pruebas de backend y 39 de frontend pasan; probado contra la base real</t>
-        </is>
-      </c>
-      <c r="N58" s="19" t="inlineStr">
-        <is>
-          <t>2026-10-25 · Tablero con fijados, no leídos y retención configurable; la notificación push de mensajes nuevos se entrega con M1-09.</t>
-        </is>
-      </c>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M58" s="19" t="inlineStr"/>
+      <c r="N58" s="19" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="18" t="inlineStr">
         <is>
-          <t>M3-12</t>
+          <t>M3-11</t>
         </is>
       </c>
       <c r="B59" s="19" t="inlineStr">
@@ -5810,12 +5810,12 @@
       </c>
       <c r="C59" s="19" t="inlineStr">
         <is>
-          <t>Reuniones: cada grupo se reúne una vez por semana en casa del líder (día y hora por grupo) y existe una reunión general de líderes, modelada como un grupo de tipo «Líderes».</t>
+          <t>Tablero de mensajes del grupo: lo publican Líder, Supervisor, Secretario y Pastor; lo leen todos los integrantes activos. Mensajes de hasta 1,000 caracteres, con opción de fijarlos, borrado lógico, contador de mensajes nuevos y conservación configurable (90 días). Pantalla «Avisos» para quien no abre la página del grupo.</t>
         </is>
       </c>
       <c r="D59" s="21" t="inlineStr">
         <is>
-          <t>Respuesta</t>
+          <t>Obs. 7</t>
         </is>
       </c>
       <c r="E59" s="19" t="inlineStr">
@@ -5830,7 +5830,7 @@
       </c>
       <c r="G59" s="19" t="inlineStr">
         <is>
-          <t>Sprint 3</t>
+          <t>Sprint 5</t>
         </is>
       </c>
       <c r="H59" s="19" t="inlineStr">
@@ -5838,14 +5838,14 @@
           <t>H3 · MVP (Grupos)</t>
         </is>
       </c>
-      <c r="I59" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
-        </is>
-      </c>
-      <c r="J59" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
+      <c r="I59" s="19" t="inlineStr">
+        <is>
+          <t>Como líder quiero un tablero de mensajes de mi grupo.</t>
+        </is>
+      </c>
+      <c r="J59" s="19" t="inlineStr">
+        <is>
+          <t>Publicar y leer mensajes del grupo.</t>
         </is>
       </c>
       <c r="K59" s="19" t="inlineStr">
@@ -5860,19 +5860,19 @@
       </c>
       <c r="M59" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/grupos-paso-3 · pruebas de backend y 81 de frontend pasan; lint, estilos y compilación limpios</t>
+          <t>Rama feature/m3-dashboard-tablero · 195 pruebas de backend y 39 de frontend pasan; probado contra la base real</t>
         </is>
       </c>
       <c r="N59" s="19" t="inlineStr">
         <is>
-          <t>2026-10-27 · Una reunión semanal por grupo y grupo tipo Líderes; filtros por día, sector, líder y estado; cada reunión muestra su asistencia, observaciones, peticiones y ofrendas.</t>
+          <t>2026-10-25 · Tablero con fijados, no leídos y retención configurable; la notificación push de mensajes nuevos se entrega con M1-09.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="18" t="inlineStr">
         <is>
-          <t>M3-13</t>
+          <t>M3-12</t>
         </is>
       </c>
       <c r="B60" s="19" t="inlineStr">
@@ -5882,7 +5882,7 @@
       </c>
       <c r="C60" s="19" t="inlineStr">
         <is>
-          <t>Parámetros configurables sin programar, con pantalla de Configuración y cada cambio en bitácora: monto máximo por ofrenda (1,000,000 por defecto) y si se permite una sola ofrenda regular por reunión. Solo Pastor y Administrador Técnico.</t>
+          <t>Reuniones: cada grupo se reúne una vez por semana en casa del líder (día y hora por grupo) y existe una reunión general de líderes, modelada como un grupo de tipo «Líderes».</t>
         </is>
       </c>
       <c r="D60" s="21" t="inlineStr">
@@ -5902,7 +5902,7 @@
       </c>
       <c r="G60" s="19" t="inlineStr">
         <is>
-          <t>Sprint 4</t>
+          <t>Sprint 3</t>
         </is>
       </c>
       <c r="H60" s="19" t="inlineStr">
@@ -5932,19 +5932,19 @@
       </c>
       <c r="M60" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/m3-ofrendas-ajustes · 121 pruebas de backend y 14 de frontend pasan</t>
+          <t>Rama feature/grupos-paso-3 · pruebas de backend y 81 de frontend pasan; lint, estilos y compilación limpios</t>
         </is>
       </c>
       <c r="N60" s="19" t="inlineStr">
         <is>
-          <t>2026-10-24 · Pantalla Configuración: monto máximo y una regular por reunión.</t>
+          <t>2026-10-27 · Una reunión semanal por grupo y grupo tipo Líderes; filtros por día, sector, líder y estado; cada reunión muestra su asistencia, observaciones, peticiones y ofrendas.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="18" t="inlineStr">
         <is>
-          <t>M3-14</t>
+          <t>M3-13</t>
         </is>
       </c>
       <c r="B61" s="19" t="inlineStr">
@@ -5954,7 +5954,7 @@
       </c>
       <c r="C61" s="19" t="inlineStr">
         <is>
-          <t>Componente de peticiones reutilizable: cualquier módulo (grupos hoy; cursos o eventos después) se registra como origen y decide quién registra y qué nivel de acceso tiene cada persona. Toda petición guarda su origen de forma inmutable (tipo, identificador y una etiqueta fija, por ejemplo «Grupo de Conexión · Norte · reunión del 22/10/2026») y lo muestra siempre en el listado.</t>
+          <t>Parámetros configurables sin programar, con pantalla de Configuración y cada cambio en bitácora: monto máximo por ofrenda (1,000,000 por defecto) y si se permite una sola ofrenda regular por reunión. Solo Pastor y Administrador Técnico.</t>
         </is>
       </c>
       <c r="D61" s="21" t="inlineStr">
@@ -6004,19 +6004,19 @@
       </c>
       <c r="M61" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/m3-peticiones-oracion · 166 pruebas de backend y 32 de frontend pasan; probado contra la base real</t>
+          <t>Rama feature/m3-ofrendas-ajustes · 121 pruebas de backend y 14 de frontend pasan</t>
         </is>
       </c>
       <c r="N61" s="19" t="inlineStr">
         <is>
-          <t>2026-10-24 · Origen inmutable y visible; probado con un segundo origen de prueba para verificar la reutilización.</t>
+          <t>2026-10-24 · Pantalla Configuración: monto máximo y una regular por reunión.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="18" t="inlineStr">
         <is>
-          <t>M3-15</t>
+          <t>M3-14</t>
         </is>
       </c>
       <c r="B62" s="19" t="inlineStr">
@@ -6026,7 +6026,7 @@
       </c>
       <c r="C62" s="19" t="inlineStr">
         <is>
-          <t>Equipo de oración: rol configurable (Equipo de oración) que se asigna a las personas que se reúnen a orar por las peticiones compartidas con ese alcance; no da acceso a nada más. Opción de ocultar el nombre de quien pide: los campos del formulario marcados «identifica a la persona» solo los ven líderes y quien registró. Al capturar se muestra una leyenda que pide confirmar la autorización de quien pide, indica quién la leerá y cuándo se borra.</t>
+          <t>Componente de peticiones reutilizable: cualquier módulo (grupos hoy; cursos o eventos después) se registra como origen y decide quién registra y qué nivel de acceso tiene cada persona. Toda petición guarda su origen de forma inmutable (tipo, identificador y una etiqueta fija, por ejemplo «Grupo de Conexión · Norte · reunión del 22/10/2026») y lo muestra siempre en el listado.</t>
         </is>
       </c>
       <c r="D62" s="21" t="inlineStr">
@@ -6081,49 +6081,49 @@
       </c>
       <c r="N62" s="19" t="inlineStr">
         <is>
-          <t>2026-10-24 · Rol Equipo de oración, nombre oculto y leyenda de privacidad al capturar. Falta el aviso de privacidad oficial de la iglesia.</t>
+          <t>2026-10-24 · Origen inmutable y visible; probado con un segundo origen de prueba para verificar la reutilización.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="18" t="inlineStr">
         <is>
-          <t>M4-01</t>
+          <t>M3-15</t>
         </is>
       </c>
       <c r="B63" s="19" t="inlineStr">
         <is>
-          <t>M4 Kids Check-In/Out</t>
+          <t>M3 Grupos de Conexión</t>
         </is>
       </c>
       <c r="C63" s="19" t="inlineStr">
         <is>
-          <t>Sustitución de la ficha física de papel.</t>
-        </is>
-      </c>
-      <c r="D63" s="19" t="inlineStr">
-        <is>
-          <t>v1 / v2</t>
+          <t>Equipo de oración: rol configurable (Equipo de oración) que se asigna a las personas que se reúnen a orar por las peticiones compartidas con ese alcance; no da acceso a nada más. Opción de ocultar el nombre de quien pide: los campos del formulario marcados «identifica a la persona» solo los ven líderes y quien registró. Al capturar se muestra una leyenda que pide confirmar la autorización de quien pide, indica quién la leerá y cuándo se borra.</t>
+        </is>
+      </c>
+      <c r="D63" s="21" t="inlineStr">
+        <is>
+          <t>Respuesta</t>
         </is>
       </c>
       <c r="E63" s="19" t="inlineStr">
         <is>
-          <t>Fuera del MVP</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="F63" s="19" t="inlineStr">
         <is>
-          <t>Fase 2</t>
+          <t>Fase 1</t>
         </is>
       </c>
       <c r="G63" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sprint 4</t>
         </is>
       </c>
       <c r="H63" s="19" t="inlineStr">
         <is>
-          <t>Posterior</t>
+          <t>H3 · MVP (Grupos)</t>
         </is>
       </c>
       <c r="I63" s="20" t="inlineStr">
@@ -6143,16 +6143,24 @@
       </c>
       <c r="L63" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M63" s="19" t="inlineStr"/>
-      <c r="N63" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M63" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/m3-peticiones-oracion · 166 pruebas de backend y 32 de frontend pasan; probado contra la base real</t>
+        </is>
+      </c>
+      <c r="N63" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-24 · Rol Equipo de oración, nombre oculto y leyenda de privacidad al capturar. Falta el aviso de privacidad oficial de la iglesia.</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="18" t="inlineStr">
         <is>
-          <t>M4-02</t>
+          <t>M4-01</t>
         </is>
       </c>
       <c r="B64" s="19" t="inlineStr">
@@ -6162,12 +6170,12 @@
       </c>
       <c r="C64" s="19" t="inlineStr">
         <is>
-          <t>Registro de ingreso del menor con salón o clase asignada y generación de código único.</t>
-        </is>
-      </c>
-      <c r="D64" s="21" t="inlineStr">
-        <is>
-          <t>v1 + Nuevo v3</t>
+          <t>Sustitución de la ficha física de papel.</t>
+        </is>
+      </c>
+      <c r="D64" s="19" t="inlineStr">
+        <is>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E64" s="19" t="inlineStr">
@@ -6216,7 +6224,7 @@
     <row r="65">
       <c r="A65" s="18" t="inlineStr">
         <is>
-          <t>M4-03</t>
+          <t>M4-02</t>
         </is>
       </c>
       <c r="B65" s="19" t="inlineStr">
@@ -6226,12 +6234,12 @@
       </c>
       <c r="C65" s="19" t="inlineStr">
         <is>
-          <t>Código QR dinámico o OTP temporal en la PWA del padre o tutor.</t>
-        </is>
-      </c>
-      <c r="D65" s="19" t="inlineStr">
-        <is>
-          <t>v2</t>
+          <t>Registro de ingreso del menor con salón o clase asignada y generación de código único.</t>
+        </is>
+      </c>
+      <c r="D65" s="21" t="inlineStr">
+        <is>
+          <t>v1 + Nuevo v3</t>
         </is>
       </c>
       <c r="E65" s="19" t="inlineStr">
@@ -6280,7 +6288,7 @@
     <row r="66">
       <c r="A66" s="18" t="inlineStr">
         <is>
-          <t>M4-04</t>
+          <t>M4-03</t>
         </is>
       </c>
       <c r="B66" s="19" t="inlineStr">
@@ -6290,7 +6298,7 @@
       </c>
       <c r="C66" s="19" t="inlineStr">
         <is>
-          <t>Validación al entregar: el servidor de Kids escanea el código y confirma identidad y fotografía del tutor autorizado en el Expediente Digital.</t>
+          <t>Código QR dinámico o OTP temporal en la PWA del padre o tutor.</t>
         </is>
       </c>
       <c r="D66" s="19" t="inlineStr">
@@ -6344,7 +6352,7 @@
     <row r="67">
       <c r="A67" s="18" t="inlineStr">
         <is>
-          <t>M4-05</t>
+          <t>M4-04</t>
         </is>
       </c>
       <c r="B67" s="19" t="inlineStr">
@@ -6354,12 +6362,12 @@
       </c>
       <c r="C67" s="19" t="inlineStr">
         <is>
-          <t>Alternativa para tutores sin smartphone, sin batería o sin conexión (p. ej. código por SMS o comprobante imprimible con identificación). Por definir.</t>
-        </is>
-      </c>
-      <c r="D67" s="21" t="inlineStr">
-        <is>
-          <t>Nuevo v3</t>
+          <t>Validación al entregar: el servidor de Kids escanea el código y confirma identidad y fotografía del tutor autorizado en el Expediente Digital.</t>
+        </is>
+      </c>
+      <c r="D67" s="19" t="inlineStr">
+        <is>
+          <t>v2</t>
         </is>
       </c>
       <c r="E67" s="19" t="inlineStr">
@@ -6394,7 +6402,7 @@
       </c>
       <c r="K67" s="19" t="inlineStr">
         <is>
-          <t>Por definir</t>
+          <t>VoBo pendiente</t>
         </is>
       </c>
       <c r="L67" s="19" t="inlineStr">
@@ -6408,7 +6416,7 @@
     <row r="68">
       <c r="A68" s="18" t="inlineStr">
         <is>
-          <t>M4-06</t>
+          <t>M4-05</t>
         </is>
       </c>
       <c r="B68" s="19" t="inlineStr">
@@ -6418,7 +6426,7 @@
       </c>
       <c r="C68" s="19" t="inlineStr">
         <is>
-          <t>Autorización temporal de un tercero para recoger al menor, con aprobación del tutor registrado.</t>
+          <t>Alternativa para tutores sin smartphone, sin batería o sin conexión (p. ej. código por SMS o comprobante imprimible con identificación). Por definir.</t>
         </is>
       </c>
       <c r="D68" s="21" t="inlineStr">
@@ -6458,7 +6466,7 @@
       </c>
       <c r="K68" s="19" t="inlineStr">
         <is>
-          <t>VoBo pendiente</t>
+          <t>Por definir</t>
         </is>
       </c>
       <c r="L68" s="19" t="inlineStr">
@@ -6472,7 +6480,7 @@
     <row r="69">
       <c r="A69" s="18" t="inlineStr">
         <is>
-          <t>M4-07</t>
+          <t>M4-06</t>
         </is>
       </c>
       <c r="B69" s="19" t="inlineStr">
@@ -6482,7 +6490,7 @@
       </c>
       <c r="C69" s="19" t="inlineStr">
         <is>
-          <t>Caducidad del código y bitácora de cada entrega (quién recogió, quién entregó, hora).</t>
+          <t>Autorización temporal de un tercero para recoger al menor, con aprobación del tutor registrado.</t>
         </is>
       </c>
       <c r="D69" s="21" t="inlineStr">
@@ -6536,7 +6544,7 @@
     <row r="70">
       <c r="A70" s="18" t="inlineStr">
         <is>
-          <t>M4-08</t>
+          <t>M4-07</t>
         </is>
       </c>
       <c r="B70" s="19" t="inlineStr">
@@ -6546,7 +6554,7 @@
       </c>
       <c r="C70" s="19" t="inlineStr">
         <is>
-          <t>Funcionamiento sin conexión o con conexión degradada para el check-out.</t>
+          <t>Caducidad del código y bitácora de cada entrega (quién recogió, quién entregó, hora).</t>
         </is>
       </c>
       <c r="D70" s="21" t="inlineStr">
@@ -6600,52 +6608,52 @@
     <row r="71">
       <c r="A71" s="18" t="inlineStr">
         <is>
-          <t>M5-01</t>
+          <t>M4-08</t>
         </is>
       </c>
       <c r="B71" s="19" t="inlineStr">
         <is>
-          <t>M5 Áreas y servidores</t>
+          <t>M4 Kids Check-In/Out</t>
         </is>
       </c>
       <c r="C71" s="19" t="inlineStr">
         <is>
-          <t>Catálogo mínimo de áreas y asignación de servidores. Versión reducida del módulo 5, necesaria para permisos por área. Sirve como primer censo.</t>
-        </is>
-      </c>
-      <c r="D71" s="19" t="inlineStr">
-        <is>
-          <t>v3</t>
+          <t>Funcionamiento sin conexión o con conexión degradada para el check-out.</t>
+        </is>
+      </c>
+      <c r="D71" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3</t>
         </is>
       </c>
       <c r="E71" s="19" t="inlineStr">
         <is>
-          <t>MVP mínimo</t>
+          <t>Fuera del MVP</t>
         </is>
       </c>
       <c r="F71" s="19" t="inlineStr">
         <is>
-          <t>Fase 0</t>
+          <t>Fase 2</t>
         </is>
       </c>
       <c r="G71" s="19" t="inlineStr">
         <is>
-          <t>Sprint 1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H71" s="19" t="inlineStr">
         <is>
-          <t>H2 · Fase 0 completa</t>
-        </is>
-      </c>
-      <c r="I71" s="19" t="inlineStr">
-        <is>
-          <t>Como pastor quiero un catálogo de áreas con su personal para conocer la estructura.</t>
-        </is>
-      </c>
-      <c r="J71" s="19" t="inlineStr">
-        <is>
-          <t>Crear un área, asignar servidores y ver el conteo real.</t>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="I71" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
+        </is>
+      </c>
+      <c r="J71" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
         </is>
       </c>
       <c r="K71" s="19" t="inlineStr">
@@ -6664,7 +6672,7 @@
     <row r="72">
       <c r="A72" s="18" t="inlineStr">
         <is>
-          <t>M5-02</t>
+          <t>M5-01</t>
         </is>
       </c>
       <c r="B72" s="19" t="inlineStr">
@@ -6674,42 +6682,42 @@
       </c>
       <c r="C72" s="19" t="inlineStr">
         <is>
-          <t>Roles jerárquicos dentro de cada área (directores, líderes, maestros, servidores).</t>
+          <t>Catálogo mínimo de áreas y asignación de servidores. Versión reducida del módulo 5, necesaria para permisos por área. Sirve como primer censo.</t>
         </is>
       </c>
       <c r="D72" s="19" t="inlineStr">
         <is>
-          <t>v1</t>
+          <t>v3</t>
         </is>
       </c>
       <c r="E72" s="19" t="inlineStr">
         <is>
-          <t>Fuera del MVP</t>
+          <t>MVP mínimo</t>
         </is>
       </c>
       <c r="F72" s="19" t="inlineStr">
         <is>
-          <t>Fase 4</t>
+          <t>Fase 0</t>
         </is>
       </c>
       <c r="G72" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sprint 1</t>
         </is>
       </c>
       <c r="H72" s="19" t="inlineStr">
         <is>
-          <t>Posterior</t>
-        </is>
-      </c>
-      <c r="I72" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
-        </is>
-      </c>
-      <c r="J72" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
+          <t>H2 · Fase 0 completa</t>
+        </is>
+      </c>
+      <c r="I72" s="19" t="inlineStr">
+        <is>
+          <t>Como pastor quiero un catálogo de áreas con su personal para conocer la estructura.</t>
+        </is>
+      </c>
+      <c r="J72" s="19" t="inlineStr">
+        <is>
+          <t>Crear un área, asignar servidores y ver el conteo real.</t>
         </is>
       </c>
       <c r="K72" s="19" t="inlineStr">
@@ -6728,7 +6736,7 @@
     <row r="73">
       <c r="A73" s="18" t="inlineStr">
         <is>
-          <t>M5-03</t>
+          <t>M5-02</t>
         </is>
       </c>
       <c r="B73" s="19" t="inlineStr">
@@ -6738,12 +6746,12 @@
       </c>
       <c r="C73" s="19" t="inlineStr">
         <is>
-          <t>Organigrama y número real de servidores activos, directores y líderes por área.</t>
+          <t>Roles jerárquicos dentro de cada área (directores, líderes, maestros, servidores).</t>
         </is>
       </c>
       <c r="D73" s="19" t="inlineStr">
         <is>
-          <t>v2</t>
+          <t>v1</t>
         </is>
       </c>
       <c r="E73" s="19" t="inlineStr">
@@ -6792,7 +6800,7 @@
     <row r="74">
       <c r="A74" s="18" t="inlineStr">
         <is>
-          <t>M5-04</t>
+          <t>M5-03</t>
         </is>
       </c>
       <c r="B74" s="19" t="inlineStr">
@@ -6802,12 +6810,12 @@
       </c>
       <c r="C74" s="19" t="inlineStr">
         <is>
-          <t>Control de asistencia a turnos o servicios.</t>
+          <t>Organigrama y número real de servidores activos, directores y líderes por área.</t>
         </is>
       </c>
       <c r="D74" s="19" t="inlineStr">
         <is>
-          <t>v1 / v2</t>
+          <t>v2</t>
         </is>
       </c>
       <c r="E74" s="19" t="inlineStr">
@@ -6856,7 +6864,7 @@
     <row r="75">
       <c r="A75" s="18" t="inlineStr">
         <is>
-          <t>M5-05</t>
+          <t>M5-04</t>
         </is>
       </c>
       <c r="B75" s="19" t="inlineStr">
@@ -6866,7 +6874,7 @@
       </c>
       <c r="C75" s="19" t="inlineStr">
         <is>
-          <t>Tablero de avisos y notificaciones interno por área.</t>
+          <t>Control de asistencia a turnos o servicios.</t>
         </is>
       </c>
       <c r="D75" s="19" t="inlineStr">
@@ -6920,7 +6928,7 @@
     <row r="76">
       <c r="A76" s="18" t="inlineStr">
         <is>
-          <t>M5-06</t>
+          <t>M5-05</t>
         </is>
       </c>
       <c r="B76" s="19" t="inlineStr">
@@ -6930,7 +6938,7 @@
       </c>
       <c r="C76" s="19" t="inlineStr">
         <is>
-          <t>Gestión financiera por área: caja chica y gastos operativos.</t>
+          <t>Tablero de avisos y notificaciones interno por área.</t>
         </is>
       </c>
       <c r="D76" s="19" t="inlineStr">
@@ -6984,22 +6992,22 @@
     <row r="77">
       <c r="A77" s="18" t="inlineStr">
         <is>
-          <t>M6-01</t>
+          <t>M5-06</t>
         </is>
       </c>
       <c r="B77" s="19" t="inlineStr">
         <is>
-          <t>M6 Ministerios de servicio</t>
+          <t>M5 Áreas y servidores</t>
         </is>
       </c>
       <c r="C77" s="19" t="inlineStr">
         <is>
-          <t>Control de personal propio de cada ministerio.</t>
-        </is>
-      </c>
-      <c r="D77" s="22" t="inlineStr">
-        <is>
-          <t>Recuperado v1</t>
+          <t>Gestión financiera por área: caja chica y gastos operativos.</t>
+        </is>
+      </c>
+      <c r="D77" s="19" t="inlineStr">
+        <is>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E77" s="19" t="inlineStr">
@@ -7048,7 +7056,7 @@
     <row r="78">
       <c r="A78" s="18" t="inlineStr">
         <is>
-          <t>M6-02</t>
+          <t>M6-01</t>
         </is>
       </c>
       <c r="B78" s="19" t="inlineStr">
@@ -7058,12 +7066,12 @@
       </c>
       <c r="C78" s="19" t="inlineStr">
         <is>
-          <t>Menú o catálogo digital interactivo (público o interno), autogestionado.</t>
-        </is>
-      </c>
-      <c r="D78" s="19" t="inlineStr">
-        <is>
-          <t>v1 / v2</t>
+          <t>Control de personal propio de cada ministerio.</t>
+        </is>
+      </c>
+      <c r="D78" s="22" t="inlineStr">
+        <is>
+          <t>Recuperado v1</t>
         </is>
       </c>
       <c r="E78" s="19" t="inlineStr">
@@ -7112,7 +7120,7 @@
     <row r="79">
       <c r="A79" s="18" t="inlineStr">
         <is>
-          <t>M6-03</t>
+          <t>M6-02</t>
         </is>
       </c>
       <c r="B79" s="19" t="inlineStr">
@@ -7122,7 +7130,7 @@
       </c>
       <c r="C79" s="19" t="inlineStr">
         <is>
-          <t>Calendario de turnos: días regulares de servicio y eventos especiales.</t>
+          <t>Menú o catálogo digital interactivo (público o interno), autogestionado.</t>
         </is>
       </c>
       <c r="D79" s="19" t="inlineStr">
@@ -7176,7 +7184,7 @@
     <row r="80">
       <c r="A80" s="18" t="inlineStr">
         <is>
-          <t>M6-04</t>
+          <t>M6-03</t>
         </is>
       </c>
       <c r="B80" s="19" t="inlineStr">
@@ -7186,7 +7194,7 @@
       </c>
       <c r="C80" s="19" t="inlineStr">
         <is>
-          <t>Registro de asistentes o personas atendidas.</t>
+          <t>Calendario de turnos: días regulares de servicio y eventos especiales.</t>
         </is>
       </c>
       <c r="D80" s="19" t="inlineStr">
@@ -7240,7 +7248,7 @@
     <row r="81">
       <c r="A81" s="18" t="inlineStr">
         <is>
-          <t>M6-05</t>
+          <t>M6-04</t>
         </is>
       </c>
       <c r="B81" s="19" t="inlineStr">
@@ -7250,7 +7258,7 @@
       </c>
       <c r="C81" s="19" t="inlineStr">
         <is>
-          <t>Control de gastos y de inventario básico.</t>
+          <t>Registro de asistentes o personas atendidas.</t>
         </is>
       </c>
       <c r="D81" s="19" t="inlineStr">
@@ -7304,7 +7312,7 @@
     <row r="82">
       <c r="A82" s="18" t="inlineStr">
         <is>
-          <t>M6-06</t>
+          <t>M6-05</t>
         </is>
       </c>
       <c r="B82" s="19" t="inlineStr">
@@ -7314,7 +7322,7 @@
       </c>
       <c r="C82" s="19" t="inlineStr">
         <is>
-          <t>Canal de comunicación directo con el área de Administración General.</t>
+          <t>Control de gastos y de inventario básico.</t>
         </is>
       </c>
       <c r="D82" s="19" t="inlineStr">
@@ -7368,7 +7376,7 @@
     <row r="83">
       <c r="A83" s="18" t="inlineStr">
         <is>
-          <t>M6-07</t>
+          <t>M6-06</t>
         </is>
       </c>
       <c r="B83" s="19" t="inlineStr">
@@ -7378,12 +7386,12 @@
       </c>
       <c r="C83" s="19" t="inlineStr">
         <is>
-          <t>Servicio Médico: los datos de salud de las personas atendidas requieren tratamiento de datos sensibles. Por definir alcance.</t>
-        </is>
-      </c>
-      <c r="D83" s="21" t="inlineStr">
-        <is>
-          <t>Nuevo v3</t>
+          <t>Canal de comunicación directo con el área de Administración General.</t>
+        </is>
+      </c>
+      <c r="D83" s="19" t="inlineStr">
+        <is>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E83" s="19" t="inlineStr">
@@ -7418,7 +7426,7 @@
       </c>
       <c r="K83" s="19" t="inlineStr">
         <is>
-          <t>Por definir</t>
+          <t>VoBo pendiente</t>
         </is>
       </c>
       <c r="L83" s="19" t="inlineStr">
@@ -7432,22 +7440,22 @@
     <row r="84">
       <c r="A84" s="18" t="inlineStr">
         <is>
-          <t>M7-01</t>
+          <t>M6-07</t>
         </is>
       </c>
       <c r="B84" s="19" t="inlineStr">
         <is>
-          <t>M7 Eventos y aforo</t>
+          <t>M6 Ministerios de servicio</t>
         </is>
       </c>
       <c r="C84" s="19" t="inlineStr">
         <is>
-          <t>Eventos abiertos o evangelísticos con formulario de inscripción rápida, sin requerir historial previo.</t>
-        </is>
-      </c>
-      <c r="D84" s="19" t="inlineStr">
-        <is>
-          <t>v1 / v2</t>
+          <t>Servicio Médico: los datos de salud de las personas atendidas requieren tratamiento de datos sensibles. Por definir alcance.</t>
+        </is>
+      </c>
+      <c r="D84" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3</t>
         </is>
       </c>
       <c r="E84" s="19" t="inlineStr">
@@ -7482,7 +7490,7 @@
       </c>
       <c r="K84" s="19" t="inlineStr">
         <is>
-          <t>VoBo pendiente</t>
+          <t>Por definir</t>
         </is>
       </c>
       <c r="L84" s="19" t="inlineStr">
@@ -7496,7 +7504,7 @@
     <row r="85">
       <c r="A85" s="18" t="inlineStr">
         <is>
-          <t>M7-02</t>
+          <t>M7-01</t>
         </is>
       </c>
       <c r="B85" s="19" t="inlineStr">
@@ -7506,12 +7514,12 @@
       </c>
       <c r="C85" s="19" t="inlineStr">
         <is>
-          <t>Consolidación (inducción de personas que asisten por primera vez) como tipo de evento.</t>
-        </is>
-      </c>
-      <c r="D85" s="22" t="inlineStr">
-        <is>
-          <t>Recuperado v1</t>
+          <t>Eventos abiertos o evangelísticos con formulario de inscripción rápida, sin requerir historial previo.</t>
+        </is>
+      </c>
+      <c r="D85" s="19" t="inlineStr">
+        <is>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E85" s="19" t="inlineStr">
@@ -7560,7 +7568,7 @@
     <row r="86">
       <c r="A86" s="18" t="inlineStr">
         <is>
-          <t>M7-03</t>
+          <t>M7-02</t>
         </is>
       </c>
       <c r="B86" s="19" t="inlineStr">
@@ -7570,7 +7578,7 @@
       </c>
       <c r="C86" s="19" t="inlineStr">
         <is>
-          <t>Encargados de evento (personal de la iglesia únicamente; no se controla personal externo).</t>
+          <t>Consolidación (inducción de personas que asisten por primera vez) como tipo de evento.</t>
         </is>
       </c>
       <c r="D86" s="22" t="inlineStr">
@@ -7624,7 +7632,7 @@
     <row r="87">
       <c r="A87" s="18" t="inlineStr">
         <is>
-          <t>M7-04</t>
+          <t>M7-03</t>
         </is>
       </c>
       <c r="B87" s="19" t="inlineStr">
@@ -7634,12 +7642,12 @@
       </c>
       <c r="C87" s="19" t="inlineStr">
         <is>
-          <t>Control de cupo en tiempo real que bloquea el sobrecupo en eventos con aforo limitado (ej. 30 o 50 lugares).</t>
-        </is>
-      </c>
-      <c r="D87" s="19" t="inlineStr">
-        <is>
-          <t>v1 / v2</t>
+          <t>Encargados de evento (personal de la iglesia únicamente; no se controla personal externo).</t>
+        </is>
+      </c>
+      <c r="D87" s="22" t="inlineStr">
+        <is>
+          <t>Recuperado v1</t>
         </is>
       </c>
       <c r="E87" s="19" t="inlineStr">
@@ -7688,7 +7696,7 @@
     <row r="88">
       <c r="A88" s="18" t="inlineStr">
         <is>
-          <t>M7-05</t>
+          <t>M7-04</t>
         </is>
       </c>
       <c r="B88" s="19" t="inlineStr">
@@ -7698,12 +7706,12 @@
       </c>
       <c r="C88" s="19" t="inlineStr">
         <is>
-          <t>Control de asistentes sin lista previa, para aforo y para dar a conocer la iglesia.</t>
+          <t>Control de cupo en tiempo real que bloquea el sobrecupo en eventos con aforo limitado (ej. 30 o 50 lugares).</t>
         </is>
       </c>
       <c r="D88" s="19" t="inlineStr">
         <is>
-          <t>v1</t>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E88" s="19" t="inlineStr">
@@ -7752,7 +7760,7 @@
     <row r="89">
       <c r="A89" s="18" t="inlineStr">
         <is>
-          <t>M7-06</t>
+          <t>M7-05</t>
         </is>
       </c>
       <c r="B89" s="19" t="inlineStr">
@@ -7762,12 +7770,12 @@
       </c>
       <c r="C89" s="19" t="inlineStr">
         <is>
-          <t>Seguimiento de personas nuevas: conversión de un invitado a Expediente Digital y canalización a un curso o Grupo de Conexión.</t>
-        </is>
-      </c>
-      <c r="D89" s="21" t="inlineStr">
-        <is>
-          <t>Nuevo v3</t>
+          <t>Control de asistentes sin lista previa, para aforo y para dar a conocer la iglesia.</t>
+        </is>
+      </c>
+      <c r="D89" s="19" t="inlineStr">
+        <is>
+          <t>v1</t>
         </is>
       </c>
       <c r="E89" s="19" t="inlineStr">
@@ -7816,52 +7824,52 @@
     <row r="90">
       <c r="A90" s="18" t="inlineStr">
         <is>
-          <t>NF-01</t>
+          <t>M7-06</t>
         </is>
       </c>
       <c r="B90" s="19" t="inlineStr">
         <is>
-          <t>No funcionales</t>
+          <t>M7 Eventos y aforo</t>
         </is>
       </c>
       <c r="C90" s="19" t="inlineStr">
         <is>
-          <t>Cumplimiento de la LFPDPPP: aviso de privacidad, consentimiento y derechos ARCO.</t>
-        </is>
-      </c>
-      <c r="D90" s="19" t="inlineStr">
-        <is>
-          <t>v3</t>
+          <t>Seguimiento de personas nuevas: conversión de un invitado a Expediente Digital y canalización a un curso o Grupo de Conexión.</t>
+        </is>
+      </c>
+      <c r="D90" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3</t>
         </is>
       </c>
       <c r="E90" s="19" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Fuera del MVP</t>
         </is>
       </c>
       <c r="F90" s="19" t="inlineStr">
         <is>
-          <t>Fase 0</t>
+          <t>Fase 4</t>
         </is>
       </c>
       <c r="G90" s="19" t="inlineStr">
         <is>
-          <t>Sprint 1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H90" s="19" t="inlineStr">
         <is>
-          <t>H1 · 18-oct (núcleo Fase 0)</t>
-        </is>
-      </c>
-      <c r="I90" s="19" t="inlineStr">
-        <is>
-          <t>Como iglesia queremos cumplir con la LFPDPPP.</t>
-        </is>
-      </c>
-      <c r="J90" s="19" t="inlineStr">
-        <is>
-          <t>Aviso de privacidad, consentimiento y atención de derechos ARCO disponibles.</t>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="I90" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
+        </is>
+      </c>
+      <c r="J90" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
         </is>
       </c>
       <c r="K90" s="19" t="inlineStr">
@@ -7880,7 +7888,7 @@
     <row r="91">
       <c r="A91" s="18" t="inlineStr">
         <is>
-          <t>NF-02</t>
+          <t>NF-01</t>
         </is>
       </c>
       <c r="B91" s="19" t="inlineStr">
@@ -7890,7 +7898,7 @@
       </c>
       <c r="C91" s="19" t="inlineStr">
         <is>
-          <t>Cifrado en tránsito y en reposo. Cifrado adicional a nivel de campo para peticiones de oración.</t>
+          <t>Cumplimiento de la LFPDPPP: aviso de privacidad, consentimiento y derechos ARCO.</t>
         </is>
       </c>
       <c r="D91" s="19" t="inlineStr">
@@ -7910,7 +7918,7 @@
       </c>
       <c r="G91" s="19" t="inlineStr">
         <is>
-          <t>Sprint 0</t>
+          <t>Sprint 1</t>
         </is>
       </c>
       <c r="H91" s="19" t="inlineStr">
@@ -7920,12 +7928,12 @@
       </c>
       <c r="I91" s="19" t="inlineStr">
         <is>
-          <t>Como iglesia queremos proteger los datos sensibles.</t>
+          <t>Como iglesia queremos cumplir con la LFPDPPP.</t>
         </is>
       </c>
       <c r="J91" s="19" t="inlineStr">
         <is>
-          <t>HTTPS obligatorio y peticiones de oración ilegibles directamente en la base.</t>
+          <t>Aviso de privacidad, consentimiento y atención de derechos ARCO disponibles.</t>
         </is>
       </c>
       <c r="K91" s="19" t="inlineStr">
@@ -7935,24 +7943,16 @@
       </c>
       <c r="L91" s="19" t="inlineStr">
         <is>
-          <t>En pruebas</t>
-        </is>
-      </c>
-      <c r="M91" s="19" t="inlineStr">
-        <is>
-          <t>Rama feature/m3-peticiones-oracion · 166 pruebas de backend y 32 de frontend pasan; probado contra la base real</t>
-        </is>
-      </c>
-      <c r="N91" s="19" t="inlineStr">
-        <is>
-          <t>2026-10-24 · Peticiones cifradas a nivel de campo; falta cifrado en reposo de toda la base (proveedor de nube).</t>
-        </is>
-      </c>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M91" s="19" t="inlineStr"/>
+      <c r="N91" s="19" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="18" t="inlineStr">
         <is>
-          <t>NF-03</t>
+          <t>NF-02</t>
         </is>
       </c>
       <c r="B92" s="19" t="inlineStr">
@@ -7962,7 +7962,7 @@
       </c>
       <c r="C92" s="19" t="inlineStr">
         <is>
-          <t>Bitácora de auditoría de solo-añadir: quién consultó o modificó expedientes, ofrendas y asistencias.</t>
+          <t>Cifrado en tránsito y en reposo. Cifrado adicional a nivel de campo para peticiones de oración.</t>
         </is>
       </c>
       <c r="D92" s="19" t="inlineStr">
@@ -7982,7 +7982,7 @@
       </c>
       <c r="G92" s="19" t="inlineStr">
         <is>
-          <t>Sprint 1</t>
+          <t>Sprint 0</t>
         </is>
       </c>
       <c r="H92" s="19" t="inlineStr">
@@ -7992,12 +7992,12 @@
       </c>
       <c r="I92" s="19" t="inlineStr">
         <is>
-          <t>Como pastor quiero una bitácora que nadie pueda alterar.</t>
+          <t>Como iglesia queremos proteger los datos sensibles.</t>
         </is>
       </c>
       <c r="J92" s="19" t="inlineStr">
         <is>
-          <t>El usuario de la aplicación no puede actualizar ni borrar registros de bitácora.</t>
+          <t>HTTPS obligatorio y peticiones de oración ilegibles directamente en la base.</t>
         </is>
       </c>
       <c r="K92" s="19" t="inlineStr">
@@ -8012,19 +8012,19 @@
       </c>
       <c r="M92" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/nf-03-bitacora · 69 pruebas de backend pasan</t>
+          <t>Rama feature/m3-peticiones-oracion · 166 pruebas de backend y 32 de frontend pasan; probado contra la base real</t>
         </is>
       </c>
       <c r="N92" s="19" t="inlineStr">
         <is>
-          <t>2026-10-10 · Bloqueo en aplicación y trigger de PostgreSQL (UPDATE/DELETE/TRUNCATE); pantalla de consulta con permiso bitacora.ver.</t>
+          <t>2026-10-24 · Peticiones cifradas a nivel de campo; falta cifrado en reposo de toda la base (proveedor de nube).</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="18" t="inlineStr">
         <is>
-          <t>NF-04</t>
+          <t>NF-03</t>
         </is>
       </c>
       <c r="B93" s="19" t="inlineStr">
@@ -8034,7 +8034,7 @@
       </c>
       <c r="C93" s="19" t="inlineStr">
         <is>
-          <t>Respaldos automáticos diarios cifrados y prueba periódica de restauración.</t>
+          <t>Bitácora de auditoría de solo-añadir: quién consultó o modificó expedientes, ofrendas y asistencias.</t>
         </is>
       </c>
       <c r="D93" s="19" t="inlineStr">
@@ -8054,7 +8054,7 @@
       </c>
       <c r="G93" s="19" t="inlineStr">
         <is>
-          <t>Sprint 0</t>
+          <t>Sprint 1</t>
         </is>
       </c>
       <c r="H93" s="19" t="inlineStr">
@@ -8064,12 +8064,12 @@
       </c>
       <c r="I93" s="19" t="inlineStr">
         <is>
-          <t>Como iglesia queremos no perder información.</t>
+          <t>Como pastor quiero una bitácora que nadie pueda alterar.</t>
         </is>
       </c>
       <c r="J93" s="19" t="inlineStr">
         <is>
-          <t>Respaldo diario cifrado y restauración probada en un ambiente de pruebas.</t>
+          <t>El usuario de la aplicación no puede actualizar ni borrar registros de bitácora.</t>
         </is>
       </c>
       <c r="K93" s="19" t="inlineStr">
@@ -8079,16 +8079,24 @@
       </c>
       <c r="L93" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M93" s="19" t="inlineStr"/>
-      <c r="N93" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M93" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/nf-03-bitacora · 69 pruebas de backend pasan</t>
+        </is>
+      </c>
+      <c r="N93" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-10 · Bloqueo en aplicación y trigger de PostgreSQL (UPDATE/DELETE/TRUNCATE); pantalla de consulta con permiso bitacora.ver.</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="18" t="inlineStr">
         <is>
-          <t>NF-05</t>
+          <t>NF-04</t>
         </is>
       </c>
       <c r="B94" s="19" t="inlineStr">
@@ -8098,47 +8106,47 @@
       </c>
       <c r="C94" s="19" t="inlineStr">
         <is>
-          <t>Disponibilidad esperada en horarios de servicio (fines de semana y reuniones de grupo). Por definir meta.</t>
-        </is>
-      </c>
-      <c r="D94" s="21" t="inlineStr">
-        <is>
-          <t>Nuevo v3</t>
+          <t>Respaldos automáticos diarios cifrados y prueba periódica de restauración.</t>
+        </is>
+      </c>
+      <c r="D94" s="19" t="inlineStr">
+        <is>
+          <t>v3</t>
         </is>
       </c>
       <c r="E94" s="19" t="inlineStr">
         <is>
-          <t>Fuera del MVP</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="F94" s="19" t="inlineStr">
         <is>
-          <t>Transversal</t>
+          <t>Fase 0</t>
         </is>
       </c>
       <c r="G94" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sprint 0</t>
         </is>
       </c>
       <c r="H94" s="19" t="inlineStr">
         <is>
-          <t>Posterior</t>
-        </is>
-      </c>
-      <c r="I94" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
-        </is>
-      </c>
-      <c r="J94" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
+          <t>H1 · 18-oct (núcleo Fase 0)</t>
+        </is>
+      </c>
+      <c r="I94" s="19" t="inlineStr">
+        <is>
+          <t>Como iglesia queremos no perder información.</t>
+        </is>
+      </c>
+      <c r="J94" s="19" t="inlineStr">
+        <is>
+          <t>Respaldo diario cifrado y restauración probada en un ambiente de pruebas.</t>
         </is>
       </c>
       <c r="K94" s="19" t="inlineStr">
         <is>
-          <t>Por definir</t>
+          <t>VoBo pendiente</t>
         </is>
       </c>
       <c r="L94" s="19" t="inlineStr">
@@ -8152,7 +8160,7 @@
     <row r="95">
       <c r="A95" s="18" t="inlineStr">
         <is>
-          <t>NF-06</t>
+          <t>NF-05</t>
         </is>
       </c>
       <c r="B95" s="19" t="inlineStr">
@@ -8162,69 +8170,61 @@
       </c>
       <c r="C95" s="19" t="inlineStr">
         <is>
-          <t>Pase de lista sin conexión con sincronización posterior (reuniones en domicilios con mala señal).</t>
-        </is>
-      </c>
-      <c r="D95" s="19" t="inlineStr">
-        <is>
-          <t>v3</t>
+          <t>Disponibilidad esperada en horarios de servicio (fines de semana y reuniones de grupo). Por definir meta.</t>
+        </is>
+      </c>
+      <c r="D95" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3</t>
         </is>
       </c>
       <c r="E95" s="19" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Fuera del MVP</t>
         </is>
       </c>
       <c r="F95" s="19" t="inlineStr">
         <is>
-          <t>Fase 0</t>
+          <t>Transversal</t>
         </is>
       </c>
       <c r="G95" s="19" t="inlineStr">
         <is>
-          <t>Sprint 3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H95" s="19" t="inlineStr">
         <is>
-          <t>H3 · MVP (Grupos)</t>
-        </is>
-      </c>
-      <c r="I95" s="19" t="inlineStr">
-        <is>
-          <t>Como secretario quiero que el pase de lista funcione sin señal.</t>
-        </is>
-      </c>
-      <c r="J95" s="19" t="inlineStr">
-        <is>
-          <t>Prueba en modo avión y sincronización al reconectar.</t>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="I95" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
+        </is>
+      </c>
+      <c r="J95" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
         </is>
       </c>
       <c r="K95" s="19" t="inlineStr">
         <is>
-          <t>VoBo pendiente</t>
+          <t>Por definir</t>
         </is>
       </c>
       <c r="L95" s="19" t="inlineStr">
         <is>
-          <t>En pruebas</t>
-        </is>
-      </c>
-      <c r="M95" s="19" t="inlineStr">
-        <is>
-          <t>Rama feature/nf-06-sin-conexion · 117 pruebas de backend y 27 de frontend; probado en Chrome real con service worker</t>
-        </is>
-      </c>
-      <c r="N95" s="19" t="inlineStr">
-        <is>
-          <t>2026-10-24 · Probado de punta a punta en Chrome (sin red → cola → sincronización). Pendiente probar en Android e iOS reales.</t>
-        </is>
-      </c>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M95" s="19" t="inlineStr"/>
+      <c r="N95" s="19" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" s="18" t="inlineStr">
         <is>
-          <t>NF-07</t>
+          <t>NF-06</t>
         </is>
       </c>
       <c r="B96" s="19" t="inlineStr">
@@ -8234,7 +8234,7 @@
       </c>
       <c r="C96" s="19" t="inlineStr">
         <is>
-          <t>Funciona en Android, iOS y escritorio. En iOS, las notificaciones push requieren instalar la PWA; el respaldo por WhatsApp cubre el resto.</t>
+          <t>Pase de lista sin conexión con sincronización posterior (reuniones en domicilios con mala señal).</t>
         </is>
       </c>
       <c r="D96" s="19" t="inlineStr">
@@ -8254,22 +8254,22 @@
       </c>
       <c r="G96" s="19" t="inlineStr">
         <is>
-          <t>Sprint 0</t>
+          <t>Sprint 3</t>
         </is>
       </c>
       <c r="H96" s="19" t="inlineStr">
         <is>
-          <t>H1 · 18-oct (núcleo Fase 0)</t>
+          <t>H3 · MVP (Grupos)</t>
         </is>
       </c>
       <c r="I96" s="19" t="inlineStr">
         <is>
-          <t>Como usuario quiero usar el sistema en mi dispositivo.</t>
+          <t>Como secretario quiero que el pase de lista funcione sin señal.</t>
         </is>
       </c>
       <c r="J96" s="19" t="inlineStr">
         <is>
-          <t>Pruebas en Android, iOS y escritorio; push en iOS con la PWA instalada y respaldo por WhatsApp.</t>
+          <t>Prueba en modo avión y sincronización al reconectar.</t>
         </is>
       </c>
       <c r="K96" s="19" t="inlineStr">
@@ -8279,16 +8279,24 @@
       </c>
       <c r="L96" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M96" s="19" t="inlineStr"/>
-      <c r="N96" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M96" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/nf-06-sin-conexion · 117 pruebas de backend y 27 de frontend; probado en Chrome real con service worker</t>
+        </is>
+      </c>
+      <c r="N96" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-24 · Probado de punta a punta en Chrome (sin red → cola → sincronización). Pendiente probar en Android e iOS reales.</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="18" t="inlineStr">
         <is>
-          <t>NF-08</t>
+          <t>NF-07</t>
         </is>
       </c>
       <c r="B97" s="19" t="inlineStr">
@@ -8298,12 +8306,12 @@
       </c>
       <c r="C97" s="19" t="inlineStr">
         <is>
-          <t>Dimensionamiento para ~1,000 personas, con picos los fines de semana, y margen de crecimiento.</t>
-        </is>
-      </c>
-      <c r="D97" s="21" t="inlineStr">
-        <is>
-          <t>Resp. P8</t>
+          <t>Funciona en Android, iOS y escritorio. En iOS, las notificaciones push requieren instalar la PWA; el respaldo por WhatsApp cubre el resto.</t>
+        </is>
+      </c>
+      <c r="D97" s="19" t="inlineStr">
+        <is>
+          <t>v3</t>
         </is>
       </c>
       <c r="E97" s="19" t="inlineStr">
@@ -8328,12 +8336,12 @@
       </c>
       <c r="I97" s="19" t="inlineStr">
         <is>
-          <t>Como iglesia queremos que el sistema soporte a ~1,000 personas.</t>
+          <t>Como usuario quiero usar el sistema en mi dispositivo.</t>
         </is>
       </c>
       <c r="J97" s="19" t="inlineStr">
         <is>
-          <t>Prueba de carga con volumen representativo (por definir) sin degradación.</t>
+          <t>Pruebas en Android, iOS y escritorio; push en iOS con la PWA instalada y respaldo por WhatsApp.</t>
         </is>
       </c>
       <c r="K97" s="19" t="inlineStr">
@@ -8352,7 +8360,7 @@
     <row r="98">
       <c r="A98" s="18" t="inlineStr">
         <is>
-          <t>NF-09</t>
+          <t>NF-08</t>
         </is>
       </c>
       <c r="B98" s="19" t="inlineStr">
@@ -8362,42 +8370,42 @@
       </c>
       <c r="C98" s="19" t="inlineStr">
         <is>
-          <t>Reportes transversales: asistencia, finanzas, crecimiento de la iglesia, exportables a Excel y PDF.</t>
+          <t>Dimensionamiento para ~1,000 personas, con picos los fines de semana, y margen de crecimiento.</t>
         </is>
       </c>
       <c r="D98" s="21" t="inlineStr">
         <is>
-          <t>Nuevo v3</t>
+          <t>Resp. P8</t>
         </is>
       </c>
       <c r="E98" s="19" t="inlineStr">
         <is>
-          <t>Fuera del MVP</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="F98" s="19" t="inlineStr">
         <is>
-          <t>Transversal</t>
+          <t>Fase 0</t>
         </is>
       </c>
       <c r="G98" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sprint 0</t>
         </is>
       </c>
       <c r="H98" s="19" t="inlineStr">
         <is>
-          <t>Posterior</t>
-        </is>
-      </c>
-      <c r="I98" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
-        </is>
-      </c>
-      <c r="J98" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
+          <t>H1 · 18-oct (núcleo Fase 0)</t>
+        </is>
+      </c>
+      <c r="I98" s="19" t="inlineStr">
+        <is>
+          <t>Como iglesia queremos que el sistema soporte a ~1,000 personas.</t>
+        </is>
+      </c>
+      <c r="J98" s="19" t="inlineStr">
+        <is>
+          <t>Prueba de carga con volumen representativo (por definir) sin degradación.</t>
         </is>
       </c>
       <c r="K98" s="19" t="inlineStr">
@@ -8416,7 +8424,7 @@
     <row r="99">
       <c r="A99" s="18" t="inlineStr">
         <is>
-          <t>NF-10</t>
+          <t>NF-09</t>
         </is>
       </c>
       <c r="B99" s="19" t="inlineStr">
@@ -8426,42 +8434,42 @@
       </c>
       <c r="C99" s="19" t="inlineStr">
         <is>
-          <t>Usabilidad para personas mayores: tipografía grande, alto contraste, flujos cortos (ver sección 5).</t>
-        </is>
-      </c>
-      <c r="D99" s="19" t="inlineStr">
-        <is>
-          <t>v3 + Obs. 1</t>
+          <t>Reportes transversales: asistencia, finanzas, crecimiento de la iglesia, exportables a Excel y PDF.</t>
+        </is>
+      </c>
+      <c r="D99" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3</t>
         </is>
       </c>
       <c r="E99" s="19" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Fuera del MVP</t>
         </is>
       </c>
       <c r="F99" s="19" t="inlineStr">
         <is>
-          <t>Fase 0</t>
+          <t>Transversal</t>
         </is>
       </c>
       <c r="G99" s="19" t="inlineStr">
         <is>
-          <t>Sprint 0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H99" s="19" t="inlineStr">
         <is>
-          <t>H1 · 18-oct (núcleo Fase 0)</t>
-        </is>
-      </c>
-      <c r="I99" s="19" t="inlineStr">
-        <is>
-          <t>Como persona mayor quiero una interfaz fácil de leer y usar.</t>
-        </is>
-      </c>
-      <c r="J99" s="19" t="inlineStr">
-        <is>
-          <t>Texto base 18 px, botones de al menos 48 px, contraste AA; prueba con usuarios mayores.</t>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="I99" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
+        </is>
+      </c>
+      <c r="J99" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
         </is>
       </c>
       <c r="K99" s="19" t="inlineStr">
@@ -8477,9 +8485,73 @@
       <c r="M99" s="19" t="inlineStr"/>
       <c r="N99" s="19" t="inlineStr"/>
     </row>
+    <row r="100">
+      <c r="A100" s="18" t="inlineStr">
+        <is>
+          <t>NF-10</t>
+        </is>
+      </c>
+      <c r="B100" s="19" t="inlineStr">
+        <is>
+          <t>No funcionales</t>
+        </is>
+      </c>
+      <c r="C100" s="19" t="inlineStr">
+        <is>
+          <t>Usabilidad para personas mayores: tipografía grande, alto contraste, flujos cortos (ver sección 5).</t>
+        </is>
+      </c>
+      <c r="D100" s="19" t="inlineStr">
+        <is>
+          <t>v3 + Obs. 1</t>
+        </is>
+      </c>
+      <c r="E100" s="19" t="inlineStr">
+        <is>
+          <t>MVP</t>
+        </is>
+      </c>
+      <c r="F100" s="19" t="inlineStr">
+        <is>
+          <t>Fase 0</t>
+        </is>
+      </c>
+      <c r="G100" s="19" t="inlineStr">
+        <is>
+          <t>Sprint 0</t>
+        </is>
+      </c>
+      <c r="H100" s="19" t="inlineStr">
+        <is>
+          <t>H1 · 18-oct (núcleo Fase 0)</t>
+        </is>
+      </c>
+      <c r="I100" s="19" t="inlineStr">
+        <is>
+          <t>Como persona mayor quiero una interfaz fácil de leer y usar.</t>
+        </is>
+      </c>
+      <c r="J100" s="19" t="inlineStr">
+        <is>
+          <t>Texto base 18 px, botones de al menos 48 px, contraste AA; prueba con usuarios mayores.</t>
+        </is>
+      </c>
+      <c r="K100" s="19" t="inlineStr">
+        <is>
+          <t>VoBo pendiente</t>
+        </is>
+      </c>
+      <c r="L100" s="19" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M100" s="19" t="inlineStr"/>
+      <c r="N100" s="19" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N99"/>
-  <conditionalFormatting sqref="L2:L99">
+  <autoFilter ref="A1:N100"/>
+  <conditionalFormatting sqref="L2:L100">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$L2="Hecho"</formula>
     </cfRule>
@@ -8496,7 +8568,7 @@
       <formula>$L2="Bloqueado"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K2:K99">
+  <conditionalFormatting sqref="K2:K100">
     <cfRule type="expression" priority="6" dxfId="0">
       <formula>$K2="Aprobado"</formula>
     </cfRule>
@@ -8504,16 +8576,16 @@
       <formula>$K2="Por definir"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H2:H99">
+  <conditionalFormatting sqref="H2:H100">
     <cfRule type="expression" priority="8" dxfId="5">
       <formula>LEFT($H2,2)="H1"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="L2:L99" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="L2:L100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Pendiente,En diseño,En desarrollo,En pruebas,Hecho,Bloqueado"</formula1>
     </dataValidation>
-    <dataValidation sqref="K2:K99" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="K2:K100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"VoBo pendiente,Aprobado,Por definir,Rechazado"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Unidades con alcance propio y avisos masivos (paso 7)
- Unidades (áreas de servicio): encargado, respaldo y servidores; cada rol
  vale solo dentro de su unidad, independiente de grupos y otras unidades
- Tablero de avisos por unidad
- Avisos masivos a toda la iglesia, grupos, unidades y personas, con permisos
  por destino; avisos recibidos agrupados en Avisos
- Cuatro permisos nuevos en la matriz de roles (unidades y avisos masivos)
- Documentos v3.20 (anexo S, requisito M1-25) y matriz de trazabilidad actualizados

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/trazabilidad/Matriz de Trazabilidad MDF.xlsx
+++ b/docs/trazabilidad/Matriz de Trazabilidad MDF.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Origen v1" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Matriz'!$A$1:$N$100</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Matriz'!$A$1:$N$101</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -897,31 +897,31 @@
         </is>
       </c>
       <c r="B5" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$100,$A5)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$101,$A5)</f>
         <v/>
       </c>
       <c r="C5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$100,$A5,Matriz!$L$2:$L$100,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$101,$A5,Matriz!$L$2:$L$101,"Pendiente")</f>
         <v/>
       </c>
       <c r="D5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$100,$A5,Matriz!$L$2:$L$100,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$101,$A5,Matriz!$L$2:$L$101,"En diseño")</f>
         <v/>
       </c>
       <c r="E5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$100,$A5,Matriz!$L$2:$L$100,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$101,$A5,Matriz!$L$2:$L$101,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$100,$A5,Matriz!$L$2:$L$100,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$101,$A5,Matriz!$L$2:$L$101,"En pruebas")</f>
         <v/>
       </c>
       <c r="G5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$100,$A5,Matriz!$L$2:$L$100,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$101,$A5,Matriz!$L$2:$L$101,"Hecho")</f>
         <v/>
       </c>
       <c r="H5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$100,$A5,Matriz!$L$2:$L$100,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$101,$A5,Matriz!$L$2:$L$101,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I5" s="13">
@@ -936,31 +936,31 @@
         </is>
       </c>
       <c r="B6" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$100,$A6)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$101,$A6)</f>
         <v/>
       </c>
       <c r="C6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$100,$A6,Matriz!$L$2:$L$100,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$101,$A6,Matriz!$L$2:$L$101,"Pendiente")</f>
         <v/>
       </c>
       <c r="D6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$100,$A6,Matriz!$L$2:$L$100,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$101,$A6,Matriz!$L$2:$L$101,"En diseño")</f>
         <v/>
       </c>
       <c r="E6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$100,$A6,Matriz!$L$2:$L$100,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$101,$A6,Matriz!$L$2:$L$101,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$100,$A6,Matriz!$L$2:$L$100,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$101,$A6,Matriz!$L$2:$L$101,"En pruebas")</f>
         <v/>
       </c>
       <c r="G6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$100,$A6,Matriz!$L$2:$L$100,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$101,$A6,Matriz!$L$2:$L$101,"Hecho")</f>
         <v/>
       </c>
       <c r="H6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$100,$A6,Matriz!$L$2:$L$100,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$101,$A6,Matriz!$L$2:$L$101,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I6" s="13">
@@ -975,31 +975,31 @@
         </is>
       </c>
       <c r="B7" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$100,$A7)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$101,$A7)</f>
         <v/>
       </c>
       <c r="C7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$100,$A7,Matriz!$L$2:$L$100,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$101,$A7,Matriz!$L$2:$L$101,"Pendiente")</f>
         <v/>
       </c>
       <c r="D7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$100,$A7,Matriz!$L$2:$L$100,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$101,$A7,Matriz!$L$2:$L$101,"En diseño")</f>
         <v/>
       </c>
       <c r="E7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$100,$A7,Matriz!$L$2:$L$100,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$101,$A7,Matriz!$L$2:$L$101,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$100,$A7,Matriz!$L$2:$L$100,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$101,$A7,Matriz!$L$2:$L$101,"En pruebas")</f>
         <v/>
       </c>
       <c r="G7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$100,$A7,Matriz!$L$2:$L$100,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$101,$A7,Matriz!$L$2:$L$101,"Hecho")</f>
         <v/>
       </c>
       <c r="H7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$100,$A7,Matriz!$L$2:$L$100,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$101,$A7,Matriz!$L$2:$L$101,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I7" s="13">
@@ -1014,31 +1014,31 @@
         </is>
       </c>
       <c r="B8" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$100,$A8)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$101,$A8)</f>
         <v/>
       </c>
       <c r="C8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$100,$A8,Matriz!$L$2:$L$100,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$101,$A8,Matriz!$L$2:$L$101,"Pendiente")</f>
         <v/>
       </c>
       <c r="D8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$100,$A8,Matriz!$L$2:$L$100,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$101,$A8,Matriz!$L$2:$L$101,"En diseño")</f>
         <v/>
       </c>
       <c r="E8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$100,$A8,Matriz!$L$2:$L$100,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$101,$A8,Matriz!$L$2:$L$101,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$100,$A8,Matriz!$L$2:$L$100,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$101,$A8,Matriz!$L$2:$L$101,"En pruebas")</f>
         <v/>
       </c>
       <c r="G8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$100,$A8,Matriz!$L$2:$L$100,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$101,$A8,Matriz!$L$2:$L$101,"Hecho")</f>
         <v/>
       </c>
       <c r="H8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$100,$A8,Matriz!$L$2:$L$100,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$101,$A8,Matriz!$L$2:$L$101,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I8" s="13">
@@ -1053,31 +1053,31 @@
         </is>
       </c>
       <c r="B9" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$100,$A9)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$101,$A9)</f>
         <v/>
       </c>
       <c r="C9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$100,$A9,Matriz!$L$2:$L$100,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$101,$A9,Matriz!$L$2:$L$101,"Pendiente")</f>
         <v/>
       </c>
       <c r="D9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$100,$A9,Matriz!$L$2:$L$100,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$101,$A9,Matriz!$L$2:$L$101,"En diseño")</f>
         <v/>
       </c>
       <c r="E9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$100,$A9,Matriz!$L$2:$L$100,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$101,$A9,Matriz!$L$2:$L$101,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$100,$A9,Matriz!$L$2:$L$100,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$101,$A9,Matriz!$L$2:$L$101,"En pruebas")</f>
         <v/>
       </c>
       <c r="G9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$100,$A9,Matriz!$L$2:$L$100,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$101,$A9,Matriz!$L$2:$L$101,"Hecho")</f>
         <v/>
       </c>
       <c r="H9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$100,$A9,Matriz!$L$2:$L$100,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$101,$A9,Matriz!$L$2:$L$101,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I9" s="13">
@@ -1092,31 +1092,31 @@
         </is>
       </c>
       <c r="B10" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$100,$A10)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$101,$A10)</f>
         <v/>
       </c>
       <c r="C10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$100,$A10,Matriz!$L$2:$L$100,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$101,$A10,Matriz!$L$2:$L$101,"Pendiente")</f>
         <v/>
       </c>
       <c r="D10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$100,$A10,Matriz!$L$2:$L$100,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$101,$A10,Matriz!$L$2:$L$101,"En diseño")</f>
         <v/>
       </c>
       <c r="E10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$100,$A10,Matriz!$L$2:$L$100,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$101,$A10,Matriz!$L$2:$L$101,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$100,$A10,Matriz!$L$2:$L$100,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$101,$A10,Matriz!$L$2:$L$101,"En pruebas")</f>
         <v/>
       </c>
       <c r="G10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$100,$A10,Matriz!$L$2:$L$100,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$101,$A10,Matriz!$L$2:$L$101,"Hecho")</f>
         <v/>
       </c>
       <c r="H10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$100,$A10,Matriz!$L$2:$L$100,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$101,$A10,Matriz!$L$2:$L$101,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I10" s="13">
@@ -1131,31 +1131,31 @@
         </is>
       </c>
       <c r="B11" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$100,$A11)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$101,$A11)</f>
         <v/>
       </c>
       <c r="C11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$100,$A11,Matriz!$L$2:$L$100,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$101,$A11,Matriz!$L$2:$L$101,"Pendiente")</f>
         <v/>
       </c>
       <c r="D11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$100,$A11,Matriz!$L$2:$L$100,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$101,$A11,Matriz!$L$2:$L$101,"En diseño")</f>
         <v/>
       </c>
       <c r="E11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$100,$A11,Matriz!$L$2:$L$100,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$101,$A11,Matriz!$L$2:$L$101,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$100,$A11,Matriz!$L$2:$L$100,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$101,$A11,Matriz!$L$2:$L$101,"En pruebas")</f>
         <v/>
       </c>
       <c r="G11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$100,$A11,Matriz!$L$2:$L$100,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$101,$A11,Matriz!$L$2:$L$101,"Hecho")</f>
         <v/>
       </c>
       <c r="H11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$100,$A11,Matriz!$L$2:$L$100,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$101,$A11,Matriz!$L$2:$L$101,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I11" s="13">
@@ -1256,31 +1256,31 @@
         </is>
       </c>
       <c r="B16" s="12">
-        <f>COUNTIF(Matriz!$H$2:$H$100,$A16)</f>
+        <f>COUNTIF(Matriz!$H$2:$H$101,$A16)</f>
         <v/>
       </c>
       <c r="C16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$100,$A16,Matriz!$L$2:$L$100,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$101,$A16,Matriz!$L$2:$L$101,"Pendiente")</f>
         <v/>
       </c>
       <c r="D16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$100,$A16,Matriz!$L$2:$L$100,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$101,$A16,Matriz!$L$2:$L$101,"En diseño")</f>
         <v/>
       </c>
       <c r="E16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$100,$A16,Matriz!$L$2:$L$100,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$101,$A16,Matriz!$L$2:$L$101,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$100,$A16,Matriz!$L$2:$L$100,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$101,$A16,Matriz!$L$2:$L$101,"En pruebas")</f>
         <v/>
       </c>
       <c r="G16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$100,$A16,Matriz!$L$2:$L$100,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$101,$A16,Matriz!$L$2:$L$101,"Hecho")</f>
         <v/>
       </c>
       <c r="H16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$100,$A16,Matriz!$L$2:$L$100,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$101,$A16,Matriz!$L$2:$L$101,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I16" s="13">
@@ -1295,31 +1295,31 @@
         </is>
       </c>
       <c r="B17" s="12">
-        <f>COUNTIF(Matriz!$H$2:$H$100,$A17)</f>
+        <f>COUNTIF(Matriz!$H$2:$H$101,$A17)</f>
         <v/>
       </c>
       <c r="C17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$100,$A17,Matriz!$L$2:$L$100,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$101,$A17,Matriz!$L$2:$L$101,"Pendiente")</f>
         <v/>
       </c>
       <c r="D17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$100,$A17,Matriz!$L$2:$L$100,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$101,$A17,Matriz!$L$2:$L$101,"En diseño")</f>
         <v/>
       </c>
       <c r="E17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$100,$A17,Matriz!$L$2:$L$100,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$101,$A17,Matriz!$L$2:$L$101,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$100,$A17,Matriz!$L$2:$L$100,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$101,$A17,Matriz!$L$2:$L$101,"En pruebas")</f>
         <v/>
       </c>
       <c r="G17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$100,$A17,Matriz!$L$2:$L$100,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$101,$A17,Matriz!$L$2:$L$101,"Hecho")</f>
         <v/>
       </c>
       <c r="H17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$100,$A17,Matriz!$L$2:$L$100,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$101,$A17,Matriz!$L$2:$L$101,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I17" s="13">
@@ -1334,31 +1334,31 @@
         </is>
       </c>
       <c r="B18" s="12">
-        <f>COUNTIF(Matriz!$H$2:$H$100,$A18)</f>
+        <f>COUNTIF(Matriz!$H$2:$H$101,$A18)</f>
         <v/>
       </c>
       <c r="C18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$100,$A18,Matriz!$L$2:$L$100,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$101,$A18,Matriz!$L$2:$L$101,"Pendiente")</f>
         <v/>
       </c>
       <c r="D18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$100,$A18,Matriz!$L$2:$L$100,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$101,$A18,Matriz!$L$2:$L$101,"En diseño")</f>
         <v/>
       </c>
       <c r="E18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$100,$A18,Matriz!$L$2:$L$100,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$101,$A18,Matriz!$L$2:$L$101,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$100,$A18,Matriz!$L$2:$L$100,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$101,$A18,Matriz!$L$2:$L$101,"En pruebas")</f>
         <v/>
       </c>
       <c r="G18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$100,$A18,Matriz!$L$2:$L$100,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$101,$A18,Matriz!$L$2:$L$101,"Hecho")</f>
         <v/>
       </c>
       <c r="H18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$100,$A18,Matriz!$L$2:$L$100,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$101,$A18,Matriz!$L$2:$L$101,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I18" s="13">
@@ -1373,31 +1373,31 @@
         </is>
       </c>
       <c r="B19" s="12">
-        <f>COUNTIF(Matriz!$H$2:$H$100,$A19)</f>
+        <f>COUNTIF(Matriz!$H$2:$H$101,$A19)</f>
         <v/>
       </c>
       <c r="C19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$100,$A19,Matriz!$L$2:$L$100,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$101,$A19,Matriz!$L$2:$L$101,"Pendiente")</f>
         <v/>
       </c>
       <c r="D19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$100,$A19,Matriz!$L$2:$L$100,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$101,$A19,Matriz!$L$2:$L$101,"En diseño")</f>
         <v/>
       </c>
       <c r="E19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$100,$A19,Matriz!$L$2:$L$100,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$101,$A19,Matriz!$L$2:$L$101,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$100,$A19,Matriz!$L$2:$L$100,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$101,$A19,Matriz!$L$2:$L$101,"En pruebas")</f>
         <v/>
       </c>
       <c r="G19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$100,$A19,Matriz!$L$2:$L$100,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$101,$A19,Matriz!$L$2:$L$101,"Hecho")</f>
         <v/>
       </c>
       <c r="H19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$100,$A19,Matriz!$L$2:$L$100,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$101,$A19,Matriz!$L$2:$L$101,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I19" s="13">
@@ -1498,31 +1498,31 @@
         </is>
       </c>
       <c r="B24" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$100,$A24)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$101,$A24)</f>
         <v/>
       </c>
       <c r="C24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$100,$A24,Matriz!$L$2:$L$100,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$101,$A24,Matriz!$L$2:$L$101,"Pendiente")</f>
         <v/>
       </c>
       <c r="D24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$100,$A24,Matriz!$L$2:$L$100,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$101,$A24,Matriz!$L$2:$L$101,"En diseño")</f>
         <v/>
       </c>
       <c r="E24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$100,$A24,Matriz!$L$2:$L$100,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$101,$A24,Matriz!$L$2:$L$101,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$100,$A24,Matriz!$L$2:$L$100,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$101,$A24,Matriz!$L$2:$L$101,"En pruebas")</f>
         <v/>
       </c>
       <c r="G24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$100,$A24,Matriz!$L$2:$L$100,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$101,$A24,Matriz!$L$2:$L$101,"Hecho")</f>
         <v/>
       </c>
       <c r="H24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$100,$A24,Matriz!$L$2:$L$100,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$101,$A24,Matriz!$L$2:$L$101,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I24" s="13">
@@ -1537,31 +1537,31 @@
         </is>
       </c>
       <c r="B25" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$100,$A25)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$101,$A25)</f>
         <v/>
       </c>
       <c r="C25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$100,$A25,Matriz!$L$2:$L$100,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$101,$A25,Matriz!$L$2:$L$101,"Pendiente")</f>
         <v/>
       </c>
       <c r="D25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$100,$A25,Matriz!$L$2:$L$100,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$101,$A25,Matriz!$L$2:$L$101,"En diseño")</f>
         <v/>
       </c>
       <c r="E25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$100,$A25,Matriz!$L$2:$L$100,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$101,$A25,Matriz!$L$2:$L$101,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$100,$A25,Matriz!$L$2:$L$100,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$101,$A25,Matriz!$L$2:$L$101,"En pruebas")</f>
         <v/>
       </c>
       <c r="G25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$100,$A25,Matriz!$L$2:$L$100,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$101,$A25,Matriz!$L$2:$L$101,"Hecho")</f>
         <v/>
       </c>
       <c r="H25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$100,$A25,Matriz!$L$2:$L$100,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$101,$A25,Matriz!$L$2:$L$101,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I25" s="13">
@@ -1576,31 +1576,31 @@
         </is>
       </c>
       <c r="B26" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$100,$A26)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$101,$A26)</f>
         <v/>
       </c>
       <c r="C26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$100,$A26,Matriz!$L$2:$L$100,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$101,$A26,Matriz!$L$2:$L$101,"Pendiente")</f>
         <v/>
       </c>
       <c r="D26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$100,$A26,Matriz!$L$2:$L$100,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$101,$A26,Matriz!$L$2:$L$101,"En diseño")</f>
         <v/>
       </c>
       <c r="E26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$100,$A26,Matriz!$L$2:$L$100,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$101,$A26,Matriz!$L$2:$L$101,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$100,$A26,Matriz!$L$2:$L$100,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$101,$A26,Matriz!$L$2:$L$101,"En pruebas")</f>
         <v/>
       </c>
       <c r="G26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$100,$A26,Matriz!$L$2:$L$100,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$101,$A26,Matriz!$L$2:$L$101,"Hecho")</f>
         <v/>
       </c>
       <c r="H26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$100,$A26,Matriz!$L$2:$L$100,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$101,$A26,Matriz!$L$2:$L$101,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I26" s="13">
@@ -1615,31 +1615,31 @@
         </is>
       </c>
       <c r="B27" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$100,$A27)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$101,$A27)</f>
         <v/>
       </c>
       <c r="C27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$100,$A27,Matriz!$L$2:$L$100,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$101,$A27,Matriz!$L$2:$L$101,"Pendiente")</f>
         <v/>
       </c>
       <c r="D27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$100,$A27,Matriz!$L$2:$L$100,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$101,$A27,Matriz!$L$2:$L$101,"En diseño")</f>
         <v/>
       </c>
       <c r="E27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$100,$A27,Matriz!$L$2:$L$100,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$101,$A27,Matriz!$L$2:$L$101,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$100,$A27,Matriz!$L$2:$L$100,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$101,$A27,Matriz!$L$2:$L$101,"En pruebas")</f>
         <v/>
       </c>
       <c r="G27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$100,$A27,Matriz!$L$2:$L$100,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$101,$A27,Matriz!$L$2:$L$101,"Hecho")</f>
         <v/>
       </c>
       <c r="H27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$100,$A27,Matriz!$L$2:$L$100,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$101,$A27,Matriz!$L$2:$L$101,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I27" s="13">
@@ -1654,31 +1654,31 @@
         </is>
       </c>
       <c r="B28" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$100,$A28)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$101,$A28)</f>
         <v/>
       </c>
       <c r="C28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$100,$A28,Matriz!$L$2:$L$100,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$101,$A28,Matriz!$L$2:$L$101,"Pendiente")</f>
         <v/>
       </c>
       <c r="D28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$100,$A28,Matriz!$L$2:$L$100,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$101,$A28,Matriz!$L$2:$L$101,"En diseño")</f>
         <v/>
       </c>
       <c r="E28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$100,$A28,Matriz!$L$2:$L$100,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$101,$A28,Matriz!$L$2:$L$101,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$100,$A28,Matriz!$L$2:$L$100,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$101,$A28,Matriz!$L$2:$L$101,"En pruebas")</f>
         <v/>
       </c>
       <c r="G28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$100,$A28,Matriz!$L$2:$L$100,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$101,$A28,Matriz!$L$2:$L$101,"Hecho")</f>
         <v/>
       </c>
       <c r="H28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$100,$A28,Matriz!$L$2:$L$100,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$101,$A28,Matriz!$L$2:$L$101,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I28" s="13">
@@ -1693,31 +1693,31 @@
         </is>
       </c>
       <c r="B29" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$100,$A29)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$101,$A29)</f>
         <v/>
       </c>
       <c r="C29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$100,$A29,Matriz!$L$2:$L$100,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$101,$A29,Matriz!$L$2:$L$101,"Pendiente")</f>
         <v/>
       </c>
       <c r="D29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$100,$A29,Matriz!$L$2:$L$100,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$101,$A29,Matriz!$L$2:$L$101,"En diseño")</f>
         <v/>
       </c>
       <c r="E29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$100,$A29,Matriz!$L$2:$L$100,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$101,$A29,Matriz!$L$2:$L$101,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$100,$A29,Matriz!$L$2:$L$100,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$101,$A29,Matriz!$L$2:$L$101,"En pruebas")</f>
         <v/>
       </c>
       <c r="G29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$100,$A29,Matriz!$L$2:$L$100,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$101,$A29,Matriz!$L$2:$L$101,"Hecho")</f>
         <v/>
       </c>
       <c r="H29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$100,$A29,Matriz!$L$2:$L$100,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$101,$A29,Matriz!$L$2:$L$101,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I29" s="13">
@@ -1732,31 +1732,31 @@
         </is>
       </c>
       <c r="B30" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$100,$A30)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$101,$A30)</f>
         <v/>
       </c>
       <c r="C30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$100,$A30,Matriz!$L$2:$L$100,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$101,$A30,Matriz!$L$2:$L$101,"Pendiente")</f>
         <v/>
       </c>
       <c r="D30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$100,$A30,Matriz!$L$2:$L$100,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$101,$A30,Matriz!$L$2:$L$101,"En diseño")</f>
         <v/>
       </c>
       <c r="E30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$100,$A30,Matriz!$L$2:$L$100,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$101,$A30,Matriz!$L$2:$L$101,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$100,$A30,Matriz!$L$2:$L$100,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$101,$A30,Matriz!$L$2:$L$101,"En pruebas")</f>
         <v/>
       </c>
       <c r="G30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$100,$A30,Matriz!$L$2:$L$100,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$101,$A30,Matriz!$L$2:$L$101,"Hecho")</f>
         <v/>
       </c>
       <c r="H30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$100,$A30,Matriz!$L$2:$L$100,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$101,$A30,Matriz!$L$2:$L$101,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I30" s="13">
@@ -1818,7 +1818,7 @@
         </is>
       </c>
       <c r="B35" s="12">
-        <f>COUNTIF(Matriz!$K$2:$K$100,A35)</f>
+        <f>COUNTIF(Matriz!$K$2:$K$101,A35)</f>
         <v/>
       </c>
     </row>
@@ -1829,7 +1829,7 @@
         </is>
       </c>
       <c r="B36" s="12">
-        <f>COUNTIF(Matriz!$K$2:$K$100,A36)</f>
+        <f>COUNTIF(Matriz!$K$2:$K$101,A36)</f>
         <v/>
       </c>
     </row>
@@ -1840,7 +1840,7 @@
         </is>
       </c>
       <c r="B37" s="12">
-        <f>COUNTIF(Matriz!$K$2:$K$100,A37)</f>
+        <f>COUNTIF(Matriz!$K$2:$K$101,A37)</f>
         <v/>
       </c>
     </row>
@@ -1851,7 +1851,7 @@
         </is>
       </c>
       <c r="B38" s="12">
-        <f>COUNTIF(Matriz!$K$2:$K$100,A38)</f>
+        <f>COUNTIF(Matriz!$K$2:$K$101,A38)</f>
         <v/>
       </c>
     </row>
@@ -1866,7 +1866,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N100"/>
+  <dimension ref="A1:N101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4008,52 +4008,52 @@
     <row r="32">
       <c r="A32" s="18" t="inlineStr">
         <is>
-          <t>M2A-01</t>
+          <t>M1-25</t>
         </is>
       </c>
       <c r="B32" s="19" t="inlineStr">
         <is>
-          <t>M2A Cursos de Vida</t>
+          <t>M1 Identidad y comunicación</t>
         </is>
       </c>
       <c r="C32" s="19" t="inlineStr">
         <is>
-          <t>Catálogo dinámico de cursos; se pueden crear nuevos sin intervención técnica. Incluye «Resolución de Varones» y «Toma de Buenas Decisiones», omitidos en v2.</t>
-        </is>
-      </c>
-      <c r="D32" s="22" t="inlineStr">
-        <is>
-          <t>Recuperado v1</t>
+          <t>Unidades: áreas de servicio de la iglesia (cafetería, librería, niños, danza, etc.), cada una con encargado, respaldo y servidores. Quien participa en una unidad ve solo esa unidad, y su rol vale únicamente dentro de ella, independiente de sus roles en grupos u otras unidades. Cada unidad tiene su propio tablero de avisos.</t>
+        </is>
+      </c>
+      <c r="D32" s="21" t="inlineStr">
+        <is>
+          <t>Respuesta v3.20</t>
         </is>
       </c>
       <c r="E32" s="19" t="inlineStr">
         <is>
-          <t>Fuera del MVP</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="F32" s="19" t="inlineStr">
         <is>
-          <t>Fase 3</t>
+          <t>Fase 0</t>
         </is>
       </c>
       <c r="G32" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sprint 5</t>
         </is>
       </c>
       <c r="H32" s="19" t="inlineStr">
         <is>
-          <t>Posterior</t>
-        </is>
-      </c>
-      <c r="I32" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
-        </is>
-      </c>
-      <c r="J32" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
+          <t>H2 · Fase 0 completa</t>
+        </is>
+      </c>
+      <c r="I32" s="19" t="inlineStr">
+        <is>
+          <t>Como encargado de una unidad quiero administrar a mi gente y mis avisos sin ver lo de otras unidades ni grupos.</t>
+        </is>
+      </c>
+      <c r="J32" s="19" t="inlineStr">
+        <is>
+          <t>Un encargado de la cafetería no ve la librería; el mismo encargado como asistente de un grupo no gestiona ese grupo; un servidor no agrega integrantes.</t>
         </is>
       </c>
       <c r="K32" s="19" t="inlineStr">
@@ -4063,16 +4063,24 @@
       </c>
       <c r="L32" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M32" s="19" t="inlineStr"/>
-      <c r="N32" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M32" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/paso-7-unidades-avisos · pruebas de backend y 103 de frontend pasan; lint, estilos y compilación limpios</t>
+        </is>
+      </c>
+      <c r="N32" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-29 · Unidades con encargado, respaldo y servidores, alcance propio por unidad y tablero de avisos. Los roles de unidad son fijos; falta moverlos a la matriz de permisos.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="18" t="inlineStr">
         <is>
-          <t>M2A-02</t>
+          <t>M2A-01</t>
         </is>
       </c>
       <c r="B33" s="19" t="inlineStr">
@@ -4082,12 +4090,12 @@
       </c>
       <c r="C33" s="19" t="inlineStr">
         <is>
-          <t>Flexibilidad operativa: sin día ni horario fijo; el día y el ponente pueden cambiar entre ediciones.</t>
-        </is>
-      </c>
-      <c r="D33" s="19" t="inlineStr">
-        <is>
-          <t>v1 / v2</t>
+          <t>Catálogo dinámico de cursos; se pueden crear nuevos sin intervención técnica. Incluye «Resolución de Varones» y «Toma de Buenas Decisiones», omitidos en v2.</t>
+        </is>
+      </c>
+      <c r="D33" s="22" t="inlineStr">
+        <is>
+          <t>Recuperado v1</t>
         </is>
       </c>
       <c r="E33" s="19" t="inlineStr">
@@ -4136,7 +4144,7 @@
     <row r="34">
       <c r="A34" s="18" t="inlineStr">
         <is>
-          <t>M2A-03</t>
+          <t>M2A-02</t>
         </is>
       </c>
       <c r="B34" s="19" t="inlineStr">
@@ -4146,7 +4154,7 @@
       </c>
       <c r="C34" s="19" t="inlineStr">
         <is>
-          <t>Reposición de clases: el inscrito puede reponer en otro grupo o con otro ponente, a decisión de quien imparte.</t>
+          <t>Flexibilidad operativa: sin día ni horario fijo; el día y el ponente pueden cambiar entre ediciones.</t>
         </is>
       </c>
       <c r="D34" s="19" t="inlineStr">
@@ -4200,7 +4208,7 @@
     <row r="35">
       <c r="A35" s="18" t="inlineStr">
         <is>
-          <t>M2A-04</t>
+          <t>M2A-03</t>
         </is>
       </c>
       <c r="B35" s="19" t="inlineStr">
@@ -4210,7 +4218,7 @@
       </c>
       <c r="C35" s="19" t="inlineStr">
         <is>
-          <t>Registro de asistencia por sesión.</t>
+          <t>Reposición de clases: el inscrito puede reponer en otro grupo o con otro ponente, a decisión de quien imparte.</t>
         </is>
       </c>
       <c r="D35" s="19" t="inlineStr">
@@ -4264,7 +4272,7 @@
     <row r="36">
       <c r="A36" s="18" t="inlineStr">
         <is>
-          <t>M2A-05</t>
+          <t>M2A-04</t>
         </is>
       </c>
       <c r="B36" s="19" t="inlineStr">
@@ -4274,7 +4282,7 @@
       </c>
       <c r="C36" s="19" t="inlineStr">
         <is>
-          <t>Seguimiento de tareas o actividades opcionales (no sumativas).</t>
+          <t>Registro de asistencia por sesión.</t>
         </is>
       </c>
       <c r="D36" s="19" t="inlineStr">
@@ -4328,7 +4336,7 @@
     <row r="37">
       <c r="A37" s="18" t="inlineStr">
         <is>
-          <t>M2A-06</t>
+          <t>M2A-05</t>
         </is>
       </c>
       <c r="B37" s="19" t="inlineStr">
@@ -4338,7 +4346,7 @@
       </c>
       <c r="C37" s="19" t="inlineStr">
         <is>
-          <t>Inscripción: quién se inscribe, cuándo lo hizo, si tiene adeudo y qué incluye el costo (materiales, hospedaje, etc.).</t>
+          <t>Seguimiento de tareas o actividades opcionales (no sumativas).</t>
         </is>
       </c>
       <c r="D37" s="19" t="inlineStr">
@@ -4392,7 +4400,7 @@
     <row r="38">
       <c r="A38" s="18" t="inlineStr">
         <is>
-          <t>M2A-07</t>
+          <t>M2A-06</t>
         </is>
       </c>
       <c r="B38" s="19" t="inlineStr">
@@ -4402,12 +4410,12 @@
       </c>
       <c r="C38" s="19" t="inlineStr">
         <is>
-          <t>Registro de pagos, saldo de adeudos y recibo. Por definir: captura manual vs. pasarela de pago, y si se requiere corte de caja.</t>
-        </is>
-      </c>
-      <c r="D38" s="21" t="inlineStr">
-        <is>
-          <t>Nuevo v3</t>
+          <t>Inscripción: quién se inscribe, cuándo lo hizo, si tiene adeudo y qué incluye el costo (materiales, hospedaje, etc.).</t>
+        </is>
+      </c>
+      <c r="D38" s="19" t="inlineStr">
+        <is>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E38" s="19" t="inlineStr">
@@ -4442,7 +4450,7 @@
       </c>
       <c r="K38" s="19" t="inlineStr">
         <is>
-          <t>Por definir</t>
+          <t>VoBo pendiente</t>
         </is>
       </c>
       <c r="L38" s="19" t="inlineStr">
@@ -4456,7 +4464,7 @@
     <row r="39">
       <c r="A39" s="18" t="inlineStr">
         <is>
-          <t>M2A-08</t>
+          <t>M2A-07</t>
         </is>
       </c>
       <c r="B39" s="19" t="inlineStr">
@@ -4466,12 +4474,12 @@
       </c>
       <c r="C39" s="19" t="inlineStr">
         <is>
-          <t>Tablero del curso tipo mensajería para avisos antes del curso y días posteriores, con notificación a los inscritos.</t>
-        </is>
-      </c>
-      <c r="D39" s="22" t="inlineStr">
-        <is>
-          <t>Recuperado v1</t>
+          <t>Registro de pagos, saldo de adeudos y recibo. Por definir: captura manual vs. pasarela de pago, y si se requiere corte de caja.</t>
+        </is>
+      </c>
+      <c r="D39" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3</t>
         </is>
       </c>
       <c r="E39" s="19" t="inlineStr">
@@ -4506,7 +4514,7 @@
       </c>
       <c r="K39" s="19" t="inlineStr">
         <is>
-          <t>VoBo pendiente</t>
+          <t>Por definir</t>
         </is>
       </c>
       <c r="L39" s="19" t="inlineStr">
@@ -4520,7 +4528,7 @@
     <row r="40">
       <c r="A40" s="18" t="inlineStr">
         <is>
-          <t>M2A-09</t>
+          <t>M2A-08</t>
         </is>
       </c>
       <c r="B40" s="19" t="inlineStr">
@@ -4530,12 +4538,12 @@
       </c>
       <c r="C40" s="19" t="inlineStr">
         <is>
-          <t>Evaluación docente configurable: formulario diseñable (tipo Google Forms) aplicado al finalizar el curso.</t>
-        </is>
-      </c>
-      <c r="D40" s="19" t="inlineStr">
-        <is>
-          <t>v1 / v2</t>
+          <t>Tablero del curso tipo mensajería para avisos antes del curso y días posteriores, con notificación a los inscritos.</t>
+        </is>
+      </c>
+      <c r="D40" s="22" t="inlineStr">
+        <is>
+          <t>Recuperado v1</t>
         </is>
       </c>
       <c r="E40" s="19" t="inlineStr">
@@ -4584,7 +4592,7 @@
     <row r="41">
       <c r="A41" s="18" t="inlineStr">
         <is>
-          <t>M2A-10</t>
+          <t>M2A-09</t>
         </is>
       </c>
       <c r="B41" s="19" t="inlineStr">
@@ -4594,12 +4602,12 @@
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>Evolución del ponente: historial de evaluaciones por ponente a lo largo del tiempo y entre ediciones.</t>
-        </is>
-      </c>
-      <c r="D41" s="22" t="inlineStr">
-        <is>
-          <t>Recuperado v1</t>
+          <t>Evaluación docente configurable: formulario diseñable (tipo Google Forms) aplicado al finalizar el curso.</t>
+        </is>
+      </c>
+      <c r="D41" s="19" t="inlineStr">
+        <is>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E41" s="19" t="inlineStr">
@@ -4648,7 +4656,7 @@
     <row r="42">
       <c r="A42" s="18" t="inlineStr">
         <is>
-          <t>M2A-11</t>
+          <t>M2A-10</t>
         </is>
       </c>
       <c r="B42" s="19" t="inlineStr">
@@ -4658,12 +4666,12 @@
       </c>
       <c r="C42" s="19" t="inlineStr">
         <is>
-          <t>Reconocimiento de participación (diploma) opcional por curso.</t>
-        </is>
-      </c>
-      <c r="D42" s="19" t="inlineStr">
-        <is>
-          <t>v1 / v2</t>
+          <t>Evolución del ponente: historial de evaluaciones por ponente a lo largo del tiempo y entre ediciones.</t>
+        </is>
+      </c>
+      <c r="D42" s="22" t="inlineStr">
+        <is>
+          <t>Recuperado v1</t>
         </is>
       </c>
       <c r="E42" s="19" t="inlineStr">
@@ -4712,17 +4720,17 @@
     <row r="43">
       <c r="A43" s="18" t="inlineStr">
         <is>
-          <t>M2B-01</t>
+          <t>M2A-11</t>
         </is>
       </c>
       <c r="B43" s="19" t="inlineStr">
         <is>
-          <t>M2B Cursos escolarizados</t>
+          <t>M2A Cursos de Vida</t>
         </is>
       </c>
       <c r="C43" s="19" t="inlineStr">
         <is>
-          <t>Control riguroso de asistencia.</t>
+          <t>Reconocimiento de participación (diploma) opcional por curso.</t>
         </is>
       </c>
       <c r="D43" s="19" t="inlineStr">
@@ -4776,7 +4784,7 @@
     <row r="44">
       <c r="A44" s="18" t="inlineStr">
         <is>
-          <t>M2B-02</t>
+          <t>M2B-01</t>
         </is>
       </c>
       <c r="B44" s="19" t="inlineStr">
@@ -4786,7 +4794,7 @@
       </c>
       <c r="C44" s="19" t="inlineStr">
         <is>
-          <t>Entrega de tareas y trabajos continuos (incluidos trabajos extra).</t>
+          <t>Control riguroso de asistencia.</t>
         </is>
       </c>
       <c r="D44" s="19" t="inlineStr">
@@ -4840,7 +4848,7 @@
     <row r="45">
       <c r="A45" s="18" t="inlineStr">
         <is>
-          <t>M2B-03</t>
+          <t>M2B-02</t>
         </is>
       </c>
       <c r="B45" s="19" t="inlineStr">
@@ -4850,7 +4858,7 @@
       </c>
       <c r="C45" s="19" t="inlineStr">
         <is>
-          <t>Ponderación de calificaciones y exámenes finales.</t>
+          <t>Entrega de tareas y trabajos continuos (incluidos trabajos extra).</t>
         </is>
       </c>
       <c r="D45" s="19" t="inlineStr">
@@ -4904,7 +4912,7 @@
     <row r="46">
       <c r="A46" s="18" t="inlineStr">
         <is>
-          <t>M2B-04</t>
+          <t>M2B-03</t>
         </is>
       </c>
       <c r="B46" s="19" t="inlineStr">
@@ -4914,12 +4922,12 @@
       </c>
       <c r="C46" s="19" t="inlineStr">
         <is>
-          <t>Creador de exámenes en línea: opción múltiple, preguntas abiertas, falso/verdadero y respuesta corta.</t>
+          <t>Ponderación de calificaciones y exámenes finales.</t>
         </is>
       </c>
       <c r="D46" s="19" t="inlineStr">
         <is>
-          <t>v2</t>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E46" s="19" t="inlineStr">
@@ -4968,7 +4976,7 @@
     <row r="47">
       <c r="A47" s="18" t="inlineStr">
         <is>
-          <t>M2B-05</t>
+          <t>M2B-04</t>
         </is>
       </c>
       <c r="B47" s="19" t="inlineStr">
@@ -4978,12 +4986,12 @@
       </c>
       <c r="C47" s="19" t="inlineStr">
         <is>
-          <t>Boleta digital con el formato definido por la iglesia. Por definir: formato oficial de la boleta.</t>
+          <t>Creador de exámenes en línea: opción múltiple, preguntas abiertas, falso/verdadero y respuesta corta.</t>
         </is>
       </c>
       <c r="D47" s="19" t="inlineStr">
         <is>
-          <t>v1 / v2</t>
+          <t>v2</t>
         </is>
       </c>
       <c r="E47" s="19" t="inlineStr">
@@ -5018,7 +5026,7 @@
       </c>
       <c r="K47" s="19" t="inlineStr">
         <is>
-          <t>Por definir</t>
+          <t>VoBo pendiente</t>
         </is>
       </c>
       <c r="L47" s="19" t="inlineStr">
@@ -5032,7 +5040,7 @@
     <row r="48">
       <c r="A48" s="18" t="inlineStr">
         <is>
-          <t>M2B-06</t>
+          <t>M2B-05</t>
         </is>
       </c>
       <c r="B48" s="19" t="inlineStr">
@@ -5042,12 +5050,12 @@
       </c>
       <c r="C48" s="19" t="inlineStr">
         <is>
-          <t>Historial académico permanente en el Expediente Digital, aunque cambie el maestro o el alumno pierda su comprobante.</t>
+          <t>Boleta digital con el formato definido por la iglesia. Por definir: formato oficial de la boleta.</t>
         </is>
       </c>
       <c r="D48" s="19" t="inlineStr">
         <is>
-          <t>v2</t>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E48" s="19" t="inlineStr">
@@ -5082,7 +5090,7 @@
       </c>
       <c r="K48" s="19" t="inlineStr">
         <is>
-          <t>VoBo pendiente</t>
+          <t>Por definir</t>
         </is>
       </c>
       <c r="L48" s="19" t="inlineStr">
@@ -5096,52 +5104,52 @@
     <row r="49">
       <c r="A49" s="18" t="inlineStr">
         <is>
-          <t>M3-01</t>
+          <t>M2B-06</t>
         </is>
       </c>
       <c r="B49" s="19" t="inlineStr">
         <is>
-          <t>M3 Grupos de Conexión</t>
+          <t>M2B Cursos escolarizados</t>
         </is>
       </c>
       <c r="C49" s="19" t="inlineStr">
         <is>
-          <t>Estructura del grupo con roles: Supervisor (supervisa uno o varios grupos y reporta al Pastor), Líder, Secretario, Anfitrión y Tesorero.</t>
+          <t>Historial académico permanente en el Expediente Digital, aunque cambie el maestro o el alumno pierda su comprobante.</t>
         </is>
       </c>
       <c r="D49" s="19" t="inlineStr">
         <is>
-          <t>v3 + Obs. 4</t>
+          <t>v2</t>
         </is>
       </c>
       <c r="E49" s="19" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Fuera del MVP</t>
         </is>
       </c>
       <c r="F49" s="19" t="inlineStr">
         <is>
-          <t>Fase 1</t>
+          <t>Fase 3</t>
         </is>
       </c>
       <c r="G49" s="19" t="inlineStr">
         <is>
-          <t>Sprint 3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H49" s="19" t="inlineStr">
         <is>
-          <t>H3 · MVP (Grupos)</t>
-        </is>
-      </c>
-      <c r="I49" s="19" t="inlineStr">
-        <is>
-          <t>Como supervisor quiero asignar Líder, Secretario, Anfitrión y Tesorero a cada grupo.</t>
-        </is>
-      </c>
-      <c r="J49" s="19" t="inlineStr">
-        <is>
-          <t>Un grupo tiene sus roles asignados; un supervisor ve varios grupos.</t>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="I49" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
+        </is>
+      </c>
+      <c r="J49" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
         </is>
       </c>
       <c r="K49" s="19" t="inlineStr">
@@ -5151,24 +5159,16 @@
       </c>
       <c r="L49" s="19" t="inlineStr">
         <is>
-          <t>En pruebas</t>
-        </is>
-      </c>
-      <c r="M49" s="19" t="inlineStr">
-        <is>
-          <t>Rama feature/grupos-paso-3 · pruebas de backend y 81 de frontend pasan; lint, estilos y compilación limpios</t>
-        </is>
-      </c>
-      <c r="N49" s="19" t="inlineStr">
-        <is>
-          <t>2026-10-27 · Supervisor, Líder, Secretario, Anfitrión, Tesorero y Asistente por grupo; ahora con cambio de rol, sector (letra), casa (número) y suspensión con motivo.</t>
-        </is>
-      </c>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M49" s="19" t="inlineStr"/>
+      <c r="N49" s="19" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="18" t="inlineStr">
         <is>
-          <t>M3-02</t>
+          <t>M3-01</t>
         </is>
       </c>
       <c r="B50" s="19" t="inlineStr">
@@ -5178,12 +5178,12 @@
       </c>
       <c r="C50" s="19" t="inlineStr">
         <is>
-          <t>Estudio semanal dentro de la app: un registro por semana con PDF para adultos, PDF para niños y audio de la lectura (PDF hasta 15 MB; audio hasta 40 MB). Lo publican Pastor o Anciano y los líderes lo abren desde la reunión, sustituyendo el envío por WhatsApp. El audio admite adelantar y retroceder en iPhone.</t>
+          <t>Estructura del grupo con roles: Supervisor (supervisa uno o varios grupos y reporta al Pastor), Líder, Secretario, Anfitrión y Tesorero.</t>
         </is>
       </c>
       <c r="D50" s="19" t="inlineStr">
         <is>
-          <t>v1 / v2 + Respuesta</t>
+          <t>v3 + Obs. 4</t>
         </is>
       </c>
       <c r="E50" s="19" t="inlineStr">
@@ -5208,12 +5208,12 @@
       </c>
       <c r="I50" s="19" t="inlineStr">
         <is>
-          <t>Como líder quiero recibir el estudio semanal en la app en lugar de WhatsApp.</t>
+          <t>Como supervisor quiero asignar Líder, Secretario, Anfitrión y Tesorero a cada grupo.</t>
         </is>
       </c>
       <c r="J50" s="19" t="inlineStr">
         <is>
-          <t>Publicar el material de la semana; el líder lo abre y queda marca de lectura.</t>
+          <t>Un grupo tiene sus roles asignados; un supervisor ve varios grupos.</t>
         </is>
       </c>
       <c r="K50" s="19" t="inlineStr">
@@ -5228,19 +5228,19 @@
       </c>
       <c r="M50" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/m3-grupos · 88 pruebas de backend y 7 de frontend pasan</t>
+          <t>Rama feature/grupos-paso-3 · pruebas de backend y 81 de frontend pasan; lint, estilos y compilación limpios</t>
         </is>
       </c>
       <c r="N50" s="19" t="inlineStr">
         <is>
-          <t>2026-10-24 · PDF adultos, PDF niños y audio por semana; audio con Range para iPhone. Pendiente probar en iOS.</t>
+          <t>2026-10-27 · Supervisor, Líder, Secretario, Anfitrión, Tesorero y Asistente por grupo; ahora con cambio de rol, sector (letra), casa (número) y suspensión con motivo.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="18" t="inlineStr">
         <is>
-          <t>M3-03</t>
+          <t>M3-02</t>
         </is>
       </c>
       <c r="B51" s="19" t="inlineStr">
@@ -5250,12 +5250,12 @@
       </c>
       <c r="C51" s="19" t="inlineStr">
         <is>
-          <t>Pase de lista digital por Secretario o Líder. El Secretario captura y corrige el mismo día; el Líder modifica siempre; el Supervisor solo consulta. Funciona sin conexión: la lista se guarda en el teléfono con la hora real de captura y se envía sola al volver la señal, sin pisar cambios más recientes hechos en línea. Una captura sin conexión se acepta hasta 7 días después y se evalúa contra el día en que se hizo; todo queda en bitácora marcado como diferido.</t>
+          <t>Estudio semanal dentro de la app: un registro por semana con PDF para adultos, PDF para niños y audio de la lectura (PDF hasta 15 MB; audio hasta 40 MB). Lo publican Pastor o Anciano y los líderes lo abren desde la reunión, sustituyendo el envío por WhatsApp. El audio admite adelantar y retroceder en iPhone.</t>
         </is>
       </c>
       <c r="D51" s="19" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>v1 / v2 + Respuesta</t>
         </is>
       </c>
       <c r="E51" s="19" t="inlineStr">
@@ -5280,12 +5280,12 @@
       </c>
       <c r="I51" s="19" t="inlineStr">
         <is>
-          <t>Como secretario quiero pasar lista aunque no haya señal.</t>
+          <t>Como líder quiero recibir el estudio semanal en la app en lugar de WhatsApp.</t>
         </is>
       </c>
       <c r="J51" s="19" t="inlineStr">
         <is>
-          <t>Pasar lista en modo avión; al reconectar se sincroniza sin duplicados.</t>
+          <t>Publicar el material de la semana; el líder lo abre y queda marca de lectura.</t>
         </is>
       </c>
       <c r="K51" s="19" t="inlineStr">
@@ -5300,19 +5300,19 @@
       </c>
       <c r="M51" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/nf-06-sin-conexion · 117 pruebas de backend y 27 de frontend; probado en Chrome real con service worker</t>
+          <t>Rama feature/m3-grupos · 88 pruebas de backend y 7 de frontend pasan</t>
         </is>
       </c>
       <c r="N51" s="19" t="inlineStr">
         <is>
-          <t>2026-10-24 · Pase de lista con y sin conexión.</t>
+          <t>2026-10-24 · PDF adultos, PDF niños y audio por semana; audio con Range para iPhone. Pendiente probar en iOS.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="18" t="inlineStr">
         <is>
-          <t>M3-04</t>
+          <t>M3-03</t>
         </is>
       </c>
       <c r="B52" s="19" t="inlineStr">
@@ -5322,12 +5322,12 @@
       </c>
       <c r="C52" s="19" t="inlineStr">
         <is>
-          <t>Ofrendas regulares y especiales (con concepto) por reunión, cuantificables. El Secretario captura el monto; si el grupo no tiene Secretario, lo suple el Líder. El Tesorero cuenta, escribe su cifra y avala volviendo a escribir su PIN; si el grupo no tiene Tesorero, avalan el Líder o el Pastor, nunca quien capturó. Si la cifra coincide queda «Avalada»; si no, se registra la diferencia y queda «Con diferencia», con aviso visible en el grupo, la reunión y la pantalla del Tesorero para quien pueda consultar. Una ofrenda ya capturada solo se corrige con motivo y vuelve a pendiente para un nuevo aval. El Pastor consulta todo, el Líder y el Supervisor consultan y el Anciano no ve finanzas. Toda suplencia, captura, aval y corrección queda en bitácora.</t>
+          <t>Pase de lista digital por Secretario o Líder. El Secretario captura y corrige el mismo día; el Líder modifica siempre; el Supervisor solo consulta. Funciona sin conexión: la lista se guarda en el teléfono con la hora real de captura y se envía sola al volver la señal, sin pisar cambios más recientes hechos en línea. Una captura sin conexión se acepta hasta 7 días después y se evalúa contra el día en que se hizo; todo queda en bitácora marcado como diferido.</t>
         </is>
       </c>
       <c r="D52" s="19" t="inlineStr">
         <is>
-          <t>v3 + Obs. 4</t>
+          <t>v3</t>
         </is>
       </c>
       <c r="E52" s="19" t="inlineStr">
@@ -5342,7 +5342,7 @@
       </c>
       <c r="G52" s="19" t="inlineStr">
         <is>
-          <t>Sprint 4</t>
+          <t>Sprint 3</t>
         </is>
       </c>
       <c r="H52" s="19" t="inlineStr">
@@ -5352,12 +5352,12 @@
       </c>
       <c r="I52" s="19" t="inlineStr">
         <is>
-          <t>Como tesorero quiero contar y avalar la ofrenda del grupo.</t>
+          <t>Como secretario quiero pasar lista aunque no haya señal.</t>
         </is>
       </c>
       <c r="J52" s="19" t="inlineStr">
         <is>
-          <t>Capturar monto; el Tesorero captura su cifra y confirma con su PIN; si difiere se registra la diferencia; con aval no se edita sin motivo.</t>
+          <t>Pasar lista en modo avión; al reconectar se sincroniza sin duplicados.</t>
         </is>
       </c>
       <c r="K52" s="19" t="inlineStr">
@@ -5372,19 +5372,19 @@
       </c>
       <c r="M52" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/m3-ofrendas-ajustes · 121 pruebas de backend y 14 de frontend pasan</t>
+          <t>Rama feature/nf-06-sin-conexion · 117 pruebas de backend y 27 de frontend; probado en Chrome real con service worker</t>
         </is>
       </c>
       <c r="N52" s="19" t="inlineStr">
         <is>
-          <t>2026-10-24 · Con suplencias del Líder, diferencias visibles y límites configurables. Falta validar con la iglesia.</t>
+          <t>2026-10-24 · Pase de lista con y sin conexión.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="18" t="inlineStr">
         <is>
-          <t>M3-05</t>
+          <t>M3-04</t>
         </is>
       </c>
       <c r="B53" s="19" t="inlineStr">
@@ -5394,12 +5394,12 @@
       </c>
       <c r="C53" s="19" t="inlineStr">
         <is>
-          <t>Peticiones de oración con formulario configurable (campos que se agregan, desactivan y reordenan sin programar; cada cambio crea una versión y los campos no se borran). Por defecto: petición, quién la pide y categoría. Las registran el Líder y el Secretario, desde la reunión o desde el grupo; el Pastor también.</t>
+          <t>Ofrendas regulares y especiales (con concepto) por reunión, cuantificables. El Secretario captura el monto; si el grupo no tiene Secretario, lo suple el Líder. El Tesorero cuenta, escribe su cifra y avala volviendo a escribir su PIN; si el grupo no tiene Tesorero, avalan el Líder o el Pastor, nunca quien capturó. Si la cifra coincide queda «Avalada»; si no, se registra la diferencia y queda «Con diferencia», con aviso visible en el grupo, la reunión y la pantalla del Tesorero para quien pueda consultar. Una ofrenda ya capturada solo se corrige con motivo y vuelve a pendiente para un nuevo aval. El Pastor consulta todo, el Líder y el Supervisor consultan y el Anciano no ve finanzas. Toda suplencia, captura, aval y corrección queda en bitácora.</t>
         </is>
       </c>
       <c r="D53" s="19" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>v3 + Obs. 4</t>
         </is>
       </c>
       <c r="E53" s="19" t="inlineStr">
@@ -5424,12 +5424,12 @@
       </c>
       <c r="I53" s="19" t="inlineStr">
         <is>
-          <t>Como líder quiero recoger peticiones de oración con un formulario configurable.</t>
+          <t>Como tesorero quiero contar y avalar la ofrenda del grupo.</t>
         </is>
       </c>
       <c r="J53" s="19" t="inlineStr">
         <is>
-          <t>Capturar una petición; el formulario se edita sin código.</t>
+          <t>Capturar monto; el Tesorero captura su cifra y confirma con su PIN; si difiere se registra la diferencia; con aval no se edita sin motivo.</t>
         </is>
       </c>
       <c r="K53" s="19" t="inlineStr">
@@ -5444,19 +5444,19 @@
       </c>
       <c r="M53" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/m3-peticiones-oracion · 166 pruebas de backend y 32 de frontend pasan; probado contra la base real</t>
+          <t>Rama feature/m3-ofrendas-ajustes · 121 pruebas de backend y 14 de frontend pasan</t>
         </is>
       </c>
       <c r="N53" s="19" t="inlineStr">
         <is>
-          <t>2026-10-24 · Formulario configurable y versionado; captura desde la reunión y el grupo.</t>
+          <t>2026-10-24 · Con suplencias del Líder, diferencias visibles y límites configurables. Falta validar con la iglesia.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="18" t="inlineStr">
         <is>
-          <t>M3-06</t>
+          <t>M3-05</t>
         </is>
       </c>
       <c r="B54" s="19" t="inlineStr">
@@ -5466,12 +5466,12 @@
       </c>
       <c r="C54" s="19" t="inlineStr">
         <is>
-          <t>Alcance de lectura de cada petición, elegido por quien la registra con autorización de quien la pide: «Solo líderes» (Líder, Supervisor, Pastor y Anciano), «Mi grupo» (todos los integrantes del grupo y los anteriores) o «Equipo de oración» (además, quien tenga el rol Equipo de oración). El alcance por defecto es configurable. Quien registra siempre ve lo que registró; el Administrador Técnico nunca ve el contenido. Solo líderes y superiores marcan una petición como atendida. Se guardan cifradas y se borran automáticamente a los 30 días, configurable. Consultarlas y atenderlas queda en bitácora sin incluir el texto.</t>
-        </is>
-      </c>
-      <c r="D54" s="21" t="inlineStr">
-        <is>
-          <t>Resp. P8 + Respuesta</t>
+          <t>Peticiones de oración con formulario configurable (campos que se agregan, desactivan y reordenan sin programar; cada cambio crea una versión y los campos no se borran). Por defecto: petición, quién la pide y categoría. Las registran el Líder y el Secretario, desde la reunión o desde el grupo; el Pastor también.</t>
+        </is>
+      </c>
+      <c r="D54" s="19" t="inlineStr">
+        <is>
+          <t>v3</t>
         </is>
       </c>
       <c r="E54" s="19" t="inlineStr">
@@ -5496,12 +5496,12 @@
       </c>
       <c r="I54" s="19" t="inlineStr">
         <is>
-          <t>Como pastor quiero que las peticiones solo las vea el Líder y superiores y se borren al vencer.</t>
+          <t>Como líder quiero recoger peticiones de oración con un formulario configurable.</t>
         </is>
       </c>
       <c r="J54" s="19" t="inlineStr">
         <is>
-          <t>El Secretario no las ve; tras el plazo configurable (por defecto 30 días) se eliminan.</t>
+          <t>Capturar una petición; el formulario se edita sin código.</t>
         </is>
       </c>
       <c r="K54" s="19" t="inlineStr">
@@ -5521,14 +5521,14 @@
       </c>
       <c r="N54" s="19" t="inlineStr">
         <is>
-          <t>2026-10-24 · Alcance por petición (líderes, grupo, equipo), cifrado y borrado a los 30 días configurable. Cambia la matriz aprobada: actualizar con la iglesia.</t>
+          <t>2026-10-24 · Formulario configurable y versionado; captura desde la reunión y el grupo.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="18" t="inlineStr">
         <is>
-          <t>M3-07</t>
+          <t>M3-06</t>
         </is>
       </c>
       <c r="B55" s="19" t="inlineStr">
@@ -5538,17 +5538,17 @@
       </c>
       <c r="C55" s="19" t="inlineStr">
         <is>
-          <t>Dashboard de supervisión («Resumen de grupos») para Supervisor, Líder, Pastor y Anciano sobre los grupos que cada uno puede consultar: asistencia por semana y por grupo, grupos sin lista esta semana, asistencia por debajo de un mínimo configurable (60 % por defecto), ofrendas avaladas, pendientes y con diferencia (solo si el rol ve finanzas) y peticiones activas (solo las que puede leer). No muestra datos de personas. El Secretario y el Tesorero no lo ven.</t>
-        </is>
-      </c>
-      <c r="D55" s="19" t="inlineStr">
-        <is>
-          <t>v3</t>
+          <t>Alcance de lectura de cada petición, elegido por quien la registra con autorización de quien la pide: «Solo líderes» (Líder, Supervisor, Pastor y Anciano), «Mi grupo» (todos los integrantes del grupo y los anteriores) o «Equipo de oración» (además, quien tenga el rol Equipo de oración). El alcance por defecto es configurable. Quien registra siempre ve lo que registró; el Administrador Técnico nunca ve el contenido. Solo líderes y superiores marcan una petición como atendida. Se guardan cifradas y se borran automáticamente a los 30 días, configurable. Consultarlas y atenderlas queda en bitácora sin incluir el texto.</t>
+        </is>
+      </c>
+      <c r="D55" s="21" t="inlineStr">
+        <is>
+          <t>Resp. P8 + Respuesta</t>
         </is>
       </c>
       <c r="E55" s="19" t="inlineStr">
         <is>
-          <t>MVP básico</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="F55" s="19" t="inlineStr">
@@ -5558,7 +5558,7 @@
       </c>
       <c r="G55" s="19" t="inlineStr">
         <is>
-          <t>Sprint 5</t>
+          <t>Sprint 4</t>
         </is>
       </c>
       <c r="H55" s="19" t="inlineStr">
@@ -5568,12 +5568,12 @@
       </c>
       <c r="I55" s="19" t="inlineStr">
         <is>
-          <t>Como supervisor quiero ver la salud de mis grupos.</t>
+          <t>Como pastor quiero que las peticiones solo las vea el Líder y superiores y se borren al vencer.</t>
         </is>
       </c>
       <c r="J55" s="19" t="inlineStr">
         <is>
-          <t>El dashboard muestra asistencia, ofrendas y crecimiento según permisos.</t>
+          <t>El Secretario no las ve; tras el plazo configurable (por defecto 30 días) se eliminan.</t>
         </is>
       </c>
       <c r="K55" s="19" t="inlineStr">
@@ -5588,19 +5588,19 @@
       </c>
       <c r="M55" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/m3-dashboard-tablero · 195 pruebas de backend y 39 de frontend pasan; probado contra la base real</t>
+          <t>Rama feature/m3-peticiones-oracion · 166 pruebas de backend y 32 de frontend pasan; probado contra la base real</t>
         </is>
       </c>
       <c r="N55" s="19" t="inlineStr">
         <is>
-          <t>2026-10-25 · Dashboard con asistencia, avisos y datos según rol; umbral configurable.</t>
+          <t>2026-10-24 · Alcance por petición (líderes, grupo, equipo), cifrado y borrado a los 30 días configurable. Cambia la matriz aprobada: actualizar con la iglesia.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="18" t="inlineStr">
         <is>
-          <t>M3-08</t>
+          <t>M3-07</t>
         </is>
       </c>
       <c r="B56" s="19" t="inlineStr">
@@ -5610,7 +5610,7 @@
       </c>
       <c r="C56" s="19" t="inlineStr">
         <is>
-          <t>Ubicación de zona del grupo para que personas cercanas lo encuentren, sin exponer el domicilio exacto. Por definir.</t>
+          <t>Dashboard de supervisión («Resumen de grupos») para Supervisor, Líder, Pastor y Anciano sobre los grupos que cada uno puede consultar: asistencia por semana y por grupo, grupos sin lista esta semana, asistencia por debajo de un mínimo configurable (60 % por defecto), ofrendas avaladas, pendientes y con diferencia (solo si el rol ve finanzas) y peticiones activas (solo las que puede leer). No muestra datos de personas. El Secretario y el Tesorero no lo ven.</t>
         </is>
       </c>
       <c r="D56" s="19" t="inlineStr">
@@ -5620,51 +5620,59 @@
       </c>
       <c r="E56" s="19" t="inlineStr">
         <is>
-          <t>Fuera del MVP</t>
+          <t>MVP básico</t>
         </is>
       </c>
       <c r="F56" s="19" t="inlineStr">
         <is>
-          <t>Fase 4</t>
+          <t>Fase 1</t>
         </is>
       </c>
       <c r="G56" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sprint 5</t>
         </is>
       </c>
       <c r="H56" s="19" t="inlineStr">
         <is>
-          <t>Posterior</t>
-        </is>
-      </c>
-      <c r="I56" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
-        </is>
-      </c>
-      <c r="J56" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
+          <t>H3 · MVP (Grupos)</t>
+        </is>
+      </c>
+      <c r="I56" s="19" t="inlineStr">
+        <is>
+          <t>Como supervisor quiero ver la salud de mis grupos.</t>
+        </is>
+      </c>
+      <c r="J56" s="19" t="inlineStr">
+        <is>
+          <t>El dashboard muestra asistencia, ofrendas y crecimiento según permisos.</t>
         </is>
       </c>
       <c r="K56" s="19" t="inlineStr">
         <is>
-          <t>Por definir</t>
+          <t>VoBo pendiente</t>
         </is>
       </c>
       <c r="L56" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M56" s="19" t="inlineStr"/>
-      <c r="N56" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M56" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/m3-dashboard-tablero · 195 pruebas de backend y 39 de frontend pasan; probado contra la base real</t>
+        </is>
+      </c>
+      <c r="N56" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-25 · Dashboard con asistencia, avisos y datos según rol; umbral configurable.</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="18" t="inlineStr">
         <is>
-          <t>M3-09</t>
+          <t>M3-08</t>
         </is>
       </c>
       <c r="B57" s="19" t="inlineStr">
@@ -5674,69 +5682,61 @@
       </c>
       <c r="C57" s="19" t="inlineStr">
         <is>
-          <t>A un grupo asisten miembros de la iglesia (vecinos o no) e invitados del grupo que no asisten a la iglesia. Los invitados se registran como Contacto con datos mínimos y se les puede invitar a consolidación.</t>
-        </is>
-      </c>
-      <c r="D57" s="21" t="inlineStr">
-        <is>
-          <t>Corrección v3.2</t>
+          <t>Ubicación de zona del grupo para que personas cercanas lo encuentren, sin exponer el domicilio exacto. Por definir.</t>
+        </is>
+      </c>
+      <c r="D57" s="19" t="inlineStr">
+        <is>
+          <t>v3</t>
         </is>
       </c>
       <c r="E57" s="19" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Fuera del MVP</t>
         </is>
       </c>
       <c r="F57" s="19" t="inlineStr">
         <is>
-          <t>Fase 1</t>
+          <t>Fase 4</t>
         </is>
       </c>
       <c r="G57" s="19" t="inlineStr">
         <is>
-          <t>Sprint 3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H57" s="19" t="inlineStr">
         <is>
-          <t>H3 · MVP (Grupos)</t>
-        </is>
-      </c>
-      <c r="I57" s="19" t="inlineStr">
-        <is>
-          <t>Como secretario quiero registrar invitados del grupo con datos mínimos.</t>
-        </is>
-      </c>
-      <c r="J57" s="19" t="inlineStr">
-        <is>
-          <t>Registrar un invitado como Contacto y marcarlo presente.</t>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="I57" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
+        </is>
+      </c>
+      <c r="J57" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
         </is>
       </c>
       <c r="K57" s="19" t="inlineStr">
         <is>
-          <t>VoBo pendiente</t>
+          <t>Por definir</t>
         </is>
       </c>
       <c r="L57" s="19" t="inlineStr">
         <is>
-          <t>En pruebas</t>
-        </is>
-      </c>
-      <c r="M57" s="19" t="inlineStr">
-        <is>
-          <t>Rama feature/paso-5-invitaciones · pruebas de backend y 93 de frontend pasan; lint, estilos y compilación limpios</t>
-        </is>
-      </c>
-      <c r="N57" s="19" t="inlineStr">
-        <is>
-          <t>2026-10-27 · Los invitados entran al grupo como Contacto cuando el líder aprueba su solicitud por enlace o QR.</t>
-        </is>
-      </c>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M57" s="19" t="inlineStr"/>
+      <c r="N57" s="19" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="18" t="inlineStr">
         <is>
-          <t>M3-10</t>
+          <t>M3-09</t>
         </is>
       </c>
       <c r="B58" s="19" t="inlineStr">
@@ -5746,12 +5746,12 @@
       </c>
       <c r="C58" s="19" t="inlineStr">
         <is>
-          <t>Confidencialidad de ofrendas y asistencias: consulta limitada por rol (matriz por definir) y modificación restringida, todo en bitácora.</t>
+          <t>A un grupo asisten miembros de la iglesia (vecinos o no) e invitados del grupo que no asisten a la iglesia. Los invitados se registran como Contacto con datos mínimos y se les puede invitar a consolidación.</t>
         </is>
       </c>
       <c r="D58" s="21" t="inlineStr">
         <is>
-          <t>Obs. 5</t>
+          <t>Corrección v3.2</t>
         </is>
       </c>
       <c r="E58" s="19" t="inlineStr">
@@ -5766,7 +5766,7 @@
       </c>
       <c r="G58" s="19" t="inlineStr">
         <is>
-          <t>Sprint 4</t>
+          <t>Sprint 3</t>
         </is>
       </c>
       <c r="H58" s="19" t="inlineStr">
@@ -5776,31 +5776,39 @@
       </c>
       <c r="I58" s="19" t="inlineStr">
         <is>
-          <t>Como pastor quiero que ofrendas y asistencias sean confidenciales.</t>
+          <t>Como secretario quiero registrar invitados del grupo con datos mínimos.</t>
         </is>
       </c>
       <c r="J58" s="19" t="inlineStr">
         <is>
-          <t>La matriz de la sección 3.3 del v3.2 se cumple en pruebas por cada rol.</t>
+          <t>Registrar un invitado como Contacto y marcarlo presente.</t>
         </is>
       </c>
       <c r="K58" s="19" t="inlineStr">
         <is>
-          <t>Por definir</t>
+          <t>VoBo pendiente</t>
         </is>
       </c>
       <c r="L58" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M58" s="19" t="inlineStr"/>
-      <c r="N58" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M58" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/paso-5-invitaciones · pruebas de backend y 93 de frontend pasan; lint, estilos y compilación limpios</t>
+        </is>
+      </c>
+      <c r="N58" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-27 · Los invitados entran al grupo como Contacto cuando el líder aprueba su solicitud por enlace o QR.</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="18" t="inlineStr">
         <is>
-          <t>M3-11</t>
+          <t>M3-10</t>
         </is>
       </c>
       <c r="B59" s="19" t="inlineStr">
@@ -5810,12 +5818,12 @@
       </c>
       <c r="C59" s="19" t="inlineStr">
         <is>
-          <t>Tablero de mensajes del grupo: lo publican Líder, Supervisor, Secretario y Pastor; lo leen todos los integrantes activos. Mensajes de hasta 1,000 caracteres, con opción de fijarlos, borrado lógico, contador de mensajes nuevos y conservación configurable (90 días). Pantalla «Avisos» para quien no abre la página del grupo.</t>
+          <t>Confidencialidad de ofrendas y asistencias: consulta limitada por rol (matriz por definir) y modificación restringida, todo en bitácora.</t>
         </is>
       </c>
       <c r="D59" s="21" t="inlineStr">
         <is>
-          <t>Obs. 7</t>
+          <t>Obs. 5</t>
         </is>
       </c>
       <c r="E59" s="19" t="inlineStr">
@@ -5830,7 +5838,7 @@
       </c>
       <c r="G59" s="19" t="inlineStr">
         <is>
-          <t>Sprint 5</t>
+          <t>Sprint 4</t>
         </is>
       </c>
       <c r="H59" s="19" t="inlineStr">
@@ -5840,39 +5848,31 @@
       </c>
       <c r="I59" s="19" t="inlineStr">
         <is>
-          <t>Como líder quiero un tablero de mensajes de mi grupo.</t>
+          <t>Como pastor quiero que ofrendas y asistencias sean confidenciales.</t>
         </is>
       </c>
       <c r="J59" s="19" t="inlineStr">
         <is>
-          <t>Publicar y leer mensajes del grupo.</t>
+          <t>La matriz de la sección 3.3 del v3.2 se cumple en pruebas por cada rol.</t>
         </is>
       </c>
       <c r="K59" s="19" t="inlineStr">
         <is>
-          <t>VoBo pendiente</t>
+          <t>Por definir</t>
         </is>
       </c>
       <c r="L59" s="19" t="inlineStr">
         <is>
-          <t>En pruebas</t>
-        </is>
-      </c>
-      <c r="M59" s="19" t="inlineStr">
-        <is>
-          <t>Rama feature/m3-dashboard-tablero · 195 pruebas de backend y 39 de frontend pasan; probado contra la base real</t>
-        </is>
-      </c>
-      <c r="N59" s="19" t="inlineStr">
-        <is>
-          <t>2026-10-25 · Tablero con fijados, no leídos y retención configurable; la notificación push de mensajes nuevos se entrega con M1-09.</t>
-        </is>
-      </c>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M59" s="19" t="inlineStr"/>
+      <c r="N59" s="19" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="18" t="inlineStr">
         <is>
-          <t>M3-12</t>
+          <t>M3-11</t>
         </is>
       </c>
       <c r="B60" s="19" t="inlineStr">
@@ -5882,12 +5882,12 @@
       </c>
       <c r="C60" s="19" t="inlineStr">
         <is>
-          <t>Reuniones: cada grupo se reúne una vez por semana en casa del líder (día y hora por grupo) y existe una reunión general de líderes, modelada como un grupo de tipo «Líderes».</t>
+          <t>Tablero de mensajes del grupo: lo publican Líder, Supervisor, Secretario y Pastor; lo leen todos los integrantes activos. Mensajes de hasta 1,000 caracteres, con opción de fijarlos, borrado lógico, contador de mensajes nuevos y conservación configurable (90 días). Pantalla «Avisos» para quien no abre la página del grupo.</t>
         </is>
       </c>
       <c r="D60" s="21" t="inlineStr">
         <is>
-          <t>Respuesta</t>
+          <t>Obs. 7</t>
         </is>
       </c>
       <c r="E60" s="19" t="inlineStr">
@@ -5902,7 +5902,7 @@
       </c>
       <c r="G60" s="19" t="inlineStr">
         <is>
-          <t>Sprint 3</t>
+          <t>Sprint 5</t>
         </is>
       </c>
       <c r="H60" s="19" t="inlineStr">
@@ -5910,14 +5910,14 @@
           <t>H3 · MVP (Grupos)</t>
         </is>
       </c>
-      <c r="I60" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
-        </is>
-      </c>
-      <c r="J60" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
+      <c r="I60" s="19" t="inlineStr">
+        <is>
+          <t>Como líder quiero un tablero de mensajes de mi grupo.</t>
+        </is>
+      </c>
+      <c r="J60" s="19" t="inlineStr">
+        <is>
+          <t>Publicar y leer mensajes del grupo.</t>
         </is>
       </c>
       <c r="K60" s="19" t="inlineStr">
@@ -5932,19 +5932,19 @@
       </c>
       <c r="M60" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/grupos-paso-3 · pruebas de backend y 81 de frontend pasan; lint, estilos y compilación limpios</t>
+          <t>Rama feature/m3-dashboard-tablero · 195 pruebas de backend y 39 de frontend pasan; probado contra la base real</t>
         </is>
       </c>
       <c r="N60" s="19" t="inlineStr">
         <is>
-          <t>2026-10-27 · Una reunión semanal por grupo y grupo tipo Líderes; filtros por día, sector, líder y estado; cada reunión muestra su asistencia, observaciones, peticiones y ofrendas.</t>
+          <t>2026-10-25 · Tablero con fijados, no leídos y retención configurable; la notificación push de mensajes nuevos se entrega con M1-09.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="18" t="inlineStr">
         <is>
-          <t>M3-13</t>
+          <t>M3-12</t>
         </is>
       </c>
       <c r="B61" s="19" t="inlineStr">
@@ -5954,7 +5954,7 @@
       </c>
       <c r="C61" s="19" t="inlineStr">
         <is>
-          <t>Parámetros configurables sin programar, con pantalla de Configuración y cada cambio en bitácora: monto máximo por ofrenda (1,000,000 por defecto) y si se permite una sola ofrenda regular por reunión. Solo Pastor y Administrador Técnico.</t>
+          <t>Reuniones: cada grupo se reúne una vez por semana en casa del líder (día y hora por grupo) y existe una reunión general de líderes, modelada como un grupo de tipo «Líderes».</t>
         </is>
       </c>
       <c r="D61" s="21" t="inlineStr">
@@ -5974,7 +5974,7 @@
       </c>
       <c r="G61" s="19" t="inlineStr">
         <is>
-          <t>Sprint 4</t>
+          <t>Sprint 3</t>
         </is>
       </c>
       <c r="H61" s="19" t="inlineStr">
@@ -6004,19 +6004,19 @@
       </c>
       <c r="M61" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/m3-ofrendas-ajustes · 121 pruebas de backend y 14 de frontend pasan</t>
+          <t>Rama feature/grupos-paso-3 · pruebas de backend y 81 de frontend pasan; lint, estilos y compilación limpios</t>
         </is>
       </c>
       <c r="N61" s="19" t="inlineStr">
         <is>
-          <t>2026-10-24 · Pantalla Configuración: monto máximo y una regular por reunión.</t>
+          <t>2026-10-27 · Una reunión semanal por grupo y grupo tipo Líderes; filtros por día, sector, líder y estado; cada reunión muestra su asistencia, observaciones, peticiones y ofrendas.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="18" t="inlineStr">
         <is>
-          <t>M3-14</t>
+          <t>M3-13</t>
         </is>
       </c>
       <c r="B62" s="19" t="inlineStr">
@@ -6026,7 +6026,7 @@
       </c>
       <c r="C62" s="19" t="inlineStr">
         <is>
-          <t>Componente de peticiones reutilizable: cualquier módulo (grupos hoy; cursos o eventos después) se registra como origen y decide quién registra y qué nivel de acceso tiene cada persona. Toda petición guarda su origen de forma inmutable (tipo, identificador y una etiqueta fija, por ejemplo «Grupo de Conexión · Norte · reunión del 22/10/2026») y lo muestra siempre en el listado.</t>
+          <t>Parámetros configurables sin programar, con pantalla de Configuración y cada cambio en bitácora: monto máximo por ofrenda (1,000,000 por defecto) y si se permite una sola ofrenda regular por reunión. Solo Pastor y Administrador Técnico.</t>
         </is>
       </c>
       <c r="D62" s="21" t="inlineStr">
@@ -6076,19 +6076,19 @@
       </c>
       <c r="M62" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/m3-peticiones-oracion · 166 pruebas de backend y 32 de frontend pasan; probado contra la base real</t>
+          <t>Rama feature/m3-ofrendas-ajustes · 121 pruebas de backend y 14 de frontend pasan</t>
         </is>
       </c>
       <c r="N62" s="19" t="inlineStr">
         <is>
-          <t>2026-10-24 · Origen inmutable y visible; probado con un segundo origen de prueba para verificar la reutilización.</t>
+          <t>2026-10-24 · Pantalla Configuración: monto máximo y una regular por reunión.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="18" t="inlineStr">
         <is>
-          <t>M3-15</t>
+          <t>M3-14</t>
         </is>
       </c>
       <c r="B63" s="19" t="inlineStr">
@@ -6098,7 +6098,7 @@
       </c>
       <c r="C63" s="19" t="inlineStr">
         <is>
-          <t>Equipo de oración: rol configurable (Equipo de oración) que se asigna a las personas que se reúnen a orar por las peticiones compartidas con ese alcance; no da acceso a nada más. Opción de ocultar el nombre de quien pide: los campos del formulario marcados «identifica a la persona» solo los ven líderes y quien registró. Al capturar se muestra una leyenda que pide confirmar la autorización de quien pide, indica quién la leerá y cuándo se borra.</t>
+          <t>Componente de peticiones reutilizable: cualquier módulo (grupos hoy; cursos o eventos después) se registra como origen y decide quién registra y qué nivel de acceso tiene cada persona. Toda petición guarda su origen de forma inmutable (tipo, identificador y una etiqueta fija, por ejemplo «Grupo de Conexión · Norte · reunión del 22/10/2026») y lo muestra siempre en el listado.</t>
         </is>
       </c>
       <c r="D63" s="21" t="inlineStr">
@@ -6153,49 +6153,49 @@
       </c>
       <c r="N63" s="19" t="inlineStr">
         <is>
-          <t>2026-10-24 · Rol Equipo de oración, nombre oculto y leyenda de privacidad al capturar. Falta el aviso de privacidad oficial de la iglesia.</t>
+          <t>2026-10-24 · Origen inmutable y visible; probado con un segundo origen de prueba para verificar la reutilización.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="18" t="inlineStr">
         <is>
-          <t>M4-01</t>
+          <t>M3-15</t>
         </is>
       </c>
       <c r="B64" s="19" t="inlineStr">
         <is>
-          <t>M4 Kids Check-In/Out</t>
+          <t>M3 Grupos de Conexión</t>
         </is>
       </c>
       <c r="C64" s="19" t="inlineStr">
         <is>
-          <t>Sustitución de la ficha física de papel.</t>
-        </is>
-      </c>
-      <c r="D64" s="19" t="inlineStr">
-        <is>
-          <t>v1 / v2</t>
+          <t>Equipo de oración: rol configurable (Equipo de oración) que se asigna a las personas que se reúnen a orar por las peticiones compartidas con ese alcance; no da acceso a nada más. Opción de ocultar el nombre de quien pide: los campos del formulario marcados «identifica a la persona» solo los ven líderes y quien registró. Al capturar se muestra una leyenda que pide confirmar la autorización de quien pide, indica quién la leerá y cuándo se borra.</t>
+        </is>
+      </c>
+      <c r="D64" s="21" t="inlineStr">
+        <is>
+          <t>Respuesta</t>
         </is>
       </c>
       <c r="E64" s="19" t="inlineStr">
         <is>
-          <t>Fuera del MVP</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="F64" s="19" t="inlineStr">
         <is>
-          <t>Fase 2</t>
+          <t>Fase 1</t>
         </is>
       </c>
       <c r="G64" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sprint 4</t>
         </is>
       </c>
       <c r="H64" s="19" t="inlineStr">
         <is>
-          <t>Posterior</t>
+          <t>H3 · MVP (Grupos)</t>
         </is>
       </c>
       <c r="I64" s="20" t="inlineStr">
@@ -6215,16 +6215,24 @@
       </c>
       <c r="L64" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M64" s="19" t="inlineStr"/>
-      <c r="N64" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M64" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/m3-peticiones-oracion · 166 pruebas de backend y 32 de frontend pasan; probado contra la base real</t>
+        </is>
+      </c>
+      <c r="N64" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-24 · Rol Equipo de oración, nombre oculto y leyenda de privacidad al capturar. Falta el aviso de privacidad oficial de la iglesia.</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="18" t="inlineStr">
         <is>
-          <t>M4-02</t>
+          <t>M4-01</t>
         </is>
       </c>
       <c r="B65" s="19" t="inlineStr">
@@ -6234,12 +6242,12 @@
       </c>
       <c r="C65" s="19" t="inlineStr">
         <is>
-          <t>Registro de ingreso del menor con salón o clase asignada y generación de código único.</t>
-        </is>
-      </c>
-      <c r="D65" s="21" t="inlineStr">
-        <is>
-          <t>v1 + Nuevo v3</t>
+          <t>Sustitución de la ficha física de papel.</t>
+        </is>
+      </c>
+      <c r="D65" s="19" t="inlineStr">
+        <is>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E65" s="19" t="inlineStr">
@@ -6288,7 +6296,7 @@
     <row r="66">
       <c r="A66" s="18" t="inlineStr">
         <is>
-          <t>M4-03</t>
+          <t>M4-02</t>
         </is>
       </c>
       <c r="B66" s="19" t="inlineStr">
@@ -6298,12 +6306,12 @@
       </c>
       <c r="C66" s="19" t="inlineStr">
         <is>
-          <t>Código QR dinámico o OTP temporal en la PWA del padre o tutor.</t>
-        </is>
-      </c>
-      <c r="D66" s="19" t="inlineStr">
-        <is>
-          <t>v2</t>
+          <t>Registro de ingreso del menor con salón o clase asignada y generación de código único.</t>
+        </is>
+      </c>
+      <c r="D66" s="21" t="inlineStr">
+        <is>
+          <t>v1 + Nuevo v3</t>
         </is>
       </c>
       <c r="E66" s="19" t="inlineStr">
@@ -6352,7 +6360,7 @@
     <row r="67">
       <c r="A67" s="18" t="inlineStr">
         <is>
-          <t>M4-04</t>
+          <t>M4-03</t>
         </is>
       </c>
       <c r="B67" s="19" t="inlineStr">
@@ -6362,7 +6370,7 @@
       </c>
       <c r="C67" s="19" t="inlineStr">
         <is>
-          <t>Validación al entregar: el servidor de Kids escanea el código y confirma identidad y fotografía del tutor autorizado en el Expediente Digital.</t>
+          <t>Código QR dinámico o OTP temporal en la PWA del padre o tutor.</t>
         </is>
       </c>
       <c r="D67" s="19" t="inlineStr">
@@ -6416,7 +6424,7 @@
     <row r="68">
       <c r="A68" s="18" t="inlineStr">
         <is>
-          <t>M4-05</t>
+          <t>M4-04</t>
         </is>
       </c>
       <c r="B68" s="19" t="inlineStr">
@@ -6426,12 +6434,12 @@
       </c>
       <c r="C68" s="19" t="inlineStr">
         <is>
-          <t>Alternativa para tutores sin smartphone, sin batería o sin conexión (p. ej. código por SMS o comprobante imprimible con identificación). Por definir.</t>
-        </is>
-      </c>
-      <c r="D68" s="21" t="inlineStr">
-        <is>
-          <t>Nuevo v3</t>
+          <t>Validación al entregar: el servidor de Kids escanea el código y confirma identidad y fotografía del tutor autorizado en el Expediente Digital.</t>
+        </is>
+      </c>
+      <c r="D68" s="19" t="inlineStr">
+        <is>
+          <t>v2</t>
         </is>
       </c>
       <c r="E68" s="19" t="inlineStr">
@@ -6466,7 +6474,7 @@
       </c>
       <c r="K68" s="19" t="inlineStr">
         <is>
-          <t>Por definir</t>
+          <t>VoBo pendiente</t>
         </is>
       </c>
       <c r="L68" s="19" t="inlineStr">
@@ -6480,7 +6488,7 @@
     <row r="69">
       <c r="A69" s="18" t="inlineStr">
         <is>
-          <t>M4-06</t>
+          <t>M4-05</t>
         </is>
       </c>
       <c r="B69" s="19" t="inlineStr">
@@ -6490,7 +6498,7 @@
       </c>
       <c r="C69" s="19" t="inlineStr">
         <is>
-          <t>Autorización temporal de un tercero para recoger al menor, con aprobación del tutor registrado.</t>
+          <t>Alternativa para tutores sin smartphone, sin batería o sin conexión (p. ej. código por SMS o comprobante imprimible con identificación). Por definir.</t>
         </is>
       </c>
       <c r="D69" s="21" t="inlineStr">
@@ -6530,7 +6538,7 @@
       </c>
       <c r="K69" s="19" t="inlineStr">
         <is>
-          <t>VoBo pendiente</t>
+          <t>Por definir</t>
         </is>
       </c>
       <c r="L69" s="19" t="inlineStr">
@@ -6544,7 +6552,7 @@
     <row r="70">
       <c r="A70" s="18" t="inlineStr">
         <is>
-          <t>M4-07</t>
+          <t>M4-06</t>
         </is>
       </c>
       <c r="B70" s="19" t="inlineStr">
@@ -6554,7 +6562,7 @@
       </c>
       <c r="C70" s="19" t="inlineStr">
         <is>
-          <t>Caducidad del código y bitácora de cada entrega (quién recogió, quién entregó, hora).</t>
+          <t>Autorización temporal de un tercero para recoger al menor, con aprobación del tutor registrado.</t>
         </is>
       </c>
       <c r="D70" s="21" t="inlineStr">
@@ -6608,7 +6616,7 @@
     <row r="71">
       <c r="A71" s="18" t="inlineStr">
         <is>
-          <t>M4-08</t>
+          <t>M4-07</t>
         </is>
       </c>
       <c r="B71" s="19" t="inlineStr">
@@ -6618,7 +6626,7 @@
       </c>
       <c r="C71" s="19" t="inlineStr">
         <is>
-          <t>Funcionamiento sin conexión o con conexión degradada para el check-out.</t>
+          <t>Caducidad del código y bitácora de cada entrega (quién recogió, quién entregó, hora).</t>
         </is>
       </c>
       <c r="D71" s="21" t="inlineStr">
@@ -6672,52 +6680,52 @@
     <row r="72">
       <c r="A72" s="18" t="inlineStr">
         <is>
-          <t>M5-01</t>
+          <t>M4-08</t>
         </is>
       </c>
       <c r="B72" s="19" t="inlineStr">
         <is>
-          <t>M5 Áreas y servidores</t>
+          <t>M4 Kids Check-In/Out</t>
         </is>
       </c>
       <c r="C72" s="19" t="inlineStr">
         <is>
-          <t>Catálogo mínimo de áreas y asignación de servidores. Versión reducida del módulo 5, necesaria para permisos por área. Sirve como primer censo.</t>
-        </is>
-      </c>
-      <c r="D72" s="19" t="inlineStr">
-        <is>
-          <t>v3</t>
+          <t>Funcionamiento sin conexión o con conexión degradada para el check-out.</t>
+        </is>
+      </c>
+      <c r="D72" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3</t>
         </is>
       </c>
       <c r="E72" s="19" t="inlineStr">
         <is>
-          <t>MVP mínimo</t>
+          <t>Fuera del MVP</t>
         </is>
       </c>
       <c r="F72" s="19" t="inlineStr">
         <is>
-          <t>Fase 0</t>
+          <t>Fase 2</t>
         </is>
       </c>
       <c r="G72" s="19" t="inlineStr">
         <is>
-          <t>Sprint 1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H72" s="19" t="inlineStr">
         <is>
-          <t>H2 · Fase 0 completa</t>
-        </is>
-      </c>
-      <c r="I72" s="19" t="inlineStr">
-        <is>
-          <t>Como pastor quiero un catálogo de áreas con su personal para conocer la estructura.</t>
-        </is>
-      </c>
-      <c r="J72" s="19" t="inlineStr">
-        <is>
-          <t>Crear un área, asignar servidores y ver el conteo real.</t>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="I72" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
+        </is>
+      </c>
+      <c r="J72" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
         </is>
       </c>
       <c r="K72" s="19" t="inlineStr">
@@ -6736,7 +6744,7 @@
     <row r="73">
       <c r="A73" s="18" t="inlineStr">
         <is>
-          <t>M5-02</t>
+          <t>M5-01</t>
         </is>
       </c>
       <c r="B73" s="19" t="inlineStr">
@@ -6746,42 +6754,42 @@
       </c>
       <c r="C73" s="19" t="inlineStr">
         <is>
-          <t>Roles jerárquicos dentro de cada área (directores, líderes, maestros, servidores).</t>
+          <t>Catálogo mínimo de áreas y asignación de servidores. Versión reducida del módulo 5, necesaria para permisos por área. Sirve como primer censo.</t>
         </is>
       </c>
       <c r="D73" s="19" t="inlineStr">
         <is>
-          <t>v1</t>
+          <t>v3</t>
         </is>
       </c>
       <c r="E73" s="19" t="inlineStr">
         <is>
-          <t>Fuera del MVP</t>
+          <t>MVP mínimo</t>
         </is>
       </c>
       <c r="F73" s="19" t="inlineStr">
         <is>
-          <t>Fase 4</t>
+          <t>Fase 0</t>
         </is>
       </c>
       <c r="G73" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sprint 1</t>
         </is>
       </c>
       <c r="H73" s="19" t="inlineStr">
         <is>
-          <t>Posterior</t>
-        </is>
-      </c>
-      <c r="I73" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
-        </is>
-      </c>
-      <c r="J73" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
+          <t>H2 · Fase 0 completa</t>
+        </is>
+      </c>
+      <c r="I73" s="19" t="inlineStr">
+        <is>
+          <t>Como pastor quiero un catálogo de áreas con su personal para conocer la estructura.</t>
+        </is>
+      </c>
+      <c r="J73" s="19" t="inlineStr">
+        <is>
+          <t>Crear un área, asignar servidores y ver el conteo real.</t>
         </is>
       </c>
       <c r="K73" s="19" t="inlineStr">
@@ -6800,7 +6808,7 @@
     <row r="74">
       <c r="A74" s="18" t="inlineStr">
         <is>
-          <t>M5-03</t>
+          <t>M5-02</t>
         </is>
       </c>
       <c r="B74" s="19" t="inlineStr">
@@ -6810,12 +6818,12 @@
       </c>
       <c r="C74" s="19" t="inlineStr">
         <is>
-          <t>Organigrama y número real de servidores activos, directores y líderes por área.</t>
+          <t>Roles jerárquicos dentro de cada área (directores, líderes, maestros, servidores).</t>
         </is>
       </c>
       <c r="D74" s="19" t="inlineStr">
         <is>
-          <t>v2</t>
+          <t>v1</t>
         </is>
       </c>
       <c r="E74" s="19" t="inlineStr">
@@ -6864,7 +6872,7 @@
     <row r="75">
       <c r="A75" s="18" t="inlineStr">
         <is>
-          <t>M5-04</t>
+          <t>M5-03</t>
         </is>
       </c>
       <c r="B75" s="19" t="inlineStr">
@@ -6874,12 +6882,12 @@
       </c>
       <c r="C75" s="19" t="inlineStr">
         <is>
-          <t>Control de asistencia a turnos o servicios.</t>
+          <t>Organigrama y número real de servidores activos, directores y líderes por área.</t>
         </is>
       </c>
       <c r="D75" s="19" t="inlineStr">
         <is>
-          <t>v1 / v2</t>
+          <t>v2</t>
         </is>
       </c>
       <c r="E75" s="19" t="inlineStr">
@@ -6928,7 +6936,7 @@
     <row r="76">
       <c r="A76" s="18" t="inlineStr">
         <is>
-          <t>M5-05</t>
+          <t>M5-04</t>
         </is>
       </c>
       <c r="B76" s="19" t="inlineStr">
@@ -6938,7 +6946,7 @@
       </c>
       <c r="C76" s="19" t="inlineStr">
         <is>
-          <t>Tablero de avisos y notificaciones interno por área.</t>
+          <t>Control de asistencia a turnos o servicios.</t>
         </is>
       </c>
       <c r="D76" s="19" t="inlineStr">
@@ -6992,7 +7000,7 @@
     <row r="77">
       <c r="A77" s="18" t="inlineStr">
         <is>
-          <t>M5-06</t>
+          <t>M5-05</t>
         </is>
       </c>
       <c r="B77" s="19" t="inlineStr">
@@ -7002,7 +7010,7 @@
       </c>
       <c r="C77" s="19" t="inlineStr">
         <is>
-          <t>Gestión financiera por área: caja chica y gastos operativos.</t>
+          <t>Tablero de avisos y notificaciones interno por área.</t>
         </is>
       </c>
       <c r="D77" s="19" t="inlineStr">
@@ -7056,22 +7064,22 @@
     <row r="78">
       <c r="A78" s="18" t="inlineStr">
         <is>
-          <t>M6-01</t>
+          <t>M5-06</t>
         </is>
       </c>
       <c r="B78" s="19" t="inlineStr">
         <is>
-          <t>M6 Ministerios de servicio</t>
+          <t>M5 Áreas y servidores</t>
         </is>
       </c>
       <c r="C78" s="19" t="inlineStr">
         <is>
-          <t>Control de personal propio de cada ministerio.</t>
-        </is>
-      </c>
-      <c r="D78" s="22" t="inlineStr">
-        <is>
-          <t>Recuperado v1</t>
+          <t>Gestión financiera por área: caja chica y gastos operativos.</t>
+        </is>
+      </c>
+      <c r="D78" s="19" t="inlineStr">
+        <is>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E78" s="19" t="inlineStr">
@@ -7120,7 +7128,7 @@
     <row r="79">
       <c r="A79" s="18" t="inlineStr">
         <is>
-          <t>M6-02</t>
+          <t>M6-01</t>
         </is>
       </c>
       <c r="B79" s="19" t="inlineStr">
@@ -7130,12 +7138,12 @@
       </c>
       <c r="C79" s="19" t="inlineStr">
         <is>
-          <t>Menú o catálogo digital interactivo (público o interno), autogestionado.</t>
-        </is>
-      </c>
-      <c r="D79" s="19" t="inlineStr">
-        <is>
-          <t>v1 / v2</t>
+          <t>Control de personal propio de cada ministerio.</t>
+        </is>
+      </c>
+      <c r="D79" s="22" t="inlineStr">
+        <is>
+          <t>Recuperado v1</t>
         </is>
       </c>
       <c r="E79" s="19" t="inlineStr">
@@ -7184,7 +7192,7 @@
     <row r="80">
       <c r="A80" s="18" t="inlineStr">
         <is>
-          <t>M6-03</t>
+          <t>M6-02</t>
         </is>
       </c>
       <c r="B80" s="19" t="inlineStr">
@@ -7194,7 +7202,7 @@
       </c>
       <c r="C80" s="19" t="inlineStr">
         <is>
-          <t>Calendario de turnos: días regulares de servicio y eventos especiales.</t>
+          <t>Menú o catálogo digital interactivo (público o interno), autogestionado.</t>
         </is>
       </c>
       <c r="D80" s="19" t="inlineStr">
@@ -7248,7 +7256,7 @@
     <row r="81">
       <c r="A81" s="18" t="inlineStr">
         <is>
-          <t>M6-04</t>
+          <t>M6-03</t>
         </is>
       </c>
       <c r="B81" s="19" t="inlineStr">
@@ -7258,7 +7266,7 @@
       </c>
       <c r="C81" s="19" t="inlineStr">
         <is>
-          <t>Registro de asistentes o personas atendidas.</t>
+          <t>Calendario de turnos: días regulares de servicio y eventos especiales.</t>
         </is>
       </c>
       <c r="D81" s="19" t="inlineStr">
@@ -7312,7 +7320,7 @@
     <row r="82">
       <c r="A82" s="18" t="inlineStr">
         <is>
-          <t>M6-05</t>
+          <t>M6-04</t>
         </is>
       </c>
       <c r="B82" s="19" t="inlineStr">
@@ -7322,7 +7330,7 @@
       </c>
       <c r="C82" s="19" t="inlineStr">
         <is>
-          <t>Control de gastos y de inventario básico.</t>
+          <t>Registro de asistentes o personas atendidas.</t>
         </is>
       </c>
       <c r="D82" s="19" t="inlineStr">
@@ -7376,7 +7384,7 @@
     <row r="83">
       <c r="A83" s="18" t="inlineStr">
         <is>
-          <t>M6-06</t>
+          <t>M6-05</t>
         </is>
       </c>
       <c r="B83" s="19" t="inlineStr">
@@ -7386,7 +7394,7 @@
       </c>
       <c r="C83" s="19" t="inlineStr">
         <is>
-          <t>Canal de comunicación directo con el área de Administración General.</t>
+          <t>Control de gastos y de inventario básico.</t>
         </is>
       </c>
       <c r="D83" s="19" t="inlineStr">
@@ -7440,7 +7448,7 @@
     <row r="84">
       <c r="A84" s="18" t="inlineStr">
         <is>
-          <t>M6-07</t>
+          <t>M6-06</t>
         </is>
       </c>
       <c r="B84" s="19" t="inlineStr">
@@ -7450,12 +7458,12 @@
       </c>
       <c r="C84" s="19" t="inlineStr">
         <is>
-          <t>Servicio Médico: los datos de salud de las personas atendidas requieren tratamiento de datos sensibles. Por definir alcance.</t>
-        </is>
-      </c>
-      <c r="D84" s="21" t="inlineStr">
-        <is>
-          <t>Nuevo v3</t>
+          <t>Canal de comunicación directo con el área de Administración General.</t>
+        </is>
+      </c>
+      <c r="D84" s="19" t="inlineStr">
+        <is>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E84" s="19" t="inlineStr">
@@ -7490,7 +7498,7 @@
       </c>
       <c r="K84" s="19" t="inlineStr">
         <is>
-          <t>Por definir</t>
+          <t>VoBo pendiente</t>
         </is>
       </c>
       <c r="L84" s="19" t="inlineStr">
@@ -7504,22 +7512,22 @@
     <row r="85">
       <c r="A85" s="18" t="inlineStr">
         <is>
-          <t>M7-01</t>
+          <t>M6-07</t>
         </is>
       </c>
       <c r="B85" s="19" t="inlineStr">
         <is>
-          <t>M7 Eventos y aforo</t>
+          <t>M6 Ministerios de servicio</t>
         </is>
       </c>
       <c r="C85" s="19" t="inlineStr">
         <is>
-          <t>Eventos abiertos o evangelísticos con formulario de inscripción rápida, sin requerir historial previo.</t>
-        </is>
-      </c>
-      <c r="D85" s="19" t="inlineStr">
-        <is>
-          <t>v1 / v2</t>
+          <t>Servicio Médico: los datos de salud de las personas atendidas requieren tratamiento de datos sensibles. Por definir alcance.</t>
+        </is>
+      </c>
+      <c r="D85" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3</t>
         </is>
       </c>
       <c r="E85" s="19" t="inlineStr">
@@ -7554,7 +7562,7 @@
       </c>
       <c r="K85" s="19" t="inlineStr">
         <is>
-          <t>VoBo pendiente</t>
+          <t>Por definir</t>
         </is>
       </c>
       <c r="L85" s="19" t="inlineStr">
@@ -7568,7 +7576,7 @@
     <row r="86">
       <c r="A86" s="18" t="inlineStr">
         <is>
-          <t>M7-02</t>
+          <t>M7-01</t>
         </is>
       </c>
       <c r="B86" s="19" t="inlineStr">
@@ -7578,12 +7586,12 @@
       </c>
       <c r="C86" s="19" t="inlineStr">
         <is>
-          <t>Consolidación (inducción de personas que asisten por primera vez) como tipo de evento.</t>
-        </is>
-      </c>
-      <c r="D86" s="22" t="inlineStr">
-        <is>
-          <t>Recuperado v1</t>
+          <t>Eventos abiertos o evangelísticos con formulario de inscripción rápida, sin requerir historial previo.</t>
+        </is>
+      </c>
+      <c r="D86" s="19" t="inlineStr">
+        <is>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E86" s="19" t="inlineStr">
@@ -7632,7 +7640,7 @@
     <row r="87">
       <c r="A87" s="18" t="inlineStr">
         <is>
-          <t>M7-03</t>
+          <t>M7-02</t>
         </is>
       </c>
       <c r="B87" s="19" t="inlineStr">
@@ -7642,7 +7650,7 @@
       </c>
       <c r="C87" s="19" t="inlineStr">
         <is>
-          <t>Encargados de evento (personal de la iglesia únicamente; no se controla personal externo).</t>
+          <t>Consolidación (inducción de personas que asisten por primera vez) como tipo de evento.</t>
         </is>
       </c>
       <c r="D87" s="22" t="inlineStr">
@@ -7696,7 +7704,7 @@
     <row r="88">
       <c r="A88" s="18" t="inlineStr">
         <is>
-          <t>M7-04</t>
+          <t>M7-03</t>
         </is>
       </c>
       <c r="B88" s="19" t="inlineStr">
@@ -7706,12 +7714,12 @@
       </c>
       <c r="C88" s="19" t="inlineStr">
         <is>
-          <t>Control de cupo en tiempo real que bloquea el sobrecupo en eventos con aforo limitado (ej. 30 o 50 lugares).</t>
-        </is>
-      </c>
-      <c r="D88" s="19" t="inlineStr">
-        <is>
-          <t>v1 / v2</t>
+          <t>Encargados de evento (personal de la iglesia únicamente; no se controla personal externo).</t>
+        </is>
+      </c>
+      <c r="D88" s="22" t="inlineStr">
+        <is>
+          <t>Recuperado v1</t>
         </is>
       </c>
       <c r="E88" s="19" t="inlineStr">
@@ -7760,7 +7768,7 @@
     <row r="89">
       <c r="A89" s="18" t="inlineStr">
         <is>
-          <t>M7-05</t>
+          <t>M7-04</t>
         </is>
       </c>
       <c r="B89" s="19" t="inlineStr">
@@ -7770,12 +7778,12 @@
       </c>
       <c r="C89" s="19" t="inlineStr">
         <is>
-          <t>Control de asistentes sin lista previa, para aforo y para dar a conocer la iglesia.</t>
+          <t>Control de cupo en tiempo real que bloquea el sobrecupo en eventos con aforo limitado (ej. 30 o 50 lugares).</t>
         </is>
       </c>
       <c r="D89" s="19" t="inlineStr">
         <is>
-          <t>v1</t>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E89" s="19" t="inlineStr">
@@ -7824,7 +7832,7 @@
     <row r="90">
       <c r="A90" s="18" t="inlineStr">
         <is>
-          <t>M7-06</t>
+          <t>M7-05</t>
         </is>
       </c>
       <c r="B90" s="19" t="inlineStr">
@@ -7834,12 +7842,12 @@
       </c>
       <c r="C90" s="19" t="inlineStr">
         <is>
-          <t>Seguimiento de personas nuevas: conversión de un invitado a Expediente Digital y canalización a un curso o Grupo de Conexión.</t>
-        </is>
-      </c>
-      <c r="D90" s="21" t="inlineStr">
-        <is>
-          <t>Nuevo v3</t>
+          <t>Control de asistentes sin lista previa, para aforo y para dar a conocer la iglesia.</t>
+        </is>
+      </c>
+      <c r="D90" s="19" t="inlineStr">
+        <is>
+          <t>v1</t>
         </is>
       </c>
       <c r="E90" s="19" t="inlineStr">
@@ -7888,52 +7896,52 @@
     <row r="91">
       <c r="A91" s="18" t="inlineStr">
         <is>
-          <t>NF-01</t>
+          <t>M7-06</t>
         </is>
       </c>
       <c r="B91" s="19" t="inlineStr">
         <is>
-          <t>No funcionales</t>
+          <t>M7 Eventos y aforo</t>
         </is>
       </c>
       <c r="C91" s="19" t="inlineStr">
         <is>
-          <t>Cumplimiento de la LFPDPPP: aviso de privacidad, consentimiento y derechos ARCO.</t>
-        </is>
-      </c>
-      <c r="D91" s="19" t="inlineStr">
-        <is>
-          <t>v3</t>
+          <t>Seguimiento de personas nuevas: conversión de un invitado a Expediente Digital y canalización a un curso o Grupo de Conexión.</t>
+        </is>
+      </c>
+      <c r="D91" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3</t>
         </is>
       </c>
       <c r="E91" s="19" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Fuera del MVP</t>
         </is>
       </c>
       <c r="F91" s="19" t="inlineStr">
         <is>
-          <t>Fase 0</t>
+          <t>Fase 4</t>
         </is>
       </c>
       <c r="G91" s="19" t="inlineStr">
         <is>
-          <t>Sprint 1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H91" s="19" t="inlineStr">
         <is>
-          <t>H1 · 18-oct (núcleo Fase 0)</t>
-        </is>
-      </c>
-      <c r="I91" s="19" t="inlineStr">
-        <is>
-          <t>Como iglesia queremos cumplir con la LFPDPPP.</t>
-        </is>
-      </c>
-      <c r="J91" s="19" t="inlineStr">
-        <is>
-          <t>Aviso de privacidad, consentimiento y atención de derechos ARCO disponibles.</t>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="I91" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
+        </is>
+      </c>
+      <c r="J91" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
         </is>
       </c>
       <c r="K91" s="19" t="inlineStr">
@@ -7952,7 +7960,7 @@
     <row r="92">
       <c r="A92" s="18" t="inlineStr">
         <is>
-          <t>NF-02</t>
+          <t>NF-01</t>
         </is>
       </c>
       <c r="B92" s="19" t="inlineStr">
@@ -7962,7 +7970,7 @@
       </c>
       <c r="C92" s="19" t="inlineStr">
         <is>
-          <t>Cifrado en tránsito y en reposo. Cifrado adicional a nivel de campo para peticiones de oración.</t>
+          <t>Cumplimiento de la LFPDPPP: aviso de privacidad, consentimiento y derechos ARCO.</t>
         </is>
       </c>
       <c r="D92" s="19" t="inlineStr">
@@ -7982,7 +7990,7 @@
       </c>
       <c r="G92" s="19" t="inlineStr">
         <is>
-          <t>Sprint 0</t>
+          <t>Sprint 1</t>
         </is>
       </c>
       <c r="H92" s="19" t="inlineStr">
@@ -7992,12 +8000,12 @@
       </c>
       <c r="I92" s="19" t="inlineStr">
         <is>
-          <t>Como iglesia queremos proteger los datos sensibles.</t>
+          <t>Como iglesia queremos cumplir con la LFPDPPP.</t>
         </is>
       </c>
       <c r="J92" s="19" t="inlineStr">
         <is>
-          <t>HTTPS obligatorio y peticiones de oración ilegibles directamente en la base.</t>
+          <t>Aviso de privacidad, consentimiento y atención de derechos ARCO disponibles.</t>
         </is>
       </c>
       <c r="K92" s="19" t="inlineStr">
@@ -8007,24 +8015,16 @@
       </c>
       <c r="L92" s="19" t="inlineStr">
         <is>
-          <t>En pruebas</t>
-        </is>
-      </c>
-      <c r="M92" s="19" t="inlineStr">
-        <is>
-          <t>Rama feature/m3-peticiones-oracion · 166 pruebas de backend y 32 de frontend pasan; probado contra la base real</t>
-        </is>
-      </c>
-      <c r="N92" s="19" t="inlineStr">
-        <is>
-          <t>2026-10-24 · Peticiones cifradas a nivel de campo; falta cifrado en reposo de toda la base (proveedor de nube).</t>
-        </is>
-      </c>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M92" s="19" t="inlineStr"/>
+      <c r="N92" s="19" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="18" t="inlineStr">
         <is>
-          <t>NF-03</t>
+          <t>NF-02</t>
         </is>
       </c>
       <c r="B93" s="19" t="inlineStr">
@@ -8034,7 +8034,7 @@
       </c>
       <c r="C93" s="19" t="inlineStr">
         <is>
-          <t>Bitácora de auditoría de solo-añadir: quién consultó o modificó expedientes, ofrendas y asistencias.</t>
+          <t>Cifrado en tránsito y en reposo. Cifrado adicional a nivel de campo para peticiones de oración.</t>
         </is>
       </c>
       <c r="D93" s="19" t="inlineStr">
@@ -8054,7 +8054,7 @@
       </c>
       <c r="G93" s="19" t="inlineStr">
         <is>
-          <t>Sprint 1</t>
+          <t>Sprint 0</t>
         </is>
       </c>
       <c r="H93" s="19" t="inlineStr">
@@ -8064,12 +8064,12 @@
       </c>
       <c r="I93" s="19" t="inlineStr">
         <is>
-          <t>Como pastor quiero una bitácora que nadie pueda alterar.</t>
+          <t>Como iglesia queremos proteger los datos sensibles.</t>
         </is>
       </c>
       <c r="J93" s="19" t="inlineStr">
         <is>
-          <t>El usuario de la aplicación no puede actualizar ni borrar registros de bitácora.</t>
+          <t>HTTPS obligatorio y peticiones de oración ilegibles directamente en la base.</t>
         </is>
       </c>
       <c r="K93" s="19" t="inlineStr">
@@ -8084,19 +8084,19 @@
       </c>
       <c r="M93" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/nf-03-bitacora · 69 pruebas de backend pasan</t>
+          <t>Rama feature/m3-peticiones-oracion · 166 pruebas de backend y 32 de frontend pasan; probado contra la base real</t>
         </is>
       </c>
       <c r="N93" s="19" t="inlineStr">
         <is>
-          <t>2026-10-10 · Bloqueo en aplicación y trigger de PostgreSQL (UPDATE/DELETE/TRUNCATE); pantalla de consulta con permiso bitacora.ver.</t>
+          <t>2026-10-24 · Peticiones cifradas a nivel de campo; falta cifrado en reposo de toda la base (proveedor de nube).</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="18" t="inlineStr">
         <is>
-          <t>NF-04</t>
+          <t>NF-03</t>
         </is>
       </c>
       <c r="B94" s="19" t="inlineStr">
@@ -8106,7 +8106,7 @@
       </c>
       <c r="C94" s="19" t="inlineStr">
         <is>
-          <t>Respaldos automáticos diarios cifrados y prueba periódica de restauración.</t>
+          <t>Bitácora de auditoría de solo-añadir: quién consultó o modificó expedientes, ofrendas y asistencias.</t>
         </is>
       </c>
       <c r="D94" s="19" t="inlineStr">
@@ -8126,7 +8126,7 @@
       </c>
       <c r="G94" s="19" t="inlineStr">
         <is>
-          <t>Sprint 0</t>
+          <t>Sprint 1</t>
         </is>
       </c>
       <c r="H94" s="19" t="inlineStr">
@@ -8136,12 +8136,12 @@
       </c>
       <c r="I94" s="19" t="inlineStr">
         <is>
-          <t>Como iglesia queremos no perder información.</t>
+          <t>Como pastor quiero una bitácora que nadie pueda alterar.</t>
         </is>
       </c>
       <c r="J94" s="19" t="inlineStr">
         <is>
-          <t>Respaldo diario cifrado y restauración probada en un ambiente de pruebas.</t>
+          <t>El usuario de la aplicación no puede actualizar ni borrar registros de bitácora.</t>
         </is>
       </c>
       <c r="K94" s="19" t="inlineStr">
@@ -8151,16 +8151,24 @@
       </c>
       <c r="L94" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M94" s="19" t="inlineStr"/>
-      <c r="N94" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M94" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/nf-03-bitacora · 69 pruebas de backend pasan</t>
+        </is>
+      </c>
+      <c r="N94" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-10 · Bloqueo en aplicación y trigger de PostgreSQL (UPDATE/DELETE/TRUNCATE); pantalla de consulta con permiso bitacora.ver.</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="18" t="inlineStr">
         <is>
-          <t>NF-05</t>
+          <t>NF-04</t>
         </is>
       </c>
       <c r="B95" s="19" t="inlineStr">
@@ -8170,47 +8178,47 @@
       </c>
       <c r="C95" s="19" t="inlineStr">
         <is>
-          <t>Disponibilidad esperada en horarios de servicio (fines de semana y reuniones de grupo). Por definir meta.</t>
-        </is>
-      </c>
-      <c r="D95" s="21" t="inlineStr">
-        <is>
-          <t>Nuevo v3</t>
+          <t>Respaldos automáticos diarios cifrados y prueba periódica de restauración.</t>
+        </is>
+      </c>
+      <c r="D95" s="19" t="inlineStr">
+        <is>
+          <t>v3</t>
         </is>
       </c>
       <c r="E95" s="19" t="inlineStr">
         <is>
-          <t>Fuera del MVP</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="F95" s="19" t="inlineStr">
         <is>
-          <t>Transversal</t>
+          <t>Fase 0</t>
         </is>
       </c>
       <c r="G95" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sprint 0</t>
         </is>
       </c>
       <c r="H95" s="19" t="inlineStr">
         <is>
-          <t>Posterior</t>
-        </is>
-      </c>
-      <c r="I95" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
-        </is>
-      </c>
-      <c r="J95" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
+          <t>H1 · 18-oct (núcleo Fase 0)</t>
+        </is>
+      </c>
+      <c r="I95" s="19" t="inlineStr">
+        <is>
+          <t>Como iglesia queremos no perder información.</t>
+        </is>
+      </c>
+      <c r="J95" s="19" t="inlineStr">
+        <is>
+          <t>Respaldo diario cifrado y restauración probada en un ambiente de pruebas.</t>
         </is>
       </c>
       <c r="K95" s="19" t="inlineStr">
         <is>
-          <t>Por definir</t>
+          <t>VoBo pendiente</t>
         </is>
       </c>
       <c r="L95" s="19" t="inlineStr">
@@ -8224,7 +8232,7 @@
     <row r="96">
       <c r="A96" s="18" t="inlineStr">
         <is>
-          <t>NF-06</t>
+          <t>NF-05</t>
         </is>
       </c>
       <c r="B96" s="19" t="inlineStr">
@@ -8234,69 +8242,61 @@
       </c>
       <c r="C96" s="19" t="inlineStr">
         <is>
-          <t>Pase de lista sin conexión con sincronización posterior (reuniones en domicilios con mala señal).</t>
-        </is>
-      </c>
-      <c r="D96" s="19" t="inlineStr">
-        <is>
-          <t>v3</t>
+          <t>Disponibilidad esperada en horarios de servicio (fines de semana y reuniones de grupo). Por definir meta.</t>
+        </is>
+      </c>
+      <c r="D96" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3</t>
         </is>
       </c>
       <c r="E96" s="19" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Fuera del MVP</t>
         </is>
       </c>
       <c r="F96" s="19" t="inlineStr">
         <is>
-          <t>Fase 0</t>
+          <t>Transversal</t>
         </is>
       </c>
       <c r="G96" s="19" t="inlineStr">
         <is>
-          <t>Sprint 3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H96" s="19" t="inlineStr">
         <is>
-          <t>H3 · MVP (Grupos)</t>
-        </is>
-      </c>
-      <c r="I96" s="19" t="inlineStr">
-        <is>
-          <t>Como secretario quiero que el pase de lista funcione sin señal.</t>
-        </is>
-      </c>
-      <c r="J96" s="19" t="inlineStr">
-        <is>
-          <t>Prueba en modo avión y sincronización al reconectar.</t>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="I96" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
+        </is>
+      </c>
+      <c r="J96" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
         </is>
       </c>
       <c r="K96" s="19" t="inlineStr">
         <is>
-          <t>VoBo pendiente</t>
+          <t>Por definir</t>
         </is>
       </c>
       <c r="L96" s="19" t="inlineStr">
         <is>
-          <t>En pruebas</t>
-        </is>
-      </c>
-      <c r="M96" s="19" t="inlineStr">
-        <is>
-          <t>Rama feature/nf-06-sin-conexion · 117 pruebas de backend y 27 de frontend; probado en Chrome real con service worker</t>
-        </is>
-      </c>
-      <c r="N96" s="19" t="inlineStr">
-        <is>
-          <t>2026-10-24 · Probado de punta a punta en Chrome (sin red → cola → sincronización). Pendiente probar en Android e iOS reales.</t>
-        </is>
-      </c>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M96" s="19" t="inlineStr"/>
+      <c r="N96" s="19" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" s="18" t="inlineStr">
         <is>
-          <t>NF-07</t>
+          <t>NF-06</t>
         </is>
       </c>
       <c r="B97" s="19" t="inlineStr">
@@ -8306,7 +8306,7 @@
       </c>
       <c r="C97" s="19" t="inlineStr">
         <is>
-          <t>Funciona en Android, iOS y escritorio. En iOS, las notificaciones push requieren instalar la PWA; el respaldo por WhatsApp cubre el resto.</t>
+          <t>Pase de lista sin conexión con sincronización posterior (reuniones en domicilios con mala señal).</t>
         </is>
       </c>
       <c r="D97" s="19" t="inlineStr">
@@ -8326,22 +8326,22 @@
       </c>
       <c r="G97" s="19" t="inlineStr">
         <is>
-          <t>Sprint 0</t>
+          <t>Sprint 3</t>
         </is>
       </c>
       <c r="H97" s="19" t="inlineStr">
         <is>
-          <t>H1 · 18-oct (núcleo Fase 0)</t>
+          <t>H3 · MVP (Grupos)</t>
         </is>
       </c>
       <c r="I97" s="19" t="inlineStr">
         <is>
-          <t>Como usuario quiero usar el sistema en mi dispositivo.</t>
+          <t>Como secretario quiero que el pase de lista funcione sin señal.</t>
         </is>
       </c>
       <c r="J97" s="19" t="inlineStr">
         <is>
-          <t>Pruebas en Android, iOS y escritorio; push en iOS con la PWA instalada y respaldo por WhatsApp.</t>
+          <t>Prueba en modo avión y sincronización al reconectar.</t>
         </is>
       </c>
       <c r="K97" s="19" t="inlineStr">
@@ -8351,16 +8351,24 @@
       </c>
       <c r="L97" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M97" s="19" t="inlineStr"/>
-      <c r="N97" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M97" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/nf-06-sin-conexion · 117 pruebas de backend y 27 de frontend; probado en Chrome real con service worker</t>
+        </is>
+      </c>
+      <c r="N97" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-24 · Probado de punta a punta en Chrome (sin red → cola → sincronización). Pendiente probar en Android e iOS reales.</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="18" t="inlineStr">
         <is>
-          <t>NF-08</t>
+          <t>NF-07</t>
         </is>
       </c>
       <c r="B98" s="19" t="inlineStr">
@@ -8370,12 +8378,12 @@
       </c>
       <c r="C98" s="19" t="inlineStr">
         <is>
-          <t>Dimensionamiento para ~1,000 personas, con picos los fines de semana, y margen de crecimiento.</t>
-        </is>
-      </c>
-      <c r="D98" s="21" t="inlineStr">
-        <is>
-          <t>Resp. P8</t>
+          <t>Funciona en Android, iOS y escritorio. En iOS, las notificaciones push requieren instalar la PWA; el respaldo por WhatsApp cubre el resto.</t>
+        </is>
+      </c>
+      <c r="D98" s="19" t="inlineStr">
+        <is>
+          <t>v3</t>
         </is>
       </c>
       <c r="E98" s="19" t="inlineStr">
@@ -8400,12 +8408,12 @@
       </c>
       <c r="I98" s="19" t="inlineStr">
         <is>
-          <t>Como iglesia queremos que el sistema soporte a ~1,000 personas.</t>
+          <t>Como usuario quiero usar el sistema en mi dispositivo.</t>
         </is>
       </c>
       <c r="J98" s="19" t="inlineStr">
         <is>
-          <t>Prueba de carga con volumen representativo (por definir) sin degradación.</t>
+          <t>Pruebas en Android, iOS y escritorio; push en iOS con la PWA instalada y respaldo por WhatsApp.</t>
         </is>
       </c>
       <c r="K98" s="19" t="inlineStr">
@@ -8424,7 +8432,7 @@
     <row r="99">
       <c r="A99" s="18" t="inlineStr">
         <is>
-          <t>NF-09</t>
+          <t>NF-08</t>
         </is>
       </c>
       <c r="B99" s="19" t="inlineStr">
@@ -8434,42 +8442,42 @@
       </c>
       <c r="C99" s="19" t="inlineStr">
         <is>
-          <t>Reportes transversales: asistencia, finanzas, crecimiento de la iglesia, exportables a Excel y PDF.</t>
+          <t>Dimensionamiento para ~1,000 personas, con picos los fines de semana, y margen de crecimiento.</t>
         </is>
       </c>
       <c r="D99" s="21" t="inlineStr">
         <is>
-          <t>Nuevo v3</t>
+          <t>Resp. P8</t>
         </is>
       </c>
       <c r="E99" s="19" t="inlineStr">
         <is>
-          <t>Fuera del MVP</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="F99" s="19" t="inlineStr">
         <is>
-          <t>Transversal</t>
+          <t>Fase 0</t>
         </is>
       </c>
       <c r="G99" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sprint 0</t>
         </is>
       </c>
       <c r="H99" s="19" t="inlineStr">
         <is>
-          <t>Posterior</t>
-        </is>
-      </c>
-      <c r="I99" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
-        </is>
-      </c>
-      <c r="J99" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
+          <t>H1 · 18-oct (núcleo Fase 0)</t>
+        </is>
+      </c>
+      <c r="I99" s="19" t="inlineStr">
+        <is>
+          <t>Como iglesia queremos que el sistema soporte a ~1,000 personas.</t>
+        </is>
+      </c>
+      <c r="J99" s="19" t="inlineStr">
+        <is>
+          <t>Prueba de carga con volumen representativo (por definir) sin degradación.</t>
         </is>
       </c>
       <c r="K99" s="19" t="inlineStr">
@@ -8488,7 +8496,7 @@
     <row r="100">
       <c r="A100" s="18" t="inlineStr">
         <is>
-          <t>NF-10</t>
+          <t>NF-09</t>
         </is>
       </c>
       <c r="B100" s="19" t="inlineStr">
@@ -8498,42 +8506,42 @@
       </c>
       <c r="C100" s="19" t="inlineStr">
         <is>
-          <t>Usabilidad para personas mayores: tipografía grande, alto contraste, flujos cortos (ver sección 5).</t>
-        </is>
-      </c>
-      <c r="D100" s="19" t="inlineStr">
-        <is>
-          <t>v3 + Obs. 1</t>
+          <t>Reportes transversales: asistencia, finanzas, crecimiento de la iglesia, exportables a Excel y PDF.</t>
+        </is>
+      </c>
+      <c r="D100" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3</t>
         </is>
       </c>
       <c r="E100" s="19" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Fuera del MVP</t>
         </is>
       </c>
       <c r="F100" s="19" t="inlineStr">
         <is>
-          <t>Fase 0</t>
+          <t>Transversal</t>
         </is>
       </c>
       <c r="G100" s="19" t="inlineStr">
         <is>
-          <t>Sprint 0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H100" s="19" t="inlineStr">
         <is>
-          <t>H1 · 18-oct (núcleo Fase 0)</t>
-        </is>
-      </c>
-      <c r="I100" s="19" t="inlineStr">
-        <is>
-          <t>Como persona mayor quiero una interfaz fácil de leer y usar.</t>
-        </is>
-      </c>
-      <c r="J100" s="19" t="inlineStr">
-        <is>
-          <t>Texto base 18 px, botones de al menos 48 px, contraste AA; prueba con usuarios mayores.</t>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="I100" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
+        </is>
+      </c>
+      <c r="J100" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
         </is>
       </c>
       <c r="K100" s="19" t="inlineStr">
@@ -8549,9 +8557,73 @@
       <c r="M100" s="19" t="inlineStr"/>
       <c r="N100" s="19" t="inlineStr"/>
     </row>
+    <row r="101">
+      <c r="A101" s="18" t="inlineStr">
+        <is>
+          <t>NF-10</t>
+        </is>
+      </c>
+      <c r="B101" s="19" t="inlineStr">
+        <is>
+          <t>No funcionales</t>
+        </is>
+      </c>
+      <c r="C101" s="19" t="inlineStr">
+        <is>
+          <t>Usabilidad para personas mayores: tipografía grande, alto contraste, flujos cortos (ver sección 5).</t>
+        </is>
+      </c>
+      <c r="D101" s="19" t="inlineStr">
+        <is>
+          <t>v3 + Obs. 1</t>
+        </is>
+      </c>
+      <c r="E101" s="19" t="inlineStr">
+        <is>
+          <t>MVP</t>
+        </is>
+      </c>
+      <c r="F101" s="19" t="inlineStr">
+        <is>
+          <t>Fase 0</t>
+        </is>
+      </c>
+      <c r="G101" s="19" t="inlineStr">
+        <is>
+          <t>Sprint 0</t>
+        </is>
+      </c>
+      <c r="H101" s="19" t="inlineStr">
+        <is>
+          <t>H1 · 18-oct (núcleo Fase 0)</t>
+        </is>
+      </c>
+      <c r="I101" s="19" t="inlineStr">
+        <is>
+          <t>Como persona mayor quiero una interfaz fácil de leer y usar.</t>
+        </is>
+      </c>
+      <c r="J101" s="19" t="inlineStr">
+        <is>
+          <t>Texto base 18 px, botones de al menos 48 px, contraste AA; prueba con usuarios mayores.</t>
+        </is>
+      </c>
+      <c r="K101" s="19" t="inlineStr">
+        <is>
+          <t>VoBo pendiente</t>
+        </is>
+      </c>
+      <c r="L101" s="19" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M101" s="19" t="inlineStr"/>
+      <c r="N101" s="19" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N100"/>
-  <conditionalFormatting sqref="L2:L100">
+  <autoFilter ref="A1:N101"/>
+  <conditionalFormatting sqref="L2:L101">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$L2="Hecho"</formula>
     </cfRule>
@@ -8568,7 +8640,7 @@
       <formula>$L2="Bloqueado"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K2:K100">
+  <conditionalFormatting sqref="K2:K101">
     <cfRule type="expression" priority="6" dxfId="0">
       <formula>$K2="Aprobado"</formula>
     </cfRule>
@@ -8576,16 +8648,16 @@
       <formula>$K2="Por definir"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H2:H100">
+  <conditionalFormatting sqref="H2:H101">
     <cfRule type="expression" priority="8" dxfId="5">
       <formula>LEFT($H2,2)="H1"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="L2:L100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="L2:L101" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Pendiente,En diseño,En desarrollo,En pruebas,Hecho,Bloqueado"</formula1>
     </dataValidation>
-    <dataValidation sqref="K2:K100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="K2:K101" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"VoBo pendiente,Aprobado,Por definir,Rechazado"</formula1>
     </dataValidation>
   </dataValidations>
@@ -9383,12 +9455,12 @@
       </c>
       <c r="D29" s="24" t="inlineStr">
         <is>
-          <t>Requiere definir ministerios como áreas de servicio.</t>
+          <t>Los ministerios se manejan como unidades (áreas de servicio). Avisos masivos a iglesia, grupos, unidades y personas, con permisos por destino, y avisos recibidos agrupados.</t>
         </is>
       </c>
       <c r="E29" s="24" t="inlineStr">
         <is>
-          <t>Planeado (paso 6)</t>
+          <t>Hecho (v3.20)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ministerios, roles de grupos y ministerios configurables, peticiones por ministerio y Mi cuenta (paso 8)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/trazabilidad/Matriz de Trazabilidad MDF.xlsx
+++ b/docs/trazabilidad/Matriz de Trazabilidad MDF.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Origen v1" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Matriz'!$A$1:$N$101</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Matriz'!$A$1:$N$103</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -897,31 +897,31 @@
         </is>
       </c>
       <c r="B5" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$101,$A5)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$103,$A5)</f>
         <v/>
       </c>
       <c r="C5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$101,$A5,Matriz!$L$2:$L$101,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$103,$A5,Matriz!$L$2:$L$103,"Pendiente")</f>
         <v/>
       </c>
       <c r="D5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$101,$A5,Matriz!$L$2:$L$101,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$103,$A5,Matriz!$L$2:$L$103,"En diseño")</f>
         <v/>
       </c>
       <c r="E5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$101,$A5,Matriz!$L$2:$L$101,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$103,$A5,Matriz!$L$2:$L$103,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$101,$A5,Matriz!$L$2:$L$101,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$103,$A5,Matriz!$L$2:$L$103,"En pruebas")</f>
         <v/>
       </c>
       <c r="G5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$101,$A5,Matriz!$L$2:$L$101,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$103,$A5,Matriz!$L$2:$L$103,"Hecho")</f>
         <v/>
       </c>
       <c r="H5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$101,$A5,Matriz!$L$2:$L$101,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$103,$A5,Matriz!$L$2:$L$103,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I5" s="13">
@@ -936,31 +936,31 @@
         </is>
       </c>
       <c r="B6" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$101,$A6)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$103,$A6)</f>
         <v/>
       </c>
       <c r="C6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$101,$A6,Matriz!$L$2:$L$101,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$103,$A6,Matriz!$L$2:$L$103,"Pendiente")</f>
         <v/>
       </c>
       <c r="D6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$101,$A6,Matriz!$L$2:$L$101,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$103,$A6,Matriz!$L$2:$L$103,"En diseño")</f>
         <v/>
       </c>
       <c r="E6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$101,$A6,Matriz!$L$2:$L$101,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$103,$A6,Matriz!$L$2:$L$103,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$101,$A6,Matriz!$L$2:$L$101,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$103,$A6,Matriz!$L$2:$L$103,"En pruebas")</f>
         <v/>
       </c>
       <c r="G6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$101,$A6,Matriz!$L$2:$L$101,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$103,$A6,Matriz!$L$2:$L$103,"Hecho")</f>
         <v/>
       </c>
       <c r="H6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$101,$A6,Matriz!$L$2:$L$101,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$103,$A6,Matriz!$L$2:$L$103,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I6" s="13">
@@ -975,31 +975,31 @@
         </is>
       </c>
       <c r="B7" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$101,$A7)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$103,$A7)</f>
         <v/>
       </c>
       <c r="C7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$101,$A7,Matriz!$L$2:$L$101,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$103,$A7,Matriz!$L$2:$L$103,"Pendiente")</f>
         <v/>
       </c>
       <c r="D7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$101,$A7,Matriz!$L$2:$L$101,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$103,$A7,Matriz!$L$2:$L$103,"En diseño")</f>
         <v/>
       </c>
       <c r="E7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$101,$A7,Matriz!$L$2:$L$101,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$103,$A7,Matriz!$L$2:$L$103,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$101,$A7,Matriz!$L$2:$L$101,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$103,$A7,Matriz!$L$2:$L$103,"En pruebas")</f>
         <v/>
       </c>
       <c r="G7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$101,$A7,Matriz!$L$2:$L$101,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$103,$A7,Matriz!$L$2:$L$103,"Hecho")</f>
         <v/>
       </c>
       <c r="H7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$101,$A7,Matriz!$L$2:$L$101,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$103,$A7,Matriz!$L$2:$L$103,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I7" s="13">
@@ -1014,31 +1014,31 @@
         </is>
       </c>
       <c r="B8" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$101,$A8)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$103,$A8)</f>
         <v/>
       </c>
       <c r="C8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$101,$A8,Matriz!$L$2:$L$101,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$103,$A8,Matriz!$L$2:$L$103,"Pendiente")</f>
         <v/>
       </c>
       <c r="D8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$101,$A8,Matriz!$L$2:$L$101,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$103,$A8,Matriz!$L$2:$L$103,"En diseño")</f>
         <v/>
       </c>
       <c r="E8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$101,$A8,Matriz!$L$2:$L$101,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$103,$A8,Matriz!$L$2:$L$103,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$101,$A8,Matriz!$L$2:$L$101,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$103,$A8,Matriz!$L$2:$L$103,"En pruebas")</f>
         <v/>
       </c>
       <c r="G8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$101,$A8,Matriz!$L$2:$L$101,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$103,$A8,Matriz!$L$2:$L$103,"Hecho")</f>
         <v/>
       </c>
       <c r="H8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$101,$A8,Matriz!$L$2:$L$101,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$103,$A8,Matriz!$L$2:$L$103,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I8" s="13">
@@ -1053,31 +1053,31 @@
         </is>
       </c>
       <c r="B9" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$101,$A9)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$103,$A9)</f>
         <v/>
       </c>
       <c r="C9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$101,$A9,Matriz!$L$2:$L$101,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$103,$A9,Matriz!$L$2:$L$103,"Pendiente")</f>
         <v/>
       </c>
       <c r="D9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$101,$A9,Matriz!$L$2:$L$101,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$103,$A9,Matriz!$L$2:$L$103,"En diseño")</f>
         <v/>
       </c>
       <c r="E9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$101,$A9,Matriz!$L$2:$L$101,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$103,$A9,Matriz!$L$2:$L$103,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$101,$A9,Matriz!$L$2:$L$101,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$103,$A9,Matriz!$L$2:$L$103,"En pruebas")</f>
         <v/>
       </c>
       <c r="G9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$101,$A9,Matriz!$L$2:$L$101,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$103,$A9,Matriz!$L$2:$L$103,"Hecho")</f>
         <v/>
       </c>
       <c r="H9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$101,$A9,Matriz!$L$2:$L$101,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$103,$A9,Matriz!$L$2:$L$103,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I9" s="13">
@@ -1092,31 +1092,31 @@
         </is>
       </c>
       <c r="B10" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$101,$A10)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$103,$A10)</f>
         <v/>
       </c>
       <c r="C10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$101,$A10,Matriz!$L$2:$L$101,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$103,$A10,Matriz!$L$2:$L$103,"Pendiente")</f>
         <v/>
       </c>
       <c r="D10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$101,$A10,Matriz!$L$2:$L$101,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$103,$A10,Matriz!$L$2:$L$103,"En diseño")</f>
         <v/>
       </c>
       <c r="E10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$101,$A10,Matriz!$L$2:$L$101,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$103,$A10,Matriz!$L$2:$L$103,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$101,$A10,Matriz!$L$2:$L$101,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$103,$A10,Matriz!$L$2:$L$103,"En pruebas")</f>
         <v/>
       </c>
       <c r="G10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$101,$A10,Matriz!$L$2:$L$101,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$103,$A10,Matriz!$L$2:$L$103,"Hecho")</f>
         <v/>
       </c>
       <c r="H10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$101,$A10,Matriz!$L$2:$L$101,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$103,$A10,Matriz!$L$2:$L$103,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I10" s="13">
@@ -1131,31 +1131,31 @@
         </is>
       </c>
       <c r="B11" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$101,$A11)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$103,$A11)</f>
         <v/>
       </c>
       <c r="C11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$101,$A11,Matriz!$L$2:$L$101,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$103,$A11,Matriz!$L$2:$L$103,"Pendiente")</f>
         <v/>
       </c>
       <c r="D11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$101,$A11,Matriz!$L$2:$L$101,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$103,$A11,Matriz!$L$2:$L$103,"En diseño")</f>
         <v/>
       </c>
       <c r="E11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$101,$A11,Matriz!$L$2:$L$101,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$103,$A11,Matriz!$L$2:$L$103,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$101,$A11,Matriz!$L$2:$L$101,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$103,$A11,Matriz!$L$2:$L$103,"En pruebas")</f>
         <v/>
       </c>
       <c r="G11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$101,$A11,Matriz!$L$2:$L$101,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$103,$A11,Matriz!$L$2:$L$103,"Hecho")</f>
         <v/>
       </c>
       <c r="H11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$101,$A11,Matriz!$L$2:$L$101,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$103,$A11,Matriz!$L$2:$L$103,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I11" s="13">
@@ -1256,31 +1256,31 @@
         </is>
       </c>
       <c r="B16" s="12">
-        <f>COUNTIF(Matriz!$H$2:$H$101,$A16)</f>
+        <f>COUNTIF(Matriz!$H$2:$H$103,$A16)</f>
         <v/>
       </c>
       <c r="C16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$101,$A16,Matriz!$L$2:$L$101,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$103,$A16,Matriz!$L$2:$L$103,"Pendiente")</f>
         <v/>
       </c>
       <c r="D16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$101,$A16,Matriz!$L$2:$L$101,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$103,$A16,Matriz!$L$2:$L$103,"En diseño")</f>
         <v/>
       </c>
       <c r="E16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$101,$A16,Matriz!$L$2:$L$101,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$103,$A16,Matriz!$L$2:$L$103,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$101,$A16,Matriz!$L$2:$L$101,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$103,$A16,Matriz!$L$2:$L$103,"En pruebas")</f>
         <v/>
       </c>
       <c r="G16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$101,$A16,Matriz!$L$2:$L$101,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$103,$A16,Matriz!$L$2:$L$103,"Hecho")</f>
         <v/>
       </c>
       <c r="H16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$101,$A16,Matriz!$L$2:$L$101,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$103,$A16,Matriz!$L$2:$L$103,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I16" s="13">
@@ -1295,31 +1295,31 @@
         </is>
       </c>
       <c r="B17" s="12">
-        <f>COUNTIF(Matriz!$H$2:$H$101,$A17)</f>
+        <f>COUNTIF(Matriz!$H$2:$H$103,$A17)</f>
         <v/>
       </c>
       <c r="C17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$101,$A17,Matriz!$L$2:$L$101,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$103,$A17,Matriz!$L$2:$L$103,"Pendiente")</f>
         <v/>
       </c>
       <c r="D17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$101,$A17,Matriz!$L$2:$L$101,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$103,$A17,Matriz!$L$2:$L$103,"En diseño")</f>
         <v/>
       </c>
       <c r="E17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$101,$A17,Matriz!$L$2:$L$101,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$103,$A17,Matriz!$L$2:$L$103,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$101,$A17,Matriz!$L$2:$L$101,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$103,$A17,Matriz!$L$2:$L$103,"En pruebas")</f>
         <v/>
       </c>
       <c r="G17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$101,$A17,Matriz!$L$2:$L$101,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$103,$A17,Matriz!$L$2:$L$103,"Hecho")</f>
         <v/>
       </c>
       <c r="H17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$101,$A17,Matriz!$L$2:$L$101,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$103,$A17,Matriz!$L$2:$L$103,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I17" s="13">
@@ -1334,31 +1334,31 @@
         </is>
       </c>
       <c r="B18" s="12">
-        <f>COUNTIF(Matriz!$H$2:$H$101,$A18)</f>
+        <f>COUNTIF(Matriz!$H$2:$H$103,$A18)</f>
         <v/>
       </c>
       <c r="C18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$101,$A18,Matriz!$L$2:$L$101,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$103,$A18,Matriz!$L$2:$L$103,"Pendiente")</f>
         <v/>
       </c>
       <c r="D18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$101,$A18,Matriz!$L$2:$L$101,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$103,$A18,Matriz!$L$2:$L$103,"En diseño")</f>
         <v/>
       </c>
       <c r="E18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$101,$A18,Matriz!$L$2:$L$101,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$103,$A18,Matriz!$L$2:$L$103,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$101,$A18,Matriz!$L$2:$L$101,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$103,$A18,Matriz!$L$2:$L$103,"En pruebas")</f>
         <v/>
       </c>
       <c r="G18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$101,$A18,Matriz!$L$2:$L$101,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$103,$A18,Matriz!$L$2:$L$103,"Hecho")</f>
         <v/>
       </c>
       <c r="H18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$101,$A18,Matriz!$L$2:$L$101,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$103,$A18,Matriz!$L$2:$L$103,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I18" s="13">
@@ -1373,31 +1373,31 @@
         </is>
       </c>
       <c r="B19" s="12">
-        <f>COUNTIF(Matriz!$H$2:$H$101,$A19)</f>
+        <f>COUNTIF(Matriz!$H$2:$H$103,$A19)</f>
         <v/>
       </c>
       <c r="C19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$101,$A19,Matriz!$L$2:$L$101,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$103,$A19,Matriz!$L$2:$L$103,"Pendiente")</f>
         <v/>
       </c>
       <c r="D19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$101,$A19,Matriz!$L$2:$L$101,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$103,$A19,Matriz!$L$2:$L$103,"En diseño")</f>
         <v/>
       </c>
       <c r="E19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$101,$A19,Matriz!$L$2:$L$101,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$103,$A19,Matriz!$L$2:$L$103,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$101,$A19,Matriz!$L$2:$L$101,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$103,$A19,Matriz!$L$2:$L$103,"En pruebas")</f>
         <v/>
       </c>
       <c r="G19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$101,$A19,Matriz!$L$2:$L$101,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$103,$A19,Matriz!$L$2:$L$103,"Hecho")</f>
         <v/>
       </c>
       <c r="H19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$101,$A19,Matriz!$L$2:$L$101,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$103,$A19,Matriz!$L$2:$L$103,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I19" s="13">
@@ -1498,31 +1498,31 @@
         </is>
       </c>
       <c r="B24" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$101,$A24)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$103,$A24)</f>
         <v/>
       </c>
       <c r="C24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$101,$A24,Matriz!$L$2:$L$101,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$103,$A24,Matriz!$L$2:$L$103,"Pendiente")</f>
         <v/>
       </c>
       <c r="D24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$101,$A24,Matriz!$L$2:$L$101,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$103,$A24,Matriz!$L$2:$L$103,"En diseño")</f>
         <v/>
       </c>
       <c r="E24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$101,$A24,Matriz!$L$2:$L$101,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$103,$A24,Matriz!$L$2:$L$103,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$101,$A24,Matriz!$L$2:$L$101,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$103,$A24,Matriz!$L$2:$L$103,"En pruebas")</f>
         <v/>
       </c>
       <c r="G24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$101,$A24,Matriz!$L$2:$L$101,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$103,$A24,Matriz!$L$2:$L$103,"Hecho")</f>
         <v/>
       </c>
       <c r="H24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$101,$A24,Matriz!$L$2:$L$101,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$103,$A24,Matriz!$L$2:$L$103,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I24" s="13">
@@ -1537,31 +1537,31 @@
         </is>
       </c>
       <c r="B25" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$101,$A25)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$103,$A25)</f>
         <v/>
       </c>
       <c r="C25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$101,$A25,Matriz!$L$2:$L$101,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$103,$A25,Matriz!$L$2:$L$103,"Pendiente")</f>
         <v/>
       </c>
       <c r="D25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$101,$A25,Matriz!$L$2:$L$101,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$103,$A25,Matriz!$L$2:$L$103,"En diseño")</f>
         <v/>
       </c>
       <c r="E25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$101,$A25,Matriz!$L$2:$L$101,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$103,$A25,Matriz!$L$2:$L$103,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$101,$A25,Matriz!$L$2:$L$101,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$103,$A25,Matriz!$L$2:$L$103,"En pruebas")</f>
         <v/>
       </c>
       <c r="G25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$101,$A25,Matriz!$L$2:$L$101,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$103,$A25,Matriz!$L$2:$L$103,"Hecho")</f>
         <v/>
       </c>
       <c r="H25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$101,$A25,Matriz!$L$2:$L$101,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$103,$A25,Matriz!$L$2:$L$103,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I25" s="13">
@@ -1576,31 +1576,31 @@
         </is>
       </c>
       <c r="B26" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$101,$A26)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$103,$A26)</f>
         <v/>
       </c>
       <c r="C26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$101,$A26,Matriz!$L$2:$L$101,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$103,$A26,Matriz!$L$2:$L$103,"Pendiente")</f>
         <v/>
       </c>
       <c r="D26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$101,$A26,Matriz!$L$2:$L$101,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$103,$A26,Matriz!$L$2:$L$103,"En diseño")</f>
         <v/>
       </c>
       <c r="E26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$101,$A26,Matriz!$L$2:$L$101,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$103,$A26,Matriz!$L$2:$L$103,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$101,$A26,Matriz!$L$2:$L$101,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$103,$A26,Matriz!$L$2:$L$103,"En pruebas")</f>
         <v/>
       </c>
       <c r="G26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$101,$A26,Matriz!$L$2:$L$101,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$103,$A26,Matriz!$L$2:$L$103,"Hecho")</f>
         <v/>
       </c>
       <c r="H26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$101,$A26,Matriz!$L$2:$L$101,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$103,$A26,Matriz!$L$2:$L$103,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I26" s="13">
@@ -1615,31 +1615,31 @@
         </is>
       </c>
       <c r="B27" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$101,$A27)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$103,$A27)</f>
         <v/>
       </c>
       <c r="C27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$101,$A27,Matriz!$L$2:$L$101,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$103,$A27,Matriz!$L$2:$L$103,"Pendiente")</f>
         <v/>
       </c>
       <c r="D27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$101,$A27,Matriz!$L$2:$L$101,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$103,$A27,Matriz!$L$2:$L$103,"En diseño")</f>
         <v/>
       </c>
       <c r="E27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$101,$A27,Matriz!$L$2:$L$101,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$103,$A27,Matriz!$L$2:$L$103,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$101,$A27,Matriz!$L$2:$L$101,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$103,$A27,Matriz!$L$2:$L$103,"En pruebas")</f>
         <v/>
       </c>
       <c r="G27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$101,$A27,Matriz!$L$2:$L$101,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$103,$A27,Matriz!$L$2:$L$103,"Hecho")</f>
         <v/>
       </c>
       <c r="H27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$101,$A27,Matriz!$L$2:$L$101,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$103,$A27,Matriz!$L$2:$L$103,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I27" s="13">
@@ -1654,31 +1654,31 @@
         </is>
       </c>
       <c r="B28" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$101,$A28)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$103,$A28)</f>
         <v/>
       </c>
       <c r="C28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$101,$A28,Matriz!$L$2:$L$101,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$103,$A28,Matriz!$L$2:$L$103,"Pendiente")</f>
         <v/>
       </c>
       <c r="D28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$101,$A28,Matriz!$L$2:$L$101,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$103,$A28,Matriz!$L$2:$L$103,"En diseño")</f>
         <v/>
       </c>
       <c r="E28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$101,$A28,Matriz!$L$2:$L$101,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$103,$A28,Matriz!$L$2:$L$103,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$101,$A28,Matriz!$L$2:$L$101,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$103,$A28,Matriz!$L$2:$L$103,"En pruebas")</f>
         <v/>
       </c>
       <c r="G28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$101,$A28,Matriz!$L$2:$L$101,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$103,$A28,Matriz!$L$2:$L$103,"Hecho")</f>
         <v/>
       </c>
       <c r="H28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$101,$A28,Matriz!$L$2:$L$101,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$103,$A28,Matriz!$L$2:$L$103,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I28" s="13">
@@ -1693,31 +1693,31 @@
         </is>
       </c>
       <c r="B29" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$101,$A29)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$103,$A29)</f>
         <v/>
       </c>
       <c r="C29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$101,$A29,Matriz!$L$2:$L$101,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$103,$A29,Matriz!$L$2:$L$103,"Pendiente")</f>
         <v/>
       </c>
       <c r="D29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$101,$A29,Matriz!$L$2:$L$101,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$103,$A29,Matriz!$L$2:$L$103,"En diseño")</f>
         <v/>
       </c>
       <c r="E29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$101,$A29,Matriz!$L$2:$L$101,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$103,$A29,Matriz!$L$2:$L$103,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$101,$A29,Matriz!$L$2:$L$101,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$103,$A29,Matriz!$L$2:$L$103,"En pruebas")</f>
         <v/>
       </c>
       <c r="G29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$101,$A29,Matriz!$L$2:$L$101,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$103,$A29,Matriz!$L$2:$L$103,"Hecho")</f>
         <v/>
       </c>
       <c r="H29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$101,$A29,Matriz!$L$2:$L$101,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$103,$A29,Matriz!$L$2:$L$103,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I29" s="13">
@@ -1732,31 +1732,31 @@
         </is>
       </c>
       <c r="B30" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$101,$A30)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$103,$A30)</f>
         <v/>
       </c>
       <c r="C30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$101,$A30,Matriz!$L$2:$L$101,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$103,$A30,Matriz!$L$2:$L$103,"Pendiente")</f>
         <v/>
       </c>
       <c r="D30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$101,$A30,Matriz!$L$2:$L$101,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$103,$A30,Matriz!$L$2:$L$103,"En diseño")</f>
         <v/>
       </c>
       <c r="E30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$101,$A30,Matriz!$L$2:$L$101,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$103,$A30,Matriz!$L$2:$L$103,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$101,$A30,Matriz!$L$2:$L$101,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$103,$A30,Matriz!$L$2:$L$103,"En pruebas")</f>
         <v/>
       </c>
       <c r="G30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$101,$A30,Matriz!$L$2:$L$101,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$103,$A30,Matriz!$L$2:$L$103,"Hecho")</f>
         <v/>
       </c>
       <c r="H30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$101,$A30,Matriz!$L$2:$L$101,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$103,$A30,Matriz!$L$2:$L$103,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I30" s="13">
@@ -1818,7 +1818,7 @@
         </is>
       </c>
       <c r="B35" s="12">
-        <f>COUNTIF(Matriz!$K$2:$K$101,A35)</f>
+        <f>COUNTIF(Matriz!$K$2:$K$103,A35)</f>
         <v/>
       </c>
     </row>
@@ -1829,7 +1829,7 @@
         </is>
       </c>
       <c r="B36" s="12">
-        <f>COUNTIF(Matriz!$K$2:$K$101,A36)</f>
+        <f>COUNTIF(Matriz!$K$2:$K$103,A36)</f>
         <v/>
       </c>
     </row>
@@ -1840,7 +1840,7 @@
         </is>
       </c>
       <c r="B37" s="12">
-        <f>COUNTIF(Matriz!$K$2:$K$101,A37)</f>
+        <f>COUNTIF(Matriz!$K$2:$K$103,A37)</f>
         <v/>
       </c>
     </row>
@@ -1851,7 +1851,7 @@
         </is>
       </c>
       <c r="B38" s="12">
-        <f>COUNTIF(Matriz!$K$2:$K$101,A38)</f>
+        <f>COUNTIF(Matriz!$K$2:$K$103,A38)</f>
         <v/>
       </c>
     </row>
@@ -1866,7 +1866,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N101"/>
+  <dimension ref="A1:N103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4018,12 +4018,12 @@
       </c>
       <c r="C32" s="19" t="inlineStr">
         <is>
-          <t>Unidades: áreas de servicio de la iglesia (cafetería, librería, niños, danza, etc.), cada una con encargado, respaldo y servidores. Quien participa en una unidad ve solo esa unidad, y su rol vale únicamente dentro de ella, independiente de sus roles en grupos u otras unidades. Cada unidad tiene su propio tablero de avisos.</t>
+          <t>Ministerios: áreas de servicio de la iglesia (cafetería, librería, niños, danza, etc.), cada uno con encargado, respaldo y servidores. Quien participa en un ministerio ve solo ese ministerio, y su rol vale únicamente dentro de él, independiente de sus roles en grupos u otros ministerios. Cada ministerio tiene su propio tablero de avisos y sus peticiones de oración.</t>
         </is>
       </c>
       <c r="D32" s="21" t="inlineStr">
         <is>
-          <t>Respuesta v3.20</t>
+          <t>Respuesta v3.21</t>
         </is>
       </c>
       <c r="E32" s="19" t="inlineStr">
@@ -4048,7 +4048,7 @@
       </c>
       <c r="I32" s="19" t="inlineStr">
         <is>
-          <t>Como encargado de una unidad quiero administrar a mi gente y mis avisos sin ver lo de otras unidades ni grupos.</t>
+          <t>Como encargado de un ministerio quiero administrar a mi gente y mis avisos sin ver lo de otros ministerios ni grupos.</t>
         </is>
       </c>
       <c r="J32" s="19" t="inlineStr">
@@ -4068,64 +4068,64 @@
       </c>
       <c r="M32" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/paso-7-unidades-avisos · pruebas de backend y 103 de frontend pasan; lint, estilos y compilación limpios</t>
+          <t>Rama feature/paso-8-ministerios-mi-cuenta · pruebas de backend y 108 de frontend pasan; lint, estilos y compilación limpios</t>
         </is>
       </c>
       <c r="N32" s="19" t="inlineStr">
         <is>
-          <t>2026-10-29 · Unidades con encargado, respaldo y servidores, alcance propio por unidad y tablero de avisos. Los roles de unidad son fijos; falta moverlos a la matriz de permisos.</t>
+          <t>2026-10-30 · Ministerios (antes unidades) con encargado, respaldo y servidores, alcance propio, tablero de avisos y peticiones de oración.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="18" t="inlineStr">
         <is>
-          <t>M2A-01</t>
+          <t>M1-26</t>
         </is>
       </c>
       <c r="B33" s="19" t="inlineStr">
         <is>
-          <t>M2A Cursos de Vida</t>
+          <t>M1 Identidad y comunicación</t>
         </is>
       </c>
       <c r="C33" s="19" t="inlineStr">
         <is>
-          <t>Catálogo dinámico de cursos; se pueden crear nuevos sin intervención técnica. Incluye «Resolución de Varones» y «Toma de Buenas Decisiones», omitidos en v2.</t>
-        </is>
-      </c>
-      <c r="D33" s="22" t="inlineStr">
-        <is>
-          <t>Recuperado v1</t>
+          <t>Roles de grupos y de ministerios configurables: encargado (líder en un grupo), respaldo y servidores, además de los roles que ya existían. Quien administra roles (Super Usuario, Pastor y Secretaria) crea roles y elige, por acción, lo que puede hacer quien los tiene dentro de un grupo o de un ministerio.</t>
+        </is>
+      </c>
+      <c r="D33" s="21" t="inlineStr">
+        <is>
+          <t>Respuesta v3.21</t>
         </is>
       </c>
       <c r="E33" s="19" t="inlineStr">
         <is>
-          <t>Fuera del MVP</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="F33" s="19" t="inlineStr">
         <is>
-          <t>Fase 3</t>
+          <t>Fase 0</t>
         </is>
       </c>
       <c r="G33" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sprint 5</t>
         </is>
       </c>
       <c r="H33" s="19" t="inlineStr">
         <is>
-          <t>Posterior</t>
-        </is>
-      </c>
-      <c r="I33" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
-        </is>
-      </c>
-      <c r="J33" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
+          <t>H2 · Fase 0 completa</t>
+        </is>
+      </c>
+      <c r="I33" s="19" t="inlineStr">
+        <is>
+          <t>Como administrador quiero definir qué puede hacer el encargado, el respaldo y los servidores de cada grupo y ministerio, para no depender de reglas fijas.</t>
+        </is>
+      </c>
+      <c r="J33" s="19" t="inlineStr">
+        <is>
+          <t>Crear un rol de ministerio con permisos; quitarle un permiso al encargado cambia lo que puede hacer; un rol que administra gente solo lo asigna la administración; un rol base no se desactiva.</t>
         </is>
       </c>
       <c r="K33" s="19" t="inlineStr">
@@ -4135,61 +4135,69 @@
       </c>
       <c r="L33" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M33" s="19" t="inlineStr"/>
-      <c r="N33" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M33" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/paso-8-ministerios-mi-cuenta · pruebas de backend y 108 de frontend pasan; lint, estilos y compilación limpios</t>
+        </is>
+      </c>
+      <c r="N33" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-30 · Roles de ministerio y de grupo configurables desde Roles y permisos; roles base y roles nuevos; las ofrendas y peticiones de grupo siguen con reglas fijas.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="18" t="inlineStr">
         <is>
-          <t>M2A-02</t>
+          <t>M1-27</t>
         </is>
       </c>
       <c r="B34" s="19" t="inlineStr">
         <is>
-          <t>M2A Cursos de Vida</t>
+          <t>M1 Identidad y comunicación</t>
         </is>
       </c>
       <c r="C34" s="19" t="inlineStr">
         <is>
-          <t>Flexibilidad operativa: sin día ni horario fijo; el día y el ponente pueden cambiar entre ediciones.</t>
-        </is>
-      </c>
-      <c r="D34" s="19" t="inlineStr">
-        <is>
-          <t>v1 / v2</t>
+          <t>Mi cuenta: la persona corrige sus datos básicos (nombre, fecha de nacimiento, domicilio, teléfono fijo, devocional, oración de familias y foto). No edita nada que afecte su acceso (WhatsApp, correo, PIN) ni sus relaciones con la iglesia (grupo, sector, ministerios, roles, nivel).</t>
+        </is>
+      </c>
+      <c r="D34" s="21" t="inlineStr">
+        <is>
+          <t>Respuesta v3.21</t>
         </is>
       </c>
       <c r="E34" s="19" t="inlineStr">
         <is>
-          <t>Fuera del MVP</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="F34" s="19" t="inlineStr">
         <is>
-          <t>Fase 3</t>
+          <t>Fase 0</t>
         </is>
       </c>
       <c r="G34" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sprint 5</t>
         </is>
       </c>
       <c r="H34" s="19" t="inlineStr">
         <is>
-          <t>Posterior</t>
-        </is>
-      </c>
-      <c r="I34" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
-        </is>
-      </c>
-      <c r="J34" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
+          <t>H2 · Fase 0 completa</t>
+        </is>
+      </c>
+      <c r="I34" s="19" t="inlineStr">
+        <is>
+          <t>Como persona quiero corregir mis datos básicos desde Mi cuenta sin poder cambiar mi acceso ni mi grupo.</t>
+        </is>
+      </c>
+      <c r="J34" s="19" t="inlineStr">
+        <is>
+          <t>Corregir nombre y domicilio; intentar cambiar WhatsApp, correo, nivel o grupo no tiene efecto; la foto pide aceptar su uso; la bitácora no guarda los valores.</t>
         </is>
       </c>
       <c r="K34" s="19" t="inlineStr">
@@ -4199,16 +4207,24 @@
       </c>
       <c r="L34" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M34" s="19" t="inlineStr"/>
-      <c r="N34" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M34" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/paso-8-ministerios-mi-cuenta · pruebas de backend y 108 de frontend pasan; lint, estilos y compilación limpios</t>
+        </is>
+      </c>
+      <c r="N34" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-30 · Mi cuenta editable: datos básicos y foto con consentimiento; sin acceso ni relaciones.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="18" t="inlineStr">
         <is>
-          <t>M2A-03</t>
+          <t>M2A-01</t>
         </is>
       </c>
       <c r="B35" s="19" t="inlineStr">
@@ -4218,12 +4234,12 @@
       </c>
       <c r="C35" s="19" t="inlineStr">
         <is>
-          <t>Reposición de clases: el inscrito puede reponer en otro grupo o con otro ponente, a decisión de quien imparte.</t>
-        </is>
-      </c>
-      <c r="D35" s="19" t="inlineStr">
-        <is>
-          <t>v1 / v2</t>
+          <t>Catálogo dinámico de cursos; se pueden crear nuevos sin intervención técnica. Incluye «Resolución de Varones» y «Toma de Buenas Decisiones», omitidos en v2.</t>
+        </is>
+      </c>
+      <c r="D35" s="22" t="inlineStr">
+        <is>
+          <t>Recuperado v1</t>
         </is>
       </c>
       <c r="E35" s="19" t="inlineStr">
@@ -4272,7 +4288,7 @@
     <row r="36">
       <c r="A36" s="18" t="inlineStr">
         <is>
-          <t>M2A-04</t>
+          <t>M2A-02</t>
         </is>
       </c>
       <c r="B36" s="19" t="inlineStr">
@@ -4282,7 +4298,7 @@
       </c>
       <c r="C36" s="19" t="inlineStr">
         <is>
-          <t>Registro de asistencia por sesión.</t>
+          <t>Flexibilidad operativa: sin día ni horario fijo; el día y el ponente pueden cambiar entre ediciones.</t>
         </is>
       </c>
       <c r="D36" s="19" t="inlineStr">
@@ -4336,7 +4352,7 @@
     <row r="37">
       <c r="A37" s="18" t="inlineStr">
         <is>
-          <t>M2A-05</t>
+          <t>M2A-03</t>
         </is>
       </c>
       <c r="B37" s="19" t="inlineStr">
@@ -4346,7 +4362,7 @@
       </c>
       <c r="C37" s="19" t="inlineStr">
         <is>
-          <t>Seguimiento de tareas o actividades opcionales (no sumativas).</t>
+          <t>Reposición de clases: el inscrito puede reponer en otro grupo o con otro ponente, a decisión de quien imparte.</t>
         </is>
       </c>
       <c r="D37" s="19" t="inlineStr">
@@ -4400,7 +4416,7 @@
     <row r="38">
       <c r="A38" s="18" t="inlineStr">
         <is>
-          <t>M2A-06</t>
+          <t>M2A-04</t>
         </is>
       </c>
       <c r="B38" s="19" t="inlineStr">
@@ -4410,7 +4426,7 @@
       </c>
       <c r="C38" s="19" t="inlineStr">
         <is>
-          <t>Inscripción: quién se inscribe, cuándo lo hizo, si tiene adeudo y qué incluye el costo (materiales, hospedaje, etc.).</t>
+          <t>Registro de asistencia por sesión.</t>
         </is>
       </c>
       <c r="D38" s="19" t="inlineStr">
@@ -4464,7 +4480,7 @@
     <row r="39">
       <c r="A39" s="18" t="inlineStr">
         <is>
-          <t>M2A-07</t>
+          <t>M2A-05</t>
         </is>
       </c>
       <c r="B39" s="19" t="inlineStr">
@@ -4474,12 +4490,12 @@
       </c>
       <c r="C39" s="19" t="inlineStr">
         <is>
-          <t>Registro de pagos, saldo de adeudos y recibo. Por definir: captura manual vs. pasarela de pago, y si se requiere corte de caja.</t>
-        </is>
-      </c>
-      <c r="D39" s="21" t="inlineStr">
-        <is>
-          <t>Nuevo v3</t>
+          <t>Seguimiento de tareas o actividades opcionales (no sumativas).</t>
+        </is>
+      </c>
+      <c r="D39" s="19" t="inlineStr">
+        <is>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E39" s="19" t="inlineStr">
@@ -4514,7 +4530,7 @@
       </c>
       <c r="K39" s="19" t="inlineStr">
         <is>
-          <t>Por definir</t>
+          <t>VoBo pendiente</t>
         </is>
       </c>
       <c r="L39" s="19" t="inlineStr">
@@ -4528,7 +4544,7 @@
     <row r="40">
       <c r="A40" s="18" t="inlineStr">
         <is>
-          <t>M2A-08</t>
+          <t>M2A-06</t>
         </is>
       </c>
       <c r="B40" s="19" t="inlineStr">
@@ -4538,12 +4554,12 @@
       </c>
       <c r="C40" s="19" t="inlineStr">
         <is>
-          <t>Tablero del curso tipo mensajería para avisos antes del curso y días posteriores, con notificación a los inscritos.</t>
-        </is>
-      </c>
-      <c r="D40" s="22" t="inlineStr">
-        <is>
-          <t>Recuperado v1</t>
+          <t>Inscripción: quién se inscribe, cuándo lo hizo, si tiene adeudo y qué incluye el costo (materiales, hospedaje, etc.).</t>
+        </is>
+      </c>
+      <c r="D40" s="19" t="inlineStr">
+        <is>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E40" s="19" t="inlineStr">
@@ -4592,7 +4608,7 @@
     <row r="41">
       <c r="A41" s="18" t="inlineStr">
         <is>
-          <t>M2A-09</t>
+          <t>M2A-07</t>
         </is>
       </c>
       <c r="B41" s="19" t="inlineStr">
@@ -4602,12 +4618,12 @@
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>Evaluación docente configurable: formulario diseñable (tipo Google Forms) aplicado al finalizar el curso.</t>
-        </is>
-      </c>
-      <c r="D41" s="19" t="inlineStr">
-        <is>
-          <t>v1 / v2</t>
+          <t>Registro de pagos, saldo de adeudos y recibo. Por definir: captura manual vs. pasarela de pago, y si se requiere corte de caja.</t>
+        </is>
+      </c>
+      <c r="D41" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3</t>
         </is>
       </c>
       <c r="E41" s="19" t="inlineStr">
@@ -4642,7 +4658,7 @@
       </c>
       <c r="K41" s="19" t="inlineStr">
         <is>
-          <t>VoBo pendiente</t>
+          <t>Por definir</t>
         </is>
       </c>
       <c r="L41" s="19" t="inlineStr">
@@ -4656,7 +4672,7 @@
     <row r="42">
       <c r="A42" s="18" t="inlineStr">
         <is>
-          <t>M2A-10</t>
+          <t>M2A-08</t>
         </is>
       </c>
       <c r="B42" s="19" t="inlineStr">
@@ -4666,7 +4682,7 @@
       </c>
       <c r="C42" s="19" t="inlineStr">
         <is>
-          <t>Evolución del ponente: historial de evaluaciones por ponente a lo largo del tiempo y entre ediciones.</t>
+          <t>Tablero del curso tipo mensajería para avisos antes del curso y días posteriores, con notificación a los inscritos.</t>
         </is>
       </c>
       <c r="D42" s="22" t="inlineStr">
@@ -4720,7 +4736,7 @@
     <row r="43">
       <c r="A43" s="18" t="inlineStr">
         <is>
-          <t>M2A-11</t>
+          <t>M2A-09</t>
         </is>
       </c>
       <c r="B43" s="19" t="inlineStr">
@@ -4730,7 +4746,7 @@
       </c>
       <c r="C43" s="19" t="inlineStr">
         <is>
-          <t>Reconocimiento de participación (diploma) opcional por curso.</t>
+          <t>Evaluación docente configurable: formulario diseñable (tipo Google Forms) aplicado al finalizar el curso.</t>
         </is>
       </c>
       <c r="D43" s="19" t="inlineStr">
@@ -4784,22 +4800,22 @@
     <row r="44">
       <c r="A44" s="18" t="inlineStr">
         <is>
-          <t>M2B-01</t>
+          <t>M2A-10</t>
         </is>
       </c>
       <c r="B44" s="19" t="inlineStr">
         <is>
-          <t>M2B Cursos escolarizados</t>
+          <t>M2A Cursos de Vida</t>
         </is>
       </c>
       <c r="C44" s="19" t="inlineStr">
         <is>
-          <t>Control riguroso de asistencia.</t>
-        </is>
-      </c>
-      <c r="D44" s="19" t="inlineStr">
-        <is>
-          <t>v1 / v2</t>
+          <t>Evolución del ponente: historial de evaluaciones por ponente a lo largo del tiempo y entre ediciones.</t>
+        </is>
+      </c>
+      <c r="D44" s="22" t="inlineStr">
+        <is>
+          <t>Recuperado v1</t>
         </is>
       </c>
       <c r="E44" s="19" t="inlineStr">
@@ -4848,17 +4864,17 @@
     <row r="45">
       <c r="A45" s="18" t="inlineStr">
         <is>
-          <t>M2B-02</t>
+          <t>M2A-11</t>
         </is>
       </c>
       <c r="B45" s="19" t="inlineStr">
         <is>
-          <t>M2B Cursos escolarizados</t>
+          <t>M2A Cursos de Vida</t>
         </is>
       </c>
       <c r="C45" s="19" t="inlineStr">
         <is>
-          <t>Entrega de tareas y trabajos continuos (incluidos trabajos extra).</t>
+          <t>Reconocimiento de participación (diploma) opcional por curso.</t>
         </is>
       </c>
       <c r="D45" s="19" t="inlineStr">
@@ -4912,7 +4928,7 @@
     <row r="46">
       <c r="A46" s="18" t="inlineStr">
         <is>
-          <t>M2B-03</t>
+          <t>M2B-01</t>
         </is>
       </c>
       <c r="B46" s="19" t="inlineStr">
@@ -4922,7 +4938,7 @@
       </c>
       <c r="C46" s="19" t="inlineStr">
         <is>
-          <t>Ponderación de calificaciones y exámenes finales.</t>
+          <t>Control riguroso de asistencia.</t>
         </is>
       </c>
       <c r="D46" s="19" t="inlineStr">
@@ -4976,7 +4992,7 @@
     <row r="47">
       <c r="A47" s="18" t="inlineStr">
         <is>
-          <t>M2B-04</t>
+          <t>M2B-02</t>
         </is>
       </c>
       <c r="B47" s="19" t="inlineStr">
@@ -4986,12 +5002,12 @@
       </c>
       <c r="C47" s="19" t="inlineStr">
         <is>
-          <t>Creador de exámenes en línea: opción múltiple, preguntas abiertas, falso/verdadero y respuesta corta.</t>
+          <t>Entrega de tareas y trabajos continuos (incluidos trabajos extra).</t>
         </is>
       </c>
       <c r="D47" s="19" t="inlineStr">
         <is>
-          <t>v2</t>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E47" s="19" t="inlineStr">
@@ -5040,7 +5056,7 @@
     <row r="48">
       <c r="A48" s="18" t="inlineStr">
         <is>
-          <t>M2B-05</t>
+          <t>M2B-03</t>
         </is>
       </c>
       <c r="B48" s="19" t="inlineStr">
@@ -5050,7 +5066,7 @@
       </c>
       <c r="C48" s="19" t="inlineStr">
         <is>
-          <t>Boleta digital con el formato definido por la iglesia. Por definir: formato oficial de la boleta.</t>
+          <t>Ponderación de calificaciones y exámenes finales.</t>
         </is>
       </c>
       <c r="D48" s="19" t="inlineStr">
@@ -5090,7 +5106,7 @@
       </c>
       <c r="K48" s="19" t="inlineStr">
         <is>
-          <t>Por definir</t>
+          <t>VoBo pendiente</t>
         </is>
       </c>
       <c r="L48" s="19" t="inlineStr">
@@ -5104,7 +5120,7 @@
     <row r="49">
       <c r="A49" s="18" t="inlineStr">
         <is>
-          <t>M2B-06</t>
+          <t>M2B-04</t>
         </is>
       </c>
       <c r="B49" s="19" t="inlineStr">
@@ -5114,7 +5130,7 @@
       </c>
       <c r="C49" s="19" t="inlineStr">
         <is>
-          <t>Historial académico permanente en el Expediente Digital, aunque cambie el maestro o el alumno pierda su comprobante.</t>
+          <t>Creador de exámenes en línea: opción múltiple, preguntas abiertas, falso/verdadero y respuesta corta.</t>
         </is>
       </c>
       <c r="D49" s="19" t="inlineStr">
@@ -5168,124 +5184,116 @@
     <row r="50">
       <c r="A50" s="18" t="inlineStr">
         <is>
-          <t>M3-01</t>
+          <t>M2B-05</t>
         </is>
       </c>
       <c r="B50" s="19" t="inlineStr">
         <is>
-          <t>M3 Grupos de Conexión</t>
+          <t>M2B Cursos escolarizados</t>
         </is>
       </c>
       <c r="C50" s="19" t="inlineStr">
         <is>
-          <t>Estructura del grupo con roles: Supervisor (supervisa uno o varios grupos y reporta al Pastor), Líder, Secretario, Anfitrión y Tesorero.</t>
+          <t>Boleta digital con el formato definido por la iglesia. Por definir: formato oficial de la boleta.</t>
         </is>
       </c>
       <c r="D50" s="19" t="inlineStr">
         <is>
-          <t>v3 + Obs. 4</t>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E50" s="19" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Fuera del MVP</t>
         </is>
       </c>
       <c r="F50" s="19" t="inlineStr">
         <is>
-          <t>Fase 1</t>
+          <t>Fase 3</t>
         </is>
       </c>
       <c r="G50" s="19" t="inlineStr">
         <is>
-          <t>Sprint 3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H50" s="19" t="inlineStr">
         <is>
-          <t>H3 · MVP (Grupos)</t>
-        </is>
-      </c>
-      <c r="I50" s="19" t="inlineStr">
-        <is>
-          <t>Como supervisor quiero asignar Líder, Secretario, Anfitrión y Tesorero a cada grupo.</t>
-        </is>
-      </c>
-      <c r="J50" s="19" t="inlineStr">
-        <is>
-          <t>Un grupo tiene sus roles asignados; un supervisor ve varios grupos.</t>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="I50" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
+        </is>
+      </c>
+      <c r="J50" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
         </is>
       </c>
       <c r="K50" s="19" t="inlineStr">
         <is>
-          <t>VoBo pendiente</t>
+          <t>Por definir</t>
         </is>
       </c>
       <c r="L50" s="19" t="inlineStr">
         <is>
-          <t>En pruebas</t>
-        </is>
-      </c>
-      <c r="M50" s="19" t="inlineStr">
-        <is>
-          <t>Rama feature/grupos-paso-3 · pruebas de backend y 81 de frontend pasan; lint, estilos y compilación limpios</t>
-        </is>
-      </c>
-      <c r="N50" s="19" t="inlineStr">
-        <is>
-          <t>2026-10-27 · Supervisor, Líder, Secretario, Anfitrión, Tesorero y Asistente por grupo; ahora con cambio de rol, sector (letra), casa (número) y suspensión con motivo.</t>
-        </is>
-      </c>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M50" s="19" t="inlineStr"/>
+      <c r="N50" s="19" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="18" t="inlineStr">
         <is>
-          <t>M3-02</t>
+          <t>M2B-06</t>
         </is>
       </c>
       <c r="B51" s="19" t="inlineStr">
         <is>
-          <t>M3 Grupos de Conexión</t>
+          <t>M2B Cursos escolarizados</t>
         </is>
       </c>
       <c r="C51" s="19" t="inlineStr">
         <is>
-          <t>Estudio semanal dentro de la app: un registro por semana con PDF para adultos, PDF para niños y audio de la lectura (PDF hasta 15 MB; audio hasta 40 MB). Lo publican Pastor o Anciano y los líderes lo abren desde la reunión, sustituyendo el envío por WhatsApp. El audio admite adelantar y retroceder en iPhone.</t>
+          <t>Historial académico permanente en el Expediente Digital, aunque cambie el maestro o el alumno pierda su comprobante.</t>
         </is>
       </c>
       <c r="D51" s="19" t="inlineStr">
         <is>
-          <t>v1 / v2 + Respuesta</t>
+          <t>v2</t>
         </is>
       </c>
       <c r="E51" s="19" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Fuera del MVP</t>
         </is>
       </c>
       <c r="F51" s="19" t="inlineStr">
         <is>
-          <t>Fase 1</t>
+          <t>Fase 3</t>
         </is>
       </c>
       <c r="G51" s="19" t="inlineStr">
         <is>
-          <t>Sprint 3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H51" s="19" t="inlineStr">
         <is>
-          <t>H3 · MVP (Grupos)</t>
-        </is>
-      </c>
-      <c r="I51" s="19" t="inlineStr">
-        <is>
-          <t>Como líder quiero recibir el estudio semanal en la app en lugar de WhatsApp.</t>
-        </is>
-      </c>
-      <c r="J51" s="19" t="inlineStr">
-        <is>
-          <t>Publicar el material de la semana; el líder lo abre y queda marca de lectura.</t>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="I51" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
+        </is>
+      </c>
+      <c r="J51" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
         </is>
       </c>
       <c r="K51" s="19" t="inlineStr">
@@ -5295,24 +5303,16 @@
       </c>
       <c r="L51" s="19" t="inlineStr">
         <is>
-          <t>En pruebas</t>
-        </is>
-      </c>
-      <c r="M51" s="19" t="inlineStr">
-        <is>
-          <t>Rama feature/m3-grupos · 88 pruebas de backend y 7 de frontend pasan</t>
-        </is>
-      </c>
-      <c r="N51" s="19" t="inlineStr">
-        <is>
-          <t>2026-10-24 · PDF adultos, PDF niños y audio por semana; audio con Range para iPhone. Pendiente probar en iOS.</t>
-        </is>
-      </c>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M51" s="19" t="inlineStr"/>
+      <c r="N51" s="19" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="18" t="inlineStr">
         <is>
-          <t>M3-03</t>
+          <t>M3-01</t>
         </is>
       </c>
       <c r="B52" s="19" t="inlineStr">
@@ -5322,12 +5322,12 @@
       </c>
       <c r="C52" s="19" t="inlineStr">
         <is>
-          <t>Pase de lista digital por Secretario o Líder. El Secretario captura y corrige el mismo día; el Líder modifica siempre; el Supervisor solo consulta. Funciona sin conexión: la lista se guarda en el teléfono con la hora real de captura y se envía sola al volver la señal, sin pisar cambios más recientes hechos en línea. Una captura sin conexión se acepta hasta 7 días después y se evalúa contra el día en que se hizo; todo queda en bitácora marcado como diferido.</t>
+          <t>Estructura del grupo con roles: Supervisor (supervisa uno o varios grupos y reporta al Pastor), Líder, Secretario, Anfitrión y Tesorero.</t>
         </is>
       </c>
       <c r="D52" s="19" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>v3 + Obs. 4</t>
         </is>
       </c>
       <c r="E52" s="19" t="inlineStr">
@@ -5352,12 +5352,12 @@
       </c>
       <c r="I52" s="19" t="inlineStr">
         <is>
-          <t>Como secretario quiero pasar lista aunque no haya señal.</t>
+          <t>Como supervisor quiero asignar Líder, Secretario, Anfitrión y Tesorero a cada grupo.</t>
         </is>
       </c>
       <c r="J52" s="19" t="inlineStr">
         <is>
-          <t>Pasar lista en modo avión; al reconectar se sincroniza sin duplicados.</t>
+          <t>Un grupo tiene sus roles asignados; un supervisor ve varios grupos.</t>
         </is>
       </c>
       <c r="K52" s="19" t="inlineStr">
@@ -5372,19 +5372,19 @@
       </c>
       <c r="M52" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/nf-06-sin-conexion · 117 pruebas de backend y 27 de frontend; probado en Chrome real con service worker</t>
+          <t>Rama feature/grupos-paso-3 · pruebas de backend y 81 de frontend pasan; lint, estilos y compilación limpios</t>
         </is>
       </c>
       <c r="N52" s="19" t="inlineStr">
         <is>
-          <t>2026-10-24 · Pase de lista con y sin conexión.</t>
+          <t>2026-10-27 · Supervisor, Líder, Secretario, Anfitrión, Tesorero y Asistente por grupo; ahora con cambio de rol, sector (letra), casa (número) y suspensión con motivo.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="18" t="inlineStr">
         <is>
-          <t>M3-04</t>
+          <t>M3-02</t>
         </is>
       </c>
       <c r="B53" s="19" t="inlineStr">
@@ -5394,12 +5394,12 @@
       </c>
       <c r="C53" s="19" t="inlineStr">
         <is>
-          <t>Ofrendas regulares y especiales (con concepto) por reunión, cuantificables. El Secretario captura el monto; si el grupo no tiene Secretario, lo suple el Líder. El Tesorero cuenta, escribe su cifra y avala volviendo a escribir su PIN; si el grupo no tiene Tesorero, avalan el Líder o el Pastor, nunca quien capturó. Si la cifra coincide queda «Avalada»; si no, se registra la diferencia y queda «Con diferencia», con aviso visible en el grupo, la reunión y la pantalla del Tesorero para quien pueda consultar. Una ofrenda ya capturada solo se corrige con motivo y vuelve a pendiente para un nuevo aval. El Pastor consulta todo, el Líder y el Supervisor consultan y el Anciano no ve finanzas. Toda suplencia, captura, aval y corrección queda en bitácora.</t>
+          <t>Estudio semanal dentro de la app: un registro por semana con PDF para adultos, PDF para niños y audio de la lectura (PDF hasta 15 MB; audio hasta 40 MB). Lo publican Pastor o Anciano y los líderes lo abren desde la reunión, sustituyendo el envío por WhatsApp. El audio admite adelantar y retroceder en iPhone.</t>
         </is>
       </c>
       <c r="D53" s="19" t="inlineStr">
         <is>
-          <t>v3 + Obs. 4</t>
+          <t>v1 / v2 + Respuesta</t>
         </is>
       </c>
       <c r="E53" s="19" t="inlineStr">
@@ -5414,7 +5414,7 @@
       </c>
       <c r="G53" s="19" t="inlineStr">
         <is>
-          <t>Sprint 4</t>
+          <t>Sprint 3</t>
         </is>
       </c>
       <c r="H53" s="19" t="inlineStr">
@@ -5424,12 +5424,12 @@
       </c>
       <c r="I53" s="19" t="inlineStr">
         <is>
-          <t>Como tesorero quiero contar y avalar la ofrenda del grupo.</t>
+          <t>Como líder quiero recibir el estudio semanal en la app en lugar de WhatsApp.</t>
         </is>
       </c>
       <c r="J53" s="19" t="inlineStr">
         <is>
-          <t>Capturar monto; el Tesorero captura su cifra y confirma con su PIN; si difiere se registra la diferencia; con aval no se edita sin motivo.</t>
+          <t>Publicar el material de la semana; el líder lo abre y queda marca de lectura.</t>
         </is>
       </c>
       <c r="K53" s="19" t="inlineStr">
@@ -5444,19 +5444,19 @@
       </c>
       <c r="M53" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/m3-ofrendas-ajustes · 121 pruebas de backend y 14 de frontend pasan</t>
+          <t>Rama feature/m3-grupos · 88 pruebas de backend y 7 de frontend pasan</t>
         </is>
       </c>
       <c r="N53" s="19" t="inlineStr">
         <is>
-          <t>2026-10-24 · Con suplencias del Líder, diferencias visibles y límites configurables. Falta validar con la iglesia.</t>
+          <t>2026-10-24 · PDF adultos, PDF niños y audio por semana; audio con Range para iPhone. Pendiente probar en iOS.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="18" t="inlineStr">
         <is>
-          <t>M3-05</t>
+          <t>M3-03</t>
         </is>
       </c>
       <c r="B54" s="19" t="inlineStr">
@@ -5466,7 +5466,7 @@
       </c>
       <c r="C54" s="19" t="inlineStr">
         <is>
-          <t>Peticiones de oración con formulario configurable (campos que se agregan, desactivan y reordenan sin programar; cada cambio crea una versión y los campos no se borran). Por defecto: petición, quién la pide y categoría. Las registran el Líder y el Secretario, desde la reunión o desde el grupo; el Pastor también.</t>
+          <t>Pase de lista digital por Secretario o Líder. El Secretario captura y corrige el mismo día; el Líder modifica siempre; el Supervisor solo consulta. Funciona sin conexión: la lista se guarda en el teléfono con la hora real de captura y se envía sola al volver la señal, sin pisar cambios más recientes hechos en línea. Una captura sin conexión se acepta hasta 7 días después y se evalúa contra el día en que se hizo; todo queda en bitácora marcado como diferido.</t>
         </is>
       </c>
       <c r="D54" s="19" t="inlineStr">
@@ -5486,7 +5486,7 @@
       </c>
       <c r="G54" s="19" t="inlineStr">
         <is>
-          <t>Sprint 4</t>
+          <t>Sprint 3</t>
         </is>
       </c>
       <c r="H54" s="19" t="inlineStr">
@@ -5496,12 +5496,12 @@
       </c>
       <c r="I54" s="19" t="inlineStr">
         <is>
-          <t>Como líder quiero recoger peticiones de oración con un formulario configurable.</t>
+          <t>Como secretario quiero pasar lista aunque no haya señal.</t>
         </is>
       </c>
       <c r="J54" s="19" t="inlineStr">
         <is>
-          <t>Capturar una petición; el formulario se edita sin código.</t>
+          <t>Pasar lista en modo avión; al reconectar se sincroniza sin duplicados.</t>
         </is>
       </c>
       <c r="K54" s="19" t="inlineStr">
@@ -5516,19 +5516,19 @@
       </c>
       <c r="M54" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/m3-peticiones-oracion · 166 pruebas de backend y 32 de frontend pasan; probado contra la base real</t>
+          <t>Rama feature/nf-06-sin-conexion · 117 pruebas de backend y 27 de frontend; probado en Chrome real con service worker</t>
         </is>
       </c>
       <c r="N54" s="19" t="inlineStr">
         <is>
-          <t>2026-10-24 · Formulario configurable y versionado; captura desde la reunión y el grupo.</t>
+          <t>2026-10-24 · Pase de lista con y sin conexión.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="18" t="inlineStr">
         <is>
-          <t>M3-06</t>
+          <t>M3-04</t>
         </is>
       </c>
       <c r="B55" s="19" t="inlineStr">
@@ -5538,12 +5538,12 @@
       </c>
       <c r="C55" s="19" t="inlineStr">
         <is>
-          <t>Alcance de lectura de cada petición, elegido por quien la registra con autorización de quien la pide: «Solo líderes» (Líder, Supervisor, Pastor y Anciano), «Mi grupo» (todos los integrantes del grupo y los anteriores) o «Equipo de oración» (además, quien tenga el rol Equipo de oración). El alcance por defecto es configurable. Quien registra siempre ve lo que registró; el Administrador Técnico nunca ve el contenido. Solo líderes y superiores marcan una petición como atendida. Se guardan cifradas y se borran automáticamente a los 30 días, configurable. Consultarlas y atenderlas queda en bitácora sin incluir el texto.</t>
-        </is>
-      </c>
-      <c r="D55" s="21" t="inlineStr">
-        <is>
-          <t>Resp. P8 + Respuesta</t>
+          <t>Ofrendas regulares y especiales (con concepto) por reunión, cuantificables. El Secretario captura el monto; si el grupo no tiene Secretario, lo suple el Líder. El Tesorero cuenta, escribe su cifra y avala volviendo a escribir su PIN; si el grupo no tiene Tesorero, avalan el Líder o el Pastor, nunca quien capturó. Si la cifra coincide queda «Avalada»; si no, se registra la diferencia y queda «Con diferencia», con aviso visible en el grupo, la reunión y la pantalla del Tesorero para quien pueda consultar. Una ofrenda ya capturada solo se corrige con motivo y vuelve a pendiente para un nuevo aval. El Pastor consulta todo, el Líder y el Supervisor consultan y el Anciano no ve finanzas. Toda suplencia, captura, aval y corrección queda en bitácora.</t>
+        </is>
+      </c>
+      <c r="D55" s="19" t="inlineStr">
+        <is>
+          <t>v3 + Obs. 4</t>
         </is>
       </c>
       <c r="E55" s="19" t="inlineStr">
@@ -5568,12 +5568,12 @@
       </c>
       <c r="I55" s="19" t="inlineStr">
         <is>
-          <t>Como pastor quiero que las peticiones solo las vea el Líder y superiores y se borren al vencer.</t>
+          <t>Como tesorero quiero contar y avalar la ofrenda del grupo.</t>
         </is>
       </c>
       <c r="J55" s="19" t="inlineStr">
         <is>
-          <t>El Secretario no las ve; tras el plazo configurable (por defecto 30 días) se eliminan.</t>
+          <t>Capturar monto; el Tesorero captura su cifra y confirma con su PIN; si difiere se registra la diferencia; con aval no se edita sin motivo.</t>
         </is>
       </c>
       <c r="K55" s="19" t="inlineStr">
@@ -5588,19 +5588,19 @@
       </c>
       <c r="M55" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/m3-peticiones-oracion · 166 pruebas de backend y 32 de frontend pasan; probado contra la base real</t>
+          <t>Rama feature/m3-ofrendas-ajustes · 121 pruebas de backend y 14 de frontend pasan</t>
         </is>
       </c>
       <c r="N55" s="19" t="inlineStr">
         <is>
-          <t>2026-10-24 · Alcance por petición (líderes, grupo, equipo), cifrado y borrado a los 30 días configurable. Cambia la matriz aprobada: actualizar con la iglesia.</t>
+          <t>2026-10-24 · Con suplencias del Líder, diferencias visibles y límites configurables. Falta validar con la iglesia.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="18" t="inlineStr">
         <is>
-          <t>M3-07</t>
+          <t>M3-05</t>
         </is>
       </c>
       <c r="B56" s="19" t="inlineStr">
@@ -5610,7 +5610,7 @@
       </c>
       <c r="C56" s="19" t="inlineStr">
         <is>
-          <t>Dashboard de supervisión («Resumen de grupos») para Supervisor, Líder, Pastor y Anciano sobre los grupos que cada uno puede consultar: asistencia por semana y por grupo, grupos sin lista esta semana, asistencia por debajo de un mínimo configurable (60 % por defecto), ofrendas avaladas, pendientes y con diferencia (solo si el rol ve finanzas) y peticiones activas (solo las que puede leer). No muestra datos de personas. El Secretario y el Tesorero no lo ven.</t>
+          <t>Peticiones de oración con formulario configurable (campos que se agregan, desactivan y reordenan sin programar; cada cambio crea una versión y los campos no se borran). Por defecto: petición, quién la pide y categoría. Las registran el Líder y el Secretario, desde la reunión o desde el grupo; el Pastor también.</t>
         </is>
       </c>
       <c r="D56" s="19" t="inlineStr">
@@ -5620,7 +5620,7 @@
       </c>
       <c r="E56" s="19" t="inlineStr">
         <is>
-          <t>MVP básico</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="F56" s="19" t="inlineStr">
@@ -5630,7 +5630,7 @@
       </c>
       <c r="G56" s="19" t="inlineStr">
         <is>
-          <t>Sprint 5</t>
+          <t>Sprint 4</t>
         </is>
       </c>
       <c r="H56" s="19" t="inlineStr">
@@ -5640,12 +5640,12 @@
       </c>
       <c r="I56" s="19" t="inlineStr">
         <is>
-          <t>Como supervisor quiero ver la salud de mis grupos.</t>
+          <t>Como líder quiero recoger peticiones de oración con un formulario configurable.</t>
         </is>
       </c>
       <c r="J56" s="19" t="inlineStr">
         <is>
-          <t>El dashboard muestra asistencia, ofrendas y crecimiento según permisos.</t>
+          <t>Capturar una petición; el formulario se edita sin código.</t>
         </is>
       </c>
       <c r="K56" s="19" t="inlineStr">
@@ -5660,19 +5660,19 @@
       </c>
       <c r="M56" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/m3-dashboard-tablero · 195 pruebas de backend y 39 de frontend pasan; probado contra la base real</t>
+          <t>Rama feature/m3-peticiones-oracion · 166 pruebas de backend y 32 de frontend pasan; probado contra la base real</t>
         </is>
       </c>
       <c r="N56" s="19" t="inlineStr">
         <is>
-          <t>2026-10-25 · Dashboard con asistencia, avisos y datos según rol; umbral configurable.</t>
+          <t>2026-10-24 · Formulario configurable y versionado; captura desde la reunión y el grupo.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="18" t="inlineStr">
         <is>
-          <t>M3-08</t>
+          <t>M3-06</t>
         </is>
       </c>
       <c r="B57" s="19" t="inlineStr">
@@ -5682,61 +5682,69 @@
       </c>
       <c r="C57" s="19" t="inlineStr">
         <is>
-          <t>Ubicación de zona del grupo para que personas cercanas lo encuentren, sin exponer el domicilio exacto. Por definir.</t>
-        </is>
-      </c>
-      <c r="D57" s="19" t="inlineStr">
-        <is>
-          <t>v3</t>
+          <t>Alcance de lectura de cada petición, elegido por quien la registra con autorización de quien la pide: «Solo líderes» (Líder, Supervisor, Pastor y Anciano), «Mi grupo» (todos los integrantes del grupo y los anteriores) o «Equipo de oración» (además, quien tenga el rol Equipo de oración). El alcance por defecto es configurable. Quien registra siempre ve lo que registró; el Administrador Técnico nunca ve el contenido. Solo líderes y superiores marcan una petición como atendida. Se guardan cifradas y se borran automáticamente a los 30 días, configurable. Consultarlas y atenderlas queda en bitácora sin incluir el texto.</t>
+        </is>
+      </c>
+      <c r="D57" s="21" t="inlineStr">
+        <is>
+          <t>Resp. P8 + Respuesta</t>
         </is>
       </c>
       <c r="E57" s="19" t="inlineStr">
         <is>
-          <t>Fuera del MVP</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="F57" s="19" t="inlineStr">
         <is>
-          <t>Fase 4</t>
+          <t>Fase 1</t>
         </is>
       </c>
       <c r="G57" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sprint 4</t>
         </is>
       </c>
       <c r="H57" s="19" t="inlineStr">
         <is>
-          <t>Posterior</t>
-        </is>
-      </c>
-      <c r="I57" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
-        </is>
-      </c>
-      <c r="J57" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
+          <t>H3 · MVP (Grupos)</t>
+        </is>
+      </c>
+      <c r="I57" s="19" t="inlineStr">
+        <is>
+          <t>Como pastor quiero que las peticiones solo las vea el Líder y superiores y se borren al vencer.</t>
+        </is>
+      </c>
+      <c r="J57" s="19" t="inlineStr">
+        <is>
+          <t>El Secretario no las ve; tras el plazo configurable (por defecto 30 días) se eliminan.</t>
         </is>
       </c>
       <c r="K57" s="19" t="inlineStr">
         <is>
-          <t>Por definir</t>
+          <t>VoBo pendiente</t>
         </is>
       </c>
       <c r="L57" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M57" s="19" t="inlineStr"/>
-      <c r="N57" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M57" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/m3-peticiones-oracion · 166 pruebas de backend y 32 de frontend pasan; probado contra la base real</t>
+        </is>
+      </c>
+      <c r="N57" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-24 · Alcance por petición (líderes, grupo, equipo), cifrado y borrado a los 30 días configurable. Cambia la matriz aprobada: actualizar con la iglesia.</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="18" t="inlineStr">
         <is>
-          <t>M3-09</t>
+          <t>M3-07</t>
         </is>
       </c>
       <c r="B58" s="19" t="inlineStr">
@@ -5746,17 +5754,17 @@
       </c>
       <c r="C58" s="19" t="inlineStr">
         <is>
-          <t>A un grupo asisten miembros de la iglesia (vecinos o no) e invitados del grupo que no asisten a la iglesia. Los invitados se registran como Contacto con datos mínimos y se les puede invitar a consolidación.</t>
-        </is>
-      </c>
-      <c r="D58" s="21" t="inlineStr">
-        <is>
-          <t>Corrección v3.2</t>
+          <t>Dashboard de supervisión («Resumen de grupos») para Supervisor, Líder, Pastor y Anciano sobre los grupos que cada uno puede consultar: asistencia por semana y por grupo, grupos sin lista esta semana, asistencia por debajo de un mínimo configurable (60 % por defecto), ofrendas avaladas, pendientes y con diferencia (solo si el rol ve finanzas) y peticiones activas (solo las que puede leer). No muestra datos de personas. El Secretario y el Tesorero no lo ven.</t>
+        </is>
+      </c>
+      <c r="D58" s="19" t="inlineStr">
+        <is>
+          <t>v3</t>
         </is>
       </c>
       <c r="E58" s="19" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>MVP básico</t>
         </is>
       </c>
       <c r="F58" s="19" t="inlineStr">
@@ -5766,7 +5774,7 @@
       </c>
       <c r="G58" s="19" t="inlineStr">
         <is>
-          <t>Sprint 3</t>
+          <t>Sprint 5</t>
         </is>
       </c>
       <c r="H58" s="19" t="inlineStr">
@@ -5776,12 +5784,12 @@
       </c>
       <c r="I58" s="19" t="inlineStr">
         <is>
-          <t>Como secretario quiero registrar invitados del grupo con datos mínimos.</t>
+          <t>Como supervisor quiero ver la salud de mis grupos.</t>
         </is>
       </c>
       <c r="J58" s="19" t="inlineStr">
         <is>
-          <t>Registrar un invitado como Contacto y marcarlo presente.</t>
+          <t>El dashboard muestra asistencia, ofrendas y crecimiento según permisos.</t>
         </is>
       </c>
       <c r="K58" s="19" t="inlineStr">
@@ -5796,19 +5804,19 @@
       </c>
       <c r="M58" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/paso-5-invitaciones · pruebas de backend y 93 de frontend pasan; lint, estilos y compilación limpios</t>
+          <t>Rama feature/m3-dashboard-tablero · 195 pruebas de backend y 39 de frontend pasan; probado contra la base real</t>
         </is>
       </c>
       <c r="N58" s="19" t="inlineStr">
         <is>
-          <t>2026-10-27 · Los invitados entran al grupo como Contacto cuando el líder aprueba su solicitud por enlace o QR.</t>
+          <t>2026-10-25 · Dashboard con asistencia, avisos y datos según rol; umbral configurable.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="18" t="inlineStr">
         <is>
-          <t>M3-10</t>
+          <t>M3-08</t>
         </is>
       </c>
       <c r="B59" s="19" t="inlineStr">
@@ -5818,42 +5826,42 @@
       </c>
       <c r="C59" s="19" t="inlineStr">
         <is>
-          <t>Confidencialidad de ofrendas y asistencias: consulta limitada por rol (matriz por definir) y modificación restringida, todo en bitácora.</t>
-        </is>
-      </c>
-      <c r="D59" s="21" t="inlineStr">
-        <is>
-          <t>Obs. 5</t>
+          <t>Ubicación de zona del grupo para que personas cercanas lo encuentren, sin exponer el domicilio exacto. Por definir.</t>
+        </is>
+      </c>
+      <c r="D59" s="19" t="inlineStr">
+        <is>
+          <t>v3</t>
         </is>
       </c>
       <c r="E59" s="19" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Fuera del MVP</t>
         </is>
       </c>
       <c r="F59" s="19" t="inlineStr">
         <is>
-          <t>Fase 1</t>
+          <t>Fase 4</t>
         </is>
       </c>
       <c r="G59" s="19" t="inlineStr">
         <is>
-          <t>Sprint 4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H59" s="19" t="inlineStr">
         <is>
-          <t>H3 · MVP (Grupos)</t>
-        </is>
-      </c>
-      <c r="I59" s="19" t="inlineStr">
-        <is>
-          <t>Como pastor quiero que ofrendas y asistencias sean confidenciales.</t>
-        </is>
-      </c>
-      <c r="J59" s="19" t="inlineStr">
-        <is>
-          <t>La matriz de la sección 3.3 del v3.2 se cumple en pruebas por cada rol.</t>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="I59" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
+        </is>
+      </c>
+      <c r="J59" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
         </is>
       </c>
       <c r="K59" s="19" t="inlineStr">
@@ -5872,7 +5880,7 @@
     <row r="60">
       <c r="A60" s="18" t="inlineStr">
         <is>
-          <t>M3-11</t>
+          <t>M3-09</t>
         </is>
       </c>
       <c r="B60" s="19" t="inlineStr">
@@ -5882,12 +5890,12 @@
       </c>
       <c r="C60" s="19" t="inlineStr">
         <is>
-          <t>Tablero de mensajes del grupo: lo publican Líder, Supervisor, Secretario y Pastor; lo leen todos los integrantes activos. Mensajes de hasta 1,000 caracteres, con opción de fijarlos, borrado lógico, contador de mensajes nuevos y conservación configurable (90 días). Pantalla «Avisos» para quien no abre la página del grupo.</t>
+          <t>A un grupo asisten miembros de la iglesia (vecinos o no) e invitados del grupo que no asisten a la iglesia. Los invitados se registran como Contacto con datos mínimos y se les puede invitar a consolidación.</t>
         </is>
       </c>
       <c r="D60" s="21" t="inlineStr">
         <is>
-          <t>Obs. 7</t>
+          <t>Corrección v3.2</t>
         </is>
       </c>
       <c r="E60" s="19" t="inlineStr">
@@ -5902,7 +5910,7 @@
       </c>
       <c r="G60" s="19" t="inlineStr">
         <is>
-          <t>Sprint 5</t>
+          <t>Sprint 3</t>
         </is>
       </c>
       <c r="H60" s="19" t="inlineStr">
@@ -5912,12 +5920,12 @@
       </c>
       <c r="I60" s="19" t="inlineStr">
         <is>
-          <t>Como líder quiero un tablero de mensajes de mi grupo.</t>
+          <t>Como secretario quiero registrar invitados del grupo con datos mínimos.</t>
         </is>
       </c>
       <c r="J60" s="19" t="inlineStr">
         <is>
-          <t>Publicar y leer mensajes del grupo.</t>
+          <t>Registrar un invitado como Contacto y marcarlo presente.</t>
         </is>
       </c>
       <c r="K60" s="19" t="inlineStr">
@@ -5932,19 +5940,19 @@
       </c>
       <c r="M60" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/m3-dashboard-tablero · 195 pruebas de backend y 39 de frontend pasan; probado contra la base real</t>
+          <t>Rama feature/paso-5-invitaciones · pruebas de backend y 93 de frontend pasan; lint, estilos y compilación limpios</t>
         </is>
       </c>
       <c r="N60" s="19" t="inlineStr">
         <is>
-          <t>2026-10-25 · Tablero con fijados, no leídos y retención configurable; la notificación push de mensajes nuevos se entrega con M1-09.</t>
+          <t>2026-10-27 · Los invitados entran al grupo como Contacto cuando el líder aprueba su solicitud por enlace o QR.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="18" t="inlineStr">
         <is>
-          <t>M3-12</t>
+          <t>M3-10</t>
         </is>
       </c>
       <c r="B61" s="19" t="inlineStr">
@@ -5954,12 +5962,12 @@
       </c>
       <c r="C61" s="19" t="inlineStr">
         <is>
-          <t>Reuniones: cada grupo se reúne una vez por semana en casa del líder (día y hora por grupo) y existe una reunión general de líderes, modelada como un grupo de tipo «Líderes».</t>
+          <t>Confidencialidad de ofrendas y asistencias: consulta limitada por rol (matriz por definir) y modificación restringida, todo en bitácora.</t>
         </is>
       </c>
       <c r="D61" s="21" t="inlineStr">
         <is>
-          <t>Respuesta</t>
+          <t>Obs. 5</t>
         </is>
       </c>
       <c r="E61" s="19" t="inlineStr">
@@ -5974,7 +5982,7 @@
       </c>
       <c r="G61" s="19" t="inlineStr">
         <is>
-          <t>Sprint 3</t>
+          <t>Sprint 4</t>
         </is>
       </c>
       <c r="H61" s="19" t="inlineStr">
@@ -5982,41 +5990,33 @@
           <t>H3 · MVP (Grupos)</t>
         </is>
       </c>
-      <c r="I61" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
-        </is>
-      </c>
-      <c r="J61" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
+      <c r="I61" s="19" t="inlineStr">
+        <is>
+          <t>Como pastor quiero que ofrendas y asistencias sean confidenciales.</t>
+        </is>
+      </c>
+      <c r="J61" s="19" t="inlineStr">
+        <is>
+          <t>La matriz de la sección 3.3 del v3.2 se cumple en pruebas por cada rol.</t>
         </is>
       </c>
       <c r="K61" s="19" t="inlineStr">
         <is>
-          <t>VoBo pendiente</t>
+          <t>Por definir</t>
         </is>
       </c>
       <c r="L61" s="19" t="inlineStr">
         <is>
-          <t>En pruebas</t>
-        </is>
-      </c>
-      <c r="M61" s="19" t="inlineStr">
-        <is>
-          <t>Rama feature/grupos-paso-3 · pruebas de backend y 81 de frontend pasan; lint, estilos y compilación limpios</t>
-        </is>
-      </c>
-      <c r="N61" s="19" t="inlineStr">
-        <is>
-          <t>2026-10-27 · Una reunión semanal por grupo y grupo tipo Líderes; filtros por día, sector, líder y estado; cada reunión muestra su asistencia, observaciones, peticiones y ofrendas.</t>
-        </is>
-      </c>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M61" s="19" t="inlineStr"/>
+      <c r="N61" s="19" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="18" t="inlineStr">
         <is>
-          <t>M3-13</t>
+          <t>M3-11</t>
         </is>
       </c>
       <c r="B62" s="19" t="inlineStr">
@@ -6026,12 +6026,12 @@
       </c>
       <c r="C62" s="19" t="inlineStr">
         <is>
-          <t>Parámetros configurables sin programar, con pantalla de Configuración y cada cambio en bitácora: monto máximo por ofrenda (1,000,000 por defecto) y si se permite una sola ofrenda regular por reunión. Solo Pastor y Administrador Técnico.</t>
+          <t>Tablero de mensajes del grupo: lo publican Líder, Supervisor, Secretario y Pastor; lo leen todos los integrantes activos. Mensajes de hasta 1,000 caracteres, con opción de fijarlos, borrado lógico, contador de mensajes nuevos y conservación configurable (90 días). Pantalla «Avisos» para quien no abre la página del grupo.</t>
         </is>
       </c>
       <c r="D62" s="21" t="inlineStr">
         <is>
-          <t>Respuesta</t>
+          <t>Obs. 7</t>
         </is>
       </c>
       <c r="E62" s="19" t="inlineStr">
@@ -6046,7 +6046,7 @@
       </c>
       <c r="G62" s="19" t="inlineStr">
         <is>
-          <t>Sprint 4</t>
+          <t>Sprint 5</t>
         </is>
       </c>
       <c r="H62" s="19" t="inlineStr">
@@ -6054,14 +6054,14 @@
           <t>H3 · MVP (Grupos)</t>
         </is>
       </c>
-      <c r="I62" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
-        </is>
-      </c>
-      <c r="J62" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
+      <c r="I62" s="19" t="inlineStr">
+        <is>
+          <t>Como líder quiero un tablero de mensajes de mi grupo.</t>
+        </is>
+      </c>
+      <c r="J62" s="19" t="inlineStr">
+        <is>
+          <t>Publicar y leer mensajes del grupo.</t>
         </is>
       </c>
       <c r="K62" s="19" t="inlineStr">
@@ -6076,19 +6076,19 @@
       </c>
       <c r="M62" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/m3-ofrendas-ajustes · 121 pruebas de backend y 14 de frontend pasan</t>
+          <t>Rama feature/m3-dashboard-tablero · 195 pruebas de backend y 39 de frontend pasan; probado contra la base real</t>
         </is>
       </c>
       <c r="N62" s="19" t="inlineStr">
         <is>
-          <t>2026-10-24 · Pantalla Configuración: monto máximo y una regular por reunión.</t>
+          <t>2026-10-25 · Tablero con fijados, no leídos y retención configurable; la notificación push de mensajes nuevos se entrega con M1-09.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="18" t="inlineStr">
         <is>
-          <t>M3-14</t>
+          <t>M3-12</t>
         </is>
       </c>
       <c r="B63" s="19" t="inlineStr">
@@ -6098,7 +6098,7 @@
       </c>
       <c r="C63" s="19" t="inlineStr">
         <is>
-          <t>Componente de peticiones reutilizable: cualquier módulo (grupos hoy; cursos o eventos después) se registra como origen y decide quién registra y qué nivel de acceso tiene cada persona. Toda petición guarda su origen de forma inmutable (tipo, identificador y una etiqueta fija, por ejemplo «Grupo de Conexión · Norte · reunión del 22/10/2026») y lo muestra siempre en el listado.</t>
+          <t>Reuniones: cada grupo se reúne una vez por semana en casa del líder (día y hora por grupo) y existe una reunión general de líderes, modelada como un grupo de tipo «Líderes».</t>
         </is>
       </c>
       <c r="D63" s="21" t="inlineStr">
@@ -6118,7 +6118,7 @@
       </c>
       <c r="G63" s="19" t="inlineStr">
         <is>
-          <t>Sprint 4</t>
+          <t>Sprint 3</t>
         </is>
       </c>
       <c r="H63" s="19" t="inlineStr">
@@ -6148,19 +6148,19 @@
       </c>
       <c r="M63" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/m3-peticiones-oracion · 166 pruebas de backend y 32 de frontend pasan; probado contra la base real</t>
+          <t>Rama feature/grupos-paso-3 · pruebas de backend y 81 de frontend pasan; lint, estilos y compilación limpios</t>
         </is>
       </c>
       <c r="N63" s="19" t="inlineStr">
         <is>
-          <t>2026-10-24 · Origen inmutable y visible; probado con un segundo origen de prueba para verificar la reutilización.</t>
+          <t>2026-10-27 · Una reunión semanal por grupo y grupo tipo Líderes; filtros por día, sector, líder y estado; cada reunión muestra su asistencia, observaciones, peticiones y ofrendas.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="18" t="inlineStr">
         <is>
-          <t>M3-15</t>
+          <t>M3-13</t>
         </is>
       </c>
       <c r="B64" s="19" t="inlineStr">
@@ -6170,7 +6170,7 @@
       </c>
       <c r="C64" s="19" t="inlineStr">
         <is>
-          <t>Equipo de oración: rol configurable (Equipo de oración) que se asigna a las personas que se reúnen a orar por las peticiones compartidas con ese alcance; no da acceso a nada más. Opción de ocultar el nombre de quien pide: los campos del formulario marcados «identifica a la persona» solo los ven líderes y quien registró. Al capturar se muestra una leyenda que pide confirmar la autorización de quien pide, indica quién la leerá y cuándo se borra.</t>
+          <t>Parámetros configurables sin programar, con pantalla de Configuración y cada cambio en bitácora: monto máximo por ofrenda (1,000,000 por defecto) y si se permite una sola ofrenda regular por reunión. Solo Pastor y Administrador Técnico.</t>
         </is>
       </c>
       <c r="D64" s="21" t="inlineStr">
@@ -6220,54 +6220,54 @@
       </c>
       <c r="M64" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/m3-peticiones-oracion · 166 pruebas de backend y 32 de frontend pasan; probado contra la base real</t>
+          <t>Rama feature/m3-ofrendas-ajustes · 121 pruebas de backend y 14 de frontend pasan</t>
         </is>
       </c>
       <c r="N64" s="19" t="inlineStr">
         <is>
-          <t>2026-10-24 · Rol Equipo de oración, nombre oculto y leyenda de privacidad al capturar. Falta el aviso de privacidad oficial de la iglesia.</t>
+          <t>2026-10-24 · Pantalla Configuración: monto máximo y una regular por reunión.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="18" t="inlineStr">
         <is>
-          <t>M4-01</t>
+          <t>M3-14</t>
         </is>
       </c>
       <c r="B65" s="19" t="inlineStr">
         <is>
-          <t>M4 Kids Check-In/Out</t>
+          <t>M3 Grupos de Conexión</t>
         </is>
       </c>
       <c r="C65" s="19" t="inlineStr">
         <is>
-          <t>Sustitución de la ficha física de papel.</t>
-        </is>
-      </c>
-      <c r="D65" s="19" t="inlineStr">
-        <is>
-          <t>v1 / v2</t>
+          <t>Componente de peticiones reutilizable: cualquier módulo (grupos hoy; cursos o eventos después) se registra como origen y decide quién registra y qué nivel de acceso tiene cada persona. Toda petición guarda su origen de forma inmutable (tipo, identificador y una etiqueta fija, por ejemplo «Grupo de Conexión · Norte · reunión del 22/10/2026») y lo muestra siempre en el listado.</t>
+        </is>
+      </c>
+      <c r="D65" s="21" t="inlineStr">
+        <is>
+          <t>Respuesta</t>
         </is>
       </c>
       <c r="E65" s="19" t="inlineStr">
         <is>
-          <t>Fuera del MVP</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="F65" s="19" t="inlineStr">
         <is>
-          <t>Fase 2</t>
+          <t>Fase 1</t>
         </is>
       </c>
       <c r="G65" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sprint 4</t>
         </is>
       </c>
       <c r="H65" s="19" t="inlineStr">
         <is>
-          <t>Posterior</t>
+          <t>H3 · MVP (Grupos)</t>
         </is>
       </c>
       <c r="I65" s="20" t="inlineStr">
@@ -6287,51 +6287,59 @@
       </c>
       <c r="L65" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M65" s="19" t="inlineStr"/>
-      <c r="N65" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M65" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/m3-peticiones-oracion · 166 pruebas de backend y 32 de frontend pasan; probado contra la base real</t>
+        </is>
+      </c>
+      <c r="N65" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-24 · Origen inmutable y visible; probado con un segundo origen de prueba para verificar la reutilización.</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="18" t="inlineStr">
         <is>
-          <t>M4-02</t>
+          <t>M3-15</t>
         </is>
       </c>
       <c r="B66" s="19" t="inlineStr">
         <is>
-          <t>M4 Kids Check-In/Out</t>
+          <t>M3 Grupos de Conexión</t>
         </is>
       </c>
       <c r="C66" s="19" t="inlineStr">
         <is>
-          <t>Registro de ingreso del menor con salón o clase asignada y generación de código único.</t>
+          <t>Equipo de oración: rol configurable (Equipo de oración) que se asigna a las personas que se reúnen a orar por las peticiones compartidas con ese alcance; no da acceso a nada más. Opción de ocultar el nombre de quien pide: los campos del formulario marcados «identifica a la persona» solo los ven líderes y quien registró. Al capturar se muestra una leyenda que pide confirmar la autorización de quien pide, indica quién la leerá y cuándo se borra.</t>
         </is>
       </c>
       <c r="D66" s="21" t="inlineStr">
         <is>
-          <t>v1 + Nuevo v3</t>
+          <t>Respuesta</t>
         </is>
       </c>
       <c r="E66" s="19" t="inlineStr">
         <is>
-          <t>Fuera del MVP</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="F66" s="19" t="inlineStr">
         <is>
-          <t>Fase 2</t>
+          <t>Fase 1</t>
         </is>
       </c>
       <c r="G66" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sprint 4</t>
         </is>
       </c>
       <c r="H66" s="19" t="inlineStr">
         <is>
-          <t>Posterior</t>
+          <t>H3 · MVP (Grupos)</t>
         </is>
       </c>
       <c r="I66" s="20" t="inlineStr">
@@ -6351,16 +6359,24 @@
       </c>
       <c r="L66" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M66" s="19" t="inlineStr"/>
-      <c r="N66" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M66" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/m3-peticiones-oracion · 166 pruebas de backend y 32 de frontend pasan; probado contra la base real</t>
+        </is>
+      </c>
+      <c r="N66" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-24 · Rol Equipo de oración, nombre oculto y leyenda de privacidad al capturar. Falta el aviso de privacidad oficial de la iglesia.</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="18" t="inlineStr">
         <is>
-          <t>M4-03</t>
+          <t>M4-01</t>
         </is>
       </c>
       <c r="B67" s="19" t="inlineStr">
@@ -6370,12 +6386,12 @@
       </c>
       <c r="C67" s="19" t="inlineStr">
         <is>
-          <t>Código QR dinámico o OTP temporal en la PWA del padre o tutor.</t>
+          <t>Sustitución de la ficha física de papel.</t>
         </is>
       </c>
       <c r="D67" s="19" t="inlineStr">
         <is>
-          <t>v2</t>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E67" s="19" t="inlineStr">
@@ -6424,7 +6440,7 @@
     <row r="68">
       <c r="A68" s="18" t="inlineStr">
         <is>
-          <t>M4-04</t>
+          <t>M4-02</t>
         </is>
       </c>
       <c r="B68" s="19" t="inlineStr">
@@ -6434,12 +6450,12 @@
       </c>
       <c r="C68" s="19" t="inlineStr">
         <is>
-          <t>Validación al entregar: el servidor de Kids escanea el código y confirma identidad y fotografía del tutor autorizado en el Expediente Digital.</t>
-        </is>
-      </c>
-      <c r="D68" s="19" t="inlineStr">
-        <is>
-          <t>v2</t>
+          <t>Registro de ingreso del menor con salón o clase asignada y generación de código único.</t>
+        </is>
+      </c>
+      <c r="D68" s="21" t="inlineStr">
+        <is>
+          <t>v1 + Nuevo v3</t>
         </is>
       </c>
       <c r="E68" s="19" t="inlineStr">
@@ -6488,7 +6504,7 @@
     <row r="69">
       <c r="A69" s="18" t="inlineStr">
         <is>
-          <t>M4-05</t>
+          <t>M4-03</t>
         </is>
       </c>
       <c r="B69" s="19" t="inlineStr">
@@ -6498,12 +6514,12 @@
       </c>
       <c r="C69" s="19" t="inlineStr">
         <is>
-          <t>Alternativa para tutores sin smartphone, sin batería o sin conexión (p. ej. código por SMS o comprobante imprimible con identificación). Por definir.</t>
-        </is>
-      </c>
-      <c r="D69" s="21" t="inlineStr">
-        <is>
-          <t>Nuevo v3</t>
+          <t>Código QR dinámico o OTP temporal en la PWA del padre o tutor.</t>
+        </is>
+      </c>
+      <c r="D69" s="19" t="inlineStr">
+        <is>
+          <t>v2</t>
         </is>
       </c>
       <c r="E69" s="19" t="inlineStr">
@@ -6538,7 +6554,7 @@
       </c>
       <c r="K69" s="19" t="inlineStr">
         <is>
-          <t>Por definir</t>
+          <t>VoBo pendiente</t>
         </is>
       </c>
       <c r="L69" s="19" t="inlineStr">
@@ -6552,7 +6568,7 @@
     <row r="70">
       <c r="A70" s="18" t="inlineStr">
         <is>
-          <t>M4-06</t>
+          <t>M4-04</t>
         </is>
       </c>
       <c r="B70" s="19" t="inlineStr">
@@ -6562,12 +6578,12 @@
       </c>
       <c r="C70" s="19" t="inlineStr">
         <is>
-          <t>Autorización temporal de un tercero para recoger al menor, con aprobación del tutor registrado.</t>
-        </is>
-      </c>
-      <c r="D70" s="21" t="inlineStr">
-        <is>
-          <t>Nuevo v3</t>
+          <t>Validación al entregar: el servidor de Kids escanea el código y confirma identidad y fotografía del tutor autorizado en el Expediente Digital.</t>
+        </is>
+      </c>
+      <c r="D70" s="19" t="inlineStr">
+        <is>
+          <t>v2</t>
         </is>
       </c>
       <c r="E70" s="19" t="inlineStr">
@@ -6616,7 +6632,7 @@
     <row r="71">
       <c r="A71" s="18" t="inlineStr">
         <is>
-          <t>M4-07</t>
+          <t>M4-05</t>
         </is>
       </c>
       <c r="B71" s="19" t="inlineStr">
@@ -6626,7 +6642,7 @@
       </c>
       <c r="C71" s="19" t="inlineStr">
         <is>
-          <t>Caducidad del código y bitácora de cada entrega (quién recogió, quién entregó, hora).</t>
+          <t>Alternativa para tutores sin smartphone, sin batería o sin conexión (p. ej. código por SMS o comprobante imprimible con identificación). Por definir.</t>
         </is>
       </c>
       <c r="D71" s="21" t="inlineStr">
@@ -6666,7 +6682,7 @@
       </c>
       <c r="K71" s="19" t="inlineStr">
         <is>
-          <t>VoBo pendiente</t>
+          <t>Por definir</t>
         </is>
       </c>
       <c r="L71" s="19" t="inlineStr">
@@ -6680,7 +6696,7 @@
     <row r="72">
       <c r="A72" s="18" t="inlineStr">
         <is>
-          <t>M4-08</t>
+          <t>M4-06</t>
         </is>
       </c>
       <c r="B72" s="19" t="inlineStr">
@@ -6690,7 +6706,7 @@
       </c>
       <c r="C72" s="19" t="inlineStr">
         <is>
-          <t>Funcionamiento sin conexión o con conexión degradada para el check-out.</t>
+          <t>Autorización temporal de un tercero para recoger al menor, con aprobación del tutor registrado.</t>
         </is>
       </c>
       <c r="D72" s="21" t="inlineStr">
@@ -6744,52 +6760,52 @@
     <row r="73">
       <c r="A73" s="18" t="inlineStr">
         <is>
-          <t>M5-01</t>
+          <t>M4-07</t>
         </is>
       </c>
       <c r="B73" s="19" t="inlineStr">
         <is>
-          <t>M5 Áreas y servidores</t>
+          <t>M4 Kids Check-In/Out</t>
         </is>
       </c>
       <c r="C73" s="19" t="inlineStr">
         <is>
-          <t>Catálogo mínimo de áreas y asignación de servidores. Versión reducida del módulo 5, necesaria para permisos por área. Sirve como primer censo.</t>
-        </is>
-      </c>
-      <c r="D73" s="19" t="inlineStr">
-        <is>
-          <t>v3</t>
+          <t>Caducidad del código y bitácora de cada entrega (quién recogió, quién entregó, hora).</t>
+        </is>
+      </c>
+      <c r="D73" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3</t>
         </is>
       </c>
       <c r="E73" s="19" t="inlineStr">
         <is>
-          <t>MVP mínimo</t>
+          <t>Fuera del MVP</t>
         </is>
       </c>
       <c r="F73" s="19" t="inlineStr">
         <is>
-          <t>Fase 0</t>
+          <t>Fase 2</t>
         </is>
       </c>
       <c r="G73" s="19" t="inlineStr">
         <is>
-          <t>Sprint 1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H73" s="19" t="inlineStr">
         <is>
-          <t>H2 · Fase 0 completa</t>
-        </is>
-      </c>
-      <c r="I73" s="19" t="inlineStr">
-        <is>
-          <t>Como pastor quiero un catálogo de áreas con su personal para conocer la estructura.</t>
-        </is>
-      </c>
-      <c r="J73" s="19" t="inlineStr">
-        <is>
-          <t>Crear un área, asignar servidores y ver el conteo real.</t>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="I73" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
+        </is>
+      </c>
+      <c r="J73" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
         </is>
       </c>
       <c r="K73" s="19" t="inlineStr">
@@ -6808,22 +6824,22 @@
     <row r="74">
       <c r="A74" s="18" t="inlineStr">
         <is>
-          <t>M5-02</t>
+          <t>M4-08</t>
         </is>
       </c>
       <c r="B74" s="19" t="inlineStr">
         <is>
-          <t>M5 Áreas y servidores</t>
+          <t>M4 Kids Check-In/Out</t>
         </is>
       </c>
       <c r="C74" s="19" t="inlineStr">
         <is>
-          <t>Roles jerárquicos dentro de cada área (directores, líderes, maestros, servidores).</t>
-        </is>
-      </c>
-      <c r="D74" s="19" t="inlineStr">
-        <is>
-          <t>v1</t>
+          <t>Funcionamiento sin conexión o con conexión degradada para el check-out.</t>
+        </is>
+      </c>
+      <c r="D74" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3</t>
         </is>
       </c>
       <c r="E74" s="19" t="inlineStr">
@@ -6833,7 +6849,7 @@
       </c>
       <c r="F74" s="19" t="inlineStr">
         <is>
-          <t>Fase 4</t>
+          <t>Fase 2</t>
         </is>
       </c>
       <c r="G74" s="19" t="inlineStr">
@@ -6872,7 +6888,7 @@
     <row r="75">
       <c r="A75" s="18" t="inlineStr">
         <is>
-          <t>M5-03</t>
+          <t>M5-01</t>
         </is>
       </c>
       <c r="B75" s="19" t="inlineStr">
@@ -6882,42 +6898,42 @@
       </c>
       <c r="C75" s="19" t="inlineStr">
         <is>
-          <t>Organigrama y número real de servidores activos, directores y líderes por área.</t>
+          <t>Catálogo mínimo de áreas y asignación de servidores. Versión reducida del módulo 5, necesaria para permisos por área. Sirve como primer censo.</t>
         </is>
       </c>
       <c r="D75" s="19" t="inlineStr">
         <is>
-          <t>v2</t>
+          <t>v3</t>
         </is>
       </c>
       <c r="E75" s="19" t="inlineStr">
         <is>
-          <t>Fuera del MVP</t>
+          <t>MVP mínimo</t>
         </is>
       </c>
       <c r="F75" s="19" t="inlineStr">
         <is>
-          <t>Fase 4</t>
+          <t>Fase 0</t>
         </is>
       </c>
       <c r="G75" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sprint 1</t>
         </is>
       </c>
       <c r="H75" s="19" t="inlineStr">
         <is>
-          <t>Posterior</t>
-        </is>
-      </c>
-      <c r="I75" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
-        </is>
-      </c>
-      <c r="J75" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
+          <t>H2 · Fase 0 completa</t>
+        </is>
+      </c>
+      <c r="I75" s="19" t="inlineStr">
+        <is>
+          <t>Como pastor quiero un catálogo de áreas con su personal para conocer la estructura.</t>
+        </is>
+      </c>
+      <c r="J75" s="19" t="inlineStr">
+        <is>
+          <t>Crear un área, asignar servidores y ver el conteo real.</t>
         </is>
       </c>
       <c r="K75" s="19" t="inlineStr">
@@ -6936,7 +6952,7 @@
     <row r="76">
       <c r="A76" s="18" t="inlineStr">
         <is>
-          <t>M5-04</t>
+          <t>M5-02</t>
         </is>
       </c>
       <c r="B76" s="19" t="inlineStr">
@@ -6946,12 +6962,12 @@
       </c>
       <c r="C76" s="19" t="inlineStr">
         <is>
-          <t>Control de asistencia a turnos o servicios.</t>
+          <t>Roles jerárquicos dentro de cada área (directores, líderes, maestros, servidores).</t>
         </is>
       </c>
       <c r="D76" s="19" t="inlineStr">
         <is>
-          <t>v1 / v2</t>
+          <t>v1</t>
         </is>
       </c>
       <c r="E76" s="19" t="inlineStr">
@@ -7000,7 +7016,7 @@
     <row r="77">
       <c r="A77" s="18" t="inlineStr">
         <is>
-          <t>M5-05</t>
+          <t>M5-03</t>
         </is>
       </c>
       <c r="B77" s="19" t="inlineStr">
@@ -7010,12 +7026,12 @@
       </c>
       <c r="C77" s="19" t="inlineStr">
         <is>
-          <t>Tablero de avisos y notificaciones interno por área.</t>
+          <t>Organigrama y número real de servidores activos, directores y líderes por área.</t>
         </is>
       </c>
       <c r="D77" s="19" t="inlineStr">
         <is>
-          <t>v1 / v2</t>
+          <t>v2</t>
         </is>
       </c>
       <c r="E77" s="19" t="inlineStr">
@@ -7064,7 +7080,7 @@
     <row r="78">
       <c r="A78" s="18" t="inlineStr">
         <is>
-          <t>M5-06</t>
+          <t>M5-04</t>
         </is>
       </c>
       <c r="B78" s="19" t="inlineStr">
@@ -7074,7 +7090,7 @@
       </c>
       <c r="C78" s="19" t="inlineStr">
         <is>
-          <t>Gestión financiera por área: caja chica y gastos operativos.</t>
+          <t>Control de asistencia a turnos o servicios.</t>
         </is>
       </c>
       <c r="D78" s="19" t="inlineStr">
@@ -7128,22 +7144,22 @@
     <row r="79">
       <c r="A79" s="18" t="inlineStr">
         <is>
-          <t>M6-01</t>
+          <t>M5-05</t>
         </is>
       </c>
       <c r="B79" s="19" t="inlineStr">
         <is>
-          <t>M6 Ministerios de servicio</t>
+          <t>M5 Áreas y servidores</t>
         </is>
       </c>
       <c r="C79" s="19" t="inlineStr">
         <is>
-          <t>Control de personal propio de cada ministerio.</t>
-        </is>
-      </c>
-      <c r="D79" s="22" t="inlineStr">
-        <is>
-          <t>Recuperado v1</t>
+          <t>Tablero de avisos y notificaciones interno por área.</t>
+        </is>
+      </c>
+      <c r="D79" s="19" t="inlineStr">
+        <is>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E79" s="19" t="inlineStr">
@@ -7192,17 +7208,17 @@
     <row r="80">
       <c r="A80" s="18" t="inlineStr">
         <is>
-          <t>M6-02</t>
+          <t>M5-06</t>
         </is>
       </c>
       <c r="B80" s="19" t="inlineStr">
         <is>
-          <t>M6 Ministerios de servicio</t>
+          <t>M5 Áreas y servidores</t>
         </is>
       </c>
       <c r="C80" s="19" t="inlineStr">
         <is>
-          <t>Menú o catálogo digital interactivo (público o interno), autogestionado.</t>
+          <t>Gestión financiera por área: caja chica y gastos operativos.</t>
         </is>
       </c>
       <c r="D80" s="19" t="inlineStr">
@@ -7256,7 +7272,7 @@
     <row r="81">
       <c r="A81" s="18" t="inlineStr">
         <is>
-          <t>M6-03</t>
+          <t>M6-01</t>
         </is>
       </c>
       <c r="B81" s="19" t="inlineStr">
@@ -7266,12 +7282,12 @@
       </c>
       <c r="C81" s="19" t="inlineStr">
         <is>
-          <t>Calendario de turnos: días regulares de servicio y eventos especiales.</t>
-        </is>
-      </c>
-      <c r="D81" s="19" t="inlineStr">
-        <is>
-          <t>v1 / v2</t>
+          <t>Control de personal propio de cada ministerio.</t>
+        </is>
+      </c>
+      <c r="D81" s="22" t="inlineStr">
+        <is>
+          <t>Recuperado v1</t>
         </is>
       </c>
       <c r="E81" s="19" t="inlineStr">
@@ -7320,7 +7336,7 @@
     <row r="82">
       <c r="A82" s="18" t="inlineStr">
         <is>
-          <t>M6-04</t>
+          <t>M6-02</t>
         </is>
       </c>
       <c r="B82" s="19" t="inlineStr">
@@ -7330,7 +7346,7 @@
       </c>
       <c r="C82" s="19" t="inlineStr">
         <is>
-          <t>Registro de asistentes o personas atendidas.</t>
+          <t>Menú o catálogo digital interactivo (público o interno), autogestionado.</t>
         </is>
       </c>
       <c r="D82" s="19" t="inlineStr">
@@ -7384,7 +7400,7 @@
     <row r="83">
       <c r="A83" s="18" t="inlineStr">
         <is>
-          <t>M6-05</t>
+          <t>M6-03</t>
         </is>
       </c>
       <c r="B83" s="19" t="inlineStr">
@@ -7394,7 +7410,7 @@
       </c>
       <c r="C83" s="19" t="inlineStr">
         <is>
-          <t>Control de gastos y de inventario básico.</t>
+          <t>Calendario de turnos: días regulares de servicio y eventos especiales.</t>
         </is>
       </c>
       <c r="D83" s="19" t="inlineStr">
@@ -7448,7 +7464,7 @@
     <row r="84">
       <c r="A84" s="18" t="inlineStr">
         <is>
-          <t>M6-06</t>
+          <t>M6-04</t>
         </is>
       </c>
       <c r="B84" s="19" t="inlineStr">
@@ -7458,7 +7474,7 @@
       </c>
       <c r="C84" s="19" t="inlineStr">
         <is>
-          <t>Canal de comunicación directo con el área de Administración General.</t>
+          <t>Registro de asistentes o personas atendidas.</t>
         </is>
       </c>
       <c r="D84" s="19" t="inlineStr">
@@ -7512,7 +7528,7 @@
     <row r="85">
       <c r="A85" s="18" t="inlineStr">
         <is>
-          <t>M6-07</t>
+          <t>M6-05</t>
         </is>
       </c>
       <c r="B85" s="19" t="inlineStr">
@@ -7522,12 +7538,12 @@
       </c>
       <c r="C85" s="19" t="inlineStr">
         <is>
-          <t>Servicio Médico: los datos de salud de las personas atendidas requieren tratamiento de datos sensibles. Por definir alcance.</t>
-        </is>
-      </c>
-      <c r="D85" s="21" t="inlineStr">
-        <is>
-          <t>Nuevo v3</t>
+          <t>Control de gastos y de inventario básico.</t>
+        </is>
+      </c>
+      <c r="D85" s="19" t="inlineStr">
+        <is>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E85" s="19" t="inlineStr">
@@ -7562,7 +7578,7 @@
       </c>
       <c r="K85" s="19" t="inlineStr">
         <is>
-          <t>Por definir</t>
+          <t>VoBo pendiente</t>
         </is>
       </c>
       <c r="L85" s="19" t="inlineStr">
@@ -7576,17 +7592,17 @@
     <row r="86">
       <c r="A86" s="18" t="inlineStr">
         <is>
-          <t>M7-01</t>
+          <t>M6-06</t>
         </is>
       </c>
       <c r="B86" s="19" t="inlineStr">
         <is>
-          <t>M7 Eventos y aforo</t>
+          <t>M6 Ministerios de servicio</t>
         </is>
       </c>
       <c r="C86" s="19" t="inlineStr">
         <is>
-          <t>Eventos abiertos o evangelísticos con formulario de inscripción rápida, sin requerir historial previo.</t>
+          <t>Canal de comunicación directo con el área de Administración General.</t>
         </is>
       </c>
       <c r="D86" s="19" t="inlineStr">
@@ -7640,22 +7656,22 @@
     <row r="87">
       <c r="A87" s="18" t="inlineStr">
         <is>
-          <t>M7-02</t>
+          <t>M6-07</t>
         </is>
       </c>
       <c r="B87" s="19" t="inlineStr">
         <is>
-          <t>M7 Eventos y aforo</t>
+          <t>M6 Ministerios de servicio</t>
         </is>
       </c>
       <c r="C87" s="19" t="inlineStr">
         <is>
-          <t>Consolidación (inducción de personas que asisten por primera vez) como tipo de evento.</t>
-        </is>
-      </c>
-      <c r="D87" s="22" t="inlineStr">
-        <is>
-          <t>Recuperado v1</t>
+          <t>Servicio Médico: los datos de salud de las personas atendidas requieren tratamiento de datos sensibles. Por definir alcance.</t>
+        </is>
+      </c>
+      <c r="D87" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3</t>
         </is>
       </c>
       <c r="E87" s="19" t="inlineStr">
@@ -7690,7 +7706,7 @@
       </c>
       <c r="K87" s="19" t="inlineStr">
         <is>
-          <t>VoBo pendiente</t>
+          <t>Por definir</t>
         </is>
       </c>
       <c r="L87" s="19" t="inlineStr">
@@ -7704,7 +7720,7 @@
     <row r="88">
       <c r="A88" s="18" t="inlineStr">
         <is>
-          <t>M7-03</t>
+          <t>M7-01</t>
         </is>
       </c>
       <c r="B88" s="19" t="inlineStr">
@@ -7714,12 +7730,12 @@
       </c>
       <c r="C88" s="19" t="inlineStr">
         <is>
-          <t>Encargados de evento (personal de la iglesia únicamente; no se controla personal externo).</t>
-        </is>
-      </c>
-      <c r="D88" s="22" t="inlineStr">
-        <is>
-          <t>Recuperado v1</t>
+          <t>Eventos abiertos o evangelísticos con formulario de inscripción rápida, sin requerir historial previo.</t>
+        </is>
+      </c>
+      <c r="D88" s="19" t="inlineStr">
+        <is>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E88" s="19" t="inlineStr">
@@ -7768,7 +7784,7 @@
     <row r="89">
       <c r="A89" s="18" t="inlineStr">
         <is>
-          <t>M7-04</t>
+          <t>M7-02</t>
         </is>
       </c>
       <c r="B89" s="19" t="inlineStr">
@@ -7778,12 +7794,12 @@
       </c>
       <c r="C89" s="19" t="inlineStr">
         <is>
-          <t>Control de cupo en tiempo real que bloquea el sobrecupo en eventos con aforo limitado (ej. 30 o 50 lugares).</t>
-        </is>
-      </c>
-      <c r="D89" s="19" t="inlineStr">
-        <is>
-          <t>v1 / v2</t>
+          <t>Consolidación (inducción de personas que asisten por primera vez) como tipo de evento.</t>
+        </is>
+      </c>
+      <c r="D89" s="22" t="inlineStr">
+        <is>
+          <t>Recuperado v1</t>
         </is>
       </c>
       <c r="E89" s="19" t="inlineStr">
@@ -7832,7 +7848,7 @@
     <row r="90">
       <c r="A90" s="18" t="inlineStr">
         <is>
-          <t>M7-05</t>
+          <t>M7-03</t>
         </is>
       </c>
       <c r="B90" s="19" t="inlineStr">
@@ -7842,12 +7858,12 @@
       </c>
       <c r="C90" s="19" t="inlineStr">
         <is>
-          <t>Control de asistentes sin lista previa, para aforo y para dar a conocer la iglesia.</t>
-        </is>
-      </c>
-      <c r="D90" s="19" t="inlineStr">
-        <is>
-          <t>v1</t>
+          <t>Encargados de evento (personal de la iglesia únicamente; no se controla personal externo).</t>
+        </is>
+      </c>
+      <c r="D90" s="22" t="inlineStr">
+        <is>
+          <t>Recuperado v1</t>
         </is>
       </c>
       <c r="E90" s="19" t="inlineStr">
@@ -7896,7 +7912,7 @@
     <row r="91">
       <c r="A91" s="18" t="inlineStr">
         <is>
-          <t>M7-06</t>
+          <t>M7-04</t>
         </is>
       </c>
       <c r="B91" s="19" t="inlineStr">
@@ -7906,12 +7922,12 @@
       </c>
       <c r="C91" s="19" t="inlineStr">
         <is>
-          <t>Seguimiento de personas nuevas: conversión de un invitado a Expediente Digital y canalización a un curso o Grupo de Conexión.</t>
-        </is>
-      </c>
-      <c r="D91" s="21" t="inlineStr">
-        <is>
-          <t>Nuevo v3</t>
+          <t>Control de cupo en tiempo real que bloquea el sobrecupo en eventos con aforo limitado (ej. 30 o 50 lugares).</t>
+        </is>
+      </c>
+      <c r="D91" s="19" t="inlineStr">
+        <is>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E91" s="19" t="inlineStr">
@@ -7960,52 +7976,52 @@
     <row r="92">
       <c r="A92" s="18" t="inlineStr">
         <is>
-          <t>NF-01</t>
+          <t>M7-05</t>
         </is>
       </c>
       <c r="B92" s="19" t="inlineStr">
         <is>
-          <t>No funcionales</t>
+          <t>M7 Eventos y aforo</t>
         </is>
       </c>
       <c r="C92" s="19" t="inlineStr">
         <is>
-          <t>Cumplimiento de la LFPDPPP: aviso de privacidad, consentimiento y derechos ARCO.</t>
+          <t>Control de asistentes sin lista previa, para aforo y para dar a conocer la iglesia.</t>
         </is>
       </c>
       <c r="D92" s="19" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>v1</t>
         </is>
       </c>
       <c r="E92" s="19" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Fuera del MVP</t>
         </is>
       </c>
       <c r="F92" s="19" t="inlineStr">
         <is>
-          <t>Fase 0</t>
+          <t>Fase 4</t>
         </is>
       </c>
       <c r="G92" s="19" t="inlineStr">
         <is>
-          <t>Sprint 1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H92" s="19" t="inlineStr">
         <is>
-          <t>H1 · 18-oct (núcleo Fase 0)</t>
-        </is>
-      </c>
-      <c r="I92" s="19" t="inlineStr">
-        <is>
-          <t>Como iglesia queremos cumplir con la LFPDPPP.</t>
-        </is>
-      </c>
-      <c r="J92" s="19" t="inlineStr">
-        <is>
-          <t>Aviso de privacidad, consentimiento y atención de derechos ARCO disponibles.</t>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="I92" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
+        </is>
+      </c>
+      <c r="J92" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
         </is>
       </c>
       <c r="K92" s="19" t="inlineStr">
@@ -8024,52 +8040,52 @@
     <row r="93">
       <c r="A93" s="18" t="inlineStr">
         <is>
-          <t>NF-02</t>
+          <t>M7-06</t>
         </is>
       </c>
       <c r="B93" s="19" t="inlineStr">
         <is>
-          <t>No funcionales</t>
+          <t>M7 Eventos y aforo</t>
         </is>
       </c>
       <c r="C93" s="19" t="inlineStr">
         <is>
-          <t>Cifrado en tránsito y en reposo. Cifrado adicional a nivel de campo para peticiones de oración.</t>
-        </is>
-      </c>
-      <c r="D93" s="19" t="inlineStr">
-        <is>
-          <t>v3</t>
+          <t>Seguimiento de personas nuevas: conversión de un invitado a Expediente Digital y canalización a un curso o Grupo de Conexión.</t>
+        </is>
+      </c>
+      <c r="D93" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3</t>
         </is>
       </c>
       <c r="E93" s="19" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Fuera del MVP</t>
         </is>
       </c>
       <c r="F93" s="19" t="inlineStr">
         <is>
-          <t>Fase 0</t>
+          <t>Fase 4</t>
         </is>
       </c>
       <c r="G93" s="19" t="inlineStr">
         <is>
-          <t>Sprint 0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H93" s="19" t="inlineStr">
         <is>
-          <t>H1 · 18-oct (núcleo Fase 0)</t>
-        </is>
-      </c>
-      <c r="I93" s="19" t="inlineStr">
-        <is>
-          <t>Como iglesia queremos proteger los datos sensibles.</t>
-        </is>
-      </c>
-      <c r="J93" s="19" t="inlineStr">
-        <is>
-          <t>HTTPS obligatorio y peticiones de oración ilegibles directamente en la base.</t>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="I93" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
+        </is>
+      </c>
+      <c r="J93" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
         </is>
       </c>
       <c r="K93" s="19" t="inlineStr">
@@ -8079,24 +8095,16 @@
       </c>
       <c r="L93" s="19" t="inlineStr">
         <is>
-          <t>En pruebas</t>
-        </is>
-      </c>
-      <c r="M93" s="19" t="inlineStr">
-        <is>
-          <t>Rama feature/m3-peticiones-oracion · 166 pruebas de backend y 32 de frontend pasan; probado contra la base real</t>
-        </is>
-      </c>
-      <c r="N93" s="19" t="inlineStr">
-        <is>
-          <t>2026-10-24 · Peticiones cifradas a nivel de campo; falta cifrado en reposo de toda la base (proveedor de nube).</t>
-        </is>
-      </c>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M93" s="19" t="inlineStr"/>
+      <c r="N93" s="19" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="18" t="inlineStr">
         <is>
-          <t>NF-03</t>
+          <t>NF-01</t>
         </is>
       </c>
       <c r="B94" s="19" t="inlineStr">
@@ -8106,7 +8114,7 @@
       </c>
       <c r="C94" s="19" t="inlineStr">
         <is>
-          <t>Bitácora de auditoría de solo-añadir: quién consultó o modificó expedientes, ofrendas y asistencias.</t>
+          <t>Cumplimiento de la LFPDPPP: aviso de privacidad, consentimiento y derechos ARCO.</t>
         </is>
       </c>
       <c r="D94" s="19" t="inlineStr">
@@ -8136,12 +8144,12 @@
       </c>
       <c r="I94" s="19" t="inlineStr">
         <is>
-          <t>Como pastor quiero una bitácora que nadie pueda alterar.</t>
+          <t>Como iglesia queremos cumplir con la LFPDPPP.</t>
         </is>
       </c>
       <c r="J94" s="19" t="inlineStr">
         <is>
-          <t>El usuario de la aplicación no puede actualizar ni borrar registros de bitácora.</t>
+          <t>Aviso de privacidad, consentimiento y atención de derechos ARCO disponibles.</t>
         </is>
       </c>
       <c r="K94" s="19" t="inlineStr">
@@ -8151,24 +8159,16 @@
       </c>
       <c r="L94" s="19" t="inlineStr">
         <is>
-          <t>En pruebas</t>
-        </is>
-      </c>
-      <c r="M94" s="19" t="inlineStr">
-        <is>
-          <t>Rama feature/nf-03-bitacora · 69 pruebas de backend pasan</t>
-        </is>
-      </c>
-      <c r="N94" s="19" t="inlineStr">
-        <is>
-          <t>2026-10-10 · Bloqueo en aplicación y trigger de PostgreSQL (UPDATE/DELETE/TRUNCATE); pantalla de consulta con permiso bitacora.ver.</t>
-        </is>
-      </c>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M94" s="19" t="inlineStr"/>
+      <c r="N94" s="19" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="18" t="inlineStr">
         <is>
-          <t>NF-04</t>
+          <t>NF-02</t>
         </is>
       </c>
       <c r="B95" s="19" t="inlineStr">
@@ -8178,7 +8178,7 @@
       </c>
       <c r="C95" s="19" t="inlineStr">
         <is>
-          <t>Respaldos automáticos diarios cifrados y prueba periódica de restauración.</t>
+          <t>Cifrado en tránsito y en reposo. Cifrado adicional a nivel de campo para peticiones de oración.</t>
         </is>
       </c>
       <c r="D95" s="19" t="inlineStr">
@@ -8208,12 +8208,12 @@
       </c>
       <c r="I95" s="19" t="inlineStr">
         <is>
-          <t>Como iglesia queremos no perder información.</t>
+          <t>Como iglesia queremos proteger los datos sensibles.</t>
         </is>
       </c>
       <c r="J95" s="19" t="inlineStr">
         <is>
-          <t>Respaldo diario cifrado y restauración probada en un ambiente de pruebas.</t>
+          <t>HTTPS obligatorio y peticiones de oración ilegibles directamente en la base.</t>
         </is>
       </c>
       <c r="K95" s="19" t="inlineStr">
@@ -8223,16 +8223,24 @@
       </c>
       <c r="L95" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M95" s="19" t="inlineStr"/>
-      <c r="N95" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M95" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/m3-peticiones-oracion · 166 pruebas de backend y 32 de frontend pasan; probado contra la base real</t>
+        </is>
+      </c>
+      <c r="N95" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-24 · Peticiones cifradas a nivel de campo; falta cifrado en reposo de toda la base (proveedor de nube).</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="18" t="inlineStr">
         <is>
-          <t>NF-05</t>
+          <t>NF-03</t>
         </is>
       </c>
       <c r="B96" s="19" t="inlineStr">
@@ -8242,61 +8250,69 @@
       </c>
       <c r="C96" s="19" t="inlineStr">
         <is>
-          <t>Disponibilidad esperada en horarios de servicio (fines de semana y reuniones de grupo). Por definir meta.</t>
-        </is>
-      </c>
-      <c r="D96" s="21" t="inlineStr">
-        <is>
-          <t>Nuevo v3</t>
+          <t>Bitácora de auditoría de solo-añadir: quién consultó o modificó expedientes, ofrendas y asistencias.</t>
+        </is>
+      </c>
+      <c r="D96" s="19" t="inlineStr">
+        <is>
+          <t>v3</t>
         </is>
       </c>
       <c r="E96" s="19" t="inlineStr">
         <is>
-          <t>Fuera del MVP</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="F96" s="19" t="inlineStr">
         <is>
-          <t>Transversal</t>
+          <t>Fase 0</t>
         </is>
       </c>
       <c r="G96" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sprint 1</t>
         </is>
       </c>
       <c r="H96" s="19" t="inlineStr">
         <is>
-          <t>Posterior</t>
-        </is>
-      </c>
-      <c r="I96" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
-        </is>
-      </c>
-      <c r="J96" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
+          <t>H1 · 18-oct (núcleo Fase 0)</t>
+        </is>
+      </c>
+      <c r="I96" s="19" t="inlineStr">
+        <is>
+          <t>Como pastor quiero una bitácora que nadie pueda alterar.</t>
+        </is>
+      </c>
+      <c r="J96" s="19" t="inlineStr">
+        <is>
+          <t>El usuario de la aplicación no puede actualizar ni borrar registros de bitácora.</t>
         </is>
       </c>
       <c r="K96" s="19" t="inlineStr">
         <is>
-          <t>Por definir</t>
+          <t>VoBo pendiente</t>
         </is>
       </c>
       <c r="L96" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M96" s="19" t="inlineStr"/>
-      <c r="N96" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M96" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/nf-03-bitacora · 69 pruebas de backend pasan</t>
+        </is>
+      </c>
+      <c r="N96" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-10 · Bloqueo en aplicación y trigger de PostgreSQL (UPDATE/DELETE/TRUNCATE); pantalla de consulta con permiso bitacora.ver.</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="18" t="inlineStr">
         <is>
-          <t>NF-06</t>
+          <t>NF-04</t>
         </is>
       </c>
       <c r="B97" s="19" t="inlineStr">
@@ -8306,7 +8322,7 @@
       </c>
       <c r="C97" s="19" t="inlineStr">
         <is>
-          <t>Pase de lista sin conexión con sincronización posterior (reuniones en domicilios con mala señal).</t>
+          <t>Respaldos automáticos diarios cifrados y prueba periódica de restauración.</t>
         </is>
       </c>
       <c r="D97" s="19" t="inlineStr">
@@ -8326,22 +8342,22 @@
       </c>
       <c r="G97" s="19" t="inlineStr">
         <is>
-          <t>Sprint 3</t>
+          <t>Sprint 0</t>
         </is>
       </c>
       <c r="H97" s="19" t="inlineStr">
         <is>
-          <t>H3 · MVP (Grupos)</t>
+          <t>H1 · 18-oct (núcleo Fase 0)</t>
         </is>
       </c>
       <c r="I97" s="19" t="inlineStr">
         <is>
-          <t>Como secretario quiero que el pase de lista funcione sin señal.</t>
+          <t>Como iglesia queremos no perder información.</t>
         </is>
       </c>
       <c r="J97" s="19" t="inlineStr">
         <is>
-          <t>Prueba en modo avión y sincronización al reconectar.</t>
+          <t>Respaldo diario cifrado y restauración probada en un ambiente de pruebas.</t>
         </is>
       </c>
       <c r="K97" s="19" t="inlineStr">
@@ -8351,24 +8367,16 @@
       </c>
       <c r="L97" s="19" t="inlineStr">
         <is>
-          <t>En pruebas</t>
-        </is>
-      </c>
-      <c r="M97" s="19" t="inlineStr">
-        <is>
-          <t>Rama feature/nf-06-sin-conexion · 117 pruebas de backend y 27 de frontend; probado en Chrome real con service worker</t>
-        </is>
-      </c>
-      <c r="N97" s="19" t="inlineStr">
-        <is>
-          <t>2026-10-24 · Probado de punta a punta en Chrome (sin red → cola → sincronización). Pendiente probar en Android e iOS reales.</t>
-        </is>
-      </c>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M97" s="19" t="inlineStr"/>
+      <c r="N97" s="19" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="18" t="inlineStr">
         <is>
-          <t>NF-07</t>
+          <t>NF-05</t>
         </is>
       </c>
       <c r="B98" s="19" t="inlineStr">
@@ -8378,47 +8386,47 @@
       </c>
       <c r="C98" s="19" t="inlineStr">
         <is>
-          <t>Funciona en Android, iOS y escritorio. En iOS, las notificaciones push requieren instalar la PWA; el respaldo por WhatsApp cubre el resto.</t>
-        </is>
-      </c>
-      <c r="D98" s="19" t="inlineStr">
-        <is>
-          <t>v3</t>
+          <t>Disponibilidad esperada en horarios de servicio (fines de semana y reuniones de grupo). Por definir meta.</t>
+        </is>
+      </c>
+      <c r="D98" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3</t>
         </is>
       </c>
       <c r="E98" s="19" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Fuera del MVP</t>
         </is>
       </c>
       <c r="F98" s="19" t="inlineStr">
         <is>
-          <t>Fase 0</t>
+          <t>Transversal</t>
         </is>
       </c>
       <c r="G98" s="19" t="inlineStr">
         <is>
-          <t>Sprint 0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H98" s="19" t="inlineStr">
         <is>
-          <t>H1 · 18-oct (núcleo Fase 0)</t>
-        </is>
-      </c>
-      <c r="I98" s="19" t="inlineStr">
-        <is>
-          <t>Como usuario quiero usar el sistema en mi dispositivo.</t>
-        </is>
-      </c>
-      <c r="J98" s="19" t="inlineStr">
-        <is>
-          <t>Pruebas en Android, iOS y escritorio; push en iOS con la PWA instalada y respaldo por WhatsApp.</t>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="I98" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
+        </is>
+      </c>
+      <c r="J98" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
         </is>
       </c>
       <c r="K98" s="19" t="inlineStr">
         <is>
-          <t>VoBo pendiente</t>
+          <t>Por definir</t>
         </is>
       </c>
       <c r="L98" s="19" t="inlineStr">
@@ -8432,7 +8440,7 @@
     <row r="99">
       <c r="A99" s="18" t="inlineStr">
         <is>
-          <t>NF-08</t>
+          <t>NF-06</t>
         </is>
       </c>
       <c r="B99" s="19" t="inlineStr">
@@ -8442,12 +8450,12 @@
       </c>
       <c r="C99" s="19" t="inlineStr">
         <is>
-          <t>Dimensionamiento para ~1,000 personas, con picos los fines de semana, y margen de crecimiento.</t>
-        </is>
-      </c>
-      <c r="D99" s="21" t="inlineStr">
-        <is>
-          <t>Resp. P8</t>
+          <t>Pase de lista sin conexión con sincronización posterior (reuniones en domicilios con mala señal).</t>
+        </is>
+      </c>
+      <c r="D99" s="19" t="inlineStr">
+        <is>
+          <t>v3</t>
         </is>
       </c>
       <c r="E99" s="19" t="inlineStr">
@@ -8462,22 +8470,22 @@
       </c>
       <c r="G99" s="19" t="inlineStr">
         <is>
-          <t>Sprint 0</t>
+          <t>Sprint 3</t>
         </is>
       </c>
       <c r="H99" s="19" t="inlineStr">
         <is>
-          <t>H1 · 18-oct (núcleo Fase 0)</t>
+          <t>H3 · MVP (Grupos)</t>
         </is>
       </c>
       <c r="I99" s="19" t="inlineStr">
         <is>
-          <t>Como iglesia queremos que el sistema soporte a ~1,000 personas.</t>
+          <t>Como secretario quiero que el pase de lista funcione sin señal.</t>
         </is>
       </c>
       <c r="J99" s="19" t="inlineStr">
         <is>
-          <t>Prueba de carga con volumen representativo (por definir) sin degradación.</t>
+          <t>Prueba en modo avión y sincronización al reconectar.</t>
         </is>
       </c>
       <c r="K99" s="19" t="inlineStr">
@@ -8487,16 +8495,24 @@
       </c>
       <c r="L99" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M99" s="19" t="inlineStr"/>
-      <c r="N99" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M99" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/nf-06-sin-conexion · 117 pruebas de backend y 27 de frontend; probado en Chrome real con service worker</t>
+        </is>
+      </c>
+      <c r="N99" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-24 · Probado de punta a punta en Chrome (sin red → cola → sincronización). Pendiente probar en Android e iOS reales.</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="18" t="inlineStr">
         <is>
-          <t>NF-09</t>
+          <t>NF-07</t>
         </is>
       </c>
       <c r="B100" s="19" t="inlineStr">
@@ -8506,42 +8522,42 @@
       </c>
       <c r="C100" s="19" t="inlineStr">
         <is>
-          <t>Reportes transversales: asistencia, finanzas, crecimiento de la iglesia, exportables a Excel y PDF.</t>
-        </is>
-      </c>
-      <c r="D100" s="21" t="inlineStr">
-        <is>
-          <t>Nuevo v3</t>
+          <t>Funciona en Android, iOS y escritorio. En iOS, las notificaciones push requieren instalar la PWA; el respaldo por WhatsApp cubre el resto.</t>
+        </is>
+      </c>
+      <c r="D100" s="19" t="inlineStr">
+        <is>
+          <t>v3</t>
         </is>
       </c>
       <c r="E100" s="19" t="inlineStr">
         <is>
-          <t>Fuera del MVP</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="F100" s="19" t="inlineStr">
         <is>
-          <t>Transversal</t>
+          <t>Fase 0</t>
         </is>
       </c>
       <c r="G100" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sprint 0</t>
         </is>
       </c>
       <c r="H100" s="19" t="inlineStr">
         <is>
-          <t>Posterior</t>
-        </is>
-      </c>
-      <c r="I100" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
-        </is>
-      </c>
-      <c r="J100" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
+          <t>H1 · 18-oct (núcleo Fase 0)</t>
+        </is>
+      </c>
+      <c r="I100" s="19" t="inlineStr">
+        <is>
+          <t>Como usuario quiero usar el sistema en mi dispositivo.</t>
+        </is>
+      </c>
+      <c r="J100" s="19" t="inlineStr">
+        <is>
+          <t>Pruebas en Android, iOS y escritorio; push en iOS con la PWA instalada y respaldo por WhatsApp.</t>
         </is>
       </c>
       <c r="K100" s="19" t="inlineStr">
@@ -8560,7 +8576,7 @@
     <row r="101">
       <c r="A101" s="18" t="inlineStr">
         <is>
-          <t>NF-10</t>
+          <t>NF-08</t>
         </is>
       </c>
       <c r="B101" s="19" t="inlineStr">
@@ -8570,12 +8586,12 @@
       </c>
       <c r="C101" s="19" t="inlineStr">
         <is>
-          <t>Usabilidad para personas mayores: tipografía grande, alto contraste, flujos cortos (ver sección 5).</t>
-        </is>
-      </c>
-      <c r="D101" s="19" t="inlineStr">
-        <is>
-          <t>v3 + Obs. 1</t>
+          <t>Dimensionamiento para ~1,000 personas, con picos los fines de semana, y margen de crecimiento.</t>
+        </is>
+      </c>
+      <c r="D101" s="21" t="inlineStr">
+        <is>
+          <t>Resp. P8</t>
         </is>
       </c>
       <c r="E101" s="19" t="inlineStr">
@@ -8600,12 +8616,12 @@
       </c>
       <c r="I101" s="19" t="inlineStr">
         <is>
-          <t>Como persona mayor quiero una interfaz fácil de leer y usar.</t>
+          <t>Como iglesia queremos que el sistema soporte a ~1,000 personas.</t>
         </is>
       </c>
       <c r="J101" s="19" t="inlineStr">
         <is>
-          <t>Texto base 18 px, botones de al menos 48 px, contraste AA; prueba con usuarios mayores.</t>
+          <t>Prueba de carga con volumen representativo (por definir) sin degradación.</t>
         </is>
       </c>
       <c r="K101" s="19" t="inlineStr">
@@ -8621,9 +8637,137 @@
       <c r="M101" s="19" t="inlineStr"/>
       <c r="N101" s="19" t="inlineStr"/>
     </row>
+    <row r="102">
+      <c r="A102" s="18" t="inlineStr">
+        <is>
+          <t>NF-09</t>
+        </is>
+      </c>
+      <c r="B102" s="19" t="inlineStr">
+        <is>
+          <t>No funcionales</t>
+        </is>
+      </c>
+      <c r="C102" s="19" t="inlineStr">
+        <is>
+          <t>Reportes transversales: asistencia, finanzas, crecimiento de la iglesia, exportables a Excel y PDF.</t>
+        </is>
+      </c>
+      <c r="D102" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3</t>
+        </is>
+      </c>
+      <c r="E102" s="19" t="inlineStr">
+        <is>
+          <t>Fuera del MVP</t>
+        </is>
+      </c>
+      <c r="F102" s="19" t="inlineStr">
+        <is>
+          <t>Transversal</t>
+        </is>
+      </c>
+      <c r="G102" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H102" s="19" t="inlineStr">
+        <is>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="I102" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
+        </is>
+      </c>
+      <c r="J102" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
+        </is>
+      </c>
+      <c r="K102" s="19" t="inlineStr">
+        <is>
+          <t>VoBo pendiente</t>
+        </is>
+      </c>
+      <c r="L102" s="19" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M102" s="19" t="inlineStr"/>
+      <c r="N102" s="19" t="inlineStr"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="18" t="inlineStr">
+        <is>
+          <t>NF-10</t>
+        </is>
+      </c>
+      <c r="B103" s="19" t="inlineStr">
+        <is>
+          <t>No funcionales</t>
+        </is>
+      </c>
+      <c r="C103" s="19" t="inlineStr">
+        <is>
+          <t>Usabilidad para personas mayores: tipografía grande, alto contraste, flujos cortos (ver sección 5).</t>
+        </is>
+      </c>
+      <c r="D103" s="19" t="inlineStr">
+        <is>
+          <t>v3 + Obs. 1</t>
+        </is>
+      </c>
+      <c r="E103" s="19" t="inlineStr">
+        <is>
+          <t>MVP</t>
+        </is>
+      </c>
+      <c r="F103" s="19" t="inlineStr">
+        <is>
+          <t>Fase 0</t>
+        </is>
+      </c>
+      <c r="G103" s="19" t="inlineStr">
+        <is>
+          <t>Sprint 0</t>
+        </is>
+      </c>
+      <c r="H103" s="19" t="inlineStr">
+        <is>
+          <t>H1 · 18-oct (núcleo Fase 0)</t>
+        </is>
+      </c>
+      <c r="I103" s="19" t="inlineStr">
+        <is>
+          <t>Como persona mayor quiero una interfaz fácil de leer y usar.</t>
+        </is>
+      </c>
+      <c r="J103" s="19" t="inlineStr">
+        <is>
+          <t>Texto base 18 px, botones de al menos 48 px, contraste AA; prueba con usuarios mayores.</t>
+        </is>
+      </c>
+      <c r="K103" s="19" t="inlineStr">
+        <is>
+          <t>VoBo pendiente</t>
+        </is>
+      </c>
+      <c r="L103" s="19" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M103" s="19" t="inlineStr"/>
+      <c r="N103" s="19" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N101"/>
-  <conditionalFormatting sqref="L2:L101">
+  <autoFilter ref="A1:N103"/>
+  <conditionalFormatting sqref="L2:L103">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$L2="Hecho"</formula>
     </cfRule>
@@ -8640,7 +8784,7 @@
       <formula>$L2="Bloqueado"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K2:K101">
+  <conditionalFormatting sqref="K2:K103">
     <cfRule type="expression" priority="6" dxfId="0">
       <formula>$K2="Aprobado"</formula>
     </cfRule>
@@ -8648,16 +8792,16 @@
       <formula>$K2="Por definir"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H2:H101">
+  <conditionalFormatting sqref="H2:H103">
     <cfRule type="expression" priority="8" dxfId="5">
       <formula>LEFT($H2,2)="H1"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="L2:L101" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="L2:L103" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Pendiente,En diseño,En desarrollo,En pruebas,Hecho,Bloqueado"</formula1>
     </dataValidation>
-    <dataValidation sqref="K2:K101" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="K2:K103" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"VoBo pendiente,Aprobado,Por definir,Rechazado"</formula1>
     </dataValidation>
   </dataValidations>
@@ -9455,7 +9599,7 @@
       </c>
       <c r="D29" s="24" t="inlineStr">
         <is>
-          <t>Los ministerios se manejan como unidades (áreas de servicio). Avisos masivos a iglesia, grupos, unidades y personas, con permisos por destino, y avisos recibidos agrupados.</t>
+          <t>Los ministerios (áreas de servicio) se llaman así en toda la aplicación. Avisos masivos a iglesia, grupos, unidades y personas, con permisos por destino, y avisos recibidos agrupados.</t>
         </is>
       </c>
       <c r="E29" s="24" t="inlineStr">
@@ -9477,17 +9621,17 @@
       </c>
       <c r="C30" s="24" t="inlineStr">
         <is>
-          <t>M1-11</t>
+          <t>M1-27</t>
         </is>
       </c>
       <c r="D30" s="24" t="inlineStr">
         <is>
-          <t>Campos editables por la persona vs. por administración.</t>
+          <t>La persona edita nombre, domicilio, datos básicos y foto; no edita acceso (WhatsApp, correo, PIN) ni relaciones (grupo, sector, ministerios, roles).</t>
         </is>
       </c>
       <c r="E30" s="24" t="inlineStr">
         <is>
-          <t>Planeado (paso 7)</t>
+          <t>Hecho (v3.21)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Oración para todos y vehículos propios en Mi cuenta (paso 9)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/trazabilidad/Matriz de Trazabilidad MDF.xlsx
+++ b/docs/trazabilidad/Matriz de Trazabilidad MDF.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Origen v1" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Matriz'!$A$1:$N$103</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Matriz'!$A$1:$N$105</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -897,31 +897,31 @@
         </is>
       </c>
       <c r="B5" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$103,$A5)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$105,$A5)</f>
         <v/>
       </c>
       <c r="C5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$103,$A5,Matriz!$L$2:$L$103,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$105,$A5,Matriz!$L$2:$L$105,"Pendiente")</f>
         <v/>
       </c>
       <c r="D5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$103,$A5,Matriz!$L$2:$L$103,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$105,$A5,Matriz!$L$2:$L$105,"En diseño")</f>
         <v/>
       </c>
       <c r="E5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$103,$A5,Matriz!$L$2:$L$103,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$105,$A5,Matriz!$L$2:$L$105,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$103,$A5,Matriz!$L$2:$L$103,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$105,$A5,Matriz!$L$2:$L$105,"En pruebas")</f>
         <v/>
       </c>
       <c r="G5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$103,$A5,Matriz!$L$2:$L$103,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$105,$A5,Matriz!$L$2:$L$105,"Hecho")</f>
         <v/>
       </c>
       <c r="H5" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$103,$A5,Matriz!$L$2:$L$103,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$105,$A5,Matriz!$L$2:$L$105,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I5" s="13">
@@ -936,31 +936,31 @@
         </is>
       </c>
       <c r="B6" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$103,$A6)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$105,$A6)</f>
         <v/>
       </c>
       <c r="C6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$103,$A6,Matriz!$L$2:$L$103,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$105,$A6,Matriz!$L$2:$L$105,"Pendiente")</f>
         <v/>
       </c>
       <c r="D6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$103,$A6,Matriz!$L$2:$L$103,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$105,$A6,Matriz!$L$2:$L$105,"En diseño")</f>
         <v/>
       </c>
       <c r="E6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$103,$A6,Matriz!$L$2:$L$103,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$105,$A6,Matriz!$L$2:$L$105,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$103,$A6,Matriz!$L$2:$L$103,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$105,$A6,Matriz!$L$2:$L$105,"En pruebas")</f>
         <v/>
       </c>
       <c r="G6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$103,$A6,Matriz!$L$2:$L$103,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$105,$A6,Matriz!$L$2:$L$105,"Hecho")</f>
         <v/>
       </c>
       <c r="H6" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$103,$A6,Matriz!$L$2:$L$103,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$105,$A6,Matriz!$L$2:$L$105,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I6" s="13">
@@ -975,31 +975,31 @@
         </is>
       </c>
       <c r="B7" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$103,$A7)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$105,$A7)</f>
         <v/>
       </c>
       <c r="C7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$103,$A7,Matriz!$L$2:$L$103,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$105,$A7,Matriz!$L$2:$L$105,"Pendiente")</f>
         <v/>
       </c>
       <c r="D7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$103,$A7,Matriz!$L$2:$L$103,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$105,$A7,Matriz!$L$2:$L$105,"En diseño")</f>
         <v/>
       </c>
       <c r="E7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$103,$A7,Matriz!$L$2:$L$103,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$105,$A7,Matriz!$L$2:$L$105,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$103,$A7,Matriz!$L$2:$L$103,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$105,$A7,Matriz!$L$2:$L$105,"En pruebas")</f>
         <v/>
       </c>
       <c r="G7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$103,$A7,Matriz!$L$2:$L$103,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$105,$A7,Matriz!$L$2:$L$105,"Hecho")</f>
         <v/>
       </c>
       <c r="H7" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$103,$A7,Matriz!$L$2:$L$103,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$105,$A7,Matriz!$L$2:$L$105,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I7" s="13">
@@ -1014,31 +1014,31 @@
         </is>
       </c>
       <c r="B8" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$103,$A8)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$105,$A8)</f>
         <v/>
       </c>
       <c r="C8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$103,$A8,Matriz!$L$2:$L$103,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$105,$A8,Matriz!$L$2:$L$105,"Pendiente")</f>
         <v/>
       </c>
       <c r="D8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$103,$A8,Matriz!$L$2:$L$103,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$105,$A8,Matriz!$L$2:$L$105,"En diseño")</f>
         <v/>
       </c>
       <c r="E8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$103,$A8,Matriz!$L$2:$L$103,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$105,$A8,Matriz!$L$2:$L$105,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$103,$A8,Matriz!$L$2:$L$103,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$105,$A8,Matriz!$L$2:$L$105,"En pruebas")</f>
         <v/>
       </c>
       <c r="G8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$103,$A8,Matriz!$L$2:$L$103,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$105,$A8,Matriz!$L$2:$L$105,"Hecho")</f>
         <v/>
       </c>
       <c r="H8" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$103,$A8,Matriz!$L$2:$L$103,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$105,$A8,Matriz!$L$2:$L$105,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I8" s="13">
@@ -1053,31 +1053,31 @@
         </is>
       </c>
       <c r="B9" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$103,$A9)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$105,$A9)</f>
         <v/>
       </c>
       <c r="C9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$103,$A9,Matriz!$L$2:$L$103,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$105,$A9,Matriz!$L$2:$L$105,"Pendiente")</f>
         <v/>
       </c>
       <c r="D9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$103,$A9,Matriz!$L$2:$L$103,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$105,$A9,Matriz!$L$2:$L$105,"En diseño")</f>
         <v/>
       </c>
       <c r="E9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$103,$A9,Matriz!$L$2:$L$103,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$105,$A9,Matriz!$L$2:$L$105,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$103,$A9,Matriz!$L$2:$L$103,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$105,$A9,Matriz!$L$2:$L$105,"En pruebas")</f>
         <v/>
       </c>
       <c r="G9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$103,$A9,Matriz!$L$2:$L$103,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$105,$A9,Matriz!$L$2:$L$105,"Hecho")</f>
         <v/>
       </c>
       <c r="H9" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$103,$A9,Matriz!$L$2:$L$103,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$105,$A9,Matriz!$L$2:$L$105,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I9" s="13">
@@ -1092,31 +1092,31 @@
         </is>
       </c>
       <c r="B10" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$103,$A10)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$105,$A10)</f>
         <v/>
       </c>
       <c r="C10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$103,$A10,Matriz!$L$2:$L$103,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$105,$A10,Matriz!$L$2:$L$105,"Pendiente")</f>
         <v/>
       </c>
       <c r="D10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$103,$A10,Matriz!$L$2:$L$103,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$105,$A10,Matriz!$L$2:$L$105,"En diseño")</f>
         <v/>
       </c>
       <c r="E10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$103,$A10,Matriz!$L$2:$L$103,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$105,$A10,Matriz!$L$2:$L$105,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$103,$A10,Matriz!$L$2:$L$103,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$105,$A10,Matriz!$L$2:$L$105,"En pruebas")</f>
         <v/>
       </c>
       <c r="G10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$103,$A10,Matriz!$L$2:$L$103,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$105,$A10,Matriz!$L$2:$L$105,"Hecho")</f>
         <v/>
       </c>
       <c r="H10" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$103,$A10,Matriz!$L$2:$L$103,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$105,$A10,Matriz!$L$2:$L$105,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I10" s="13">
@@ -1131,31 +1131,31 @@
         </is>
       </c>
       <c r="B11" s="12">
-        <f>COUNTIF(Matriz!$F$2:$F$103,$A11)</f>
+        <f>COUNTIF(Matriz!$F$2:$F$105,$A11)</f>
         <v/>
       </c>
       <c r="C11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$103,$A11,Matriz!$L$2:$L$103,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$105,$A11,Matriz!$L$2:$L$105,"Pendiente")</f>
         <v/>
       </c>
       <c r="D11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$103,$A11,Matriz!$L$2:$L$103,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$105,$A11,Matriz!$L$2:$L$105,"En diseño")</f>
         <v/>
       </c>
       <c r="E11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$103,$A11,Matriz!$L$2:$L$103,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$105,$A11,Matriz!$L$2:$L$105,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$103,$A11,Matriz!$L$2:$L$103,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$105,$A11,Matriz!$L$2:$L$105,"En pruebas")</f>
         <v/>
       </c>
       <c r="G11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$103,$A11,Matriz!$L$2:$L$103,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$105,$A11,Matriz!$L$2:$L$105,"Hecho")</f>
         <v/>
       </c>
       <c r="H11" s="12">
-        <f>COUNTIFS(Matriz!$F$2:$F$103,$A11,Matriz!$L$2:$L$103,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$F$2:$F$105,$A11,Matriz!$L$2:$L$105,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I11" s="13">
@@ -1256,31 +1256,31 @@
         </is>
       </c>
       <c r="B16" s="12">
-        <f>COUNTIF(Matriz!$H$2:$H$103,$A16)</f>
+        <f>COUNTIF(Matriz!$H$2:$H$105,$A16)</f>
         <v/>
       </c>
       <c r="C16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$103,$A16,Matriz!$L$2:$L$103,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$105,$A16,Matriz!$L$2:$L$105,"Pendiente")</f>
         <v/>
       </c>
       <c r="D16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$103,$A16,Matriz!$L$2:$L$103,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$105,$A16,Matriz!$L$2:$L$105,"En diseño")</f>
         <v/>
       </c>
       <c r="E16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$103,$A16,Matriz!$L$2:$L$103,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$105,$A16,Matriz!$L$2:$L$105,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$103,$A16,Matriz!$L$2:$L$103,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$105,$A16,Matriz!$L$2:$L$105,"En pruebas")</f>
         <v/>
       </c>
       <c r="G16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$103,$A16,Matriz!$L$2:$L$103,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$105,$A16,Matriz!$L$2:$L$105,"Hecho")</f>
         <v/>
       </c>
       <c r="H16" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$103,$A16,Matriz!$L$2:$L$103,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$105,$A16,Matriz!$L$2:$L$105,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I16" s="13">
@@ -1295,31 +1295,31 @@
         </is>
       </c>
       <c r="B17" s="12">
-        <f>COUNTIF(Matriz!$H$2:$H$103,$A17)</f>
+        <f>COUNTIF(Matriz!$H$2:$H$105,$A17)</f>
         <v/>
       </c>
       <c r="C17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$103,$A17,Matriz!$L$2:$L$103,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$105,$A17,Matriz!$L$2:$L$105,"Pendiente")</f>
         <v/>
       </c>
       <c r="D17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$103,$A17,Matriz!$L$2:$L$103,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$105,$A17,Matriz!$L$2:$L$105,"En diseño")</f>
         <v/>
       </c>
       <c r="E17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$103,$A17,Matriz!$L$2:$L$103,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$105,$A17,Matriz!$L$2:$L$105,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$103,$A17,Matriz!$L$2:$L$103,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$105,$A17,Matriz!$L$2:$L$105,"En pruebas")</f>
         <v/>
       </c>
       <c r="G17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$103,$A17,Matriz!$L$2:$L$103,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$105,$A17,Matriz!$L$2:$L$105,"Hecho")</f>
         <v/>
       </c>
       <c r="H17" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$103,$A17,Matriz!$L$2:$L$103,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$105,$A17,Matriz!$L$2:$L$105,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I17" s="13">
@@ -1334,31 +1334,31 @@
         </is>
       </c>
       <c r="B18" s="12">
-        <f>COUNTIF(Matriz!$H$2:$H$103,$A18)</f>
+        <f>COUNTIF(Matriz!$H$2:$H$105,$A18)</f>
         <v/>
       </c>
       <c r="C18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$103,$A18,Matriz!$L$2:$L$103,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$105,$A18,Matriz!$L$2:$L$105,"Pendiente")</f>
         <v/>
       </c>
       <c r="D18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$103,$A18,Matriz!$L$2:$L$103,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$105,$A18,Matriz!$L$2:$L$105,"En diseño")</f>
         <v/>
       </c>
       <c r="E18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$103,$A18,Matriz!$L$2:$L$103,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$105,$A18,Matriz!$L$2:$L$105,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$103,$A18,Matriz!$L$2:$L$103,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$105,$A18,Matriz!$L$2:$L$105,"En pruebas")</f>
         <v/>
       </c>
       <c r="G18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$103,$A18,Matriz!$L$2:$L$103,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$105,$A18,Matriz!$L$2:$L$105,"Hecho")</f>
         <v/>
       </c>
       <c r="H18" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$103,$A18,Matriz!$L$2:$L$103,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$105,$A18,Matriz!$L$2:$L$105,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I18" s="13">
@@ -1373,31 +1373,31 @@
         </is>
       </c>
       <c r="B19" s="12">
-        <f>COUNTIF(Matriz!$H$2:$H$103,$A19)</f>
+        <f>COUNTIF(Matriz!$H$2:$H$105,$A19)</f>
         <v/>
       </c>
       <c r="C19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$103,$A19,Matriz!$L$2:$L$103,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$105,$A19,Matriz!$L$2:$L$105,"Pendiente")</f>
         <v/>
       </c>
       <c r="D19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$103,$A19,Matriz!$L$2:$L$103,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$105,$A19,Matriz!$L$2:$L$105,"En diseño")</f>
         <v/>
       </c>
       <c r="E19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$103,$A19,Matriz!$L$2:$L$103,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$105,$A19,Matriz!$L$2:$L$105,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$103,$A19,Matriz!$L$2:$L$103,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$105,$A19,Matriz!$L$2:$L$105,"En pruebas")</f>
         <v/>
       </c>
       <c r="G19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$103,$A19,Matriz!$L$2:$L$103,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$105,$A19,Matriz!$L$2:$L$105,"Hecho")</f>
         <v/>
       </c>
       <c r="H19" s="12">
-        <f>COUNTIFS(Matriz!$H$2:$H$103,$A19,Matriz!$L$2:$L$103,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$H$2:$H$105,$A19,Matriz!$L$2:$L$105,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I19" s="13">
@@ -1498,31 +1498,31 @@
         </is>
       </c>
       <c r="B24" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$103,$A24)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$105,$A24)</f>
         <v/>
       </c>
       <c r="C24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$103,$A24,Matriz!$L$2:$L$103,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$105,$A24,Matriz!$L$2:$L$105,"Pendiente")</f>
         <v/>
       </c>
       <c r="D24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$103,$A24,Matriz!$L$2:$L$103,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$105,$A24,Matriz!$L$2:$L$105,"En diseño")</f>
         <v/>
       </c>
       <c r="E24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$103,$A24,Matriz!$L$2:$L$103,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$105,$A24,Matriz!$L$2:$L$105,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$103,$A24,Matriz!$L$2:$L$103,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$105,$A24,Matriz!$L$2:$L$105,"En pruebas")</f>
         <v/>
       </c>
       <c r="G24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$103,$A24,Matriz!$L$2:$L$103,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$105,$A24,Matriz!$L$2:$L$105,"Hecho")</f>
         <v/>
       </c>
       <c r="H24" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$103,$A24,Matriz!$L$2:$L$103,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$105,$A24,Matriz!$L$2:$L$105,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I24" s="13">
@@ -1537,31 +1537,31 @@
         </is>
       </c>
       <c r="B25" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$103,$A25)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$105,$A25)</f>
         <v/>
       </c>
       <c r="C25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$103,$A25,Matriz!$L$2:$L$103,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$105,$A25,Matriz!$L$2:$L$105,"Pendiente")</f>
         <v/>
       </c>
       <c r="D25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$103,$A25,Matriz!$L$2:$L$103,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$105,$A25,Matriz!$L$2:$L$105,"En diseño")</f>
         <v/>
       </c>
       <c r="E25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$103,$A25,Matriz!$L$2:$L$103,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$105,$A25,Matriz!$L$2:$L$105,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$103,$A25,Matriz!$L$2:$L$103,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$105,$A25,Matriz!$L$2:$L$105,"En pruebas")</f>
         <v/>
       </c>
       <c r="G25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$103,$A25,Matriz!$L$2:$L$103,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$105,$A25,Matriz!$L$2:$L$105,"Hecho")</f>
         <v/>
       </c>
       <c r="H25" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$103,$A25,Matriz!$L$2:$L$103,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$105,$A25,Matriz!$L$2:$L$105,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I25" s="13">
@@ -1576,31 +1576,31 @@
         </is>
       </c>
       <c r="B26" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$103,$A26)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$105,$A26)</f>
         <v/>
       </c>
       <c r="C26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$103,$A26,Matriz!$L$2:$L$103,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$105,$A26,Matriz!$L$2:$L$105,"Pendiente")</f>
         <v/>
       </c>
       <c r="D26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$103,$A26,Matriz!$L$2:$L$103,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$105,$A26,Matriz!$L$2:$L$105,"En diseño")</f>
         <v/>
       </c>
       <c r="E26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$103,$A26,Matriz!$L$2:$L$103,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$105,$A26,Matriz!$L$2:$L$105,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$103,$A26,Matriz!$L$2:$L$103,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$105,$A26,Matriz!$L$2:$L$105,"En pruebas")</f>
         <v/>
       </c>
       <c r="G26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$103,$A26,Matriz!$L$2:$L$103,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$105,$A26,Matriz!$L$2:$L$105,"Hecho")</f>
         <v/>
       </c>
       <c r="H26" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$103,$A26,Matriz!$L$2:$L$103,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$105,$A26,Matriz!$L$2:$L$105,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I26" s="13">
@@ -1615,31 +1615,31 @@
         </is>
       </c>
       <c r="B27" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$103,$A27)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$105,$A27)</f>
         <v/>
       </c>
       <c r="C27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$103,$A27,Matriz!$L$2:$L$103,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$105,$A27,Matriz!$L$2:$L$105,"Pendiente")</f>
         <v/>
       </c>
       <c r="D27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$103,$A27,Matriz!$L$2:$L$103,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$105,$A27,Matriz!$L$2:$L$105,"En diseño")</f>
         <v/>
       </c>
       <c r="E27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$103,$A27,Matriz!$L$2:$L$103,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$105,$A27,Matriz!$L$2:$L$105,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$103,$A27,Matriz!$L$2:$L$103,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$105,$A27,Matriz!$L$2:$L$105,"En pruebas")</f>
         <v/>
       </c>
       <c r="G27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$103,$A27,Matriz!$L$2:$L$103,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$105,$A27,Matriz!$L$2:$L$105,"Hecho")</f>
         <v/>
       </c>
       <c r="H27" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$103,$A27,Matriz!$L$2:$L$103,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$105,$A27,Matriz!$L$2:$L$105,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I27" s="13">
@@ -1654,31 +1654,31 @@
         </is>
       </c>
       <c r="B28" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$103,$A28)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$105,$A28)</f>
         <v/>
       </c>
       <c r="C28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$103,$A28,Matriz!$L$2:$L$103,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$105,$A28,Matriz!$L$2:$L$105,"Pendiente")</f>
         <v/>
       </c>
       <c r="D28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$103,$A28,Matriz!$L$2:$L$103,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$105,$A28,Matriz!$L$2:$L$105,"En diseño")</f>
         <v/>
       </c>
       <c r="E28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$103,$A28,Matriz!$L$2:$L$103,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$105,$A28,Matriz!$L$2:$L$105,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$103,$A28,Matriz!$L$2:$L$103,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$105,$A28,Matriz!$L$2:$L$105,"En pruebas")</f>
         <v/>
       </c>
       <c r="G28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$103,$A28,Matriz!$L$2:$L$103,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$105,$A28,Matriz!$L$2:$L$105,"Hecho")</f>
         <v/>
       </c>
       <c r="H28" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$103,$A28,Matriz!$L$2:$L$103,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$105,$A28,Matriz!$L$2:$L$105,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I28" s="13">
@@ -1693,31 +1693,31 @@
         </is>
       </c>
       <c r="B29" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$103,$A29)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$105,$A29)</f>
         <v/>
       </c>
       <c r="C29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$103,$A29,Matriz!$L$2:$L$103,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$105,$A29,Matriz!$L$2:$L$105,"Pendiente")</f>
         <v/>
       </c>
       <c r="D29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$103,$A29,Matriz!$L$2:$L$103,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$105,$A29,Matriz!$L$2:$L$105,"En diseño")</f>
         <v/>
       </c>
       <c r="E29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$103,$A29,Matriz!$L$2:$L$103,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$105,$A29,Matriz!$L$2:$L$105,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$103,$A29,Matriz!$L$2:$L$103,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$105,$A29,Matriz!$L$2:$L$105,"En pruebas")</f>
         <v/>
       </c>
       <c r="G29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$103,$A29,Matriz!$L$2:$L$103,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$105,$A29,Matriz!$L$2:$L$105,"Hecho")</f>
         <v/>
       </c>
       <c r="H29" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$103,$A29,Matriz!$L$2:$L$103,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$105,$A29,Matriz!$L$2:$L$105,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I29" s="13">
@@ -1732,31 +1732,31 @@
         </is>
       </c>
       <c r="B30" s="12">
-        <f>COUNTIF(Matriz!$G$2:$G$103,$A30)</f>
+        <f>COUNTIF(Matriz!$G$2:$G$105,$A30)</f>
         <v/>
       </c>
       <c r="C30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$103,$A30,Matriz!$L$2:$L$103,"Pendiente")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$105,$A30,Matriz!$L$2:$L$105,"Pendiente")</f>
         <v/>
       </c>
       <c r="D30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$103,$A30,Matriz!$L$2:$L$103,"En diseño")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$105,$A30,Matriz!$L$2:$L$105,"En diseño")</f>
         <v/>
       </c>
       <c r="E30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$103,$A30,Matriz!$L$2:$L$103,"En desarrollo")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$105,$A30,Matriz!$L$2:$L$105,"En desarrollo")</f>
         <v/>
       </c>
       <c r="F30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$103,$A30,Matriz!$L$2:$L$103,"En pruebas")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$105,$A30,Matriz!$L$2:$L$105,"En pruebas")</f>
         <v/>
       </c>
       <c r="G30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$103,$A30,Matriz!$L$2:$L$103,"Hecho")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$105,$A30,Matriz!$L$2:$L$105,"Hecho")</f>
         <v/>
       </c>
       <c r="H30" s="12">
-        <f>COUNTIFS(Matriz!$G$2:$G$103,$A30,Matriz!$L$2:$L$103,"Bloqueado")</f>
+        <f>COUNTIFS(Matriz!$G$2:$G$105,$A30,Matriz!$L$2:$L$105,"Bloqueado")</f>
         <v/>
       </c>
       <c r="I30" s="13">
@@ -1818,7 +1818,7 @@
         </is>
       </c>
       <c r="B35" s="12">
-        <f>COUNTIF(Matriz!$K$2:$K$103,A35)</f>
+        <f>COUNTIF(Matriz!$K$2:$K$105,A35)</f>
         <v/>
       </c>
     </row>
@@ -1829,7 +1829,7 @@
         </is>
       </c>
       <c r="B36" s="12">
-        <f>COUNTIF(Matriz!$K$2:$K$103,A36)</f>
+        <f>COUNTIF(Matriz!$K$2:$K$105,A36)</f>
         <v/>
       </c>
     </row>
@@ -1840,7 +1840,7 @@
         </is>
       </c>
       <c r="B37" s="12">
-        <f>COUNTIF(Matriz!$K$2:$K$103,A37)</f>
+        <f>COUNTIF(Matriz!$K$2:$K$105,A37)</f>
         <v/>
       </c>
     </row>
@@ -1851,7 +1851,7 @@
         </is>
       </c>
       <c r="B38" s="12">
-        <f>COUNTIF(Matriz!$K$2:$K$103,A38)</f>
+        <f>COUNTIF(Matriz!$K$2:$K$105,A38)</f>
         <v/>
       </c>
     </row>
@@ -1866,7 +1866,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N103"/>
+  <dimension ref="A1:N105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4224,52 +4224,52 @@
     <row r="35">
       <c r="A35" s="18" t="inlineStr">
         <is>
-          <t>M2A-01</t>
+          <t>M1-28</t>
         </is>
       </c>
       <c r="B35" s="19" t="inlineStr">
         <is>
-          <t>M2A Cursos de Vida</t>
+          <t>M1 Identidad y comunicación</t>
         </is>
       </c>
       <c r="C35" s="19" t="inlineStr">
         <is>
-          <t>Catálogo dinámico de cursos; se pueden crear nuevos sin intervención técnica. Incluye «Resolución de Varones» y «Toma de Buenas Decisiones», omitidos en v2.</t>
-        </is>
-      </c>
-      <c r="D35" s="22" t="inlineStr">
-        <is>
-          <t>Recuperado v1</t>
+          <t>Peticiones de oración personales: toda persona con sesión puede pedir oración y ve la sección de oración. Ve las suyas; las ve también la dirección que consulta todas las peticiones, y el equipo de oración si las comparte con él.</t>
+        </is>
+      </c>
+      <c r="D35" s="21" t="inlineStr">
+        <is>
+          <t>Respuesta v3.22</t>
         </is>
       </c>
       <c r="E35" s="19" t="inlineStr">
         <is>
-          <t>Fuera del MVP</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="F35" s="19" t="inlineStr">
         <is>
-          <t>Fase 3</t>
+          <t>Fase 0</t>
         </is>
       </c>
       <c r="G35" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sprint 5</t>
         </is>
       </c>
       <c r="H35" s="19" t="inlineStr">
         <is>
-          <t>Posterior</t>
-        </is>
-      </c>
-      <c r="I35" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
-        </is>
-      </c>
-      <c r="J35" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
+          <t>H2 · Fase 0 completa</t>
+        </is>
+      </c>
+      <c r="I35" s="19" t="inlineStr">
+        <is>
+          <t>Como persona quiero pedir oración desde la aplicación y ver mis peticiones.</t>
+        </is>
+      </c>
+      <c r="J35" s="19" t="inlineStr">
+        <is>
+          <t>Cualquier cuenta registra una petición personal y la ve; otra cuenta no; el equipo de oración solo lee las compartidas con él.</t>
         </is>
       </c>
       <c r="K35" s="19" t="inlineStr">
@@ -4279,61 +4279,69 @@
       </c>
       <c r="L35" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M35" s="19" t="inlineStr"/>
-      <c r="N35" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M35" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/paso-9-oraciones-vehiculos · pruebas de backend y 110 de frontend pasan; lint, estilos y compilación limpios</t>
+        </is>
+      </c>
+      <c r="N35" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-30 · Origen de peticiones personales para toda cuenta.</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="18" t="inlineStr">
         <is>
-          <t>M2A-02</t>
+          <t>M1-29</t>
         </is>
       </c>
       <c r="B36" s="19" t="inlineStr">
         <is>
-          <t>M2A Cursos de Vida</t>
+          <t>M1 Identidad y comunicación</t>
         </is>
       </c>
       <c r="C36" s="19" t="inlineStr">
         <is>
-          <t>Flexibilidad operativa: sin día ni horario fijo; el día y el ponente pueden cambiar entre ediciones.</t>
-        </is>
-      </c>
-      <c r="D36" s="19" t="inlineStr">
-        <is>
-          <t>v1 / v2</t>
+          <t>Bienes ligados (vehículos): cada persona registra, corrige y quita sus vehículos (tipo, marca, modelo, año, color y placas) desde Mi cuenta. Quien consulta expedientes los ve en la ficha, sin poder cambiarlos.</t>
+        </is>
+      </c>
+      <c r="D36" s="21" t="inlineStr">
+        <is>
+          <t>Respuesta v3.22</t>
         </is>
       </c>
       <c r="E36" s="19" t="inlineStr">
         <is>
-          <t>Fuera del MVP</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="F36" s="19" t="inlineStr">
         <is>
-          <t>Fase 3</t>
+          <t>Fase 0</t>
         </is>
       </c>
       <c r="G36" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sprint 5</t>
         </is>
       </c>
       <c r="H36" s="19" t="inlineStr">
         <is>
-          <t>Posterior</t>
-        </is>
-      </c>
-      <c r="I36" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
-        </is>
-      </c>
-      <c r="J36" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
+          <t>H2 · Fase 0 completa</t>
+        </is>
+      </c>
+      <c r="I36" s="19" t="inlineStr">
+        <is>
+          <t>Como persona quiero registrar mis vehículos para que la iglesia los conozca.</t>
+        </is>
+      </c>
+      <c r="J36" s="19" t="inlineStr">
+        <is>
+          <t>Agregar, editar y quitar un vehículo propio; no se puede tocar el de otra persona; queda en la bitácora.</t>
         </is>
       </c>
       <c r="K36" s="19" t="inlineStr">
@@ -4343,16 +4351,24 @@
       </c>
       <c r="L36" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M36" s="19" t="inlineStr"/>
-      <c r="N36" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M36" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/paso-9-oraciones-vehiculos · pruebas de backend y 110 de frontend pasan; lint, estilos y compilación limpios</t>
+        </is>
+      </c>
+      <c r="N36" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-30 · Vehículos propios en Mi cuenta y consulta en la ficha.</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="18" t="inlineStr">
         <is>
-          <t>M2A-03</t>
+          <t>M2A-01</t>
         </is>
       </c>
       <c r="B37" s="19" t="inlineStr">
@@ -4362,12 +4378,12 @@
       </c>
       <c r="C37" s="19" t="inlineStr">
         <is>
-          <t>Reposición de clases: el inscrito puede reponer en otro grupo o con otro ponente, a decisión de quien imparte.</t>
-        </is>
-      </c>
-      <c r="D37" s="19" t="inlineStr">
-        <is>
-          <t>v1 / v2</t>
+          <t>Catálogo dinámico de cursos; se pueden crear nuevos sin intervención técnica. Incluye «Resolución de Varones» y «Toma de Buenas Decisiones», omitidos en v2.</t>
+        </is>
+      </c>
+      <c r="D37" s="22" t="inlineStr">
+        <is>
+          <t>Recuperado v1</t>
         </is>
       </c>
       <c r="E37" s="19" t="inlineStr">
@@ -4416,7 +4432,7 @@
     <row r="38">
       <c r="A38" s="18" t="inlineStr">
         <is>
-          <t>M2A-04</t>
+          <t>M2A-02</t>
         </is>
       </c>
       <c r="B38" s="19" t="inlineStr">
@@ -4426,7 +4442,7 @@
       </c>
       <c r="C38" s="19" t="inlineStr">
         <is>
-          <t>Registro de asistencia por sesión.</t>
+          <t>Flexibilidad operativa: sin día ni horario fijo; el día y el ponente pueden cambiar entre ediciones.</t>
         </is>
       </c>
       <c r="D38" s="19" t="inlineStr">
@@ -4480,7 +4496,7 @@
     <row r="39">
       <c r="A39" s="18" t="inlineStr">
         <is>
-          <t>M2A-05</t>
+          <t>M2A-03</t>
         </is>
       </c>
       <c r="B39" s="19" t="inlineStr">
@@ -4490,7 +4506,7 @@
       </c>
       <c r="C39" s="19" t="inlineStr">
         <is>
-          <t>Seguimiento de tareas o actividades opcionales (no sumativas).</t>
+          <t>Reposición de clases: el inscrito puede reponer en otro grupo o con otro ponente, a decisión de quien imparte.</t>
         </is>
       </c>
       <c r="D39" s="19" t="inlineStr">
@@ -4544,7 +4560,7 @@
     <row r="40">
       <c r="A40" s="18" t="inlineStr">
         <is>
-          <t>M2A-06</t>
+          <t>M2A-04</t>
         </is>
       </c>
       <c r="B40" s="19" t="inlineStr">
@@ -4554,7 +4570,7 @@
       </c>
       <c r="C40" s="19" t="inlineStr">
         <is>
-          <t>Inscripción: quién se inscribe, cuándo lo hizo, si tiene adeudo y qué incluye el costo (materiales, hospedaje, etc.).</t>
+          <t>Registro de asistencia por sesión.</t>
         </is>
       </c>
       <c r="D40" s="19" t="inlineStr">
@@ -4608,7 +4624,7 @@
     <row r="41">
       <c r="A41" s="18" t="inlineStr">
         <is>
-          <t>M2A-07</t>
+          <t>M2A-05</t>
         </is>
       </c>
       <c r="B41" s="19" t="inlineStr">
@@ -4618,12 +4634,12 @@
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>Registro de pagos, saldo de adeudos y recibo. Por definir: captura manual vs. pasarela de pago, y si se requiere corte de caja.</t>
-        </is>
-      </c>
-      <c r="D41" s="21" t="inlineStr">
-        <is>
-          <t>Nuevo v3</t>
+          <t>Seguimiento de tareas o actividades opcionales (no sumativas).</t>
+        </is>
+      </c>
+      <c r="D41" s="19" t="inlineStr">
+        <is>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E41" s="19" t="inlineStr">
@@ -4658,7 +4674,7 @@
       </c>
       <c r="K41" s="19" t="inlineStr">
         <is>
-          <t>Por definir</t>
+          <t>VoBo pendiente</t>
         </is>
       </c>
       <c r="L41" s="19" t="inlineStr">
@@ -4672,7 +4688,7 @@
     <row r="42">
       <c r="A42" s="18" t="inlineStr">
         <is>
-          <t>M2A-08</t>
+          <t>M2A-06</t>
         </is>
       </c>
       <c r="B42" s="19" t="inlineStr">
@@ -4682,12 +4698,12 @@
       </c>
       <c r="C42" s="19" t="inlineStr">
         <is>
-          <t>Tablero del curso tipo mensajería para avisos antes del curso y días posteriores, con notificación a los inscritos.</t>
-        </is>
-      </c>
-      <c r="D42" s="22" t="inlineStr">
-        <is>
-          <t>Recuperado v1</t>
+          <t>Inscripción: quién se inscribe, cuándo lo hizo, si tiene adeudo y qué incluye el costo (materiales, hospedaje, etc.).</t>
+        </is>
+      </c>
+      <c r="D42" s="19" t="inlineStr">
+        <is>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E42" s="19" t="inlineStr">
@@ -4736,7 +4752,7 @@
     <row r="43">
       <c r="A43" s="18" t="inlineStr">
         <is>
-          <t>M2A-09</t>
+          <t>M2A-07</t>
         </is>
       </c>
       <c r="B43" s="19" t="inlineStr">
@@ -4746,12 +4762,12 @@
       </c>
       <c r="C43" s="19" t="inlineStr">
         <is>
-          <t>Evaluación docente configurable: formulario diseñable (tipo Google Forms) aplicado al finalizar el curso.</t>
-        </is>
-      </c>
-      <c r="D43" s="19" t="inlineStr">
-        <is>
-          <t>v1 / v2</t>
+          <t>Registro de pagos, saldo de adeudos y recibo. Por definir: captura manual vs. pasarela de pago, y si se requiere corte de caja.</t>
+        </is>
+      </c>
+      <c r="D43" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3</t>
         </is>
       </c>
       <c r="E43" s="19" t="inlineStr">
@@ -4786,7 +4802,7 @@
       </c>
       <c r="K43" s="19" t="inlineStr">
         <is>
-          <t>VoBo pendiente</t>
+          <t>Por definir</t>
         </is>
       </c>
       <c r="L43" s="19" t="inlineStr">
@@ -4800,7 +4816,7 @@
     <row r="44">
       <c r="A44" s="18" t="inlineStr">
         <is>
-          <t>M2A-10</t>
+          <t>M2A-08</t>
         </is>
       </c>
       <c r="B44" s="19" t="inlineStr">
@@ -4810,7 +4826,7 @@
       </c>
       <c r="C44" s="19" t="inlineStr">
         <is>
-          <t>Evolución del ponente: historial de evaluaciones por ponente a lo largo del tiempo y entre ediciones.</t>
+          <t>Tablero del curso tipo mensajería para avisos antes del curso y días posteriores, con notificación a los inscritos.</t>
         </is>
       </c>
       <c r="D44" s="22" t="inlineStr">
@@ -4864,7 +4880,7 @@
     <row r="45">
       <c r="A45" s="18" t="inlineStr">
         <is>
-          <t>M2A-11</t>
+          <t>M2A-09</t>
         </is>
       </c>
       <c r="B45" s="19" t="inlineStr">
@@ -4874,7 +4890,7 @@
       </c>
       <c r="C45" s="19" t="inlineStr">
         <is>
-          <t>Reconocimiento de participación (diploma) opcional por curso.</t>
+          <t>Evaluación docente configurable: formulario diseñable (tipo Google Forms) aplicado al finalizar el curso.</t>
         </is>
       </c>
       <c r="D45" s="19" t="inlineStr">
@@ -4928,22 +4944,22 @@
     <row r="46">
       <c r="A46" s="18" t="inlineStr">
         <is>
-          <t>M2B-01</t>
+          <t>M2A-10</t>
         </is>
       </c>
       <c r="B46" s="19" t="inlineStr">
         <is>
-          <t>M2B Cursos escolarizados</t>
+          <t>M2A Cursos de Vida</t>
         </is>
       </c>
       <c r="C46" s="19" t="inlineStr">
         <is>
-          <t>Control riguroso de asistencia.</t>
-        </is>
-      </c>
-      <c r="D46" s="19" t="inlineStr">
-        <is>
-          <t>v1 / v2</t>
+          <t>Evolución del ponente: historial de evaluaciones por ponente a lo largo del tiempo y entre ediciones.</t>
+        </is>
+      </c>
+      <c r="D46" s="22" t="inlineStr">
+        <is>
+          <t>Recuperado v1</t>
         </is>
       </c>
       <c r="E46" s="19" t="inlineStr">
@@ -4992,17 +5008,17 @@
     <row r="47">
       <c r="A47" s="18" t="inlineStr">
         <is>
-          <t>M2B-02</t>
+          <t>M2A-11</t>
         </is>
       </c>
       <c r="B47" s="19" t="inlineStr">
         <is>
-          <t>M2B Cursos escolarizados</t>
+          <t>M2A Cursos de Vida</t>
         </is>
       </c>
       <c r="C47" s="19" t="inlineStr">
         <is>
-          <t>Entrega de tareas y trabajos continuos (incluidos trabajos extra).</t>
+          <t>Reconocimiento de participación (diploma) opcional por curso.</t>
         </is>
       </c>
       <c r="D47" s="19" t="inlineStr">
@@ -5056,7 +5072,7 @@
     <row r="48">
       <c r="A48" s="18" t="inlineStr">
         <is>
-          <t>M2B-03</t>
+          <t>M2B-01</t>
         </is>
       </c>
       <c r="B48" s="19" t="inlineStr">
@@ -5066,7 +5082,7 @@
       </c>
       <c r="C48" s="19" t="inlineStr">
         <is>
-          <t>Ponderación de calificaciones y exámenes finales.</t>
+          <t>Control riguroso de asistencia.</t>
         </is>
       </c>
       <c r="D48" s="19" t="inlineStr">
@@ -5120,7 +5136,7 @@
     <row r="49">
       <c r="A49" s="18" t="inlineStr">
         <is>
-          <t>M2B-04</t>
+          <t>M2B-02</t>
         </is>
       </c>
       <c r="B49" s="19" t="inlineStr">
@@ -5130,12 +5146,12 @@
       </c>
       <c r="C49" s="19" t="inlineStr">
         <is>
-          <t>Creador de exámenes en línea: opción múltiple, preguntas abiertas, falso/verdadero y respuesta corta.</t>
+          <t>Entrega de tareas y trabajos continuos (incluidos trabajos extra).</t>
         </is>
       </c>
       <c r="D49" s="19" t="inlineStr">
         <is>
-          <t>v2</t>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E49" s="19" t="inlineStr">
@@ -5184,7 +5200,7 @@
     <row r="50">
       <c r="A50" s="18" t="inlineStr">
         <is>
-          <t>M2B-05</t>
+          <t>M2B-03</t>
         </is>
       </c>
       <c r="B50" s="19" t="inlineStr">
@@ -5194,7 +5210,7 @@
       </c>
       <c r="C50" s="19" t="inlineStr">
         <is>
-          <t>Boleta digital con el formato definido por la iglesia. Por definir: formato oficial de la boleta.</t>
+          <t>Ponderación de calificaciones y exámenes finales.</t>
         </is>
       </c>
       <c r="D50" s="19" t="inlineStr">
@@ -5234,7 +5250,7 @@
       </c>
       <c r="K50" s="19" t="inlineStr">
         <is>
-          <t>Por definir</t>
+          <t>VoBo pendiente</t>
         </is>
       </c>
       <c r="L50" s="19" t="inlineStr">
@@ -5248,7 +5264,7 @@
     <row r="51">
       <c r="A51" s="18" t="inlineStr">
         <is>
-          <t>M2B-06</t>
+          <t>M2B-04</t>
         </is>
       </c>
       <c r="B51" s="19" t="inlineStr">
@@ -5258,7 +5274,7 @@
       </c>
       <c r="C51" s="19" t="inlineStr">
         <is>
-          <t>Historial académico permanente en el Expediente Digital, aunque cambie el maestro o el alumno pierda su comprobante.</t>
+          <t>Creador de exámenes en línea: opción múltiple, preguntas abiertas, falso/verdadero y respuesta corta.</t>
         </is>
       </c>
       <c r="D51" s="19" t="inlineStr">
@@ -5312,124 +5328,116 @@
     <row r="52">
       <c r="A52" s="18" t="inlineStr">
         <is>
-          <t>M3-01</t>
+          <t>M2B-05</t>
         </is>
       </c>
       <c r="B52" s="19" t="inlineStr">
         <is>
-          <t>M3 Grupos de Conexión</t>
+          <t>M2B Cursos escolarizados</t>
         </is>
       </c>
       <c r="C52" s="19" t="inlineStr">
         <is>
-          <t>Estructura del grupo con roles: Supervisor (supervisa uno o varios grupos y reporta al Pastor), Líder, Secretario, Anfitrión y Tesorero.</t>
+          <t>Boleta digital con el formato definido por la iglesia. Por definir: formato oficial de la boleta.</t>
         </is>
       </c>
       <c r="D52" s="19" t="inlineStr">
         <is>
-          <t>v3 + Obs. 4</t>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E52" s="19" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Fuera del MVP</t>
         </is>
       </c>
       <c r="F52" s="19" t="inlineStr">
         <is>
-          <t>Fase 1</t>
+          <t>Fase 3</t>
         </is>
       </c>
       <c r="G52" s="19" t="inlineStr">
         <is>
-          <t>Sprint 3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H52" s="19" t="inlineStr">
         <is>
-          <t>H3 · MVP (Grupos)</t>
-        </is>
-      </c>
-      <c r="I52" s="19" t="inlineStr">
-        <is>
-          <t>Como supervisor quiero asignar Líder, Secretario, Anfitrión y Tesorero a cada grupo.</t>
-        </is>
-      </c>
-      <c r="J52" s="19" t="inlineStr">
-        <is>
-          <t>Un grupo tiene sus roles asignados; un supervisor ve varios grupos.</t>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="I52" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
+        </is>
+      </c>
+      <c r="J52" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
         </is>
       </c>
       <c r="K52" s="19" t="inlineStr">
         <is>
-          <t>VoBo pendiente</t>
+          <t>Por definir</t>
         </is>
       </c>
       <c r="L52" s="19" t="inlineStr">
         <is>
-          <t>En pruebas</t>
-        </is>
-      </c>
-      <c r="M52" s="19" t="inlineStr">
-        <is>
-          <t>Rama feature/grupos-paso-3 · pruebas de backend y 81 de frontend pasan; lint, estilos y compilación limpios</t>
-        </is>
-      </c>
-      <c r="N52" s="19" t="inlineStr">
-        <is>
-          <t>2026-10-27 · Supervisor, Líder, Secretario, Anfitrión, Tesorero y Asistente por grupo; ahora con cambio de rol, sector (letra), casa (número) y suspensión con motivo.</t>
-        </is>
-      </c>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M52" s="19" t="inlineStr"/>
+      <c r="N52" s="19" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="18" t="inlineStr">
         <is>
-          <t>M3-02</t>
+          <t>M2B-06</t>
         </is>
       </c>
       <c r="B53" s="19" t="inlineStr">
         <is>
-          <t>M3 Grupos de Conexión</t>
+          <t>M2B Cursos escolarizados</t>
         </is>
       </c>
       <c r="C53" s="19" t="inlineStr">
         <is>
-          <t>Estudio semanal dentro de la app: un registro por semana con PDF para adultos, PDF para niños y audio de la lectura (PDF hasta 15 MB; audio hasta 40 MB). Lo publican Pastor o Anciano y los líderes lo abren desde la reunión, sustituyendo el envío por WhatsApp. El audio admite adelantar y retroceder en iPhone.</t>
+          <t>Historial académico permanente en el Expediente Digital, aunque cambie el maestro o el alumno pierda su comprobante.</t>
         </is>
       </c>
       <c r="D53" s="19" t="inlineStr">
         <is>
-          <t>v1 / v2 + Respuesta</t>
+          <t>v2</t>
         </is>
       </c>
       <c r="E53" s="19" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Fuera del MVP</t>
         </is>
       </c>
       <c r="F53" s="19" t="inlineStr">
         <is>
-          <t>Fase 1</t>
+          <t>Fase 3</t>
         </is>
       </c>
       <c r="G53" s="19" t="inlineStr">
         <is>
-          <t>Sprint 3</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H53" s="19" t="inlineStr">
         <is>
-          <t>H3 · MVP (Grupos)</t>
-        </is>
-      </c>
-      <c r="I53" s="19" t="inlineStr">
-        <is>
-          <t>Como líder quiero recibir el estudio semanal en la app en lugar de WhatsApp.</t>
-        </is>
-      </c>
-      <c r="J53" s="19" t="inlineStr">
-        <is>
-          <t>Publicar el material de la semana; el líder lo abre y queda marca de lectura.</t>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="I53" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
+        </is>
+      </c>
+      <c r="J53" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
         </is>
       </c>
       <c r="K53" s="19" t="inlineStr">
@@ -5439,24 +5447,16 @@
       </c>
       <c r="L53" s="19" t="inlineStr">
         <is>
-          <t>En pruebas</t>
-        </is>
-      </c>
-      <c r="M53" s="19" t="inlineStr">
-        <is>
-          <t>Rama feature/m3-grupos · 88 pruebas de backend y 7 de frontend pasan</t>
-        </is>
-      </c>
-      <c r="N53" s="19" t="inlineStr">
-        <is>
-          <t>2026-10-24 · PDF adultos, PDF niños y audio por semana; audio con Range para iPhone. Pendiente probar en iOS.</t>
-        </is>
-      </c>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M53" s="19" t="inlineStr"/>
+      <c r="N53" s="19" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="18" t="inlineStr">
         <is>
-          <t>M3-03</t>
+          <t>M3-01</t>
         </is>
       </c>
       <c r="B54" s="19" t="inlineStr">
@@ -5466,12 +5466,12 @@
       </c>
       <c r="C54" s="19" t="inlineStr">
         <is>
-          <t>Pase de lista digital por Secretario o Líder. El Secretario captura y corrige el mismo día; el Líder modifica siempre; el Supervisor solo consulta. Funciona sin conexión: la lista se guarda en el teléfono con la hora real de captura y se envía sola al volver la señal, sin pisar cambios más recientes hechos en línea. Una captura sin conexión se acepta hasta 7 días después y se evalúa contra el día en que se hizo; todo queda en bitácora marcado como diferido.</t>
+          <t>Estructura del grupo con roles: Supervisor (supervisa uno o varios grupos y reporta al Pastor), Líder, Secretario, Anfitrión y Tesorero.</t>
         </is>
       </c>
       <c r="D54" s="19" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>v3 + Obs. 4</t>
         </is>
       </c>
       <c r="E54" s="19" t="inlineStr">
@@ -5496,12 +5496,12 @@
       </c>
       <c r="I54" s="19" t="inlineStr">
         <is>
-          <t>Como secretario quiero pasar lista aunque no haya señal.</t>
+          <t>Como supervisor quiero asignar Líder, Secretario, Anfitrión y Tesorero a cada grupo.</t>
         </is>
       </c>
       <c r="J54" s="19" t="inlineStr">
         <is>
-          <t>Pasar lista en modo avión; al reconectar se sincroniza sin duplicados.</t>
+          <t>Un grupo tiene sus roles asignados; un supervisor ve varios grupos.</t>
         </is>
       </c>
       <c r="K54" s="19" t="inlineStr">
@@ -5516,19 +5516,19 @@
       </c>
       <c r="M54" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/nf-06-sin-conexion · 117 pruebas de backend y 27 de frontend; probado en Chrome real con service worker</t>
+          <t>Rama feature/grupos-paso-3 · pruebas de backend y 81 de frontend pasan; lint, estilos y compilación limpios</t>
         </is>
       </c>
       <c r="N54" s="19" t="inlineStr">
         <is>
-          <t>2026-10-24 · Pase de lista con y sin conexión.</t>
+          <t>2026-10-27 · Supervisor, Líder, Secretario, Anfitrión, Tesorero y Asistente por grupo; ahora con cambio de rol, sector (letra), casa (número) y suspensión con motivo.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="18" t="inlineStr">
         <is>
-          <t>M3-04</t>
+          <t>M3-02</t>
         </is>
       </c>
       <c r="B55" s="19" t="inlineStr">
@@ -5538,12 +5538,12 @@
       </c>
       <c r="C55" s="19" t="inlineStr">
         <is>
-          <t>Ofrendas regulares y especiales (con concepto) por reunión, cuantificables. El Secretario captura el monto; si el grupo no tiene Secretario, lo suple el Líder. El Tesorero cuenta, escribe su cifra y avala volviendo a escribir su PIN; si el grupo no tiene Tesorero, avalan el Líder o el Pastor, nunca quien capturó. Si la cifra coincide queda «Avalada»; si no, se registra la diferencia y queda «Con diferencia», con aviso visible en el grupo, la reunión y la pantalla del Tesorero para quien pueda consultar. Una ofrenda ya capturada solo se corrige con motivo y vuelve a pendiente para un nuevo aval. El Pastor consulta todo, el Líder y el Supervisor consultan y el Anciano no ve finanzas. Toda suplencia, captura, aval y corrección queda en bitácora.</t>
+          <t>Estudio semanal dentro de la app: un registro por semana con PDF para adultos, PDF para niños y audio de la lectura (PDF hasta 15 MB; audio hasta 40 MB). Lo publican Pastor o Anciano y los líderes lo abren desde la reunión, sustituyendo el envío por WhatsApp. El audio admite adelantar y retroceder en iPhone.</t>
         </is>
       </c>
       <c r="D55" s="19" t="inlineStr">
         <is>
-          <t>v3 + Obs. 4</t>
+          <t>v1 / v2 + Respuesta</t>
         </is>
       </c>
       <c r="E55" s="19" t="inlineStr">
@@ -5558,7 +5558,7 @@
       </c>
       <c r="G55" s="19" t="inlineStr">
         <is>
-          <t>Sprint 4</t>
+          <t>Sprint 3</t>
         </is>
       </c>
       <c r="H55" s="19" t="inlineStr">
@@ -5568,12 +5568,12 @@
       </c>
       <c r="I55" s="19" t="inlineStr">
         <is>
-          <t>Como tesorero quiero contar y avalar la ofrenda del grupo.</t>
+          <t>Como líder quiero recibir el estudio semanal en la app en lugar de WhatsApp.</t>
         </is>
       </c>
       <c r="J55" s="19" t="inlineStr">
         <is>
-          <t>Capturar monto; el Tesorero captura su cifra y confirma con su PIN; si difiere se registra la diferencia; con aval no se edita sin motivo.</t>
+          <t>Publicar el material de la semana; el líder lo abre y queda marca de lectura.</t>
         </is>
       </c>
       <c r="K55" s="19" t="inlineStr">
@@ -5588,19 +5588,19 @@
       </c>
       <c r="M55" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/m3-ofrendas-ajustes · 121 pruebas de backend y 14 de frontend pasan</t>
+          <t>Rama feature/m3-grupos · 88 pruebas de backend y 7 de frontend pasan</t>
         </is>
       </c>
       <c r="N55" s="19" t="inlineStr">
         <is>
-          <t>2026-10-24 · Con suplencias del Líder, diferencias visibles y límites configurables. Falta validar con la iglesia.</t>
+          <t>2026-10-24 · PDF adultos, PDF niños y audio por semana; audio con Range para iPhone. Pendiente probar en iOS.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="18" t="inlineStr">
         <is>
-          <t>M3-05</t>
+          <t>M3-03</t>
         </is>
       </c>
       <c r="B56" s="19" t="inlineStr">
@@ -5610,7 +5610,7 @@
       </c>
       <c r="C56" s="19" t="inlineStr">
         <is>
-          <t>Peticiones de oración con formulario configurable (campos que se agregan, desactivan y reordenan sin programar; cada cambio crea una versión y los campos no se borran). Por defecto: petición, quién la pide y categoría. Las registran el Líder y el Secretario, desde la reunión o desde el grupo; el Pastor también.</t>
+          <t>Pase de lista digital por Secretario o Líder. El Secretario captura y corrige el mismo día; el Líder modifica siempre; el Supervisor solo consulta. Funciona sin conexión: la lista se guarda en el teléfono con la hora real de captura y se envía sola al volver la señal, sin pisar cambios más recientes hechos en línea. Una captura sin conexión se acepta hasta 7 días después y se evalúa contra el día en que se hizo; todo queda en bitácora marcado como diferido.</t>
         </is>
       </c>
       <c r="D56" s="19" t="inlineStr">
@@ -5630,7 +5630,7 @@
       </c>
       <c r="G56" s="19" t="inlineStr">
         <is>
-          <t>Sprint 4</t>
+          <t>Sprint 3</t>
         </is>
       </c>
       <c r="H56" s="19" t="inlineStr">
@@ -5640,12 +5640,12 @@
       </c>
       <c r="I56" s="19" t="inlineStr">
         <is>
-          <t>Como líder quiero recoger peticiones de oración con un formulario configurable.</t>
+          <t>Como secretario quiero pasar lista aunque no haya señal.</t>
         </is>
       </c>
       <c r="J56" s="19" t="inlineStr">
         <is>
-          <t>Capturar una petición; el formulario se edita sin código.</t>
+          <t>Pasar lista en modo avión; al reconectar se sincroniza sin duplicados.</t>
         </is>
       </c>
       <c r="K56" s="19" t="inlineStr">
@@ -5660,19 +5660,19 @@
       </c>
       <c r="M56" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/m3-peticiones-oracion · 166 pruebas de backend y 32 de frontend pasan; probado contra la base real</t>
+          <t>Rama feature/nf-06-sin-conexion · 117 pruebas de backend y 27 de frontend; probado en Chrome real con service worker</t>
         </is>
       </c>
       <c r="N56" s="19" t="inlineStr">
         <is>
-          <t>2026-10-24 · Formulario configurable y versionado; captura desde la reunión y el grupo.</t>
+          <t>2026-10-24 · Pase de lista con y sin conexión.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="18" t="inlineStr">
         <is>
-          <t>M3-06</t>
+          <t>M3-04</t>
         </is>
       </c>
       <c r="B57" s="19" t="inlineStr">
@@ -5682,12 +5682,12 @@
       </c>
       <c r="C57" s="19" t="inlineStr">
         <is>
-          <t>Alcance de lectura de cada petición, elegido por quien la registra con autorización de quien la pide: «Solo líderes» (Líder, Supervisor, Pastor y Anciano), «Mi grupo» (todos los integrantes del grupo y los anteriores) o «Equipo de oración» (además, quien tenga el rol Equipo de oración). El alcance por defecto es configurable. Quien registra siempre ve lo que registró; el Administrador Técnico nunca ve el contenido. Solo líderes y superiores marcan una petición como atendida. Se guardan cifradas y se borran automáticamente a los 30 días, configurable. Consultarlas y atenderlas queda en bitácora sin incluir el texto.</t>
-        </is>
-      </c>
-      <c r="D57" s="21" t="inlineStr">
-        <is>
-          <t>Resp. P8 + Respuesta</t>
+          <t>Ofrendas regulares y especiales (con concepto) por reunión, cuantificables. El Secretario captura el monto; si el grupo no tiene Secretario, lo suple el Líder. El Tesorero cuenta, escribe su cifra y avala volviendo a escribir su PIN; si el grupo no tiene Tesorero, avalan el Líder o el Pastor, nunca quien capturó. Si la cifra coincide queda «Avalada»; si no, se registra la diferencia y queda «Con diferencia», con aviso visible en el grupo, la reunión y la pantalla del Tesorero para quien pueda consultar. Una ofrenda ya capturada solo se corrige con motivo y vuelve a pendiente para un nuevo aval. El Pastor consulta todo, el Líder y el Supervisor consultan y el Anciano no ve finanzas. Toda suplencia, captura, aval y corrección queda en bitácora.</t>
+        </is>
+      </c>
+      <c r="D57" s="19" t="inlineStr">
+        <is>
+          <t>v3 + Obs. 4</t>
         </is>
       </c>
       <c r="E57" s="19" t="inlineStr">
@@ -5712,12 +5712,12 @@
       </c>
       <c r="I57" s="19" t="inlineStr">
         <is>
-          <t>Como pastor quiero que las peticiones solo las vea el Líder y superiores y se borren al vencer.</t>
+          <t>Como tesorero quiero contar y avalar la ofrenda del grupo.</t>
         </is>
       </c>
       <c r="J57" s="19" t="inlineStr">
         <is>
-          <t>El Secretario no las ve; tras el plazo configurable (por defecto 30 días) se eliminan.</t>
+          <t>Capturar monto; el Tesorero captura su cifra y confirma con su PIN; si difiere se registra la diferencia; con aval no se edita sin motivo.</t>
         </is>
       </c>
       <c r="K57" s="19" t="inlineStr">
@@ -5732,19 +5732,19 @@
       </c>
       <c r="M57" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/m3-peticiones-oracion · 166 pruebas de backend y 32 de frontend pasan; probado contra la base real</t>
+          <t>Rama feature/m3-ofrendas-ajustes · 121 pruebas de backend y 14 de frontend pasan</t>
         </is>
       </c>
       <c r="N57" s="19" t="inlineStr">
         <is>
-          <t>2026-10-24 · Alcance por petición (líderes, grupo, equipo), cifrado y borrado a los 30 días configurable. Cambia la matriz aprobada: actualizar con la iglesia.</t>
+          <t>2026-10-24 · Con suplencias del Líder, diferencias visibles y límites configurables. Falta validar con la iglesia.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="18" t="inlineStr">
         <is>
-          <t>M3-07</t>
+          <t>M3-05</t>
         </is>
       </c>
       <c r="B58" s="19" t="inlineStr">
@@ -5754,7 +5754,7 @@
       </c>
       <c r="C58" s="19" t="inlineStr">
         <is>
-          <t>Dashboard de supervisión («Resumen de grupos») para Supervisor, Líder, Pastor y Anciano sobre los grupos que cada uno puede consultar: asistencia por semana y por grupo, grupos sin lista esta semana, asistencia por debajo de un mínimo configurable (60 % por defecto), ofrendas avaladas, pendientes y con diferencia (solo si el rol ve finanzas) y peticiones activas (solo las que puede leer). No muestra datos de personas. El Secretario y el Tesorero no lo ven.</t>
+          <t>Peticiones de oración con formulario configurable (campos que se agregan, desactivan y reordenan sin programar; cada cambio crea una versión y los campos no se borran). Por defecto: petición, quién la pide y categoría. Las registran el Líder y el Secretario, desde la reunión o desde el grupo; el Pastor también.</t>
         </is>
       </c>
       <c r="D58" s="19" t="inlineStr">
@@ -5764,7 +5764,7 @@
       </c>
       <c r="E58" s="19" t="inlineStr">
         <is>
-          <t>MVP básico</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="F58" s="19" t="inlineStr">
@@ -5774,7 +5774,7 @@
       </c>
       <c r="G58" s="19" t="inlineStr">
         <is>
-          <t>Sprint 5</t>
+          <t>Sprint 4</t>
         </is>
       </c>
       <c r="H58" s="19" t="inlineStr">
@@ -5784,12 +5784,12 @@
       </c>
       <c r="I58" s="19" t="inlineStr">
         <is>
-          <t>Como supervisor quiero ver la salud de mis grupos.</t>
+          <t>Como líder quiero recoger peticiones de oración con un formulario configurable.</t>
         </is>
       </c>
       <c r="J58" s="19" t="inlineStr">
         <is>
-          <t>El dashboard muestra asistencia, ofrendas y crecimiento según permisos.</t>
+          <t>Capturar una petición; el formulario se edita sin código.</t>
         </is>
       </c>
       <c r="K58" s="19" t="inlineStr">
@@ -5804,19 +5804,19 @@
       </c>
       <c r="M58" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/m3-dashboard-tablero · 195 pruebas de backend y 39 de frontend pasan; probado contra la base real</t>
+          <t>Rama feature/m3-peticiones-oracion · 166 pruebas de backend y 32 de frontend pasan; probado contra la base real</t>
         </is>
       </c>
       <c r="N58" s="19" t="inlineStr">
         <is>
-          <t>2026-10-25 · Dashboard con asistencia, avisos y datos según rol; umbral configurable.</t>
+          <t>2026-10-24 · Formulario configurable y versionado; captura desde la reunión y el grupo.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="18" t="inlineStr">
         <is>
-          <t>M3-08</t>
+          <t>M3-06</t>
         </is>
       </c>
       <c r="B59" s="19" t="inlineStr">
@@ -5826,61 +5826,69 @@
       </c>
       <c r="C59" s="19" t="inlineStr">
         <is>
-          <t>Ubicación de zona del grupo para que personas cercanas lo encuentren, sin exponer el domicilio exacto. Por definir.</t>
-        </is>
-      </c>
-      <c r="D59" s="19" t="inlineStr">
-        <is>
-          <t>v3</t>
+          <t>Alcance de lectura de cada petición, elegido por quien la registra con autorización de quien la pide: «Solo líderes» (Líder, Supervisor, Pastor y Anciano), «Mi grupo» (todos los integrantes del grupo y los anteriores) o «Equipo de oración» (además, quien tenga el rol Equipo de oración). El alcance por defecto es configurable. Quien registra siempre ve lo que registró; el Administrador Técnico nunca ve el contenido. Solo líderes y superiores marcan una petición como atendida. Se guardan cifradas y se borran automáticamente a los 30 días, configurable. Consultarlas y atenderlas queda en bitácora sin incluir el texto.</t>
+        </is>
+      </c>
+      <c r="D59" s="21" t="inlineStr">
+        <is>
+          <t>Resp. P8 + Respuesta</t>
         </is>
       </c>
       <c r="E59" s="19" t="inlineStr">
         <is>
-          <t>Fuera del MVP</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="F59" s="19" t="inlineStr">
         <is>
-          <t>Fase 4</t>
+          <t>Fase 1</t>
         </is>
       </c>
       <c r="G59" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sprint 4</t>
         </is>
       </c>
       <c r="H59" s="19" t="inlineStr">
         <is>
-          <t>Posterior</t>
-        </is>
-      </c>
-      <c r="I59" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
-        </is>
-      </c>
-      <c r="J59" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
+          <t>H3 · MVP (Grupos)</t>
+        </is>
+      </c>
+      <c r="I59" s="19" t="inlineStr">
+        <is>
+          <t>Como pastor quiero que las peticiones solo las vea el Líder y superiores y se borren al vencer.</t>
+        </is>
+      </c>
+      <c r="J59" s="19" t="inlineStr">
+        <is>
+          <t>El Secretario no las ve; tras el plazo configurable (por defecto 30 días) se eliminan.</t>
         </is>
       </c>
       <c r="K59" s="19" t="inlineStr">
         <is>
-          <t>Por definir</t>
+          <t>VoBo pendiente</t>
         </is>
       </c>
       <c r="L59" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M59" s="19" t="inlineStr"/>
-      <c r="N59" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M59" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/m3-peticiones-oracion · 166 pruebas de backend y 32 de frontend pasan; probado contra la base real</t>
+        </is>
+      </c>
+      <c r="N59" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-24 · Alcance por petición (líderes, grupo, equipo), cifrado y borrado a los 30 días configurable. Cambia la matriz aprobada: actualizar con la iglesia.</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="18" t="inlineStr">
         <is>
-          <t>M3-09</t>
+          <t>M3-07</t>
         </is>
       </c>
       <c r="B60" s="19" t="inlineStr">
@@ -5890,17 +5898,17 @@
       </c>
       <c r="C60" s="19" t="inlineStr">
         <is>
-          <t>A un grupo asisten miembros de la iglesia (vecinos o no) e invitados del grupo que no asisten a la iglesia. Los invitados se registran como Contacto con datos mínimos y se les puede invitar a consolidación.</t>
-        </is>
-      </c>
-      <c r="D60" s="21" t="inlineStr">
-        <is>
-          <t>Corrección v3.2</t>
+          <t>Dashboard de supervisión («Resumen de grupos») para Supervisor, Líder, Pastor y Anciano sobre los grupos que cada uno puede consultar: asistencia por semana y por grupo, grupos sin lista esta semana, asistencia por debajo de un mínimo configurable (60 % por defecto), ofrendas avaladas, pendientes y con diferencia (solo si el rol ve finanzas) y peticiones activas (solo las que puede leer). No muestra datos de personas. El Secretario y el Tesorero no lo ven.</t>
+        </is>
+      </c>
+      <c r="D60" s="19" t="inlineStr">
+        <is>
+          <t>v3</t>
         </is>
       </c>
       <c r="E60" s="19" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>MVP básico</t>
         </is>
       </c>
       <c r="F60" s="19" t="inlineStr">
@@ -5910,7 +5918,7 @@
       </c>
       <c r="G60" s="19" t="inlineStr">
         <is>
-          <t>Sprint 3</t>
+          <t>Sprint 5</t>
         </is>
       </c>
       <c r="H60" s="19" t="inlineStr">
@@ -5920,12 +5928,12 @@
       </c>
       <c r="I60" s="19" t="inlineStr">
         <is>
-          <t>Como secretario quiero registrar invitados del grupo con datos mínimos.</t>
+          <t>Como supervisor quiero ver la salud de mis grupos.</t>
         </is>
       </c>
       <c r="J60" s="19" t="inlineStr">
         <is>
-          <t>Registrar un invitado como Contacto y marcarlo presente.</t>
+          <t>El dashboard muestra asistencia, ofrendas y crecimiento según permisos.</t>
         </is>
       </c>
       <c r="K60" s="19" t="inlineStr">
@@ -5940,19 +5948,19 @@
       </c>
       <c r="M60" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/paso-5-invitaciones · pruebas de backend y 93 de frontend pasan; lint, estilos y compilación limpios</t>
+          <t>Rama feature/m3-dashboard-tablero · 195 pruebas de backend y 39 de frontend pasan; probado contra la base real</t>
         </is>
       </c>
       <c r="N60" s="19" t="inlineStr">
         <is>
-          <t>2026-10-27 · Los invitados entran al grupo como Contacto cuando el líder aprueba su solicitud por enlace o QR.</t>
+          <t>2026-10-25 · Dashboard con asistencia, avisos y datos según rol; umbral configurable.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="18" t="inlineStr">
         <is>
-          <t>M3-10</t>
+          <t>M3-08</t>
         </is>
       </c>
       <c r="B61" s="19" t="inlineStr">
@@ -5962,42 +5970,42 @@
       </c>
       <c r="C61" s="19" t="inlineStr">
         <is>
-          <t>Confidencialidad de ofrendas y asistencias: consulta limitada por rol (matriz por definir) y modificación restringida, todo en bitácora.</t>
-        </is>
-      </c>
-      <c r="D61" s="21" t="inlineStr">
-        <is>
-          <t>Obs. 5</t>
+          <t>Ubicación de zona del grupo para que personas cercanas lo encuentren, sin exponer el domicilio exacto. Por definir.</t>
+        </is>
+      </c>
+      <c r="D61" s="19" t="inlineStr">
+        <is>
+          <t>v3</t>
         </is>
       </c>
       <c r="E61" s="19" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Fuera del MVP</t>
         </is>
       </c>
       <c r="F61" s="19" t="inlineStr">
         <is>
-          <t>Fase 1</t>
+          <t>Fase 4</t>
         </is>
       </c>
       <c r="G61" s="19" t="inlineStr">
         <is>
-          <t>Sprint 4</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H61" s="19" t="inlineStr">
         <is>
-          <t>H3 · MVP (Grupos)</t>
-        </is>
-      </c>
-      <c r="I61" s="19" t="inlineStr">
-        <is>
-          <t>Como pastor quiero que ofrendas y asistencias sean confidenciales.</t>
-        </is>
-      </c>
-      <c r="J61" s="19" t="inlineStr">
-        <is>
-          <t>La matriz de la sección 3.3 del v3.2 se cumple en pruebas por cada rol.</t>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="I61" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
+        </is>
+      </c>
+      <c r="J61" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
         </is>
       </c>
       <c r="K61" s="19" t="inlineStr">
@@ -6016,7 +6024,7 @@
     <row r="62">
       <c r="A62" s="18" t="inlineStr">
         <is>
-          <t>M3-11</t>
+          <t>M3-09</t>
         </is>
       </c>
       <c r="B62" s="19" t="inlineStr">
@@ -6026,12 +6034,12 @@
       </c>
       <c r="C62" s="19" t="inlineStr">
         <is>
-          <t>Tablero de mensajes del grupo: lo publican Líder, Supervisor, Secretario y Pastor; lo leen todos los integrantes activos. Mensajes de hasta 1,000 caracteres, con opción de fijarlos, borrado lógico, contador de mensajes nuevos y conservación configurable (90 días). Pantalla «Avisos» para quien no abre la página del grupo.</t>
+          <t>A un grupo asisten miembros de la iglesia (vecinos o no) e invitados del grupo que no asisten a la iglesia. Los invitados se registran como Contacto con datos mínimos y se les puede invitar a consolidación.</t>
         </is>
       </c>
       <c r="D62" s="21" t="inlineStr">
         <is>
-          <t>Obs. 7</t>
+          <t>Corrección v3.2</t>
         </is>
       </c>
       <c r="E62" s="19" t="inlineStr">
@@ -6046,7 +6054,7 @@
       </c>
       <c r="G62" s="19" t="inlineStr">
         <is>
-          <t>Sprint 5</t>
+          <t>Sprint 3</t>
         </is>
       </c>
       <c r="H62" s="19" t="inlineStr">
@@ -6056,12 +6064,12 @@
       </c>
       <c r="I62" s="19" t="inlineStr">
         <is>
-          <t>Como líder quiero un tablero de mensajes de mi grupo.</t>
+          <t>Como secretario quiero registrar invitados del grupo con datos mínimos.</t>
         </is>
       </c>
       <c r="J62" s="19" t="inlineStr">
         <is>
-          <t>Publicar y leer mensajes del grupo.</t>
+          <t>Registrar un invitado como Contacto y marcarlo presente.</t>
         </is>
       </c>
       <c r="K62" s="19" t="inlineStr">
@@ -6076,19 +6084,19 @@
       </c>
       <c r="M62" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/m3-dashboard-tablero · 195 pruebas de backend y 39 de frontend pasan; probado contra la base real</t>
+          <t>Rama feature/paso-5-invitaciones · pruebas de backend y 93 de frontend pasan; lint, estilos y compilación limpios</t>
         </is>
       </c>
       <c r="N62" s="19" t="inlineStr">
         <is>
-          <t>2026-10-25 · Tablero con fijados, no leídos y retención configurable; la notificación push de mensajes nuevos se entrega con M1-09.</t>
+          <t>2026-10-27 · Los invitados entran al grupo como Contacto cuando el líder aprueba su solicitud por enlace o QR.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="18" t="inlineStr">
         <is>
-          <t>M3-12</t>
+          <t>M3-10</t>
         </is>
       </c>
       <c r="B63" s="19" t="inlineStr">
@@ -6098,12 +6106,12 @@
       </c>
       <c r="C63" s="19" t="inlineStr">
         <is>
-          <t>Reuniones: cada grupo se reúne una vez por semana en casa del líder (día y hora por grupo) y existe una reunión general de líderes, modelada como un grupo de tipo «Líderes».</t>
+          <t>Confidencialidad de ofrendas y asistencias: consulta limitada por rol (matriz por definir) y modificación restringida, todo en bitácora.</t>
         </is>
       </c>
       <c r="D63" s="21" t="inlineStr">
         <is>
-          <t>Respuesta</t>
+          <t>Obs. 5</t>
         </is>
       </c>
       <c r="E63" s="19" t="inlineStr">
@@ -6118,7 +6126,7 @@
       </c>
       <c r="G63" s="19" t="inlineStr">
         <is>
-          <t>Sprint 3</t>
+          <t>Sprint 4</t>
         </is>
       </c>
       <c r="H63" s="19" t="inlineStr">
@@ -6126,41 +6134,33 @@
           <t>H3 · MVP (Grupos)</t>
         </is>
       </c>
-      <c r="I63" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
-        </is>
-      </c>
-      <c r="J63" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
+      <c r="I63" s="19" t="inlineStr">
+        <is>
+          <t>Como pastor quiero que ofrendas y asistencias sean confidenciales.</t>
+        </is>
+      </c>
+      <c r="J63" s="19" t="inlineStr">
+        <is>
+          <t>La matriz de la sección 3.3 del v3.2 se cumple en pruebas por cada rol.</t>
         </is>
       </c>
       <c r="K63" s="19" t="inlineStr">
         <is>
-          <t>VoBo pendiente</t>
+          <t>Por definir</t>
         </is>
       </c>
       <c r="L63" s="19" t="inlineStr">
         <is>
-          <t>En pruebas</t>
-        </is>
-      </c>
-      <c r="M63" s="19" t="inlineStr">
-        <is>
-          <t>Rama feature/grupos-paso-3 · pruebas de backend y 81 de frontend pasan; lint, estilos y compilación limpios</t>
-        </is>
-      </c>
-      <c r="N63" s="19" t="inlineStr">
-        <is>
-          <t>2026-10-27 · Una reunión semanal por grupo y grupo tipo Líderes; filtros por día, sector, líder y estado; cada reunión muestra su asistencia, observaciones, peticiones y ofrendas.</t>
-        </is>
-      </c>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M63" s="19" t="inlineStr"/>
+      <c r="N63" s="19" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="18" t="inlineStr">
         <is>
-          <t>M3-13</t>
+          <t>M3-11</t>
         </is>
       </c>
       <c r="B64" s="19" t="inlineStr">
@@ -6170,12 +6170,12 @@
       </c>
       <c r="C64" s="19" t="inlineStr">
         <is>
-          <t>Parámetros configurables sin programar, con pantalla de Configuración y cada cambio en bitácora: monto máximo por ofrenda (1,000,000 por defecto) y si se permite una sola ofrenda regular por reunión. Solo Pastor y Administrador Técnico.</t>
+          <t>Tablero de mensajes del grupo: lo publican Líder, Supervisor, Secretario y Pastor; lo leen todos los integrantes activos. Mensajes de hasta 1,000 caracteres, con opción de fijarlos, borrado lógico, contador de mensajes nuevos y conservación configurable (90 días). Pantalla «Avisos» para quien no abre la página del grupo.</t>
         </is>
       </c>
       <c r="D64" s="21" t="inlineStr">
         <is>
-          <t>Respuesta</t>
+          <t>Obs. 7</t>
         </is>
       </c>
       <c r="E64" s="19" t="inlineStr">
@@ -6190,7 +6190,7 @@
       </c>
       <c r="G64" s="19" t="inlineStr">
         <is>
-          <t>Sprint 4</t>
+          <t>Sprint 5</t>
         </is>
       </c>
       <c r="H64" s="19" t="inlineStr">
@@ -6198,14 +6198,14 @@
           <t>H3 · MVP (Grupos)</t>
         </is>
       </c>
-      <c r="I64" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
-        </is>
-      </c>
-      <c r="J64" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
+      <c r="I64" s="19" t="inlineStr">
+        <is>
+          <t>Como líder quiero un tablero de mensajes de mi grupo.</t>
+        </is>
+      </c>
+      <c r="J64" s="19" t="inlineStr">
+        <is>
+          <t>Publicar y leer mensajes del grupo.</t>
         </is>
       </c>
       <c r="K64" s="19" t="inlineStr">
@@ -6220,19 +6220,19 @@
       </c>
       <c r="M64" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/m3-ofrendas-ajustes · 121 pruebas de backend y 14 de frontend pasan</t>
+          <t>Rama feature/m3-dashboard-tablero · 195 pruebas de backend y 39 de frontend pasan; probado contra la base real</t>
         </is>
       </c>
       <c r="N64" s="19" t="inlineStr">
         <is>
-          <t>2026-10-24 · Pantalla Configuración: monto máximo y una regular por reunión.</t>
+          <t>2026-10-25 · Tablero con fijados, no leídos y retención configurable; la notificación push de mensajes nuevos se entrega con M1-09.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="18" t="inlineStr">
         <is>
-          <t>M3-14</t>
+          <t>M3-12</t>
         </is>
       </c>
       <c r="B65" s="19" t="inlineStr">
@@ -6242,7 +6242,7 @@
       </c>
       <c r="C65" s="19" t="inlineStr">
         <is>
-          <t>Componente de peticiones reutilizable: cualquier módulo (grupos hoy; cursos o eventos después) se registra como origen y decide quién registra y qué nivel de acceso tiene cada persona. Toda petición guarda su origen de forma inmutable (tipo, identificador y una etiqueta fija, por ejemplo «Grupo de Conexión · Norte · reunión del 22/10/2026») y lo muestra siempre en el listado.</t>
+          <t>Reuniones: cada grupo se reúne una vez por semana en casa del líder (día y hora por grupo) y existe una reunión general de líderes, modelada como un grupo de tipo «Líderes».</t>
         </is>
       </c>
       <c r="D65" s="21" t="inlineStr">
@@ -6262,7 +6262,7 @@
       </c>
       <c r="G65" s="19" t="inlineStr">
         <is>
-          <t>Sprint 4</t>
+          <t>Sprint 3</t>
         </is>
       </c>
       <c r="H65" s="19" t="inlineStr">
@@ -6292,19 +6292,19 @@
       </c>
       <c r="M65" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/m3-peticiones-oracion · 166 pruebas de backend y 32 de frontend pasan; probado contra la base real</t>
+          <t>Rama feature/grupos-paso-3 · pruebas de backend y 81 de frontend pasan; lint, estilos y compilación limpios</t>
         </is>
       </c>
       <c r="N65" s="19" t="inlineStr">
         <is>
-          <t>2026-10-24 · Origen inmutable y visible; probado con un segundo origen de prueba para verificar la reutilización.</t>
+          <t>2026-10-27 · Una reunión semanal por grupo y grupo tipo Líderes; filtros por día, sector, líder y estado; cada reunión muestra su asistencia, observaciones, peticiones y ofrendas.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="18" t="inlineStr">
         <is>
-          <t>M3-15</t>
+          <t>M3-13</t>
         </is>
       </c>
       <c r="B66" s="19" t="inlineStr">
@@ -6314,7 +6314,7 @@
       </c>
       <c r="C66" s="19" t="inlineStr">
         <is>
-          <t>Equipo de oración: rol configurable (Equipo de oración) que se asigna a las personas que se reúnen a orar por las peticiones compartidas con ese alcance; no da acceso a nada más. Opción de ocultar el nombre de quien pide: los campos del formulario marcados «identifica a la persona» solo los ven líderes y quien registró. Al capturar se muestra una leyenda que pide confirmar la autorización de quien pide, indica quién la leerá y cuándo se borra.</t>
+          <t>Parámetros configurables sin programar, con pantalla de Configuración y cada cambio en bitácora: monto máximo por ofrenda (1,000,000 por defecto) y si se permite una sola ofrenda regular por reunión. Solo Pastor y Administrador Técnico.</t>
         </is>
       </c>
       <c r="D66" s="21" t="inlineStr">
@@ -6364,54 +6364,54 @@
       </c>
       <c r="M66" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/m3-peticiones-oracion · 166 pruebas de backend y 32 de frontend pasan; probado contra la base real</t>
+          <t>Rama feature/m3-ofrendas-ajustes · 121 pruebas de backend y 14 de frontend pasan</t>
         </is>
       </c>
       <c r="N66" s="19" t="inlineStr">
         <is>
-          <t>2026-10-24 · Rol Equipo de oración, nombre oculto y leyenda de privacidad al capturar. Falta el aviso de privacidad oficial de la iglesia.</t>
+          <t>2026-10-24 · Pantalla Configuración: monto máximo y una regular por reunión.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="18" t="inlineStr">
         <is>
-          <t>M4-01</t>
+          <t>M3-14</t>
         </is>
       </c>
       <c r="B67" s="19" t="inlineStr">
         <is>
-          <t>M4 Kids Check-In/Out</t>
+          <t>M3 Grupos de Conexión</t>
         </is>
       </c>
       <c r="C67" s="19" t="inlineStr">
         <is>
-          <t>Sustitución de la ficha física de papel.</t>
-        </is>
-      </c>
-      <c r="D67" s="19" t="inlineStr">
-        <is>
-          <t>v1 / v2</t>
+          <t>Componente de peticiones reutilizable: cualquier módulo (grupos hoy; cursos o eventos después) se registra como origen y decide quién registra y qué nivel de acceso tiene cada persona. Toda petición guarda su origen de forma inmutable (tipo, identificador y una etiqueta fija, por ejemplo «Grupo de Conexión · Norte · reunión del 22/10/2026») y lo muestra siempre en el listado.</t>
+        </is>
+      </c>
+      <c r="D67" s="21" t="inlineStr">
+        <is>
+          <t>Respuesta</t>
         </is>
       </c>
       <c r="E67" s="19" t="inlineStr">
         <is>
-          <t>Fuera del MVP</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="F67" s="19" t="inlineStr">
         <is>
-          <t>Fase 2</t>
+          <t>Fase 1</t>
         </is>
       </c>
       <c r="G67" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sprint 4</t>
         </is>
       </c>
       <c r="H67" s="19" t="inlineStr">
         <is>
-          <t>Posterior</t>
+          <t>H3 · MVP (Grupos)</t>
         </is>
       </c>
       <c r="I67" s="20" t="inlineStr">
@@ -6431,51 +6431,59 @@
       </c>
       <c r="L67" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M67" s="19" t="inlineStr"/>
-      <c r="N67" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M67" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/m3-peticiones-oracion · 166 pruebas de backend y 32 de frontend pasan; probado contra la base real</t>
+        </is>
+      </c>
+      <c r="N67" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-24 · Origen inmutable y visible; probado con un segundo origen de prueba para verificar la reutilización.</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="18" t="inlineStr">
         <is>
-          <t>M4-02</t>
+          <t>M3-15</t>
         </is>
       </c>
       <c r="B68" s="19" t="inlineStr">
         <is>
-          <t>M4 Kids Check-In/Out</t>
+          <t>M3 Grupos de Conexión</t>
         </is>
       </c>
       <c r="C68" s="19" t="inlineStr">
         <is>
-          <t>Registro de ingreso del menor con salón o clase asignada y generación de código único.</t>
+          <t>Equipo de oración: rol configurable (Equipo de oración) que se asigna a las personas que se reúnen a orar por las peticiones compartidas con ese alcance; no da acceso a nada más. Opción de ocultar el nombre de quien pide: los campos del formulario marcados «identifica a la persona» solo los ven líderes y quien registró. Al capturar se muestra una leyenda que pide confirmar la autorización de quien pide, indica quién la leerá y cuándo se borra.</t>
         </is>
       </c>
       <c r="D68" s="21" t="inlineStr">
         <is>
-          <t>v1 + Nuevo v3</t>
+          <t>Respuesta</t>
         </is>
       </c>
       <c r="E68" s="19" t="inlineStr">
         <is>
-          <t>Fuera del MVP</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="F68" s="19" t="inlineStr">
         <is>
-          <t>Fase 2</t>
+          <t>Fase 1</t>
         </is>
       </c>
       <c r="G68" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sprint 4</t>
         </is>
       </c>
       <c r="H68" s="19" t="inlineStr">
         <is>
-          <t>Posterior</t>
+          <t>H3 · MVP (Grupos)</t>
         </is>
       </c>
       <c r="I68" s="20" t="inlineStr">
@@ -6495,16 +6503,24 @@
       </c>
       <c r="L68" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M68" s="19" t="inlineStr"/>
-      <c r="N68" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M68" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/m3-peticiones-oracion · 166 pruebas de backend y 32 de frontend pasan; probado contra la base real</t>
+        </is>
+      </c>
+      <c r="N68" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-24 · Rol Equipo de oración, nombre oculto y leyenda de privacidad al capturar. Falta el aviso de privacidad oficial de la iglesia.</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="18" t="inlineStr">
         <is>
-          <t>M4-03</t>
+          <t>M4-01</t>
         </is>
       </c>
       <c r="B69" s="19" t="inlineStr">
@@ -6514,12 +6530,12 @@
       </c>
       <c r="C69" s="19" t="inlineStr">
         <is>
-          <t>Código QR dinámico o OTP temporal en la PWA del padre o tutor.</t>
+          <t>Sustitución de la ficha física de papel.</t>
         </is>
       </c>
       <c r="D69" s="19" t="inlineStr">
         <is>
-          <t>v2</t>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E69" s="19" t="inlineStr">
@@ -6568,7 +6584,7 @@
     <row r="70">
       <c r="A70" s="18" t="inlineStr">
         <is>
-          <t>M4-04</t>
+          <t>M4-02</t>
         </is>
       </c>
       <c r="B70" s="19" t="inlineStr">
@@ -6578,12 +6594,12 @@
       </c>
       <c r="C70" s="19" t="inlineStr">
         <is>
-          <t>Validación al entregar: el servidor de Kids escanea el código y confirma identidad y fotografía del tutor autorizado en el Expediente Digital.</t>
-        </is>
-      </c>
-      <c r="D70" s="19" t="inlineStr">
-        <is>
-          <t>v2</t>
+          <t>Registro de ingreso del menor con salón o clase asignada y generación de código único.</t>
+        </is>
+      </c>
+      <c r="D70" s="21" t="inlineStr">
+        <is>
+          <t>v1 + Nuevo v3</t>
         </is>
       </c>
       <c r="E70" s="19" t="inlineStr">
@@ -6632,7 +6648,7 @@
     <row r="71">
       <c r="A71" s="18" t="inlineStr">
         <is>
-          <t>M4-05</t>
+          <t>M4-03</t>
         </is>
       </c>
       <c r="B71" s="19" t="inlineStr">
@@ -6642,12 +6658,12 @@
       </c>
       <c r="C71" s="19" t="inlineStr">
         <is>
-          <t>Alternativa para tutores sin smartphone, sin batería o sin conexión (p. ej. código por SMS o comprobante imprimible con identificación). Por definir.</t>
-        </is>
-      </c>
-      <c r="D71" s="21" t="inlineStr">
-        <is>
-          <t>Nuevo v3</t>
+          <t>Código QR dinámico o OTP temporal en la PWA del padre o tutor.</t>
+        </is>
+      </c>
+      <c r="D71" s="19" t="inlineStr">
+        <is>
+          <t>v2</t>
         </is>
       </c>
       <c r="E71" s="19" t="inlineStr">
@@ -6682,7 +6698,7 @@
       </c>
       <c r="K71" s="19" t="inlineStr">
         <is>
-          <t>Por definir</t>
+          <t>VoBo pendiente</t>
         </is>
       </c>
       <c r="L71" s="19" t="inlineStr">
@@ -6696,7 +6712,7 @@
     <row r="72">
       <c r="A72" s="18" t="inlineStr">
         <is>
-          <t>M4-06</t>
+          <t>M4-04</t>
         </is>
       </c>
       <c r="B72" s="19" t="inlineStr">
@@ -6706,12 +6722,12 @@
       </c>
       <c r="C72" s="19" t="inlineStr">
         <is>
-          <t>Autorización temporal de un tercero para recoger al menor, con aprobación del tutor registrado.</t>
-        </is>
-      </c>
-      <c r="D72" s="21" t="inlineStr">
-        <is>
-          <t>Nuevo v3</t>
+          <t>Validación al entregar: el servidor de Kids escanea el código y confirma identidad y fotografía del tutor autorizado en el Expediente Digital.</t>
+        </is>
+      </c>
+      <c r="D72" s="19" t="inlineStr">
+        <is>
+          <t>v2</t>
         </is>
       </c>
       <c r="E72" s="19" t="inlineStr">
@@ -6760,7 +6776,7 @@
     <row r="73">
       <c r="A73" s="18" t="inlineStr">
         <is>
-          <t>M4-07</t>
+          <t>M4-05</t>
         </is>
       </c>
       <c r="B73" s="19" t="inlineStr">
@@ -6770,7 +6786,7 @@
       </c>
       <c r="C73" s="19" t="inlineStr">
         <is>
-          <t>Caducidad del código y bitácora de cada entrega (quién recogió, quién entregó, hora).</t>
+          <t>Alternativa para tutores sin smartphone, sin batería o sin conexión (p. ej. código por SMS o comprobante imprimible con identificación). Por definir.</t>
         </is>
       </c>
       <c r="D73" s="21" t="inlineStr">
@@ -6810,7 +6826,7 @@
       </c>
       <c r="K73" s="19" t="inlineStr">
         <is>
-          <t>VoBo pendiente</t>
+          <t>Por definir</t>
         </is>
       </c>
       <c r="L73" s="19" t="inlineStr">
@@ -6824,7 +6840,7 @@
     <row r="74">
       <c r="A74" s="18" t="inlineStr">
         <is>
-          <t>M4-08</t>
+          <t>M4-06</t>
         </is>
       </c>
       <c r="B74" s="19" t="inlineStr">
@@ -6834,7 +6850,7 @@
       </c>
       <c r="C74" s="19" t="inlineStr">
         <is>
-          <t>Funcionamiento sin conexión o con conexión degradada para el check-out.</t>
+          <t>Autorización temporal de un tercero para recoger al menor, con aprobación del tutor registrado.</t>
         </is>
       </c>
       <c r="D74" s="21" t="inlineStr">
@@ -6888,52 +6904,52 @@
     <row r="75">
       <c r="A75" s="18" t="inlineStr">
         <is>
-          <t>M5-01</t>
+          <t>M4-07</t>
         </is>
       </c>
       <c r="B75" s="19" t="inlineStr">
         <is>
-          <t>M5 Áreas y servidores</t>
+          <t>M4 Kids Check-In/Out</t>
         </is>
       </c>
       <c r="C75" s="19" t="inlineStr">
         <is>
-          <t>Catálogo mínimo de áreas y asignación de servidores. Versión reducida del módulo 5, necesaria para permisos por área. Sirve como primer censo.</t>
-        </is>
-      </c>
-      <c r="D75" s="19" t="inlineStr">
-        <is>
-          <t>v3</t>
+          <t>Caducidad del código y bitácora de cada entrega (quién recogió, quién entregó, hora).</t>
+        </is>
+      </c>
+      <c r="D75" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3</t>
         </is>
       </c>
       <c r="E75" s="19" t="inlineStr">
         <is>
-          <t>MVP mínimo</t>
+          <t>Fuera del MVP</t>
         </is>
       </c>
       <c r="F75" s="19" t="inlineStr">
         <is>
-          <t>Fase 0</t>
+          <t>Fase 2</t>
         </is>
       </c>
       <c r="G75" s="19" t="inlineStr">
         <is>
-          <t>Sprint 1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H75" s="19" t="inlineStr">
         <is>
-          <t>H2 · Fase 0 completa</t>
-        </is>
-      </c>
-      <c r="I75" s="19" t="inlineStr">
-        <is>
-          <t>Como pastor quiero un catálogo de áreas con su personal para conocer la estructura.</t>
-        </is>
-      </c>
-      <c r="J75" s="19" t="inlineStr">
-        <is>
-          <t>Crear un área, asignar servidores y ver el conteo real.</t>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="I75" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
+        </is>
+      </c>
+      <c r="J75" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
         </is>
       </c>
       <c r="K75" s="19" t="inlineStr">
@@ -6952,22 +6968,22 @@
     <row r="76">
       <c r="A76" s="18" t="inlineStr">
         <is>
-          <t>M5-02</t>
+          <t>M4-08</t>
         </is>
       </c>
       <c r="B76" s="19" t="inlineStr">
         <is>
-          <t>M5 Áreas y servidores</t>
+          <t>M4 Kids Check-In/Out</t>
         </is>
       </c>
       <c r="C76" s="19" t="inlineStr">
         <is>
-          <t>Roles jerárquicos dentro de cada área (directores, líderes, maestros, servidores).</t>
-        </is>
-      </c>
-      <c r="D76" s="19" t="inlineStr">
-        <is>
-          <t>v1</t>
+          <t>Funcionamiento sin conexión o con conexión degradada para el check-out.</t>
+        </is>
+      </c>
+      <c r="D76" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3</t>
         </is>
       </c>
       <c r="E76" s="19" t="inlineStr">
@@ -6977,7 +6993,7 @@
       </c>
       <c r="F76" s="19" t="inlineStr">
         <is>
-          <t>Fase 4</t>
+          <t>Fase 2</t>
         </is>
       </c>
       <c r="G76" s="19" t="inlineStr">
@@ -7016,7 +7032,7 @@
     <row r="77">
       <c r="A77" s="18" t="inlineStr">
         <is>
-          <t>M5-03</t>
+          <t>M5-01</t>
         </is>
       </c>
       <c r="B77" s="19" t="inlineStr">
@@ -7026,42 +7042,42 @@
       </c>
       <c r="C77" s="19" t="inlineStr">
         <is>
-          <t>Organigrama y número real de servidores activos, directores y líderes por área.</t>
+          <t>Catálogo mínimo de áreas y asignación de servidores. Versión reducida del módulo 5, necesaria para permisos por área. Sirve como primer censo.</t>
         </is>
       </c>
       <c r="D77" s="19" t="inlineStr">
         <is>
-          <t>v2</t>
+          <t>v3</t>
         </is>
       </c>
       <c r="E77" s="19" t="inlineStr">
         <is>
-          <t>Fuera del MVP</t>
+          <t>MVP mínimo</t>
         </is>
       </c>
       <c r="F77" s="19" t="inlineStr">
         <is>
-          <t>Fase 4</t>
+          <t>Fase 0</t>
         </is>
       </c>
       <c r="G77" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sprint 1</t>
         </is>
       </c>
       <c r="H77" s="19" t="inlineStr">
         <is>
-          <t>Posterior</t>
-        </is>
-      </c>
-      <c r="I77" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
-        </is>
-      </c>
-      <c r="J77" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
+          <t>H2 · Fase 0 completa</t>
+        </is>
+      </c>
+      <c r="I77" s="19" t="inlineStr">
+        <is>
+          <t>Como pastor quiero un catálogo de áreas con su personal para conocer la estructura.</t>
+        </is>
+      </c>
+      <c r="J77" s="19" t="inlineStr">
+        <is>
+          <t>Crear un área, asignar servidores y ver el conteo real.</t>
         </is>
       </c>
       <c r="K77" s="19" t="inlineStr">
@@ -7080,7 +7096,7 @@
     <row r="78">
       <c r="A78" s="18" t="inlineStr">
         <is>
-          <t>M5-04</t>
+          <t>M5-02</t>
         </is>
       </c>
       <c r="B78" s="19" t="inlineStr">
@@ -7090,12 +7106,12 @@
       </c>
       <c r="C78" s="19" t="inlineStr">
         <is>
-          <t>Control de asistencia a turnos o servicios.</t>
+          <t>Roles jerárquicos dentro de cada área (directores, líderes, maestros, servidores).</t>
         </is>
       </c>
       <c r="D78" s="19" t="inlineStr">
         <is>
-          <t>v1 / v2</t>
+          <t>v1</t>
         </is>
       </c>
       <c r="E78" s="19" t="inlineStr">
@@ -7144,7 +7160,7 @@
     <row r="79">
       <c r="A79" s="18" t="inlineStr">
         <is>
-          <t>M5-05</t>
+          <t>M5-03</t>
         </is>
       </c>
       <c r="B79" s="19" t="inlineStr">
@@ -7154,12 +7170,12 @@
       </c>
       <c r="C79" s="19" t="inlineStr">
         <is>
-          <t>Tablero de avisos y notificaciones interno por área.</t>
+          <t>Organigrama y número real de servidores activos, directores y líderes por área.</t>
         </is>
       </c>
       <c r="D79" s="19" t="inlineStr">
         <is>
-          <t>v1 / v2</t>
+          <t>v2</t>
         </is>
       </c>
       <c r="E79" s="19" t="inlineStr">
@@ -7208,7 +7224,7 @@
     <row r="80">
       <c r="A80" s="18" t="inlineStr">
         <is>
-          <t>M5-06</t>
+          <t>M5-04</t>
         </is>
       </c>
       <c r="B80" s="19" t="inlineStr">
@@ -7218,7 +7234,7 @@
       </c>
       <c r="C80" s="19" t="inlineStr">
         <is>
-          <t>Gestión financiera por área: caja chica y gastos operativos.</t>
+          <t>Control de asistencia a turnos o servicios.</t>
         </is>
       </c>
       <c r="D80" s="19" t="inlineStr">
@@ -7272,22 +7288,22 @@
     <row r="81">
       <c r="A81" s="18" t="inlineStr">
         <is>
-          <t>M6-01</t>
+          <t>M5-05</t>
         </is>
       </c>
       <c r="B81" s="19" t="inlineStr">
         <is>
-          <t>M6 Ministerios de servicio</t>
+          <t>M5 Áreas y servidores</t>
         </is>
       </c>
       <c r="C81" s="19" t="inlineStr">
         <is>
-          <t>Control de personal propio de cada ministerio.</t>
-        </is>
-      </c>
-      <c r="D81" s="22" t="inlineStr">
-        <is>
-          <t>Recuperado v1</t>
+          <t>Tablero de avisos y notificaciones interno por área.</t>
+        </is>
+      </c>
+      <c r="D81" s="19" t="inlineStr">
+        <is>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E81" s="19" t="inlineStr">
@@ -7336,17 +7352,17 @@
     <row r="82">
       <c r="A82" s="18" t="inlineStr">
         <is>
-          <t>M6-02</t>
+          <t>M5-06</t>
         </is>
       </c>
       <c r="B82" s="19" t="inlineStr">
         <is>
-          <t>M6 Ministerios de servicio</t>
+          <t>M5 Áreas y servidores</t>
         </is>
       </c>
       <c r="C82" s="19" t="inlineStr">
         <is>
-          <t>Menú o catálogo digital interactivo (público o interno), autogestionado.</t>
+          <t>Gestión financiera por área: caja chica y gastos operativos.</t>
         </is>
       </c>
       <c r="D82" s="19" t="inlineStr">
@@ -7400,7 +7416,7 @@
     <row r="83">
       <c r="A83" s="18" t="inlineStr">
         <is>
-          <t>M6-03</t>
+          <t>M6-01</t>
         </is>
       </c>
       <c r="B83" s="19" t="inlineStr">
@@ -7410,12 +7426,12 @@
       </c>
       <c r="C83" s="19" t="inlineStr">
         <is>
-          <t>Calendario de turnos: días regulares de servicio y eventos especiales.</t>
-        </is>
-      </c>
-      <c r="D83" s="19" t="inlineStr">
-        <is>
-          <t>v1 / v2</t>
+          <t>Control de personal propio de cada ministerio.</t>
+        </is>
+      </c>
+      <c r="D83" s="22" t="inlineStr">
+        <is>
+          <t>Recuperado v1</t>
         </is>
       </c>
       <c r="E83" s="19" t="inlineStr">
@@ -7464,7 +7480,7 @@
     <row r="84">
       <c r="A84" s="18" t="inlineStr">
         <is>
-          <t>M6-04</t>
+          <t>M6-02</t>
         </is>
       </c>
       <c r="B84" s="19" t="inlineStr">
@@ -7474,7 +7490,7 @@
       </c>
       <c r="C84" s="19" t="inlineStr">
         <is>
-          <t>Registro de asistentes o personas atendidas.</t>
+          <t>Menú o catálogo digital interactivo (público o interno), autogestionado.</t>
         </is>
       </c>
       <c r="D84" s="19" t="inlineStr">
@@ -7528,7 +7544,7 @@
     <row r="85">
       <c r="A85" s="18" t="inlineStr">
         <is>
-          <t>M6-05</t>
+          <t>M6-03</t>
         </is>
       </c>
       <c r="B85" s="19" t="inlineStr">
@@ -7538,7 +7554,7 @@
       </c>
       <c r="C85" s="19" t="inlineStr">
         <is>
-          <t>Control de gastos y de inventario básico.</t>
+          <t>Calendario de turnos: días regulares de servicio y eventos especiales.</t>
         </is>
       </c>
       <c r="D85" s="19" t="inlineStr">
@@ -7592,7 +7608,7 @@
     <row r="86">
       <c r="A86" s="18" t="inlineStr">
         <is>
-          <t>M6-06</t>
+          <t>M6-04</t>
         </is>
       </c>
       <c r="B86" s="19" t="inlineStr">
@@ -7602,7 +7618,7 @@
       </c>
       <c r="C86" s="19" t="inlineStr">
         <is>
-          <t>Canal de comunicación directo con el área de Administración General.</t>
+          <t>Registro de asistentes o personas atendidas.</t>
         </is>
       </c>
       <c r="D86" s="19" t="inlineStr">
@@ -7656,7 +7672,7 @@
     <row r="87">
       <c r="A87" s="18" t="inlineStr">
         <is>
-          <t>M6-07</t>
+          <t>M6-05</t>
         </is>
       </c>
       <c r="B87" s="19" t="inlineStr">
@@ -7666,12 +7682,12 @@
       </c>
       <c r="C87" s="19" t="inlineStr">
         <is>
-          <t>Servicio Médico: los datos de salud de las personas atendidas requieren tratamiento de datos sensibles. Por definir alcance.</t>
-        </is>
-      </c>
-      <c r="D87" s="21" t="inlineStr">
-        <is>
-          <t>Nuevo v3</t>
+          <t>Control de gastos y de inventario básico.</t>
+        </is>
+      </c>
+      <c r="D87" s="19" t="inlineStr">
+        <is>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E87" s="19" t="inlineStr">
@@ -7706,7 +7722,7 @@
       </c>
       <c r="K87" s="19" t="inlineStr">
         <is>
-          <t>Por definir</t>
+          <t>VoBo pendiente</t>
         </is>
       </c>
       <c r="L87" s="19" t="inlineStr">
@@ -7720,17 +7736,17 @@
     <row r="88">
       <c r="A88" s="18" t="inlineStr">
         <is>
-          <t>M7-01</t>
+          <t>M6-06</t>
         </is>
       </c>
       <c r="B88" s="19" t="inlineStr">
         <is>
-          <t>M7 Eventos y aforo</t>
+          <t>M6 Ministerios de servicio</t>
         </is>
       </c>
       <c r="C88" s="19" t="inlineStr">
         <is>
-          <t>Eventos abiertos o evangelísticos con formulario de inscripción rápida, sin requerir historial previo.</t>
+          <t>Canal de comunicación directo con el área de Administración General.</t>
         </is>
       </c>
       <c r="D88" s="19" t="inlineStr">
@@ -7784,22 +7800,22 @@
     <row r="89">
       <c r="A89" s="18" t="inlineStr">
         <is>
-          <t>M7-02</t>
+          <t>M6-07</t>
         </is>
       </c>
       <c r="B89" s="19" t="inlineStr">
         <is>
-          <t>M7 Eventos y aforo</t>
+          <t>M6 Ministerios de servicio</t>
         </is>
       </c>
       <c r="C89" s="19" t="inlineStr">
         <is>
-          <t>Consolidación (inducción de personas que asisten por primera vez) como tipo de evento.</t>
-        </is>
-      </c>
-      <c r="D89" s="22" t="inlineStr">
-        <is>
-          <t>Recuperado v1</t>
+          <t>Servicio Médico: los datos de salud de las personas atendidas requieren tratamiento de datos sensibles. Por definir alcance.</t>
+        </is>
+      </c>
+      <c r="D89" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3</t>
         </is>
       </c>
       <c r="E89" s="19" t="inlineStr">
@@ -7834,7 +7850,7 @@
       </c>
       <c r="K89" s="19" t="inlineStr">
         <is>
-          <t>VoBo pendiente</t>
+          <t>Por definir</t>
         </is>
       </c>
       <c r="L89" s="19" t="inlineStr">
@@ -7848,7 +7864,7 @@
     <row r="90">
       <c r="A90" s="18" t="inlineStr">
         <is>
-          <t>M7-03</t>
+          <t>M7-01</t>
         </is>
       </c>
       <c r="B90" s="19" t="inlineStr">
@@ -7858,12 +7874,12 @@
       </c>
       <c r="C90" s="19" t="inlineStr">
         <is>
-          <t>Encargados de evento (personal de la iglesia únicamente; no se controla personal externo).</t>
-        </is>
-      </c>
-      <c r="D90" s="22" t="inlineStr">
-        <is>
-          <t>Recuperado v1</t>
+          <t>Eventos abiertos o evangelísticos con formulario de inscripción rápida, sin requerir historial previo.</t>
+        </is>
+      </c>
+      <c r="D90" s="19" t="inlineStr">
+        <is>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E90" s="19" t="inlineStr">
@@ -7912,7 +7928,7 @@
     <row r="91">
       <c r="A91" s="18" t="inlineStr">
         <is>
-          <t>M7-04</t>
+          <t>M7-02</t>
         </is>
       </c>
       <c r="B91" s="19" t="inlineStr">
@@ -7922,12 +7938,12 @@
       </c>
       <c r="C91" s="19" t="inlineStr">
         <is>
-          <t>Control de cupo en tiempo real que bloquea el sobrecupo en eventos con aforo limitado (ej. 30 o 50 lugares).</t>
-        </is>
-      </c>
-      <c r="D91" s="19" t="inlineStr">
-        <is>
-          <t>v1 / v2</t>
+          <t>Consolidación (inducción de personas que asisten por primera vez) como tipo de evento.</t>
+        </is>
+      </c>
+      <c r="D91" s="22" t="inlineStr">
+        <is>
+          <t>Recuperado v1</t>
         </is>
       </c>
       <c r="E91" s="19" t="inlineStr">
@@ -7976,7 +7992,7 @@
     <row r="92">
       <c r="A92" s="18" t="inlineStr">
         <is>
-          <t>M7-05</t>
+          <t>M7-03</t>
         </is>
       </c>
       <c r="B92" s="19" t="inlineStr">
@@ -7986,12 +8002,12 @@
       </c>
       <c r="C92" s="19" t="inlineStr">
         <is>
-          <t>Control de asistentes sin lista previa, para aforo y para dar a conocer la iglesia.</t>
-        </is>
-      </c>
-      <c r="D92" s="19" t="inlineStr">
-        <is>
-          <t>v1</t>
+          <t>Encargados de evento (personal de la iglesia únicamente; no se controla personal externo).</t>
+        </is>
+      </c>
+      <c r="D92" s="22" t="inlineStr">
+        <is>
+          <t>Recuperado v1</t>
         </is>
       </c>
       <c r="E92" s="19" t="inlineStr">
@@ -8040,7 +8056,7 @@
     <row r="93">
       <c r="A93" s="18" t="inlineStr">
         <is>
-          <t>M7-06</t>
+          <t>M7-04</t>
         </is>
       </c>
       <c r="B93" s="19" t="inlineStr">
@@ -8050,12 +8066,12 @@
       </c>
       <c r="C93" s="19" t="inlineStr">
         <is>
-          <t>Seguimiento de personas nuevas: conversión de un invitado a Expediente Digital y canalización a un curso o Grupo de Conexión.</t>
-        </is>
-      </c>
-      <c r="D93" s="21" t="inlineStr">
-        <is>
-          <t>Nuevo v3</t>
+          <t>Control de cupo en tiempo real que bloquea el sobrecupo en eventos con aforo limitado (ej. 30 o 50 lugares).</t>
+        </is>
+      </c>
+      <c r="D93" s="19" t="inlineStr">
+        <is>
+          <t>v1 / v2</t>
         </is>
       </c>
       <c r="E93" s="19" t="inlineStr">
@@ -8104,52 +8120,52 @@
     <row r="94">
       <c r="A94" s="18" t="inlineStr">
         <is>
-          <t>NF-01</t>
+          <t>M7-05</t>
         </is>
       </c>
       <c r="B94" s="19" t="inlineStr">
         <is>
-          <t>No funcionales</t>
+          <t>M7 Eventos y aforo</t>
         </is>
       </c>
       <c r="C94" s="19" t="inlineStr">
         <is>
-          <t>Cumplimiento de la LFPDPPP: aviso de privacidad, consentimiento y derechos ARCO.</t>
+          <t>Control de asistentes sin lista previa, para aforo y para dar a conocer la iglesia.</t>
         </is>
       </c>
       <c r="D94" s="19" t="inlineStr">
         <is>
-          <t>v3</t>
+          <t>v1</t>
         </is>
       </c>
       <c r="E94" s="19" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Fuera del MVP</t>
         </is>
       </c>
       <c r="F94" s="19" t="inlineStr">
         <is>
-          <t>Fase 0</t>
+          <t>Fase 4</t>
         </is>
       </c>
       <c r="G94" s="19" t="inlineStr">
         <is>
-          <t>Sprint 1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H94" s="19" t="inlineStr">
         <is>
-          <t>H1 · 18-oct (núcleo Fase 0)</t>
-        </is>
-      </c>
-      <c r="I94" s="19" t="inlineStr">
-        <is>
-          <t>Como iglesia queremos cumplir con la LFPDPPP.</t>
-        </is>
-      </c>
-      <c r="J94" s="19" t="inlineStr">
-        <is>
-          <t>Aviso de privacidad, consentimiento y atención de derechos ARCO disponibles.</t>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="I94" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
+        </is>
+      </c>
+      <c r="J94" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
         </is>
       </c>
       <c r="K94" s="19" t="inlineStr">
@@ -8168,52 +8184,52 @@
     <row r="95">
       <c r="A95" s="18" t="inlineStr">
         <is>
-          <t>NF-02</t>
+          <t>M7-06</t>
         </is>
       </c>
       <c r="B95" s="19" t="inlineStr">
         <is>
-          <t>No funcionales</t>
+          <t>M7 Eventos y aforo</t>
         </is>
       </c>
       <c r="C95" s="19" t="inlineStr">
         <is>
-          <t>Cifrado en tránsito y en reposo. Cifrado adicional a nivel de campo para peticiones de oración.</t>
-        </is>
-      </c>
-      <c r="D95" s="19" t="inlineStr">
-        <is>
-          <t>v3</t>
+          <t>Seguimiento de personas nuevas: conversión de un invitado a Expediente Digital y canalización a un curso o Grupo de Conexión.</t>
+        </is>
+      </c>
+      <c r="D95" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3</t>
         </is>
       </c>
       <c r="E95" s="19" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Fuera del MVP</t>
         </is>
       </c>
       <c r="F95" s="19" t="inlineStr">
         <is>
-          <t>Fase 0</t>
+          <t>Fase 4</t>
         </is>
       </c>
       <c r="G95" s="19" t="inlineStr">
         <is>
-          <t>Sprint 0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H95" s="19" t="inlineStr">
         <is>
-          <t>H1 · 18-oct (núcleo Fase 0)</t>
-        </is>
-      </c>
-      <c r="I95" s="19" t="inlineStr">
-        <is>
-          <t>Como iglesia queremos proteger los datos sensibles.</t>
-        </is>
-      </c>
-      <c r="J95" s="19" t="inlineStr">
-        <is>
-          <t>HTTPS obligatorio y peticiones de oración ilegibles directamente en la base.</t>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="I95" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
+        </is>
+      </c>
+      <c r="J95" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
         </is>
       </c>
       <c r="K95" s="19" t="inlineStr">
@@ -8223,24 +8239,16 @@
       </c>
       <c r="L95" s="19" t="inlineStr">
         <is>
-          <t>En pruebas</t>
-        </is>
-      </c>
-      <c r="M95" s="19" t="inlineStr">
-        <is>
-          <t>Rama feature/m3-peticiones-oracion · 166 pruebas de backend y 32 de frontend pasan; probado contra la base real</t>
-        </is>
-      </c>
-      <c r="N95" s="19" t="inlineStr">
-        <is>
-          <t>2026-10-24 · Peticiones cifradas a nivel de campo; falta cifrado en reposo de toda la base (proveedor de nube).</t>
-        </is>
-      </c>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M95" s="19" t="inlineStr"/>
+      <c r="N95" s="19" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" s="18" t="inlineStr">
         <is>
-          <t>NF-03</t>
+          <t>NF-01</t>
         </is>
       </c>
       <c r="B96" s="19" t="inlineStr">
@@ -8250,7 +8258,7 @@
       </c>
       <c r="C96" s="19" t="inlineStr">
         <is>
-          <t>Bitácora de auditoría de solo-añadir: quién consultó o modificó expedientes, ofrendas y asistencias.</t>
+          <t>Cumplimiento de la LFPDPPP: aviso de privacidad, consentimiento y derechos ARCO.</t>
         </is>
       </c>
       <c r="D96" s="19" t="inlineStr">
@@ -8280,12 +8288,12 @@
       </c>
       <c r="I96" s="19" t="inlineStr">
         <is>
-          <t>Como pastor quiero una bitácora que nadie pueda alterar.</t>
+          <t>Como iglesia queremos cumplir con la LFPDPPP.</t>
         </is>
       </c>
       <c r="J96" s="19" t="inlineStr">
         <is>
-          <t>El usuario de la aplicación no puede actualizar ni borrar registros de bitácora.</t>
+          <t>Aviso de privacidad, consentimiento y atención de derechos ARCO disponibles.</t>
         </is>
       </c>
       <c r="K96" s="19" t="inlineStr">
@@ -8295,24 +8303,16 @@
       </c>
       <c r="L96" s="19" t="inlineStr">
         <is>
-          <t>En pruebas</t>
-        </is>
-      </c>
-      <c r="M96" s="19" t="inlineStr">
-        <is>
-          <t>Rama feature/nf-03-bitacora · 69 pruebas de backend pasan</t>
-        </is>
-      </c>
-      <c r="N96" s="19" t="inlineStr">
-        <is>
-          <t>2026-10-10 · Bloqueo en aplicación y trigger de PostgreSQL (UPDATE/DELETE/TRUNCATE); pantalla de consulta con permiso bitacora.ver.</t>
-        </is>
-      </c>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M96" s="19" t="inlineStr"/>
+      <c r="N96" s="19" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" s="18" t="inlineStr">
         <is>
-          <t>NF-04</t>
+          <t>NF-02</t>
         </is>
       </c>
       <c r="B97" s="19" t="inlineStr">
@@ -8322,7 +8322,7 @@
       </c>
       <c r="C97" s="19" t="inlineStr">
         <is>
-          <t>Respaldos automáticos diarios cifrados y prueba periódica de restauración.</t>
+          <t>Cifrado en tránsito y en reposo. Cifrado adicional a nivel de campo para peticiones de oración.</t>
         </is>
       </c>
       <c r="D97" s="19" t="inlineStr">
@@ -8352,12 +8352,12 @@
       </c>
       <c r="I97" s="19" t="inlineStr">
         <is>
-          <t>Como iglesia queremos no perder información.</t>
+          <t>Como iglesia queremos proteger los datos sensibles.</t>
         </is>
       </c>
       <c r="J97" s="19" t="inlineStr">
         <is>
-          <t>Respaldo diario cifrado y restauración probada en un ambiente de pruebas.</t>
+          <t>HTTPS obligatorio y peticiones de oración ilegibles directamente en la base.</t>
         </is>
       </c>
       <c r="K97" s="19" t="inlineStr">
@@ -8367,16 +8367,24 @@
       </c>
       <c r="L97" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M97" s="19" t="inlineStr"/>
-      <c r="N97" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M97" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/m3-peticiones-oracion · 166 pruebas de backend y 32 de frontend pasan; probado contra la base real</t>
+        </is>
+      </c>
+      <c r="N97" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-24 · Peticiones cifradas a nivel de campo; falta cifrado en reposo de toda la base (proveedor de nube).</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="18" t="inlineStr">
         <is>
-          <t>NF-05</t>
+          <t>NF-03</t>
         </is>
       </c>
       <c r="B98" s="19" t="inlineStr">
@@ -8386,61 +8394,69 @@
       </c>
       <c r="C98" s="19" t="inlineStr">
         <is>
-          <t>Disponibilidad esperada en horarios de servicio (fines de semana y reuniones de grupo). Por definir meta.</t>
-        </is>
-      </c>
-      <c r="D98" s="21" t="inlineStr">
-        <is>
-          <t>Nuevo v3</t>
+          <t>Bitácora de auditoría de solo-añadir: quién consultó o modificó expedientes, ofrendas y asistencias.</t>
+        </is>
+      </c>
+      <c r="D98" s="19" t="inlineStr">
+        <is>
+          <t>v3</t>
         </is>
       </c>
       <c r="E98" s="19" t="inlineStr">
         <is>
-          <t>Fuera del MVP</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="F98" s="19" t="inlineStr">
         <is>
-          <t>Transversal</t>
+          <t>Fase 0</t>
         </is>
       </c>
       <c r="G98" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sprint 1</t>
         </is>
       </c>
       <c r="H98" s="19" t="inlineStr">
         <is>
-          <t>Posterior</t>
-        </is>
-      </c>
-      <c r="I98" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
-        </is>
-      </c>
-      <c r="J98" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
+          <t>H1 · 18-oct (núcleo Fase 0)</t>
+        </is>
+      </c>
+      <c r="I98" s="19" t="inlineStr">
+        <is>
+          <t>Como pastor quiero una bitácora que nadie pueda alterar.</t>
+        </is>
+      </c>
+      <c r="J98" s="19" t="inlineStr">
+        <is>
+          <t>El usuario de la aplicación no puede actualizar ni borrar registros de bitácora.</t>
         </is>
       </c>
       <c r="K98" s="19" t="inlineStr">
         <is>
-          <t>Por definir</t>
+          <t>VoBo pendiente</t>
         </is>
       </c>
       <c r="L98" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M98" s="19" t="inlineStr"/>
-      <c r="N98" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M98" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/nf-03-bitacora · 69 pruebas de backend pasan</t>
+        </is>
+      </c>
+      <c r="N98" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-10 · Bloqueo en aplicación y trigger de PostgreSQL (UPDATE/DELETE/TRUNCATE); pantalla de consulta con permiso bitacora.ver.</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="18" t="inlineStr">
         <is>
-          <t>NF-06</t>
+          <t>NF-04</t>
         </is>
       </c>
       <c r="B99" s="19" t="inlineStr">
@@ -8450,7 +8466,7 @@
       </c>
       <c r="C99" s="19" t="inlineStr">
         <is>
-          <t>Pase de lista sin conexión con sincronización posterior (reuniones en domicilios con mala señal).</t>
+          <t>Respaldos automáticos diarios cifrados y prueba periódica de restauración.</t>
         </is>
       </c>
       <c r="D99" s="19" t="inlineStr">
@@ -8470,22 +8486,22 @@
       </c>
       <c r="G99" s="19" t="inlineStr">
         <is>
-          <t>Sprint 3</t>
+          <t>Sprint 0</t>
         </is>
       </c>
       <c r="H99" s="19" t="inlineStr">
         <is>
-          <t>H3 · MVP (Grupos)</t>
+          <t>H1 · 18-oct (núcleo Fase 0)</t>
         </is>
       </c>
       <c r="I99" s="19" t="inlineStr">
         <is>
-          <t>Como secretario quiero que el pase de lista funcione sin señal.</t>
+          <t>Como iglesia queremos no perder información.</t>
         </is>
       </c>
       <c r="J99" s="19" t="inlineStr">
         <is>
-          <t>Prueba en modo avión y sincronización al reconectar.</t>
+          <t>Respaldo diario cifrado y restauración probada en un ambiente de pruebas.</t>
         </is>
       </c>
       <c r="K99" s="19" t="inlineStr">
@@ -8495,24 +8511,16 @@
       </c>
       <c r="L99" s="19" t="inlineStr">
         <is>
-          <t>En pruebas</t>
-        </is>
-      </c>
-      <c r="M99" s="19" t="inlineStr">
-        <is>
-          <t>Rama feature/nf-06-sin-conexion · 117 pruebas de backend y 27 de frontend; probado en Chrome real con service worker</t>
-        </is>
-      </c>
-      <c r="N99" s="19" t="inlineStr">
-        <is>
-          <t>2026-10-24 · Probado de punta a punta en Chrome (sin red → cola → sincronización). Pendiente probar en Android e iOS reales.</t>
-        </is>
-      </c>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M99" s="19" t="inlineStr"/>
+      <c r="N99" s="19" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" s="18" t="inlineStr">
         <is>
-          <t>NF-07</t>
+          <t>NF-05</t>
         </is>
       </c>
       <c r="B100" s="19" t="inlineStr">
@@ -8522,47 +8530,47 @@
       </c>
       <c r="C100" s="19" t="inlineStr">
         <is>
-          <t>Funciona en Android, iOS y escritorio. En iOS, las notificaciones push requieren instalar la PWA; el respaldo por WhatsApp cubre el resto.</t>
-        </is>
-      </c>
-      <c r="D100" s="19" t="inlineStr">
-        <is>
-          <t>v3</t>
+          <t>Disponibilidad esperada en horarios de servicio (fines de semana y reuniones de grupo). Por definir meta.</t>
+        </is>
+      </c>
+      <c r="D100" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3</t>
         </is>
       </c>
       <c r="E100" s="19" t="inlineStr">
         <is>
-          <t>MVP</t>
+          <t>Fuera del MVP</t>
         </is>
       </c>
       <c r="F100" s="19" t="inlineStr">
         <is>
-          <t>Fase 0</t>
+          <t>Transversal</t>
         </is>
       </c>
       <c r="G100" s="19" t="inlineStr">
         <is>
-          <t>Sprint 0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H100" s="19" t="inlineStr">
         <is>
-          <t>H1 · 18-oct (núcleo Fase 0)</t>
-        </is>
-      </c>
-      <c r="I100" s="19" t="inlineStr">
-        <is>
-          <t>Como usuario quiero usar el sistema en mi dispositivo.</t>
-        </is>
-      </c>
-      <c r="J100" s="19" t="inlineStr">
-        <is>
-          <t>Pruebas en Android, iOS y escritorio; push en iOS con la PWA instalada y respaldo por WhatsApp.</t>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="I100" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
+        </is>
+      </c>
+      <c r="J100" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
         </is>
       </c>
       <c r="K100" s="19" t="inlineStr">
         <is>
-          <t>VoBo pendiente</t>
+          <t>Por definir</t>
         </is>
       </c>
       <c r="L100" s="19" t="inlineStr">
@@ -8576,7 +8584,7 @@
     <row r="101">
       <c r="A101" s="18" t="inlineStr">
         <is>
-          <t>NF-08</t>
+          <t>NF-06</t>
         </is>
       </c>
       <c r="B101" s="19" t="inlineStr">
@@ -8586,12 +8594,12 @@
       </c>
       <c r="C101" s="19" t="inlineStr">
         <is>
-          <t>Dimensionamiento para ~1,000 personas, con picos los fines de semana, y margen de crecimiento.</t>
-        </is>
-      </c>
-      <c r="D101" s="21" t="inlineStr">
-        <is>
-          <t>Resp. P8</t>
+          <t>Pase de lista sin conexión con sincronización posterior (reuniones en domicilios con mala señal).</t>
+        </is>
+      </c>
+      <c r="D101" s="19" t="inlineStr">
+        <is>
+          <t>v3</t>
         </is>
       </c>
       <c r="E101" s="19" t="inlineStr">
@@ -8606,22 +8614,22 @@
       </c>
       <c r="G101" s="19" t="inlineStr">
         <is>
-          <t>Sprint 0</t>
+          <t>Sprint 3</t>
         </is>
       </c>
       <c r="H101" s="19" t="inlineStr">
         <is>
-          <t>H1 · 18-oct (núcleo Fase 0)</t>
+          <t>H3 · MVP (Grupos)</t>
         </is>
       </c>
       <c r="I101" s="19" t="inlineStr">
         <is>
-          <t>Como iglesia queremos que el sistema soporte a ~1,000 personas.</t>
+          <t>Como secretario quiero que el pase de lista funcione sin señal.</t>
         </is>
       </c>
       <c r="J101" s="19" t="inlineStr">
         <is>
-          <t>Prueba de carga con volumen representativo (por definir) sin degradación.</t>
+          <t>Prueba en modo avión y sincronización al reconectar.</t>
         </is>
       </c>
       <c r="K101" s="19" t="inlineStr">
@@ -8631,16 +8639,24 @@
       </c>
       <c r="L101" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M101" s="19" t="inlineStr"/>
-      <c r="N101" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M101" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/nf-06-sin-conexion · 117 pruebas de backend y 27 de frontend; probado en Chrome real con service worker</t>
+        </is>
+      </c>
+      <c r="N101" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-24 · Probado de punta a punta en Chrome (sin red → cola → sincronización). Pendiente probar en Android e iOS reales.</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="18" t="inlineStr">
         <is>
-          <t>NF-09</t>
+          <t>NF-07</t>
         </is>
       </c>
       <c r="B102" s="19" t="inlineStr">
@@ -8650,42 +8666,42 @@
       </c>
       <c r="C102" s="19" t="inlineStr">
         <is>
-          <t>Reportes transversales: asistencia, finanzas, crecimiento de la iglesia, exportables a Excel y PDF.</t>
-        </is>
-      </c>
-      <c r="D102" s="21" t="inlineStr">
-        <is>
-          <t>Nuevo v3</t>
+          <t>Funciona en Android, iOS y escritorio. En iOS, las notificaciones push requieren instalar la PWA; el respaldo por WhatsApp cubre el resto.</t>
+        </is>
+      </c>
+      <c r="D102" s="19" t="inlineStr">
+        <is>
+          <t>v3</t>
         </is>
       </c>
       <c r="E102" s="19" t="inlineStr">
         <is>
-          <t>Fuera del MVP</t>
+          <t>MVP</t>
         </is>
       </c>
       <c r="F102" s="19" t="inlineStr">
         <is>
-          <t>Transversal</t>
+          <t>Fase 0</t>
         </is>
       </c>
       <c r="G102" s="19" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Sprint 0</t>
         </is>
       </c>
       <c r="H102" s="19" t="inlineStr">
         <is>
-          <t>Posterior</t>
-        </is>
-      </c>
-      <c r="I102" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
-        </is>
-      </c>
-      <c r="J102" s="20" t="inlineStr">
-        <is>
-          <t>Se define al iniciar la fase.</t>
+          <t>H1 · 18-oct (núcleo Fase 0)</t>
+        </is>
+      </c>
+      <c r="I102" s="19" t="inlineStr">
+        <is>
+          <t>Como usuario quiero usar el sistema en mi dispositivo.</t>
+        </is>
+      </c>
+      <c r="J102" s="19" t="inlineStr">
+        <is>
+          <t>Pruebas en Android, iOS y escritorio; push en iOS con la PWA instalada y respaldo por WhatsApp.</t>
         </is>
       </c>
       <c r="K102" s="19" t="inlineStr">
@@ -8704,7 +8720,7 @@
     <row r="103">
       <c r="A103" s="18" t="inlineStr">
         <is>
-          <t>NF-10</t>
+          <t>NF-08</t>
         </is>
       </c>
       <c r="B103" s="19" t="inlineStr">
@@ -8714,12 +8730,12 @@
       </c>
       <c r="C103" s="19" t="inlineStr">
         <is>
-          <t>Usabilidad para personas mayores: tipografía grande, alto contraste, flujos cortos (ver sección 5).</t>
-        </is>
-      </c>
-      <c r="D103" s="19" t="inlineStr">
-        <is>
-          <t>v3 + Obs. 1</t>
+          <t>Dimensionamiento para ~1,000 personas, con picos los fines de semana, y margen de crecimiento.</t>
+        </is>
+      </c>
+      <c r="D103" s="21" t="inlineStr">
+        <is>
+          <t>Resp. P8</t>
         </is>
       </c>
       <c r="E103" s="19" t="inlineStr">
@@ -8744,12 +8760,12 @@
       </c>
       <c r="I103" s="19" t="inlineStr">
         <is>
-          <t>Como persona mayor quiero una interfaz fácil de leer y usar.</t>
+          <t>Como iglesia queremos que el sistema soporte a ~1,000 personas.</t>
         </is>
       </c>
       <c r="J103" s="19" t="inlineStr">
         <is>
-          <t>Texto base 18 px, botones de al menos 48 px, contraste AA; prueba con usuarios mayores.</t>
+          <t>Prueba de carga con volumen representativo (por definir) sin degradación.</t>
         </is>
       </c>
       <c r="K103" s="19" t="inlineStr">
@@ -8765,9 +8781,137 @@
       <c r="M103" s="19" t="inlineStr"/>
       <c r="N103" s="19" t="inlineStr"/>
     </row>
+    <row r="104">
+      <c r="A104" s="18" t="inlineStr">
+        <is>
+          <t>NF-09</t>
+        </is>
+      </c>
+      <c r="B104" s="19" t="inlineStr">
+        <is>
+          <t>No funcionales</t>
+        </is>
+      </c>
+      <c r="C104" s="19" t="inlineStr">
+        <is>
+          <t>Reportes transversales: asistencia, finanzas, crecimiento de la iglesia, exportables a Excel y PDF.</t>
+        </is>
+      </c>
+      <c r="D104" s="21" t="inlineStr">
+        <is>
+          <t>Nuevo v3</t>
+        </is>
+      </c>
+      <c r="E104" s="19" t="inlineStr">
+        <is>
+          <t>Fuera del MVP</t>
+        </is>
+      </c>
+      <c r="F104" s="19" t="inlineStr">
+        <is>
+          <t>Transversal</t>
+        </is>
+      </c>
+      <c r="G104" s="19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H104" s="19" t="inlineStr">
+        <is>
+          <t>Posterior</t>
+        </is>
+      </c>
+      <c r="I104" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
+        </is>
+      </c>
+      <c r="J104" s="20" t="inlineStr">
+        <is>
+          <t>Se define al iniciar la fase.</t>
+        </is>
+      </c>
+      <c r="K104" s="19" t="inlineStr">
+        <is>
+          <t>VoBo pendiente</t>
+        </is>
+      </c>
+      <c r="L104" s="19" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M104" s="19" t="inlineStr"/>
+      <c r="N104" s="19" t="inlineStr"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="18" t="inlineStr">
+        <is>
+          <t>NF-10</t>
+        </is>
+      </c>
+      <c r="B105" s="19" t="inlineStr">
+        <is>
+          <t>No funcionales</t>
+        </is>
+      </c>
+      <c r="C105" s="19" t="inlineStr">
+        <is>
+          <t>Usabilidad para personas mayores: tipografía grande, alto contraste, flujos cortos (ver sección 5).</t>
+        </is>
+      </c>
+      <c r="D105" s="19" t="inlineStr">
+        <is>
+          <t>v3 + Obs. 1</t>
+        </is>
+      </c>
+      <c r="E105" s="19" t="inlineStr">
+        <is>
+          <t>MVP</t>
+        </is>
+      </c>
+      <c r="F105" s="19" t="inlineStr">
+        <is>
+          <t>Fase 0</t>
+        </is>
+      </c>
+      <c r="G105" s="19" t="inlineStr">
+        <is>
+          <t>Sprint 0</t>
+        </is>
+      </c>
+      <c r="H105" s="19" t="inlineStr">
+        <is>
+          <t>H1 · 18-oct (núcleo Fase 0)</t>
+        </is>
+      </c>
+      <c r="I105" s="19" t="inlineStr">
+        <is>
+          <t>Como persona mayor quiero una interfaz fácil de leer y usar.</t>
+        </is>
+      </c>
+      <c r="J105" s="19" t="inlineStr">
+        <is>
+          <t>Texto base 18 px, botones de al menos 48 px, contraste AA; prueba con usuarios mayores.</t>
+        </is>
+      </c>
+      <c r="K105" s="19" t="inlineStr">
+        <is>
+          <t>VoBo pendiente</t>
+        </is>
+      </c>
+      <c r="L105" s="19" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M105" s="19" t="inlineStr"/>
+      <c r="N105" s="19" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N103"/>
-  <conditionalFormatting sqref="L2:L103">
+  <autoFilter ref="A1:N105"/>
+  <conditionalFormatting sqref="L2:L105">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$L2="Hecho"</formula>
     </cfRule>
@@ -8784,7 +8928,7 @@
       <formula>$L2="Bloqueado"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K2:K103">
+  <conditionalFormatting sqref="K2:K105">
     <cfRule type="expression" priority="6" dxfId="0">
       <formula>$K2="Aprobado"</formula>
     </cfRule>
@@ -8792,16 +8936,16 @@
       <formula>$K2="Por definir"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H2:H103">
+  <conditionalFormatting sqref="H2:H105">
     <cfRule type="expression" priority="8" dxfId="5">
       <formula>LEFT($H2,2)="H1"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="L2:L103" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="L2:L105" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Pendiente,En diseño,En desarrollo,En pruebas,Hecho,Bloqueado"</formula1>
     </dataValidation>
-    <dataValidation sqref="K2:K103" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="K2:K105" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"VoBo pendiente,Aprobado,Por definir,Rechazado"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Matriz de trazabilidad al día con el paso 10
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/trazabilidad/Matriz de Trazabilidad MDF.xlsx
+++ b/docs/trazabilidad/Matriz de Trazabilidad MDF.xlsx
@@ -4356,12 +4356,12 @@
       </c>
       <c r="M36" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/paso-9-oraciones-vehiculos · pruebas de backend y 110 de frontend pasan; lint, estilos y compilación limpios</t>
+          <t>Rama feature/paso-10-cerrar-sesion · 111 pruebas de frontend pasan; lint y compilación limpios</t>
         </is>
       </c>
       <c r="N36" s="19" t="inlineStr">
         <is>
-          <t>2026-10-30 · Vehículos propios en Mi cuenta y consulta en la ficha.</t>
+          <t>2026-10-30 · Vehículos propios en Mi cuenta y consulta en la ficha; leyenda de uso exclusivo para ubicar a la persona.</t>
         </is>
       </c>
     </row>
@@ -9505,7 +9505,7 @@
       </c>
       <c r="E20" s="24" t="inlineStr">
         <is>
-          <t>Corregido (v3.14)</t>
+          <t>Corregido (v3.14); reforzado el 30-oct-2026: si el servidor ya no reconoce la sesión, igual se limpia el dispositivo y se vuelve al login</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Formularios configurables y aviso de privacidad sustituible (paso 11)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/trazabilidad/Matriz de Trazabilidad MDF.xlsx
+++ b/docs/trazabilidad/Matriz de Trazabilidad MDF.xlsx
@@ -2015,11 +2015,19 @@
       </c>
       <c r="L2" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M2" s="19" t="inlineStr"/>
-      <c r="N2" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M2" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/paso-11-formularios · pruebas de backend y 116 de frontend pasan; lint, estilos y compilación limpios</t>
+        </is>
+      </c>
+      <c r="N2" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-30 · Diseñador de campos adicionales para Personas y Grupos (más el de peticiones, ya existente), con siete tipos de campo.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="18" t="inlineStr">
@@ -2271,11 +2279,19 @@
       </c>
       <c r="L6" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M6" s="19" t="inlineStr"/>
-      <c r="N6" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M6" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/paso-11-formularios · pruebas de backend y 116 de frontend pasan; lint, estilos y compilación limpios</t>
+        </is>
+      </c>
+      <c r="N6" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-30 · El diseñador de formularios ya está disponible; layouts y flujos avanzados siguen en Fase 5.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="18" t="inlineStr">
@@ -2335,11 +2351,19 @@
       </c>
       <c r="L7" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M7" s="19" t="inlineStr"/>
-      <c r="N7" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M7" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/paso-11-formularios · pruebas de backend y 116 de frontend pasan; lint, estilos y compilación limpios</t>
+        </is>
+      </c>
+      <c r="N7" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-30 · Modelo híbrido para Persona y Grupo (campos extra en el propio registro). Pendiente: Reunión y Ofrenda.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="18" t="inlineStr">
@@ -2399,11 +2423,19 @@
       </c>
       <c r="L8" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M8" s="19" t="inlineStr"/>
-      <c r="N8" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M8" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/paso-11-formularios · pruebas de backend y 116 de frontend pasan; lint, estilos y compilación limpios</t>
+        </is>
+      </c>
+      <c r="N8" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-30 · Campos de relación a persona, grupo o ministerio con vínculo por id; el reporte cruza una persona elegida con su grupo.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="18" t="inlineStr">
@@ -2463,11 +2495,19 @@
       </c>
       <c r="L9" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M9" s="19" t="inlineStr"/>
-      <c r="N9" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M9" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/paso-11-formularios · pruebas de backend y 116 de frontend pasan; lint, estilos y compilación limpios</t>
+        </is>
+      </c>
+      <c r="N9" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-30 · Los campos solo se desactivan, cada cambio crea versión y los marcados como reportables aparecen en el reporte.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="18" t="inlineStr">
@@ -2599,11 +2639,19 @@
       </c>
       <c r="L11" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M11" s="19" t="inlineStr"/>
-      <c r="N11" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M11" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/paso-11-formularios · pruebas de backend y 116 de frontend pasan; lint, estilos y compilación limpios</t>
+        </is>
+      </c>
+      <c r="N11" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-30 · Campos configurables del expediente visibles en el alta y en la ficha.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="18" t="inlineStr">
@@ -3162,7 +3210,7 @@
       </c>
       <c r="C20" s="19" t="inlineStr">
         <is>
-          <t>Aviso de privacidad y consentimiento al registrar a cualquier persona o activar una cuenta, con consentimiento aparte para la foto. Cada consentimiento guarda la versión del aviso y la fecha. Por ahora el texto es genérico de ejemplo y debe sustituirse por el oficial antes de producción.</t>
+          <t>Aviso de privacidad y consentimiento al registrar a cualquier persona o activar una cuenta, con consentimiento aparte para la foto. Cada consentimiento guarda la versión del aviso y la fecha. El texto vigente se publica desde la aplicación (Aviso de privacidad); cuando cambia, cada persona debe aceptar la versión nueva. Hoy rige un texto provisional que debe sustituirse por el oficial antes de producción.</t>
         </is>
       </c>
       <c r="D20" s="19" t="inlineStr">
@@ -3212,12 +3260,12 @@
       </c>
       <c r="M20" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/m1-01-expediente · 56 pruebas de backend y 6 de frontend pasan</t>
+          <t>Rama feature/paso-11-formularios · pruebas de backend y 116 de frontend pasan; lint, estilos y compilación limpios</t>
         </is>
       </c>
       <c r="N20" s="19" t="inlineStr">
         <is>
-          <t>2026-10-05 · Texto del aviso genérico; sustituir por el oficial antes de producción.</t>
+          <t>2026-10-30 · El aviso se publica desde la aplicación y cada persona acepta la versión nueva; rige un texto provisional (0.2) que incluye vehículos y formularios. Falta el texto oficial.</t>
         </is>
       </c>
     </row>
@@ -4356,12 +4404,12 @@
       </c>
       <c r="M36" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/paso-9-oraciones-vehiculos · pruebas de backend y 110 de frontend pasan; lint, estilos y compilación limpios</t>
+          <t>Rama feature/paso-10-cerrar-sesion · 111 pruebas de frontend pasan; lint y compilación limpios</t>
         </is>
       </c>
       <c r="N36" s="19" t="inlineStr">
         <is>
-          <t>2026-10-30 · Vehículos propios en Mi cuenta y consulta en la ficha.</t>
+          <t>2026-10-30 · Vehículos propios en Mi cuenta y consulta en la ficha; leyenda de uso exclusivo para ubicar a la persona.</t>
         </is>
       </c>
     </row>
@@ -9505,7 +9553,7 @@
       </c>
       <c r="E20" s="24" t="inlineStr">
         <is>
-          <t>Corregido (v3.14)</t>
+          <t>Corregido (v3.14); reforzado el 30-oct-2026: si el servidor ya no reconoce la sesión, igual se limpia el dispositivo y se vuelve al login</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Manual de usuario, presentación y pendientes de definición
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/trazabilidad/Matriz de Trazabilidad MDF.xlsx
+++ b/docs/trazabilidad/Matriz de Trazabilidad MDF.xlsx
@@ -2015,11 +2015,19 @@
       </c>
       <c r="L2" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M2" s="19" t="inlineStr"/>
-      <c r="N2" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M2" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/paso-11-formularios · pruebas de backend y 116 de frontend pasan; lint, estilos y compilación limpios</t>
+        </is>
+      </c>
+      <c r="N2" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-30 · Diseñador de campos adicionales para Personas y Grupos (más el de peticiones, ya existente), con siete tipos de campo.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="18" t="inlineStr">
@@ -2271,11 +2279,19 @@
       </c>
       <c r="L6" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M6" s="19" t="inlineStr"/>
-      <c r="N6" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M6" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/paso-11-formularios · pruebas de backend y 116 de frontend pasan; lint, estilos y compilación limpios</t>
+        </is>
+      </c>
+      <c r="N6" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-30 · El diseñador de formularios ya está disponible; layouts y flujos avanzados siguen en Fase 5.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="18" t="inlineStr">
@@ -2335,11 +2351,19 @@
       </c>
       <c r="L7" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M7" s="19" t="inlineStr"/>
-      <c r="N7" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M7" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/paso-11-formularios · pruebas de backend y 116 de frontend pasan; lint, estilos y compilación limpios</t>
+        </is>
+      </c>
+      <c r="N7" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-30 · Modelo híbrido para Persona y Grupo (campos extra en el propio registro). Pendiente: Reunión y Ofrenda.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="18" t="inlineStr">
@@ -2399,11 +2423,19 @@
       </c>
       <c r="L8" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M8" s="19" t="inlineStr"/>
-      <c r="N8" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M8" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/paso-11-formularios · pruebas de backend y 116 de frontend pasan; lint, estilos y compilación limpios</t>
+        </is>
+      </c>
+      <c r="N8" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-30 · Campos de relación a persona, grupo o ministerio con vínculo por id; el reporte cruza una persona elegida con su grupo.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="18" t="inlineStr">
@@ -2463,11 +2495,19 @@
       </c>
       <c r="L9" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M9" s="19" t="inlineStr"/>
-      <c r="N9" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M9" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/paso-11-formularios · pruebas de backend y 116 de frontend pasan; lint, estilos y compilación limpios</t>
+        </is>
+      </c>
+      <c r="N9" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-30 · Los campos solo se desactivan, cada cambio crea versión y los marcados como reportables aparecen en el reporte.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="18" t="inlineStr">
@@ -2599,11 +2639,19 @@
       </c>
       <c r="L11" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M11" s="19" t="inlineStr"/>
-      <c r="N11" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M11" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/paso-11-formularios · pruebas de backend y 116 de frontend pasan; lint, estilos y compilación limpios</t>
+        </is>
+      </c>
+      <c r="N11" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-30 · Campos configurables del expediente visibles en el alta y en la ficha.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="18" t="inlineStr">
@@ -3162,7 +3210,7 @@
       </c>
       <c r="C20" s="19" t="inlineStr">
         <is>
-          <t>Aviso de privacidad y consentimiento al registrar a cualquier persona o activar una cuenta, con consentimiento aparte para la foto. Cada consentimiento guarda la versión del aviso y la fecha. Por ahora el texto es genérico de ejemplo y debe sustituirse por el oficial antes de producción.</t>
+          <t>Aviso de privacidad y consentimiento al registrar a cualquier persona o activar una cuenta, con consentimiento aparte para la foto. Cada consentimiento guarda la versión del aviso y la fecha. El texto vigente se publica desde la aplicación (Aviso de privacidad); cuando cambia, cada persona debe aceptar la versión nueva. Hoy rige un texto provisional que debe sustituirse por el oficial antes de producción.</t>
         </is>
       </c>
       <c r="D20" s="19" t="inlineStr">
@@ -3212,12 +3260,12 @@
       </c>
       <c r="M20" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/m1-01-expediente · 56 pruebas de backend y 6 de frontend pasan</t>
+          <t>Rama feature/paso-11-formularios · pruebas de backend y 116 de frontend pasan; lint, estilos y compilación limpios</t>
         </is>
       </c>
       <c r="N20" s="19" t="inlineStr">
         <is>
-          <t>2026-10-05 · Texto del aviso genérico; sustituir por el oficial antes de producción.</t>
+          <t>2026-10-30 · El aviso se publica desde la aplicación y cada persona acepta la versión nueva; rige un texto provisional (0.2) que incluye vehículos y formularios. Falta el texto oficial.</t>
         </is>
       </c>
     </row>
@@ -4356,12 +4404,12 @@
       </c>
       <c r="M36" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/paso-9-oraciones-vehiculos · pruebas de backend y 110 de frontend pasan; lint, estilos y compilación limpios</t>
+          <t>Rama feature/paso-10-cerrar-sesion · 111 pruebas de frontend pasan; lint y compilación limpios</t>
         </is>
       </c>
       <c r="N36" s="19" t="inlineStr">
         <is>
-          <t>2026-10-30 · Vehículos propios en Mi cuenta y consulta en la ficha.</t>
+          <t>2026-10-30 · Vehículos propios en Mi cuenta y consulta en la ficha; leyenda de uso exclusivo para ubicar a la persona.</t>
         </is>
       </c>
     </row>
@@ -9505,7 +9553,7 @@
       </c>
       <c r="E20" s="24" t="inlineStr">
         <is>
-          <t>Corregido (v3.14)</t>
+          <t>Corregido (v3.14); reforzado el 30-oct-2026: si el servidor ya no reconoce la sesión, igual se limpia el dispositivo y se vuelve al login</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ofrendas, peticiones y bajas configurables por rol (paso 12)
- Roles de grupo: permisos de ofrendas (ver, capturar, avalar y suplencias) y de
  peticiones (registrar, ver); las reglas de seguridad del dinero siguen fijas
- Baja, traslado y reactivación: permiso de rol con alcance (su grupo)
- Publicar avisos en el grupo se decide por el permiso del rol
- Requerimientos v3.24 y matriz de trazabilidad

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/trazabilidad/Matriz de Trazabilidad MDF.xlsx
+++ b/docs/trazabilidad/Matriz de Trazabilidad MDF.xlsx
@@ -2775,11 +2775,19 @@
       </c>
       <c r="L13" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="M13" s="19" t="inlineStr"/>
-      <c r="N13" s="19" t="inlineStr"/>
+          <t>En pruebas</t>
+        </is>
+      </c>
+      <c r="M13" s="19" t="inlineStr">
+        <is>
+          <t>Rama feature/paso-11-formularios · pruebas de backend y 116 de frontend pasan; lint, estilos y compilación limpios</t>
+        </is>
+      </c>
+      <c r="N13" s="19" t="inlineStr">
+        <is>
+          <t>2026-10-30 · Parcial: ya se registran los vehículos de cada persona (Mi cuenta). Faltan otros bienes y las alertas por placa (M1-05 y M1-06).</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="18" t="inlineStr">
@@ -2972,12 +2980,12 @@
       </c>
       <c r="M16" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/paso-6-roles-permisos · pruebas de backend y 97 de frontend pasan; lint, estilos y compilación limpios</t>
+          <t>Rama feature/paso-12-roles-ofrendas-bajas · pruebas de backend y 116 de frontend pasan; lint, estilos y compilación limpios</t>
         </is>
       </c>
       <c r="N16" s="19" t="inlineStr">
         <is>
-          <t>2026-10-29 · Roles base más la Secretaria; asignación con jerarquía (nadie otorga un rol más alto que el suyo, solo el Super Usuario asigna Super Usuario); baja y traslado solo por un superior.</t>
+          <t>2026-10-30 · Roles base más la Secretaria; asignación con jerarquía (nadie otorga un rol más alto que el suyo); la baja es un permiso de rol, solo hacia abajo en la jerarquía y dentro del alcance de cada quien (su grupo).</t>
         </is>
       </c>
     </row>
@@ -4188,12 +4196,12 @@
       </c>
       <c r="M33" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/paso-8-ministerios-mi-cuenta · pruebas de backend y 108 de frontend pasan; lint, estilos y compilación limpios</t>
+          <t>Rama feature/paso-12-roles-ofrendas-bajas · pruebas de backend y 116 de frontend pasan; lint, estilos y compilación limpios</t>
         </is>
       </c>
       <c r="N33" s="19" t="inlineStr">
         <is>
-          <t>2026-10-30 · Roles de ministerio y de grupo configurables desde Roles y permisos; roles base y roles nuevos; las ofrendas y peticiones de grupo siguen con reglas fijas.</t>
+          <t>2026-10-30 · Roles de ministerio y de grupo configurables desde Roles y permisos, incluidas las ofrendas (ver, capturar, avalar y suplencias) y las peticiones del grupo. Las reglas de seguridad del dinero siguen fijas.</t>
         </is>
       </c>
     </row>
@@ -5780,12 +5788,12 @@
       </c>
       <c r="M57" s="19" t="inlineStr">
         <is>
-          <t>Rama feature/m3-ofrendas-ajustes · 121 pruebas de backend y 14 de frontend pasan</t>
+          <t>Rama feature/paso-12-roles-ofrendas-bajas · pruebas de backend y 116 de frontend pasan; lint, estilos y compilación limpios</t>
         </is>
       </c>
       <c r="N57" s="19" t="inlineStr">
         <is>
-          <t>2026-10-24 · Con suplencias del Líder, diferencias visibles y límites configurables. Falta validar con la iglesia.</t>
+          <t>2026-10-30 · Quién ve, captura y avala (y las suplencias) se configura por rol del grupo; quien captura no avala, el aval pide PIN. Falta validar con la iglesia.</t>
         </is>
       </c>
     </row>

</xml_diff>